<commit_message>
Mueve el análisis de «Contra el canon» a analisis/ y cataloga Giunta 2014
- Traslada «Sistematización - Contra el canon (Giunta).md» de
  Sistematización/ a la carpeta analisis/.
- Cataloga «Teoría/Giunta2014_CuandoEmpiezaElArteContemporaneo.md»
  (¿Cuándo empieza el arte contemporáneo?, arteBA, 2014) en
  tabla-teoria.csv con resumen de ~250 palabras y citas literales
  verificadas. Teoría pasa a 68 filas.
- Regenera tablas-sistematizacion.xlsx con la hoja Teoría actualizada.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bob4w11uQRyAcv1Qayw1V
</commit_message>
<xml_diff>
--- a/Sistematización/tablas-sistematizacion.xlsx
+++ b/Sistematización/tablas-sistematizacion.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$72</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cap 3 - Análisis'!$A$1:$F$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Teoría'!$A$1:$F$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Teoría'!$A$1:$F$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Extras'!$A$1:$F$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4409,7 +4409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5260,27 +5260,27 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Groys - Volverse público. Las transformaciones del arte en el ágora contemporánea (2014) [Caja Negra].md</t>
+          <t>Giunta2014_CuandoEmpiezaElArteContemporaneo.md</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>n/d (ensayo teórico; con referencias a la vanguardia histórica del siglo XX y a la cultura digital contemporánea)</t>
+          <t>Años sesenta–presente (la contemporaneidad como crisis del régimen moderno; foco desde los años 1960)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Libro (ensayos), 2014 [orig. Going Public, 2010]</t>
+          <t>Ensayo/libro bilingüe (español-inglés), 2014 (Fundación arteBA, Buenos Aires; ISBN 978-987-28023-3-2)</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Boris Groys; Immanuel Kant; G. W. F. Hegel; Marcel Duchamp; Kazimir Malevich; Walter Benjamin; Michel Foucault; Clement Greenberg; Hugo Ball; Paola Cortés Rocca (trad.); Caja Negra Editora</t>
+          <t>Andrea Giunta; Agustín Diez Fischer (notas); Tamara Stuby (traducción); Fundación arteBA; Tucumán arde</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Groys reúne ensayos que buscan escribir sobre arte de un modo no estético, invirtiendo la perspectiva dominante desde Kant. Su tesis central es que la actitud estética es la del espectador-consumidor, que subordina la producción al consumo y la teoría del arte a la sociología, y que además vuelve superflua a la obra (la vida misma ofrece mejores experiencias estéticas); frente a ella propone la poética, la perspectiva del productor, la poiesis o techné. En la modernidad tardía, con la proliferación de medios visuales e Internet, la antigua dicotomía artista/espectador colapsa: hoy hay más gente interesada en producir imágenes que en mirarlas, y todos debemos diseñar una "persona pública", un doble artificial, en un ejercicio de autopoética por el que somos ética y políticamente responsables. Relee así la vanguardia (Malevich, Ball, Duchamp) como autopoiesis, producción del propio Yo público desde el grado cero de la forma, no como shock ni transgresión. Otros ensayos desarrollan: la obligación del diseño de sí y la producción de sinceridad; la política de la instalación como espacio donde el artista actúa cual legislador soberano y heterotópico, poniendo en cuestión la reducción foucaultiana del poder a mecanismos impersonales; una crítica al ensayo de Benjamin sobre el aura, sustituyendo la pérdida irreversible por un juego contemporáneo de desterritorializaciones y re-auratizaciones donde toda copia deviene nuevo original; el universalismo débil; Marx después de Duchamp; los trabajadores del arte entre utopía y archivo; y Google como máquina filosófica que resuelve la deconstrucción.</t>
+          <t>Ensayo bilingüe (español-inglés) de Andrea Giunta publicado por Fundación arteBA (Buenos Aires, 2014), con notas de la autora y Agustín Diez Fischer. Es el núcleo germinal de su libro posterior «Contra el canon» (2020). Parte de una pregunta historiográfica —«¿Existe un arte específicamente contemporáneo?»— para sostener que «el régimen moderno ha entrado en crisis» y que la contemporaneidad se define por «la pulsión del presente, de lo inmediato», un presente «atravesado por los rastros de otras temporalidades». Rechaza explícitamente el modelo difusionista: «se sostiene la invalidez del esquema de centros y periferias para el estudio del arte contemporáneo» y propone «la noción de vanguardias simultáneas» para analizar obras insertas en la lógica global del arte pero que «activan situaciones específicas». Metodológicamente, el texto se organiza como fragmentos o pequeños ensayos temáticos (lenguajes, estrategias de comunicación, técnicas, materiales, agendas y temas), en los que las obras tienen «un rol protagónico» y no pueden «deducirse ni de las genealogías ni de los contextos»; la descripción detallada de cada pieza funciona como archivo y punto de partida interpretativo. Sitúa el umbral de la contemporaneidad en la politización y el experimentalismo de los años sesenta —cuando se quiebra la autonomía moderna del lenguaje— antes que en 1989. Aunque atiende sobre todo al arte latinoamericano (con casos como Tucumán arde), piensa la contemporaneidad como fenómeno global y situado. Anticipa así los conceptos —vanguardias simultáneas, obra como acontecimiento, crítica al canon centro-periferia— que desarrollará en extenso en «Contra el canon».</t>
         </is>
       </c>
     </row>
@@ -5292,27 +5292,27 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Harris - The Global Contemporary Art World. A Rough Guide (2017) [Wiley, ISBN 9781118288917].md</t>
+          <t>Groys - Volverse público. Las transformaciones del arte en el ágora contemporánea (2014) [Caja Negra].md</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Arte contemporáneo global posterior a 1989 (décadas de 1990-2016), con genealogía en la modernidad y el sistema colonial occidental</t>
+          <t>n/d (ensayo teórico; con referencias a la vanguardia histórica del siglo XX y a la cultura digital contemporánea)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Libro, 2017</t>
+          <t>Libro (ensayos), 2014 [orig. Going Public, 2010]</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Jonathan Harris; Bashir Makhoul; Nicholas Serota; Damien Hirst; Jeff Koons; Charles Saatchi; Hans Ulrich Obrist; Raymond Williams; Edward Said; David Harvey; Tate Modern / Art Basel; Wiley-Blackwell</t>
+          <t>Boris Groys; Immanuel Kant; G. W. F. Hegel; Marcel Duchamp; Kazimir Malevich; Walter Benjamin; Michel Foucault; Clement Greenberg; Hugo Ball; Paola Cortés Rocca (trad.); Caja Negra Editora</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Cierre de la trilogía de Harris, el libro sostiene que el mundo del arte contemporáneo global no está separado del mundo, sino que constituye un subsistema —relativamente autónomo pero funcional— del "orden/desorden mundial" globalizado, conducido por alianzas cambiantes de estados y corporaciones bajo el capitalismo neoliberal surgido en los años ochenta (Reagan, Thatcher). El marco conceptual, deudor de Williams, Said y Harvey, insiste en el carácter fundamentalmente asimétrico del sistema: las instituciones "guardianas" occidentales (Sotheby's, Christie's, Art Basel, Frieze, Tate, MoMA, Guggenheim, galerías como Gagosian y White Cube) conservan el poder de validar y explotar económicamente un arte crecientemente producido fuera de Occidente. Harris amplía la noción de "productor" más allá del artista para incluir directores, curadores y coleccionistas (Serota, Saatchi, Obrist), y subraya la borrosa frontera entre lo público y lo privado. Metodológicamente rechaza el formato de "survey": el número reducido de obras analizadas tiene valor heurístico dentro de un análisis sistémico. El cuerpo del libro se organiza en cinco estudios de caso de la "gran Asia", todos de pasado poscolonial compartido: las ferias de Hong Kong (negocio offshore y desarrollo desigual y combinado), el nuevo media art y el globalismo cultural en Corea del Sur, la Bienal de Kochi como forma retórica en India, la reproducción social y el branding del "arte chino contemporáneo" en la educación superior de la RPC, y la "ONG-ización" del arte en el Estado de Palestina. Reflexiona además sobre las categorías "global", "contemporáneo", "arte" y "mundo", y sobre la modernidad como problema no resuelto de igualdad.</t>
+          <t>Groys reúne ensayos que buscan escribir sobre arte de un modo no estético, invirtiendo la perspectiva dominante desde Kant. Su tesis central es que la actitud estética es la del espectador-consumidor, que subordina la producción al consumo y la teoría del arte a la sociología, y que además vuelve superflua a la obra (la vida misma ofrece mejores experiencias estéticas); frente a ella propone la poética, la perspectiva del productor, la poiesis o techné. En la modernidad tardía, con la proliferación de medios visuales e Internet, la antigua dicotomía artista/espectador colapsa: hoy hay más gente interesada en producir imágenes que en mirarlas, y todos debemos diseñar una "persona pública", un doble artificial, en un ejercicio de autopoética por el que somos ética y políticamente responsables. Relee así la vanguardia (Malevich, Ball, Duchamp) como autopoiesis, producción del propio Yo público desde el grado cero de la forma, no como shock ni transgresión. Otros ensayos desarrollan: la obligación del diseño de sí y la producción de sinceridad; la política de la instalación como espacio donde el artista actúa cual legislador soberano y heterotópico, poniendo en cuestión la reducción foucaultiana del poder a mecanismos impersonales; una crítica al ensayo de Benjamin sobre el aura, sustituyendo la pérdida irreversible por un juego contemporáneo de desterritorializaciones y re-auratizaciones donde toda copia deviene nuevo original; el universalismo débil; Marx después de Duchamp; los trabajadores del arte entre utopía y archivo; y Google como máquina filosófica que resuelve la deconstrucción.</t>
         </is>
       </c>
     </row>
@@ -5324,27 +5324,27 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Heinich - Un nuevo paradigma. El arte contemporáneo como revolución artística.md</t>
+          <t>Harris - The Global Contemporary Art World. A Rough Guide (2017) [Wiley, ISBN 9781118288917].md</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Décadas de 1950 en adelante (arte contemporáneo); c. 1860-1950 (arte moderno)</t>
+          <t>Arte contemporáneo global posterior a 1989 (décadas de 1990-2016), con genealogía en la modernidad y el sistema colonial occidental</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro, 2014</t>
+          <t>Libro, 2017</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Nathalie Heinich; Thomas S. Kuhn; Thierry de Duve; Robert Rauschenberg; Yves Klein; Marcel Duchamp; Clement Greenberg; Harold Rosenberg; Krzysztof Pomian; Jean-Pierre Cometti; Julie Verlaine; Pierre Restany</t>
+          <t>Jonathan Harris; Bashir Makhoul; Nicholas Serota; Damien Hirst; Jeff Koons; Charles Saatchi; Hans Ulrich Obrist; Raymond Williams; Edward Said; David Harvey; Tate Modern / Art Basel; Wiley-Blackwell</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Heinich sostiene que el arte contemporáneo no es una etapa cronológica de la historia del arte, sino un nuevo paradigma artístico, incompatible con los paradigmas clásico y moderno que lo precedieron. Revisando su propuesta anterior de 1999 —que lo definía como un mero "género" para pacificar la polémica—, la autora la considera insuficiente y opta por transponer al arte el concepto kuhniano de paradigma tomado de La estructura de las revoluciones científicas. El objeto de estudio es la ruptura ontológica inaugurada por gestos como el dibujo borrado de De Kooning por Rauschenberg (1953), la Exposición del vacío de Klein (1958) o el premio de la Bienal de Venecia de 1964, que desplazan el arte desde la expresión de la interioridad (paradigma moderno) hacia un juego reflexivo con los límites mismos de lo que cuenta como obra. El marco conceptual articula sociología pragmática, análisis lexicométrico (los tres léxicos crítico-artísticos de Martin: clásico, moderno, contemporáneo) y la noción de "ciencia normal". Conceptos clave: paradigma, incompatibilidad entre paradigmas, conversión frente a demostración, transgresión ontológica, y la solidaridad entre dimensiones estéticas, jurídicas, económicas e institucionales que constituye "la fuerza del paradigma". Su tesis es que la disputa entre modernos y contemporáneos es irresoluble por argumentación, pues cada prueba solo vale dentro de su propio paradigma. El aporte central consiste en reencuadrar la controversia sobre el arte contemporáneo como una auténtica "revolución artística", descriptiva y no valorativa, cuyo alcance excede la naturaleza de las obras para abarcar todo el mundo del arte.</t>
+          <t>Cierre de la trilogía de Harris, el libro sostiene que el mundo del arte contemporáneo global no está separado del mundo, sino que constituye un subsistema —relativamente autónomo pero funcional— del "orden/desorden mundial" globalizado, conducido por alianzas cambiantes de estados y corporaciones bajo el capitalismo neoliberal surgido en los años ochenta (Reagan, Thatcher). El marco conceptual, deudor de Williams, Said y Harvey, insiste en el carácter fundamentalmente asimétrico del sistema: las instituciones "guardianas" occidentales (Sotheby's, Christie's, Art Basel, Frieze, Tate, MoMA, Guggenheim, galerías como Gagosian y White Cube) conservan el poder de validar y explotar económicamente un arte crecientemente producido fuera de Occidente. Harris amplía la noción de "productor" más allá del artista para incluir directores, curadores y coleccionistas (Serota, Saatchi, Obrist), y subraya la borrosa frontera entre lo público y lo privado. Metodológicamente rechaza el formato de "survey": el número reducido de obras analizadas tiene valor heurístico dentro de un análisis sistémico. El cuerpo del libro se organiza en cinco estudios de caso de la "gran Asia", todos de pasado poscolonial compartido: las ferias de Hong Kong (negocio offshore y desarrollo desigual y combinado), el nuevo media art y el globalismo cultural en Corea del Sur, la Bienal de Kochi como forma retórica en India, la reproducción social y el branding del "arte chino contemporáneo" en la educación superior de la RPC, y la "ONG-ización" del arte en el Estado de Palestina. Reflexiona además sobre las categorías "global", "contemporáneo", "arte" y "mundo", y sobre la modernidad como problema no resuelto de igualdad.</t>
         </is>
       </c>
     </row>
@@ -5356,27 +5356,27 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Holtaway - World-Forming and Contemporary Art (2021) [Routledge, ISBN 9780367628390].md</t>
+          <t>Heinich - Un nuevo paradigma. El arte contemporáneo como revolución artística.md</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>2010-2020 (prácticas artísticas y curatoriales analizadas)</t>
+          <t>Décadas de 1950 en adelante (arte contemporáneo); c. 1860-1950 (arte moderno)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Libro, 2021</t>
+          <t>Capítulo de libro, 2014</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Jessica Holtaway; Jean-Luc Nancy; Liberate Tate; Art Action UK; Arnolfini (Bristol); Georges Bataille; Hannah Arendt; Maurice Blanchot; Paolo Virno; Carl Schmitt; Jacques Rancière; Nicolas Bourriaud</t>
+          <t>Nathalie Heinich; Thomas S. Kuhn; Thierry de Duve; Robert Rauschenberg; Yves Klein; Marcel Duchamp; Clement Greenberg; Harold Rosenberg; Krzysztof Pomian; Jean-Pierre Cometti; Julie Verlaine; Pierre Restany</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Holtaway explora cómo el arte contemporáneo puede alterar los modos en que visualizamos y conceptualizamos el mundo y las relaciones sociales que lo configuran, frente a los aparatos del capitalismo global. Su tesis central, apoyada en la filosofía de Jean-Luc Nancy, es la de "recomponer" (recomposing) la imagen del mundo mediante la noción de "world-forming" (mondialisation frente a globalización). El libro traza una "inclinación" (incline) desde la ontología nanciana hacia lo político a través de tres conceptos —spacing (espaciamiento), exscribing (exscripción) y co-appearing (co-aparición)— y tres prácticas participativas estudiadas desde dentro: el colectivo activista Liberate Tate (contra el patrocinio petrolero de la Tate por BP), la práctica curatorial de Art Action UK (arte tras el desastre nuclear de Fukushima de 2011) y las prácticas institucionales y evaluativas del Arnolfini de Bristol (crítica a las Quality Metrics del Arts Council). El marco conceptual moviliza la ontología del "ser singular plural", la "comunidad inoperante", el "desobramiento" (unworking), la comunicación como "contagio" (Bataille) y el "espacio de aparición" de Arendt. Conceptos clave: separación compartida, exposición, intencionalidad no fenomenológica, retirada (retreat) y singularidad inaprehensible del arte. La autora defiende una investigación práctica y encarnada, que afirma la indivisibilidad de teoría y práctica, y sostiene que las intervenciones micropolíticas pueden desplazar los valores de las instituciones y suscitar cambio social. Su aporte es renovar la lectura de Nancy hacia lo institucional, mostrando cómo el arte sostiene una libertad crítica y una agencia abierta frente a la mercantilización neoliberal de la cultura.</t>
+          <t>Heinich sostiene que el arte contemporáneo no es una etapa cronológica de la historia del arte, sino un nuevo paradigma artístico, incompatible con los paradigmas clásico y moderno que lo precedieron. Revisando su propuesta anterior de 1999 —que lo definía como un mero "género" para pacificar la polémica—, la autora la considera insuficiente y opta por transponer al arte el concepto kuhniano de paradigma tomado de La estructura de las revoluciones científicas. El objeto de estudio es la ruptura ontológica inaugurada por gestos como el dibujo borrado de De Kooning por Rauschenberg (1953), la Exposición del vacío de Klein (1958) o el premio de la Bienal de Venecia de 1964, que desplazan el arte desde la expresión de la interioridad (paradigma moderno) hacia un juego reflexivo con los límites mismos de lo que cuenta como obra. El marco conceptual articula sociología pragmática, análisis lexicométrico (los tres léxicos crítico-artísticos de Martin: clásico, moderno, contemporáneo) y la noción de "ciencia normal". Conceptos clave: paradigma, incompatibilidad entre paradigmas, conversión frente a demostración, transgresión ontológica, y la solidaridad entre dimensiones estéticas, jurídicas, económicas e institucionales que constituye "la fuerza del paradigma". Su tesis es que la disputa entre modernos y contemporáneos es irresoluble por argumentación, pues cada prueba solo vale dentro de su propio paradigma. El aporte central consiste en reencuadrar la controversia sobre el arte contemporáneo como una auténtica "revolución artística", descriptiva y no valorativa, cuyo alcance excede la naturaleza de las obras para abarcar todo el mundo del arte.</t>
         </is>
       </c>
     </row>
@@ -5388,27 +5388,27 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Jelinek - This Is Not Art. Activism and Other «Not-Art» (2013) [I. B. Tauris, ISBN 9780755604920].md</t>
+          <t>Holtaway - World-Forming and Contemporary Art (2021) [Routledge, ISBN 9780367628390].md</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Escena artística de Londres, décadas de 1990-2010 (contexto neoliberal)</t>
+          <t>2010-2020 (prácticas artísticas y curatoriales analizadas)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Libro, 2013</t>
+          <t>Libro, 2021</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Alana Jelinek; PLATFORM; George Dickie; Arthur Danto; Michel Foucault; Hannah Arendt; Clement Greenberg; Allan Kaprow; David Harvey; Pierre Bourdieu; Gregory Sholette; Alfred Gell</t>
+          <t>Jessica Holtaway; Jean-Luc Nancy; Liberate Tate; Art Action UK; Arnolfini (Bristol); Georges Bataille; Hannah Arendt; Maurice Blanchot; Paolo Virno; Carl Schmitt; Jacques Rancière; Nicolas Bourriaud</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Jelinek, artista y teórica, escribe desde una perspectiva deliberadamente londinense para cuestionar los supuestos compartidos por el mundo del arte y el activismo sobre el arte "político" o "ético". Su tesis es que la mayor parte del arte contemporáneo que reclama radicalidad reproduce, en lugar de socavar, los valores y estructuras del neoliberalismo, fracasando a la vez como arte y como activismo. El libro, en seis capítulos, articula: (1) una descripción de cómo el mundo del arte —mercado, casas de subastas, bienales estatales— replica la privatización, liberalización comercial y desregulación neoliberales (con David Harvey, Gadrey, Callon, Velthuis); (2) la definición Institucional del arte (Dickie, Danto) de la tradición analítica angloamericana, que revela que la función del mundo del arte es definir y vigilar los límites del arte; (3) los modelos binarios marxistas del poder (Gramsci, Escuela de Frankfurt) frente a la concepción foucaultiana del poder como fluido y constitutivo; (4) la dicotomía Greenberg-Kaprow, "arte" versus "vida", estética versus ética, que propone colapsar. Conceptos clave: neoliberalismo, definición institucional, cliché de resistencia, disciplina, agencia y autonomía. Su aporte y posición: comprender la práctica artística como una disciplina formadora de conocimiento, con valores endógenos que permitan juzgar por sí misma qué es bueno, en lugar de ceder ese juicio al mercado o al Estado. Recurriendo a Arendt, Foucault y la antropología de Gell, defiende el poder singular del arte para narrar historias individuales, complejas y matizadas que subvierten la ortodoxia dominante y constituyen la esfera pública.</t>
+          <t>Holtaway explora cómo el arte contemporáneo puede alterar los modos en que visualizamos y conceptualizamos el mundo y las relaciones sociales que lo configuran, frente a los aparatos del capitalismo global. Su tesis central, apoyada en la filosofía de Jean-Luc Nancy, es la de "recomponer" (recomposing) la imagen del mundo mediante la noción de "world-forming" (mondialisation frente a globalización). El libro traza una "inclinación" (incline) desde la ontología nanciana hacia lo político a través de tres conceptos —spacing (espaciamiento), exscribing (exscripción) y co-appearing (co-aparición)— y tres prácticas participativas estudiadas desde dentro: el colectivo activista Liberate Tate (contra el patrocinio petrolero de la Tate por BP), la práctica curatorial de Art Action UK (arte tras el desastre nuclear de Fukushima de 2011) y las prácticas institucionales y evaluativas del Arnolfini de Bristol (crítica a las Quality Metrics del Arts Council). El marco conceptual moviliza la ontología del "ser singular plural", la "comunidad inoperante", el "desobramiento" (unworking), la comunicación como "contagio" (Bataille) y el "espacio de aparición" de Arendt. Conceptos clave: separación compartida, exposición, intencionalidad no fenomenológica, retirada (retreat) y singularidad inaprehensible del arte. La autora defiende una investigación práctica y encarnada, que afirma la indivisibilidad de teoría y práctica, y sostiene que las intervenciones micropolíticas pueden desplazar los valores de las instituciones y suscitar cambio social. Su aporte es renovar la lectura de Nancy hacia lo institucional, mostrando cómo el arte sostiene una libertad crítica y una agencia abierta frente a la mercantilización neoliberal de la cultura.</t>
         </is>
       </c>
     </row>
@@ -5420,27 +5420,27 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Keane - On Semiotic Ideology (2018) [Signs and Society].md</t>
+          <t>Jelinek - This Is Not Art. Activism and Other «Not-Art» (2013) [I. B. Tauris, ISBN 9780755604920].md</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>n/d (ejemplos históricos: Reforma protestante, Revolución bolchevique, Francia de mediados del s. XX)</t>
+          <t>Escena artística de Londres, décadas de 1990-2010 (contexto neoliberal)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico, 2018</t>
+          <t>Libro, 2013</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Webb Keane; Michael Silverstein; Charles Sanders Peirce; Richard Parmentier; Gregory Bateson; Pierre Bourdieu; Benedict Anderson; Christopher Ball; Susan Gal; Harvey Sacks; E. E. Evans-Pritchard</t>
+          <t>Alana Jelinek; PLATFORM; George Dickie; Arthur Danto; Michel Foucault; Hannah Arendt; Clement Greenberg; Allan Kaprow; David Harvey; Pierre Bourdieu; Gregory Sholette; Alfred Gell</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Keane revisa y sistematiza el concepto de "ideología semiótica", entendido como los supuestos subyacentes de las personas sobre qué son los signos, qué funciones cumplen y qué consecuencias producen. Su tesis central es que la ideología semiótica no es una falsa conciencia ni algo que unos poseen y otros no, sino una manifestación de la reflexividad inherente a la capacidad humana general de usar signos; varía histórica y socialmente y vincula los procesos semióticos generales con juicios éticos y políticos particulares. El objeto es articular la semiótica peirceana (las tres tricotomías: cualisigno/sinsigno/legisigno; icono/índice/símbolo; rema/dicente/argumento) con el análisis etnográfico y social. El marco conceptual retoma a Silverstein (ideología lingüística), Peirce, Bateson (mapa y territorio, negación de la mediación) y la "economía representacional". Conceptos clave: reflexividad, abducción, ground (fundamento del signo), affordances, rematización y dicentización (procesos de naturalización), y la ontología en disputa de los objetos del signo. Dos ejemplos vertebran el argumento: el análisis de la clase social en Bourdieu (el habitus como ícono indexical, donde analista y lego difieren sobre el objeto del signo corporal) y los choques religiosos —la campaña bolchevique de exhumación de reliquias, la Reforma— donde la propia existencia del objeto del signo está en disputa. Su aporte es mostrar que no hay ground determinado a priori de un signo: tomar un signo de cierta manera es tomar en serio el mundo que presupone y la vida que ese mundo recomienda, dotando a la existencia social de su carácter constructivo, incierto y conflictivo.</t>
+          <t>Jelinek, artista y teórica, escribe desde una perspectiva deliberadamente londinense para cuestionar los supuestos compartidos por el mundo del arte y el activismo sobre el arte "político" o "ético". Su tesis es que la mayor parte del arte contemporáneo que reclama radicalidad reproduce, en lugar de socavar, los valores y estructuras del neoliberalismo, fracasando a la vez como arte y como activismo. El libro, en seis capítulos, articula: (1) una descripción de cómo el mundo del arte —mercado, casas de subastas, bienales estatales— replica la privatización, liberalización comercial y desregulación neoliberales (con David Harvey, Gadrey, Callon, Velthuis); (2) la definición Institucional del arte (Dickie, Danto) de la tradición analítica angloamericana, que revela que la función del mundo del arte es definir y vigilar los límites del arte; (3) los modelos binarios marxistas del poder (Gramsci, Escuela de Frankfurt) frente a la concepción foucaultiana del poder como fluido y constitutivo; (4) la dicotomía Greenberg-Kaprow, "arte" versus "vida", estética versus ética, que propone colapsar. Conceptos clave: neoliberalismo, definición institucional, cliché de resistencia, disciplina, agencia y autonomía. Su aporte y posición: comprender la práctica artística como una disciplina formadora de conocimiento, con valores endógenos que permitan juzgar por sí misma qué es bueno, en lugar de ceder ese juicio al mercado o al Estado. Recurriendo a Arendt, Foucault y la antropología de Gell, defiende el poder singular del arte para narrar historias individuales, complejas y matizadas que subvierten la ortodoxia dominante y constituyen la esfera pública.</t>
         </is>
       </c>
     </row>
@@ -5452,27 +5452,27 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Keane - Perspectives on Affordances, or the Anthropologically Real. The 2018 Daryll Forde Lecture.md</t>
+          <t>Keane - On Semiotic Ideology (2018) [Signs and Society].md</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>n/d (casos: feminismo estadounidense de la segunda ola, fines de 1960; etnografía melanesia contemporánea)</t>
+          <t>n/d (ejemplos históricos: Reforma protestante, Revolución bolchevique, Francia de mediados del s. XX)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Conferencia académica (Daryll Forde Lecture) publicada en HAU, 2018</t>
+          <t>Artículo académico, 2018</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Webb Keane; James J. Gibson; Daryll Forde; Franz Boas; Alfred Kroeber; Bruno Latour; George Herbert Mead; Rupert Stasch; Joel Robbins; Bambi Schieffelin; University College London; HAU: Journal of Ethnographic Theory</t>
+          <t>Webb Keane; Michael Silverstein; Charles Sanders Peirce; Richard Parmentier; Gregory Bateson; Pierre Bourdieu; Benedict Anderson; Christopher Ball; Susan Gal; Harvey Sacks; E. E. Evans-Pritchard</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>En esta conferencia Keane propone la "perspectiva de las affordances" (disposiciones o posibilidades de acción) como alternativa tanto al determinismo reductivo como a las versiones fuertes del constructivismo social, articulando un "realismo antropológico". Partiendo de la antropología de cuatro campos de Daryll Forde y de la distinción de Boas entre el conocimiento idiográfico del geógrafo y el nomotético del físico, plantea la pregunta por qué hace que algo sea una "cuestión de interés" (matter of concern, Latour) y para qué "nosotros". Su tesis: las personas descubren continuamente cosas sobre sí mismas y sus mundos que no pusieron allí, porque las affordances (Gibson, Mead) son propiedades objetivas y reales que solo existen como tales en combinaciones contingentes y relativas a las actividades y proyectos de un agente. Conceptos clave: potencialidad frente a determinación, proyecto, reflexividad, el "nosotros" emergente, y la coexistencia de significado y causalidad. Dos ejemplos desarrollan el argumento: la toma de conciencia (consciousness-raising) del feminismo estadounidense de fines de los 1960, donde la ira personal se reconfigura como crítica política y emerge un nuevo "nosotras" (apoyado en el experimento de Schachter y Singer sobre la epinefrina); y la "doctrina de la opacidad" de las mentes en Melanesia (Stasch, Robbins, Schieffelin), donde negar una affordance —el acceso a las intenciones ajenas— es en sí una respuesta ética y política que valora la autonomía. El aporte es una antropología realista pero no reductivista: el mundo excede nuestras conceptualizaciones, y los autodescubrimientos redefinen las fronteras de quiénes somos "nosotros".</t>
+          <t>Keane revisa y sistematiza el concepto de "ideología semiótica", entendido como los supuestos subyacentes de las personas sobre qué son los signos, qué funciones cumplen y qué consecuencias producen. Su tesis central es que la ideología semiótica no es una falsa conciencia ni algo que unos poseen y otros no, sino una manifestación de la reflexividad inherente a la capacidad humana general de usar signos; varía histórica y socialmente y vincula los procesos semióticos generales con juicios éticos y políticos particulares. El objeto es articular la semiótica peirceana (las tres tricotomías: cualisigno/sinsigno/legisigno; icono/índice/símbolo; rema/dicente/argumento) con el análisis etnográfico y social. El marco conceptual retoma a Silverstein (ideología lingüística), Peirce, Bateson (mapa y territorio, negación de la mediación) y la "economía representacional". Conceptos clave: reflexividad, abducción, ground (fundamento del signo), affordances, rematización y dicentización (procesos de naturalización), y la ontología en disputa de los objetos del signo. Dos ejemplos vertebran el argumento: el análisis de la clase social en Bourdieu (el habitus como ícono indexical, donde analista y lego difieren sobre el objeto del signo corporal) y los choques religiosos —la campaña bolchevique de exhumación de reliquias, la Reforma— donde la propia existencia del objeto del signo está en disputa. Su aporte es mostrar que no hay ground determinado a priori de un signo: tomar un signo de cierta manera es tomar en serio el mundo que presupone y la vida que ese mundo recomienda, dotando a la existencia social de su carácter constructivo, incierto y conflictivo.</t>
         </is>
       </c>
     </row>
@@ -5484,27 +5484,27 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Keane - Semiotics and the Social Analysis of Material Things (2003) [Language &amp; Communication 23, pp. 409-425].md</t>
+          <t>Keane - Perspectives on Affordances, or the Anthropologically Real. The 2018 Daryll Forde Lecture.md</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>n/d (trabajo de campo en Sumba, Indonesia; teoría social)</t>
+          <t>n/d (casos: feminismo estadounidense de la segunda ola, fines de 1960; etnografía melanesia contemporánea)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico, 2003</t>
+          <t>Conferencia académica (Daryll Forde Lecture) publicada en HAU, 2018</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Webb Keane; Charles Sanders Peirce; Ferdinand de Saussure; Jacques Derrida; Nancy Munn; Pierre Bourdieu; Alfred Gell; Michael Silverstein; Martin Heidegger; Karl Marx; Judith Irvine; Roman Jakobson</t>
+          <t>Webb Keane; James J. Gibson; Daryll Forde; Franz Boas; Alfred Kroeber; Bruno Latour; George Herbert Mead; Rupert Stasch; Joel Robbins; Bambi Schieffelin; University College London; HAU: Journal of Ethnographic Theory</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Keane examina cómo la semiótica peirceana puede contribuir al análisis social de los artefactos materiales, superando la persistente dicotomía entre "espíritu" y "materia", ideas y cosas, que él rastrea en el linaje que va de Saussure al posestructuralismo. Su tesis es que el modelo triádico de Peirce —al incluir el objeto de la significación— permite reintroducir la materialidad, la causalidad y la contingencia (el "choque exterior" que Peirce reprochaba a Hegel) sin caer en reduccionismos materialistas ni en el idealismo. El objeto de estudio son la iconicidad y la indexicalidad y su papel al mediar contingencia, causalidad y acciones posibles. Como "iconos e índices en sí mismos no afirman nada", sus funciones sociales dependen de su mediación por la "Terceridad" (orientación al futuro, ley general), lo que exige una teoría de las ideologías semióticas y su encarnación en "economías representacionales". Conceptos clave: cualisigno, bundling (empaquetamiento de cualidades), biografía de las cosas, naturalización (conversión de indexicalidad en iconismo), objetualización y semiotización. Recurre a Munn (valor y "levedad" en Gawa), Bourdieu (el connaisseur y el habitus), Marx y Heidegger (trabajo no alienado, útiles), y a su propio trabajo de campo en Sumba, donde signos que él tomaba por "naturales" eran interpretados como "no naturales", registro de intenciones de agentes. El aporte es doble: mostrar la historicidad implícita en la semiótica y reclamar un concepto más rico de las múltiples modalidades de objetualización en la vida social, contra las romantizaciones que la identifican solo con el capitalismo, la ciencia o el protestantismo.</t>
+          <t>En esta conferencia Keane propone la "perspectiva de las affordances" (disposiciones o posibilidades de acción) como alternativa tanto al determinismo reductivo como a las versiones fuertes del constructivismo social, articulando un "realismo antropológico". Partiendo de la antropología de cuatro campos de Daryll Forde y de la distinción de Boas entre el conocimiento idiográfico del geógrafo y el nomotético del físico, plantea la pregunta por qué hace que algo sea una "cuestión de interés" (matter of concern, Latour) y para qué "nosotros". Su tesis: las personas descubren continuamente cosas sobre sí mismas y sus mundos que no pusieron allí, porque las affordances (Gibson, Mead) son propiedades objetivas y reales que solo existen como tales en combinaciones contingentes y relativas a las actividades y proyectos de un agente. Conceptos clave: potencialidad frente a determinación, proyecto, reflexividad, el "nosotros" emergente, y la coexistencia de significado y causalidad. Dos ejemplos desarrollan el argumento: la toma de conciencia (consciousness-raising) del feminismo estadounidense de fines de los 1960, donde la ira personal se reconfigura como crítica política y emerge un nuevo "nosotras" (apoyado en el experimento de Schachter y Singer sobre la epinefrina); y la "doctrina de la opacidad" de las mentes en Melanesia (Stasch, Robbins, Schieffelin), donde negar una affordance —el acceso a las intenciones ajenas— es en sí una respuesta ética y política que valora la autonomía. El aporte es una antropología realista pero no reductivista: el mundo excede nuestras conceptualizaciones, y los autodescubrimientos redefinen las fronteras de quiénes somos "nosotros".</t>
         </is>
       </c>
     </row>
@@ -5516,27 +5516,27 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Knox y Gambino - Infrastructure [entrada de enciclopedia, fuente sin confirmar].md</t>
+          <t>Keane - Semiotics and the Social Analysis of Material Things (2003) [Language &amp; Communication 23, pp. 409-425].md</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>n/d (revisión teórica; casos desde el siglo XIX hasta la actualidad, incluyendo crisis del COVID-19 y la guerra en Ucrania)</t>
+          <t>n/d (trabajo de campo en Sumba, Indonesia; teoría social)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Entrada de enciclopedia (antropología), c. 2023 (fecha sin confirmar)</t>
+          <t>Artículo académico, 2003</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Hannah Knox (University College London); Evelina Gambino (University of Cambridge); Brian Larkin; Bruno Latour; Susan Leigh Star; AbdouMaliq Simone; Ashley Carse; Stephen Collier; Nikhil Anand, Akhil Gupta y Hannah Appel; Penny Harvey; Anna Tsing; Duke University Press</t>
+          <t>Webb Keane; Charles Sanders Peirce; Ferdinand de Saussure; Jacques Derrida; Nancy Munn; Pierre Bourdieu; Alfred Gell; Michael Silverstein; Martin Heidegger; Karl Marx; Judith Irvine; Roman Jakobson</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Esta entrada enciclopédica ofrece una cartografía del campo emergente de la antropología de la infraestructura, argumentando que atender a las infraestructuras —carreteras, cables, tuberías, redes de datos, contratos— permite a la etnografía extender su análisis a través de múltiples escalas y estudiar sistemas de gran envergadura (Estado, capitalismo, colonialismo) sin abandonar la observación situada. Las autoras subrayan la ontología dual de la infraestructura, que es a la vez cosa material y relación entre cosas (Larkin: «matter that moves matter»), y su naturaleza relacional: siguiendo a Star y Ruhleder, no cabe preguntar «qué» es una infraestructura sino «cuándo» algo deviene infraestructural. El texto sintetiza marcos teóricos convergentes: teoría del actor-red, estudios de ciencia y tecnología, los «nuevos materialismos» y la STS feminista (Haraway, Barad, Stengers). Organiza la literatura en cuatro ejes. Primero, infraestructura y Estado: las obras públicas materializan y a la vez descosen la soberanía, y encarnan lógicas coloniales y de securitización (Collier, Von Schnitzler, Appel, Vaughn). Segundo, espacio/tiempo: las infraestructuras «trabajan sobre el tiempo», producen sublimidad tecnológica, promesa de futuro y compresión espacio-temporal, aunque la etnografía revela la lentitud y fricción reales del acelerar (Starosielski). Tercero, medio ambiente: bosques, suelo o agua se vuelven infraestructurales, vinculando la disciplina al Antropoceno (Carse, Tsing, Hetherington). Cuarto, infraestructuras contrapolíticas: prácticas bottom-up, de código abierto y de cuidado que reconfiguran la comprensión antropológica de la política (Simone). La conclusión recoge las críticas a la sobreextensión del concepto y aboga por detectar cuándo la cualidad infraestructural de las cosas empieza a importar.</t>
+          <t>Keane examina cómo la semiótica peirceana puede contribuir al análisis social de los artefactos materiales, superando la persistente dicotomía entre "espíritu" y "materia", ideas y cosas, que él rastrea en el linaje que va de Saussure al posestructuralismo. Su tesis es que el modelo triádico de Peirce —al incluir el objeto de la significación— permite reintroducir la materialidad, la causalidad y la contingencia (el "choque exterior" que Peirce reprochaba a Hegel) sin caer en reduccionismos materialistas ni en el idealismo. El objeto de estudio son la iconicidad y la indexicalidad y su papel al mediar contingencia, causalidad y acciones posibles. Como "iconos e índices en sí mismos no afirman nada", sus funciones sociales dependen de su mediación por la "Terceridad" (orientación al futuro, ley general), lo que exige una teoría de las ideologías semióticas y su encarnación en "economías representacionales". Conceptos clave: cualisigno, bundling (empaquetamiento de cualidades), biografía de las cosas, naturalización (conversión de indexicalidad en iconismo), objetualización y semiotización. Recurre a Munn (valor y "levedad" en Gawa), Bourdieu (el connaisseur y el habitus), Marx y Heidegger (trabajo no alienado, útiles), y a su propio trabajo de campo en Sumba, donde signos que él tomaba por "naturales" eran interpretados como "no naturales", registro de intenciones de agentes. El aporte es doble: mostrar la historicidad implícita en la semiótica y reclamar un concepto más rico de las múltiples modalidades de objetualización en la vida social, contra las romantizaciones que la identifican solo con el capitalismo, la ciencia o el protestantismo.</t>
         </is>
       </c>
     </row>
@@ -5548,27 +5548,27 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Kosmala e Imas (eds.) - Precarious Spaces. The Arts, Social and Organizational Change [ISBN 9781783205936].md</t>
+          <t>Knox y Gambino - Infrastructure [entrada de enciclopedia, fuente sin confirmar].md</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Contemporáneo (décadas de 2000 y 2010, con referencia al modernismo latinoamericano de los años 1920-1930)</t>
+          <t>n/d (revisión teórica; casos desde el siglo XIX hasta la actualidad, incluyendo crisis del COVID-19 y la guerra en Ucrania)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Libro editado (colección académica), 2016 (Intellect, Bristol/Chicago)</t>
+          <t>Entrada de enciclopedia (antropología), c. 2023 (fecha sin confirmar)</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Katarzyna Kosmala y Miguel Imas (editores); Maria Ceci Misoczky (prefacio); Diana Brydon; Judith Butler; Zygmunt Bauman; Gregory Sholette; Claire Bishop; Grant Kester; Nicolas Bourriaud; Gonzalo Olmos y Valeria Biffi (capítulo sobre Lima); Intellect</t>
+          <t>Hannah Knox (University College London); Evelina Gambino (University of Cambridge); Brian Larkin; Bruno Latour; Susan Leigh Star; AbdouMaliq Simone; Ashley Carse; Stephen Collier; Nikhil Anand, Akhil Gupta y Hannah Appel; Penny Harvey; Anna Tsing; Duke University Press</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Volumen colectivo interdisciplinario que examina la relación entre prácticas artísticas de base, precariedad y cambio social y organizacional en espacios periféricos, priorizando experiencias del Sur Global (Brasil, México, Perú, Argentina, Chile) para luego proyectarlas hacia el Norte. La introducción de Kosmala e Imas distingue, siguiendo a Butler, la precariedad como condición compartida de toda vida frente a la precarity políticamente inducida por el neoliberalismo, y moviliza a Bauman (modernidad líquida), Wacquant, Standing y Sholette (el «dark matter» de artistas fracasados que sostiene el mundo del arte) para conceptualizar el precariado como clase en formación. El marco estético central es la estética dialógica y relacional (Kester, Bourriaud, Bishop), donde el objeto artístico cede protagonismo al proceso participativo y a la especificidad de sitio (Kwon) como espacio de encuentro y coproducción, aunque los editores advierten sobre la cooptación neoliberal de la agencia política del arte. El capítulo teórico de Brydon articula autonomía relacional y planetariedad como categorías para reencuadrar el debate desde una ecología de saberes descolonial (Santos, Mignolo, Spivak). Las secciones «Emancipating» y «Resisting» reúnen estudios de caso: el Complexo da Maré y la Favela Painting en Río, la Autoconstrucción de Abraham Cruzvillegas en Ciudad de México, el FOLi Lab de la Bienal de Fotografía de Lima, campamentos Mbyá-Guaraní, fábricas recuperadas, activismo mediático (Mídia Ninja) y organización cultural en favelas. El aporte del libro es tender puentes entre teoría del arte, estudios organizacionales y urbanismo desde el Sur, evitando privilegiar los marcos filosóficos del Norte y proponiendo la indagación basada en las artes como método y como intervención transformadora hacia vidas más «vivibles».</t>
+          <t>Esta entrada enciclopédica ofrece una cartografía del campo emergente de la antropología de la infraestructura, argumentando que atender a las infraestructuras —carreteras, cables, tuberías, redes de datos, contratos— permite a la etnografía extender su análisis a través de múltiples escalas y estudiar sistemas de gran envergadura (Estado, capitalismo, colonialismo) sin abandonar la observación situada. Las autoras subrayan la ontología dual de la infraestructura, que es a la vez cosa material y relación entre cosas (Larkin: «matter that moves matter»), y su naturaleza relacional: siguiendo a Star y Ruhleder, no cabe preguntar «qué» es una infraestructura sino «cuándo» algo deviene infraestructural. El texto sintetiza marcos teóricos convergentes: teoría del actor-red, estudios de ciencia y tecnología, los «nuevos materialismos» y la STS feminista (Haraway, Barad, Stengers). Organiza la literatura en cuatro ejes. Primero, infraestructura y Estado: las obras públicas materializan y a la vez descosen la soberanía, y encarnan lógicas coloniales y de securitización (Collier, Von Schnitzler, Appel, Vaughn). Segundo, espacio/tiempo: las infraestructuras «trabajan sobre el tiempo», producen sublimidad tecnológica, promesa de futuro y compresión espacio-temporal, aunque la etnografía revela la lentitud y fricción reales del acelerar (Starosielski). Tercero, medio ambiente: bosques, suelo o agua se vuelven infraestructurales, vinculando la disciplina al Antropoceno (Carse, Tsing, Hetherington). Cuarto, infraestructuras contrapolíticas: prácticas bottom-up, de código abierto y de cuidado que reconfiguran la comprensión antropológica de la política (Simone). La conclusión recoge las críticas a la sobreextensión del concepto y aboga por detectar cuándo la cualidad infraestructural de las cosas empieza a importar.</t>
         </is>
       </c>
     </row>
@@ -5580,27 +5580,27 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Kuoni (ed.) - Words of Wisdom. A Curator's Vade Mecum on Contemporary Art [Nueva York, ISBN 9780916365608].md</t>
+          <t>Kosmala e Imas (eds.) - Precarious Spaces. The Arts, Social and Organizational Change [ISBN 9781783205936].md</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>1975-2001 (veinticinco años de práctica curatorial y expositiva)</t>
+          <t>Contemporáneo (décadas de 2000 y 2010, con referencia al modernismo latinoamericano de los años 1920-1930)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Libro (antología de ensayos curatoriales), 2001 (Independent Curators International, Nueva York)</t>
+          <t>Libro editado (colección académica), 2016 (Intellect, Bristol/Chicago)</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Carin Kuoni (editora); Judith Olch Richards (ICI); Jean-Christophe Ammann; Harald Szeemann; Hans-Ulrich Obrist; Thelma Golden; Hou Hanru; Mari Carmen Ramírez; Gerardo Mosquera; Lucy Lippard; Mary Jane Jacob; Robert Storr; Jean-Hubert Martin; Seth Siegelaub; Independent Curators International (ICI)</t>
+          <t>Katarzyna Kosmala y Miguel Imas (editores); Maria Ceci Misoczky (prefacio); Diana Brydon; Judith Butler; Zygmunt Bauman; Gregory Sholette; Claire Bishop; Grant Kester; Nicolas Bourriaud; Gonzalo Olmos y Valeria Biffi (capítulo sobre Lima); Intellect</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Antología publicada por Independent Curators International (ICI) con motivo de su 25º aniversario, que reúne alrededor de sesenta ensayos breves de curadores internacionales de contemporáneo, concebida como un vade mecum —manual portátil de oficio, en analogía con los manuales gremiales medievales— dirigido especialmente a curadores jóvenes. Kuoni plantea en la introducción una paradoja fundacional: el libro «no debería existir», pues de los textos se desprende que en el trabajo curatorial no hay reglas y que toda exposición solo aborda las cuestiones del momento particular en que se creó, de modo que codificar estrategias contradice ese talante ahistórico. A los colaboradores se les propuso responder a un cuestionario sobre audiencia, financiamiento, marco institucional, responsabilidad y rendición de cuentas, y el correo electrónico sirvió como vehículo informal de ideas jotadas rápidamente. El volumen contextualiza la historia expositiva reciente: los intercambios transatlánticos de los años setenta y ochenta (Martin: Paris-New York, Paris-Moscou), los primeros ensayos multiculturales (Les Magiciens de la Terre, The Decade Show), las «culture wars» estadounidenses, la exposición site-specific (Jacob: Places with a Past) y el arte de nuevos medios y web. Las contribuciones oscilan entre visiones del curador como agitador cultural, «comadrona», antropólogo visual o corrector del canon dominado por el mercado, y enfatizan recurrentemente el privilegio de trabajar con los artistas vivos. Los curadores más jóvenes reclaman inversión a largo plazo y exposiciones entendidas como constructos volátiles y discursivos. El ejemplo de Ammann ofrece veintiséis máximas (confiar en el arte y no en los discursos, entrenar la intuición, evadir el zeitgeist). El aporte del libro reside en registrar, sin jerarquizar, la pluralidad contradictoria del oficio curatorial contemporáneo.</t>
+          <t>Volumen colectivo interdisciplinario que examina la relación entre prácticas artísticas de base, precariedad y cambio social y organizacional en espacios periféricos, priorizando experiencias del Sur Global (Brasil, México, Perú, Argentina, Chile) para luego proyectarlas hacia el Norte. La introducción de Kosmala e Imas distingue, siguiendo a Butler, la precariedad como condición compartida de toda vida frente a la precarity políticamente inducida por el neoliberalismo, y moviliza a Bauman (modernidad líquida), Wacquant, Standing y Sholette (el «dark matter» de artistas fracasados que sostiene el mundo del arte) para conceptualizar el precariado como clase en formación. El marco estético central es la estética dialógica y relacional (Kester, Bourriaud, Bishop), donde el objeto artístico cede protagonismo al proceso participativo y a la especificidad de sitio (Kwon) como espacio de encuentro y coproducción, aunque los editores advierten sobre la cooptación neoliberal de la agencia política del arte. El capítulo teórico de Brydon articula autonomía relacional y planetariedad como categorías para reencuadrar el debate desde una ecología de saberes descolonial (Santos, Mignolo, Spivak). Las secciones «Emancipating» y «Resisting» reúnen estudios de caso: el Complexo da Maré y la Favela Painting en Río, la Autoconstrucción de Abraham Cruzvillegas en Ciudad de México, el FOLi Lab de la Bienal de Fotografía de Lima, campamentos Mbyá-Guaraní, fábricas recuperadas, activismo mediático (Mídia Ninja) y organización cultural en favelas. El aporte del libro es tender puentes entre teoría del arte, estudios organizacionales y urbanismo desde el Sur, evitando privilegiar los marcos filosóficos del Norte y proponiendo la indagación basada en las artes como método y como intervención transformadora hacia vidas más «vivibles».</t>
         </is>
       </c>
     </row>
@@ -5612,27 +5612,27 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Larkin - The Politics and Poetics of Infrastructure (2013) [Annual Review of Anthropology 42, pp. 327-343].md</t>
+          <t>Kuoni (ed.) - Words of Wisdom. A Curator's Vade Mecum on Contemporary Art [Nueva York, ISBN 9780916365608].md</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>n/d (reseña teórica; ejemplos del siglo XIX a la contemporaneidad)</t>
+          <t>1975-2001 (veinticinco años de práctica curatorial y expositiva)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico (reseña), 2013 (Annual Review of Anthropology 42, pp. 327-343)</t>
+          <t>Libro (antología de ensayos curatoriales), 2001 (Independent Curators International, Nueva York)</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Brian Larkin (Barnard College, Columbia University); Susan Leigh Star; Thomas Hughes; Bruno Latour; Roman Jakobson; Michel Foucault; Achille Mbembe; Nikhil Anand; Antina von Schnitzler; Stephen Collier; Rudolf Mrázek; Walter Benjamin; Annual Review of Anthropology</t>
+          <t>Carin Kuoni (editora); Judith Olch Richards (ICI); Jean-Christophe Ammann; Harald Szeemann; Hans-Ulrich Obrist; Thelma Golden; Hou Hanru; Mari Carmen Ramírez; Gerardo Mosquera; Lucy Lippard; Mary Jane Jacob; Robert Storr; Jean-Hubert Martin; Seth Siegelaub; Independent Curators International (ICI)</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Artículo de reseña que se ha vuelto seminal para la antropología de la infraestructura. Larkin define las infraestructuras como formas materiales que posibilitan el intercambio sobre el espacio: redes construidas que canalizan bienes, personas, ideas, desechos y capital, y cuya ontología es dual, pues son a la vez cosas y la relación entre cosas. Sostiene que definir una infraestructura es siempre un acto categorial y epistemológico, ya que las redes son recursivas y dispersas (el ejemplo del computador y la electricidad). El texto traza tres grandes aproximaciones. Primero, el pensamiento sistémico y la tecnopolítica: apoyándose en Hughes, la STS y la teoría del actor-red, y en el liberalismo foucaultiano como gobierno que se autodisimula, revisa etnografías del agua (Anand en Mumbai, «ciudadanía hidráulica»; Von Schnitzler y el medidor como productor de un «sujeto calculador» en Soweto) y la biopolítica de la electricidad soviética (Collier). Segundo, y su aporte más original, la «poética» de la infraestructura: retomando la función poética de Jakobson, argumenta que la forma se desliga de la función técnica y que las infraestructuras operan sobre el deseo, la fantasía y el sublime tecnológico, generando la promesa de modernidad y sus abyecciones (Mrázek, Mbembe, el «desdoblamiento» donde la tubería deviene documento). Tercero, la estética como aisthesis: recuperando a Buck-Morss, describe cómo los materiales (hierro, concreto, luz) producen experiencias sensoriales y ambientales de la modernidad. Larkin refuta la tesis de la invisibilidad de la infraestructura (Star), mostrando su hipervisibilidad, y concluye que la elección metodológica sobre qué es infraestructura es una cuestión teórica de primer orden.</t>
+          <t>Antología publicada por Independent Curators International (ICI) con motivo de su 25º aniversario, que reúne alrededor de sesenta ensayos breves de curadores internacionales de contemporáneo, concebida como un vade mecum —manual portátil de oficio, en analogía con los manuales gremiales medievales— dirigido especialmente a curadores jóvenes. Kuoni plantea en la introducción una paradoja fundacional: el libro «no debería existir», pues de los textos se desprende que en el trabajo curatorial no hay reglas y que toda exposición solo aborda las cuestiones del momento particular en que se creó, de modo que codificar estrategias contradice ese talante ahistórico. A los colaboradores se les propuso responder a un cuestionario sobre audiencia, financiamiento, marco institucional, responsabilidad y rendición de cuentas, y el correo electrónico sirvió como vehículo informal de ideas jotadas rápidamente. El volumen contextualiza la historia expositiva reciente: los intercambios transatlánticos de los años setenta y ochenta (Martin: Paris-New York, Paris-Moscou), los primeros ensayos multiculturales (Les Magiciens de la Terre, The Decade Show), las «culture wars» estadounidenses, la exposición site-specific (Jacob: Places with a Past) y el arte de nuevos medios y web. Las contribuciones oscilan entre visiones del curador como agitador cultural, «comadrona», antropólogo visual o corrector del canon dominado por el mercado, y enfatizan recurrentemente el privilegio de trabajar con los artistas vivos. Los curadores más jóvenes reclaman inversión a largo plazo y exposiciones entendidas como constructos volátiles y discursivos. El ejemplo de Ammann ofrece veintiséis máximas (confiar en el arte y no en los discursos, entrenar la intuición, evadir el zeitgeist). El aporte del libro reside en registrar, sin jerarquizar, la pluralidad contradictoria del oficio curatorial contemporáneo.</t>
         </is>
       </c>
     </row>
@@ -5644,27 +5644,27 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Leone, Keane y Nakassis - Semiotic Ideology. A Dialogue across Semiotic Traditions.md</t>
+          <t>Larkin - The Politics and Poetics of Infrastructure (2013) [Annual Review of Anthropology 42, pp. 327-343].md</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>n/d (diálogo teórico; recorrido histórico del concepto de ideología desde fines del siglo XVIII hasta el presente)</t>
+          <t>n/d (reseña teórica; ejemplos del siglo XIX a la contemporaneidad)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Diálogo académico (transcripción editada de una sesión del 23 de junio de 2025), publicado en 2025</t>
+          <t>Artículo académico (reseña), 2013 (Annual Review of Anthropology 42, pp. 327-343)</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Massimo Leone (Università di Torino); Webb Keane (University of Michigan); Constantine V. Nakassis (University of Chicago); Simona Stano; Michael Silverstein; Umberto Eco; Charles S. Peirce; Karl Marx; Destutt de Tracy; Fondazione Bruno Kessler (Trento); Lexia</t>
+          <t>Brian Larkin (Barnard College, Columbia University); Susan Leigh Star; Thomas Hughes; Bruno Latour; Roman Jakobson; Michel Foucault; Achille Mbembe; Nikhil Anand; Antina von Schnitzler; Stephen Collier; Rudolf Mrázek; Walter Benjamin; Annual Review of Anthropology</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Transcripción editada de un diálogo entre el semiótico continental Massimo Leone y el antropólogo lingüístico Webb Keane, moderado y prologado por Constantine Nakassis, que explora convergencias y divergencias entre la semiótica continental (Saussure, Greimas, Lotman, Eco) y la antropología lingüística norteamericana peirceana en torno a la noción de «ideología semiótica». Nakassis reconstruye la genealogía del término ideología: de la «ciencia de las ideas» materialista y antimetafísica de Destutt de Tracy, pasando por la resignificación peyorativa que impuso Napoleón vía enregisterment, hasta la doble crítica marxiana en La ideología alemana. Argumenta que la ideología no es falsa conciencia ni epifenómeno, sino mediación performativa constitutiva de lo social —ejemplificada en el fetichismo de la mercancía—, y que su espacio problemático coincide con el de la semiótica misma. Keane sostiene, desde el pragmatismo peirceano, que la semiosis importa menos por lo que nombra que por lo que trae al ser; introduce su concepto de «economía representacional» (transformaciones causales no significantes que reconfiguran las affordances del sentido, como la fotografía respecto de la pintura) y sitúa la abducción no como método hermenéutico del analista sino como el proceso cotidiano, falible y dialógico por el que la gente da sentido a los signos (rhema, dicent, argumento como modos de ideología semiótica). Ambos aceptan que el análisis es él mismo situado e ideológico, rechazando el objetivismo. Leone describe la ideología semiótica como espacio de tensión entre el yo-tú dialógico y la enunciación en tercera persona (el «it»), y como trampolín de autorreflexividad existencial. El debate aborda además la disolución del concepto de cultura y la unidad social de la ideología, implícita en las prácticas.</t>
+          <t>Artículo de reseña que se ha vuelto seminal para la antropología de la infraestructura. Larkin define las infraestructuras como formas materiales que posibilitan el intercambio sobre el espacio: redes construidas que canalizan bienes, personas, ideas, desechos y capital, y cuya ontología es dual, pues son a la vez cosas y la relación entre cosas. Sostiene que definir una infraestructura es siempre un acto categorial y epistemológico, ya que las redes son recursivas y dispersas (el ejemplo del computador y la electricidad). El texto traza tres grandes aproximaciones. Primero, el pensamiento sistémico y la tecnopolítica: apoyándose en Hughes, la STS y la teoría del actor-red, y en el liberalismo foucaultiano como gobierno que se autodisimula, revisa etnografías del agua (Anand en Mumbai, «ciudadanía hidráulica»; Von Schnitzler y el medidor como productor de un «sujeto calculador» en Soweto) y la biopolítica de la electricidad soviética (Collier). Segundo, y su aporte más original, la «poética» de la infraestructura: retomando la función poética de Jakobson, argumenta que la forma se desliga de la función técnica y que las infraestructuras operan sobre el deseo, la fantasía y el sublime tecnológico, generando la promesa de modernidad y sus abyecciones (Mrázek, Mbembe, el «desdoblamiento» donde la tubería deviene documento). Tercero, la estética como aisthesis: recuperando a Buck-Morss, describe cómo los materiales (hierro, concreto, luz) producen experiencias sensoriales y ambientales de la modernidad. Larkin refuta la tesis de la invisibilidad de la infraestructura (Star), mostrando su hipervisibilidad, y concluye que la elección metodológica sobre qué es infraestructura es una cuestión teórica de primer orden.</t>
         </is>
       </c>
     </row>
@@ -5676,27 +5676,27 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Marcus - Arte, etnografía y diseño. Reconfigurando el arte y la antropología hoy.md</t>
+          <t>Leone, Keane y Nakassis - Semiotic Ideology. A Dialogue across Semiotic Traditions.md</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>n/d (práctica etnográfica contemporánea desde los años 1980 hasta la década de 2010)</t>
+          <t>n/d (diálogo teórico; recorrido histórico del concepto de ideología desde fines del siglo XVIII hasta el presente)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Capítulo/ensayo académico, c. 2015 (traducción al español de Sidney Evans, revisión de Giuliana Borea)</t>
+          <t>Diálogo académico (transcripción editada de una sesión del 23 de junio de 2025), publicado en 2025</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>George E. Marcus (Center for Ethnography, University of California, Irvine); James Clifford; Claire Bishop; Nicolas Bourriaud; Hal Foster; Kim Fortun; Michael Fischer; Luke Cantarella; Christine Hegel; Anna Tsing; Bruno Latour; Cultural Anthropology (Writing Culture)</t>
+          <t>Massimo Leone (Università di Torino); Webb Keane (University of Michigan); Constantine V. Nakassis (University of Chicago); Simona Stano; Michael Silverstein; Umberto Eco; Charles S. Peirce; Karl Marx; Destutt de Tracy; Fondazione Bruno Kessler (Trento); Lexia</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Ensayo en que George Marcus reflexiona, desde el legado de Writing Culture (1986) y su balance en el 25º aniversario (Duke, 2011), sobre la convergencia entre el método etnográfico y las prácticas del arte contemporáneo y el diseño. Su preocupación no es una antropología del arte ni como arte, sino cómo los métodos colaborativos de taller y el arte conceptual site-specific se infiltran en la producción etnográfica, incentivando un «hacer» activo con otros durante el trabajo de campo, en las formas intermedias que median entre las notas de campo privadas y el texto etnográfico terminado. Marcus identifica cuatro tendencias post-ochenta en la etnografía y privilegia la cuarta —la colaboración— que convierte al informante en «socio epistémico» y a la teoría en forma primaria del dato (para-etnografía). Recupera y reencuadra su noción de etnografía multisituada (1995): ya no como seguimiento literal de procesos entre sitios, sino como construcción de micropúblicos, recepciones y «encuentros productivos» mediante «artilugios» (gizmos) que trasladan prototipos de pensamiento antes de su «anclaje» en la autoridad académica. Relata los experimentos del Center for Ethnography (UCI): colaboración, pedagogía, terceros espacios, parasitios, plataformas digitales (los Asthma Files de los Fortun). Dialoga con Artificial Hells de Claire Bishop y con el ensayo de Hal Foster «The Artist as Ethnographer?», sosteniendo que el arte participativo comparte con la etnografía el problema de generar públicos secundarios. Concluye con el proyecto ejemplar «214 Sq. Ft.» (coescrito con Cantarella y Hegel), instalación inmersiva sobre familias sin techo en el condado de Orange que, itinerando por sitios diversos, elicita etnográficamente la conciencia de la desigualdad entre los privilegiados, reformulando la «inmersión» como «amplificación».</t>
+          <t>Transcripción editada de un diálogo entre el semiótico continental Massimo Leone y el antropólogo lingüístico Webb Keane, moderado y prologado por Constantine Nakassis, que explora convergencias y divergencias entre la semiótica continental (Saussure, Greimas, Lotman, Eco) y la antropología lingüística norteamericana peirceana en torno a la noción de «ideología semiótica». Nakassis reconstruye la genealogía del término ideología: de la «ciencia de las ideas» materialista y antimetafísica de Destutt de Tracy, pasando por la resignificación peyorativa que impuso Napoleón vía enregisterment, hasta la doble crítica marxiana en La ideología alemana. Argumenta que la ideología no es falsa conciencia ni epifenómeno, sino mediación performativa constitutiva de lo social —ejemplificada en el fetichismo de la mercancía—, y que su espacio problemático coincide con el de la semiótica misma. Keane sostiene, desde el pragmatismo peirceano, que la semiosis importa menos por lo que nombra que por lo que trae al ser; introduce su concepto de «economía representacional» (transformaciones causales no significantes que reconfiguran las affordances del sentido, como la fotografía respecto de la pintura) y sitúa la abducción no como método hermenéutico del analista sino como el proceso cotidiano, falible y dialógico por el que la gente da sentido a los signos (rhema, dicent, argumento como modos de ideología semiótica). Ambos aceptan que el análisis es él mismo situado e ideológico, rechazando el objetivismo. Leone describe la ideología semiótica como espacio de tensión entre el yo-tú dialógico y la enunciación en tercera persona (el «it»), y como trampolín de autorreflexividad existencial. El debate aborda además la disolución del concepto de cultura y la unidad social de la ideología, implícita en las prácticas.</t>
         </is>
       </c>
     </row>
@@ -5708,27 +5708,27 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Marcus y Holmes - Collaboration Today and the Re-Imagination of the Classic Scene of Fieldwork Encounter (2008).md</t>
+          <t>Marcus - Arte, etnografía y diseño. Reconfigurando el arte y la antropología hoy.md</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Décadas de 1990-2000 (presente etnográfico contemporáneo)</t>
+          <t>n/d (práctica etnográfica contemporánea desde los años 1980 hasta la década de 2010)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico, 2008</t>
+          <t>Capítulo/ensayo académico, c. 2015 (traducción al español de Sidney Evans, revisión de Giuliana Borea)</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Douglas R. Holmes; George E. Marcus; David "Bert" Westbrook; Marc Abélès; Justin Richland; Pascal Lamy; Collaborative Anthropologies (University of Nebraska Press); Center for Ethnography (UC Irvine); proyecto Late Editions (Rice University); OMC</t>
+          <t>George E. Marcus (Center for Ethnography, University of California, Irvine); James Clifford; Claire Bishop; Nicolas Bourriaud; Hal Foster; Kim Fortun; Michael Fischer; Luke Cantarella; Christine Hegel; Anna Tsing; Bruno Latour; Cultural Anthropology (Writing Culture)</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Holmes y Marcus proponen reconceptualizar la colaboración como núcleo de un "refuncionamiento" (refunctioning) de la etnografía, más allá de dos sentidos que rechazan: la colaboración implícita y desigual del trabajo de campo malinowskiano clásico, y la ideología contemporánea del trabajo colectivo como mero entorno de investigación. Su tesis central es que la etnografía actual opera en comunidades epistémicas y de expertise (bancos centrales, laboratorios, ONG, espacios de arte, burocracias) donde los sujetos son ya reflexivos y practican una "para-etnografía": poseen una conciencia analítica y curiosidad que anticipa interlocutores. El concepto clave es la deferencia a la apropiación (deferral to appropriation): el etnógrafo debe ceder ante los marcos conceptuales de sus sujetos-socios epistémicos para que la investigación avance. El argumento se despliega narrativamente a través de la relación de los autores con el jurista Westbrook, quien, al escribir Navigators of the Contemporary, los "apropió" como informantes, invirtiendo la autoridad etnográfica y funcionando como simulacro o prototipo para pensar el trabajo de campo colaborativo. Recorren su genealogía intelectual (el proyecto Late Editions de los noventa, la etnografía multisituada, el tropo de la "complicidad") y ejemplifican con proyectos posteriores a 2000: la etnografía de Holmes sobre los bancos centrales y sus "alegorías econométricas" y el inflation targeting, y las intervenciones "para-site" del Center for Ethnography en la formación doctoral. Cierran con su participación en un estudio etnográfico de la OMC. El texto se posiciona como una reformulación de la escena clásica del encuentro de campo, sustituyendo el "punto de vista del nativo" por una negociación conceptual mutua con sujetos-interlocutores expertos.</t>
+          <t>Ensayo en que George Marcus reflexiona, desde el legado de Writing Culture (1986) y su balance en el 25º aniversario (Duke, 2011), sobre la convergencia entre el método etnográfico y las prácticas del arte contemporáneo y el diseño. Su preocupación no es una antropología del arte ni como arte, sino cómo los métodos colaborativos de taller y el arte conceptual site-specific se infiltran en la producción etnográfica, incentivando un «hacer» activo con otros durante el trabajo de campo, en las formas intermedias que median entre las notas de campo privadas y el texto etnográfico terminado. Marcus identifica cuatro tendencias post-ochenta en la etnografía y privilegia la cuarta —la colaboración— que convierte al informante en «socio epistémico» y a la teoría en forma primaria del dato (para-etnografía). Recupera y reencuadra su noción de etnografía multisituada (1995): ya no como seguimiento literal de procesos entre sitios, sino como construcción de micropúblicos, recepciones y «encuentros productivos» mediante «artilugios» (gizmos) que trasladan prototipos de pensamiento antes de su «anclaje» en la autoridad académica. Relata los experimentos del Center for Ethnography (UCI): colaboración, pedagogía, terceros espacios, parasitios, plataformas digitales (los Asthma Files de los Fortun). Dialoga con Artificial Hells de Claire Bishop y con el ensayo de Hal Foster «The Artist as Ethnographer?», sosteniendo que el arte participativo comparte con la etnografía el problema de generar públicos secundarios. Concluye con el proyecto ejemplar «214 Sq. Ft.» (coescrito con Cantarella y Hegel), instalación inmersiva sobre familias sin techo en el condado de Orange que, itinerando por sitios diversos, elicita etnográficamente la conciencia de la desigualdad entre los privilegiados, reformulando la «inmersión» como «amplificación».</t>
         </is>
       </c>
     </row>
@@ -5740,27 +5740,27 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Nakassis - A Linguistic Anthropology of Images (2023) [Annual Review of Anthropology 52, pp. 73-91].md</t>
+          <t>Marcus y Holmes - Collaboration Today and the Re-Imagination of the Classic Scene of Fieldwork Encounter (2008).md</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>Décadas de 1990-2000 (presente etnográfico contemporáneo)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Artículo de revisión académica, 2023</t>
+          <t>Artículo académico, 2008</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Constantine V. Nakassis (University of Chicago); Michael Silverstein; Roman Jakobson; Sol Worth; W. J. T. Mitchell; Erving Goffman; Asif Agha; Susan Gal e Judith Irvine; Webb Keane; Charles S. Peirce; Annual Review of Anthropology</t>
+          <t>Douglas R. Holmes; George E. Marcus; David "Bert" Westbrook; Marc Abélès; Justin Richland; Pascal Lamy; Collaborative Anthropologies (University of Nebraska Press); Center for Ethnography (UC Irvine); proyecto Late Editions (Rice University); OMC</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Nakassis esboza una antropología lingüística de las imágenes que rechaza toda distinción tajante entre lenguaje e imagen. Su argumento central es que la antropología lingüística, en su crítica pragmática al estructuralismo, desarrolló ya una teoría de la imagen "avant l'image": una imagen inmanente al discurso. Introduce el concepto de image-text (imagen-texto), un diagrama peirceano cuyas partes son imágenes, que emerge por entextualización cuando signos en contigüidad indexical figuran icónicamente una textura estética. Distingue image (tipo metasemiótico) de picture (la instancia material, token), retomando a Mitchell. Sostiene que las imágenes no son necesariamente visuales, existen en toda modalidad y son procesos temporales, no marcos espaciales estáticos. Repasa cuatro dimensiones semióticas para teorizar la imagen: entextualización y circulación (Shankar sobre publicidad y "diversidad", Hardy sobre el cine bhojpuri que coproduce lengua e industria); performatividad (la dicentización de Ball, los títeres de Barker, los altares de Santería de Wirtz, las caricaturas danesas de Keane y la mediación por ideologías semióticas); perspectiva (la "visión profesional" de Goodwin en el caso Rodney King, el "envisioning" de Chumley); y enregisterment (Agha, Gal e Irvine, con el realismo cinematográfico y los ejemplos tamiles del propio autor, distinguiendo estilos, registros y géneros narrativos como metasemióticas intertextuales). Recurre a las tres iconicidades de Peirce (imagen, diagrama, metáfora). Concluye ampliando el proyecto a una "antropología lingüística de...", un horizonte abierto de objetos unidos como antropología lingüística. La posición del texto es programática: no aislar la imagen como medio específico, sino generalizar desde ella los principios semióticos que atraviesan todo signo, incluido el lenguaje.</t>
+          <t>Holmes y Marcus proponen reconceptualizar la colaboración como núcleo de un "refuncionamiento" (refunctioning) de la etnografía, más allá de dos sentidos que rechazan: la colaboración implícita y desigual del trabajo de campo malinowskiano clásico, y la ideología contemporánea del trabajo colectivo como mero entorno de investigación. Su tesis central es que la etnografía actual opera en comunidades epistémicas y de expertise (bancos centrales, laboratorios, ONG, espacios de arte, burocracias) donde los sujetos son ya reflexivos y practican una "para-etnografía": poseen una conciencia analítica y curiosidad que anticipa interlocutores. El concepto clave es la deferencia a la apropiación (deferral to appropriation): el etnógrafo debe ceder ante los marcos conceptuales de sus sujetos-socios epistémicos para que la investigación avance. El argumento se despliega narrativamente a través de la relación de los autores con el jurista Westbrook, quien, al escribir Navigators of the Contemporary, los "apropió" como informantes, invirtiendo la autoridad etnográfica y funcionando como simulacro o prototipo para pensar el trabajo de campo colaborativo. Recorren su genealogía intelectual (el proyecto Late Editions de los noventa, la etnografía multisituada, el tropo de la "complicidad") y ejemplifican con proyectos posteriores a 2000: la etnografía de Holmes sobre los bancos centrales y sus "alegorías econométricas" y el inflation targeting, y las intervenciones "para-site" del Center for Ethnography en la formación doctoral. Cierran con su participación en un estudio etnográfico de la OMC. El texto se posiciona como una reformulación de la escena clásica del encuentro de campo, sustituyendo el "punto de vista del nativo" por una negociación conceptual mutua con sujetos-interlocutores expertos.</t>
         </is>
       </c>
     </row>
@@ -5772,7 +5772,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Nakassis - Indexicality's Ambivalent Ground [Signs and Society].md</t>
+          <t>Nakassis - A Linguistic Anthropology of Images (2023) [Annual Review of Anthropology 52, pp. 73-91].md</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -5782,17 +5782,17 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico, 2018</t>
+          <t>Artículo de revisión académica, 2023</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Constantine V. Nakassis (University of Chicago); Michael Silverstein; Charles S. Peirce; Roman Jakobson; Jacques Derrida; Martin Heidegger; Ferdinand de Saussure; Gottlob Frege; W. V. O. Quine; Rajinikanth; Signs and Society (Semiosis Research Center, Hankuk University)</t>
+          <t>Constantine V. Nakassis (University of Chicago); Michael Silverstein; Roman Jakobson; Sol Worth; W. J. T. Mitchell; Erving Goffman; Asif Agha; Susan Gal e Judith Irvine; Webb Keane; Charles S. Peirce; Annual Review of Anthropology</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Nakassis somete la categoría de indexicalidad —central a la antropología lingüística desde Silverstein— a una lectura reflexiva y deconstructiva. Su tesis es que la vitalidad teórica de la indexicalidad emerge de una ambivalencia fundacional e irresoluble entre inmediatez/presencia y mediación/representación. Aunque la indexicalidad se invocó para anclar el lenguaje en su contexto de uso y refutar las ideologías idealistas y representacionalistas de la filosofía "SAE" (Standard Average European) —Frege, Saussure y la reducción semantizante del lenguaje a denotación autónoma—, conserva paradójicamente algo de la metafísica de la presencia que critica: promete acercarnos a los fenómenos en su actualidad. Analiza la "escena primigenia" de la indexicalidad (el dedo índice que señala), mostrando, vía Quine ("Gavagai"), Heidegger ("La época de la imagen del mundo") y Derrida, su régimen ocularcéntrico y su deseo de inmediación. Propone reformular la indexicalidad mediante "etnografías de la presencia", ilustrándolo con su estudio de las imágenes cinematográficas del "mass hero" tamil Rajinikanth, donde el índice del actor no señala sino que engloba e incorpora a la audiencia en un idioma de darśan y soberanía cine-política; allí el fundamento indexical no es co-presencia autoevidente sino relación mediada de abarcamiento. Examina luego cómo la disciplina ha trabajado esta ambivalencia mediante un incesante desdoblamiento (presuponente/creativo, referencial/no referencial, orden n-ésimo/n+1) y suplementación (metapragmática, ideología, orden indexical). Concluye que la ambivalencia no debe resolverse sino mantenerse visible y escrutarse etnográficamente, pues expresa el realismo semiótico mismo: mediación e inmediatez como fases de una dialéctica irreductible que impulsa toda semiosis.</t>
+          <t>Nakassis esboza una antropología lingüística de las imágenes que rechaza toda distinción tajante entre lenguaje e imagen. Su argumento central es que la antropología lingüística, en su crítica pragmática al estructuralismo, desarrolló ya una teoría de la imagen "avant l'image": una imagen inmanente al discurso. Introduce el concepto de image-text (imagen-texto), un diagrama peirceano cuyas partes son imágenes, que emerge por entextualización cuando signos en contigüidad indexical figuran icónicamente una textura estética. Distingue image (tipo metasemiótico) de picture (la instancia material, token), retomando a Mitchell. Sostiene que las imágenes no son necesariamente visuales, existen en toda modalidad y son procesos temporales, no marcos espaciales estáticos. Repasa cuatro dimensiones semióticas para teorizar la imagen: entextualización y circulación (Shankar sobre publicidad y "diversidad", Hardy sobre el cine bhojpuri que coproduce lengua e industria); performatividad (la dicentización de Ball, los títeres de Barker, los altares de Santería de Wirtz, las caricaturas danesas de Keane y la mediación por ideologías semióticas); perspectiva (la "visión profesional" de Goodwin en el caso Rodney King, el "envisioning" de Chumley); y enregisterment (Agha, Gal e Irvine, con el realismo cinematográfico y los ejemplos tamiles del propio autor, distinguiendo estilos, registros y géneros narrativos como metasemióticas intertextuales). Recurre a las tres iconicidades de Peirce (imagen, diagrama, metáfora). Concluye ampliando el proyecto a una "antropología lingüística de...", un horizonte abierto de objetos unidos como antropología lingüística. La posición del texto es programática: no aislar la imagen como medio específico, sino generalizar desde ella los principios semióticos que atraviesan todo signo, incluido el lenguaje.</t>
         </is>
       </c>
     </row>
@@ -5804,7 +5804,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Nöth - Peirce's Iconicity and His Image-Diagram-Metaphor Triad Revisited. Complements to Stjernfelt's «Sheets, Diagrams, and Realism» (2024) [Semiotica 258, pp. 143-167].md</t>
+          <t>Nakassis - Indexicality's Ambivalent Ground [Signs and Society].md</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -5814,17 +5814,17 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Artículo de reseña académica (review article), 2024</t>
+          <t>Artículo académico, 2018</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Winfried Nöth (Pontifícia Universidade Católica de São Paulo); Frederik Stjernfelt; Charles S. Peirce; Charles Morris; Lucia Santaella; Aristóteles; Douglas R. Anderson; Semiotica (De Gruyter); serie Peirceana</t>
+          <t>Constantine V. Nakassis (University of Chicago); Michael Silverstein; Charles S. Peirce; Roman Jakobson; Jacques Derrida; Martin Heidegger; Ferdinand de Saussure; Gottlob Frege; W. V. O. Quine; Rajinikanth; Signs and Society (Semiosis Research Center, Hankuk University)</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Este artículo-reseña de Sheets, Diagrams, and Realism in Peirce (2022) de Frederik Stjernfelt reconoce la obra como un avance mayor en la semiótica peirceana, pero argumenta contra su reducción de la teoría de la iconicidad a la iconicidad diagramática. La tesis de Nöth es que el fundamento de la subdivisión triádica del icono —imagen, diagrama, metáfora— no está en la lógica diagramática de los Gráficos Existenciales sino en las categorías cenopitagóricas de Peirce (primeridad, segundidad, terceridad). Muestra que Peirce apenas usó el término "iconicity" (dos veces), y que la noción de grados de iconicidad proviene en realidad de Charles Morris, cuya escala (mayor iconicidad = más detalles, culminando en la identidad signo-objeto) es incompatible con Peirce: para él la iconicidad es máxima cuando la semioticidad es mínima (el icono puro o cualisigno), y decrece de la imagen a la metáfora, mientras que una fotografía perfecta es índice, no icono. Corrige varias interpretaciones de Stjernfelt: que el diagrama sea siempre un tipo/legisigno (lo que eliminaría el sinsigno icónico), el uso equívoco de "degenerate" y "generic", y la aplicabilidad de la generalidad a los iconos (insight peirceano de 1903). El núcleo del texto defiende la terceridad en la primeridad de la metáfora: esta no es una relación de adicidad triádica (valencia verbal) sino un "paralelismo en algo más" (tertium comparationis) que también abarca símiles, comparaciones, analogías, argumentos por analogía y ejemplos, apoyándose en la retórica clásica (Aristóteles, Lausberg) y en el manuscrito de 1903 donde Peirce usa "example" como variante de "metaphor". Reconstruye finalmente los fundamentos categoriales de la tríada con apoyo diagramático.</t>
+          <t>Nakassis somete la categoría de indexicalidad —central a la antropología lingüística desde Silverstein— a una lectura reflexiva y deconstructiva. Su tesis es que la vitalidad teórica de la indexicalidad emerge de una ambivalencia fundacional e irresoluble entre inmediatez/presencia y mediación/representación. Aunque la indexicalidad se invocó para anclar el lenguaje en su contexto de uso y refutar las ideologías idealistas y representacionalistas de la filosofía "SAE" (Standard Average European) —Frege, Saussure y la reducción semantizante del lenguaje a denotación autónoma—, conserva paradójicamente algo de la metafísica de la presencia que critica: promete acercarnos a los fenómenos en su actualidad. Analiza la "escena primigenia" de la indexicalidad (el dedo índice que señala), mostrando, vía Quine ("Gavagai"), Heidegger ("La época de la imagen del mundo") y Derrida, su régimen ocularcéntrico y su deseo de inmediación. Propone reformular la indexicalidad mediante "etnografías de la presencia", ilustrándolo con su estudio de las imágenes cinematográficas del "mass hero" tamil Rajinikanth, donde el índice del actor no señala sino que engloba e incorpora a la audiencia en un idioma de darśan y soberanía cine-política; allí el fundamento indexical no es co-presencia autoevidente sino relación mediada de abarcamiento. Examina luego cómo la disciplina ha trabajado esta ambivalencia mediante un incesante desdoblamiento (presuponente/creativo, referencial/no referencial, orden n-ésimo/n+1) y suplementación (metapragmática, ideología, orden indexical). Concluye que la ambivalencia no debe resolverse sino mantenerse visible y escrutarse etnográficamente, pues expresa el realismo semiótico mismo: mediación e inmediatez como fases de una dialéctica irreductible que impulsa toda semiosis.</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Nöth - Visual Semiotics. Key Features and an Application to Picture Ads (2011) [The SAGE Handbook of Visual Research Methods, cap. 16].md</t>
+          <t>Nöth - Peirce's Iconicity and His Image-Diagram-Metaphor Triad Revisited. Complements to Stjernfelt's «Sheets, Diagrams, and Realism» (2024) [Semiotica 258, pp. 143-167].md</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -5846,17 +5846,17 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro / manual académico, 2011</t>
+          <t>Artículo de reseña académica (review article), 2024</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Winfried Nöth; Charles S. Peirce; Roland Barthes; Ferdinand de Saussure; Louis Hjelmslev; Jean-Marie Floch; Lucia Santaella; Grupo µ (Escuela de Lieja); Escuela de París; Umberto Eco; The SAGE Handbook of Visual Research Methods; International Association for Visual Semiotics</t>
+          <t>Winfried Nöth (Pontifícia Universidade Católica de São Paulo); Frederik Stjernfelt; Charles S. Peirce; Charles Morris; Lucia Santaella; Aristóteles; Douglas R. Anderson; Semiotica (De Gruyter); serie Peirceana</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Capítulo panorámico que expone las características centrales de la semiótica visual como rama de la semiótica aplicada, restringido a la imagen fija (pinturas, fotografías, imágenes de prensa). Nöth traza la historia del campo desde su fundación en los años sesenta por lingüistas estructurales, con Barthes y su "retórica de la imagen" apoyada en Saussure y Hjelmslev, y distingue las principales escuelas: la retórica visual del Grupo µ de Lieja, la Escuela de París (con analogías entre imagen y lengua, planos de expresión y contenido, oposiciones binarias) y el enfoque peirceano. Discute el potencial semiótico diferencial y complementario de palabra e imagen (linealidad temporal vs. espacialidad bidimensional) y refuta el logocentrismo de Barthes sobre la dependencia verbal de la imagen. Desarrolla el modelo triádico del signo de Peirce (representamen, objeto, interpretante) aplicado a la imagen, y la tricotomía icono-índice-símbolo como sistema de inclusión: las imágenes son típicamente icónicas, pero las fotografías son índices (conexión causal por proyección lumínica e identificación de un objeto singular), y muchas incorporan símbolos que requieren conocimiento cultural. Aborda por qué las pinturas abstractas son signos (signos plásticos, icono puro autorreferencial), la sintaxis y semántica visuales, y una pragmática visual centrada en la imposibilidad de actos pictóricos directos (las imágenes carecen de metasignos, no pueden afirmar ni mentir explícitamente, solo mostrar). Concluye con dos estudios de caso de anuncios de prensa: el análisis de la Escuela de París de Floch sobre la campaña de cigarrillos "News" (1980) con su oposición identidad/alteridad, y el enfoque peirceano de Santaella y Nöth sobre un aviso de ginebra Beefeater (1974) como transferencia de valor simbólico de la corona a la marca.</t>
+          <t>Este artículo-reseña de Sheets, Diagrams, and Realism in Peirce (2022) de Frederik Stjernfelt reconoce la obra como un avance mayor en la semiótica peirceana, pero argumenta contra su reducción de la teoría de la iconicidad a la iconicidad diagramática. La tesis de Nöth es que el fundamento de la subdivisión triádica del icono —imagen, diagrama, metáfora— no está en la lógica diagramática de los Gráficos Existenciales sino en las categorías cenopitagóricas de Peirce (primeridad, segundidad, terceridad). Muestra que Peirce apenas usó el término "iconicity" (dos veces), y que la noción de grados de iconicidad proviene en realidad de Charles Morris, cuya escala (mayor iconicidad = más detalles, culminando en la identidad signo-objeto) es incompatible con Peirce: para él la iconicidad es máxima cuando la semioticidad es mínima (el icono puro o cualisigno), y decrece de la imagen a la metáfora, mientras que una fotografía perfecta es índice, no icono. Corrige varias interpretaciones de Stjernfelt: que el diagrama sea siempre un tipo/legisigno (lo que eliminaría el sinsigno icónico), el uso equívoco de "degenerate" y "generic", y la aplicabilidad de la generalidad a los iconos (insight peirceano de 1903). El núcleo del texto defiende la terceridad en la primeridad de la metáfora: esta no es una relación de adicidad triádica (valencia verbal) sino un "paralelismo en algo más" (tertium comparationis) que también abarca símiles, comparaciones, analogías, argumentos por analogía y ejemplos, apoyándose en la retórica clásica (Aristóteles, Lausberg) y en el manuscrito de 1903 donde Peirce usa "example" como variante de "metaphor". Reconstruye finalmente los fundamentos categoriales de la tríada con apoyo diagramático.</t>
         </is>
       </c>
     </row>
@@ -5868,27 +5868,27 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Pinochet Cobos - Antropologías del arte en tiempo presente. Una aproximación (2020).md</t>
+          <t>Nöth - Visual Semiotics. Key Features and an Application to Picture Ads (2011) [The SAGE Handbook of Visual Research Methods, cap. 16].md</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>n/d (tiempo presente; escenas artísticas contemporáneas)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico (introducción a dossier temático), 2020</t>
+          <t>Capítulo de libro / manual académico, 2011</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Carla Pinochet Cobos (Universidad Alberto Hurtado); Alfred Gell; Néstor García Canclini; Pierre Bourdieu; Howard Becker; Nathalie Heinich; James Clifford; Sally Price; George Marcus y Fred Myers; María Paz Peirano, Sebastián Muñoz y Mijail Mitrovic (autores del dossier); FONDECYT</t>
+          <t>Winfried Nöth; Charles S. Peirce; Roland Barthes; Ferdinand de Saussure; Louis Hjelmslev; Jean-Marie Floch; Lucia Santaella; Grupo µ (Escuela de Lieja); Escuela de París; Umberto Eco; The SAGE Handbook of Visual Research Methods; International Association for Visual Semiotics</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Pinochet ofrece una aproximación a las antropologías del arte atendiendo a cómo sus tensiones constitutivas históricas adquieren forma contemporánea en América Latina. Su lugar de enunciación reivindica el derecho de las antropologías latinoamericanas a ocuparse de la complejidad de sus propias escenas artísticas —no solo del arte indígena o popular de la otredad—, sin ceder a las demandas exotizantes ni neoprimitivistas del campo académico y artístico metropolitano, en la senda de The Traffic in Culture (Marcus y Myers). Revisa tres nudos: el lugar de enunciación, el objeto de estudio y los modelos teóricos. Retomando a Gell, plantea que la antropología del arte exige un "desmontaje" del ethos esteticista del investigador (el arte como "religión de los intelectuales"), operando un desanclaje entre arte y estética —esta última un régimen de identificación entre otros, provincializado por las críticas poscoloniales y decoloniales— que impone un "filisteísmo metodológico". Sobre la especificidad del objeto, articula la mirada semiótica de Geertz con la propuesta pragmatista de García Canclini (el arte posautónomo como "inminencia", contrato oblicuo con lo real) y Heinich, y con la teoría de la agencia de Gell (las obras como agentes sociales; anclaje, circulación y valor, según Borea). Contrapone luego los modelos del campo artístico de Bourdieu (jerarquía, lucha, capital) y de los mundos del arte de Becker (cooperación, convención). La segunda mitad, empírica, discute la profesionalización artística a partir de tres etnografías del dossier (cine chileno, rap bonaerense, artes visuales limeñas), leyéndolas como gestión de las contradicciones del trabajo creativo en torno a la autonomía, la singularidad y la sustentabilidad, marcadas por precariedad, entusiasmo y multiactividad.</t>
+          <t>Capítulo panorámico que expone las características centrales de la semiótica visual como rama de la semiótica aplicada, restringido a la imagen fija (pinturas, fotografías, imágenes de prensa). Nöth traza la historia del campo desde su fundación en los años sesenta por lingüistas estructurales, con Barthes y su "retórica de la imagen" apoyada en Saussure y Hjelmslev, y distingue las principales escuelas: la retórica visual del Grupo µ de Lieja, la Escuela de París (con analogías entre imagen y lengua, planos de expresión y contenido, oposiciones binarias) y el enfoque peirceano. Discute el potencial semiótico diferencial y complementario de palabra e imagen (linealidad temporal vs. espacialidad bidimensional) y refuta el logocentrismo de Barthes sobre la dependencia verbal de la imagen. Desarrolla el modelo triádico del signo de Peirce (representamen, objeto, interpretante) aplicado a la imagen, y la tricotomía icono-índice-símbolo como sistema de inclusión: las imágenes son típicamente icónicas, pero las fotografías son índices (conexión causal por proyección lumínica e identificación de un objeto singular), y muchas incorporan símbolos que requieren conocimiento cultural. Aborda por qué las pinturas abstractas son signos (signos plásticos, icono puro autorreferencial), la sintaxis y semántica visuales, y una pragmática visual centrada en la imposibilidad de actos pictóricos directos (las imágenes carecen de metasignos, no pueden afirmar ni mentir explícitamente, solo mostrar). Concluye con dos estudios de caso de anuncios de prensa: el análisis de la Escuela de París de Floch sobre la campaña de cigarrillos "News" (1980) con su oposición identidad/alteridad, y el enfoque peirceano de Santaella y Nöth sobre un aviso de ginebra Beefeater (1974) como transferencia de valor simbólico de la corona a la marca.</t>
         </is>
       </c>
     </row>
@@ -5900,27 +5900,27 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Pinochet Cobos - Arte, comunidad y polifonía. Acerca de la noción de investigación en arte y antropología.md</t>
+          <t>Pinochet Cobos - Antropologías del arte en tiempo presente. Una aproximación (2020).md</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>n/d (prácticas contemporáneas posteriores al «giro etnográfico» de fines de los años noventa)</t>
+          <t>n/d (tiempo presente; escenas artísticas contemporáneas)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico, s/f</t>
+          <t>Artículo académico (introducción a dossier temático), 2020</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Carla Pinochet Cobos; Hal Foster; Natascha Sadr Haghighian; Sherry Ortner; Chantal Mouffe; Jacques Rancière; Pilar Riaño; Leticia Katzer y Agustín Samprón</t>
+          <t>Carla Pinochet Cobos (Universidad Alberto Hurtado); Alfred Gell; Néstor García Canclini; Pierre Bourdieu; Howard Becker; Nathalie Heinich; James Clifford; Sally Price; George Marcus y Fred Myers; María Paz Peirano, Sebastián Muñoz y Mijail Mitrovic (autores del dossier); FONDECYT</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>El ensayo interroga la noción de investigación como bisagra conceptual del cruce contemporáneo entre arte y antropología, en un escenario marcado por el «giro etnográfico» (Foster) y la proliferación de proyectos comunitarios, colaborativos y de mediación cultural. Pinochet Cobos sostiene que investigar admite significados divergentes y propone una tipología de tres figuras del investigador: el «traductor», que asume una mirada parcial y traduce entre registros remitidos a la subjetividad; el «detective», que busca desclasificar, visibilizar o denunciar un saber oculto preexistente; y el «procesualista», que produce un conocimiento emergente inexistente de antemano, construido experimentalmente en el encuentro. La autora privilegia este tercer modelo por habilitar una producción interdisciplinaria genuinamente dialógica, un «construir con otros» de raíz polifónica heredada de la antropología posmoderna. Estructura su reflexión en cuatro niveles —las preguntas, los caminos, las herramientas y los resultados— y señala en cada uno las encrucijadas específicas de ambas disciplinas: la antropología debe romper con la lógica del «informante» y su racionalidad rígida; el arte debe abandonar la autoría del genio y la sensibilidad privilegiada del artista individual. Advierte que las metodologías compartidas (observación participante, entrevista, mapeo, bitácoras) no bastan: deben devenir vías para una voz colectiva, una «investigación sin garantías». El texto cierra con una crítica a las estructuras institucionales de la economía del conocimiento, que dificultan lo lento, colaborativo y no replicable. Define la cooperación no como armonía sino como choque de significados, disenso y conflicto antagonista, condición de una emergencia cognitiva compartida.</t>
+          <t>Pinochet ofrece una aproximación a las antropologías del arte atendiendo a cómo sus tensiones constitutivas históricas adquieren forma contemporánea en América Latina. Su lugar de enunciación reivindica el derecho de las antropologías latinoamericanas a ocuparse de la complejidad de sus propias escenas artísticas —no solo del arte indígena o popular de la otredad—, sin ceder a las demandas exotizantes ni neoprimitivistas del campo académico y artístico metropolitano, en la senda de The Traffic in Culture (Marcus y Myers). Revisa tres nudos: el lugar de enunciación, el objeto de estudio y los modelos teóricos. Retomando a Gell, plantea que la antropología del arte exige un "desmontaje" del ethos esteticista del investigador (el arte como "religión de los intelectuales"), operando un desanclaje entre arte y estética —esta última un régimen de identificación entre otros, provincializado por las críticas poscoloniales y decoloniales— que impone un "filisteísmo metodológico". Sobre la especificidad del objeto, articula la mirada semiótica de Geertz con la propuesta pragmatista de García Canclini (el arte posautónomo como "inminencia", contrato oblicuo con lo real) y Heinich, y con la teoría de la agencia de Gell (las obras como agentes sociales; anclaje, circulación y valor, según Borea). Contrapone luego los modelos del campo artístico de Bourdieu (jerarquía, lucha, capital) y de los mundos del arte de Becker (cooperación, convención). La segunda mitad, empírica, discute la profesionalización artística a partir de tres etnografías del dossier (cine chileno, rap bonaerense, artes visuales limeñas), leyéndolas como gestión de las contradicciones del trabajo creativo en torno a la autonomía, la singularidad y la sustentabilidad, marcadas por precariedad, entusiasmo y multiactividad.</t>
         </is>
       </c>
     </row>
@@ -5932,27 +5932,27 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Pinochet Cobos y Tobar Tapia - El giro creativo en el trabajo contemporáneo (2021).md</t>
+          <t>Pinochet Cobos - Arte, comunidad y polifonía. Acerca de la noción de investigación en arte y antropología.md</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>2017-2019 (trabajo de campo en Santiago de Chile)</t>
+          <t>n/d (prácticas contemporáneas posteriores al «giro etnográfico» de fines de los años noventa)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico, 2021 (revista CUHSO, Universidad Católica de Temuco)</t>
+          <t>Ensayo académico, s/f</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Carla Pinochet Cobos (U. Alberto Hurtado); Constanza Tobar Tapia (U. de Chile); Luc Boltanski y Ève Chiapello; Maurizio Lazzarato; Bojana Kunst; Richard Florida; Angela McRobbie; Isabell Lorey; Nathalie Heinich; Howard Becker; revista CUHSO</t>
+          <t>Carla Pinochet Cobos; Hal Foster; Natascha Sadr Haghighian; Sherry Ortner; Chantal Mouffe; Jacques Rancière; Pilar Riaño; Leticia Katzer y Agustín Samprón</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>El artículo examina los fundamentos del «giro creativo» del trabajo contemporáneo: el proceso por el cual el modo de vida artístico —flexible, apasionado, autodirigido— se convierte en referente laboral exportable a otros sectores productivos en el marco del capitalismo flexible o postfordista. A partir de un estudio cualitativo (64 casos de artistas, creativos e intelectuales de Santiago, con bitácoras autoetnográficas y entrevistas en profundidad entre 2017 y 2019), las autoras contraponen a los discursos celebratorios (Florida, ciudades y economías creativas) el reverso precario del oficio. Movilizan a Boltanski y Chiapello (absorción de la «crítica artista» por el nuevo espíritu del capitalismo), Lazzarato (el «empresario de sí mismo») y Kunst (la homología entre arte y capitalismo como apropiación de la vida) para mostrar cómo la labor creativa niega su propia condición productiva. Organizan los costos subjetivos en torno a tres ejes conflictivos —el tiempo (intermitencia, multiactividad, indistinción trabajo/ocio), el dinero (trabajo impago, economías afectivas del favor y la visibilidad) y la gestión (autogestión permanente)—, que derivan en sobrecarga y en una intensa regulación emocional. Restituyen la agencia de los sujetos identificando tácticas cotidianas y estrategias de largo plazo, y acuñan la categoría de «trabajo experimentado como propio», núcleo que infunde sentido a la identidad laboral. La tesis final es que los creativos no se enuncian ni como trabajadores ni como empresarios, sino desde discursos de excepción (excentricidad, privilegio, carencia) anclados en el «régimen de singularidad», matizando en la periferia santiaguina las retóricas del autoemprendimiento neoliberal.</t>
+          <t>El ensayo interroga la noción de investigación como bisagra conceptual del cruce contemporáneo entre arte y antropología, en un escenario marcado por el «giro etnográfico» (Foster) y la proliferación de proyectos comunitarios, colaborativos y de mediación cultural. Pinochet Cobos sostiene que investigar admite significados divergentes y propone una tipología de tres figuras del investigador: el «traductor», que asume una mirada parcial y traduce entre registros remitidos a la subjetividad; el «detective», que busca desclasificar, visibilizar o denunciar un saber oculto preexistente; y el «procesualista», que produce un conocimiento emergente inexistente de antemano, construido experimentalmente en el encuentro. La autora privilegia este tercer modelo por habilitar una producción interdisciplinaria genuinamente dialógica, un «construir con otros» de raíz polifónica heredada de la antropología posmoderna. Estructura su reflexión en cuatro niveles —las preguntas, los caminos, las herramientas y los resultados— y señala en cada uno las encrucijadas específicas de ambas disciplinas: la antropología debe romper con la lógica del «informante» y su racionalidad rígida; el arte debe abandonar la autoría del genio y la sensibilidad privilegiada del artista individual. Advierte que las metodologías compartidas (observación participante, entrevista, mapeo, bitácoras) no bastan: deben devenir vías para una voz colectiva, una «investigación sin garantías». El texto cierra con una crítica a las estructuras institucionales de la economía del conocimiento, que dificultan lo lento, colaborativo y no replicable. Define la cooperación no como armonía sino como choque de significados, disenso y conflicto antagonista, condición de una emergencia cognitiva compartida.</t>
         </is>
       </c>
     </row>
@@ -5964,27 +5964,27 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Rabinow - Unconsolable Contemporary. Observing Gerhard Richter.md</t>
+          <t>Pinochet Cobos y Tobar Tapia - El giro creativo en el trabajo contemporáneo (2021).md</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Segunda mitad del siglo XX hasta 2014 (trayectoria de Gerhard Richter; serie Birkenau)</t>
+          <t>2017-2019 (trabajo de campo en Santiago de Chile)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Libro, 2017 (Duke University Press)</t>
+          <t>Artículo académico, 2021 (revista CUHSO, Universidad Católica de Temuco)</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Paul Rabinow; Gerhard Richter; Benjamin H. D. Buchloh; Mark Godfrey; Georges Didi-Huberman; Aby Warburg; Michel Foucault; Jean-François Lyotard; Theodor Adorno; Michaël Fœssel; revista October; Duke University Press</t>
+          <t>Carla Pinochet Cobos (U. Alberto Hurtado); Constanza Tobar Tapia (U. de Chile); Luc Boltanski y Ève Chiapello; Maurizio Lazzarato; Bojana Kunst; Richard Florida; Angela McRobbie; Isabell Lorey; Nathalie Heinich; Howard Becker; revista CUHSO</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Rabinow propone un experimento de antropología del contemporáneo tomando la obra y la práctica de Gerhard Richter como ocasión —no como ejemplo ni como teoría de la pintura— para articular un «ethos contemporáneo». Desde una posición declarada de «amateur» y de «adyacencia», ensaya una observación de segundo orden sobre el ensamblaje heterogéneo que rodea a Richter: críticos, curadores, instituciones y mercados. El concepto central es el de «lo contemporáneo», definido como ratio móvil de la modernidad que atraviesa el pasado reciente y el futuro próximo en un espacio no lineal; rechaza la existencia de un «posmoderno» definitivo y, siguiendo a Warburg y Didi-Huberman, postula un Nachleben (pervivencia, «vida póstuma») de lo moderno y una Pathosformel que Richter integra en su producción de imágenes. Distingue analíticamente lo moderno (batalla por la forma, según Foucault) y la modernidad (separación weberiana de las esferas de valor). El libro discute críticamente la lectura de Buchloh —de cuño frankfurtiano y de la revista October— sobre las pinturas Birkenau (2014) y sobre el arte tras Auschwitz (Adorno), oponiéndole la interpretación más matizada de Godfrey y la noción de «differend» de Lyotard: dar testimonio de lo irrepresentable sin inscribirlo de un modo que garantice su olvido. Rabinow valora el kairós de Richter no en el Holocausto sino en la relación devenida histórica entre modernismo y modernidad. La figura del título —lo «inconsolable» (Fœssel)— nombra un ethos restivo y recalcitrante que rechaza la consolación como resultado, sosteniéndola solo como deseo y protesta ética.</t>
+          <t>El artículo examina los fundamentos del «giro creativo» del trabajo contemporáneo: el proceso por el cual el modo de vida artístico —flexible, apasionado, autodirigido— se convierte en referente laboral exportable a otros sectores productivos en el marco del capitalismo flexible o postfordista. A partir de un estudio cualitativo (64 casos de artistas, creativos e intelectuales de Santiago, con bitácoras autoetnográficas y entrevistas en profundidad entre 2017 y 2019), las autoras contraponen a los discursos celebratorios (Florida, ciudades y economías creativas) el reverso precario del oficio. Movilizan a Boltanski y Chiapello (absorción de la «crítica artista» por el nuevo espíritu del capitalismo), Lazzarato (el «empresario de sí mismo») y Kunst (la homología entre arte y capitalismo como apropiación de la vida) para mostrar cómo la labor creativa niega su propia condición productiva. Organizan los costos subjetivos en torno a tres ejes conflictivos —el tiempo (intermitencia, multiactividad, indistinción trabajo/ocio), el dinero (trabajo impago, economías afectivas del favor y la visibilidad) y la gestión (autogestión permanente)—, que derivan en sobrecarga y en una intensa regulación emocional. Restituyen la agencia de los sujetos identificando tácticas cotidianas y estrategias de largo plazo, y acuñan la categoría de «trabajo experimentado como propio», núcleo que infunde sentido a la identidad laboral. La tesis final es que los creativos no se enuncian ni como trabajadores ni como empresarios, sino desde discursos de excepción (excentricidad, privilegio, carencia) anclados en el «régimen de singularidad», matizando en la periferia santiaguina las retóricas del autoemprendimiento neoliberal.</t>
         </is>
       </c>
     </row>
@@ -5996,27 +5996,27 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Rancière - El malestar en la estética.md</t>
+          <t>Rabinow - Unconsolable Contemporary. Observing Gerhard Richter.md</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>n/d (texto teórico; referencias a la constitución del régimen estético desde fines del s. XVIII)</t>
+          <t>Segunda mitad del siglo XX hasta 2014 (trayectoria de Gerhard Richter; serie Birkenau)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Libro, 2011 (Capital Intelectual, Buenos Aires; orig. «Malaise dans l'esthétique», Galilée, 2004)</t>
+          <t>Libro, 2017 (Duke University Press)</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Jacques Rancière; Immanuel Kant; Friedrich Schiller; G. W. F. Hegel; Pierre Bourdieu; Alain Badiou; Jean-François Lyotard; Theodor Adorno; F. W. J. Schelling; Barnett Newman; Capital Intelectual</t>
+          <t>Paul Rabinow; Gerhard Richter; Benjamin H. D. Buchloh; Mark Godfrey; Georges Didi-Huberman; Aby Warburg; Michel Foucault; Jean-François Lyotard; Theodor Adorno; Michaël Fœssel; revista October; Duke University Press</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Rancière responde a la «mala reputación» contemporánea de la estética —acusada, desde Bourdieu al «antiaesthetic» posmoderno, de encubrir lo social o de sostener promesas revolucionarias falaces— invirtiendo los términos del reproche. Su tesis es que «estética» no designa una disciplina ni una teoría de la sensibilidad, sino un régimen de identificación del arte históricamente constituido hace dos siglos. Frente al «régimen representativo», gobernado por la mímesis y por una relación reglada entre poiesis y aisthesis garantizada por la «naturaleza humana», el «régimen estético del arte» nace de la ruina de esa relación tripartita: disuelve la jerarquía de temas y géneros, iguala lo noble y lo ínfimo (la bomba de agua de Stendhal, los mendigos de Murillo), y liga las obras a una potencia anónima —pueblo, historia— ofreciéndolas a una mirada cualquiera. La estética es el pensamiento de ese «sensorium paradójico» donde se unen sin concepto actividad y pasividad, lo querido y lo no querido. Rancière argumenta que este régimen conlleva intrínsecamente una política o metapolítica: la promesa schilleriana del «libre juego» y de una humanidad por venir. El libro despliega esta matriz en capítulos sobre la estética como política, los problemas del arte crítico, las antinomias del modernismo (con una crítica a la «inestética» de Badiou), la estética de lo sublime en Lyotard como contralectura de Kant, y el «giro ético» que hoy disuelve arte y política en la indistinción de la comunidad ética. El «malestar», concluye, es tan antiguo y constitutivo como la estética misma.</t>
+          <t>Rabinow propone un experimento de antropología del contemporáneo tomando la obra y la práctica de Gerhard Richter como ocasión —no como ejemplo ni como teoría de la pintura— para articular un «ethos contemporáneo». Desde una posición declarada de «amateur» y de «adyacencia», ensaya una observación de segundo orden sobre el ensamblaje heterogéneo que rodea a Richter: críticos, curadores, instituciones y mercados. El concepto central es el de «lo contemporáneo», definido como ratio móvil de la modernidad que atraviesa el pasado reciente y el futuro próximo en un espacio no lineal; rechaza la existencia de un «posmoderno» definitivo y, siguiendo a Warburg y Didi-Huberman, postula un Nachleben (pervivencia, «vida póstuma») de lo moderno y una Pathosformel que Richter integra en su producción de imágenes. Distingue analíticamente lo moderno (batalla por la forma, según Foucault) y la modernidad (separación weberiana de las esferas de valor). El libro discute críticamente la lectura de Buchloh —de cuño frankfurtiano y de la revista October— sobre las pinturas Birkenau (2014) y sobre el arte tras Auschwitz (Adorno), oponiéndole la interpretación más matizada de Godfrey y la noción de «differend» de Lyotard: dar testimonio de lo irrepresentable sin inscribirlo de un modo que garantice su olvido. Rabinow valora el kairós de Richter no en el Holocausto sino en la relación devenida histórica entre modernismo y modernidad. La figura del título —lo «inconsolable» (Fœssel)— nombra un ethos restivo y recalcitrante que rechaza la consolación como resultado, sosteniéndola solo como deseo y protesta ética.</t>
         </is>
       </c>
     </row>
@@ -6028,27 +6028,27 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Rancière - El reparto de lo sensible. Estética y política (2014) [Prometeo, trad. Mónica Padró, ISBN 9789875745797].md</t>
+          <t>Rancière - El malestar en la estética.md</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>n/d (texto teórico; genealogía de los regímenes del arte de la Antigüedad al presente)</t>
+          <t>n/d (texto teórico; referencias a la constitución del régimen estético desde fines del s. XVIII)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Libro (entrevista-ensayo), 2014 (Prometeo, Buenos Aires; orig. «Le Partage du sensible», La Fabrique, 2000)</t>
+          <t>Libro, 2011 (Capital Intelectual, Buenos Aires; orig. «Malaise dans l'esthétique», Galilée, 2004)</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Jacques Rancière; Mónica Padró (trad.); Marcelo G. Burello; María Beatriz Greco (estudio preliminar); Platón; Aristóteles; Friedrich Schiller; Prometeo Libros; La Fabrique</t>
+          <t>Jacques Rancière; Immanuel Kant; Friedrich Schiller; G. W. F. Hegel; Pierre Bourdieu; Alain Badiou; Jean-François Lyotard; Theodor Adorno; F. W. J. Schelling; Barnett Newman; Capital Intelectual</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>En este texto seminal, estructurado como serie de respuestas a preguntas, Rancière expone la noción que articula su pensamiento estético-político: el «reparto de lo sensible», entendido como el sistema de evidencias sensibles que hace ver simultáneamente la existencia de un común y los recortes que definen los lugares y partes de cada quien. Todo reparto distribuye tiempos, espacios y formas de actividad, y determina quién tiene parte en lo común: el ciudadano aristotélico frente al esclavo que comprende pero no «posee» el lenguaje, o los artesanos platónicos que, por no tener tiempo, no pueden ocupar otro lugar que su trabajo. La política y el arte no son esferas separadas sino dos formas de división de lo sensible dependientes de regímenes de identificación. Rancière distingue tres regímenes del arte: el ético de las imágenes (Platón, donde el arte no se distingue como tal y se juzga por su verdad y sus efectos), el representativo o poético (la mímesis y su jerarquía de géneros) y el estético (que libera al arte de la regla mimética y lo define por un sensorium específico, singular y autónomo). Critica la noción de «modernidad» y de vanguardia como relatos empobrecidos del «fin» y el «retorno», y aborda la promoción estética de los anónimos por las artes mecánicas (fotografía, cine), los modos de la ficción frente a la historia, y la relación entre arte y trabajo. La estética emerge así como pensamiento de la igualdad y del disenso inscrito en las formas mismas de la experiencia sensible.</t>
+          <t>Rancière responde a la «mala reputación» contemporánea de la estética —acusada, desde Bourdieu al «antiaesthetic» posmoderno, de encubrir lo social o de sostener promesas revolucionarias falaces— invirtiendo los términos del reproche. Su tesis es que «estética» no designa una disciplina ni una teoría de la sensibilidad, sino un régimen de identificación del arte históricamente constituido hace dos siglos. Frente al «régimen representativo», gobernado por la mímesis y por una relación reglada entre poiesis y aisthesis garantizada por la «naturaleza humana», el «régimen estético del arte» nace de la ruina de esa relación tripartita: disuelve la jerarquía de temas y géneros, iguala lo noble y lo ínfimo (la bomba de agua de Stendhal, los mendigos de Murillo), y liga las obras a una potencia anónima —pueblo, historia— ofreciéndolas a una mirada cualquiera. La estética es el pensamiento de ese «sensorium paradójico» donde se unen sin concepto actividad y pasividad, lo querido y lo no querido. Rancière argumenta que este régimen conlleva intrínsecamente una política o metapolítica: la promesa schilleriana del «libre juego» y de una humanidad por venir. El libro despliega esta matriz en capítulos sobre la estética como política, los problemas del arte crítico, las antinomias del modernismo (con una crítica a la «inestética» de Badiou), la estética de lo sublime en Lyotard como contralectura de Kant, y el «giro ético» que hoy disuelve arte y política en la indistinción de la comunidad ética. El «malestar», concluye, es tan antiguo y constitutivo como la estética misma.</t>
         </is>
       </c>
     </row>
@@ -6060,27 +6060,27 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Rancière - La estética como política [cap. de El malestar en la estética, que también tienes entero].md</t>
+          <t>Rancière - El reparto de lo sensible. Estética y política (2014) [Prometeo, trad. Mónica Padró, ISBN 9789875745797].md</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>n/d (texto teórico; referencia central a Schiller, 1795, y al arte contemporáneo)</t>
+          <t>n/d (texto teórico; genealogía de los regímenes del arte de la Antigüedad al presente)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro, 2011 (de «El malestar en la estética», Capital Intelectual; elaborado para un seminario en el MACBA, 2002)</t>
+          <t>Libro (entrevista-ensayo), 2014 (Prometeo, Buenos Aires; orig. «Le Partage du sensible», La Fabrique, 2000)</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Jacques Rancière; Friedrich Schiller; Immanuel Kant; Jean-François Lyotard; Barnett Newman; Thierry de Duve; Pierre Huyghe; Nicolas Bourriaud (arte relacional); Platón; Aristóteles; MACBA</t>
+          <t>Jacques Rancière; Mónica Padró (trad.); Marcelo G. Burello; María Beatriz Greco (estudio preliminar); Platón; Aristóteles; Friedrich Schiller; Prometeo Libros; La Fabrique</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Capítulo de «El malestar en la estética» que reconstruye la lógica de la relación «estética» entre arte y política ante el diagnóstico compartido del fin de la utopía estética. Rancière identifica dos concepciones «post-utópicas» del presente del arte: la de los filósofos, que aísla la radicalidad artística bajo el signo kantiano de lo sublime (sea como instauración de un ser-en-común, sea, con Lyotard, como testimonio negativo de lo impresentable), derivando en una comunidad ética que revoca la emancipación; y la de artistas e instituciones, que propone un arte modesto, relacional (Bourriaud, Huyghe), de microsituaciones que recrean lazos. Ambas, muestra, son fragmentos de una misma alianza rota entre radicalidad artística y política, y ambas reafirman una función comunitaria del arte. Su tesis: el arte no es político por sus mensajes ni por representar estructuras o conflictos sociales, sino por la distancia que toma respecto de sus funciones, por el tiempo y el espacio que instituye —por su modo de recortar el «reparto de lo sensible». La política, a su vez, no es ejercicio del poder sino configuración de un espacio de experiencia común y litigio sobre quién posee la palabra y no solo la voz. Mediante la lectura de la carta decimoquinta de Schiller sobre la «Juno Ludovisi» —la «apariencia libre» y el «libre juego» que suspenden el poder de la forma sobre la materia, del entendimiento sobre la sensibilidad—, Rancière funda la politicidad del arte en su autonomía misma, refutación sensible de la división entre dos humanidades.</t>
+          <t>En este texto seminal, estructurado como serie de respuestas a preguntas, Rancière expone la noción que articula su pensamiento estético-político: el «reparto de lo sensible», entendido como el sistema de evidencias sensibles que hace ver simultáneamente la existencia de un común y los recortes que definen los lugares y partes de cada quien. Todo reparto distribuye tiempos, espacios y formas de actividad, y determina quién tiene parte en lo común: el ciudadano aristotélico frente al esclavo que comprende pero no «posee» el lenguaje, o los artesanos platónicos que, por no tener tiempo, no pueden ocupar otro lugar que su trabajo. La política y el arte no son esferas separadas sino dos formas de división de lo sensible dependientes de regímenes de identificación. Rancière distingue tres regímenes del arte: el ético de las imágenes (Platón, donde el arte no se distingue como tal y se juzga por su verdad y sus efectos), el representativo o poético (la mímesis y su jerarquía de géneros) y el estético (que libera al arte de la regla mimética y lo define por un sensorium específico, singular y autónomo). Critica la noción de «modernidad» y de vanguardia como relatos empobrecidos del «fin» y el «retorno», y aborda la promoción estética de los anónimos por las artes mecánicas (fotografía, cine), los modos de la ficción frente a la historia, y la relación entre arte y trabajo. La estética emerge así como pensamiento de la igualdad y del disenso inscrito en las formas mismas de la experiencia sensible.</t>
         </is>
       </c>
     </row>
@@ -6092,27 +6092,27 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Richard - Fracturas de la memoria. Arte y pensamiento crítico (2007) [col. Arte y pensamiento dir. Andrea Giunta, Buenos Aires, ISBN 9789871220786].md</t>
+          <t>Rancière - La estética como política [cap. de El malestar en la estética, que también tienes entero].md</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Chile, 1973-2006 (dictadura de Pinochet, transición y globalización)</t>
+          <t>n/d (texto teórico; referencia central a Schiller, 1795, y al arte contemporáneo)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Libro (recopilación de ensayos), 2007</t>
+          <t>Capítulo de libro, 2011 (de «El malestar en la estética», Capital Intelectual; elaborado para un seminario en el MACBA, 2002)</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Nelly Richard; Andrea Giunta (dir. colección); Escena de Avanzada (Carlos Leppe, Eugenio Dittborn, Diamela Eltit, Raúl Zurita, Lotty Rosenfeld, CADA, Catalina Parra, Juan Dávila); Walter Benjamin; Michel Foucault; Jean Baudrillard; Fredric Jameson; Rosalind Krauss y Hal Foster (revista October); Siglo XXI Editores Argentina; revista Estudios Visuales</t>
+          <t>Jacques Rancière; Friedrich Schiller; Immanuel Kant; Jean-François Lyotard; Barnett Newman; Thierry de Duve; Pierre Huyghe; Nicolas Bourriaud (arte relacional); Platón; Aristóteles; MACBA</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>Compilación de ensayos de Nelly Richard, escritos entre 1987 y 2005, que traza un itinerario crítico sobre las relaciones entre arte, política y memoria en el Chile de la dictadura y la postdictadura. La tesis central sostiene que la Escena de Avanzada —surgida hacia 1977 bajo el régimen de Pinochet— reformuló el nexo arte/política desde un materialismo crítico de los signos, distanciándose tanto de la censura oficial como del realismo denunciante de la izquierda militante. Richard analiza prácticas neovanguardistas (CADA, Leppe, Dittborn, Rosenfeld, Eltit, Zurita) que trabajaron el cuerpo y la ciudad como soportes, la elipsis y la metáfora como tácticas frente a la censura, y el fragmento como poética de una temporalidad rota. El marco conceptual combina deconstrucción, la crítica benjaminiana de la Historia (discontinuidad, alegoría, aura) y referencias a Foucault, Baudrillard y Jameson. El libro se organiza en dos ejes: «Lo crítico y lo político en el arte» (márgenes e instituciones, ciencias sociales y poéticas de la crisis, régimen crítico-estético en la globalización, estudios visuales) y «Dramas y tramas de la memoria» (roturas y discontinuidades, la cita de la violencia, la captura de Pinochet en 1998, el contratiempo crítico de la memoria). Richard defiende un arte crítico que reintroduzca «peso» simbólico en la imaginería plana del capitalismo visual y resista la homogeneización mercantil. Su aporte es una crítica cultural latinoamericana que articula análisis sociopolítico, teoría estética y escritura, reivindicando la opacidad del significante contra el consenso neoliberal y sus poéticas de la transparencia.</t>
+          <t>Capítulo de «El malestar en la estética» que reconstruye la lógica de la relación «estética» entre arte y política ante el diagnóstico compartido del fin de la utopía estética. Rancière identifica dos concepciones «post-utópicas» del presente del arte: la de los filósofos, que aísla la radicalidad artística bajo el signo kantiano de lo sublime (sea como instauración de un ser-en-común, sea, con Lyotard, como testimonio negativo de lo impresentable), derivando en una comunidad ética que revoca la emancipación; y la de artistas e instituciones, que propone un arte modesto, relacional (Bourriaud, Huyghe), de microsituaciones que recrean lazos. Ambas, muestra, son fragmentos de una misma alianza rota entre radicalidad artística y política, y ambas reafirman una función comunitaria del arte. Su tesis: el arte no es político por sus mensajes ni por representar estructuras o conflictos sociales, sino por la distancia que toma respecto de sus funciones, por el tiempo y el espacio que instituye —por su modo de recortar el «reparto de lo sensible». La política, a su vez, no es ejercicio del poder sino configuración de un espacio de experiencia común y litigio sobre quién posee la palabra y no solo la voz. Mediante la lectura de la carta decimoquinta de Schiller sobre la «Juno Ludovisi» —la «apariencia libre» y el «libre juego» que suspenden el poder de la forma sobre la materia, del entendimiento sobre la sensibilidad—, Rancière funda la politicidad del arte en su autonomía misma, refutación sensible de la división entre dos humanidades.</t>
         </is>
       </c>
     </row>
@@ -6124,27 +6124,27 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Richard - La insubordinación de los signos. Cambio político, transformaciones culturales y poéticas de la crisis [Cuarto Propio, Santiago, ISBN 9789562600576].md</t>
+          <t>Richard - Fracturas de la memoria. Arte y pensamiento crítico (2007) [col. Arte y pensamiento dir. Andrea Giunta, Buenos Aires, ISBN 9789871220786].md</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Chile, 1973-1994 (dictadura y transición democrática)</t>
+          <t>Chile, 1973-2006 (dictadura de Pinochet, transición y globalización)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Libro (ensayo), 1994</t>
+          <t>Libro (recopilación de ensayos), 2007</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Nelly Richard; Germán Bravo, Martín Hopenhayn, Adriana Valdés (conversación final); Eugenio Dittborn; Diamela Eltit; Paz Errázuriz; Gonzalo Muñoz; Diego Maquieira; Walter Benjamin; José Joaquín Brunner; Editorial Cuarto Propio (Serie Debates), Santiago</t>
+          <t>Nelly Richard; Andrea Giunta (dir. colección); Escena de Avanzada (Carlos Leppe, Eugenio Dittborn, Diamela Eltit, Raúl Zurita, Lotty Rosenfeld, CADA, Catalina Parra, Juan Dávila); Walter Benjamin; Michel Foucault; Jean Baudrillard; Fredric Jameson; Rosalind Krauss y Hal Foster (revista October); Siglo XXI Editores Argentina; revista Estudios Visuales</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>Ensayo seminal de Nelly Richard (Editorial Cuarto Propio, Santiago, 1994) que inaugura la «Serie Debates» y analiza las transformaciones culturales del Chile de la dictadura y la transición democrática. Su tesis: frente al quiebre de 1973, ciertas prácticas artístico-literarias —la «nueva escena» o Escena de Avanzada— insubordinaron los signos, rechazando tanto la lengua oficial del poder como el molde ideológico del arte militante y el racionalismo de las ciencias sociales. El objeto de estudio son obras de Eugenio Dittborn, Diamela Eltit, Paz Errázuriz, Gonzalo Muñoz, Diego Maquieira y otros, leídas desde un marco benjaminiano (memoria, discontinuidad, alegoría, reproductibilidad técnica, la fotografía como delación). Richard articula conceptos clave: «poéticas de la crisis», arte refractario, estéticas del desecho, des-identidad, y la crítica a la Historia como continuidad de los opresores frente a la discontinuidad de los oprimidos. Los capítulos recorren memoria y roturas; la cita limítrofe entre neovanguardia y postvanguardia; destrucción, reconstrucción y desconstrucción; las ciencias sociales; y el escenario democrático y la política de las diferencias, donde examina la paradoja de la transición: la energía crítica se subsume en la negociación consensual y el intelectual se institucionaliza. El libro cierra con una conversación entre Germán Bravo, Martín Hopenhayn, Nelly Richard y Adriana Valdés. Su aporte es fundar una crítica cultural que valoriza la cultura como escenario de mediaciones simbólicas, resistente a la transparencia comunicativa del consenso neoliberal, y que rescata la opacidad, el fragmento y la ambigüedad como formas de memoria disidente y de subjetivación crítica.</t>
+          <t>Compilación de ensayos de Nelly Richard, escritos entre 1987 y 2005, que traza un itinerario crítico sobre las relaciones entre arte, política y memoria en el Chile de la dictadura y la postdictadura. La tesis central sostiene que la Escena de Avanzada —surgida hacia 1977 bajo el régimen de Pinochet— reformuló el nexo arte/política desde un materialismo crítico de los signos, distanciándose tanto de la censura oficial como del realismo denunciante de la izquierda militante. Richard analiza prácticas neovanguardistas (CADA, Leppe, Dittborn, Rosenfeld, Eltit, Zurita) que trabajaron el cuerpo y la ciudad como soportes, la elipsis y la metáfora como tácticas frente a la censura, y el fragmento como poética de una temporalidad rota. El marco conceptual combina deconstrucción, la crítica benjaminiana de la Historia (discontinuidad, alegoría, aura) y referencias a Foucault, Baudrillard y Jameson. El libro se organiza en dos ejes: «Lo crítico y lo político en el arte» (márgenes e instituciones, ciencias sociales y poéticas de la crisis, régimen crítico-estético en la globalización, estudios visuales) y «Dramas y tramas de la memoria» (roturas y discontinuidades, la cita de la violencia, la captura de Pinochet en 1998, el contratiempo crítico de la memoria). Richard defiende un arte crítico que reintroduzca «peso» simbólico en la imaginería plana del capitalismo visual y resista la homogeneización mercantil. Su aporte es una crítica cultural latinoamericana que articula análisis sociopolítico, teoría estética y escritura, reivindicando la opacidad del significante contra el consenso neoliberal y sus poéticas de la transparencia.</t>
         </is>
       </c>
     </row>
@@ -6156,27 +6156,27 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Sansi (ed.) - The Anthropologist as Curator (2019) [Bloomsbury Academic, ISBN 9781350081901].md</t>
+          <t>Richard - La insubordinación de los signos. Cambio político, transformaciones culturales y poéticas de la crisis [Cuarto Propio, Santiago, ISBN 9789562600576].md</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>n/d (arte contemporáneo y giro curatorial, ca. 1990-2018)</t>
+          <t>Chile, 1973-1994 (dictadura y transición democrática)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Libro editado (volumen colectivo), 2019</t>
+          <t>Libro (ensayo), 1994</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Roger Sansi (ed.); Tarek Elhaik; George Marcus; Jonas Tinius; Sharon Macdonald; Silvia Forni; Ivan Bargna; Ethnographic Terminalia; Jennifer Clarke; Rafael Schacter; Alex Flynn; Okwui Enwezor; Hal Foster; Hans-Ulrich Obrist; Irit Rogoff; Bloomsbury Academic; EASA / Pirelli HangarBicocca</t>
+          <t>Nelly Richard; Germán Bravo, Martín Hopenhayn, Adriana Valdés (conversación final); Eugenio Dittborn; Diamela Eltit; Paz Errázuriz; Gonzalo Muñoz; Diego Maquieira; Walter Benjamin; José Joaquín Brunner; Editorial Cuarto Propio (Serie Debates), Santiago</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Volumen colectivo editado por Roger Sansi (Bloomsbury Academic, 2019) que examina la figura del «antropólogo como curador» y, recíprocamente, del curador como etnógrafo. Partiendo del ensayo de Hal Foster sobre el «giro etnográfico» y de la analogía de Okwui Enwezor entre viaje curatorial y trabajo de campo, el libro sostiene que la curaduría se ha vuelto un término omniabarcante en la era del capitalismo cognitivo, y pregunta qué puede aprender la antropología de esa expansión sin diluir su especificidad. La introducción de Sansi mapea la curaduría participativa, el «laboratorio curatorial» (Obrist, Latour, prototipos), y propuestas como el «assemblage-work» y la «para-site» de Marcus o el «conceptualismo etnográfico» de Ssorin-Chaikov. Los capítulos reúnen antropólogos con experiencia curatorial: Elhaik y Marcus debaten la curaduría como posible «tercer método» antropológico tras el comparativo y el etnográfico; Tinius y Macdonald elaboran la «recursividad» del par arte/antropología; Forni y Bargna reflexionan desde museos etnográficos africanos y el debate sobre descolonización y representación; Ethnographic Terminalia describe sus exposiciones como prototipos; Winter y Clarke escriben desde «Knowing from the Inside» (Ingold) y proponen una «ecología de prácticas» (Stengers); Schacter, Flynn, Theunissen, Favero y Lobley extienden lo curatorial al arte urbano, la expografía, lo digital y el sonido. El marco conceptual gira en torno a la mediación, la experimentación, la infraestructura del trabajo y una ontología relacional. El aporte del libro no es proclamar un nuevo «giro», sino describir etnográficamente los procesos, restricciones y anécdotas de la labor curatorial para repensar qué es hoy el trabajo antropológico.</t>
+          <t>Ensayo seminal de Nelly Richard (Editorial Cuarto Propio, Santiago, 1994) que inaugura la «Serie Debates» y analiza las transformaciones culturales del Chile de la dictadura y la transición democrática. Su tesis: frente al quiebre de 1973, ciertas prácticas artístico-literarias —la «nueva escena» o Escena de Avanzada— insubordinaron los signos, rechazando tanto la lengua oficial del poder como el molde ideológico del arte militante y el racionalismo de las ciencias sociales. El objeto de estudio son obras de Eugenio Dittborn, Diamela Eltit, Paz Errázuriz, Gonzalo Muñoz, Diego Maquieira y otros, leídas desde un marco benjaminiano (memoria, discontinuidad, alegoría, reproductibilidad técnica, la fotografía como delación). Richard articula conceptos clave: «poéticas de la crisis», arte refractario, estéticas del desecho, des-identidad, y la crítica a la Historia como continuidad de los opresores frente a la discontinuidad de los oprimidos. Los capítulos recorren memoria y roturas; la cita limítrofe entre neovanguardia y postvanguardia; destrucción, reconstrucción y desconstrucción; las ciencias sociales; y el escenario democrático y la política de las diferencias, donde examina la paradoja de la transición: la energía crítica se subsume en la negociación consensual y el intelectual se institucionaliza. El libro cierra con una conversación entre Germán Bravo, Martín Hopenhayn, Nelly Richard y Adriana Valdés. Su aporte es fundar una crítica cultural que valoriza la cultura como escenario de mediaciones simbólicas, resistente a la transparencia comunicativa del consenso neoliberal, y que rescata la opacidad, el fragmento y la ambigüedad como formas de memoria disidente y de subjetivación crítica.</t>
         </is>
       </c>
     </row>
@@ -6188,27 +6188,27 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Sansi - Art, Anthropology and the Gift (2015) [Bloomsbury Academic, ISBN 9780857857811].md</t>
+          <t>Sansi (ed.) - The Anthropologist as Curator (2019) [Bloomsbury Academic, ISBN 9781350081901].md</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>n/d (arte contemporáneo y antropología, ca. 1990-2013)</t>
+          <t>n/d (arte contemporáneo y giro curatorial, ca. 1990-2018)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Libro (monografía), 2015</t>
+          <t>Libro editado (volumen colectivo), 2019</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Roger Sansi; Marcel Mauss; Marilyn Strathern; Alfred Gell; Nicolas Bourriaud; Hal Foster; Claire Bishop; Rirkrit Tiravanija; Félix González-Torres; Santiago Sierra; George Marcus; Goldsmiths / Bloomsbury Academic</t>
+          <t>Roger Sansi (ed.); Tarek Elhaik; George Marcus; Jonas Tinius; Sharon Macdonald; Silvia Forni; Ivan Bargna; Ethnographic Terminalia; Jennifer Clarke; Rafael Schacter; Alex Flynn; Okwui Enwezor; Hal Foster; Hans-Ulrich Obrist; Irit Rogoff; Bloomsbury Academic; EASA / Pirelli HangarBicocca</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Monografía de Roger Sansi (Bloomsbury Academic, 2015) que examina las «afinidades profundas» entre arte contemporáneo y antropología más allá del uso compartido de métodos etnográficos. Su tesis: el «giro social» del arte —prácticas de social practice, arte relacional, colaborativo y contextual desde los años noventa— reactiva conceptos antropológicos clásicos, en particular el don de Mauss («on se donne en donnant»). Sansi articula la «persona partible» de Marilyn Strathern y la «persona distribuida» y las «trampas de agencia» de Alfred Gell para analizar obras de Félix González-Torres, Rirkrit Tiravanija y Santiago Sierra, mostrando cómo el arte no solo representa sino que hace: produce relaciones, situaciones y acontecimientos. El libro discute críticamente la «estética relacional» de Bourriaud (y sus objeciones desde Bishop y Kester), distinguiendo la relación estética de la relación antropológica. Los capítulos recorren el arte como antropología; trampas y dispositivos; estética y política; participación y don; trabajo y vida; campos y laboratorios; y etnografía y utopía. El marco conceptual combina la teoría del don, las ontologías relacionales, la crítica institucional paralela en ambas disciplinas (la «crisis de la representación» de Marcus y Fischer) y una lectura de la participación que no celebra ingenuamente la igualdad, sino que atiende a la jerarquía, el poder y la ambigüedad. El aporte de Sansi es desplazar el debate desde la representación (identidad, alteridad, el «ethnographer's envy» de Foster) hacia la práctica social y la agencia: entender el arte contemporáneo como un laboratorio experimental de las formas mínimas de la vida cotidiana y del intercambio, y repensar desde ahí la propia labor de la antropología.</t>
+          <t>Volumen colectivo editado por Roger Sansi (Bloomsbury Academic, 2019) que examina la figura del «antropólogo como curador» y, recíprocamente, del curador como etnógrafo. Partiendo del ensayo de Hal Foster sobre el «giro etnográfico» y de la analogía de Okwui Enwezor entre viaje curatorial y trabajo de campo, el libro sostiene que la curaduría se ha vuelto un término omniabarcante en la era del capitalismo cognitivo, y pregunta qué puede aprender la antropología de esa expansión sin diluir su especificidad. La introducción de Sansi mapea la curaduría participativa, el «laboratorio curatorial» (Obrist, Latour, prototipos), y propuestas como el «assemblage-work» y la «para-site» de Marcus o el «conceptualismo etnográfico» de Ssorin-Chaikov. Los capítulos reúnen antropólogos con experiencia curatorial: Elhaik y Marcus debaten la curaduría como posible «tercer método» antropológico tras el comparativo y el etnográfico; Tinius y Macdonald elaboran la «recursividad» del par arte/antropología; Forni y Bargna reflexionan desde museos etnográficos africanos y el debate sobre descolonización y representación; Ethnographic Terminalia describe sus exposiciones como prototipos; Winter y Clarke escriben desde «Knowing from the Inside» (Ingold) y proponen una «ecología de prácticas» (Stengers); Schacter, Flynn, Theunissen, Favero y Lobley extienden lo curatorial al arte urbano, la expografía, lo digital y el sonido. El marco conceptual gira en torno a la mediación, la experimentación, la infraestructura del trabajo y una ontología relacional. El aporte del libro no es proclamar un nuevo «giro», sino describir etnográficamente los procesos, restricciones y anécdotas de la labor curatorial para repensar qué es hoy el trabajo antropológico.</t>
         </is>
       </c>
     </row>
@@ -6220,27 +6220,27 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Sansi - Introduction. Anthropology and Curation through the Looking Glass (2019) [The Anthropologist as Curator, que también tienes entero].md</t>
+          <t>Sansi - Art, Anthropology and the Gift (2015) [Bloomsbury Academic, ISBN 9780857857811].md</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>n/d (arte contemporáneo y curaduría, ca. 1990-2018)</t>
+          <t>n/d (arte contemporáneo y antropología, ca. 1990-2013)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro (introducción), 2019</t>
+          <t>Libro (monografía), 2015</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Roger Sansi; Okwui Enwezor; Hal Foster; Hans-Ulrich Obrist; Tarek Elhaik; George Marcus; Nikolai Ssorin-Chaikov; Irit Rogoff; Carolyn Christov-Bakargiev; Bruno Latour; Bloomsbury Academic</t>
+          <t>Roger Sansi; Marcel Mauss; Marilyn Strathern; Alfred Gell; Nicolas Bourriaud; Hal Foster; Claire Bishop; Rirkrit Tiravanija; Félix González-Torres; Santiago Sierra; George Marcus; Goldsmiths / Bloomsbury Academic</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Capítulo introductorio de Roger Sansi al volumen colectivo «The Anthropologist as Curator» (Bloomsbury, 2019/2020), titulado «Anthropology and curation through the looking glass». Plantea que, mientras la relación entre arte y antropología —abierta por el ensayo de Hal Foster (1995)— ha sido ampliamente discutida, la del «antropólogo como curador» apenas se ha explorado, pese a la creciente preeminencia del curador en el mundo del arte y a que muchos antropólogos han organizado exposiciones. Sansi invierte primero la pregunta («el curador como etnógrafo») a partir de la analogía de Okwui Enwezor entre el trabajo de campo curatorial y la errancia etnográfica en un mundo de desplazamientos y proximidades conflictivas. Traza luego los efectos del «giro etnográfico»: la globalización del arte contemporáneo, la «descolonización» como consigna, la curaduría participativa (Obrist, «Do it»), los enfoques duracionales y el «laboratorio curatorial» (Basu y Macdonald, Latour). Introduce conceptos clave —montaje (Enwezor), assemblage-work y para-site (Rabinow, Marcus), conceptualismo etnográfico (Ssorin-Chaikov), el «campo expandido» de lo curatorial (Rogoff), el curador como «trabajador emblemático de la era cognitiva» (Christov-Bakargiev, Boltanski y Chiapello)— y presenta los capítulos del libro. Su posición evita proclamar un «giro curatorial» o defender la pureza disciplinar por «desapego»; propone, en cambio, describir etnográficamente la experiencia, las infraestructuras y las anécdotas del trabajo curatorial. El aporte es replantear qué ha llegado a ser la labor de la antropología en una sociedad «relacional», y advertir sobre un tercer agente: las infraestructuras digitales que se autocuran mediante algoritmos.</t>
+          <t>Monografía de Roger Sansi (Bloomsbury Academic, 2015) que examina las «afinidades profundas» entre arte contemporáneo y antropología más allá del uso compartido de métodos etnográficos. Su tesis: el «giro social» del arte —prácticas de social practice, arte relacional, colaborativo y contextual desde los años noventa— reactiva conceptos antropológicos clásicos, en particular el don de Mauss («on se donne en donnant»). Sansi articula la «persona partible» de Marilyn Strathern y la «persona distribuida» y las «trampas de agencia» de Alfred Gell para analizar obras de Félix González-Torres, Rirkrit Tiravanija y Santiago Sierra, mostrando cómo el arte no solo representa sino que hace: produce relaciones, situaciones y acontecimientos. El libro discute críticamente la «estética relacional» de Bourriaud (y sus objeciones desde Bishop y Kester), distinguiendo la relación estética de la relación antropológica. Los capítulos recorren el arte como antropología; trampas y dispositivos; estética y política; participación y don; trabajo y vida; campos y laboratorios; y etnografía y utopía. El marco conceptual combina la teoría del don, las ontologías relacionales, la crítica institucional paralela en ambas disciplinas (la «crisis de la representación» de Marcus y Fischer) y una lectura de la participación que no celebra ingenuamente la igualdad, sino que atiende a la jerarquía, el poder y la ambigüedad. El aporte de Sansi es desplazar el debate desde la representación (identidad, alteridad, el «ethnographer's envy» de Foster) hacia la práctica social y la agencia: entender el arte contemporáneo como un laboratorio experimental de las formas mínimas de la vida cotidiana y del intercambio, y repensar desde ahí la propia labor de la antropología.</t>
         </is>
       </c>
     </row>
@@ -6252,27 +6252,27 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Schneider y Wright (eds.) - Anthropology and Art Practice (2013) [Bloomsbury Academic].md</t>
+          <t>Sansi - Introduction. Anthropology and Curation through the Looking Glass (2019) [The Anthropologist as Curator, que también tienes entero].md</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>n/d (arte contemporáneo y antropología, ca. 1990-2013)</t>
+          <t>n/d (arte contemporáneo y curaduría, ca. 1990-2018)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Libro editado (volumen colectivo), 2013</t>
+          <t>Capítulo de libro (introducción), 2019</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Arnd Schneider y Christopher Wright (eds.); Pia Arke; Franz Ackermann; Fiamma Montezemolo; Anthony Luvera; Rupert Cox y Angus Carlyle; Craig Campbell; Jennifer Deger; Caterina Pasqualino; Okwui Enwezor; Hal Foster; Alfred Gell; Marc Augé; Bloomsbury Academic / Goldsmiths / University of Oslo</t>
+          <t>Roger Sansi; Okwui Enwezor; Hal Foster; Hans-Ulrich Obrist; Tarek Elhaik; George Marcus; Nikolai Ssorin-Chaikov; Irit Rogoff; Carolyn Christov-Bakargiev; Bruno Latour; Bloomsbury Academic</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Volumen colectivo editado por Arnd Schneider y Christopher Wright (Bloomsbury Academic, 2013), tercero de una trilogía tras «Contemporary Art and Anthropology» (2006) y «Between Art and Anthropology» (2010). Su tesis: el foco debe desplazarse hacia «las maneras de trabajar» (ways of working) de artistas y antropólogos, entendiendo la creatividad y el significado como emergentes —no prefigurados— y situando la teoría dentro del hacer y no fuera de él. El objeto son prácticas y colaboraciones que difuminan las fronteras entre arte contemporáneo y etnografía: procesos abiertos, fragmentarios y de larga duración donde el trabajo con personas y materiales importa tanto o más que el producto final. La introducción, «Ways of Working», articula el argumento mediante casos como Pia Arke (fotografía, colonialidad y la «condición mestiza» en Groenlandia), Franz Ackermann (mapas mentales y no-lugares de la supermodernidad, Augé), Fiamma Montezemolo (frontera México-EE.UU., biocartografía) y Anthony Luvera (trabajo prolongado con personas sin hogar). El marco conceptual dialoga con Foster, Enwezor («Intense Proximity»), Gell (materialidad, relacionalidad, personhood) y la genealogía surrealista de «Documents». El libro adopta un formato deliberadamente heterogéneo —ensayos breves, conversaciones y relatos de artistas en primera persona (Campbell, Orrantia, Mjaaland, Lammer, Ramey, Deger, Ortega Ayala, Cox y Carlyle, Pasqualino)— que performa la propia colaboración interdisciplinaria que estudia. Su aporte es reclamar un compromiso entre las prácticas artísticas y la teoría antropológica actual (materialidad, sensorialidad, colaboración) capaz de renovar ambos campos, superando la mera yuxtaposición disciplinaria y proponiendo la co-autoría y la incertidumbre epistemológica como métodos productivos.</t>
+          <t>Capítulo introductorio de Roger Sansi al volumen colectivo «The Anthropologist as Curator» (Bloomsbury, 2019/2020), titulado «Anthropology and curation through the looking glass». Plantea que, mientras la relación entre arte y antropología —abierta por el ensayo de Hal Foster (1995)— ha sido ampliamente discutida, la del «antropólogo como curador» apenas se ha explorado, pese a la creciente preeminencia del curador en el mundo del arte y a que muchos antropólogos han organizado exposiciones. Sansi invierte primero la pregunta («el curador como etnógrafo») a partir de la analogía de Okwui Enwezor entre el trabajo de campo curatorial y la errancia etnográfica en un mundo de desplazamientos y proximidades conflictivas. Traza luego los efectos del «giro etnográfico»: la globalización del arte contemporáneo, la «descolonización» como consigna, la curaduría participativa (Obrist, «Do it»), los enfoques duracionales y el «laboratorio curatorial» (Basu y Macdonald, Latour). Introduce conceptos clave —montaje (Enwezor), assemblage-work y para-site (Rabinow, Marcus), conceptualismo etnográfico (Ssorin-Chaikov), el «campo expandido» de lo curatorial (Rogoff), el curador como «trabajador emblemático de la era cognitiva» (Christov-Bakargiev, Boltanski y Chiapello)— y presenta los capítulos del libro. Su posición evita proclamar un «giro curatorial» o defender la pureza disciplinar por «desapego»; propone, en cambio, describir etnográficamente la experiencia, las infraestructuras y las anécdotas del trabajo curatorial. El aporte es replantear qué ha llegado a ser la labor de la antropología en una sociedad «relacional», y advertir sobre un tercer agente: las infraestructuras digitales que se autocuran mediante algoritmos.</t>
         </is>
       </c>
     </row>
@@ -6284,27 +6284,27 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Schneider y Wright (eds.) - Between Art and Anthropology. Contemporary Ethnographic Practice (2010).md</t>
+          <t>Schneider y Wright (eds.) - Anthropology and Art Practice (2013) [Bloomsbury Academic].md</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Prácticas artísticas y etnográficas contemporáneas, ca. 1960-2010</t>
+          <t>n/d (arte contemporáneo y antropología, ca. 1990-2013)</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Libro (volumen colectivo editado), 2010</t>
+          <t>Libro editado (volumen colectivo), 2013</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Arnd Schneider; Christopher Wright; Lucy R. Lippard; George E. Marcus; Steven Feld; Virginia Ryan; Anna Grimshaw; Amanda Ravetz; Tim Ingold; Alfred Gell; Nicolas Bourriaud; Berg Publishers / conferencia Fieldworks (Tate Modern, 2003)</t>
+          <t>Arnd Schneider y Christopher Wright (eds.); Pia Arke; Franz Ackermann; Fiamma Montezemolo; Anthony Luvera; Rupert Cox y Angus Carlyle; Craig Campbell; Jennifer Deger; Caterina Pasqualino; Okwui Enwezor; Hal Foster; Alfred Gell; Marc Augé; Bloomsbury Academic / Goldsmiths / University of Oslo</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Volumen colectivo, derivado de la conferencia «Fieldworks: Dialogues between Art and Anthropology» (Tate Modern, 2003), que cartografía las «inter-zonas» productivas entre el arte contemporáneo y la antropología. En su extensa introducción, Schneider y Wright sostienen que ambos campos comparten el impulso de documentar la cultura, pero que la antropología ha cultivado una persistente «iconofobia» y un conservadurismo textualista que relegan la experimentación formal y sensorial al margen de lo que cuenta como investigación legítima. La tesis central es doble: reclamar una práctica antropológica «con» artistas (no meramente «sobre» artistas) y una práctica artística con antropólogos, tratando la diferencia disciplinar (epistemológica, ética, cognitiva) no como obstáculo sino como «irritante productivo». El marco conceptual articula el giro etnográfico en el arte y el giro hacia el arte en la antropología, apoyándose en la estética relacional de Bourriaud, la teoría de la agencia de Gell, la antropología de los sentidos, la fenomenología de la percepción y la ecología perceptual de Ingold, así como en la noción de apropiación de Schneider. Se examinan la experimentación en el trabajo de campo, el cine estructuralista y multipantalla, la etnografía panóptica de Griaule, el montaje, la materialidad y los «materiales inteligentes», el olfato como medio de investigación y las políticas de exhibición y del «circuito de bienales». Los capítulos de Lippard, Marcus, Feld/Ryan, Grimshaw/Owen/Ravetz, Salmond/Raymond, Perkins, Wynne, entre otros, ilustran colaboraciones concretas. El aporte del libro es programático: legitimar formas experimentales, sensoriales y colaborativas de producir y presentar conocimiento etnográfico, ampliando el repertorio de la antropología visual hacia una antropología audiovisual y sensorial.</t>
+          <t>Volumen colectivo editado por Arnd Schneider y Christopher Wright (Bloomsbury Academic, 2013), tercero de una trilogía tras «Contemporary Art and Anthropology» (2006) y «Between Art and Anthropology» (2010). Su tesis: el foco debe desplazarse hacia «las maneras de trabajar» (ways of working) de artistas y antropólogos, entendiendo la creatividad y el significado como emergentes —no prefigurados— y situando la teoría dentro del hacer y no fuera de él. El objeto son prácticas y colaboraciones que difuminan las fronteras entre arte contemporáneo y etnografía: procesos abiertos, fragmentarios y de larga duración donde el trabajo con personas y materiales importa tanto o más que el producto final. La introducción, «Ways of Working», articula el argumento mediante casos como Pia Arke (fotografía, colonialidad y la «condición mestiza» en Groenlandia), Franz Ackermann (mapas mentales y no-lugares de la supermodernidad, Augé), Fiamma Montezemolo (frontera México-EE.UU., biocartografía) y Anthony Luvera (trabajo prolongado con personas sin hogar). El marco conceptual dialoga con Foster, Enwezor («Intense Proximity»), Gell (materialidad, relacionalidad, personhood) y la genealogía surrealista de «Documents». El libro adopta un formato deliberadamente heterogéneo —ensayos breves, conversaciones y relatos de artistas en primera persona (Campbell, Orrantia, Mjaaland, Lammer, Ramey, Deger, Ortega Ayala, Cox y Carlyle, Pasqualino)— que performa la propia colaboración interdisciplinaria que estudia. Su aporte es reclamar un compromiso entre las prácticas artísticas y la teoría antropológica actual (materialidad, sensorialidad, colaboración) capaz de renovar ambos campos, superando la mera yuxtaposición disciplinaria y proponiendo la co-autoría y la incertidumbre epistemológica como métodos productivos.</t>
         </is>
       </c>
     </row>
@@ -6316,27 +6316,27 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Sedgwick - Paranoid Reading and Reparative Reading, or, You're So Paranoid, You Probably Think This Essay Is About You [Touching Feeling, cap. 4].md</t>
+          <t>Schneider y Wright (eds.) - Between Art and Anthropology. Contemporary Ethnographic Practice (2010).md</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>Prácticas artísticas y etnográficas contemporáneas, ca. 1960-2010</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro, 2003 (Touching Feeling, Duke University Press)</t>
+          <t>Libro (volumen colectivo editado), 2010</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Eve Kosofsky Sedgwick; Cindy Patton; Paul Ricoeur; Sigmund Freud; Melanie Klein; Silvan Tomkins; Judith Butler; D. A. Miller; Guy Hocquenghem; Leo Bersani; Michel Foucault; Richard Hofstadter</t>
+          <t>Arnd Schneider; Christopher Wright; Lucy R. Lippard; George E. Marcus; Steven Feld; Virginia Ryan; Anna Grimshaw; Amanda Ravetz; Tim Ingold; Alfred Gell; Nicolas Bourriaud; Berg Publishers / conferencia Fieldworks (Tate Modern, 2003)</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Ensayo seminal que interroga la hegemonía de la «hermenéutica de la sospecha» (Ricoeur, a partir de Marx, Nietzsche y Freud) en la teoría crítica, la teoría queer y feminista contemporáneas. Sedgwick argumenta que la sospecha y la paranoia, de descripción taxonómica, han devenido un imperativo metodológico casi obligatorio, confundido con la crítica misma. Su tesis no es refutar la verdad de las lecturas paranoides, sino desnaturalizar su condición de único modo legítimo de conocer, desplazando la pregunta de si un saber es verdadero hacia qué hace el saber: cómo es performativo. Caracteriza la lectura paranoide mediante cinco rasgos: es anticipatoria (no debe haber malas sorpresas), reflexiva y mimética, una «teoría fuerte» (Tomkins) de reducción totalizante, una teoría de los afectos negativos, y deposita una fe desmedida en la exposición y el desvelamiento. Frente a ella, recuperando el concepto de «posiciones» de Melanie Klein (esquizo-paranoide frente a depresiva) y la teoría del afecto de Tomkins, propone la lectura reparativa: aditiva, acretiva, abierta a la sorpresa, la esperanza y el placer, orientada a ensamblar objetos parciales en totalidades que nutran al self. Analiza críticamente Gender Trouble de Butler y The Novel and the Police de D. A. Miller como ejemplos de teoría fuerte paranoide, y muestra la datación histórica de la fe en la exposición en un contexto de violencia hipervisible y cinismo generalizado (Sloterdijk). El aporte: pluralizar las prácticas de conocimiento, revalorizar el camp y las intertextualidades queer como prácticas reparativas, y ligar temporalidad, afecto y contingencia.</t>
+          <t>Volumen colectivo, derivado de la conferencia «Fieldworks: Dialogues between Art and Anthropology» (Tate Modern, 2003), que cartografía las «inter-zonas» productivas entre el arte contemporáneo y la antropología. En su extensa introducción, Schneider y Wright sostienen que ambos campos comparten el impulso de documentar la cultura, pero que la antropología ha cultivado una persistente «iconofobia» y un conservadurismo textualista que relegan la experimentación formal y sensorial al margen de lo que cuenta como investigación legítima. La tesis central es doble: reclamar una práctica antropológica «con» artistas (no meramente «sobre» artistas) y una práctica artística con antropólogos, tratando la diferencia disciplinar (epistemológica, ética, cognitiva) no como obstáculo sino como «irritante productivo». El marco conceptual articula el giro etnográfico en el arte y el giro hacia el arte en la antropología, apoyándose en la estética relacional de Bourriaud, la teoría de la agencia de Gell, la antropología de los sentidos, la fenomenología de la percepción y la ecología perceptual de Ingold, así como en la noción de apropiación de Schneider. Se examinan la experimentación en el trabajo de campo, el cine estructuralista y multipantalla, la etnografía panóptica de Griaule, el montaje, la materialidad y los «materiales inteligentes», el olfato como medio de investigación y las políticas de exhibición y del «circuito de bienales». Los capítulos de Lippard, Marcus, Feld/Ryan, Grimshaw/Owen/Ravetz, Salmond/Raymond, Perkins, Wynne, entre otros, ilustran colaboraciones concretas. El aporte del libro es programático: legitimar formas experimentales, sensoriales y colaborativas de producir y presentar conocimiento etnográfico, ampliando el repertorio de la antropología visual hacia una antropología audiovisual y sensorial.</t>
         </is>
       </c>
     </row>
@@ -6348,7 +6348,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Star - The Ethnography of Infrastructure (1999) [American Behavioral Scientist 43(3), pp. 377-391].md</t>
+          <t>Sedgwick - Paranoid Reading and Reparative Reading, or, You're So Paranoid, You Probably Think This Essay Is About You [Touching Feeling, cap. 4].md</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -6358,17 +6358,17 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico, 1999 (American Behavioral Scientist 43(3))</t>
+          <t>Capítulo de libro, 2003 (Touching Feeling, Duke University Press)</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Susan Leigh Star; Geoffrey C. Bowker; Anselm Strauss; Gregory Bateson; Howard Becker; Bruno Latour; Langdon Winner; Karen Ruhleder; American Behavioral Scientist / Sage</t>
+          <t>Eve Kosofsky Sedgwick; Cindy Patton; Paul Ricoeur; Sigmund Freud; Melanie Klein; Silvan Tomkins; Judith Butler; D. A. Miller; Guy Hocquenghem; Leo Bersani; Michel Foucault; Richard Hofstadter</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Artículo metodológico que propone estudiar la infraestructura como objeto etnográfico, formulado como un «llamado a estudiar cosas aburridas»: enchufes, estándares, formularios, clasificaciones y protocolos que subyacen invisiblemente al trabajo. Star sostiene que la infraestructura no es una cosa sino una propiedad fundamentalmente relacional y ecológica: es infraestructura solo en relación con prácticas organizadas («cuándo», no «qué», es una infraestructura); lo que para uno es sustrato transparente, para otro es tópico o barrera (el ejemplo de la escalera y la persona en silla de ruedas). Define nueve dimensiones: encaje (embeddedness), transparencia, alcance espacio-temporal, aprendizaje como parte de la membresía, vínculo con convenciones de práctica, encarnación de estándares, construcción sobre una base instalada, visibilidad ante el fallo y reparación modular. El marco proviene del interaccionismo simbólico (Strauss), los estudios sociales de la ciencia y la «inversión infraestructural» de Bowker, que lleva al primer plano lo que suele quedar de trasfondo. Metodológicamente combina análisis histórico y literario, entrevistas, observación, análisis de sistemas y estudios de usabilidad, y ofrece «trucos del oficio»: identificar narrativas maestras y sus «otros» silenciados, hacer visible el trabajo invisible y de articulación, atender a las paradojas (transparente/opaco) y precisar el estatus epistemológico de los indicadores (artefacto material, huella o representación verídica). Aborda además el problema de escala en la etnografía de sistemas distribuidos y la política inscrita en el diseño (Winner, los puentes de Moses, categorías raciales del censo). Su aporte: fundar una ética y una justicia distributiva de la infraestructura informacional.</t>
+          <t>Ensayo seminal que interroga la hegemonía de la «hermenéutica de la sospecha» (Ricoeur, a partir de Marx, Nietzsche y Freud) en la teoría crítica, la teoría queer y feminista contemporáneas. Sedgwick argumenta que la sospecha y la paranoia, de descripción taxonómica, han devenido un imperativo metodológico casi obligatorio, confundido con la crítica misma. Su tesis no es refutar la verdad de las lecturas paranoides, sino desnaturalizar su condición de único modo legítimo de conocer, desplazando la pregunta de si un saber es verdadero hacia qué hace el saber: cómo es performativo. Caracteriza la lectura paranoide mediante cinco rasgos: es anticipatoria (no debe haber malas sorpresas), reflexiva y mimética, una «teoría fuerte» (Tomkins) de reducción totalizante, una teoría de los afectos negativos, y deposita una fe desmedida en la exposición y el desvelamiento. Frente a ella, recuperando el concepto de «posiciones» de Melanie Klein (esquizo-paranoide frente a depresiva) y la teoría del afecto de Tomkins, propone la lectura reparativa: aditiva, acretiva, abierta a la sorpresa, la esperanza y el placer, orientada a ensamblar objetos parciales en totalidades que nutran al self. Analiza críticamente Gender Trouble de Butler y The Novel and the Police de D. A. Miller como ejemplos de teoría fuerte paranoide, y muestra la datación histórica de la fe en la exposición en un contexto de violencia hipervisible y cinismo generalizado (Sloterdijk). El aporte: pluralizar las prácticas de conocimiento, revalorizar el camp y las intertextualidades queer como prácticas reparativas, y ligar temporalidad, afecto y contingencia.</t>
         </is>
       </c>
     </row>
@@ -6380,27 +6380,27 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Star y Ruhleder - Steps Toward an Ecology of Infrastructure. Design and Access for Large Information Spaces (1996) [Information Systems Research 7(1), desde p. 111].md</t>
+          <t>Star - The Ethnography of Infrastructure (1999) [American Behavioral Scientist 43(3), pp. 377-391].md</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>1991-1994 (estudio del Worm Community System)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico, 1996 (Information Systems Research 7(1))</t>
+          <t>Artículo académico, 1999 (American Behavioral Scientist 43(3))</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Susan Leigh Star; Karen Ruhleder; Gregory Bateson; Bruce Schatz; Yrjö Engeström; Geoffrey Bowker; Bruno Latour; Information Systems Research / INFORMS</t>
+          <t>Susan Leigh Star; Geoffrey C. Bowker; Anselm Strauss; Gregory Bateson; Howard Becker; Bruno Latour; Langdon Winner; Karen Ruhleder; American Behavioral Scientist / Sage</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Estudio empírico y teórico basado en tres años de etnografía (1991-1994) sobre el Worm Community System (WCS), software colaborativo para una comunidad dispersa de genetistas de C. elegans. Pese a alta satisfacción de usuarios, extensa evaluación de necesidades y prototipado participativo, la mayoría no llegó a usar el sistema, que fracasó en su meta de convertirse en la infraestructura comunicativa central; muchos migraron a Gopher y Mosaic durante el auge de internet. Las autoras usan este «fracaso» para elaborar un marco analítico sobre la relación entre infraestructura de gran escala y transformación organizacional. Definen la infraestructura como concepto relacional («cuándo es una infraestructura», por analogía con el «¿cuándo es una herramienta?» de Engeström) y enumeran sus ocho dimensiones (encaje, transparencia, alcance, aprendizaje por membresía, vínculo con convenciones, encarnación de estándares, base instalada, visibilidad ante el fallo). Sostienen que no existen universales en el diseño de tecnología a gran escala: el estándar de uno es el caos de otro, y la tensión entre lo local-flexible y lo global-estandarizado es constitutiva. Aplicando los niveles de aprendizaje y comunicación de Bateson (de Steps to an Ecology of Mind), distinguen tres órdenes de problemas en el «signing on / hooking up»: de primer orden (recursos, información, acceso), de segundo orden (efectos contextuales imprevistos, choques de culturas técnicas, paradojas de infraestructura, restricciones-como-recursos) y de tercer orden (disputas políticas permanentes). Su aporte: teorizar las discontinuidades entre contextos y advertir que diseñar sistemas ciegos a estos niveles produce organizaciones escindidas y desigualdades profundizadas.</t>
+          <t>Artículo metodológico que propone estudiar la infraestructura como objeto etnográfico, formulado como un «llamado a estudiar cosas aburridas»: enchufes, estándares, formularios, clasificaciones y protocolos que subyacen invisiblemente al trabajo. Star sostiene que la infraestructura no es una cosa sino una propiedad fundamentalmente relacional y ecológica: es infraestructura solo en relación con prácticas organizadas («cuándo», no «qué», es una infraestructura); lo que para uno es sustrato transparente, para otro es tópico o barrera (el ejemplo de la escalera y la persona en silla de ruedas). Define nueve dimensiones: encaje (embeddedness), transparencia, alcance espacio-temporal, aprendizaje como parte de la membresía, vínculo con convenciones de práctica, encarnación de estándares, construcción sobre una base instalada, visibilidad ante el fallo y reparación modular. El marco proviene del interaccionismo simbólico (Strauss), los estudios sociales de la ciencia y la «inversión infraestructural» de Bowker, que lleva al primer plano lo que suele quedar de trasfondo. Metodológicamente combina análisis histórico y literario, entrevistas, observación, análisis de sistemas y estudios de usabilidad, y ofrece «trucos del oficio»: identificar narrativas maestras y sus «otros» silenciados, hacer visible el trabajo invisible y de articulación, atender a las paradojas (transparente/opaco) y precisar el estatus epistemológico de los indicadores (artefacto material, huella o representación verídica). Aborda además el problema de escala en la etnografía de sistemas distribuidos y la política inscrita en el diseño (Winner, los puentes de Moses, categorías raciales del censo). Su aporte: fundar una ética y una justicia distributiva de la infraestructura informacional.</t>
         </is>
       </c>
     </row>
@@ -6412,27 +6412,27 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Stjernfelt - Diagrammatology. An Investigation on the Borderlines of Phenomenology, Ontology, and Semiotics (2007) [Synthese Library, ISBN 9781402056512, pp. 49-107, cap. 3 «How to Learn More. An Apology for a Strong Concept of Iconicity»].md</t>
+          <t>Star y Ruhleder - Steps Toward an Ecology of Infrastructure. Design and Access for Large Information Spaces (1996) [Information Systems Research 7(1), desde p. 111].md</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>1991-1994 (estudio del Worm Community System)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro, 2007 (Synthese Library, Springer)</t>
+          <t>Artículo académico, 1996 (Information Systems Research 7(1))</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Frederik Stjernfelt; Charles S. Peirce; Edmund Husserl; Nelson Goodman; W. V. O. Quine; Friedrich Nietzsche; Alexius Meinong; Carl Stumpf; Springer / Synthese Library</t>
+          <t>Susan Leigh Star; Karen Ruhleder; Gregory Bateson; Bruce Schatz; Yrjö Engeström; Geoffrey Bowker; Bruno Latour; Information Systems Research / INFORMS</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Capítulo tercero de la diagramatología de Stjernfelt, que defiende un concepto «fuerte» u operacional de iconicidad como piedra angular de una semiótica realista de raíz peirceana (leída junto a Husserl). Frente a la mala prensa de la semejanza en el siglo XX, atacada tanto desde el flanco «nietzscheano» de las filosofías de la diferencia (que subordinan toda identidad a la diferencia) como desde el nominalismo analítico de Quine y Goodman (que reducen o eliminan la semejanza), Stjernfelt sostiene que el icono no se define por la mera semejanza objetiva —insuficiente, pues cualquier cosa se parece a otra en algún respecto— sino por la semejanza puesta en función significante mediante el uso o la intencionalidad. Su tesis decisiva es el criterio operacional peirceano del «aprender más» (to learn more): el icono es el único signo cuya contemplación y manipulación permite descubrir sobre su objeto verdades no contenidas en las instrucciones de su construcción. Este criterio, no circular, hace de la iconicidad el único signo que aporta evidencia y significado: todo índice y todo símbolo deben terminar en un icono para no estar vacíos (paralelo a Kant: intuiciones sin conceptos ciegas, conceptos sin intuiciones vacíos). De ahí que la iconicidad abarque incluso el álgebra y los cálculos formales, «iconos por excelencia» en la medida en que son manipulables y fértiles, distinguiendo así formalizaciones productivas de estériles. El icono contiene una generalidad potencial (continuo) que fundamenta el pensamiento riguroso, cuyo caso privilegiado es el diagrama. El aporte: cimentar una epistemología evolutiva y una gramática icónica que anticipan la teoría del diagrama del capítulo siguiente.</t>
+          <t>Estudio empírico y teórico basado en tres años de etnografía (1991-1994) sobre el Worm Community System (WCS), software colaborativo para una comunidad dispersa de genetistas de C. elegans. Pese a alta satisfacción de usuarios, extensa evaluación de necesidades y prototipado participativo, la mayoría no llegó a usar el sistema, que fracasó en su meta de convertirse en la infraestructura comunicativa central; muchos migraron a Gopher y Mosaic durante el auge de internet. Las autoras usan este «fracaso» para elaborar un marco analítico sobre la relación entre infraestructura de gran escala y transformación organizacional. Definen la infraestructura como concepto relacional («cuándo es una infraestructura», por analogía con el «¿cuándo es una herramienta?» de Engeström) y enumeran sus ocho dimensiones (encaje, transparencia, alcance, aprendizaje por membresía, vínculo con convenciones, encarnación de estándares, base instalada, visibilidad ante el fallo). Sostienen que no existen universales en el diseño de tecnología a gran escala: el estándar de uno es el caos de otro, y la tensión entre lo local-flexible y lo global-estandarizado es constitutiva. Aplicando los niveles de aprendizaje y comunicación de Bateson (de Steps to an Ecology of Mind), distinguen tres órdenes de problemas en el «signing on / hooking up»: de primer orden (recursos, información, acceso), de segundo orden (efectos contextuales imprevistos, choques de culturas técnicas, paradojas de infraestructura, restricciones-como-recursos) y de tercer orden (disputas políticas permanentes). Su aporte: teorizar las discontinuidades entre contextos y advertir que diseñar sistemas ciegos a estos niveles produce organizaciones escindidas y desigualdades profundizadas.</t>
         </is>
       </c>
     </row>
@@ -6444,7 +6444,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Trninić - Political Nature of Contemporary Culture and Art. Negation of Dominant and-or Affirmation of Marginal Culture [en serbio, con resumen en inglés].md</t>
+          <t>Stjernfelt - Diagrammatology. An Investigation on the Borderlines of Phenomenology, Ontology, and Semiotics (2007) [Synthese Library, ISBN 9781402056512, pp. 49-107, cap. 3 «How to Learn More. An Apology for a Strong Concept of Iconicity»].md</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -6454,17 +6454,17 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico (reseña científica), 2022</t>
+          <t>Capítulo de libro, 2007 (Synthese Library, Springer)</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Duško Trninić; Terry Eagleton; Raymond Williams; Stuart Hall; Theodor Adorno; Max Horkheimer; Walter Benjamin; Homi K. Bhabha; Fredric Jameson; Slavoj Žižek; Marina Abramović; Universidad de Banja Luka (Sociološki godišnjak)</t>
+          <t>Frederik Stjernfelt; Charles S. Peirce; Edmund Husserl; Nelson Goodman; W. V. O. Quine; Friedrich Nietzsche; Alexius Meinong; Carl Stumpf; Springer / Synthese Library</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Artículo teórico (reseña científica, en serbio con resumen en inglés) que argumenta la necesidad de redefinir la cultura y examina la politización de la cultura y del arte contemporáneos. Frente a la definición tradicional que insistía en la permanencia, inmutabilidad y jerarquía de la cultura —fijada por élites que distinguían alta y baja cultura—, Trninić rastrea, desde los «estudios culturales» del CCCS de Birmingham (Hoggart, Williams, Hall), el giro que concibe la cultura como fluida, ordinaria, cotidiana y política. Recorre las críticas a la cultura de masas (los leavisistas y Eliot desde la derecha; Adorno y Horkheimer y la «industria cultural» desde la izquierda) y la conciliación benjaminiana entre cultura elitista y de masas vía la reproductibilidad técnica. Apoyándose en Terry Eagleton y su noción de «guerras culturales», y en la tipología de Williams (cultura como ideal, documento y práctica social; niveles de cultura vivida, registrada y tradición selectiva), sostiene que introducir lo político e ideológico en el campo cultural convirtió a la cultura y a las prácticas artísticas contemporáneas en terrenos de luchas identitarias por el reconocimiento de grupos minoritarios y marginados. El marco moviliza el postestructuralismo (Derrida, différance, deconstrucción), el «mapeo cognitivo» de Jameson, el tercer espacio híbrido de Bhabha y la crítica de Žižek al multiculturalismo como «nuevo racismo». Concluye que estas luchas siguen dos vías —autoconciencia y demanda de reconocimiento de las minorías frente a la resistencia de la cultura dominante a des-privilegiarse— y propone dos soluciones: mostrar y aceptar modos de vida, e inclusión social y política efectiva. Cita a Abramović y Laibach como emblemas del arte politizado.</t>
+          <t>Capítulo tercero de la diagramatología de Stjernfelt, que defiende un concepto «fuerte» u operacional de iconicidad como piedra angular de una semiótica realista de raíz peirceana (leída junto a Husserl). Frente a la mala prensa de la semejanza en el siglo XX, atacada tanto desde el flanco «nietzscheano» de las filosofías de la diferencia (que subordinan toda identidad a la diferencia) como desde el nominalismo analítico de Quine y Goodman (que reducen o eliminan la semejanza), Stjernfelt sostiene que el icono no se define por la mera semejanza objetiva —insuficiente, pues cualquier cosa se parece a otra en algún respecto— sino por la semejanza puesta en función significante mediante el uso o la intencionalidad. Su tesis decisiva es el criterio operacional peirceano del «aprender más» (to learn more): el icono es el único signo cuya contemplación y manipulación permite descubrir sobre su objeto verdades no contenidas en las instrucciones de su construcción. Este criterio, no circular, hace de la iconicidad el único signo que aporta evidencia y significado: todo índice y todo símbolo deben terminar en un icono para no estar vacíos (paralelo a Kant: intuiciones sin conceptos ciegas, conceptos sin intuiciones vacíos). De ahí que la iconicidad abarque incluso el álgebra y los cálculos formales, «iconos por excelencia» en la medida en que son manipulables y fértiles, distinguiendo así formalizaciones productivas de estériles. El icono contiene una generalidad potencial (continuo) que fundamenta el pensamiento riguroso, cuyo caso privilegiado es el diagrama. El aporte: cimentar una epistemología evolutiva y una gramática icónica que anticipan la teoría del diagrama del capítulo siguiente.</t>
         </is>
       </c>
     </row>
@@ -6476,27 +6476,27 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>canepa_kg_2006_p132-167.pdf</t>
+          <t>Trninić - Political Nature of Contemporary Culture and Art. Negation of Dominant and-or Affirmation of Marginal Culture [en serbio, con resumen en inglés].md</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>1970-2006 (con referencias históricas desde el siglo XIX)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro, 2006</t>
+          <t>Artículo académico (reseña científica), 2022</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Giuliana Borea Labarthe; Gisela Cánepa Koch (ed.); Sandra Gamarra (LiMAC); Instituto de Arte Contemporáneo (IAC); Fernando de Szyszlo; Gerardo Chávez; Mario Vargas Llosa; Ramiro Llona; Instituto Nacional de Cultura; ICOM; Museo de la Nación; Museo Nacional de la Cultura Peruana; Alfonso Castrillón</t>
+          <t>Duško Trninić; Terry Eagleton; Raymond Williams; Stuart Hall; Theodor Adorno; Max Horkheimer; Walter Benjamin; Homi K. Bhabha; Fredric Jameson; Slavoj Žižek; Marina Abramović; Universidad de Banja Luka (Sociološki godišnjak)</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Capítulo de Giuliana Borea Labarthe ('Museos y esfera pública: espacio, discursos y prácticas. Reflexiones en torno a la ciudad de Lima') incluido en el volumen editado por Gisela Cánepa Koch, 'Mirando la esfera pública desde la cultura en el Perú' (2006). Partiendo de las nociones de esfera pública (Habermas), cultura pública (Appadurai) y de la nueva museología surgida de las crisis de los años 70-80 (Mesa de Santiago 1972, redefinición del ICOM 1974, ecomuseos), Borea concibe el museo como contenedor y contenido, plataforma y discurso, esfera de poder y arena de disputa por la representación. Analiza tres casos limeños. Primero, el posicionamiento urbano de los museos: mediante una encuesta a transeúntes y taxistas muestra que solo el Museo de la Nación y el Museo de Arte de Lima son hitos reconocidos, mientras la mayoría oscila entre lugar simbólico y lugar anónimo por la falta de señalización y de alianzas municipales. Segundo, la polémica de 2006 por el proyecto del Museo de Arte Contemporáneo (MAC) del IAC, detonada por el intento de nombrarlo 'Fernando de Szyszlo': reconstruye siete momentos del debate mediático (comunicados de artistas, la columna 'Escaramuzas en Liliput' de Vargas Llosa), la falta de plan museológico y de diálogo con artistas donantes y con Barranco, y destaca la contrapropuesta crítica LiMAC de Sandra Gamarra frente al silencio del INC. Tercero, compara las puestas en escena sobre peruanidad y diversidad de cinco museos (Cultura Peruana, de la Nación, Etnográfico, Inmigración Japonesa, MNAAHP), evidenciando discursos lejanos, fragmentados y ahistóricos en los grandes museos nacionales frente a autorrepresentaciones más políticas en los pequeños. Cierra con Castrillón: Lima como escenario de emplazamiento, no de reflexión.</t>
+          <t>Artículo teórico (reseña científica, en serbio con resumen en inglés) que argumenta la necesidad de redefinir la cultura y examina la politización de la cultura y del arte contemporáneos. Frente a la definición tradicional que insistía en la permanencia, inmutabilidad y jerarquía de la cultura —fijada por élites que distinguían alta y baja cultura—, Trninić rastrea, desde los «estudios culturales» del CCCS de Birmingham (Hoggart, Williams, Hall), el giro que concibe la cultura como fluida, ordinaria, cotidiana y política. Recorre las críticas a la cultura de masas (los leavisistas y Eliot desde la derecha; Adorno y Horkheimer y la «industria cultural» desde la izquierda) y la conciliación benjaminiana entre cultura elitista y de masas vía la reproductibilidad técnica. Apoyándose en Terry Eagleton y su noción de «guerras culturales», y en la tipología de Williams (cultura como ideal, documento y práctica social; niveles de cultura vivida, registrada y tradición selectiva), sostiene que introducir lo político e ideológico en el campo cultural convirtió a la cultura y a las prácticas artísticas contemporáneas en terrenos de luchas identitarias por el reconocimiento de grupos minoritarios y marginados. El marco moviliza el postestructuralismo (Derrida, différance, deconstrucción), el «mapeo cognitivo» de Jameson, el tercer espacio híbrido de Bhabha y la crítica de Žižek al multiculturalismo como «nuevo racismo». Concluye que estas luchas siguen dos vías —autoconciencia y demanda de reconocimiento de las minorías frente a la resistencia de la cultura dominante a des-privilegiarse— y propone dos soluciones: mostrar y aceptar modos de vida, e inclusión social y política efectiva. Cita a Abramović y Laibach como emblemas del arte politizado.</t>
         </is>
       </c>
     </row>
@@ -6508,27 +6508,27 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>canepa_kg_2006_p14-34.pdf</t>
+          <t>canepa_kg_2006_p132-167.pdf</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>n/d (marco teórico); con referencias al Perú y América Latina de la década de 2000 (Fujimori 2000, Toledo, Alan García)</t>
+          <t>1970-2006 (con referencias históricas desde el siglo XIX)</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro académico, 2006</t>
+          <t>Capítulo de libro, 2006</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Gisela Cánepa Koch; Jürgen Habermas; Nancy Fraser; Arjun Appadurai; Carol Breckenridge; George Yúdice; Michel Foucault; Pierre Bourdieu; Terence Turner; Jon McKenzie; Harold Mah; Renato Rosaldo</t>
+          <t>Giuliana Borea Labarthe; Gisela Cánepa Koch (ed.); Sandra Gamarra (LiMAC); Instituto de Arte Contemporáneo (IAC); Fernando de Szyszlo; Gerardo Chávez; Mario Vargas Llosa; Ramiro Llona; Instituto Nacional de Cultura; ICOM; Museo de la Nación; Museo Nacional de la Cultura Peruana; Alfonso Castrillón</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>La antropóloga Gisela Cánepa Koch reflexiona sobre la relación entre cultura y política proponiendo desplazar el análisis del campo político institucional hacia la comprensión del sujeto público. Su tesis central sostiene que, en un contexto de despolitización, retraimiento del Estado y crisis de representatividad partidaria, la cultura ha dejado de ser un mero medio de expresión de la diferencia para convertirse en un recurso de acción (Yúdice) y en un mecanismo fundamental de gobierno. El objeto de estudio es la esfera pública, que la autora somete a una crítica del modelo habermasiano: siguiendo a Nancy Fraser, Geoff Eley y Harold Mah, muestra que la esfera pública burguesa fue excluyente no solo por el acceso desigual, sino por codificar en sus estilos retóricos —la argumentación racional, viril y 'distinguida' en el sentido de Bourdieu— la hegemonía de una clase que hace pasar su interés particular por universal. Frente a ese modelo representacional, Cánepa adopta la noción de cultura pública de Appadurai y Breckenridge, que borra la frontera entre lo privado y lo público y admite lenguajes corporales, visuales y escénicos. Su marco conceptual articula la performatividad (McKenzie, Schechner: el imperativo del 'mostrar hacer'), el sujeto que ejerce poder (Foucault) y la ciudadanía cultural (Rosaldo). Analiza casos peruanos y latinoamericanos: la espectacularización presidencial (Fujimori, Toledo, Alan García), los asháninka, los zapatistas y la 'cultura del parque' limeña como espacio donde la opinión deviene acción. Aporta una reconceptualización del sujeto público como agente situado y performativo, cuya politización cotidiana ampliaría la democratización más allá de la mera representación.</t>
+          <t>Capítulo de Giuliana Borea Labarthe ('Museos y esfera pública: espacio, discursos y prácticas. Reflexiones en torno a la ciudad de Lima') incluido en el volumen editado por Gisela Cánepa Koch, 'Mirando la esfera pública desde la cultura en el Perú' (2006). Partiendo de las nociones de esfera pública (Habermas), cultura pública (Appadurai) y de la nueva museología surgida de las crisis de los años 70-80 (Mesa de Santiago 1972, redefinición del ICOM 1974, ecomuseos), Borea concibe el museo como contenedor y contenido, plataforma y discurso, esfera de poder y arena de disputa por la representación. Analiza tres casos limeños. Primero, el posicionamiento urbano de los museos: mediante una encuesta a transeúntes y taxistas muestra que solo el Museo de la Nación y el Museo de Arte de Lima son hitos reconocidos, mientras la mayoría oscila entre lugar simbólico y lugar anónimo por la falta de señalización y de alianzas municipales. Segundo, la polémica de 2006 por el proyecto del Museo de Arte Contemporáneo (MAC) del IAC, detonada por el intento de nombrarlo 'Fernando de Szyszlo': reconstruye siete momentos del debate mediático (comunicados de artistas, la columna 'Escaramuzas en Liliput' de Vargas Llosa), la falta de plan museológico y de diálogo con artistas donantes y con Barranco, y destaca la contrapropuesta crítica LiMAC de Sandra Gamarra frente al silencio del INC. Tercero, compara las puestas en escena sobre peruanidad y diversidad de cinco museos (Cultura Peruana, de la Nación, Etnográfico, Inmigración Japonesa, MNAAHP), evidenciando discursos lejanos, fragmentados y ahistóricos en los grandes museos nacionales frente a autorrepresentaciones más políticas en los pequeños. Cierra con Castrillón: Lima como escenario de emplazamiento, no de reflexión.</t>
         </is>
       </c>
     </row>
@@ -6540,27 +6540,27 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>poscrisis.md</t>
+          <t>canepa_kg_2006_p14-34.pdf</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>2001-2009 (arte argentino de la poscrisis)</t>
+          <t>n/d (marco teórico); con referencias al Perú y América Latina de la década de 2000 (Fujimori 2000, Toledo, Alan García)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Libro (OCR de la edición impresa), 2009</t>
+          <t>Capítulo de libro académico, 2006</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Andrea Giunta; León Ferrari; Roberto Jacoby; Graciela Sacco; Marcelo Pombo; Jorge Macchi; Liliana Maresca; Santiago Sierra; Taller Popular de Serigrafía; Nicolás Bourriaud; MALBA; Museo Nacional de Bellas Artes / Centro Cultural Recoleta; Siglo Veintiuno Editores</t>
+          <t>Gisela Cánepa Koch; Jürgen Habermas; Nancy Fraser; Arjun Appadurai; Carol Breckenridge; George Yúdice; Michel Foucault; Pierre Bourdieu; Terence Turner; Jon McKenzie; Harold Mah; Renato Rosaldo</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Reunión de ensayos de la historiadora del arte Andrea Giunta que analiza el arte argentino producido tras el colapso económico, político y social de diciembre de 2001. La tesis central sostiene que la crisis, lejos de paralizar, resultó fértil: activó una intensa colectivización de la práctica artística y una creatividad social que buscó salidas imaginarias frente a la corrupción y la incertidumbre. El objeto de estudio es la escena cultural porteña (y rosarina) entre 2001 y 2009, leída en cuatro escenarios: la ciudad de Buenos Aires como escenario del arte, el nuevo mapa museográfico (inauguración del MALBA, del MACRO, la federalización del patrimonio del MNBA), el 'caso Ferrari' como experiencia de ciudadanía y libertad de expresión, y las preguntas sobre la forma y la sensibilidad del presente. El marco conceptual combina biopolítica, gentrificación y posfordismo, la estética relacional y la posproducción de Bourriaud, y el debate reactivado sobre arte y política, vanguardia y autonomía. Giunta articula las prácticas de protesta popular (cortes de ruta, piquetes, cacerolazos, escraches, asambleas) con la organización colectiva de los artistas, sin homologarlas, y documenta la internacionalización de la crisis en el arte (La Traslación de una cacerolada, de Santiago Sierra). El libro incluye escritos de coyuntura sobre exposiciones y un glosario de términos emergentes (corralito, gentrificación, posproducción). Aparecen León Ferrari, Roberto Jacoby, Graciela Sacco, Marcelo Pombo, Jorge Macchi, Liliana Maresca y el Taller Popular de Serigrafía. Su aporte es una lectura de época, testimonial y confiada, que piensa el arte como agente activo en la reconstitución de la trama social argentina de la poscrisis.</t>
+          <t>La antropóloga Gisela Cánepa Koch reflexiona sobre la relación entre cultura y política proponiendo desplazar el análisis del campo político institucional hacia la comprensión del sujeto público. Su tesis central sostiene que, en un contexto de despolitización, retraimiento del Estado y crisis de representatividad partidaria, la cultura ha dejado de ser un mero medio de expresión de la diferencia para convertirse en un recurso de acción (Yúdice) y en un mecanismo fundamental de gobierno. El objeto de estudio es la esfera pública, que la autora somete a una crítica del modelo habermasiano: siguiendo a Nancy Fraser, Geoff Eley y Harold Mah, muestra que la esfera pública burguesa fue excluyente no solo por el acceso desigual, sino por codificar en sus estilos retóricos —la argumentación racional, viril y 'distinguida' en el sentido de Bourdieu— la hegemonía de una clase que hace pasar su interés particular por universal. Frente a ese modelo representacional, Cánepa adopta la noción de cultura pública de Appadurai y Breckenridge, que borra la frontera entre lo privado y lo público y admite lenguajes corporales, visuales y escénicos. Su marco conceptual articula la performatividad (McKenzie, Schechner: el imperativo del 'mostrar hacer'), el sujeto que ejerce poder (Foucault) y la ciudadanía cultural (Rosaldo). Analiza casos peruanos y latinoamericanos: la espectacularización presidencial (Fujimori, Toledo, Alan García), los asháninka, los zapatistas y la 'cultura del parque' limeña como espacio donde la opinión deviene acción. Aporta una reconceptualización del sujeto público como agente situado y performativo, cuya politización cotidiana ampliaría la democratización más allá de la mera representación.</t>
         </is>
       </c>
     </row>
@@ -6572,32 +6572,64 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
+          <t>poscrisis.md</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>2001-2009 (arte argentino de la poscrisis)</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Libro (OCR de la edición impresa), 2009</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Andrea Giunta; León Ferrari; Roberto Jacoby; Graciela Sacco; Marcelo Pombo; Jorge Macchi; Liliana Maresca; Santiago Sierra; Taller Popular de Serigrafía; Nicolás Bourriaud; MALBA; Museo Nacional de Bellas Artes / Centro Cultural Recoleta; Siglo Veintiuno Editores</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Reunión de ensayos de la historiadora del arte Andrea Giunta que analiza el arte argentino producido tras el colapso económico, político y social de diciembre de 2001. La tesis central sostiene que la crisis, lejos de paralizar, resultó fértil: activó una intensa colectivización de la práctica artística y una creatividad social que buscó salidas imaginarias frente a la corrupción y la incertidumbre. El objeto de estudio es la escena cultural porteña (y rosarina) entre 2001 y 2009, leída en cuatro escenarios: la ciudad de Buenos Aires como escenario del arte, el nuevo mapa museográfico (inauguración del MALBA, del MACRO, la federalización del patrimonio del MNBA), el 'caso Ferrari' como experiencia de ciudadanía y libertad de expresión, y las preguntas sobre la forma y la sensibilidad del presente. El marco conceptual combina biopolítica, gentrificación y posfordismo, la estética relacional y la posproducción de Bourriaud, y el debate reactivado sobre arte y política, vanguardia y autonomía. Giunta articula las prácticas de protesta popular (cortes de ruta, piquetes, cacerolazos, escraches, asambleas) con la organización colectiva de los artistas, sin homologarlas, y documenta la internacionalización de la crisis en el arte (La Traslación de una cacerolada, de Santiago Sierra). El libro incluye escritos de coyuntura sobre exposiciones y un glosario de términos emergentes (corralito, gentrificación, posproducción). Aparecen León Ferrari, Roberto Jacoby, Graciela Sacco, Marcelo Pombo, Jorge Macchi, Liliana Maresca y el Taller Popular de Serigrafía. Su aporte es una lectura de época, testimonial y confiada, que piensa el arte como agente activo en la reconstitución de la trama social argentina de la poscrisis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Teoría</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
           <t>Índice de «Anthropology and Art Practice» de Schneider y Wright. Solo la tabla de contenidos, 257 palabras, no es el libro.md</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>Índice / tabla de contenidos de libro, 2013</t>
         </is>
       </c>
-      <c r="E68" s="3" t="inlineStr">
+      <c r="E69" s="3" t="inlineStr">
         <is>
           <t>Arnd Schneider; Christopher Wright; Craig Campbell; Anthony Luvera; Thera Mjaaland; Christina Lammer; Kathryn Ramey; Brad Butler; Karen Mirza; Raul Ortega Ayala; Rupert Cox y Angus Carlyle; Bloomsbury Academic</t>
         </is>
       </c>
-      <c r="F68" s="3" t="inlineStr">
+      <c r="F69" s="3" t="inlineStr">
         <is>
           <t>Este documento no es el libro sino, exclusivamente, la tabla de contenidos (índice, unas 257 palabras) de «Anthropology and Art Practice», volumen editado por Arnd Schneider y Christopher Wright y publicado por Bloomsbury Academic en 2013. Por su naturaleza paratextual, no contiene argumentación desarrollada, sino la nómina de capítulos, autores y páginas, además de las secciones preliminares (lista de ilustraciones, agradecimientos, colaboradores) y el índice analítico final. El sumario permite reconstruir la arquitectura conceptual de la obra: se abre con el ensayo programático «Ways of Working», de los editores, que enmarca el cruce entre práctica artística y práctica antropológica como campo metodológico y epistemológico. Los capítulos siguientes, en su mayoría escritos por artistas-investigadores o formulados como conversaciones (con figuras como Anthony Luvera, Brad Butler y Karen Mirza, o Raul Ortega Ayala), privilegian el relato en primera persona sobre el proceso creativo antes que la teorización clásica. Los títulos anuncian los ejes recurrentes del volumen: la ambigüedad y la incertidumbre epistemológica (Thera Mjaaland), la liminalidad y la experiencia del cuerpo (Ruth Jones, Christina Lammer), lo sensorial y lo audiovisual (Laurent Van Lancker, Caterina Pasqualino), el cine experimental y etnográfico (Kathryn Ramey, Craig Campbell) y la colaboración entre arte, antropología y ciencia (Rupert Cox y Angus Carlyle). En conjunto, el índice evidencia la apuesta editorial por un giro práctico y colaborativo en la antropología del arte, que desplaza el foco desde la representación etnográfica hacia formas experimentales de conocimiento compartido. Como fuente, su utilidad es referencial: sirve para localizar autores, temas y aportes del libro, pero no sustituye la lectura de sus capítulos.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F68"/>
+  <autoFilter ref="A1:F69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Cataloga «La Construcción del Lugar Común» (MAC-Lima, 2008)
- Añade Cap 2 - Historia/mac-proyecto-2008.md a tabla-cap2-historia.csv
  con año referenciado, periodo, personas e instituciones y resumen de
  ~250 palabras. Cap 2 pasa a 72 filas.
- Regenera tablas-sistematizacion.xlsx con la hoja Cap 2 - Historia al día.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bob4w11uQRyAcv1Qayw1V
</commit_message>
<xml_diff>
--- a/Sistematización/tablas-sistematizacion.xlsx
+++ b/Sistematización/tablas-sistematizacion.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Extras" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cap 3 - Análisis'!$A$1:$F$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Teoría'!$A$1:$F$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Extras'!$A$1:$F$4</definedName>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2366,59 +2366,59 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>sura.md</t>
+          <t>mac-proyecto-2008.md</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>mediados de la década de 1960 a 2013 (arte contemporáneo peruano)</t>
+          <t>2008 (exposición feb.–mar. 2008; con historia del sitio desde 1944)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de colección museística, 2013</t>
+          <t>Catálogo de exposición, mayo 2008 (Instituto de Arte Contemporáneo — MAC-Lima; OCR)</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner (ed.); Museo de Arte de Lima (MALI); Grupo SURA; Mirko Lauer; E.P.S. Huayco; Charo Noriega; Ramiro Llona; Flavia Gandolfo; Armando Andrade Tudela; Ricardo Wiesse; Eduardo Villanes; Miguel A. López; Rodrigo Quijano</t>
+          <t>Jorge Villacorta; Miguel Zegarra (curadores); Instituto de Arte Contemporáneo (IAC); MAC-Lima; Giuliana Borea; George Gruenberg; Ricardo Ramón Jarne; José Carlos Martinat; Ishmael Randall Weeks; Elena Damiani; Sergio Abugattás; Raura Oblitas</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Catálogo de la colección de arte contemporáneo del Museo de Arte de Lima (MALI), editado por la curadora Sharon Lerner y publicado con el patrocinio del grupo SURA. El volumen traza los derroteros del arte peruano reciente a partir del acervo del museo, sin pretender definir un 'arte peruano' esencial. La colección se articula bajo dos principios: identificar momentos de ruptura en la producción artística de fines del siglo XX y perfilar la producción reciente mediante ejes temáticos comunes. El ensayo central de Lerner establece como punto de partida mediados de la década de 1960 (grupos de vanguardia ligados al Pop y al no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, tras las reformas del Gobierno Militar, cuando —según la célebre frase de Mirko Lauer para la muestra Arte al paso del colectivo E.P.S. Huayco (1980)— 'en el Perú hoy solo lo popular es moderno'. Analiza la irrupción de la migración interna, el conflicto armado interno, el autogolpe de Fujimori (1992) y la virtual desaparición de la esfera pública, así como la Bienal Iberoamericana de Lima (1997) como puesta al día forzada y descontextualizada. El catálogo se organiza en núcleos temáticos: modernidad popular y transformación de Lima, f(r)icciones cosmopolitas, reconsideración del pasado y configuración del Perú, sistema artístico y utopías museales, desplazamientos, y signos de violencia, resistencia y memoria. Incluye obras de Charo Noriega, Ramiro Llona, Flavia Gandolfo, Armando Andrade Tudela, Herman Schwarz, Ricardo Wiesse y Eduardo Villanes, entre otros, y textos críticos complementarios. Su aporte es consolidar un relato historiográfico y crítico del arte contemporáneo peruano desde una institución museal.</t>
+          <t>Catálogo de la exposición «La Construcción del Lugar Común» (MAC-Lima, 5 de febrero–30 de marzo de 2008), editado por el Instituto de Arte Contemporáneo (IAC) y curado por Jorge Villacorta y Miguel Zegarra. Documenta una intervención colectiva de quince artistas peruanos emergentes —Sergio Abugattás, Miguel Andrade, Víctor Castro, Elena Damiani, Giuseppe De Bernardi, Nicole Franchy, Alejandro Jaime, Manuel Larrea, Martín Jiménez Paz, Christians Luna, José Carlos Martinat, José Miyashiro, Raura Oblitas, Ishmael Randall Weeks e Iliana Scheggia— que ocuparon el edificio del Museo de Arte Contemporáneo de Lima cuando aún estaba a medio construir. La muestra convirtió la arquitectura inconclusa y su entorno (el parque de la antigua «laguna» de Barranco) en soporte y tema: las obras tematizan la construcción/destrucción, el paisaje, la memoria del sitio y la disputa pública por el museo, cuyo proceso estuvo marcado por conflictos municipales y un intento de clausura respondido con el gesto «CLAUSURADO = INAUGURADO». El catálogo reúne textos institucionales (George Gruenberg, presidente del IAC), una pieza literaria de Ricardo Ramón Jarne («La maldición de la laguna»), un ensayo antropológico de Giuliana Borea sobre la construcción del lugar y el «lugar común» en la esfera pública (apoyado en Augé, Appadurai, Certeau y Casey), el texto curatorial de Villacorta y Zegarra, y los statements de cada artista. Como fuente histórica documenta un episodio clave de institucionalización del arte contemporáneo en Lima —la génesis del MAC— y las prácticas site-specific, de crítica institucional y de intervención en el espacio público de una generación emergente peruana de fines de la década de 2000.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Arte al Paso 2011</t>
+          <t>Cap 2 - Historia</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Arte al Paso - Texto Investigación.md</t>
+          <t>sura.md</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 1960 – 2010 (con foco en las décadas de 1970-2000 y el conflicto armado interno 1980-2000)</t>
+          <t>mediados de la década de 1960 a 2013 (arte contemporáneo peruano)</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Ensayo curatorial de catálogo (exposición Arte al paso, Pinacoteca do Estado de São Paulo, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Catálogo de colección museística, 2013</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Pinacoteca de São Paulo; Emilio Hernández Saavedra; E.P.S. Huayco; Jesús Ruiz Durand; Sandra Gamarra; Alfredo Márquez / Taller NN; Fernando Bryce; José Carlos Martinat; Susana Torres</t>
+          <t>Sharon Lerner (ed.); Museo de Arte de Lima (MALI); Grupo SURA; Mirko Lauer; E.P.S. Huayco; Charo Noriega; Ramiro Llona; Flavia Gandolfo; Armando Andrade Tudela; Ricardo Wiesse; Eduardo Villanes; Miguel A. López; Rodrigo Quijano</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Ensayo curatorial extenso y bilingüe (castellano/portugués) de Tatiana Cuevas y Rodrigo Quijano para la muestra Arte al paso, que exhibió la coleccion contemporanea del MALI en la Estacion Pinacoteca de Sao Paulo. El texto toma como punto de partida la imagen El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra para diagnosticar los vacios institucionales y la distancia entre el discurso cultural cosmopolita y la practica real en el Peru de la segunda mitad del siglo XX. Su argumento articula el arte contemporaneo peruano con las transformaciones sociales derivadas de la masiva migracion rural a Lima, la explosion de la economia informal y la emergencia de una nueva cultura popular urbana. Rastrea las primeras vinculaciones locales con vanguardias internacionales (op, pop, conceptualismo, no-objetualismo), el pop achorado de Jesus Ruiz Durand y sus afiches de la Reforma Agraria velasquista, y las experiencias colectivas Contacta 79 y Arte al paso de E.P.S. Huayco (1980), que propusieron un arte callejero y antiinstitucional. Analiza la critica a la institucionalidad faltante (el museo ficticio LiMAC de Sandra Gamarra), el uso ironico del pasado prehispanico (Susana Torres, Rodriguez Larrain, Bryce, Cordova, Martinat), el tema del paisaje y el territorio, y la irrupcion tardia de la fotografia y la serigrafia como medios. Dedica una seccion central a la memoria de la violencia del conflicto armado interno (1980-2000) —Sendero Luminoso, MRTA, la Comision de la Verdad, 69.280 muertos— y su tratamiento por el Taller NN, Alfredo Marquez (Katatay), Carlos Dominguez, Ricardo Wiesse, Eduardo Villanes, Fernando Bryce y Milagros de la Torre.</t>
+          <t>Catálogo de la colección de arte contemporáneo del Museo de Arte de Lima (MALI), editado por la curadora Sharon Lerner y publicado con el patrocinio del grupo SURA. El volumen traza los derroteros del arte peruano reciente a partir del acervo del museo, sin pretender definir un 'arte peruano' esencial. La colección se articula bajo dos principios: identificar momentos de ruptura en la producción artística de fines del siglo XX y perfilar la producción reciente mediante ejes temáticos comunes. El ensayo central de Lerner establece como punto de partida mediados de la década de 1960 (grupos de vanguardia ligados al Pop y al no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, tras las reformas del Gobierno Militar, cuando —según la célebre frase de Mirko Lauer para la muestra Arte al paso del colectivo E.P.S. Huayco (1980)— 'en el Perú hoy solo lo popular es moderno'. Analiza la irrupción de la migración interna, el conflicto armado interno, el autogolpe de Fujimori (1992) y la virtual desaparición de la esfera pública, así como la Bienal Iberoamericana de Lima (1997) como puesta al día forzada y descontextualizada. El catálogo se organiza en núcleos temáticos: modernidad popular y transformación de Lima, f(r)icciones cosmopolitas, reconsideración del pasado y configuración del Perú, sistema artístico y utopías museales, desplazamientos, y signos de violencia, resistencia y memoria. Incluye obras de Charo Noriega, Ramiro Llona, Flavia Gandolfo, Armando Andrade Tudela, Herman Schwarz, Ricardo Wiesse y Eduardo Villanes, entre otros, y textos críticos complementarios. Su aporte es consolidar un relato historiográfico y crítico del arte contemporáneo peruano desde una institución museal.</t>
         </is>
       </c>
     </row>
@@ -2430,27 +2430,27 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Cronología Político Artistica - Arte al Paso 2011.md</t>
+          <t>Arte al Paso - Texto Investigación.md</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>1962 – 2010</t>
+          <t>Fines de los años 1960 – 2010 (con foco en las décadas de 1970-2000 y el conflicto armado interno 1980-2000)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Cronología y bibliografía de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Ensayo curatorial de catálogo (exposición Arte al paso, Pinacoteca do Estado de São Paulo, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Museo de Arte de Lima (MALI); Grupo Arte Nuevo; Grupo Señal; E.P.S. Huayco; Taller NN; Colectivo Sociedad Civil; Gustavo Buntinx; Joaquín López Antay; Comisión de la Verdad y Reconciliación; Sendero Luminoso; Alberto Fujimori; Juan Velasco Alvarado</t>
+          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Pinacoteca de São Paulo; Emilio Hernández Saavedra; E.P.S. Huayco; Jesús Ruiz Durand; Sandra Gamarra; Alfredo Márquez / Taller NN; Fernando Bryce; José Carlos Martinat; Susana Torres</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Cronologia politico-artistica bilingue (castellano/portugues) incluida en el catalogo Arte al paso, que entrelaza en paralelo tres series de acontecimientos —eventos politicos, eventos artisticos y adquisiciones de la coleccion de arte contemporaneo del MALI— entre 1962 y 2010. El documento funciona como aparato historiografico que contextualiza la escena artistica peruana dentro de sus convulsiones politicas: rebeliones campesinas y golpes militares de los anos sesenta, el Gobierno Revolucionario de las Fuerzas Armadas de Velasco Alvarado (1968) y la Reforma Agraria, el estallido del conflicto armado interno con Sendero Luminoso y el MRTA (1980), las masacres de Barrios Altos y La Cantuta, el autogolpe y la dictadura de Alberto Fujimori (1990-2000), la Marcha de los Cuatro Suyos y el Informe de la Comision de la Verdad y Reconciliacion (2003). En el plano artistico registra la formacion de los grupos Senal y Arte Nuevo, las Bienales de Lima e Iberoamericanas, los festivales Contacta e Inkarri, el Taller E.P.S. Huayco y el Taller NN, la premiacion de Joaquin Lopez Antay, y acciones de arte critico como Cantuta de Ricardo Wiesse, Gloria evaporada de Eduardo Villanes y Lava la bandera del Colectivo Sociedad Civil. Una tercera linea traza la institucionalizacion del MALI: el ciclo curatorial Miradas de fin de siglo, la creacion del Comite de Adquisiciones (2007) y la reapertura del museo (2010). Se acompana de una extensa bibliografia especializada (Buntinx, Castrillon, Lauer, Majluf, Lopez, Tarazona, Quijano, Villacorta), fuente clave para la historiografia del arte peruano contemporaneo.</t>
+          <t>Ensayo curatorial extenso y bilingüe (castellano/portugués) de Tatiana Cuevas y Rodrigo Quijano para la muestra Arte al paso, que exhibió la coleccion contemporanea del MALI en la Estacion Pinacoteca de Sao Paulo. El texto toma como punto de partida la imagen El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra para diagnosticar los vacios institucionales y la distancia entre el discurso cultural cosmopolita y la practica real en el Peru de la segunda mitad del siglo XX. Su argumento articula el arte contemporaneo peruano con las transformaciones sociales derivadas de la masiva migracion rural a Lima, la explosion de la economia informal y la emergencia de una nueva cultura popular urbana. Rastrea las primeras vinculaciones locales con vanguardias internacionales (op, pop, conceptualismo, no-objetualismo), el pop achorado de Jesus Ruiz Durand y sus afiches de la Reforma Agraria velasquista, y las experiencias colectivas Contacta 79 y Arte al paso de E.P.S. Huayco (1980), que propusieron un arte callejero y antiinstitucional. Analiza la critica a la institucionalidad faltante (el museo ficticio LiMAC de Sandra Gamarra), el uso ironico del pasado prehispanico (Susana Torres, Rodriguez Larrain, Bryce, Cordova, Martinat), el tema del paisaje y el territorio, y la irrupcion tardia de la fotografia y la serigrafia como medios. Dedica una seccion central a la memoria de la violencia del conflicto armado interno (1980-2000) —Sendero Luminoso, MRTA, la Comision de la Verdad, 69.280 muertos— y su tratamiento por el Taller NN, Alfredo Marquez (Katatay), Carlos Dominguez, Ricardo Wiesse, Eduardo Villanes, Fernando Bryce y Milagros de la Torre.</t>
         </is>
       </c>
     </row>
@@ -2462,59 +2462,59 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Texto de la exposición Arte al Paso 2011.md</t>
+          <t>Cronología Político Artistica - Arte al Paso 2011.md</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 1960 – 2010 (unos 40 años; foco en las décadas de 1970-1980)</t>
+          <t>1962 – 2010</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Texto de sala / presentación de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Cronología y bibliografía de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Emilio Hernández Saavedra; E.P.S. Huayco; Grupo Paréntesis; Sandra Gamarra; Susana Torres; Emilio Rodríguez Larraín; Juan Javier Salazar; William Cordova; José Carlos Martinat</t>
+          <t>Museo de Arte de Lima (MALI); Grupo Arte Nuevo; Grupo Señal; E.P.S. Huayco; Taller NN; Colectivo Sociedad Civil; Gustavo Buntinx; Joaquín López Antay; Comisión de la Verdad y Reconciliación; Sendero Luminoso; Alberto Fujimori; Juan Velasco Alvarado</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Texto de sala o presentacion general de la exposicion Arte al paso (coleccion contemporanea del MALI en la Pinacoteca de Sao Paulo), firmado por los curadores Tatiana Cuevas y Rodrigo Quijano, en edicion bilingue castellano/portugues. Es una version sintetica del argumento curatorial: parte nuevamente de El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra como metafora de la ausencia institucional y punto de arranque para examinar la escena artistica peruana desde fines de los anos sesenta. Explica el titulo de la muestra a partir de la accion Arte al paso de E.P.S. Huayco (1980) —que, aludiendo a los puestos informales de comida al paso surgidos con la migracion y la economia informal, propuso un arte para consumirse en la calle, opuesto al museo y la galeria ausentes, un arte para pensar y no para sentir que dejaba atras el modernismo conservador de mediados de siglo. Sintetiza cuarenta anos de produccion cultural marcados por oposiciones ocultas y explicitas, los primeros acercamientos al conceptualismo y a las vanguardias internacionales, y la creciente proyeccion internacional de artistas peruanos. Una segunda seccion, Critica ante una institucionalidad faltante y al poder redentor del pasado, reune a Hernandez Saavedra, los grupos Parentesis y E.P.S. Huayco y el museo ficticio de Sandra Gamarra como estrategias de critica institucional apropiadas del conceptualismo y del imaginario popular urbano, con recurrente uso del humor. Aborda ademas la critica a la explotacion comercial y politica de lo prehispanico (Museo Neo-Inka de Susana Torres) y el vinculo entre la retorica del glorioso pasado incaico y los fracasos politicos y economicos del presente en obras de Rodriguez Larrain, Salazar, Cordova y Martinat.</t>
+          <t>Cronologia politico-artistica bilingue (castellano/portugues) incluida en el catalogo Arte al paso, que entrelaza en paralelo tres series de acontecimientos —eventos politicos, eventos artisticos y adquisiciones de la coleccion de arte contemporaneo del MALI— entre 1962 y 2010. El documento funciona como aparato historiografico que contextualiza la escena artistica peruana dentro de sus convulsiones politicas: rebeliones campesinas y golpes militares de los anos sesenta, el Gobierno Revolucionario de las Fuerzas Armadas de Velasco Alvarado (1968) y la Reforma Agraria, el estallido del conflicto armado interno con Sendero Luminoso y el MRTA (1980), las masacres de Barrios Altos y La Cantuta, el autogolpe y la dictadura de Alberto Fujimori (1990-2000), la Marcha de los Cuatro Suyos y el Informe de la Comision de la Verdad y Reconciliacion (2003). En el plano artistico registra la formacion de los grupos Senal y Arte Nuevo, las Bienales de Lima e Iberoamericanas, los festivales Contacta e Inkarri, el Taller E.P.S. Huayco y el Taller NN, la premiacion de Joaquin Lopez Antay, y acciones de arte critico como Cantuta de Ricardo Wiesse, Gloria evaporada de Eduardo Villanes y Lava la bandera del Colectivo Sociedad Civil. Una tercera linea traza la institucionalizacion del MALI: el ciclo curatorial Miradas de fin de siglo, la creacion del Comite de Adquisiciones (2007) y la reapertura del museo (2010). Se acompana de una extensa bibliografia especializada (Buntinx, Castrillon, Lauer, Majluf, Lopez, Tarazona, Quijano, Villacorta), fuente clave para la historiografia del arte peruano contemporaneo.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Hueso Húmero 18</t>
+          <t>Cap 2 - Historia/Arte al Paso 2011</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - Arte joven peruano, ¿el sueño del mercado propio? Una conversación con Claudia Polar (1983) [Hueso Húmero 18, pp. 94-107].md</t>
+          <t>Texto de la exposición Arte al Paso 2011.md</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>1974-1983</t>
+          <t>Fines de los años 1960 – 2010 (unos 40 años; foco en las décadas de 1970-1980)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Entrevista en revista (Hueso Húmero 18), 1983</t>
+          <t>Texto de sala / presentación de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Claudia Polar; Galería Forum; Elida Román; Hernán Pazos; Esther Vainstein; Ramiro Llona; Bill Caro; Herbert Rodríguez; EAPUC; ENBA; Hueso Húmero</t>
+          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Emilio Hernández Saavedra; E.P.S. Huayco; Grupo Paréntesis; Sandra Gamarra; Susana Torres; Emilio Rodríguez Larraín; Juan Javier Salazar; William Cordova; José Carlos Martinat</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Entrevista conducida por Gustavo Buntinx a Claudia Polar, directora de la Galería Forum, concebida como contraparte de un reportaje previo a Elida Román para perfilar el mercado del arte joven peruano. Polar reconstruye la fundación de Forum en diciembre de 1974 como un espacio destinado a priorizar a los artistas jóvenes y a gestar deliberadamente un mercado y coleccionistas nuevos, mediante becas, premios, subvenciones informales (incluso marcos y pasajes) y una política de "riesgo total" sostenida por la venta de stock. El diálogo traza una periodización económica de la plástica: expansión del mercado hacia 1974-1976, auge en 1978 atribuido a la restricción de importaciones bajo Morales Bermúdez, y recesión desde 1980 con la apertura de Belaúnde, siendo 1983 el año más difícil. Se discute la naturaleza del público comprador (gente joven, profesionales, empresarios, bancos como el de Crédito y el Continental) y la débil proporción de compradores habituales, apenas un 5% con relación económica. Buntinx presiona sobre las mediaciones de clase: el vínculo de Forum con la Universidad Católica frente a la ENBA, la identidad ideológica compartida, y el papel de las relaciones públicas como "gatillo" de casi toda venta en un mercado de "sala de estar". Polar aborda la diferencia entre lo culto y lo popular, el fracaso de asociar galerías, las cotizaciones (Llona, Caro, Pazos, Vainstein) y la explotación del artista acostumbrado a vender barato. El aporte documental es excepcional: registra desde dentro la lógica comercial, simbólica y provinciana del circuito limeño de principios de los ochenta.</t>
+          <t>Texto de sala o presentacion general de la exposicion Arte al paso (coleccion contemporanea del MALI en la Pinacoteca de Sao Paulo), firmado por los curadores Tatiana Cuevas y Rodrigo Quijano, en edicion bilingue castellano/portugues. Es una version sintetica del argumento curatorial: parte nuevamente de El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra como metafora de la ausencia institucional y punto de arranque para examinar la escena artistica peruana desde fines de los anos sesenta. Explica el titulo de la muestra a partir de la accion Arte al paso de E.P.S. Huayco (1980) —que, aludiendo a los puestos informales de comida al paso surgidos con la migracion y la economia informal, propuso un arte para consumirse en la calle, opuesto al museo y la galeria ausentes, un arte para pensar y no para sentir que dejaba atras el modernismo conservador de mediados de siglo. Sintetiza cuarenta anos de produccion cultural marcados por oposiciones ocultas y explicitas, los primeros acercamientos al conceptualismo y a las vanguardias internacionales, y la creciente proyeccion internacional de artistas peruanos. Una segunda seccion, Critica ante una institucionalidad faltante y al poder redentor del pasado, reune a Hernandez Saavedra, los grupos Parentesis y E.P.S. Huayco y el museo ficticio de Sandra Gamarra como estrategias de critica institucional apropiadas del conceptualismo y del imaginario popular urbano, con recurrente uso del humor. Aborda ademas la critica a la explotacion comercial y politica de lo prehispanico (Museo Neo-Inka de Susana Torres) y el vinculo entre la retorica del glorioso pasado incaico y los fracasos politicos y economicos del presente en obras de Rodriguez Larrain, Salazar, Cordova y Martinat.</t>
         </is>
       </c>
     </row>
@@ -2526,27 +2526,27 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - ¿Entre lo popular y lo moderno? Alternativas pretendidas o reales en la joven plástica peruana (1983) [Hueso Húmero 18, pp. 61-85].md</t>
+          <t>Buntinx - Arte joven peruano, ¿el sueño del mercado propio? Una conversación con Claudia Polar (1983) [Hueso Húmero 18, pp. 94-107].md</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>1960-1984 (con énfasis en los años 70)</t>
+          <t>1974-1983</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
+          <t>Entrevista en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Mirko Lauer; Juan Acha; Francisco Mariotti; Huayco E.P.S.; Herbert Rodríguez; Juan Javier Salazar; Jesús Ruiz Durand; Fernando de Szyszlo; IAC; Galería Forum; SINAMOS; Néstor García Canclini</t>
+          <t>Gustavo Buntinx; Claudia Polar; Galería Forum; Elida Román; Hernán Pazos; Esther Vainstein; Ramiro Llona; Bill Caro; Herbert Rodríguez; EAPUC; ENBA; Hueso Húmero</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Ensayo teórico-histórico que propone hipótesis de trabajo sobre lo que fue o pretendió ser alternativo en el arte erudito peruano desde la transición al primer belaundismo hasta los años ochenta, articulando dos tópicos móviles: lo popular y lo moderno. Retomando y ampliando a Mirko Lauer, Buntinx sostiene que las opciones estéticas no reflejan mecánicamente la época sino que reproducen una inserción particular en el mercado, entendido como trama compleja de producción, intermediación y consumo (soporte social). Recorre así una secuencia de "soportes": el corporativo (IAC financiado por IPC, IBM, Tecnoquímica) que sostuvo la Teoría de las Raíces Nacionales de Szyszlo; el soporte "de punta" del frenesí pop cosmopolita (Acha, Arte Nuevo, Fundación para las Artes, 1966-1969); el soporte estatal velasquista con sus cuatro alternativas (comunicación masiva de Ruiz Durand con su "pop achorado", festivales de arte-total como Contacta e Inkarri, revaloración de lo artesanal, López Antay); y la frustrada búsqueda de un soporte alternativo hacia 1977-1980. El caso central es Huayco E.P.S., cuyo proyecto Sarita Colonia codifica una modernidad sincrética limeña sostenida por una pequeña burguesía ilustrada radicalizada, y cuya dispersión coincide con el agotamiento de la izquierda y el repliegue hacia el mercado galerístico (Forum). El marco conceptual bebe de García Canclini. La tesis es incisiva: el tránsito de la imagen telúrica a la industrial, agraria y migrante revela apropiaciones sucesivas de una idea variable de lo popular, siempre con una radicalidad deficiente y una relación desigual con la cultura interpretada.</t>
+          <t>Entrevista conducida por Gustavo Buntinx a Claudia Polar, directora de la Galería Forum, concebida como contraparte de un reportaje previo a Elida Román para perfilar el mercado del arte joven peruano. Polar reconstruye la fundación de Forum en diciembre de 1974 como un espacio destinado a priorizar a los artistas jóvenes y a gestar deliberadamente un mercado y coleccionistas nuevos, mediante becas, premios, subvenciones informales (incluso marcos y pasajes) y una política de "riesgo total" sostenida por la venta de stock. El diálogo traza una periodización económica de la plástica: expansión del mercado hacia 1974-1976, auge en 1978 atribuido a la restricción de importaciones bajo Morales Bermúdez, y recesión desde 1980 con la apertura de Belaúnde, siendo 1983 el año más difícil. Se discute la naturaleza del público comprador (gente joven, profesionales, empresarios, bancos como el de Crédito y el Continental) y la débil proporción de compradores habituales, apenas un 5% con relación económica. Buntinx presiona sobre las mediaciones de clase: el vínculo de Forum con la Universidad Católica frente a la ENBA, la identidad ideológica compartida, y el papel de las relaciones públicas como "gatillo" de casi toda venta en un mercado de "sala de estar". Polar aborda la diferencia entre lo culto y lo popular, el fracaso de asociar galerías, las cotizaciones (Llona, Caro, Pazos, Vainstein) y la explotación del artista acostumbrado a vender barato. El aporte documental es excepcional: registra desde dentro la lógica comercial, simbólica y provinciana del circuito limeño de principios de los ochenta.</t>
         </is>
       </c>
     </row>
@@ -2558,27 +2558,27 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Freire - Herbert Rodríguez, azote y azúcar con el sistema (1983) [Hueso Húmero 18, pdf pp. 178-185].md</t>
+          <t>Buntinx - ¿Entre lo popular y lo moderno? Alternativas pretendidas o reales en la joven plástica peruana (1983) [Hueso Húmero 18, pp. 61-85].md</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>1979-1983 (con antecedentes desde 1968)</t>
+          <t>1960-1984 (con énfasis en los años 70)</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Reseña crítica en revista (Hueso Húmero 18), 1983</t>
+          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Luis Freire S.; Herbert Rodríguez; Francisco Mariotti; Huayco E.P.S.; Juan Acha; Fernando Bedoya; Juan Javier Salazar; Bienal de Sao Paulo; Galería La Rama Dorada; Galería Forum; EAPUC; ENBAP</t>
+          <t>Gustavo Buntinx; Mirko Lauer; Juan Acha; Francisco Mariotti; Huayco E.P.S.; Herbert Rodríguez; Juan Javier Salazar; Jesús Ruiz Durand; Fernando de Szyszlo; IAC; Galería Forum; SINAMOS; Néstor García Canclini</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Perfil crítico dedicado a Herbert Rodríguez Huachín en la sección "Individuales" de Hueso Húmero, escrito por Luis Freire, que examina el salto vertiginoso del artista desde la suspensión disciplinaria en la Escuela de Artes Plásticas de la Católica (1981) hasta su presencia en la XVII Bienal de Sao Paulo (1983). Freire sitúa a Rodríguez como imposible de explicar sin el proceso ideológico del populismo velasquista y sin la figura mediadora de Francisco Mariotti, artista suizo-peruano formado en la Documenta de Kassel y la vanguardia europea, catalizador de Contacta y de la EPS Huayco. El texto reconstruye la genealogía Mariotti-Huayco-Rodríguez: los ensamblajes y "reciclajes" del suizo-peruano derivan en los "altares" de Rodríguez, hibridación entre constructivismo geométrico, expresionismo "pobre" y antiestético, y estructuras rituales de la religiosidad popular andina. Argumenta que Rodríguez encarna las contradicciones de una pequeña burguesía radical: dinamita el circuito con una mano y lo enluce con la otra, camuflando "bellamente" materiales pobres y reciclados en obras a la vez contestatarias y comerciables, con lo que ironiza sobre el culto al oficio del arte establecido. Analiza su heterogeneidad de lenguajes (expresionismo abstracto, figuración dura, conceptualismo informal, collage, fotocopia, ensamblaje) como búsqueda pero también como crisis, y sus "altares al Yo" exhibidos en Forum (1983) y la Bienal. Freire lo define como un artista religioso-existencial populista sin referentes sólidos, en formación, tensionado entre enriquecer el jardín burgués que quiere pisotear o saltar a opciones más radicales de ruptura.</t>
+          <t>Ensayo teórico-histórico que propone hipótesis de trabajo sobre lo que fue o pretendió ser alternativo en el arte erudito peruano desde la transición al primer belaundismo hasta los años ochenta, articulando dos tópicos móviles: lo popular y lo moderno. Retomando y ampliando a Mirko Lauer, Buntinx sostiene que las opciones estéticas no reflejan mecánicamente la época sino que reproducen una inserción particular en el mercado, entendido como trama compleja de producción, intermediación y consumo (soporte social). Recorre así una secuencia de "soportes": el corporativo (IAC financiado por IPC, IBM, Tecnoquímica) que sostuvo la Teoría de las Raíces Nacionales de Szyszlo; el soporte "de punta" del frenesí pop cosmopolita (Acha, Arte Nuevo, Fundación para las Artes, 1966-1969); el soporte estatal velasquista con sus cuatro alternativas (comunicación masiva de Ruiz Durand con su "pop achorado", festivales de arte-total como Contacta e Inkarri, revaloración de lo artesanal, López Antay); y la frustrada búsqueda de un soporte alternativo hacia 1977-1980. El caso central es Huayco E.P.S., cuyo proyecto Sarita Colonia codifica una modernidad sincrética limeña sostenida por una pequeña burguesía ilustrada radicalizada, y cuya dispersión coincide con el agotamiento de la izquierda y el repliegue hacia el mercado galerístico (Forum). El marco conceptual bebe de García Canclini. La tesis es incisiva: el tránsito de la imagen telúrica a la industrial, agraria y migrante revela apropiaciones sucesivas de una idea variable de lo popular, siempre con una radicalidad deficiente y una relación desigual con la cultura interpretada.</t>
         </is>
       </c>
     </row>
@@ -2590,59 +2590,59 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Lama - Los años de la resaca (1983) [Hueso Húmero 18, pdf pp. 136-156].md</t>
+          <t>Freire - Herbert Rodríguez, azote y azúcar con el sistema (1983) [Hueso Húmero 18, pdf pp. 178-185].md</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>1974-1983 (con antecedentes en los años 60-70)</t>
+          <t>1979-1983 (con antecedentes desde 1968)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
+          <t>Reseña crítica en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Luis Lama; Hernán Pazos; Francisco Mariotti; Contacta; grupo Huayco; Juan Javier Salazar; Herbert Rodríguez; Alfonso Castrillón; Escuela Nacional de Bellas Artes; Galería Forum; Galería 9; Ugarte Eléspuru</t>
+          <t>Luis Freire S.; Herbert Rodríguez; Francisco Mariotti; Huayco E.P.S.; Juan Acha; Fernando Bedoya; Juan Javier Salazar; Bienal de Sao Paulo; Galería La Rama Dorada; Galería Forum; EAPUC; ENBAP</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Ensayo de Luis Lama que narra el paso de la "ebullición ideológica" de los años setenta a la "resaca" del segundo belaundismo, articulando historia social del arte y crítica biográfica. La primera parte reconstruye los antecedentes: el terremoto de 1974 y el reflujo de artistas jóvenes hacia Barranco, la gravitación de Francisco Mariotti que transforma el arte de sistemas en movimiento grupal con Contacta e Inkari bajo auspicio de SINAMOS, las tomas y la crisis de la Escuela Nacional de Bellas Artes (1974-1976), y la gestación del taller de Pedro de Osma que devendría núcleo del grupo Huayco (Juan Javier Salazar, Herbert Rodríguez, Charo Noriega, Fernando Bedoya, Lucy Angulo). Lama describe la consolidación paradójica del mercado del arte al amparo de la prohibición de importaciones, con galerías que proliferan mientras la formación académica alcanza sus niveles más bajos. Diagnostica el fin de los happenings sesenteros y el retorno de un expresionismo "de crisis" impulsado desde los predios católicos (Williams, Polanco, Velarde, Hamann), junto a indagaciones matéricas de Wiesse y el conceptualismo de Vainstein. La segunda mitad es un retrato extenso de Hernán Pazos: su formación entre Derecho, la Católica y París, su tránsito del conceptualismo (los cielos y nubes de Galería 9) a la abstracción cromática, las series de los Quipus y los dibujos infantiles, su gestión en Rama Dorada y su individualismo parricida. Lama lo consagra como el artista más destacado de la década, emblema lúcido de las "amargas frustraciones" nacionales bajo el liberalismo económico belaundista.</t>
+          <t>Perfil crítico dedicado a Herbert Rodríguez Huachín en la sección "Individuales" de Hueso Húmero, escrito por Luis Freire, que examina el salto vertiginoso del artista desde la suspensión disciplinaria en la Escuela de Artes Plásticas de la Católica (1981) hasta su presencia en la XVII Bienal de Sao Paulo (1983). Freire sitúa a Rodríguez como imposible de explicar sin el proceso ideológico del populismo velasquista y sin la figura mediadora de Francisco Mariotti, artista suizo-peruano formado en la Documenta de Kassel y la vanguardia europea, catalizador de Contacta y de la EPS Huayco. El texto reconstruye la genealogía Mariotti-Huayco-Rodríguez: los ensamblajes y "reciclajes" del suizo-peruano derivan en los "altares" de Rodríguez, hibridación entre constructivismo geométrico, expresionismo "pobre" y antiestético, y estructuras rituales de la religiosidad popular andina. Argumenta que Rodríguez encarna las contradicciones de una pequeña burguesía radical: dinamita el circuito con una mano y lo enluce con la otra, camuflando "bellamente" materiales pobres y reciclados en obras a la vez contestatarias y comerciables, con lo que ironiza sobre el culto al oficio del arte establecido. Analiza su heterogeneidad de lenguajes (expresionismo abstracto, figuración dura, conceptualismo informal, collage, fotocopia, ensamblaje) como búsqueda pero también como crisis, y sus "altares al Yo" exhibidos en Forum (1983) y la Bienal. Freire lo define como un artista religioso-existencial populista sin referentes sólidos, en formación, tensionado entre enriquecer el jardín burgués que quiere pisotear o saltar a opciones más radicales de ruptura.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/MALI</t>
+          <t>Cap 2 - Historia/Hueso Húmero 18</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - El poder y la ilusión. Pérdida y restauración del aura en la «República de Weimar peruana» 1980-1992 [MALI].md</t>
+          <t>Lama - Los años de la resaca (1983) [Hueso Húmero 18, pdf pp. 136-156].md</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>1980-1992</t>
+          <t>1974-1983 (con antecedentes en los años 60-70)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico (versión MALI), 2013 [escrito 1991-1994]</t>
+          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; E.P.S. Huayco; Taller NN; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; Walter Benjamin; Jesús Ruiz Durand; Andy Warhol; Mirko Lauer; Museo de Arte de Lima (MALI); III Bienal de La Habana</t>
+          <t>Luis Lama; Hernán Pazos; Francisco Mariotti; Contacta; grupo Huayco; Juan Javier Salazar; Herbert Rodríguez; Alfonso Castrillón; Escuela Nacional de Bellas Artes; Galería Forum; Galería 9; Ugarte Eléspuru</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Ensayo seminal de Gustavo Buntinx —redactado entre 1991 y 1994, difundido en inglés en «Beyond the Fantastic» (1995) y publicado por primera vez en Perú en esta versión del MALI (2013)— que interpreta el radical cambio de época del arte peruano entre 1980 y 1992, periodo que denomina metafóricamente «República de Weimar peruana». Su marco conceptual adapta la dialéctica benjaminiana entre proximidad y distancia (el aura, su pérdida por la reproductibilidad técnica y su posible restauración) y las categorías de alegoría, montaje y apropiación de Owens, Foster y Craig Owens a una periferia extrema. El argumento se sostiene sobre el análisis iconográfico minucioso de dos o tres obras que abren y cierran la década. La primera, «Arte al paso» y sobre todo «Sarita Colonia» (1980) del taller E.P.S. Huayco: una enorme estampa de la santa migrante pintada sobre diez mil latas de leche y emplazada en la Panamericana Sur, que Buntinx lee como huaca (post)moderna y exvoto donde lo pequeñoburgués radical se articula figuradamente a lo popular en emergencia (el «pop achorado» y «chicha»). La segunda, «Maorilyn» / «Viva el maoísmo» (1989) del Taller NN: una serigrafía que travistió el rostro de Mao con labios warholianos, alegoría ambivalente de la violencia senderista y la estetización de la política. Su tesis vincula la desintegración social —hiperinflación, guerra civil, movida subte punk— con el desarrollo de una condición alegórica y neo-aurática; su aporte es un modelo teórico para leer el colectivismo y la (post)modernidad popular peruana.</t>
+          <t>Ensayo de Luis Lama que narra el paso de la "ebullición ideológica" de los años setenta a la "resaca" del segundo belaundismo, articulando historia social del arte y crítica biográfica. La primera parte reconstruye los antecedentes: el terremoto de 1974 y el reflujo de artistas jóvenes hacia Barranco, la gravitación de Francisco Mariotti que transforma el arte de sistemas en movimiento grupal con Contacta e Inkari bajo auspicio de SINAMOS, las tomas y la crisis de la Escuela Nacional de Bellas Artes (1974-1976), y la gestación del taller de Pedro de Osma que devendría núcleo del grupo Huayco (Juan Javier Salazar, Herbert Rodríguez, Charo Noriega, Fernando Bedoya, Lucy Angulo). Lama describe la consolidación paradójica del mercado del arte al amparo de la prohibición de importaciones, con galerías que proliferan mientras la formación académica alcanza sus niveles más bajos. Diagnostica el fin de los happenings sesenteros y el retorno de un expresionismo "de crisis" impulsado desde los predios católicos (Williams, Polanco, Velarde, Hamann), junto a indagaciones matéricas de Wiesse y el conceptualismo de Vainstein. La segunda mitad es un retrato extenso de Hernán Pazos: su formación entre Derecho, la Católica y París, su tránsito del conceptualismo (los cielos y nubes de Galería 9) a la abstracción cromática, las series de los Quipus y los dibujos infantiles, su gestión en Rama Dorada y su individualismo parricida. Lama lo consagra como el artista más destacado de la década, emblema lúcido de las "amargas frustraciones" nacionales bajo el liberalismo económico belaundista.</t>
         </is>
       </c>
     </row>
@@ -2654,27 +2654,27 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Lerner - Formando la colección de arte contemporáneo del MALI (2013).txt</t>
+          <t>Buntinx - El poder y la ilusión. Pérdida y restauración del aura en la «República de Weimar peruana» 1980-1992 [MALI].md</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>mediados de los años 60 - 2013 (con foco en 1980-2000)</t>
+          <t>1980-1992</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo de colección, 2013</t>
+          <t>Ensayo académico (versión MALI), 2013 [escrito 1991-1994]</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Museo de Arte de Lima (MALI); Tatiana Cuevas; Miguel A. López; Gustavo Buntinx; Rodrigo Quijano; Jorge Villacorta; Natalia Majluf; E.P.S. Huayco; Teresa Burga; Milagros de la Torre; Flavia Gandolfo</t>
+          <t>Gustavo Buntinx; E.P.S. Huayco; Taller NN; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; Walter Benjamin; Jesús Ruiz Durand; Andy Warhol; Mirko Lauer; Museo de Arte de Lima (MALI); III Bienal de La Habana</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Ensayo introductorio de Sharon Lerner al libro que presenta la colección de arte contemporáneo del Museo de Arte de Lima (MALI), articulado como una lectura —entre muchas posibles— de la historia del arte reciente peruano a partir del acervo. Su tesis metodológica es que en el Perú el tránsito a la contemporaneidad no ocurre como un quiebre radical, sino como una serie de pequeños cambios discontinuos, por lo que la colección se organiza en dos principios: identificar momentos de ruptura de fines del siglo XX y perfilar la producción reciente por ejes temáticos. El recorrido histórico parte de mediados de los sesenta (vanguardias pop, experimentalismo, no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, cuando la migración y la sentencia de Mirko Lauer —«En el Perú, hoy, solo lo popular es moderno»— enmarcan la obra de E.P.S. Huayco. Recorre luego la hegemonía de la abstracción en los ochenta, el arte de derechos humanos de Ricardo Wiesse y Eduardo Villanes bajo el fujimorato, la irrupción de la Bienal Iberoamericana de Lima (1997) y el «bienalismo», y la generación de los 2000 (Flavia Gandolfo, Gilda Mantilla, Armando Andrade Tudela) vinculada al espacio La Culpable. El texto presenta además los ensayos de Miguel López, Gustavo Buntinx y Rodrigo Quijano incluidos en el volumen y la conversación de seis críticos (2011). Su aporte es explicitar la política de adquisiciones del MALI y su ambición de llenar el vacío institucional y discursivo, construyendo un marco regional e internacional para el arte peruano.</t>
+          <t>Ensayo seminal de Gustavo Buntinx —redactado entre 1991 y 1994, difundido en inglés en «Beyond the Fantastic» (1995) y publicado por primera vez en Perú en esta versión del MALI (2013)— que interpreta el radical cambio de época del arte peruano entre 1980 y 1992, periodo que denomina metafóricamente «República de Weimar peruana». Su marco conceptual adapta la dialéctica benjaminiana entre proximidad y distancia (el aura, su pérdida por la reproductibilidad técnica y su posible restauración) y las categorías de alegoría, montaje y apropiación de Owens, Foster y Craig Owens a una periferia extrema. El argumento se sostiene sobre el análisis iconográfico minucioso de dos o tres obras que abren y cierran la década. La primera, «Arte al paso» y sobre todo «Sarita Colonia» (1980) del taller E.P.S. Huayco: una enorme estampa de la santa migrante pintada sobre diez mil latas de leche y emplazada en la Panamericana Sur, que Buntinx lee como huaca (post)moderna y exvoto donde lo pequeñoburgués radical se articula figuradamente a lo popular en emergencia (el «pop achorado» y «chicha»). La segunda, «Maorilyn» / «Viva el maoísmo» (1989) del Taller NN: una serigrafía que travistió el rostro de Mao con labios warholianos, alegoría ambivalente de la violencia senderista y la estetización de la política. Su tesis vincula la desintegración social —hiperinflación, guerra civil, movida subte punk— con el desarrollo de una condición alegórica y neo-aurática; su aporte es un modelo teórico para leer el colectivismo y la (post)modernidad popular peruana.</t>
         </is>
       </c>
     </row>
@@ -2686,27 +2686,27 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - F(r)icciones cosmopolitas. Redefiniciones estéticas y políticas de una idea de vanguardia en los años 60s.txt</t>
+          <t>Lerner - Formando la colección de arte contemporáneo del MALI (2013).txt</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>1960-1976 (con antecedentes desde 1942-1947)</t>
+          <t>mediados de los años 60 - 2013 (con foco en 1980-2000)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico / capítulo de catálogo (MALI), s/f</t>
+          <t>Ensayo de catálogo de colección, 2013</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Emilio Tarazona; Juan Acha; Fernando de Szyszlo; Jorge Romero Brest; Teresa Burga; Rafael Hastings; Grupo Arte Nuevo; Jesús Ruiz Durand; José Gómez Sicre; Marta Traba; Instituto de Arte Contemporáneo (IAC); MoMA / Instituto Di Tella</t>
+          <t>Sharon Lerner; Museo de Arte de Lima (MALI); Tatiana Cuevas; Miguel A. López; Gustavo Buntinx; Rodrigo Quijano; Jorge Villacorta; Natalia Majluf; E.P.S. Huayco; Teresa Burga; Milagros de la Torre; Flavia Gandolfo</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>López reconstruye las mutaciones semánticas y políticas de la noción de vanguardia en el Perú entre los años sesenta y setenta, argumentando que la euforia cosmopolita del periodo fue el espejismo de una modernidad desarrollista tan prometedora como inacabada en un país socialmente fracturado. El objeto de estudio son las plataformas institucionales privadas (IAC, galerías, bienales americanas, concursos empresariales) que, apuntaladas por el panamericanismo de la Guerra Fría, la Alianza para el Progreso y la política curatorial estadounidense de José Gómez Sicre, promovieron primero la abstracción y luego el arte óptico, el pop y las ambientaciones. El texto traza el paso del declive de la abstracción szyszliana hacia el experimentalismo detonado por las conferencias de Jorge Romero Brest (1965) y la irrupción beligerante del grupo Arte Nuevo (1966-1968) contra el Festival Americano de Pintura. El marco conceptual articula la relación entre desarrollismo y vanguardia, y su posterior tensión con el subdesarrollo, siguiendo la radicalización de Juan Acha, quien tras 1968 y el golpe de Velasco redefine la vanguardia como 'guerrilla cultural' y horizonte revolucionario, hasta su exilio a México en 1971. López destaca las reconversiones de Teresa Burga y Rafael Hastings, el 'pop achorado' de Ruiz Durand al servicio de la Reforma Agraria, los festivales Contacta y las Carreras de chasquis. Su aporte es mostrar cómo la condición local, provinciana y periférica de las prácticas de los setenta y ochenta (Paréntesis, E.P.S. Huayco, Grupo Chaclacayo) actualizó de modo radical las pretensiones críticas sesenteras, canibalizando los conceptos metropolitanos de arte conceptual.</t>
+          <t>Ensayo introductorio de Sharon Lerner al libro que presenta la colección de arte contemporáneo del Museo de Arte de Lima (MALI), articulado como una lectura —entre muchas posibles— de la historia del arte reciente peruano a partir del acervo. Su tesis metodológica es que en el Perú el tránsito a la contemporaneidad no ocurre como un quiebre radical, sino como una serie de pequeños cambios discontinuos, por lo que la colección se organiza en dos principios: identificar momentos de ruptura de fines del siglo XX y perfilar la producción reciente por ejes temáticos. El recorrido histórico parte de mediados de los sesenta (vanguardias pop, experimentalismo, no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, cuando la migración y la sentencia de Mirko Lauer —«En el Perú, hoy, solo lo popular es moderno»— enmarcan la obra de E.P.S. Huayco. Recorre luego la hegemonía de la abstracción en los ochenta, el arte de derechos humanos de Ricardo Wiesse y Eduardo Villanes bajo el fujimorato, la irrupción de la Bienal Iberoamericana de Lima (1997) y el «bienalismo», y la generación de los 2000 (Flavia Gandolfo, Gilda Mantilla, Armando Andrade Tudela) vinculada al espacio La Culpable. El texto presenta además los ensayos de Miguel López, Gustavo Buntinx y Rodrigo Quijano incluidos en el volumen y la conversación de seis críticos (2011). Su aporte es explicitar la política de adquisiciones del MALI y su ambición de llenar el vacío institucional y discursivo, construyendo un marco regional e internacional para el arte peruano.</t>
         </is>
       </c>
     </row>
@@ -2718,27 +2718,27 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Quijano - Notas incompletas sobre el sitio de la fotografía peruana.md</t>
+          <t>López, Miguel A. - F(r)icciones cosmopolitas. Redefiniciones estéticas y políticas de una idea de vanguardia en los años 60s.txt</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>1900-2011 (con énfasis en 1920-1998)</t>
+          <t>1960-1976 (con antecedentes desde 1942-1947)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo (MALI), s/f</t>
+          <t>Ensayo académico / capítulo de catálogo (MALI), s/f</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Quijano; Martín Chambi; José María Eguren; Carlos 'Chino' Domínguez; Aaron Siskind; Jesús Ruiz Durand; Claudia Martínez Garay; Daniela Ortiz; Foto Galería Secuencia; TAFOS; Taller NN; E.P.S. Huayco</t>
+          <t>Miguel A. López; Emilio Tarazona; Juan Acha; Fernando de Szyszlo; Jorge Romero Brest; Teresa Burga; Rafael Hastings; Grupo Arte Nuevo; Jesús Ruiz Durand; José Gómez Sicre; Marta Traba; Instituto de Arte Contemporáneo (IAC); MoMA / Instituto Di Tella</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Quijano ensaya una genealogía del 'sitio' de la fotografía peruana, sosteniendo que este medio inauguró un margen de creación moderno al margen de la institucionalidad académica de las bellas artes, alcanzando una temprana ubicuidad territorial y una masividad que condicionó la percepción misma de una realidad nacional. El texto, de estructura fragmentaria y numerada, contrapone dos matrices fundacionales: Martín Chambi como 'modernista sin modernidad' y profesional de la imagen surgido de una familia campesina andina —una 'oportunidad nacional'— frente a la miniatura pinhole intimista y hermética de José María Eguren, que prefigura la figura del fotógrafo-artista individual. Analiza a Carlos 'Chino' Domínguez como ojo testimonial de la urbanización y la nueva cultura popular (La resaca del Inca, el 'Cholo' Sotil, el filme Cholo y su reedición Mi cholo de Gruenberg), y la experiencia de la fotogalería Secuencia (1977-1980), que reinventó una tradición y un discurso del oficio adoptando a Minor White y Aaron Siskind. El marco conceptual enlaza fotografía, prensa y democratización de la imagen en el contexto del auge sindical y la repolitización popular de fines de los setenta, y la aparición de la fotoserigrafía disidente (Bedoya, Williams, Mariotti, Salazar) como catalizador de una nueva condición fotográfica colectiva, desde E.P.S. Huayco hasta el Taller NN. El aporte del texto es leer la fotografía como dispositivo de documento, archivo, memoria y duelo frente a la violencia política (Uchuraccay, Yuyanapaq), rastreando su 'grado cero' icónico en obras de Ruiz Durand, Claudia Martínez Garay y Daniela Ortiz, que develan la mirada colonial y la invisibilización étnica.</t>
+          <t>López reconstruye las mutaciones semánticas y políticas de la noción de vanguardia en el Perú entre los años sesenta y setenta, argumentando que la euforia cosmopolita del periodo fue el espejismo de una modernidad desarrollista tan prometedora como inacabada en un país socialmente fracturado. El objeto de estudio son las plataformas institucionales privadas (IAC, galerías, bienales americanas, concursos empresariales) que, apuntaladas por el panamericanismo de la Guerra Fría, la Alianza para el Progreso y la política curatorial estadounidense de José Gómez Sicre, promovieron primero la abstracción y luego el arte óptico, el pop y las ambientaciones. El texto traza el paso del declive de la abstracción szyszliana hacia el experimentalismo detonado por las conferencias de Jorge Romero Brest (1965) y la irrupción beligerante del grupo Arte Nuevo (1966-1968) contra el Festival Americano de Pintura. El marco conceptual articula la relación entre desarrollismo y vanguardia, y su posterior tensión con el subdesarrollo, siguiendo la radicalización de Juan Acha, quien tras 1968 y el golpe de Velasco redefine la vanguardia como 'guerrilla cultural' y horizonte revolucionario, hasta su exilio a México en 1971. López destaca las reconversiones de Teresa Burga y Rafael Hastings, el 'pop achorado' de Ruiz Durand al servicio de la Reforma Agraria, los festivales Contacta y las Carreras de chasquis. Su aporte es mostrar cómo la condición local, provinciana y periférica de las prácticas de los setenta y ochenta (Paréntesis, E.P.S. Huayco, Grupo Chaclacayo) actualizó de modo radical las pretensiones críticas sesenteras, canibalizando los conceptos metropolitanos de arte conceptual.</t>
         </is>
       </c>
     </row>
@@ -2750,32 +2750,64 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
+          <t>Quijano - Notas incompletas sobre el sitio de la fotografía peruana.md</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>1900-2011 (con énfasis en 1920-1998)</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Ensayo de catálogo (MALI), s/f</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>Rodrigo Quijano; Martín Chambi; José María Eguren; Carlos 'Chino' Domínguez; Aaron Siskind; Jesús Ruiz Durand; Claudia Martínez Garay; Daniela Ortiz; Foto Galería Secuencia; TAFOS; Taller NN; E.P.S. Huayco</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Quijano ensaya una genealogía del 'sitio' de la fotografía peruana, sosteniendo que este medio inauguró un margen de creación moderno al margen de la institucionalidad académica de las bellas artes, alcanzando una temprana ubicuidad territorial y una masividad que condicionó la percepción misma de una realidad nacional. El texto, de estructura fragmentaria y numerada, contrapone dos matrices fundacionales: Martín Chambi como 'modernista sin modernidad' y profesional de la imagen surgido de una familia campesina andina —una 'oportunidad nacional'— frente a la miniatura pinhole intimista y hermética de José María Eguren, que prefigura la figura del fotógrafo-artista individual. Analiza a Carlos 'Chino' Domínguez como ojo testimonial de la urbanización y la nueva cultura popular (La resaca del Inca, el 'Cholo' Sotil, el filme Cholo y su reedición Mi cholo de Gruenberg), y la experiencia de la fotogalería Secuencia (1977-1980), que reinventó una tradición y un discurso del oficio adoptando a Minor White y Aaron Siskind. El marco conceptual enlaza fotografía, prensa y democratización de la imagen en el contexto del auge sindical y la repolitización popular de fines de los setenta, y la aparición de la fotoserigrafía disidente (Bedoya, Williams, Mariotti, Salazar) como catalizador de una nueva condición fotográfica colectiva, desde E.P.S. Huayco hasta el Taller NN. El aporte del texto es leer la fotografía como dispositivo de documento, archivo, memoria y duelo frente a la violencia política (Uchuraccay, Yuyanapaq), rastreando su 'grado cero' icónico en obras de Ruiz Durand, Claudia Martínez Garay y Daniela Ortiz, que develan la mirada colonial y la invisibilización étnica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Cap 2 - Historia/MALI</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
           <t>Villacorta (ed.) - ¿Un arte visual a contrapelo de los dictados metropolitanos? En el Perú, el arte moderno es un gesto tardío [conversación en el MALI, 2011].txt</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>1947-2011 (con eje en 1960-2002)</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>Transcripción editada de conversación (MALI), 2011</t>
         </is>
       </c>
-      <c r="E72" s="3" t="inlineStr">
+      <c r="E73" s="3" t="inlineStr">
         <is>
           <t>Jorge Villacorta; Gustavo Buntinx; Miguel A. López; Rodrigo Quijano; Tatiana Cuevas; Natalia Majluf; E.P.S. Huayco; Grupo Arte Nuevo; Taller NN; Grupo Chaclacayo; Christian Bendayán; Fernando Bryce; MALI / Micromuseo</t>
         </is>
       </c>
-      <c r="F72" s="3" t="inlineStr">
+      <c r="F73" s="3" t="inlineStr">
         <is>
           <t>Editada por Villacorta a partir de dos sesiones de 2011 en el MALI, esta conversación a seis voces indaga si lo moderno está clausurado en el arte peruano de modo que permita definir lo contemporáneo. La tesis articuladora, propuesta por Quijano, es que en el Perú lo moderno solo ha podido darse 'a contrapelo' y como 'gesto tardío', a destiempo de las modernidades metropolitanas; López y Buntinx la matizan con la idea de temporalidades dislocadas y friccionadas que impiden toda historia lineal. El objeto de estudio es la genealogía de la vanguardia local: la contraposición entre Arte Nuevo (1966-1968), leído como destello cosmopolita fugaz, y E.P.S. Huayco y Paréntesis, cuya apropiación de Sarita Colonia y el 'pop achorado' marca una ruptura más perdurable y pertinente al medio. Buntinx despliega una secuencia estilístico-conceptual en clave pop/místico-libidinal —de la Twiggy de Emilio Hernández a Quistococha de Bendayán, pasando por el afiche de Ruiz Durand, la Maoirilyn del Taller NN y La Pachakuti de Alfredo Márquez— ligada a periodos políticos (desarrollismo, velasquismo, utopía socialista, dictadura fujimorista, revolución capitalista). Majluf sitúa el quiebre epocal de fin de siglo en el ingreso de la 'referencia' fotográfica (Bryce, Milagros de la Torre, Juan Enrique Bedoya, Mantilla), frente al neobarroco. El texto discute además la construcción de públicos, la institucionalidad faltante, el rol del curador, el mercado 'social' peruano, las subastas del MALI y la 'normalización de la diferencia' como riesgo de la consagración institucional del pasado radical.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F72"/>
+  <autoFilter ref="A1:F73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Añade y cataloga el volante de Mirko Lauer «Arte al paso / Tome uno» (1980)
- Sube a Cap 2 - Historia la transcripción del volante de Mirko Lauer que
  acompañó la exposición de E.P.S. Huayco en la Galería Forum (Lima, mayo
  de 1980), transcrito desde una fotografía del original.
- Lo cataloga en tabla-cap2-historia.csv (Cap 2 pasa a 73 filas) y
  regenera tablas-sistematizacion.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bob4w11uQRyAcv1Qayw1V
</commit_message>
<xml_diff>
--- a/Sistematización/tablas-sistematizacion.xlsx
+++ b/Sistematización/tablas-sistematizacion.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Extras" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cap 3 - Análisis'!$A$1:$F$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Teoría'!$A$1:$F$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Extras'!$A$1:$F$4</definedName>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1502,27 +1502,27 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. (ed.) - Hay algo incomestible en la garganta. Poéticas antipatriarcales y nueva escena en los años noventa (2021) [catálogo ICPNA].md</t>
+          <t>Lauer, Mirko - Arte al paso, Tome uno (1980) [volante Galería Forum, E.P.S. Huayco].md</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>1988-2002</t>
+          <t>1980 (exposición Arte al paso, E.P.S. Huayco; contexto de la plástica joven peruana de fin de los años 70)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de exposición, 2021</t>
+          <t>Volante/panfleto de exposición, mayo de 1980 (Galería Forum, Lima); transcripción manual de fotografía, 2026</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López (curaduría); Issela Ccoyllo; Carmen Ilizarbe; Susana Torres; María Eugenia Yllia; Montserrat Álvarez; Irene Rojas; Elena Tejada-Herrera; Natalia Iguíñiz; Flavia Gandolfo; Movimiento Manuela Ramos / TAFOS; ICPNA</t>
+          <t>Mirko Lauer (texto); E.P.S. Huayco; María Luy; Francisco Mariotti; Charo Noriega; Juan Javier Salazar; Mariela Zevallos; Guillermo Orbegoso; Roberto Cores; Galería Forum</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Catálogo bilingüe de la exposición homónima curada por Miguel A. López en el ICPNA de Lima con motivo del Bicentenario, que reúne más de doscientas obras de cerca de noventa creadoras, colectivas y talleres para examinar la producción visual y las transformaciones sociopolíticas peruanas entre 1988 y 2002. Su tesis central sostiene que, al cierre del siglo XX, fueron las mujeres y los cuerpos feminizados quienes reorientaron el rumbo del arte, desplegando lo que López denomina «poéticas antipatriarcales»: vocabularios estéticos surgidos para enfrentar una misoginia naturalizada y la violencia colonial, racial y patriarcal. El marco conceptual articula feminismo, crítica al neoliberalismo (el «hechizo» de la privatización y el individualismo), teoría social del arte y una lectura de clase del campo cultural, rechazando una absorción de la heterogeneidad bajo la categoría occidental de «arte». El proyecto yuxtapone deliberadamente circuitos antagónicos: obras de galerías, museos y bienales junto a arpilleras de asociaciones de mujeres y clubes de madres, los Talleres de Fotografía Social (TAFOS) y el proyecto Mercomujer del Movimiento Manuela Ramos. Se organiza en diez ejes temáticos (autorrepresentación, misoginia, deseo y disidencia de género, políticas de cuidado, acción colectiva, poder androcéntrico, reciprocidad, cuerpos gestantes, pieles e hilos, violencia política) y ensayos complementarios de Susana Torres, Issela Ccoyllo, María Eugenia Yllia y Carmen Ilizarbe. Su aporte reside en construir una genealogía transfeminista que rescata prácticas invisibilizadas —arpilleristas migrantes, artistas indígenas y campesinas, transformismo, autogestión— y las inscribe como agentes decisivas de la reconfiguración de la esfera pública peruana frente a la dictadura fujimorista.</t>
+          <t>Volante o panfleto bifronte («Arte al paso» / «Tome uno») escrito por Mirko Lauer para acompañar la exposición homónima del colectivo E.P.S. Huayco en la Galería Forum de Lima (mayo de 1980); el proyecto reúne a María Luy, Francisco Mariotti, Charo Noriega, Juan Javier Salazar y Mariela Zevallos, con fotografías de Guillermo Orbegoso y Roberto Cores. El texto, organizado como una serie de definiciones anafóricas («Arte al paso: …»), es un manifiesto programático del no-objetualismo peruano y del arte crítico. Lauer presenta la obra como una «contestación» que combina serigrafía, detritus industriales, fórmulas teóricas, fotos y «expendio de salchipapas» para sostener que «la realidad del arte es más compleja que la realidad de las 'Bellas Artes'». Articula tres operaciones críticas: contra el mercado y las galerías como «escaparates» de la transacción comercial; contra los «métodos religioso-expresionistas» que enseñan a «sentir y no pensar»; y contra «una falsa modernidad de importación», rematando con la consigna que se volvería célebre: «Sólo lo popular es realmente moderno hoy en el Perú». Reivindica el trabajo colectivo frente al «aislamiento» y el «desamparo teórico» del plástico joven, propone un «ejercicio ecológico» que revela el «cordón umbilical» entre los desechos de la ciudad y su arte, y ancla la práctica en «esa realidad fundamental del arte en América Latina que es la miseria». Contra el «arte bobo», postula un arte popular, político y antipublicitario. Constituye una fuente primaria clave para la historia del arte crítico y no-objetual peruano de fines de los años setenta e inicios de los ochenta.</t>
         </is>
       </c>
     </row>
@@ -1534,27 +1534,27 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - How Do We Know What Latin American Conceptualism Looks Like?.md</t>
+          <t>López, Miguel A. (ed.) - Hay algo incomestible en la garganta. Poéticas antipatriarcales y nueva escena en los años noventa (2021) [catálogo ICPNA].md</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>años 60-70 (con foco en 1968: Tucumán Arde)</t>
+          <t>1988-2002</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico (Afterall), ca. 2010</t>
+          <t>Catálogo de exposición, 2021</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Mari Carmen Ramírez; Luis Camnitzer; Jane Farver; Rachel Weiss; Paul B. (Beatriz) Preciado; Graciela Carnevale; Ana Longoni; Fernando Davis; Eduardo Costa; Roberto Jacoby; Queens Museum of Art / MoMA / Red Conceptualismos del Sur</t>
+          <t>Miguel A. López (curaduría); Issela Ccoyllo; Carmen Ilizarbe; Susana Torres; María Eugenia Yllia; Montserrat Álvarez; Irene Rojas; Elena Tejada-Herrera; Natalia Iguíñiz; Flavia Gandolfo; Movimiento Manuela Ramos / TAFOS; ICPNA</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Ensayo historiográfico de Miguel A. López que problematiza cómo se ha construido y estabilizado la categoría «conceptualismo latinoamericano». Su objeto de estudio son los dispositivos discursivos y expositivos que fijaron una imagen canónica de la producción crítica de los años sesenta y setenta, tomando como bisagras la muestra «Global Conceptualism: Points of Origin» (Queens Museum, 1999) y el ensayo fundacional «Blueprint Circuits» (1993) de Mari Carmen Ramírez. El marco conceptual proviene de una crítica queer de la representación: siguiendo a Paul B. Preciado y a Guattari, López contrapone una «cartografía de identidades» —que rastrea, clasifica y verifica obras conceptuales— a una «cartografía crítica» que expone las relaciones de poder y las tecnologías de producción de subjetividad implicadas en el acto de historizar. Argumenta que la distinción binaria entre un conceptualismo «analítico» anglosajón (Kosuth) y uno «ideológico» latinoamericano, consolidada por Ramírez y repetida por Osborne y Alberro, reinscribe la lógica centro/periferia que dice combatir y fija un estereotipo de arte subversivo. El texto examina la mitificación de «Tucumán Arde» (1968) y su recuperación en la exposición «Inventario 1965-1975. Archivo Graciela Carnevale» (Rosario, 2008), primer experimento curatorial de la Red Conceptualismos del Sur, que activa el archivo para desmontar la narrativa única. Recupera conceptos «menores» (desmaterialización de Masotta, no-objetualismo de Acha, deshabituación de Carreira) y cierra con la pieza de Eduardo Costa: su aporte es proponer una historiografía infiel, anacrónica y desestabilizadora que traicione las certezas del relato consensual.</t>
+          <t>Catálogo bilingüe de la exposición homónima curada por Miguel A. López en el ICPNA de Lima con motivo del Bicentenario, que reúne más de doscientas obras de cerca de noventa creadoras, colectivas y talleres para examinar la producción visual y las transformaciones sociopolíticas peruanas entre 1988 y 2002. Su tesis central sostiene que, al cierre del siglo XX, fueron las mujeres y los cuerpos feminizados quienes reorientaron el rumbo del arte, desplegando lo que López denomina «poéticas antipatriarcales»: vocabularios estéticos surgidos para enfrentar una misoginia naturalizada y la violencia colonial, racial y patriarcal. El marco conceptual articula feminismo, crítica al neoliberalismo (el «hechizo» de la privatización y el individualismo), teoría social del arte y una lectura de clase del campo cultural, rechazando una absorción de la heterogeneidad bajo la categoría occidental de «arte». El proyecto yuxtapone deliberadamente circuitos antagónicos: obras de galerías, museos y bienales junto a arpilleras de asociaciones de mujeres y clubes de madres, los Talleres de Fotografía Social (TAFOS) y el proyecto Mercomujer del Movimiento Manuela Ramos. Se organiza en diez ejes temáticos (autorrepresentación, misoginia, deseo y disidencia de género, políticas de cuidado, acción colectiva, poder androcéntrico, reciprocidad, cuerpos gestantes, pieles e hilos, violencia política) y ensayos complementarios de Susana Torres, Issela Ccoyllo, María Eugenia Yllia y Carmen Ilizarbe. Su aporte reside en construir una genealogía transfeminista que rescata prácticas invisibilizadas —arpilleristas migrantes, artistas indígenas y campesinas, transformismo, autogestión— y las inscribe como agentes decisivas de la reconfiguración de la esfera pública peruana frente a la dictadura fujimorista.</t>
         </is>
       </c>
     </row>
@@ -1566,27 +1566,27 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - Los feminismos van a vencer. Una introducción [con presentación de Claudia Salazar Jiménez, dic. 2018].md</t>
+          <t>López, Miguel A. - How Do We Know What Latin American Conceptualism Looks Like?.md</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>años 60-90 (textos escritos 2012-2018; activismo 2015-2018)</t>
+          <t>años 60-70 (con foco en 1968: Tucumán Arde)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Introducción de libro, 2018</t>
+          <t>Artículo académico (Afterall), ca. 2010</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Claudia Salazar Jiménez; Rita Segato; Frantz Fanon; Julia Bryan-Wilson; Gladys Tzul Tzul; Aníbal Quijano; Paul B. Preciado; Giuseppe Campuzano; Víctor Manuel Rodríguez; TEOR/éTica / MACBA</t>
+          <t>Miguel A. López; Mari Carmen Ramírez; Luis Camnitzer; Jane Farver; Rachel Weiss; Paul B. (Beatriz) Preciado; Graciela Carnevale; Ana Longoni; Fernando Davis; Eduardo Costa; Roberto Jacoby; Queens Museum of Art / MoMA / Red Conceptualismos del Sur</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Texto introductorio de López al libro que reúne sus ensayos sobre poéticas antipatriarcales (escritos entre 2012 y 2018), precedido por una presentación de la escritora Claudia Salazar Jiménez. Su tesis define los feminismos no como una identidad ni un periodo, sino como una «metodología para mirar» y un método de investigación afectivo: una política del afecto, la escucha y la resistencia colectiva que redefine el horizonte de acción y desconfía del esencialismo identitario. El marco conceptual entrelaza la «pedagogía de la crueldad» y el «mandato de la masculinidad» de Rita Segato, la distinción de Fanon entre «zona del ser» y «zona del no-ser», la «colonialidad del poder» de Aníbal Quijano y el «modelo metodológico afectivo» de Julia Bryan-Wilson, junto a referencias a Gladys Tzul Tzul y Paul B. Preciado. López sostiene que el arte, la performance y la escritura funcionan como refugio y resistencia frente a la exclusión, y que la tarea no es incorporar episodios omitidos a un inventario, sino analizar las condiciones políticas, materiales y afectivas que hacen emerger ciertas representaciones. Discute críticamente el rol de los museos como lugares de disputa capaces de redefinir la esfera pública, apoyándose en su experiencia en el MACBA y en la dirección colectiva de TEOR/éTica. Situado geopolíticamente en Lima pero atento a sus ausencias (la Amazonía, las provincias, el centralismo), el ensayo propone una genealogía transfeminista de la cultura visual que reactive «parientes extraviados» y reorganice la historia del arte como reserva de sororidad y alianzas.</t>
+          <t>Ensayo historiográfico de Miguel A. López que problematiza cómo se ha construido y estabilizado la categoría «conceptualismo latinoamericano». Su objeto de estudio son los dispositivos discursivos y expositivos que fijaron una imagen canónica de la producción crítica de los años sesenta y setenta, tomando como bisagras la muestra «Global Conceptualism: Points of Origin» (Queens Museum, 1999) y el ensayo fundacional «Blueprint Circuits» (1993) de Mari Carmen Ramírez. El marco conceptual proviene de una crítica queer de la representación: siguiendo a Paul B. Preciado y a Guattari, López contrapone una «cartografía de identidades» —que rastrea, clasifica y verifica obras conceptuales— a una «cartografía crítica» que expone las relaciones de poder y las tecnologías de producción de subjetividad implicadas en el acto de historizar. Argumenta que la distinción binaria entre un conceptualismo «analítico» anglosajón (Kosuth) y uno «ideológico» latinoamericano, consolidada por Ramírez y repetida por Osborne y Alberro, reinscribe la lógica centro/periferia que dice combatir y fija un estereotipo de arte subversivo. El texto examina la mitificación de «Tucumán Arde» (1968) y su recuperación en la exposición «Inventario 1965-1975. Archivo Graciela Carnevale» (Rosario, 2008), primer experimento curatorial de la Red Conceptualismos del Sur, que activa el archivo para desmontar la narrativa única. Recupera conceptos «menores» (desmaterialización de Masotta, no-objetualismo de Acha, deshabituación de Carreira) y cierra con la pieza de Eduardo Costa: su aporte es proponer una historiografía infiel, anacrónica y desestabilizadora que traicione las certezas del relato consensual.</t>
         </is>
       </c>
     </row>
@@ -1598,27 +1598,27 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - Parientes extraviados, Cuerpo vehículo político y A contratiempo. Tres ensayos sobre poéticas antipatriarcales.md</t>
+          <t>López, Miguel A. - Los feminismos van a vencer. Una introducción [con presentación de Claudia Salazar Jiménez, dic. 2018].md</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>años 60-80 (con proyección al presente)</t>
+          <t>años 60-90 (textos escritos 2012-2018; activismo 2015-2018)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Capítulos de libro, 2019</t>
+          <t>Introducción de libro, 2018</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Teresa Burga; Gloria Gómez-Sánchez; Cristina Portocarrero; Victoria Santa Cruz; Johanna Hamann; Tilsa Tsuchiya; Marisa Godínez; María T-Ta (María Roncal); Grupo Chaclacayo; ALIMUPER / Movimiento Manuela Ramos / Centro Flora Tristán</t>
+          <t>Miguel A. López; Claudia Salazar Jiménez; Rita Segato; Frantz Fanon; Julia Bryan-Wilson; Gladys Tzul Tzul; Aníbal Quijano; Paul B. Preciado; Giuseppe Campuzano; Víctor Manuel Rodríguez; TEOR/éTica / MACBA</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Conjunto de tres ensayos de López que trazan una genealogía de poéticas antipatriarcales en el arte peruano entre los años sesenta y ochenta, entendidas como «parientes extraviados» de las luchas feministas y sexodisidentes actuales. «Parientes extraviados» reconstruye la contribución de las artistas mujeres al experimentalismo: las ambientaciones y objetos de Teresa Burga y Gloria Gómez-Sánchez en el grupo Arte Nuevo (1966-1968), que desmantelaban el régimen masculino de la mirada; el tránsito de Cristina Portocarrero del arte a la militancia en ALIMUPER; y la revaloración de las artes de tradición andina (Apolonia Dorregaray) bajo el velasquismo. «Cuerpo, vehículo político» analiza cómo diversas creadoras abandonaron pintura y escultura para usar el propio cuerpo como crítica: el «Antiballet» de Yvonne von Mollendorff, el «Autorretrato» clínico de Burga (1972), la declamación antirracista «Me gritaron negra» de Victoria Santa Cruz, las «Barrigas» de Johanna Hamann y la gráfica militante de Marisa Godínez para Flora Tristán. Aborda además la teatralidad, el travestismo y lo performativo de los ochenta —Grupo Chaclacayo, Jaime Higa, la escena drag documentada por Flavia Gandolfo, la punk María T-Ta, Támira Bassallo, Susana Torres— como respuestas a una guerra tanto armada como misógina y homofóbica. El tercer ensayo, «A contratiempo», explora las «cronodisidencias» de Burga y su temporalidad improductiva del dibujo. El marco conceptual moviliza teoría feminista y queer (Preciado, Bryan-Wilson, Richard); su aporte es reinscribir prácticas borradas como antagonismo estético-político y desmentir el diagnóstico de su supuesta inexistencia.</t>
+          <t>Texto introductorio de López al libro que reúne sus ensayos sobre poéticas antipatriarcales (escritos entre 2012 y 2018), precedido por una presentación de la escritora Claudia Salazar Jiménez. Su tesis define los feminismos no como una identidad ni un periodo, sino como una «metodología para mirar» y un método de investigación afectivo: una política del afecto, la escucha y la resistencia colectiva que redefine el horizonte de acción y desconfía del esencialismo identitario. El marco conceptual entrelaza la «pedagogía de la crueldad» y el «mandato de la masculinidad» de Rita Segato, la distinción de Fanon entre «zona del ser» y «zona del no-ser», la «colonialidad del poder» de Aníbal Quijano y el «modelo metodológico afectivo» de Julia Bryan-Wilson, junto a referencias a Gladys Tzul Tzul y Paul B. Preciado. López sostiene que el arte, la performance y la escritura funcionan como refugio y resistencia frente a la exclusión, y que la tarea no es incorporar episodios omitidos a un inventario, sino analizar las condiciones políticas, materiales y afectivas que hacen emerger ciertas representaciones. Discute críticamente el rol de los museos como lugares de disputa capaces de redefinir la esfera pública, apoyándose en su experiencia en el MACBA y en la dirección colectiva de TEOR/éTica. Situado geopolíticamente en Lima pero atento a sus ausencias (la Amazonía, las provincias, el centralismo), el ensayo propone una genealogía transfeminista de la cultura visual que reactive «parientes extraviados» y reorganice la historia del arte como reserva de sororidad y alianzas.</t>
         </is>
       </c>
     </row>
@@ -1630,27 +1630,27 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Mesa - Arte contemporáneo peruano. Portocarrero, Aramburu y Lerner (2022) [MALBA].transcripcion.md</t>
+          <t>López, Miguel A. - Parientes extraviados, Cuerpo vehículo político y A contratiempo. Tres ensayos sobre poéticas antipatriarcales.md</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>1930-2022 (con énfasis en 1976-2022)</t>
+          <t>años 60-80 (con proyección al presente)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Transcripción de mesa redonda (MALBA/MALVA), 2022</t>
+          <t>Capítulos de libro, 2019</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Florencia Portocarrero; Iosu Aramburu; Verónica Rossi; Ana Teresa Barboza; Mirko Lauer; Joaquín López Antay; Miguel Aguirre; Elvia Paucar; Centro de Textiles Tradicionales del Cusco; MALI</t>
+          <t>Miguel A. López; Teresa Burga; Gloria Gómez-Sánchez; Cristina Portocarrero; Victoria Santa Cruz; Johanna Hamann; Tilsa Tsuchiya; Marisa Godínez; María T-Ta (María Roncal); Grupo Chaclacayo; ALIMUPER / Movimiento Manuela Ramos / Centro Flora Tristán</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Transcripción (borrador sin refinar) de una mesa redonda organizada en torno a la exposición 'Tejer las Piedras' de Ana Teresa Barboza, que toma el pulso a los debates del arte contemporáneo peruano actual, con foco en la relación entre arte y artesanía. Sharon Lerner abre con un recorrido por veinte años de la obra de Barboza, desde el bordado autobiográfico de cuerpos y heridas —leído por Gabriela Germaná y Augusto del Valle como inversión de la representación sexista— hacia un trabajo colaborativo con tejido, telar de cintura y tintes naturales que reflexiona sobre paisaje, sostenibilidad y territorio, situándolo en la tradición anglosajona del craft y en la reinserción de lo personal, según Whitney Chadwick, característica del feminismo desde los setenta. Portocarrero y Aramburu estructuran su intervención con los tres 'universos estéticos' de Mirko Lauer (precolombino, erudito/bellas artes, tradicional/popular), entendidos como compartimentos estancos ligados a una estructura colonial y racista, y examinan sus cruces históricos: el Instituto de Arte Peruano indigenista, la apropiación de lo prehispánico en los sesenta, el escándalo del Premio Nacional a Joaquín López Antay (1976). El marco conceptual sostiene que, a diferencia de aquel premio otorgado por un jurado, artistas indígenas contemporáneos como Venuca Evanán y Chonon Bensho hoy postulan conscientemente e ingresan por agencia propia a los circuitos del arte contemporáneo. Se analizan la colaboración de largo aliento entre Miguel Aguirre y la tejedora Elvia Paucar y el proyecto Ser Payay en Cusco, como casos de 'vocabularios colaborados' que problematizan la coautoría, la mediación y las lógicas de mercado diferenciadas entre arte y artesanía.</t>
+          <t>Conjunto de tres ensayos de López que trazan una genealogía de poéticas antipatriarcales en el arte peruano entre los años sesenta y ochenta, entendidas como «parientes extraviados» de las luchas feministas y sexodisidentes actuales. «Parientes extraviados» reconstruye la contribución de las artistas mujeres al experimentalismo: las ambientaciones y objetos de Teresa Burga y Gloria Gómez-Sánchez en el grupo Arte Nuevo (1966-1968), que desmantelaban el régimen masculino de la mirada; el tránsito de Cristina Portocarrero del arte a la militancia en ALIMUPER; y la revaloración de las artes de tradición andina (Apolonia Dorregaray) bajo el velasquismo. «Cuerpo, vehículo político» analiza cómo diversas creadoras abandonaron pintura y escultura para usar el propio cuerpo como crítica: el «Antiballet» de Yvonne von Mollendorff, el «Autorretrato» clínico de Burga (1972), la declamación antirracista «Me gritaron negra» de Victoria Santa Cruz, las «Barrigas» de Johanna Hamann y la gráfica militante de Marisa Godínez para Flora Tristán. Aborda además la teatralidad, el travestismo y lo performativo de los ochenta —Grupo Chaclacayo, Jaime Higa, la escena drag documentada por Flavia Gandolfo, la punk María T-Ta, Támira Bassallo, Susana Torres— como respuestas a una guerra tanto armada como misógina y homofóbica. El tercer ensayo, «A contratiempo», explora las «cronodisidencias» de Burga y su temporalidad improductiva del dibujo. El marco conceptual moviliza teoría feminista y queer (Preciado, Bryan-Wilson, Richard); su aporte es reinscribir prácticas borradas como antagonismo estético-político y desmentir el diagnóstico de su supuesta inexistencia.</t>
         </is>
       </c>
     </row>
@@ -1662,27 +1662,27 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Mesa - Coleccionando desde la institución (2025) [Charlas de colección, Foro Pinta Lima].transcripcion.md</t>
+          <t>Mesa - Arte contemporáneo peruano. Portocarrero, Aramburu y Lerner (2022) [MALBA].transcripcion.md</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>1960s-2025 (con eje en 2006-2025)</t>
+          <t>1930-2022 (con énfasis en 1976-2022)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Transcripción de conversatorio (Foro Pinta Lima 2025), 2025</t>
+          <t>Transcripción de mesa redonda (MALBA/MALVA), 2022</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Pablo León de la Barra; Sharon Lerner; Manuel Segade; MALI; Museo Reina Sofía; Museo Guggenheim; Comité de Adquisiciones de Arte Contemporáneo del MALI; Suset Sánchez; Amanda de la Garza; Tatiana Cuevas; Fundación Museo Reina Sofía</t>
+          <t>Sharon Lerner; Florencia Portocarrero; Iosu Aramburu; Verónica Rossi; Ana Teresa Barboza; Mirko Lauer; Joaquín López Antay; Miguel Aguirre; Elvia Paucar; Centro de Textiles Tradicionales del Cusco; MALI</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Transcripción (borrador) del conversatorio 'Coleccionando desde la institución' del Foro Pinta Lima 2025, moderado por Pablo León de la Barra (Guggenheim), que confronta dos modelos museales públicos: el MALI de Lima y el Museo Reina Sofía de Madrid. La tesis compartida es que coleccionar implica un pensamiento crítico que puede cuestionar el canon, reparar asimetrías históricas de género, raza e identidad y llenar vacíos. Sharon Lerner expone la trayectoria del Comité de Adquisiciones de Arte Contemporáneo del MALI (casi veinte años, modelado sobre el Latin American Acquisitions Committee de la Tate), la curaduría contemporánea iniciada por Tatiana Cuevas en 2008, y el trabajo 'trenzado' entre colección histórica y contemporánea que atraviesa exposiciones como Arte al Paso, Amazonías y Otras historias posibles, y la reestructuración pospandemia con el programa Salas Abiertas. Detalla la visibilización de artistas amazónicos e indígenas (Sara Flores, Chonon Bensho, Venuca Evanán), la incorporación del textil y proyectos como Línea de Vida de Giuseppe Campuzano, junto a comisiones y trabajo comunitario con Cantagallo. Manuel Segade analiza la dimensión colonial del Reina Sofía —cuya colección latinoamericana se inauguró en 1992— y las condiciones estructurales, funcionariales y presupuestarias que la condicionan, citando las preguntas ontológicas de Suset Sánchez y el Instituto Cader de arte centroamericano como vía de restitución frente al extractivismo cultural. El diálogo aborda el rol de los públicos, la crispación política, la censura, el cierre del Lugar de la Memoria y la misión histórica del museo como plataforma de tensiones críticas de la sociedad civil.</t>
+          <t>Transcripción (borrador sin refinar) de una mesa redonda organizada en torno a la exposición 'Tejer las Piedras' de Ana Teresa Barboza, que toma el pulso a los debates del arte contemporáneo peruano actual, con foco en la relación entre arte y artesanía. Sharon Lerner abre con un recorrido por veinte años de la obra de Barboza, desde el bordado autobiográfico de cuerpos y heridas —leído por Gabriela Germaná y Augusto del Valle como inversión de la representación sexista— hacia un trabajo colaborativo con tejido, telar de cintura y tintes naturales que reflexiona sobre paisaje, sostenibilidad y territorio, situándolo en la tradición anglosajona del craft y en la reinserción de lo personal, según Whitney Chadwick, característica del feminismo desde los setenta. Portocarrero y Aramburu estructuran su intervención con los tres 'universos estéticos' de Mirko Lauer (precolombino, erudito/bellas artes, tradicional/popular), entendidos como compartimentos estancos ligados a una estructura colonial y racista, y examinan sus cruces históricos: el Instituto de Arte Peruano indigenista, la apropiación de lo prehispánico en los sesenta, el escándalo del Premio Nacional a Joaquín López Antay (1976). El marco conceptual sostiene que, a diferencia de aquel premio otorgado por un jurado, artistas indígenas contemporáneos como Venuca Evanán y Chonon Bensho hoy postulan conscientemente e ingresan por agencia propia a los circuitos del arte contemporáneo. Se analizan la colaboración de largo aliento entre Miguel Aguirre y la tejedora Elvia Paucar y el proyecto Ser Payay en Cusco, como casos de 'vocabularios colaborados' que problematizan la coautoría, la mediación y las lógicas de mercado diferenciadas entre arte y artesanía.</t>
         </is>
       </c>
     </row>
@@ -1694,27 +1694,27 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Ministerio de Cultura - Contemporáneos. Cinco mil años de visualidad peruana (2019) [catálogo, Perú país invitado ARCOmadrid].md</t>
+          <t>Mesa - Coleccionando desde la institución (2025) [Charlas de colección, Foro Pinta Lima].transcripcion.md</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>200 a.C.-2019 (Nasca, virreinato y arte contemporáneo reciente)</t>
+          <t>1960s-2025 (con eje en 2006-2025)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Catálogo institucional de feria/exposición (ARCOmadrid), 2019</t>
+          <t>Transcripción de conversatorio (Foro Pinta Lima 2025), 2025</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Ministerio de Cultura del Perú; Jorge Villacorta; Sharon Lerner; Fietta Jarque; Miguel A. López; Teresa Burga; Fernando Bryce; Sandra Gamarra; Natalia Majluf; MALI; ARCOmadrid / IFEMA; Museo Reina Sofía / Museo del Prado</t>
+          <t>Pablo León de la Barra; Sharon Lerner; Manuel Segade; MALI; Museo Reina Sofía; Museo Guggenheim; Comité de Adquisiciones de Arte Contemporáneo del MALI; Suset Sánchez; Amanda de la Garza; Tatiana Cuevas; Fundación Museo Reina Sofía</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Catálogo institucional de la participación de Perú como País Invitado en ARCOmadrid 2019, que reúne los textos curatoriales del stand del Estado, la zona de galerías y el programa oficial de más de treinta exposiciones y actividades en Madrid. El ensayo de Jorge Villacorta, 'Contemporáneos: cinco mil años de visualidad peruana', propone lo contemporáneo como actitud y coexistencia antes que como novedad, avanzando la hipótesis de que la contemporaneidad peruana es continuidad de una matriz cultural andino-amazónica con incrustaciones occidentales, un tiempo cíclico que supera categorías como arte popular o artesanía. Sharon Lerner, en 'Texto, tactibilidad y trama', encuadra la selección de galerías —que por primera vez combina representación local e internacional— como un corte no representativo de un 'arte nacional', destacando líneas transversales: el uso del texto, la cita y el archivo para desmontar discursos de la historia oficial; las tensiones del colonialismo y los criterios étnicos y de clase; la mirada al territorio y a lo extractivo; y la fragilidad táctil del textil, la arcilla y el cuerpo. El catálogo perfila a artistas como Teresa Burga, Rita Ponce de León, Ximena Garrido Lecca, Herbert Rodríguez, Fernando Bryce, Sandra Gamarra, Milagros de la Torre y Antonio Paucar, y documenta las conferencias curadas por Miguel A. López sobre el Bicentenario, la contemporaneidad andina, indígena y amazónica, y las transformaciones institucionales y de mercado. El programa oficial, presentado por Fietta Jarque, articula un relato de cinco mil años: Nasca, el Matrimonio de Martín de Loyola, Huamán Poma, la revista Amauta de Mariátegui, Amazonías y colecciones privadas (Hochschild, CIFO, Jan Mulder).</t>
+          <t>Transcripción (borrador) del conversatorio 'Coleccionando desde la institución' del Foro Pinta Lima 2025, moderado por Pablo León de la Barra (Guggenheim), que confronta dos modelos museales públicos: el MALI de Lima y el Museo Reina Sofía de Madrid. La tesis compartida es que coleccionar implica un pensamiento crítico que puede cuestionar el canon, reparar asimetrías históricas de género, raza e identidad y llenar vacíos. Sharon Lerner expone la trayectoria del Comité de Adquisiciones de Arte Contemporáneo del MALI (casi veinte años, modelado sobre el Latin American Acquisitions Committee de la Tate), la curaduría contemporánea iniciada por Tatiana Cuevas en 2008, y el trabajo 'trenzado' entre colección histórica y contemporánea que atraviesa exposiciones como Arte al Paso, Amazonías y Otras historias posibles, y la reestructuración pospandemia con el programa Salas Abiertas. Detalla la visibilización de artistas amazónicos e indígenas (Sara Flores, Chonon Bensho, Venuca Evanán), la incorporación del textil y proyectos como Línea de Vida de Giuseppe Campuzano, junto a comisiones y trabajo comunitario con Cantagallo. Manuel Segade analiza la dimensión colonial del Reina Sofía —cuya colección latinoamericana se inauguró en 1992— y las condiciones estructurales, funcionariales y presupuestarias que la condicionan, citando las preguntas ontológicas de Suset Sánchez y el Instituto Cader de arte centroamericano como vía de restitución frente al extractivismo cultural. El diálogo aborda el rol de los públicos, la crispación política, la censura, el cierre del Lugar de la Memoria y la misión histórica del museo como plataforma de tensiones críticas de la sociedad civil.</t>
         </is>
       </c>
     </row>
@@ -1726,27 +1726,27 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Mitrovic - Extravíos de la forma. Vanguardia, modernismo popular y arte contemporáneo en Lima desde los 60 (2019).md</t>
+          <t>Ministerio de Cultura - Contemporáneos. Cinco mil años de visualidad peruana (2019) [catálogo, Perú país invitado ARCOmadrid].md</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>1960-2018 (desde los sesenta hasta el presente)</t>
+          <t>200 a.C.-2019 (Nasca, virreinato y arte contemporáneo reciente)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Libro académico, 2019 (Fondo Editorial FAU-PUCP)</t>
+          <t>Catálogo institucional de feria/exposición (ARCOmadrid), 2019</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Mijail Mitrovic; Gustavo Buntinx; Mirko Lauer; Sharon Lerner; Miguel A. López; Emilio Tarazona; Fernando de Szyszlo; E.P.S. Huayco; Taller NN; José Carlos Martinat; Museo de Arte de Lima (MALI); PUCP; Fredric Jameson</t>
+          <t>Ministerio de Cultura del Perú; Jorge Villacorta; Sharon Lerner; Fietta Jarque; Miguel A. López; Teresa Burga; Fernando Bryce; Sandra Gamarra; Natalia Majluf; MALI; ARCOmadrid / IFEMA; Museo Reina Sofía / Museo del Prado</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Ensayo de historia y teoría del arte que impugna el «relato convencional» sobre el arte contemporáneo en Lima, entendido como una fábula épica que narra el tránsito de la vanguardia de los sesenta al arte contemporáneo global mediante el «encuentro con lo popular». Desde un marco marxista-dialéctico (Adorno, Jameson, Bürger, Osborne, Lukács), Mitrovic reivindica la totalización y la periodización frente al historicismo posmoderno que celebra heterogeneidad y discontinuidad. Su tesis central es que la «desidealización» del arte —su reducción a hecho social e institucional— siguió en Lima una trayectoria específica: de la teoría de las raíces nacionales (Szyszlo, Lauer) y el altomodernismo, a la radicalización de la vanguardia bajo el velasquismo, que el autor conceptualiza como «modernismo popular» (E.P.S. Huayco, Paréntesis, la frase de Lauer «solo lo popular es moderno»). Con Sendero Luminoso y la crisis de los ochenta, la utopía colapsa y el arte se reorienta hacia la denuncia ética de la violencia, prolongada durante el fujimorato (Colectivo Sociedad Civil, «Lava la bandera»). El cambio de siglo consuma la «contemporaneización» mediante las Bienales de Lima y el mercado. El último capítulo analiza obras (Polanco, Guerra García, Huarcaya, Aguirre, Andrade Valdez, Martinat) para mostrar cómo lo popular deviene «neocostumbrismo» y «renta de monopolio»: sello local que certifica autenticidad cultural en el circuito global, mientras se evacúa el horizonte futuro y el «pueblo» se reduce a «población». Frente a la nostalgia y la reoligarquización simbólica, Mitrovic propone recuperar las potencialidades utópicas hoy reprimidas.</t>
+          <t>Catálogo institucional de la participación de Perú como País Invitado en ARCOmadrid 2019, que reúne los textos curatoriales del stand del Estado, la zona de galerías y el programa oficial de más de treinta exposiciones y actividades en Madrid. El ensayo de Jorge Villacorta, 'Contemporáneos: cinco mil años de visualidad peruana', propone lo contemporáneo como actitud y coexistencia antes que como novedad, avanzando la hipótesis de que la contemporaneidad peruana es continuidad de una matriz cultural andino-amazónica con incrustaciones occidentales, un tiempo cíclico que supera categorías como arte popular o artesanía. Sharon Lerner, en 'Texto, tactibilidad y trama', encuadra la selección de galerías —que por primera vez combina representación local e internacional— como un corte no representativo de un 'arte nacional', destacando líneas transversales: el uso del texto, la cita y el archivo para desmontar discursos de la historia oficial; las tensiones del colonialismo y los criterios étnicos y de clase; la mirada al territorio y a lo extractivo; y la fragilidad táctil del textil, la arcilla y el cuerpo. El catálogo perfila a artistas como Teresa Burga, Rita Ponce de León, Ximena Garrido Lecca, Herbert Rodríguez, Fernando Bryce, Sandra Gamarra, Milagros de la Torre y Antonio Paucar, y documenta las conferencias curadas por Miguel A. López sobre el Bicentenario, la contemporaneidad andina, indígena y amazónica, y las transformaciones institucionales y de mercado. El programa oficial, presentado por Fietta Jarque, articula un relato de cinco mil años: Nasca, el Matrimonio de Martín de Loyola, Huamán Poma, la revista Amauta de Mariátegui, Amazonías y colecciones privadas (Hochschild, CIFO, Jan Mulder).</t>
         </is>
       </c>
     </row>
@@ -1758,27 +1758,27 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Peralta - Lo que la Bienal de Lima se llevó. Balance a cinco años de su desactivación.md</t>
+          <t>Mitrovic - Extravíos de la forma. Vanguardia, modernismo popular y arte contemporáneo en Lima desde los 60 (2019).md</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>1997-2003 (Bienales de Lima y su desactivación)</t>
+          <t>1960-2018 (desde los sesenta hasta el presente)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Artículo/ensayo de balance, ca. 2007-2008</t>
+          <t>Libro académico, 2019 (Fondo Editorial FAU-PUCP)</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Juan Peralta; Luis Lama; Jorge Villacorta; Emilio Santisteban; Elena Tejada; Gustavo Buntinx; Alfonso Castrillón; Élida Román; Allora &amp; Calzadilla; Francis Alÿs; Cuauhtémoc Medina; Alberto Andrade; Luis Castañeda Lossio; Municipalidad Metropolitana de Lima; UCCI</t>
+          <t>Mijail Mitrovic; Gustavo Buntinx; Mirko Lauer; Sharon Lerner; Miguel A. López; Emilio Tarazona; Fernando de Szyszlo; E.P.S. Huayco; Taller NN; José Carlos Martinat; Museo de Arte de Lima (MALI); PUCP; Fredric Jameson</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Balance crítico sobre la desaparición de la Bienal de Lima, escrito por Juan Peralta a cinco años de su desactivación. El texto reconstruye el contexto político-cultural en que surgió el megaevento ideado por Luis Lama: el régimen fujimorista, el programa municipal «Volver al Centro» y el Plan Maestro del Centro Histórico impulsado por la gestión de Alberto Andrade, articulados con redes internacionales (UCCI, CIDEU) y el título de «Lima, Capital de la Cultura Iberoamericana». Peralta sostiene que la Bienal (1997-2002), en sus versiones nacional e iberoamericana, funcionó como núcleo de reactivación cultural y descentralización mediante salones regionales, atrajo atención internacional y sirvió de modelo de gestión, pero fue cancelada por desinterés político —especialmente de Luis Castañeda Lossio— y por la incapacidad del propio medio artístico de defender su función social. Documenta episodios polémicos: la crítica de Alfonso Castrillón a la autoría de una obra de García Zapatero, la performance «Señorita de buena presencia busca empleo» de Elena Tejada, la muestra paralela «Emergencia Artística» (1999) gestada por Emilio Santisteban y Gustavo Buntinx tras el veto a «Crisis», y la intervención «Chalk» de Allora &amp; Calzadilla, resignificada por trabajadores municipales. A través de testimonios (Santisteban, Élida Román, Natalia Velit, el propio Lama), el autor argumenta que la orfandad cultural persiste por la ausencia de políticas públicas y la subordinación al mercado. El texto se posiciona a favor de una gestión cultural audaz, descentralizada y socialmente participativa, lamentando que nada haya reemplazado la escala y el alcance de la Bienal.</t>
+          <t>Ensayo de historia y teoría del arte que impugna el «relato convencional» sobre el arte contemporáneo en Lima, entendido como una fábula épica que narra el tránsito de la vanguardia de los sesenta al arte contemporáneo global mediante el «encuentro con lo popular». Desde un marco marxista-dialéctico (Adorno, Jameson, Bürger, Osborne, Lukács), Mitrovic reivindica la totalización y la periodización frente al historicismo posmoderno que celebra heterogeneidad y discontinuidad. Su tesis central es que la «desidealización» del arte —su reducción a hecho social e institucional— siguió en Lima una trayectoria específica: de la teoría de las raíces nacionales (Szyszlo, Lauer) y el altomodernismo, a la radicalización de la vanguardia bajo el velasquismo, que el autor conceptualiza como «modernismo popular» (E.P.S. Huayco, Paréntesis, la frase de Lauer «solo lo popular es moderno»). Con Sendero Luminoso y la crisis de los ochenta, la utopía colapsa y el arte se reorienta hacia la denuncia ética de la violencia, prolongada durante el fujimorato (Colectivo Sociedad Civil, «Lava la bandera»). El cambio de siglo consuma la «contemporaneización» mediante las Bienales de Lima y el mercado. El último capítulo analiza obras (Polanco, Guerra García, Huarcaya, Aguirre, Andrade Valdez, Martinat) para mostrar cómo lo popular deviene «neocostumbrismo» y «renta de monopolio»: sello local que certifica autenticidad cultural en el circuito global, mientras se evacúa el horizonte futuro y el «pueblo» se reduce a «población». Frente a la nostalgia y la reoligarquización simbólica, Mitrovic propone recuperar las potencialidades utópicas hoy reprimidas.</t>
         </is>
       </c>
     </row>
@@ -1790,27 +1790,27 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Ponencia - Villacorta, Jorge - Puntos cardinales (2019) [CEdA].transcripcion.txt</t>
+          <t>Peralta - Lo que la Bienal de Lima se llevó. Balance a cinco años de su desactivación.md</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>1979-2019 (énfasis en 2001-2019: obra de los ochenta y ARCO 2019)</t>
+          <t>1997-2003 (Bienales de Lima y su desactivación)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Transcripción de ponencia/conferencia, 2019 (Fundación SEDA-CEdA, Santiago)</t>
+          <t>Artículo/ensayo de balance, ca. 2007-2008</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Sebastián Vidal; Fundación SEDA; Sandra Gamarra (LiMac); Juan Javier Salazar; Herbert Rodríguez; Rodrigo Quijano; grupo Huayco; MALI; Fundación Reina Sofía; ARCOmadrid; galería Enrique Faria; galería Revólver; Alexis Fabri</t>
+          <t>Juan Peralta; Luis Lama; Jorge Villacorta; Emilio Santisteban; Elena Tejada; Gustavo Buntinx; Alfonso Castrillón; Élida Román; Allora &amp; Calzadilla; Francis Alÿs; Cuauhtémoc Medina; Alberto Andrade; Luis Castañeda Lossio; Municipalidad Metropolitana de Lima; UCCI</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Transcripción de una ponencia de Jorge Villacorta en la Fundación SEDA (Santiago de Chile), presentada por Sebastián Vidal, en el marco de su participación en el pabellón peruano de ARCOmadrid 2019. Partiendo de dos exposiciones fundacionales de Sandra Gamarra (Living Room, 2001; el proyecto LiMac, 2002), Villacorta reflexiona sobre la desconexión histórica del sistema del arte limeño respecto del circuito internacional y su condición estructuralmente «coja». El eje del argumento es un contraste entre dos artistas del grupo Huayco: Juan Javier Salazar y Herbert Rodríguez. Salazar, considerado durante dos décadas el artista contemporáneo peruano por excelencia (Perú País del Mañana, El cuartucho, los náufragos), cultivó una obra frágil, localista y ácida sobre la desidia nacional, pero fue «maltratado» tras su muerte: descartado en ARCO 2019, cosmetizado en la Bienal de Venecia 2017 y regateado por el capítulo peruano de la Fundación Reina Sofía. Rodríguez, artista afrodescendiente y sistemático archivista de su obra (fotocopias, murales antisenderistas en San Marcos, fotoserigrafía), experimenta en cambio un ascenso internacional inesperado (galería Enrique Faria, Reina Sofía, Fundación Cartier), pese al desdén histórico del medio limeño y del MALI. Villacorta articula estas trayectorias con una crítica al coleccionismo peruano, a la lógica del mercado (galería Revólver, ferias, matching funds de arteBA), a la desatención de la crítica y las galerías, y a las jerarquías raciales y clasistas del establishment cultural limeño (Szyszlo, Armando Andrade). El texto plantea el problema del legado, el valor simbólico y la posibilidad de un arte con «testigos» frente a un arte subordinado al mercado.</t>
+          <t>Balance crítico sobre la desaparición de la Bienal de Lima, escrito por Juan Peralta a cinco años de su desactivación. El texto reconstruye el contexto político-cultural en que surgió el megaevento ideado por Luis Lama: el régimen fujimorista, el programa municipal «Volver al Centro» y el Plan Maestro del Centro Histórico impulsado por la gestión de Alberto Andrade, articulados con redes internacionales (UCCI, CIDEU) y el título de «Lima, Capital de la Cultura Iberoamericana». Peralta sostiene que la Bienal (1997-2002), en sus versiones nacional e iberoamericana, funcionó como núcleo de reactivación cultural y descentralización mediante salones regionales, atrajo atención internacional y sirvió de modelo de gestión, pero fue cancelada por desinterés político —especialmente de Luis Castañeda Lossio— y por la incapacidad del propio medio artístico de defender su función social. Documenta episodios polémicos: la crítica de Alfonso Castrillón a la autoría de una obra de García Zapatero, la performance «Señorita de buena presencia busca empleo» de Elena Tejada, la muestra paralela «Emergencia Artística» (1999) gestada por Emilio Santisteban y Gustavo Buntinx tras el veto a «Crisis», y la intervención «Chalk» de Allora &amp; Calzadilla, resignificada por trabajadores municipales. A través de testimonios (Santisteban, Élida Román, Natalia Velit, el propio Lama), el autor argumenta que la orfandad cultural persiste por la ausencia de políticas públicas y la subordinación al mercado. El texto se posiciona a favor de una gestión cultural audaz, descentralizada y socialmente participativa, lamentando que nada haya reemplazado la escala y el alcance de la Bienal.</t>
         </is>
       </c>
     </row>
@@ -1822,27 +1822,27 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Por Qué no vivo en el Perú.md</t>
+          <t>Ponencia - Villacorta, Jorge - Puntos cardinales (2019) [CEdA].transcripcion.txt</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>ca. 1972 en adelante (emigración de Juan Acha a México y comparación Perú/México de los años setenta)</t>
+          <t>1979-2019 (énfasis en 2001-2019: obra de los ochenta y ARCO 2019)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Encuesta/testimonio en revista literaria (Hueso Húmero), ca. 1980; transcripción en Markdown, s/f</t>
+          <t>Transcripción de ponencia/conferencia, 2019 (Fundación SEDA-CEdA, Santiago)</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Juan Acha; revista Hueso Húmero; museos, institutos y universidades de México</t>
+          <t>Jorge Villacorta; Sebastián Vidal; Fundación SEDA; Sandra Gamarra (LiMac); Juan Javier Salazar; Herbert Rodríguez; Rodrigo Quijano; grupo Huayco; MALI; Fundación Reina Sofía; ARCOmadrid; galería Enrique Faria; galería Revólver; Alexis Fabri</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Transcripción de la respuesta de Juan Acha a la encuesta 'Por qué no vivo en el Perú', iniciada por la revista Hueso Húmero para indagar las razones del éxodo de creadores e intelectuales peruanos. Acha —crítico y teórico del arte dedicado a los problemas latinoamericanos, radicado en México— distingue razones 'de afuera' y 'de adentro', otorgando mayor peso a las primeras: sólo abandona su país quien encuentra en otro las condiciones para desarrollar con dignidad su trabajo profesional, mientras que las circunstancias personales o los factores nacionales negativos serían secundarios en su caso. Enumera lo que México le ofreció y el Perú le negaba: amplias posibilidades de publicar en diarios y revistas, de colaborar en museos e institutos y de investigar y enseñar en universidades, todo ello remunerado con dignidad; libertad de expresión intelectual e intensa circulación de ideas marxistas en libros, revistas y simposios; prestigio nacional de las artes visuales con apoyo estatal, política museográfica y de simposios activa, y facilidades para viajar y contactar con el arte de otras latitudes. Valora, además, el mejor enfoque de los problemas artísticos y culturales latinoamericanos posible desde México, cuya escala demográfica y potente industria editorial concentran las investigaciones de toda la región y anticipan fenómenos que luego se difunden. El testimonio —que el archivo conserva incompleto, interrumpido al mencionar una 'identificación cultural más conflictiva y acorde a la realidad concreta'— condensa la autojustificación del exilio intelectual como decisión productiva antes que como queja, y funciona como documento sobre las carencias institucionales del campo artístico peruano frente a las condiciones del México de esos años.</t>
+          <t>Transcripción de una ponencia de Jorge Villacorta en la Fundación SEDA (Santiago de Chile), presentada por Sebastián Vidal, en el marco de su participación en el pabellón peruano de ARCOmadrid 2019. Partiendo de dos exposiciones fundacionales de Sandra Gamarra (Living Room, 2001; el proyecto LiMac, 2002), Villacorta reflexiona sobre la desconexión histórica del sistema del arte limeño respecto del circuito internacional y su condición estructuralmente «coja». El eje del argumento es un contraste entre dos artistas del grupo Huayco: Juan Javier Salazar y Herbert Rodríguez. Salazar, considerado durante dos décadas el artista contemporáneo peruano por excelencia (Perú País del Mañana, El cuartucho, los náufragos), cultivó una obra frágil, localista y ácida sobre la desidia nacional, pero fue «maltratado» tras su muerte: descartado en ARCO 2019, cosmetizado en la Bienal de Venecia 2017 y regateado por el capítulo peruano de la Fundación Reina Sofía. Rodríguez, artista afrodescendiente y sistemático archivista de su obra (fotocopias, murales antisenderistas en San Marcos, fotoserigrafía), experimenta en cambio un ascenso internacional inesperado (galería Enrique Faria, Reina Sofía, Fundación Cartier), pese al desdén histórico del medio limeño y del MALI. Villacorta articula estas trayectorias con una crítica al coleccionismo peruano, a la lógica del mercado (galería Revólver, ferias, matching funds de arteBA), a la desatención de la crítica y las galerías, y a las jerarquías raciales y clasistas del establishment cultural limeño (Szyszlo, Armando Andrade). El texto plantea el problema del legado, el valor simbólico y la posibilidad de un arte con «testigos» frente a un arte subordinado al mercado.</t>
         </is>
       </c>
     </row>
@@ -1854,27 +1854,27 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>QUEHACER 19_watermark_p120-128.pdf</t>
+          <t>Por Qué no vivo en el Perú.md</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>1940-1982 (arte peruano del siglo XX: indigenismo, velasquismo y transición belaundista)</t>
+          <t>ca. 1972 en adelante (emigración de Juan Acha a México y comparación Perú/México de los años setenta)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Entrevista en revista (Quehacer n.º 19, DESCO), ca. 1982</t>
+          <t>Encuesta/testimonio en revista literaria (Hueso Húmero), ca. 1980; transcripción en Markdown, s/f</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Mirko Lauer; Sebastián Gris; Juan Acha; DESCO; Alfonso Castrillón; José Sabogal; Josué Sánchez; Ramiro Llona; José Carlos Ramos; Joaquín López Antay; Fernando de Szyszlo; Juan Manuel Ugarte Eléspuru; Bienal de Medellín</t>
+          <t>Juan Acha; revista Hueso Húmero; museos, institutos y universidades de México</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Entrevista de Sebastián Gris a Mirko Lauer publicada en la revista Quehacer (n.º 19, DESCO) bajo el título 'Está naciendo algo…'. El diálogo presenta el giro teórico de Lauer —poeta y crítico literario— hacia una teoría social de la cultura y del objeto plástico, formulada en su libro 'Crítica de la artesanía' y anticipada, junto al ausente Juan Acha, en el Coloquio de Arte No-objetual de Medellín. Lauer relee su 'Introducción a la pintura peruana del siglo XX': sostiene que hacia 1960 culmina, con la 'Teoría de las Raíces Nacionales', el ciclo abierto por el indigenismo de Sabogal, mientras los años setenta traen la revaloración del arte popular y su confluencia con una tradición artesanal. Critica el neo-indigenismo como coartada del populismo velasquista y de la Reforma Agraria: un país que, sin atreverse a enfrentar lo popular real, se inventa un seudo-país mistificado (el 'colmenazo', el arte turístico de José Carlos Ramos). Diagnostica, tras la restauración belaundista (posterior a 1977), una 'pérdida de direccionalidad' y un caos del mercado que ahora impone valor. Discute los límites de la propuesta conceptual y no-objetual, el Premio Nacional López Antay y la labor de Alfonso Castrillón, y reivindica la crítica de arte como oficio concreto —ni estética idealista ni 'estética marxista'—. Finalmente aborda la marginalidad y el desprecio hacia el intelectual peruano. Aparecen Josué Sánchez, Ramiro Llona, Szyszlo, Ugarte Eléspuru y la Bienal de Medellín. Su aporte es proponer el estudio del objeto plástico desde su existencia social y desde una perspectiva popular.</t>
+          <t>Transcripción de la respuesta de Juan Acha a la encuesta 'Por qué no vivo en el Perú', iniciada por la revista Hueso Húmero para indagar las razones del éxodo de creadores e intelectuales peruanos. Acha —crítico y teórico del arte dedicado a los problemas latinoamericanos, radicado en México— distingue razones 'de afuera' y 'de adentro', otorgando mayor peso a las primeras: sólo abandona su país quien encuentra en otro las condiciones para desarrollar con dignidad su trabajo profesional, mientras que las circunstancias personales o los factores nacionales negativos serían secundarios en su caso. Enumera lo que México le ofreció y el Perú le negaba: amplias posibilidades de publicar en diarios y revistas, de colaborar en museos e institutos y de investigar y enseñar en universidades, todo ello remunerado con dignidad; libertad de expresión intelectual e intensa circulación de ideas marxistas en libros, revistas y simposios; prestigio nacional de las artes visuales con apoyo estatal, política museográfica y de simposios activa, y facilidades para viajar y contactar con el arte de otras latitudes. Valora, además, el mejor enfoque de los problemas artísticos y culturales latinoamericanos posible desde México, cuya escala demográfica y potente industria editorial concentran las investigaciones de toda la región y anticipan fenómenos que luego se difunden. El testimonio —que el archivo conserva incompleto, interrumpido al mencionar una 'identificación cultural más conflictiva y acorde a la realidad concreta'— condensa la autojustificación del exilio intelectual como decisión productiva antes que como queja, y funciona como documento sobre las carencias institucionales del campo artístico peruano frente a las condiciones del México de esos años.</t>
         </is>
       </c>
     </row>
@@ -1886,27 +1886,27 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Román, Elida - I Bienal Nacional de Lima. Algunos deslindes.md</t>
+          <t>QUEHACER 19_watermark_p120-128.pdf</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>1997-1998 (I Bienal Nacional de Lima; referencias a 1987 y 1997)</t>
+          <t>1940-1982 (arte peruano del siglo XX: indigenismo, velasquismo y transición belaundista)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Artículo/reseña crítica, 1998</t>
+          <t>Entrevista en revista (Quehacer n.º 19, DESCO), ca. 1982</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Élida Román; Luis Lama; UCCI; Municipalidad Metropolitana de Lima; Centro de Artes Visuales (CAV); Virginia Pérez-Ratton; Museo de Arte de Lima; Luz María Bedoya; Mariella Agois; Bienal de Trujillo</t>
+          <t>Mirko Lauer; Sebastián Gris; Juan Acha; DESCO; Alfonso Castrillón; José Sabogal; Josué Sánchez; Ramiro Llona; José Carlos Ramos; Joaquín López Antay; Fernando de Szyszlo; Juan Manuel Ugarte Eléspuru; Bienal de Medellín</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Nota crítica de la crítica de arte Élida Román sobre la I Bienal Nacional de Lima (1998), que deslinda sus antecedentes y examina su lógica organizativa. Román recuerda que un evento similar existió en la III Bienal de Trujillo (1987) con el núcleo «Mirada hacia adentro», y sitúa la Bienal Nacional como mecanismo para seleccionar —mediante salones regionales y comités— la representación peruana a la II Bienal Iberoamericana. Enmarca el evento en el proyecto municipal de recuperación del Centro Histórico y en la designación de Lima como «Plaza Mayor de la Cultura Iberoamericana» por la UCCI, señalando el apresuramiento organizativo y los defectos museográficos derivados del uso de casonas no adecuadas a fines museológicos. Su argumento central cuestiona el discurso «modernizador» y globalizador de los organizadores (Luis Lama), advirtiendo que tras las nociones de ruptura, novedad y globalización se esconden la moda, el esnobismo y «roles forzados» e intereses extraculturales. Critica el centralismo y paternalismo de los salones regionales, que perpetúan la posición privilegiada de Lima sin una política real de desarrollo en provincias. Román reclama definir los propósitos de la actividad artística e interroga la falsa dicotomía entre arte «popular» y «culto», recordando la polémica por el Premio Nacional otorgado a un artesano ayacuchano. Frente a la comparación con estándares metropolitanos, aboga por una modernidad entendida como apertura multidisciplinaria y actitud cohesionadora e identitaria, apoyada en la historia, la antropología y las ciencias sociales. El texto, denso en interrogantes, defiende la reflexión teórica y el debate, y cierra evocando la consigna «¡La imaginación al poder!».</t>
+          <t>Entrevista de Sebastián Gris a Mirko Lauer publicada en la revista Quehacer (n.º 19, DESCO) bajo el título 'Está naciendo algo…'. El diálogo presenta el giro teórico de Lauer —poeta y crítico literario— hacia una teoría social de la cultura y del objeto plástico, formulada en su libro 'Crítica de la artesanía' y anticipada, junto al ausente Juan Acha, en el Coloquio de Arte No-objetual de Medellín. Lauer relee su 'Introducción a la pintura peruana del siglo XX': sostiene que hacia 1960 culmina, con la 'Teoría de las Raíces Nacionales', el ciclo abierto por el indigenismo de Sabogal, mientras los años setenta traen la revaloración del arte popular y su confluencia con una tradición artesanal. Critica el neo-indigenismo como coartada del populismo velasquista y de la Reforma Agraria: un país que, sin atreverse a enfrentar lo popular real, se inventa un seudo-país mistificado (el 'colmenazo', el arte turístico de José Carlos Ramos). Diagnostica, tras la restauración belaundista (posterior a 1977), una 'pérdida de direccionalidad' y un caos del mercado que ahora impone valor. Discute los límites de la propuesta conceptual y no-objetual, el Premio Nacional López Antay y la labor de Alfonso Castrillón, y reivindica la crítica de arte como oficio concreto —ni estética idealista ni 'estética marxista'—. Finalmente aborda la marginalidad y el desprecio hacia el intelectual peruano. Aparecen Josué Sánchez, Ramiro Llona, Szyszlo, Ugarte Eléspuru y la Bienal de Medellín. Su aporte es proponer el estudio del objeto plástico desde su existencia social y desde una perspectiva popular.</t>
         </is>
       </c>
     </row>
@@ -1918,27 +1918,27 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Screen Shot 2026-07-16 at 08.22.07.png</t>
+          <t>Román, Elida - I Bienal Nacional de Lima. Algunos deslindes.md</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>1980-1981 (obra 'Arte al Paso' y culto vigente a Sarita Colonia); Sarita Colonia 1914-1940</t>
+          <t>1997-1998 (I Bienal Nacional de Lima; referencias a 1987 y 1997)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Captura de pantalla, 16-07-2026 (de artículo de la revista MARKA, Lima, 14-05-1981, p. 34; archivo UNMSM-CEDOC)</t>
+          <t>Artículo/reseña crítica, 1998</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Sarita Colonia; Taller de Estética de Proyección Social 'Huayco' (E.P.S. Huayco); Francisco Mariotti; María Luy; Gerbert Rodríguez; Mariella Zevallos; Armando Williams; Charo Noriega; revista MARKA; UNMSM-CEDOC</t>
+          <t>Élida Román; Luis Lama; UCCI; Municipalidad Metropolitana de Lima; Centro de Artes Visuales (CAV); Virginia Pérez-Ratton; Museo de Arte de Lima; Luz María Bedoya; Mariella Agois; Bienal de Trujillo</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Captura de una página de la revista MARKA (Lima, 14 de mayo de 1981, p. 34; sello de archivo UNMSM-CEDOC) con el artículo 'La imagen y la fuerza milagrosa', dedicado al culto a Sarita Colonia y a su tratamiento en el arte. El texto interpreta la devoción popular a Sarita como caso patente de realización simbólica donde el elemento religioso se ensambla con el gusto estético popular, uniendo pensamiento mágico y realidad social inmediata; el símbolo religioso operaría como continente de mitos que resuelven imaginariamente las contradicciones de la vida. Recuerda que Sarita nació en Huaraz en 1914 y murió en el Callao en 1940, donde surgió su culto —hoy extendido entre los más desvalidos: el mundo del hampa, la prostitución, estibadores y choferes—, con un mausoleo-santuario rodeado de exvotos y comerciantes ambulantes. La sección 'Sarita en el arte' presenta y reproduce la obra 'Arte al Paso', un enorme rostro de Sarita compuesto con cerca de 12,000 latas de leche, realizado por un conjunto de artistas jóvenes reunidos en el Taller de Estética de Proyección Social 'Huayco' (E.P.S. Huayco): Francisco Mariotti, María Luy, Gerbert Rodríguez, Mariella Zevallos, Armando Williams y Charo Noriega. Instalada desde enero de ese año a la vera del sur, la obra recoge en clave colectiva la significación sociocultural de Sarita para ofrecer a viajeros y peregrinos una exposición permanente de esa imagen, integrando la escala monumental, la soledad del paisaje y una identificación plástica con el misterio cotidiano. Es documento clave sobre el vínculo entre religiosidad popular, migración andina y vanguardia peruana de inicios de los ochenta.</t>
+          <t>Nota crítica de la crítica de arte Élida Román sobre la I Bienal Nacional de Lima (1998), que deslinda sus antecedentes y examina su lógica organizativa. Román recuerda que un evento similar existió en la III Bienal de Trujillo (1987) con el núcleo «Mirada hacia adentro», y sitúa la Bienal Nacional como mecanismo para seleccionar —mediante salones regionales y comités— la representación peruana a la II Bienal Iberoamericana. Enmarca el evento en el proyecto municipal de recuperación del Centro Histórico y en la designación de Lima como «Plaza Mayor de la Cultura Iberoamericana» por la UCCI, señalando el apresuramiento organizativo y los defectos museográficos derivados del uso de casonas no adecuadas a fines museológicos. Su argumento central cuestiona el discurso «modernizador» y globalizador de los organizadores (Luis Lama), advirtiendo que tras las nociones de ruptura, novedad y globalización se esconden la moda, el esnobismo y «roles forzados» e intereses extraculturales. Critica el centralismo y paternalismo de los salones regionales, que perpetúan la posición privilegiada de Lima sin una política real de desarrollo en provincias. Román reclama definir los propósitos de la actividad artística e interroga la falsa dicotomía entre arte «popular» y «culto», recordando la polémica por el Premio Nacional otorgado a un artesano ayacuchano. Frente a la comparación con estándares metropolitanos, aboga por una modernidad entendida como apertura multidisciplinaria y actitud cohesionadora e identitaria, apoyada en la historia, la antropología y las ciencias sociales. El texto, denso en interrogantes, defiende la reflexión teórica y el debate, y cierra evocando la consigna «¡La imaginación al poder!».</t>
         </is>
       </c>
     </row>
@@ -1950,27 +1950,27 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Screen Shot 2026-07-16 at 08.37.09.png</t>
+          <t>Screen Shot 2026-07-16 at 08.22.07.png</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>1965-1984</t>
+          <t>1980-1981 (obra 'Arte al Paso' y culto vigente a Sarita Colonia); Sarita Colonia 1914-1940</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Captura de pantalla, 16-07-2026 (de un cuadro/gráfico basado en el informe de Alfonso Castrillón, 'Reflexiones sobre el arte conceptual en el Perú y sus proyecciones', Hueso Húmero n.º 7; sello UNMSM)</t>
+          <t>Captura de pantalla, 16-07-2026 (de artículo de la revista MARKA, Lima, 14-05-1981, p. 34; archivo UNMSM-CEDOC)</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Alfonso Castrillón; Juan Acha; Teresa Burga; Emilio Hernández; Rafael Hastings; Francisco Mariotti; Luis Arias Vera; Jorge Eielson; Wiley Ludeña; Herbert Rodríguez; E.P.S. Huayco; Grupo Paréntesis; UNMSM</t>
+          <t>Sarita Colonia; Taller de Estética de Proyección Social 'Huayco' (E.P.S. Huayco); Francisco Mariotti; María Luy; Gerbert Rodríguez; Mariella Zevallos; Armando Williams; Charo Noriega; revista MARKA; UNMSM-CEDOC</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Captura de pantalla de un cuadro cronológico ('Gráfico 1') que sistematiza el desarrollo del arte conceptual y no-objetual en el Perú entre 1965 y 1984, elaborado 'en base al informe de Alfonso Castrillón: Reflexiones sobre el arte conceptual en el Perú y sus proyecciones' (Hueso Húmero 7). El cuadro organiza la información en cuatro columnas —Fecha, Tendencia, Operador (artistas y grupos) y Lugar— trazando la sucesión de tendencias: pop y op (1965, Galería Lima, IAC), concepto y ambientes (1969-1970, con Juan Acha, 'Cultura y Libertad'), acciones y eventos (1972-1975: Teresa Burga, Rafael Hastings, Francisco Mariotti, CONTACTA, Premio López Antay, Festival Inkarri), y las prácticas de no-objeto y performance de fines de los setenta y de los ochenta. Registra los colectivos 'Signo x signo' (Patricia López, Armando Williams, Rossana Agois, Wiley Ludeña, Hugo Salazar), el Grupo USM de Alfonso Castrillón, 'Paréntesis' (Charo Noriega, Armando Williams, María Luy, Francisco Mariotti, Fernando Bedoya, Juan J. Salazar, Mariela Zevallos) y 'Huayco EPS' (Herbert Rodríguez, Lucy Angulo, José Morales), junto a nombres como Luis Arias Vera, Emilio Hernández, Jorge Eielson, Hernán Pazos, Esther Vainstein, Cecilia Paredes y Sergio Zevallos. Consigna hitos y sedes: encuestas, la Bienal no-objetual de Medellín, la Bienal de São Paulo (1983), la acción 'Cuidado pintores…', y espacios como el Instituto Italiano, la Universidad de San Marcos y galerías limeñas. Funciona como mapa genealógico de la vanguardia experimental peruana y de sus operadores institucionales, útil para periodizar el paso del conceptualismo a la performance y al arte no-objetual.</t>
+          <t>Captura de una página de la revista MARKA (Lima, 14 de mayo de 1981, p. 34; sello de archivo UNMSM-CEDOC) con el artículo 'La imagen y la fuerza milagrosa', dedicado al culto a Sarita Colonia y a su tratamiento en el arte. El texto interpreta la devoción popular a Sarita como caso patente de realización simbólica donde el elemento religioso se ensambla con el gusto estético popular, uniendo pensamiento mágico y realidad social inmediata; el símbolo religioso operaría como continente de mitos que resuelven imaginariamente las contradicciones de la vida. Recuerda que Sarita nació en Huaraz en 1914 y murió en el Callao en 1940, donde surgió su culto —hoy extendido entre los más desvalidos: el mundo del hampa, la prostitución, estibadores y choferes—, con un mausoleo-santuario rodeado de exvotos y comerciantes ambulantes. La sección 'Sarita en el arte' presenta y reproduce la obra 'Arte al Paso', un enorme rostro de Sarita compuesto con cerca de 12,000 latas de leche, realizado por un conjunto de artistas jóvenes reunidos en el Taller de Estética de Proyección Social 'Huayco' (E.P.S. Huayco): Francisco Mariotti, María Luy, Gerbert Rodríguez, Mariella Zevallos, Armando Williams y Charo Noriega. Instalada desde enero de ese año a la vera del sur, la obra recoge en clave colectiva la significación sociocultural de Sarita para ofrecer a viajeros y peregrinos una exposición permanente de esa imagen, integrando la escala monumental, la soledad del paisaje y una identificación plástica con el misterio cotidiano. Es documento clave sobre el vínculo entre religiosidad popular, migración andina y vanguardia peruana de inicios de los ochenta.</t>
         </is>
       </c>
     </row>
@@ -1982,27 +1982,27 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Screen Shot 2026-07-16 at 13.03.35.png</t>
+          <t>Screen Shot 2026-07-16 at 08.37.09.png</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>1970-1981</t>
+          <t>1965-1984</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Captura de pantalla (16-07-2026) de artículo de revista, 1981</t>
+          <t>Captura de pantalla, 16-07-2026 (de un cuadro/gráfico basado en el informe de Alfonso Castrillón, 'Reflexiones sobre el arte conceptual en el Perú y sus proyecciones', Hueso Húmero n.º 7; sello UNMSM)</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Juan Acha; Hueso Húmero (revista); UNMSM; José Carlos Mariátegui (contexto marxista); El Sexto (prisión); México D.F.</t>
+          <t>Alfonso Castrillón; Juan Acha; Teresa Burga; Emilio Hernández; Rafael Hastings; Francisco Mariotti; Luis Arias Vera; Jorge Eielson; Wiley Ludeña; Herbert Rodríguez; E.P.S. Huayco; Grupo Paréntesis; UNMSM</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>La captura reproduce la primera página del texto autobiográfico y ensayístico de Juan Acha titulado 'Por qué no vivo en el Perú', encabezado por una nota editorial de la revista Hueso Húmero que enmarca el escrito dentro de una indagación colectiva sobre los creadores e intelectuales peruanos que optaron por emigrar, problema que la publicación se propone tratar con seriedad y continuar en números sucesivos. Acha, crítico y teórico del arte dedicado a los problemas latinoamericanos, ordena sus razones para no residir en el Perú en dos clases jerarquizadas: las 'de afuera', que considera principales, y las 'de adentro', secundarias. Bajo las primeras enumera lo que encontró en México y le faltaba en su país: amplias posibilidades de publicar en diarios y revistas, colaborar en museos e institutos, investigar y enseñar en universidades como crítico de arte, todo ello remunerado con dignidad; libertad de expresión e intensa circulación de ideas marxistas en libros, revistas y simposios; y un prestigio nacional de las artes visuales sostenido por el Estado, con una activa política museográfica y de simposios además de facilidades para viajar y entrar en contacto con el arte de otras latitudes. El fragmento evidencia la tesis central del autor: la emigración no responde a un rechazo personal sino a la asimetría estructural entre el medio cultural peruano, precario y cerrado, y el mexicano, mejor equipado y más poroso al quehacer cultural latinoamericano. El documento funciona como fuente primaria sobre las condiciones institucionales del campo artístico peruano y sobre la trayectoria del propio Acha como figura clave de la teoría del arte no objetual en América Latina.</t>
+          <t>Captura de pantalla de un cuadro cronológico ('Gráfico 1') que sistematiza el desarrollo del arte conceptual y no-objetual en el Perú entre 1965 y 1984, elaborado 'en base al informe de Alfonso Castrillón: Reflexiones sobre el arte conceptual en el Perú y sus proyecciones' (Hueso Húmero 7). El cuadro organiza la información en cuatro columnas —Fecha, Tendencia, Operador (artistas y grupos) y Lugar— trazando la sucesión de tendencias: pop y op (1965, Galería Lima, IAC), concepto y ambientes (1969-1970, con Juan Acha, 'Cultura y Libertad'), acciones y eventos (1972-1975: Teresa Burga, Rafael Hastings, Francisco Mariotti, CONTACTA, Premio López Antay, Festival Inkarri), y las prácticas de no-objeto y performance de fines de los setenta y de los ochenta. Registra los colectivos 'Signo x signo' (Patricia López, Armando Williams, Rossana Agois, Wiley Ludeña, Hugo Salazar), el Grupo USM de Alfonso Castrillón, 'Paréntesis' (Charo Noriega, Armando Williams, María Luy, Francisco Mariotti, Fernando Bedoya, Juan J. Salazar, Mariela Zevallos) y 'Huayco EPS' (Herbert Rodríguez, Lucy Angulo, José Morales), junto a nombres como Luis Arias Vera, Emilio Hernández, Jorge Eielson, Hernán Pazos, Esther Vainstein, Cecilia Paredes y Sergio Zevallos. Consigna hitos y sedes: encuestas, la Bienal no-objetual de Medellín, la Bienal de São Paulo (1983), la acción 'Cuidado pintores…', y espacios como el Instituto Italiano, la Universidad de San Marcos y galerías limeñas. Funciona como mapa genealógico de la vanguardia experimental peruana y de sus operadores institucionales, útil para periodizar el paso del conceptualismo a la performance y al arte no-objetual.</t>
         </is>
       </c>
     </row>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Screen Shot 2026-07-16 at 13.03.44.png</t>
+          <t>Screen Shot 2026-07-16 at 13.03.35.png</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2029,12 +2029,12 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Juan Acha; Hueso Húmero (revista); El Sexto (prisión de Lima); México D.F.; UNMSM</t>
+          <t>Juan Acha; Hueso Húmero (revista); UNMSM; José Carlos Mariátegui (contexto marxista); El Sexto (prisión); México D.F.</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>La captura corresponde a la página 109 (sección 'Encuesta') y continúa el texto de Juan Acha 'Por qué no vivo en el Perú', cerrando la argumentación iniciada en la página anterior. Bajo las razones 'de afuera' Acha añade dos motivos vinculados a su vocación latinoamericanista: México ofrece un mejor enfoque de los problemas artísticos y culturales de 'nuestra América' porque, por su tamaño demográfico e importancia y por su industria editora, allí confluyen antes que en otros países los fenómenos y las investigaciones del resto de Latinoamérica; y propicia una identificación cultural más conflictiva y acorde a la realidad concreta, con un aprecio por la cultura popular en la que halla semejanzas con el Perú. Luego expone tres razones 'secundarias', personales, que lo empujaron a salir: haber vivido y formado universitariamente fuera del país trabajando como químico en varios países latinoamericanos, lo que facilitó su salida y le dio mejor visión de virtudes y defectos nacionales; el clima represivo y discriminante de la capital, producto del 'aristocratismo limeño' y su racismo disimulado, del nepotismo de las clases dominantes y la represión de lo popular; y, sobre todo, haber sido fichado en 1970 como supuesto inculpado de tráfico de drogas al asistir a una fiesta de artistas jóvenes, sufriendo diez días de vejaciones en la prisión El Sexto por negligencia judicial antes de ser declarado inocente. El texto, firmado en México D.F. en febrero de 1981, articula crítica estructural del campo cultural peruano con testimonio personal de exclusión y violencia institucional.</t>
+          <t>La captura reproduce la primera página del texto autobiográfico y ensayístico de Juan Acha titulado 'Por qué no vivo en el Perú', encabezado por una nota editorial de la revista Hueso Húmero que enmarca el escrito dentro de una indagación colectiva sobre los creadores e intelectuales peruanos que optaron por emigrar, problema que la publicación se propone tratar con seriedad y continuar en números sucesivos. Acha, crítico y teórico del arte dedicado a los problemas latinoamericanos, ordena sus razones para no residir en el Perú en dos clases jerarquizadas: las 'de afuera', que considera principales, y las 'de adentro', secundarias. Bajo las primeras enumera lo que encontró en México y le faltaba en su país: amplias posibilidades de publicar en diarios y revistas, colaborar en museos e institutos, investigar y enseñar en universidades como crítico de arte, todo ello remunerado con dignidad; libertad de expresión e intensa circulación de ideas marxistas en libros, revistas y simposios; y un prestigio nacional de las artes visuales sostenido por el Estado, con una activa política museográfica y de simposios además de facilidades para viajar y entrar en contacto con el arte de otras latitudes. El fragmento evidencia la tesis central del autor: la emigración no responde a un rechazo personal sino a la asimetría estructural entre el medio cultural peruano, precario y cerrado, y el mexicano, mejor equipado y más poroso al quehacer cultural latinoamericano. El documento funciona como fuente primaria sobre las condiciones institucionales del campo artístico peruano y sobre la trayectoria del propio Acha como figura clave de la teoría del arte no objetual en América Latina.</t>
         </is>
       </c>
     </row>
@@ -2046,27 +2046,27 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>VVAA - El desencantamiento del arte. Conversación de egresados con Jorge Villacorta [Ansible].md</t>
+          <t>Screen Shot 2026-07-16 at 13.03.44.png</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>2013-2018 (coyuntura reciente, con referencias a los años ochenta)</t>
+          <t>1970-1981</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Conversación colectiva publicada en revista (Ansible), ca. 2018 (s/f exacta)</t>
+          <t>Captura de pantalla (16-07-2026) de artículo de revista, 1981</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Adriana Bickel; Rafael Nolte; Rox Monteverde; Kenji Quispe; Mariana Román; Raúl Silva; Michael Prado; Alfredo Bernal; PUCP; ENSABAP; Corriente Alterna; Centro de la Imagen; galería 80m2 Livia Benavides; Revolver; Mario Testino; Rodrigo Quijano</t>
+          <t>Juan Acha; Hueso Húmero (revista); El Sexto (prisión de Lima); México D.F.; UNMSM</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Conversación colectiva entre egresados y estudiantes recientes de las principales escuelas de artes visuales de Lima (PUCP, ENSABAP-Bellas Artes, Corriente Alterna, Centro de la Imagen), con intervención del crítico Jorge Villacorta, publicada en la revista Ansible. El diálogo diagnostica un momento de «desencantamiento» e inflexión entre un pasado precario y un futuro incierto en el campo laboral del arte. Los participantes (Adriana Bickel, Rafael Nolte, Rox Monteverde, Kenji Quispe, Mariana Román, Raúl Silva, Michael Prado, Alfredo Bernal) analizan factores recientes: el surgimiento de ferias (P.Ar.C., Art Lima), la internacionalización de galerías (Revolver, 80m2 Livia Benavides), las vanity gallery, el coleccionismo concentrado de Hochschild y Verme, el libro de Mario Testino, la gentrificación de Monumental Callao y el escándalo del pabellón peruano en la Bienal de Venecia 2017 (obra de Juan Javier Salazar, retirada del curador Rodrigo Quijano). El eje conceptual gira en torno al mercado como fuerza hegemónica que guía la cultura, la ausencia de aparato crítico e histórico, el auge de la autogestión como «arma de doble filo» y la imposibilidad de agremiación en un medio fragmentado y competitivo. Villacorta aporta la memoria histórica de la ASPAP (años ochenta) y el contraste con la colegiatura profesional y la AICA. Se debaten la profesionalización, la legitimación externa del artista (por sociólogos, curadores, museos), la deficiente formación que provoca el éxodo de artistas, los cambios curriculares hacia el «artista-investigador» (2010-2011) y lo aspiracional del éxito comercial. El texto expone críticamente la vulnerabilidad estructural del artista joven limeño.</t>
+          <t>La captura corresponde a la página 109 (sección 'Encuesta') y continúa el texto de Juan Acha 'Por qué no vivo en el Perú', cerrando la argumentación iniciada en la página anterior. Bajo las razones 'de afuera' Acha añade dos motivos vinculados a su vocación latinoamericanista: México ofrece un mejor enfoque de los problemas artísticos y culturales de 'nuestra América' porque, por su tamaño demográfico e importancia y por su industria editora, allí confluyen antes que en otros países los fenómenos y las investigaciones del resto de Latinoamérica; y propicia una identificación cultural más conflictiva y acorde a la realidad concreta, con un aprecio por la cultura popular en la que halla semejanzas con el Perú. Luego expone tres razones 'secundarias', personales, que lo empujaron a salir: haber vivido y formado universitariamente fuera del país trabajando como químico en varios países latinoamericanos, lo que facilitó su salida y le dio mejor visión de virtudes y defectos nacionales; el clima represivo y discriminante de la capital, producto del 'aristocratismo limeño' y su racismo disimulado, del nepotismo de las clases dominantes y la represión de lo popular; y, sobre todo, haber sido fichado en 1970 como supuesto inculpado de tráfico de drogas al asistir a una fiesta de artistas jóvenes, sufriendo diez días de vejaciones en la prisión El Sexto por negligencia judicial antes de ser declarado inocente. El texto, firmado en México D.F. en febrero de 1981, articula crítica estructural del campo cultural peruano con testimonio personal de exclusión y violencia institucional.</t>
         </is>
       </c>
     </row>
@@ -2078,27 +2078,27 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>VVAA - Lima se anima. Debates en la escena artística peruana (2009) [ramona 89].md</t>
+          <t>VVAA - El desencantamiento del arte. Conversación de egresados con Jorge Villacorta [Ansible].md</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>1997-2009 (última década, de la Bienal Iberoamericana al presente)</t>
+          <t>2013-2018 (coyuntura reciente, con referencias a los años ochenta)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Dossier de revista (ramona nº 89), abril 2009</t>
+          <t>Conversación colectiva publicada en revista (Ansible), ca. 2018 (s/f exacta)</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Quijano; Eliana Otta; Miguel López; Max Hernández-Calvo; Gustavo Buntinx; Jorge Villacorta; Alfredo Márquez; Fernando Bryce; Gilda Mantilla; Philippe Gruenberg; Giancarlo Scaglia; revista Juanacha; La Culpable; MALI; galería Revólver</t>
+          <t>Jorge Villacorta; Adriana Bickel; Rafael Nolte; Rox Monteverde; Kenji Quispe; Mariana Román; Raúl Silva; Michael Prado; Alfredo Bernal; PUCP; ENSABAP; Corriente Alterna; Centro de la Imagen; galería 80m2 Livia Benavides; Revolver; Mario Testino; Rodrigo Quijano</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Dossier «Lima se anima» de la revista argentina ramona (nº 89, abril 2009), coeditado con la publicación limeña Juanacha por Rodrigo Quijano y Eliana Otta, que ofrece una radiografía crítica de la escena artística peruana ante su reciente revinculación con el circuito internacional. Reúne una conversación entre artistas («Perú, ¿país blindado?») con Alfredo Márquez, Fernando Bryce, Gilda Mantilla, Philippe Gruenberg y Giancarlo Scaglia; ensayos de Miguel López y Max Hernández-Calvo; un debate virtual del blog Arte-Nuevo sobre las políticas museales; un texto de Gustavo Buntinx (Micromuseo) y una entrevista a Jorge Villacorta. El hilo común es la interrogación del supuesto «boom» del arte contemporáneo limeño de la última década: los participantes coinciden en que la internacionalización y el crecimiento del mercado y del coleccionismo (impulsado por el MALI) han producido una escena «contrahecha», con brazos de mercado pero sin instituciones, crítica, educación ni políticas culturales. Márquez denuncia el carácter colonial y exótico de esa visibilidad; López («Boo(o)m: Morir de éxito») teoriza un proceso de despolitización y domesticación que diluye el conflicto y convierte la autonomía en aquiescencia entre agentes; Hernández-Calvo («Una coyuntura que no fue») analiza cómo las Bienales de Lima (1997-2002) forzaron una «contemporaneización» de instalación y video sin sustento curatorial ni educativo, generando escisiones entre circuito oficial y alternativo. Se abordan además el éxodo de artistas por la deficiente formación, la toma estudiantil de Bellas Artes, la autogestión (La Culpable) y las disputas por el Museo de la Memoria. El dossier reivindica la autonomía, el disenso y el filo crítico histórico del arte peruano.</t>
+          <t>Conversación colectiva entre egresados y estudiantes recientes de las principales escuelas de artes visuales de Lima (PUCP, ENSABAP-Bellas Artes, Corriente Alterna, Centro de la Imagen), con intervención del crítico Jorge Villacorta, publicada en la revista Ansible. El diálogo diagnostica un momento de «desencantamiento» e inflexión entre un pasado precario y un futuro incierto en el campo laboral del arte. Los participantes (Adriana Bickel, Rafael Nolte, Rox Monteverde, Kenji Quispe, Mariana Román, Raúl Silva, Michael Prado, Alfredo Bernal) analizan factores recientes: el surgimiento de ferias (P.Ar.C., Art Lima), la internacionalización de galerías (Revolver, 80m2 Livia Benavides), las vanity gallery, el coleccionismo concentrado de Hochschild y Verme, el libro de Mario Testino, la gentrificación de Monumental Callao y el escándalo del pabellón peruano en la Bienal de Venecia 2017 (obra de Juan Javier Salazar, retirada del curador Rodrigo Quijano). El eje conceptual gira en torno al mercado como fuerza hegemónica que guía la cultura, la ausencia de aparato crítico e histórico, el auge de la autogestión como «arma de doble filo» y la imposibilidad de agremiación en un medio fragmentado y competitivo. Villacorta aporta la memoria histórica de la ASPAP (años ochenta) y el contraste con la colegiatura profesional y la AICA. Se debaten la profesionalización, la legitimación externa del artista (por sociólogos, curadores, museos), la deficiente formación que provoca el éxodo de artistas, los cambios curriculares hacia el «artista-investigador» (2010-2011) y lo aspiracional del éxito comercial. El texto expone críticamente la vulnerabilidad estructural del artista joven limeño.</t>
         </is>
       </c>
     </row>
@@ -2110,27 +2110,27 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>VVAA - Memorias del subdesarrollo. Arte y el giro descolonial en América Latina, 1960-1985 [catálogo MCASD].md</t>
+          <t>VVAA - Lima se anima. Debates en la escena artística peruana (2009) [ramona 89].md</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>1960-1985 (con foco 1967-1981)</t>
+          <t>1997-2009 (última década, de la Bienal Iberoamericana al presente)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de exposición / ensayo académico, 2018 (MCASD)</t>
+          <t>Dossier de revista (ramona nº 89), abril 2009</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Julieta González; Andrea Giunta; Jacopo Crivelli Visconti; Juan Acha; Marta Traba; Ferreira Gullar; Teresa Burga; E.P.S. Huayco; Grupo Paréntesis; Jesús Ruiz Durand; Fernando 'Coco' Bedoya; MALI; Museum of Contemporary Art San Diego</t>
+          <t>Rodrigo Quijano; Eliana Otta; Miguel López; Max Hernández-Calvo; Gustavo Buntinx; Jorge Villacorta; Alfredo Márquez; Fernando Bryce; Gilda Mantilla; Philippe Gruenberg; Giancarlo Scaglia; revista Juanacha; La Culpable; MALI; galería Revólver</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>El ensayo de Sharon Lerner incluido en el catálogo de la exposición 'Memorias del subdesarrollo: arte y el giro descolonial en América Latina, 1960-1985' inserta la escena peruana de 1967-1981 en una narrativa continental que postula una ruptura epistémica con lo moderno mediante la noción de subdesarrollo y el deseo de descolonizar los cánones estéticos impuestos. Su tesis desplaza el foco del paradigma formalista modernista hacia el contexto social, la apropiación de tradiciones locales y lo 'popular' como categoría clave, cuya heterogeneidad histórica advierte no homogeneizar. Reconstruye el debate entre Juan Acha y Marta Traba sobre el pop cosmopolita y la dependencia cultural, apoyándose en Mariátegui, Ferreira Gullar y Mário Pedrosa, y en la teoría de la dependencia. Analiza casos peruanos: los afiches de la Reforma Agraria de Jesús Ruiz Durand y su 'pop achorado' dentro de SINAMOS; los festivales Contacta y las Carreras de Chasquis de Luis Arias Vera bajo el velasquismo; el Grupo Paréntesis y el Contacta 79 (Becerro de oro, Coquito) de Fernando Bedoya; y sobre todo E.P.S. Huayco, con 'Arte al paso (Salchipapas)' y 'Sarita Colonia', leídos vía Buntinx y Lauer como articulación de lo popular urbano migrante. Suma el caso aislado de Teresa Burga y 'Perfil de la mujer peruana' (1980-81) como acercamiento conceptual a género y clase. Recurriendo a Bürger y Giunta, discute la definición de vanguardia y concluye que estas prácticas oscilaron entre dependencia y autonomía, sin lograr plataformas de continuidad, siendo Huayco el caso más próximo a una vanguardia local pese a su disolución.</t>
+          <t>Dossier «Lima se anima» de la revista argentina ramona (nº 89, abril 2009), coeditado con la publicación limeña Juanacha por Rodrigo Quijano y Eliana Otta, que ofrece una radiografía crítica de la escena artística peruana ante su reciente revinculación con el circuito internacional. Reúne una conversación entre artistas («Perú, ¿país blindado?») con Alfredo Márquez, Fernando Bryce, Gilda Mantilla, Philippe Gruenberg y Giancarlo Scaglia; ensayos de Miguel López y Max Hernández-Calvo; un debate virtual del blog Arte-Nuevo sobre las políticas museales; un texto de Gustavo Buntinx (Micromuseo) y una entrevista a Jorge Villacorta. El hilo común es la interrogación del supuesto «boom» del arte contemporáneo limeño de la última década: los participantes coinciden en que la internacionalización y el crecimiento del mercado y del coleccionismo (impulsado por el MALI) han producido una escena «contrahecha», con brazos de mercado pero sin instituciones, crítica, educación ni políticas culturales. Márquez denuncia el carácter colonial y exótico de esa visibilidad; López («Boo(o)m: Morir de éxito») teoriza un proceso de despolitización y domesticación que diluye el conflicto y convierte la autonomía en aquiescencia entre agentes; Hernández-Calvo («Una coyuntura que no fue») analiza cómo las Bienales de Lima (1997-2002) forzaron una «contemporaneización» de instalación y video sin sustento curatorial ni educativo, generando escisiones entre circuito oficial y alternativo. Se abordan además el éxodo de artistas por la deficiente formación, la toma estudiantil de Bellas Artes, la autogestión (La Culpable) y las disputas por el Museo de la Memoria. El dossier reivindica la autonomía, el disenso y el filo crítico histórico del arte peruano.</t>
         </is>
       </c>
     </row>
@@ -2142,27 +2142,27 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Vich - La violencia, la dictadura y la globalización. Arte y política en el Perú contemporáneo.md</t>
+          <t>VVAA - Memorias del subdesarrollo. Arte y el giro descolonial en América Latina, 1960-1985 [catálogo MCASD].md</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>1980-2009 (violencia política, dictadura fujimorista y posconflicto)</t>
+          <t>1960-1985 (con foco 1967-1981)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Ensayo / capítulo de libro académico, c. 2013-2015</t>
+          <t>Catálogo de exposición / ensayo académico, 2018 (MCASD)</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Víctor Vich; Eduardo Tokeshi; Colectivo Sociedad Civil; Natalia Iguíñiz; Sandro Venturo; Piero Quijano; Luz Letts; Víctor Delfín; Miguel Cordero; Jaime Higa; Herbert Rodríguez; Claudia Martínez; Santiago Quintanilla; Rudolph Castro; Felipe López; Gustavo Buntinx</t>
+          <t>Sharon Lerner; Julieta González; Andrea Giunta; Jacopo Crivelli Visconti; Juan Acha; Marta Traba; Ferreira Gullar; Teresa Burga; E.P.S. Huayco; Grupo Paréntesis; Jesús Ruiz Durand; Fernando 'Coco' Bedoya; MALI; Museum of Contemporary Art San Diego</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>Víctor Vich propone una lectura desde la crítica cultural del arte peruano contemporáneo, sosteniendo que, frente al discurso triunfalista del crecimiento económico, un sector de artistas sigue nombrando al país a partir de sus heridas históricas. Estructura el ensayo en torno a tres acontecimientos: la violencia política, el autoritarismo corrupto del fujimontesinismo y la globalización neoliberal. Apoyándose en Žižek, Hall, Jameson, Foucault y Badiou, entiende lo simbólico no como reflejo sino como soporte de la realidad y campo de batalla donde se disputan sentidos de ciudadanía. Analiza obras emblemáticas: 'Bandera VIII' (2000) de Eduardo Tokeshi, leída como 'la patria en cuidados intensivos'; 'Lava la bandera' del Colectivo Sociedad Civil; la instalación 'Patria' de Natalia Iguíñiz y Sandro Venturo; el afiche censurado de Piero Quijano sobre La Cantuta e Iwo Jima; 'El azar como destino' de Luz Letts; 'El hermoso general' de Víctor Delfín; el saco militar de Miguel Cordero; y las serigrafías de César Vallejo de Jaime Higa sobre posmodernismo y cultura de masas. En una segunda sección sobre memoria generacional examina a artistas nacidos en los ochenta que 'traducen' la violencia con lenguajes heredados de la infancia: la serie 'Invisible' de Claudia Martínez, el trabajo de archivo y cómic de Santiago Quintanilla, los juguetes siniestros (Lego, Playmobil) de Rudolph Castro y las fotografías de nichos ayacuchanos de Felipe López. Su aporte es articular teoría psicoanalítica y poscolonial con un corpus visual peruano, mostrando el arte crítico como agente que interrumpe la ficción neoliberal y recompone la comunidad desde el orden simbólico.</t>
+          <t>El ensayo de Sharon Lerner incluido en el catálogo de la exposición 'Memorias del subdesarrollo: arte y el giro descolonial en América Latina, 1960-1985' inserta la escena peruana de 1967-1981 en una narrativa continental que postula una ruptura epistémica con lo moderno mediante la noción de subdesarrollo y el deseo de descolonizar los cánones estéticos impuestos. Su tesis desplaza el foco del paradigma formalista modernista hacia el contexto social, la apropiación de tradiciones locales y lo 'popular' como categoría clave, cuya heterogeneidad histórica advierte no homogeneizar. Reconstruye el debate entre Juan Acha y Marta Traba sobre el pop cosmopolita y la dependencia cultural, apoyándose en Mariátegui, Ferreira Gullar y Mário Pedrosa, y en la teoría de la dependencia. Analiza casos peruanos: los afiches de la Reforma Agraria de Jesús Ruiz Durand y su 'pop achorado' dentro de SINAMOS; los festivales Contacta y las Carreras de Chasquis de Luis Arias Vera bajo el velasquismo; el Grupo Paréntesis y el Contacta 79 (Becerro de oro, Coquito) de Fernando Bedoya; y sobre todo E.P.S. Huayco, con 'Arte al paso (Salchipapas)' y 'Sarita Colonia', leídos vía Buntinx y Lauer como articulación de lo popular urbano migrante. Suma el caso aislado de Teresa Burga y 'Perfil de la mujer peruana' (1980-81) como acercamiento conceptual a género y clase. Recurriendo a Bürger y Giunta, discute la definición de vanguardia y concluye que estas prácticas oscilaron entre dependencia y autonomía, sin lograr plataformas de continuidad, siendo Huayco el caso más próximo a una vanguardia local pese a su disolución.</t>
         </is>
       </c>
     </row>
@@ -2174,27 +2174,27 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Vidarte - Exhibiciones y adquisiciones para la construcción de narrativas en la historia del arte contemporáneo peruano.md</t>
+          <t>Vich - La violencia, la dictadura y la globalización. Arte y política en el Perú contemporáneo.md</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>2015-2023</t>
+          <t>1980-2009 (violencia política, dictadura fujimorista y posconflicto)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Ensayo curatorial de catálogo, 2023</t>
+          <t>Ensayo / capítulo de libro académico, c. 2013-2015</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Giuliana Vidarte; ICPNA; Natalia Iguíñiz; Carlos García Montero; Venuca Evanán; Nereida Apaza; Gloria Quispe; Cristina Flores; Antonio Paucar; Andrés Argüelles Vigo; Carolina Estrada; Santiago Yahuarcani; Ana de Orbegoso</t>
+          <t>Víctor Vich; Eduardo Tokeshi; Colectivo Sociedad Civil; Natalia Iguíñiz; Sandro Venturo; Piero Quijano; Luz Letts; Víctor Delfín; Miguel Cordero; Jaime Higa; Herbert Rodríguez; Claudia Martínez; Santiago Quintanilla; Rudolph Castro; Felipe López; Gustavo Buntinx</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>Giuliana Vidarte reflexiona sobre la exposición 'Miradas contemporáneas. Nuevas adquisiciones en la colección ICPNA (2015-2023)', presentada en el Espacio Juan Pardo Heeren del ICPNA de Lima entre agosto y septiembre de 2023. Su argumento central es que las exhibiciones y adquisiciones institucionales son dispositivos para la construcción de narrativas y memoria crítica en la historia del arte contemporáneo peruano: una colección formada a partir de obras que fueron parte de la propia programación expositiva constituye un testimonio de los modos de creación y conserva la memoria de la historia de las exposiciones en el país. Parte de dos ganadoras del Premio ICPNA de Arte Contemporáneo, Venuca Evanán y Nereida Apaza, para introducir cómo el arte contribuye a pensar la realidad mediante reflexiones colectivas sobre violencia de género, identidad y nación. Describe los cinco ejes curatoriales de la muestra —revalorando intimidades, discursos críticos, develando entornos, reinterpretar tradiciones y estéticas disímiles— y analiza diálogos entre obras: el cuerpo y la caja torácica en Gloria Quispe, Cristina Flores y Antonio Paucar; la crítica a la representación colonial y republicana en Andrés Argüelles Vigo y Carolina Estrada/Teodoro Ramírez; el paisaje y la crisis medioambiental amazónica en Silvia Westphalen y Nicole Franchy; la reinterpretación de saberes ancestrales en Santiago Yahuarcani y Ana de Orbegoso. Destaca que las fichas incorporan citas de textos curatoriales previos, nutriendo la exposición del archivo documental institucional. Concluye que estos conjuntos abren líneas múltiples de lectura y afirman el valor del esfuerzo colectivo de gestores, curadores e investigadores en la formación de colecciones y en la escritura de la historia del arte peruano reciente.</t>
+          <t>Víctor Vich propone una lectura desde la crítica cultural del arte peruano contemporáneo, sosteniendo que, frente al discurso triunfalista del crecimiento económico, un sector de artistas sigue nombrando al país a partir de sus heridas históricas. Estructura el ensayo en torno a tres acontecimientos: la violencia política, el autoritarismo corrupto del fujimontesinismo y la globalización neoliberal. Apoyándose en Žižek, Hall, Jameson, Foucault y Badiou, entiende lo simbólico no como reflejo sino como soporte de la realidad y campo de batalla donde se disputan sentidos de ciudadanía. Analiza obras emblemáticas: 'Bandera VIII' (2000) de Eduardo Tokeshi, leída como 'la patria en cuidados intensivos'; 'Lava la bandera' del Colectivo Sociedad Civil; la instalación 'Patria' de Natalia Iguíñiz y Sandro Venturo; el afiche censurado de Piero Quijano sobre La Cantuta e Iwo Jima; 'El azar como destino' de Luz Letts; 'El hermoso general' de Víctor Delfín; el saco militar de Miguel Cordero; y las serigrafías de César Vallejo de Jaime Higa sobre posmodernismo y cultura de masas. En una segunda sección sobre memoria generacional examina a artistas nacidos en los ochenta que 'traducen' la violencia con lenguajes heredados de la infancia: la serie 'Invisible' de Claudia Martínez, el trabajo de archivo y cómic de Santiago Quintanilla, los juguetes siniestros (Lego, Playmobil) de Rudolph Castro y las fotografías de nichos ayacuchanos de Felipe López. Su aporte es articular teoría psicoanalítica y poscolonial con un corpus visual peruano, mostrando el arte crítico como agente que interrumpe la ficción neoliberal y recompone la comunidad desde el orden simbólico.</t>
         </is>
       </c>
     </row>
@@ -2206,27 +2206,27 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Villacorta - La colección Hochschild.md</t>
+          <t>Vidarte - Exhibiciones y adquisiciones para la construcción de narrativas en la historia del arte contemporáneo peruano.md</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>1980-2016 (con énfasis en el arte peruano desde 2000)</t>
+          <t>2015-2023</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo de colección, c. 2016</t>
+          <t>Ensayo curatorial de catálogo, 2023</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta Chávez; Eduardo y Mariana Hochschild; Octavio Zaya; Luis Pérez Oramas; Giancarlo Scaglia; Fernando Bryce; Teresa Burga; Tilsa Tsuchiya; Jorge Eduardo Eielson; Regina Aprijaskis; MALI; MoMA; Tate Modern</t>
+          <t>Giuliana Vidarte; ICPNA; Natalia Iguíñiz; Carlos García Montero; Venuca Evanán; Nereida Apaza; Gloria Quispe; Cristina Flores; Antonio Paucar; Andrés Argüelles Vigo; Carolina Estrada; Santiago Yahuarcani; Ana de Orbegoso</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta analiza la Colección Hochschild como caso paradigmático del coleccionismo privado de arte contemporáneo peruano, sosteniendo que todo desarrollo artístico notable requiere un coleccionismo a la altura de su ambición, junto con crítica y testimonio histórico escrito. El coleccionista, figura clave de todo sistema artístico moderno, opera a la vez como catalizador de la escena y motor del mercado. Iniciada en 2009 por Eduardo y Mariana Hochschild, la colección se distingue por seguir la dinámica actual del sistema de las artes visuales en un medio que careció de coleccionismo corporativo sostenido, escasa crítica periodística y pocas publicaciones especializadas —una 'orfandad' de los artistas. Villacorta subraya que los Hochschild rompieron el molde del coleccionismo centrado en el arte moderno al adquirir netamente arte contemporáneo con asesoramiento profesional (Luis Pérez Oramas, Giancarlo Scaglia) en ausencia de una historiografía orgánica del arte peruano desde 1980. Contextualiza el aislamiento económico y la violencia de los años ochenta y noventa que invisibilizaron a dos generaciones de artistas, y el dinamismo que trajeron la Bienal Iberoamericana de Lima (1997) y el Festival de Video/Arte Electrónico (1998). Comenta la selección de Octavio Zaya para 'Próxima parada' y la tríada Aprijaskis-Eielson-Burga como artistas que escapan al arte moderno local e inauguran lo contemporáneo. Ejemplifica el 'punto ciego' del coleccionista limeño con 'Atlas Perú' de Fernando Bryce, vendido al exterior, y aborda la tensión entre relevancia cultural nacional y reconocimiento del mercado internacional. Cita cimientos modernos (Sabogal, Szyszlo, Tsuchiya) y fortalezas en escultura, instalación y fotografía (Chambi, Testino, Martinat, Damiani), afirmando que la colección materializa una visión cabal del arte peruano contemporáneo.</t>
+          <t>Giuliana Vidarte reflexiona sobre la exposición 'Miradas contemporáneas. Nuevas adquisiciones en la colección ICPNA (2015-2023)', presentada en el Espacio Juan Pardo Heeren del ICPNA de Lima entre agosto y septiembre de 2023. Su argumento central es que las exhibiciones y adquisiciones institucionales son dispositivos para la construcción de narrativas y memoria crítica en la historia del arte contemporáneo peruano: una colección formada a partir de obras que fueron parte de la propia programación expositiva constituye un testimonio de los modos de creación y conserva la memoria de la historia de las exposiciones en el país. Parte de dos ganadoras del Premio ICPNA de Arte Contemporáneo, Venuca Evanán y Nereida Apaza, para introducir cómo el arte contribuye a pensar la realidad mediante reflexiones colectivas sobre violencia de género, identidad y nación. Describe los cinco ejes curatoriales de la muestra —revalorando intimidades, discursos críticos, develando entornos, reinterpretar tradiciones y estéticas disímiles— y analiza diálogos entre obras: el cuerpo y la caja torácica en Gloria Quispe, Cristina Flores y Antonio Paucar; la crítica a la representación colonial y republicana en Andrés Argüelles Vigo y Carolina Estrada/Teodoro Ramírez; el paisaje y la crisis medioambiental amazónica en Silvia Westphalen y Nicole Franchy; la reinterpretación de saberes ancestrales en Santiago Yahuarcani y Ana de Orbegoso. Destaca que las fichas incorporan citas de textos curatoriales previos, nutriendo la exposición del archivo documental institucional. Concluye que estos conjuntos abren líneas múltiples de lectura y afirman el valor del esfuerzo colectivo de gestores, curadores e investigadores en la formación de colecciones y en la escritura de la historia del arte peruano reciente.</t>
         </is>
       </c>
     </row>
@@ -2238,27 +2238,27 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Villacorta - Un arte cuestionador. De Dadá a La Cantuta [Quehacer 102, pdf pp. 96-105].md</t>
+          <t>Villacorta - La colección Hochschild.md</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>1916-1996 (vanguardias históricas y arte peruano 1979-1995)</t>
+          <t>1980-2016 (con énfasis en el arte peruano desde 2000)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Artículo de revista (Quehacer 102, DESCO), c. 1996</t>
+          <t>Ensayo de catálogo de colección, c. 2016</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Francisco Mariotti; Herbert Rodríguez; Ricardo Wiesse; Eduardo Villanes; Hugo Salazar del Alcázar; E.P.S. Huayco; Grupo Paréntesis; Los Bestias; Carpa Teatro del Puente Santa Rosa; Sendero Luminoso</t>
+          <t>Jorge Villacorta Chávez; Eduardo y Mariana Hochschild; Octavio Zaya; Luis Pérez Oramas; Giancarlo Scaglia; Fernando Bryce; Teresa Burga; Tilsa Tsuchiya; Jorge Eduardo Eielson; Regina Aprijaskis; MALI; MoMA; Tate Modern</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>En este artículo para la revista Quehacer (DESCO), dedicado in memoriam a Hugo Salazar del Alcázar, Jorge Villacorta traza una genealogía del arte peruano contestatario que la generación más joven de artistas visuales estaría redescubriendo como una tradición alternativa o 'canon no-oficial', paralelo al aceptado. Su tesis vincula esa tradición local con las vanguardias históricas internacionales: la deuda con Dadá (Zúrich, 1916) como rechazo crítico de la civilización occidental tras la carnicería bélica, el manifiesto como obra del futurismo, y el constructivismo ruso con su noción de arte como agit-prop. Aplica ese marco a la 'movida barranquina' de fines de los años setenta, primera generación ligada a una cultura juvenil limeña irreverente y a los medios masivos, donde grupos como Paréntesis y Huayco entendieron la creación como provocación y enfrentamiento; destaca la serigrafía enseñada por Mariotti y la salida de Huayco de la galería hacia el kilómetro 54 de la Panamericana Sur. Narra luego cómo la violencia de Sendero Luminoso desde 1980, el fracaso de Izquierda Unida y la crisis marcaron el clima cultural: la exposición de Artistas Visuales Asociados (1983) y 'Por el Derecho a la Vida' (1985). Analiza la escena subterránea y la Carpa Teatro del Puente Santa Rosa (1986), con Los Bestias y el fanzine, y el proyecto solitario Arte Vida de Herbert Rodríguez en San Marcos entre 1986 y 1992. Concluye con la respuesta ética ante el caso La Cantuta: la exposición de Eduardo Villanes con cajas de leche Gloria (1994) y la acción ambiental de Ricardo Wiesse con flores de cantuta en Cieneguilla (1995), afirmando un arte que asume responsabilidades éticas frente a los desaparecidos.</t>
+          <t>Jorge Villacorta analiza la Colección Hochschild como caso paradigmático del coleccionismo privado de arte contemporáneo peruano, sosteniendo que todo desarrollo artístico notable requiere un coleccionismo a la altura de su ambición, junto con crítica y testimonio histórico escrito. El coleccionista, figura clave de todo sistema artístico moderno, opera a la vez como catalizador de la escena y motor del mercado. Iniciada en 2009 por Eduardo y Mariana Hochschild, la colección se distingue por seguir la dinámica actual del sistema de las artes visuales en un medio que careció de coleccionismo corporativo sostenido, escasa crítica periodística y pocas publicaciones especializadas —una 'orfandad' de los artistas. Villacorta subraya que los Hochschild rompieron el molde del coleccionismo centrado en el arte moderno al adquirir netamente arte contemporáneo con asesoramiento profesional (Luis Pérez Oramas, Giancarlo Scaglia) en ausencia de una historiografía orgánica del arte peruano desde 1980. Contextualiza el aislamiento económico y la violencia de los años ochenta y noventa que invisibilizaron a dos generaciones de artistas, y el dinamismo que trajeron la Bienal Iberoamericana de Lima (1997) y el Festival de Video/Arte Electrónico (1998). Comenta la selección de Octavio Zaya para 'Próxima parada' y la tríada Aprijaskis-Eielson-Burga como artistas que escapan al arte moderno local e inauguran lo contemporáneo. Ejemplifica el 'punto ciego' del coleccionista limeño con 'Atlas Perú' de Fernando Bryce, vendido al exterior, y aborda la tensión entre relevancia cultural nacional y reconocimiento del mercado internacional. Cita cimientos modernos (Sabogal, Szyszlo, Tsuchiya) y fortalezas en escultura, instalación y fotografía (Chambi, Testino, Martinat, Damiani), afirmando que la colección materializa una visión cabal del arte peruano contemporáneo.</t>
         </is>
       </c>
     </row>
@@ -2270,27 +2270,27 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Villacorta y Del Valle - Incertidumbre y certezas en el arte peruano reciente. Imaginarios de Lima en transformación 1980-2006 [Post-Ilusiones].txt</t>
+          <t>Villacorta - Un arte cuestionador. De Dadá a La Cantuta [Quehacer 102, pdf pp. 96-105].md</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>1919-2006 (con eje central 1980-2006)</t>
+          <t>1916-1996 (vanguardias históricas y arte peruano 1979-1995)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de libro/catálogo (Post-Ilusiones), c. 2007</t>
+          <t>Artículo de revista (Quehacer 102, DESCO), c. 1996</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta Chávez; Augusto del Valle Cárdenas; José Sabogal; Juan Acha; Marta Traba; Fernando de Szyszlo; Jorge Eduardo Eielson; Emilio Rodríguez Larraín; E.P.S. Huayco; Escuela Nacional de Bellas Artes; IAC; Agrupación Espacio</t>
+          <t>Jorge Villacorta; Francisco Mariotti; Herbert Rodríguez; Ricardo Wiesse; Eduardo Villanes; Hugo Salazar del Alcázar; E.P.S. Huayco; Grupo Paréntesis; Los Bestias; Carpa Teatro del Puente Santa Rosa; Sendero Luminoso</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta y Augusto del Valle proponen un ensayo panorámico sobre el arte peruano reciente que lee la transformación de los imaginarios de Lima entre 1980 y 2006 a partir de una tesis de fondo: en el Perú la academia y sus modelos artísticos comenzaron tarde e hicieron crisis temprano. Recorren la fundación de la Escuela Nacional de Bellas Artes (1919), la retorización del indigenismo de Sabogal como vanguardia institucionalizada, el rol del IAC (1955-1972) en la difusión del arte 'culto' y su negociación con modelos norteamericanos, y la tensión entre 'alta' y 'baja' cultura heredada de la intelligentsia marxista tras la Revolución cubana. Interpretan el populismo cultural del gobierno militar (Velasco y Morales Bermúdez), el premio a López Antay (1975) y el receso de Bellas Artes (1977) como síntomas del agotamiento de una visión del arte, frente al modelo pedagógico expresivo-trascendente de Winternitz en la PUCP. El eje del texto es la categoría de no-objetualismo de Juan Acha, que articulan en dos oleadas: un primer no-objetualismo utópico de izquierda (E.P.S. Huayco) y un segundo, ligado a la Movida Subterránea y a la Carpa Teatro del Puente Santa Rosa (1986). Analizan la precariedad de los años ochenta bajo la violencia y la crisis del primer gobierno de García, el neoliberalismo autocrático fujimorista como silenciador del arte crítico y productor de espectáculo, y la centralidad creciente de la fotografía, el video y el arte electrónico desde las bienales de Lima (1997) y el Festival de Video (1998). Concluyen con el tránsito del no-objetualismo político al poético y con la 'choledad digital' y la globalización del imaginario como horizonte contemporáneo.</t>
+          <t>En este artículo para la revista Quehacer (DESCO), dedicado in memoriam a Hugo Salazar del Alcázar, Jorge Villacorta traza una genealogía del arte peruano contestatario que la generación más joven de artistas visuales estaría redescubriendo como una tradición alternativa o 'canon no-oficial', paralelo al aceptado. Su tesis vincula esa tradición local con las vanguardias históricas internacionales: la deuda con Dadá (Zúrich, 1916) como rechazo crítico de la civilización occidental tras la carnicería bélica, el manifiesto como obra del futurismo, y el constructivismo ruso con su noción de arte como agit-prop. Aplica ese marco a la 'movida barranquina' de fines de los años setenta, primera generación ligada a una cultura juvenil limeña irreverente y a los medios masivos, donde grupos como Paréntesis y Huayco entendieron la creación como provocación y enfrentamiento; destaca la serigrafía enseñada por Mariotti y la salida de Huayco de la galería hacia el kilómetro 54 de la Panamericana Sur. Narra luego cómo la violencia de Sendero Luminoso desde 1980, el fracaso de Izquierda Unida y la crisis marcaron el clima cultural: la exposición de Artistas Visuales Asociados (1983) y 'Por el Derecho a la Vida' (1985). Analiza la escena subterránea y la Carpa Teatro del Puente Santa Rosa (1986), con Los Bestias y el fanzine, y el proyecto solitario Arte Vida de Herbert Rodríguez en San Marcos entre 1986 y 1992. Concluye con la respuesta ética ante el caso La Cantuta: la exposición de Eduardo Villanes con cajas de leche Gloria (1994) y la acción ambiental de Ricardo Wiesse con flores de cantuta en Cieneguilla (1995), afirmando un arte que asume responsabilidades éticas frente a los desaparecidos.</t>
         </is>
       </c>
     </row>
@@ -2302,27 +2302,27 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Villegas_Fernando_La_relacion_entre_arte.pdf</t>
+          <t>Villacorta y Del Valle - Incertidumbre y certezas en el arte peruano reciente. Imaginarios de Lima en transformación 1980-2006 [Post-Ilusiones].txt</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>1920-1976 (con proyecciones hasta 2013)</t>
+          <t>1919-2006 (con eje central 1980-2006)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico, 2013 (Revista de Historiografía, N.º 19)</t>
+          <t>Ensayo de libro/catálogo (Post-Ilusiones), c. 2007</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Fernando Villegas; José Sabogal; Joaquín López Antay; José Carlos Mariátegui; Fernando de Szyszlo; Carlos Quízpez Asín; Instituto de Arte Peruano; Amauta; ASPAP; Juan Velasco Alvarado; Universidad Complutense de Madrid; Néstor García Canclini</t>
+          <t>Jorge Villacorta Chávez; Augusto del Valle Cárdenas; José Sabogal; Juan Acha; Marta Traba; Fernando de Szyszlo; Jorge Eduardo Eielson; Emilio Rodríguez Larraín; E.P.S. Huayco; Escuela Nacional de Bellas Artes; IAC; Agrupación Espacio</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Artículo de Fernando Villegas (Universidad Complutense de Madrid), publicado en la Revista de Historiografía N.º 19 (2013, pp. 75-87), que rastrea la evolución de los enfoques ideológicos sobre el arte popular peruano vinculando arte y política en dos momentos clave. El primero es el proyecto mestizo de José Sabogal en los años veinte: tras su viaje a México (1923) y en sintonía con la búsqueda de peruanidad de Mariátegui y la revista Amauta, Sabogal revaloriza mates burilados, queros y retablos como productos mestizos, fusión de lo indígena precolombino y lo virreinal hispano. Desde el Instituto de Arte Peruano (1931) su grupo estudia la cerámica precolombina, el color y las artes populares, legitimando estos objetos por su origen indígena pero desplazando al artista popular como creador (los pintores urbanos se autoproclaman sus 'descubridores'). El segundo momento es la polémica de 1975-1976, cuando el gobierno militar de Velasco otorgó el Premio Nacional de Cultura al retablista ayacuchano Joaquín López Antay; la ASPAP y artistas académicos lo descalificaron como 'artesano', reproduciendo la jerarquía social y racial limeña. Villegas argumenta que ambos episodios responden a gobiernos autoritarios que legitimaron el arte popular para oponerse a la oligarquía limeña, y que el criterio de validación siempre fue estético-cronológico, ignorando el proceso histórico. El marco conceptual moviliza a Mariátegui, a Clifford (apropiación de objetos de otras culturas) y a García Canclini (descontextualización). Su aporte es evidenciar la ausencia del artista popular como sujeto de su propia obra y la carga étnica y de clase que desnaturaliza el proceso creativo andino en el circuito artístico peruano.</t>
+          <t>Jorge Villacorta y Augusto del Valle proponen un ensayo panorámico sobre el arte peruano reciente que lee la transformación de los imaginarios de Lima entre 1980 y 2006 a partir de una tesis de fondo: en el Perú la academia y sus modelos artísticos comenzaron tarde e hicieron crisis temprano. Recorren la fundación de la Escuela Nacional de Bellas Artes (1919), la retorización del indigenismo de Sabogal como vanguardia institucionalizada, el rol del IAC (1955-1972) en la difusión del arte 'culto' y su negociación con modelos norteamericanos, y la tensión entre 'alta' y 'baja' cultura heredada de la intelligentsia marxista tras la Revolución cubana. Interpretan el populismo cultural del gobierno militar (Velasco y Morales Bermúdez), el premio a López Antay (1975) y el receso de Bellas Artes (1977) como síntomas del agotamiento de una visión del arte, frente al modelo pedagógico expresivo-trascendente de Winternitz en la PUCP. El eje del texto es la categoría de no-objetualismo de Juan Acha, que articulan en dos oleadas: un primer no-objetualismo utópico de izquierda (E.P.S. Huayco) y un segundo, ligado a la Movida Subterránea y a la Carpa Teatro del Puente Santa Rosa (1986). Analizan la precariedad de los años ochenta bajo la violencia y la crisis del primer gobierno de García, el neoliberalismo autocrático fujimorista como silenciador del arte crítico y productor de espectáculo, y la centralidad creciente de la fotografía, el video y el arte electrónico desde las bienales de Lima (1997) y el Festival de Video (1998). Concluyen con el tránsito del no-objetualismo político al poético y con la 'choledad digital' y la globalización del imaginario como horizonte contemporáneo.</t>
         </is>
       </c>
     </row>
@@ -2334,27 +2334,27 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>canepa_kg_2006_p132-167.pdf</t>
+          <t>Villegas_Fernando_La_relacion_entre_arte.pdf</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>1970-2006 (con referencias históricas desde el siglo XIX)</t>
+          <t>1920-1976 (con proyecciones hasta 2013)</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro, 2006</t>
+          <t>Artículo académico, 2013 (Revista de Historiografía, N.º 19)</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Giuliana Borea Labarthe; Gisela Cánepa Koch (ed.); Sandra Gamarra (LiMAC); Instituto de Arte Contemporáneo (IAC); Fernando de Szyszlo; Gerardo Chávez; Mario Vargas Llosa; Ramiro Llona; Instituto Nacional de Cultura; ICOM; Museo de la Nación; Museo Nacional de la Cultura Peruana; Alfonso Castrillón</t>
+          <t>Fernando Villegas; José Sabogal; Joaquín López Antay; José Carlos Mariátegui; Fernando de Szyszlo; Carlos Quízpez Asín; Instituto de Arte Peruano; Amauta; ASPAP; Juan Velasco Alvarado; Universidad Complutense de Madrid; Néstor García Canclini</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Capítulo de Giuliana Borea Labarthe ('Museos y esfera pública: espacio, discursos y prácticas. Reflexiones en torno a la ciudad de Lima') incluido en el volumen editado por Gisela Cánepa Koch, 'Mirando la esfera pública desde la cultura en el Perú' (2006). Partiendo de las nociones de esfera pública (Habermas), cultura pública (Appadurai) y de la nueva museología surgida de las crisis de los años 70-80 (Mesa de Santiago 1972, redefinición del ICOM 1974, ecomuseos), Borea concibe el museo como contenedor y contenido, plataforma y discurso, esfera de poder y arena de disputa por la representación. Analiza tres casos limeños. Primero, el posicionamiento urbano de los museos: mediante una encuesta a transeúntes y taxistas muestra que solo el Museo de la Nación y el Museo de Arte de Lima son hitos reconocidos, mientras la mayoría oscila entre lugar simbólico y lugar anónimo por la falta de señalización y de alianzas municipales. Segundo, la polémica de 2006 por el proyecto del Museo de Arte Contemporáneo (MAC) del IAC, detonada por el intento de nombrarlo 'Fernando de Szyszlo': reconstruye siete momentos del debate mediático (comunicados de artistas, la columna 'Escaramuzas en Liliput' de Vargas Llosa), la falta de plan museológico y de diálogo con artistas donantes y con Barranco, y destaca la contrapropuesta crítica LiMAC de Sandra Gamarra frente al silencio del INC. Tercero, compara las puestas en escena sobre peruanidad y diversidad de cinco museos (Cultura Peruana, de la Nación, Etnográfico, Inmigración Japonesa, MNAAHP), evidenciando discursos lejanos, fragmentados y ahistóricos en los grandes museos nacionales frente a autorrepresentaciones más políticas en los pequeños. Cierra con Castrillón: Lima como escenario de emplazamiento, no de reflexión.</t>
+          <t>Artículo de Fernando Villegas (Universidad Complutense de Madrid), publicado en la Revista de Historiografía N.º 19 (2013, pp. 75-87), que rastrea la evolución de los enfoques ideológicos sobre el arte popular peruano vinculando arte y política en dos momentos clave. El primero es el proyecto mestizo de José Sabogal en los años veinte: tras su viaje a México (1923) y en sintonía con la búsqueda de peruanidad de Mariátegui y la revista Amauta, Sabogal revaloriza mates burilados, queros y retablos como productos mestizos, fusión de lo indígena precolombino y lo virreinal hispano. Desde el Instituto de Arte Peruano (1931) su grupo estudia la cerámica precolombina, el color y las artes populares, legitimando estos objetos por su origen indígena pero desplazando al artista popular como creador (los pintores urbanos se autoproclaman sus 'descubridores'). El segundo momento es la polémica de 1975-1976, cuando el gobierno militar de Velasco otorgó el Premio Nacional de Cultura al retablista ayacuchano Joaquín López Antay; la ASPAP y artistas académicos lo descalificaron como 'artesano', reproduciendo la jerarquía social y racial limeña. Villegas argumenta que ambos episodios responden a gobiernos autoritarios que legitimaron el arte popular para oponerse a la oligarquía limeña, y que el criterio de validación siempre fue estético-cronológico, ignorando el proceso histórico. El marco conceptual moviliza a Mariátegui, a Clifford (apropiación de objetos de otras culturas) y a García Canclini (descontextualización). Su aporte es evidenciar la ausencia del artista popular como sujeto de su propia obra y la carga étnica y de clase que desnaturaliza el proceso creativo andino en el circuito artístico peruano.</t>
         </is>
       </c>
     </row>
@@ -2366,27 +2366,27 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>mac-proyecto-2008.md</t>
+          <t>canepa_kg_2006_p132-167.pdf</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>2008 (exposición feb.–mar. 2008; con historia del sitio desde 1944)</t>
+          <t>1970-2006 (con referencias históricas desde el siglo XIX)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de exposición, mayo 2008 (Instituto de Arte Contemporáneo — MAC-Lima; OCR)</t>
+          <t>Capítulo de libro, 2006</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Miguel Zegarra (curadores); Instituto de Arte Contemporáneo (IAC); MAC-Lima; Giuliana Borea; George Gruenberg; Ricardo Ramón Jarne; José Carlos Martinat; Ishmael Randall Weeks; Elena Damiani; Sergio Abugattás; Raura Oblitas</t>
+          <t>Giuliana Borea Labarthe; Gisela Cánepa Koch (ed.); Sandra Gamarra (LiMAC); Instituto de Arte Contemporáneo (IAC); Fernando de Szyszlo; Gerardo Chávez; Mario Vargas Llosa; Ramiro Llona; Instituto Nacional de Cultura; ICOM; Museo de la Nación; Museo Nacional de la Cultura Peruana; Alfonso Castrillón</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Catálogo de la exposición «La Construcción del Lugar Común» (MAC-Lima, 5 de febrero–30 de marzo de 2008), editado por el Instituto de Arte Contemporáneo (IAC) y curado por Jorge Villacorta y Miguel Zegarra. Documenta una intervención colectiva de quince artistas peruanos emergentes —Sergio Abugattás, Miguel Andrade, Víctor Castro, Elena Damiani, Giuseppe De Bernardi, Nicole Franchy, Alejandro Jaime, Manuel Larrea, Martín Jiménez Paz, Christians Luna, José Carlos Martinat, José Miyashiro, Raura Oblitas, Ishmael Randall Weeks e Iliana Scheggia— que ocuparon el edificio del Museo de Arte Contemporáneo de Lima cuando aún estaba a medio construir. La muestra convirtió la arquitectura inconclusa y su entorno (el parque de la antigua «laguna» de Barranco) en soporte y tema: las obras tematizan la construcción/destrucción, el paisaje, la memoria del sitio y la disputa pública por el museo, cuyo proceso estuvo marcado por conflictos municipales y un intento de clausura respondido con el gesto «CLAUSURADO = INAUGURADO». El catálogo reúne textos institucionales (George Gruenberg, presidente del IAC), una pieza literaria de Ricardo Ramón Jarne («La maldición de la laguna»), un ensayo antropológico de Giuliana Borea sobre la construcción del lugar y el «lugar común» en la esfera pública (apoyado en Augé, Appadurai, Certeau y Casey), el texto curatorial de Villacorta y Zegarra, y los statements de cada artista. Como fuente histórica documenta un episodio clave de institucionalización del arte contemporáneo en Lima —la génesis del MAC— y las prácticas site-specific, de crítica institucional y de intervención en el espacio público de una generación emergente peruana de fines de la década de 2000.</t>
+          <t>Capítulo de Giuliana Borea Labarthe ('Museos y esfera pública: espacio, discursos y prácticas. Reflexiones en torno a la ciudad de Lima') incluido en el volumen editado por Gisela Cánepa Koch, 'Mirando la esfera pública desde la cultura en el Perú' (2006). Partiendo de las nociones de esfera pública (Habermas), cultura pública (Appadurai) y de la nueva museología surgida de las crisis de los años 70-80 (Mesa de Santiago 1972, redefinición del ICOM 1974, ecomuseos), Borea concibe el museo como contenedor y contenido, plataforma y discurso, esfera de poder y arena de disputa por la representación. Analiza tres casos limeños. Primero, el posicionamiento urbano de los museos: mediante una encuesta a transeúntes y taxistas muestra que solo el Museo de la Nación y el Museo de Arte de Lima son hitos reconocidos, mientras la mayoría oscila entre lugar simbólico y lugar anónimo por la falta de señalización y de alianzas municipales. Segundo, la polémica de 2006 por el proyecto del Museo de Arte Contemporáneo (MAC) del IAC, detonada por el intento de nombrarlo 'Fernando de Szyszlo': reconstruye siete momentos del debate mediático (comunicados de artistas, la columna 'Escaramuzas en Liliput' de Vargas Llosa), la falta de plan museológico y de diálogo con artistas donantes y con Barranco, y destaca la contrapropuesta crítica LiMAC de Sandra Gamarra frente al silencio del INC. Tercero, compara las puestas en escena sobre peruanidad y diversidad de cinco museos (Cultura Peruana, de la Nación, Etnográfico, Inmigración Japonesa, MNAAHP), evidenciando discursos lejanos, fragmentados y ahistóricos en los grandes museos nacionales frente a autorrepresentaciones más políticas en los pequeños. Cierra con Castrillón: Lima como escenario de emplazamiento, no de reflexión.</t>
         </is>
       </c>
     </row>
@@ -2398,59 +2398,59 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>sura.md</t>
+          <t>mac-proyecto-2008.md</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>mediados de la década de 1960 a 2013 (arte contemporáneo peruano)</t>
+          <t>2008 (exposición feb.–mar. 2008; con historia del sitio desde 1944)</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de colección museística, 2013</t>
+          <t>Catálogo de exposición, mayo 2008 (Instituto de Arte Contemporáneo — MAC-Lima; OCR)</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner (ed.); Museo de Arte de Lima (MALI); Grupo SURA; Mirko Lauer; E.P.S. Huayco; Charo Noriega; Ramiro Llona; Flavia Gandolfo; Armando Andrade Tudela; Ricardo Wiesse; Eduardo Villanes; Miguel A. López; Rodrigo Quijano</t>
+          <t>Jorge Villacorta; Miguel Zegarra (curadores); Instituto de Arte Contemporáneo (IAC); MAC-Lima; Giuliana Borea; George Gruenberg; Ricardo Ramón Jarne; José Carlos Martinat; Ishmael Randall Weeks; Elena Damiani; Sergio Abugattás; Raura Oblitas</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Catálogo de la colección de arte contemporáneo del Museo de Arte de Lima (MALI), editado por la curadora Sharon Lerner y publicado con el patrocinio del grupo SURA. El volumen traza los derroteros del arte peruano reciente a partir del acervo del museo, sin pretender definir un 'arte peruano' esencial. La colección se articula bajo dos principios: identificar momentos de ruptura en la producción artística de fines del siglo XX y perfilar la producción reciente mediante ejes temáticos comunes. El ensayo central de Lerner establece como punto de partida mediados de la década de 1960 (grupos de vanguardia ligados al Pop y al no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, tras las reformas del Gobierno Militar, cuando —según la célebre frase de Mirko Lauer para la muestra Arte al paso del colectivo E.P.S. Huayco (1980)— 'en el Perú hoy solo lo popular es moderno'. Analiza la irrupción de la migración interna, el conflicto armado interno, el autogolpe de Fujimori (1992) y la virtual desaparición de la esfera pública, así como la Bienal Iberoamericana de Lima (1997) como puesta al día forzada y descontextualizada. El catálogo se organiza en núcleos temáticos: modernidad popular y transformación de Lima, f(r)icciones cosmopolitas, reconsideración del pasado y configuración del Perú, sistema artístico y utopías museales, desplazamientos, y signos de violencia, resistencia y memoria. Incluye obras de Charo Noriega, Ramiro Llona, Flavia Gandolfo, Armando Andrade Tudela, Herman Schwarz, Ricardo Wiesse y Eduardo Villanes, entre otros, y textos críticos complementarios. Su aporte es consolidar un relato historiográfico y crítico del arte contemporáneo peruano desde una institución museal.</t>
+          <t>Catálogo de la exposición «La Construcción del Lugar Común» (MAC-Lima, 5 de febrero–30 de marzo de 2008), editado por el Instituto de Arte Contemporáneo (IAC) y curado por Jorge Villacorta y Miguel Zegarra. Documenta una intervención colectiva de quince artistas peruanos emergentes —Sergio Abugattás, Miguel Andrade, Víctor Castro, Elena Damiani, Giuseppe De Bernardi, Nicole Franchy, Alejandro Jaime, Manuel Larrea, Martín Jiménez Paz, Christians Luna, José Carlos Martinat, José Miyashiro, Raura Oblitas, Ishmael Randall Weeks e Iliana Scheggia— que ocuparon el edificio del Museo de Arte Contemporáneo de Lima cuando aún estaba a medio construir. La muestra convirtió la arquitectura inconclusa y su entorno (el parque de la antigua «laguna» de Barranco) en soporte y tema: las obras tematizan la construcción/destrucción, el paisaje, la memoria del sitio y la disputa pública por el museo, cuyo proceso estuvo marcado por conflictos municipales y un intento de clausura respondido con el gesto «CLAUSURADO = INAUGURADO». El catálogo reúne textos institucionales (George Gruenberg, presidente del IAC), una pieza literaria de Ricardo Ramón Jarne («La maldición de la laguna»), un ensayo antropológico de Giuliana Borea sobre la construcción del lugar y el «lugar común» en la esfera pública (apoyado en Augé, Appadurai, Certeau y Casey), el texto curatorial de Villacorta y Zegarra, y los statements de cada artista. Como fuente histórica documenta un episodio clave de institucionalización del arte contemporáneo en Lima —la génesis del MAC— y las prácticas site-specific, de crítica institucional y de intervención en el espacio público de una generación emergente peruana de fines de la década de 2000.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Arte al Paso 2011</t>
+          <t>Cap 2 - Historia</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Arte al Paso - Texto Investigación.md</t>
+          <t>sura.md</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 1960 – 2010 (con foco en las décadas de 1970-2000 y el conflicto armado interno 1980-2000)</t>
+          <t>mediados de la década de 1960 a 2013 (arte contemporáneo peruano)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Ensayo curatorial de catálogo (exposición Arte al paso, Pinacoteca do Estado de São Paulo, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Catálogo de colección museística, 2013</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Pinacoteca de São Paulo; Emilio Hernández Saavedra; E.P.S. Huayco; Jesús Ruiz Durand; Sandra Gamarra; Alfredo Márquez / Taller NN; Fernando Bryce; José Carlos Martinat; Susana Torres</t>
+          <t>Sharon Lerner (ed.); Museo de Arte de Lima (MALI); Grupo SURA; Mirko Lauer; E.P.S. Huayco; Charo Noriega; Ramiro Llona; Flavia Gandolfo; Armando Andrade Tudela; Ricardo Wiesse; Eduardo Villanes; Miguel A. López; Rodrigo Quijano</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Ensayo curatorial extenso y bilingüe (castellano/portugués) de Tatiana Cuevas y Rodrigo Quijano para la muestra Arte al paso, que exhibió la coleccion contemporanea del MALI en la Estacion Pinacoteca de Sao Paulo. El texto toma como punto de partida la imagen El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra para diagnosticar los vacios institucionales y la distancia entre el discurso cultural cosmopolita y la practica real en el Peru de la segunda mitad del siglo XX. Su argumento articula el arte contemporaneo peruano con las transformaciones sociales derivadas de la masiva migracion rural a Lima, la explosion de la economia informal y la emergencia de una nueva cultura popular urbana. Rastrea las primeras vinculaciones locales con vanguardias internacionales (op, pop, conceptualismo, no-objetualismo), el pop achorado de Jesus Ruiz Durand y sus afiches de la Reforma Agraria velasquista, y las experiencias colectivas Contacta 79 y Arte al paso de E.P.S. Huayco (1980), que propusieron un arte callejero y antiinstitucional. Analiza la critica a la institucionalidad faltante (el museo ficticio LiMAC de Sandra Gamarra), el uso ironico del pasado prehispanico (Susana Torres, Rodriguez Larrain, Bryce, Cordova, Martinat), el tema del paisaje y el territorio, y la irrupcion tardia de la fotografia y la serigrafia como medios. Dedica una seccion central a la memoria de la violencia del conflicto armado interno (1980-2000) —Sendero Luminoso, MRTA, la Comision de la Verdad, 69.280 muertos— y su tratamiento por el Taller NN, Alfredo Marquez (Katatay), Carlos Dominguez, Ricardo Wiesse, Eduardo Villanes, Fernando Bryce y Milagros de la Torre.</t>
+          <t>Catálogo de la colección de arte contemporáneo del Museo de Arte de Lima (MALI), editado por la curadora Sharon Lerner y publicado con el patrocinio del grupo SURA. El volumen traza los derroteros del arte peruano reciente a partir del acervo del museo, sin pretender definir un 'arte peruano' esencial. La colección se articula bajo dos principios: identificar momentos de ruptura en la producción artística de fines del siglo XX y perfilar la producción reciente mediante ejes temáticos comunes. El ensayo central de Lerner establece como punto de partida mediados de la década de 1960 (grupos de vanguardia ligados al Pop y al no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, tras las reformas del Gobierno Militar, cuando —según la célebre frase de Mirko Lauer para la muestra Arte al paso del colectivo E.P.S. Huayco (1980)— 'en el Perú hoy solo lo popular es moderno'. Analiza la irrupción de la migración interna, el conflicto armado interno, el autogolpe de Fujimori (1992) y la virtual desaparición de la esfera pública, así como la Bienal Iberoamericana de Lima (1997) como puesta al día forzada y descontextualizada. El catálogo se organiza en núcleos temáticos: modernidad popular y transformación de Lima, f(r)icciones cosmopolitas, reconsideración del pasado y configuración del Perú, sistema artístico y utopías museales, desplazamientos, y signos de violencia, resistencia y memoria. Incluye obras de Charo Noriega, Ramiro Llona, Flavia Gandolfo, Armando Andrade Tudela, Herman Schwarz, Ricardo Wiesse y Eduardo Villanes, entre otros, y textos críticos complementarios. Su aporte es consolidar un relato historiográfico y crítico del arte contemporáneo peruano desde una institución museal.</t>
         </is>
       </c>
     </row>
@@ -2462,27 +2462,27 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Cronología Político Artistica - Arte al Paso 2011.md</t>
+          <t>Arte al Paso - Texto Investigación.md</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>1962 – 2010</t>
+          <t>Fines de los años 1960 – 2010 (con foco en las décadas de 1970-2000 y el conflicto armado interno 1980-2000)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Cronología y bibliografía de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Ensayo curatorial de catálogo (exposición Arte al paso, Pinacoteca do Estado de São Paulo, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Museo de Arte de Lima (MALI); Grupo Arte Nuevo; Grupo Señal; E.P.S. Huayco; Taller NN; Colectivo Sociedad Civil; Gustavo Buntinx; Joaquín López Antay; Comisión de la Verdad y Reconciliación; Sendero Luminoso; Alberto Fujimori; Juan Velasco Alvarado</t>
+          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Pinacoteca de São Paulo; Emilio Hernández Saavedra; E.P.S. Huayco; Jesús Ruiz Durand; Sandra Gamarra; Alfredo Márquez / Taller NN; Fernando Bryce; José Carlos Martinat; Susana Torres</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Cronologia politico-artistica bilingue (castellano/portugues) incluida en el catalogo Arte al paso, que entrelaza en paralelo tres series de acontecimientos —eventos politicos, eventos artisticos y adquisiciones de la coleccion de arte contemporaneo del MALI— entre 1962 y 2010. El documento funciona como aparato historiografico que contextualiza la escena artistica peruana dentro de sus convulsiones politicas: rebeliones campesinas y golpes militares de los anos sesenta, el Gobierno Revolucionario de las Fuerzas Armadas de Velasco Alvarado (1968) y la Reforma Agraria, el estallido del conflicto armado interno con Sendero Luminoso y el MRTA (1980), las masacres de Barrios Altos y La Cantuta, el autogolpe y la dictadura de Alberto Fujimori (1990-2000), la Marcha de los Cuatro Suyos y el Informe de la Comision de la Verdad y Reconciliacion (2003). En el plano artistico registra la formacion de los grupos Senal y Arte Nuevo, las Bienales de Lima e Iberoamericanas, los festivales Contacta e Inkarri, el Taller E.P.S. Huayco y el Taller NN, la premiacion de Joaquin Lopez Antay, y acciones de arte critico como Cantuta de Ricardo Wiesse, Gloria evaporada de Eduardo Villanes y Lava la bandera del Colectivo Sociedad Civil. Una tercera linea traza la institucionalizacion del MALI: el ciclo curatorial Miradas de fin de siglo, la creacion del Comite de Adquisiciones (2007) y la reapertura del museo (2010). Se acompana de una extensa bibliografia especializada (Buntinx, Castrillon, Lauer, Majluf, Lopez, Tarazona, Quijano, Villacorta), fuente clave para la historiografia del arte peruano contemporaneo.</t>
+          <t>Ensayo curatorial extenso y bilingüe (castellano/portugués) de Tatiana Cuevas y Rodrigo Quijano para la muestra Arte al paso, que exhibió la coleccion contemporanea del MALI en la Estacion Pinacoteca de Sao Paulo. El texto toma como punto de partida la imagen El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra para diagnosticar los vacios institucionales y la distancia entre el discurso cultural cosmopolita y la practica real en el Peru de la segunda mitad del siglo XX. Su argumento articula el arte contemporaneo peruano con las transformaciones sociales derivadas de la masiva migracion rural a Lima, la explosion de la economia informal y la emergencia de una nueva cultura popular urbana. Rastrea las primeras vinculaciones locales con vanguardias internacionales (op, pop, conceptualismo, no-objetualismo), el pop achorado de Jesus Ruiz Durand y sus afiches de la Reforma Agraria velasquista, y las experiencias colectivas Contacta 79 y Arte al paso de E.P.S. Huayco (1980), que propusieron un arte callejero y antiinstitucional. Analiza la critica a la institucionalidad faltante (el museo ficticio LiMAC de Sandra Gamarra), el uso ironico del pasado prehispanico (Susana Torres, Rodriguez Larrain, Bryce, Cordova, Martinat), el tema del paisaje y el territorio, y la irrupcion tardia de la fotografia y la serigrafia como medios. Dedica una seccion central a la memoria de la violencia del conflicto armado interno (1980-2000) —Sendero Luminoso, MRTA, la Comision de la Verdad, 69.280 muertos— y su tratamiento por el Taller NN, Alfredo Marquez (Katatay), Carlos Dominguez, Ricardo Wiesse, Eduardo Villanes, Fernando Bryce y Milagros de la Torre.</t>
         </is>
       </c>
     </row>
@@ -2494,59 +2494,59 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Texto de la exposición Arte al Paso 2011.md</t>
+          <t>Cronología Político Artistica - Arte al Paso 2011.md</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 1960 – 2010 (unos 40 años; foco en las décadas de 1970-1980)</t>
+          <t>1962 – 2010</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Texto de sala / presentación de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Cronología y bibliografía de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Emilio Hernández Saavedra; E.P.S. Huayco; Grupo Paréntesis; Sandra Gamarra; Susana Torres; Emilio Rodríguez Larraín; Juan Javier Salazar; William Cordova; José Carlos Martinat</t>
+          <t>Museo de Arte de Lima (MALI); Grupo Arte Nuevo; Grupo Señal; E.P.S. Huayco; Taller NN; Colectivo Sociedad Civil; Gustavo Buntinx; Joaquín López Antay; Comisión de la Verdad y Reconciliación; Sendero Luminoso; Alberto Fujimori; Juan Velasco Alvarado</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Texto de sala o presentacion general de la exposicion Arte al paso (coleccion contemporanea del MALI en la Pinacoteca de Sao Paulo), firmado por los curadores Tatiana Cuevas y Rodrigo Quijano, en edicion bilingue castellano/portugues. Es una version sintetica del argumento curatorial: parte nuevamente de El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra como metafora de la ausencia institucional y punto de arranque para examinar la escena artistica peruana desde fines de los anos sesenta. Explica el titulo de la muestra a partir de la accion Arte al paso de E.P.S. Huayco (1980) —que, aludiendo a los puestos informales de comida al paso surgidos con la migracion y la economia informal, propuso un arte para consumirse en la calle, opuesto al museo y la galeria ausentes, un arte para pensar y no para sentir que dejaba atras el modernismo conservador de mediados de siglo. Sintetiza cuarenta anos de produccion cultural marcados por oposiciones ocultas y explicitas, los primeros acercamientos al conceptualismo y a las vanguardias internacionales, y la creciente proyeccion internacional de artistas peruanos. Una segunda seccion, Critica ante una institucionalidad faltante y al poder redentor del pasado, reune a Hernandez Saavedra, los grupos Parentesis y E.P.S. Huayco y el museo ficticio de Sandra Gamarra como estrategias de critica institucional apropiadas del conceptualismo y del imaginario popular urbano, con recurrente uso del humor. Aborda ademas la critica a la explotacion comercial y politica de lo prehispanico (Museo Neo-Inka de Susana Torres) y el vinculo entre la retorica del glorioso pasado incaico y los fracasos politicos y economicos del presente en obras de Rodriguez Larrain, Salazar, Cordova y Martinat.</t>
+          <t>Cronologia politico-artistica bilingue (castellano/portugues) incluida en el catalogo Arte al paso, que entrelaza en paralelo tres series de acontecimientos —eventos politicos, eventos artisticos y adquisiciones de la coleccion de arte contemporaneo del MALI— entre 1962 y 2010. El documento funciona como aparato historiografico que contextualiza la escena artistica peruana dentro de sus convulsiones politicas: rebeliones campesinas y golpes militares de los anos sesenta, el Gobierno Revolucionario de las Fuerzas Armadas de Velasco Alvarado (1968) y la Reforma Agraria, el estallido del conflicto armado interno con Sendero Luminoso y el MRTA (1980), las masacres de Barrios Altos y La Cantuta, el autogolpe y la dictadura de Alberto Fujimori (1990-2000), la Marcha de los Cuatro Suyos y el Informe de la Comision de la Verdad y Reconciliacion (2003). En el plano artistico registra la formacion de los grupos Senal y Arte Nuevo, las Bienales de Lima e Iberoamericanas, los festivales Contacta e Inkarri, el Taller E.P.S. Huayco y el Taller NN, la premiacion de Joaquin Lopez Antay, y acciones de arte critico como Cantuta de Ricardo Wiesse, Gloria evaporada de Eduardo Villanes y Lava la bandera del Colectivo Sociedad Civil. Una tercera linea traza la institucionalizacion del MALI: el ciclo curatorial Miradas de fin de siglo, la creacion del Comite de Adquisiciones (2007) y la reapertura del museo (2010). Se acompana de una extensa bibliografia especializada (Buntinx, Castrillon, Lauer, Majluf, Lopez, Tarazona, Quijano, Villacorta), fuente clave para la historiografia del arte peruano contemporaneo.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Hueso Húmero 18</t>
+          <t>Cap 2 - Historia/Arte al Paso 2011</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - Arte joven peruano, ¿el sueño del mercado propio? Una conversación con Claudia Polar (1983) [Hueso Húmero 18, pp. 94-107].md</t>
+          <t>Texto de la exposición Arte al Paso 2011.md</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>1974-1983</t>
+          <t>Fines de los años 1960 – 2010 (unos 40 años; foco en las décadas de 1970-1980)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Entrevista en revista (Hueso Húmero 18), 1983</t>
+          <t>Texto de sala / presentación de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Claudia Polar; Galería Forum; Elida Román; Hernán Pazos; Esther Vainstein; Ramiro Llona; Bill Caro; Herbert Rodríguez; EAPUC; ENBA; Hueso Húmero</t>
+          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Emilio Hernández Saavedra; E.P.S. Huayco; Grupo Paréntesis; Sandra Gamarra; Susana Torres; Emilio Rodríguez Larraín; Juan Javier Salazar; William Cordova; José Carlos Martinat</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Entrevista conducida por Gustavo Buntinx a Claudia Polar, directora de la Galería Forum, concebida como contraparte de un reportaje previo a Elida Román para perfilar el mercado del arte joven peruano. Polar reconstruye la fundación de Forum en diciembre de 1974 como un espacio destinado a priorizar a los artistas jóvenes y a gestar deliberadamente un mercado y coleccionistas nuevos, mediante becas, premios, subvenciones informales (incluso marcos y pasajes) y una política de "riesgo total" sostenida por la venta de stock. El diálogo traza una periodización económica de la plástica: expansión del mercado hacia 1974-1976, auge en 1978 atribuido a la restricción de importaciones bajo Morales Bermúdez, y recesión desde 1980 con la apertura de Belaúnde, siendo 1983 el año más difícil. Se discute la naturaleza del público comprador (gente joven, profesionales, empresarios, bancos como el de Crédito y el Continental) y la débil proporción de compradores habituales, apenas un 5% con relación económica. Buntinx presiona sobre las mediaciones de clase: el vínculo de Forum con la Universidad Católica frente a la ENBA, la identidad ideológica compartida, y el papel de las relaciones públicas como "gatillo" de casi toda venta en un mercado de "sala de estar". Polar aborda la diferencia entre lo culto y lo popular, el fracaso de asociar galerías, las cotizaciones (Llona, Caro, Pazos, Vainstein) y la explotación del artista acostumbrado a vender barato. El aporte documental es excepcional: registra desde dentro la lógica comercial, simbólica y provinciana del circuito limeño de principios de los ochenta.</t>
+          <t>Texto de sala o presentacion general de la exposicion Arte al paso (coleccion contemporanea del MALI en la Pinacoteca de Sao Paulo), firmado por los curadores Tatiana Cuevas y Rodrigo Quijano, en edicion bilingue castellano/portugues. Es una version sintetica del argumento curatorial: parte nuevamente de El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra como metafora de la ausencia institucional y punto de arranque para examinar la escena artistica peruana desde fines de los anos sesenta. Explica el titulo de la muestra a partir de la accion Arte al paso de E.P.S. Huayco (1980) —que, aludiendo a los puestos informales de comida al paso surgidos con la migracion y la economia informal, propuso un arte para consumirse en la calle, opuesto al museo y la galeria ausentes, un arte para pensar y no para sentir que dejaba atras el modernismo conservador de mediados de siglo. Sintetiza cuarenta anos de produccion cultural marcados por oposiciones ocultas y explicitas, los primeros acercamientos al conceptualismo y a las vanguardias internacionales, y la creciente proyeccion internacional de artistas peruanos. Una segunda seccion, Critica ante una institucionalidad faltante y al poder redentor del pasado, reune a Hernandez Saavedra, los grupos Parentesis y E.P.S. Huayco y el museo ficticio de Sandra Gamarra como estrategias de critica institucional apropiadas del conceptualismo y del imaginario popular urbano, con recurrente uso del humor. Aborda ademas la critica a la explotacion comercial y politica de lo prehispanico (Museo Neo-Inka de Susana Torres) y el vinculo entre la retorica del glorioso pasado incaico y los fracasos politicos y economicos del presente en obras de Rodriguez Larrain, Salazar, Cordova y Martinat.</t>
         </is>
       </c>
     </row>
@@ -2558,27 +2558,27 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - ¿Entre lo popular y lo moderno? Alternativas pretendidas o reales en la joven plástica peruana (1983) [Hueso Húmero 18, pp. 61-85].md</t>
+          <t>Buntinx - Arte joven peruano, ¿el sueño del mercado propio? Una conversación con Claudia Polar (1983) [Hueso Húmero 18, pp. 94-107].md</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>1960-1984 (con énfasis en los años 70)</t>
+          <t>1974-1983</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
+          <t>Entrevista en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Mirko Lauer; Juan Acha; Francisco Mariotti; Huayco E.P.S.; Herbert Rodríguez; Juan Javier Salazar; Jesús Ruiz Durand; Fernando de Szyszlo; IAC; Galería Forum; SINAMOS; Néstor García Canclini</t>
+          <t>Gustavo Buntinx; Claudia Polar; Galería Forum; Elida Román; Hernán Pazos; Esther Vainstein; Ramiro Llona; Bill Caro; Herbert Rodríguez; EAPUC; ENBA; Hueso Húmero</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Ensayo teórico-histórico que propone hipótesis de trabajo sobre lo que fue o pretendió ser alternativo en el arte erudito peruano desde la transición al primer belaundismo hasta los años ochenta, articulando dos tópicos móviles: lo popular y lo moderno. Retomando y ampliando a Mirko Lauer, Buntinx sostiene que las opciones estéticas no reflejan mecánicamente la época sino que reproducen una inserción particular en el mercado, entendido como trama compleja de producción, intermediación y consumo (soporte social). Recorre así una secuencia de "soportes": el corporativo (IAC financiado por IPC, IBM, Tecnoquímica) que sostuvo la Teoría de las Raíces Nacionales de Szyszlo; el soporte "de punta" del frenesí pop cosmopolita (Acha, Arte Nuevo, Fundación para las Artes, 1966-1969); el soporte estatal velasquista con sus cuatro alternativas (comunicación masiva de Ruiz Durand con su "pop achorado", festivales de arte-total como Contacta e Inkarri, revaloración de lo artesanal, López Antay); y la frustrada búsqueda de un soporte alternativo hacia 1977-1980. El caso central es Huayco E.P.S., cuyo proyecto Sarita Colonia codifica una modernidad sincrética limeña sostenida por una pequeña burguesía ilustrada radicalizada, y cuya dispersión coincide con el agotamiento de la izquierda y el repliegue hacia el mercado galerístico (Forum). El marco conceptual bebe de García Canclini. La tesis es incisiva: el tránsito de la imagen telúrica a la industrial, agraria y migrante revela apropiaciones sucesivas de una idea variable de lo popular, siempre con una radicalidad deficiente y una relación desigual con la cultura interpretada.</t>
+          <t>Entrevista conducida por Gustavo Buntinx a Claudia Polar, directora de la Galería Forum, concebida como contraparte de un reportaje previo a Elida Román para perfilar el mercado del arte joven peruano. Polar reconstruye la fundación de Forum en diciembre de 1974 como un espacio destinado a priorizar a los artistas jóvenes y a gestar deliberadamente un mercado y coleccionistas nuevos, mediante becas, premios, subvenciones informales (incluso marcos y pasajes) y una política de "riesgo total" sostenida por la venta de stock. El diálogo traza una periodización económica de la plástica: expansión del mercado hacia 1974-1976, auge en 1978 atribuido a la restricción de importaciones bajo Morales Bermúdez, y recesión desde 1980 con la apertura de Belaúnde, siendo 1983 el año más difícil. Se discute la naturaleza del público comprador (gente joven, profesionales, empresarios, bancos como el de Crédito y el Continental) y la débil proporción de compradores habituales, apenas un 5% con relación económica. Buntinx presiona sobre las mediaciones de clase: el vínculo de Forum con la Universidad Católica frente a la ENBA, la identidad ideológica compartida, y el papel de las relaciones públicas como "gatillo" de casi toda venta en un mercado de "sala de estar". Polar aborda la diferencia entre lo culto y lo popular, el fracaso de asociar galerías, las cotizaciones (Llona, Caro, Pazos, Vainstein) y la explotación del artista acostumbrado a vender barato. El aporte documental es excepcional: registra desde dentro la lógica comercial, simbólica y provinciana del circuito limeño de principios de los ochenta.</t>
         </is>
       </c>
     </row>
@@ -2590,27 +2590,27 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Freire - Herbert Rodríguez, azote y azúcar con el sistema (1983) [Hueso Húmero 18, pdf pp. 178-185].md</t>
+          <t>Buntinx - ¿Entre lo popular y lo moderno? Alternativas pretendidas o reales en la joven plástica peruana (1983) [Hueso Húmero 18, pp. 61-85].md</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>1979-1983 (con antecedentes desde 1968)</t>
+          <t>1960-1984 (con énfasis en los años 70)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Reseña crítica en revista (Hueso Húmero 18), 1983</t>
+          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Luis Freire S.; Herbert Rodríguez; Francisco Mariotti; Huayco E.P.S.; Juan Acha; Fernando Bedoya; Juan Javier Salazar; Bienal de Sao Paulo; Galería La Rama Dorada; Galería Forum; EAPUC; ENBAP</t>
+          <t>Gustavo Buntinx; Mirko Lauer; Juan Acha; Francisco Mariotti; Huayco E.P.S.; Herbert Rodríguez; Juan Javier Salazar; Jesús Ruiz Durand; Fernando de Szyszlo; IAC; Galería Forum; SINAMOS; Néstor García Canclini</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Perfil crítico dedicado a Herbert Rodríguez Huachín en la sección "Individuales" de Hueso Húmero, escrito por Luis Freire, que examina el salto vertiginoso del artista desde la suspensión disciplinaria en la Escuela de Artes Plásticas de la Católica (1981) hasta su presencia en la XVII Bienal de Sao Paulo (1983). Freire sitúa a Rodríguez como imposible de explicar sin el proceso ideológico del populismo velasquista y sin la figura mediadora de Francisco Mariotti, artista suizo-peruano formado en la Documenta de Kassel y la vanguardia europea, catalizador de Contacta y de la EPS Huayco. El texto reconstruye la genealogía Mariotti-Huayco-Rodríguez: los ensamblajes y "reciclajes" del suizo-peruano derivan en los "altares" de Rodríguez, hibridación entre constructivismo geométrico, expresionismo "pobre" y antiestético, y estructuras rituales de la religiosidad popular andina. Argumenta que Rodríguez encarna las contradicciones de una pequeña burguesía radical: dinamita el circuito con una mano y lo enluce con la otra, camuflando "bellamente" materiales pobres y reciclados en obras a la vez contestatarias y comerciables, con lo que ironiza sobre el culto al oficio del arte establecido. Analiza su heterogeneidad de lenguajes (expresionismo abstracto, figuración dura, conceptualismo informal, collage, fotocopia, ensamblaje) como búsqueda pero también como crisis, y sus "altares al Yo" exhibidos en Forum (1983) y la Bienal. Freire lo define como un artista religioso-existencial populista sin referentes sólidos, en formación, tensionado entre enriquecer el jardín burgués que quiere pisotear o saltar a opciones más radicales de ruptura.</t>
+          <t>Ensayo teórico-histórico que propone hipótesis de trabajo sobre lo que fue o pretendió ser alternativo en el arte erudito peruano desde la transición al primer belaundismo hasta los años ochenta, articulando dos tópicos móviles: lo popular y lo moderno. Retomando y ampliando a Mirko Lauer, Buntinx sostiene que las opciones estéticas no reflejan mecánicamente la época sino que reproducen una inserción particular en el mercado, entendido como trama compleja de producción, intermediación y consumo (soporte social). Recorre así una secuencia de "soportes": el corporativo (IAC financiado por IPC, IBM, Tecnoquímica) que sostuvo la Teoría de las Raíces Nacionales de Szyszlo; el soporte "de punta" del frenesí pop cosmopolita (Acha, Arte Nuevo, Fundación para las Artes, 1966-1969); el soporte estatal velasquista con sus cuatro alternativas (comunicación masiva de Ruiz Durand con su "pop achorado", festivales de arte-total como Contacta e Inkarri, revaloración de lo artesanal, López Antay); y la frustrada búsqueda de un soporte alternativo hacia 1977-1980. El caso central es Huayco E.P.S., cuyo proyecto Sarita Colonia codifica una modernidad sincrética limeña sostenida por una pequeña burguesía ilustrada radicalizada, y cuya dispersión coincide con el agotamiento de la izquierda y el repliegue hacia el mercado galerístico (Forum). El marco conceptual bebe de García Canclini. La tesis es incisiva: el tránsito de la imagen telúrica a la industrial, agraria y migrante revela apropiaciones sucesivas de una idea variable de lo popular, siempre con una radicalidad deficiente y una relación desigual con la cultura interpretada.</t>
         </is>
       </c>
     </row>
@@ -2622,59 +2622,59 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Lama - Los años de la resaca (1983) [Hueso Húmero 18, pdf pp. 136-156].md</t>
+          <t>Freire - Herbert Rodríguez, azote y azúcar con el sistema (1983) [Hueso Húmero 18, pdf pp. 178-185].md</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>1974-1983 (con antecedentes en los años 60-70)</t>
+          <t>1979-1983 (con antecedentes desde 1968)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
+          <t>Reseña crítica en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Luis Lama; Hernán Pazos; Francisco Mariotti; Contacta; grupo Huayco; Juan Javier Salazar; Herbert Rodríguez; Alfonso Castrillón; Escuela Nacional de Bellas Artes; Galería Forum; Galería 9; Ugarte Eléspuru</t>
+          <t>Luis Freire S.; Herbert Rodríguez; Francisco Mariotti; Huayco E.P.S.; Juan Acha; Fernando Bedoya; Juan Javier Salazar; Bienal de Sao Paulo; Galería La Rama Dorada; Galería Forum; EAPUC; ENBAP</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Ensayo de Luis Lama que narra el paso de la "ebullición ideológica" de los años setenta a la "resaca" del segundo belaundismo, articulando historia social del arte y crítica biográfica. La primera parte reconstruye los antecedentes: el terremoto de 1974 y el reflujo de artistas jóvenes hacia Barranco, la gravitación de Francisco Mariotti que transforma el arte de sistemas en movimiento grupal con Contacta e Inkari bajo auspicio de SINAMOS, las tomas y la crisis de la Escuela Nacional de Bellas Artes (1974-1976), y la gestación del taller de Pedro de Osma que devendría núcleo del grupo Huayco (Juan Javier Salazar, Herbert Rodríguez, Charo Noriega, Fernando Bedoya, Lucy Angulo). Lama describe la consolidación paradójica del mercado del arte al amparo de la prohibición de importaciones, con galerías que proliferan mientras la formación académica alcanza sus niveles más bajos. Diagnostica el fin de los happenings sesenteros y el retorno de un expresionismo "de crisis" impulsado desde los predios católicos (Williams, Polanco, Velarde, Hamann), junto a indagaciones matéricas de Wiesse y el conceptualismo de Vainstein. La segunda mitad es un retrato extenso de Hernán Pazos: su formación entre Derecho, la Católica y París, su tránsito del conceptualismo (los cielos y nubes de Galería 9) a la abstracción cromática, las series de los Quipus y los dibujos infantiles, su gestión en Rama Dorada y su individualismo parricida. Lama lo consagra como el artista más destacado de la década, emblema lúcido de las "amargas frustraciones" nacionales bajo el liberalismo económico belaundista.</t>
+          <t>Perfil crítico dedicado a Herbert Rodríguez Huachín en la sección "Individuales" de Hueso Húmero, escrito por Luis Freire, que examina el salto vertiginoso del artista desde la suspensión disciplinaria en la Escuela de Artes Plásticas de la Católica (1981) hasta su presencia en la XVII Bienal de Sao Paulo (1983). Freire sitúa a Rodríguez como imposible de explicar sin el proceso ideológico del populismo velasquista y sin la figura mediadora de Francisco Mariotti, artista suizo-peruano formado en la Documenta de Kassel y la vanguardia europea, catalizador de Contacta y de la EPS Huayco. El texto reconstruye la genealogía Mariotti-Huayco-Rodríguez: los ensamblajes y "reciclajes" del suizo-peruano derivan en los "altares" de Rodríguez, hibridación entre constructivismo geométrico, expresionismo "pobre" y antiestético, y estructuras rituales de la religiosidad popular andina. Argumenta que Rodríguez encarna las contradicciones de una pequeña burguesía radical: dinamita el circuito con una mano y lo enluce con la otra, camuflando "bellamente" materiales pobres y reciclados en obras a la vez contestatarias y comerciables, con lo que ironiza sobre el culto al oficio del arte establecido. Analiza su heterogeneidad de lenguajes (expresionismo abstracto, figuración dura, conceptualismo informal, collage, fotocopia, ensamblaje) como búsqueda pero también como crisis, y sus "altares al Yo" exhibidos en Forum (1983) y la Bienal. Freire lo define como un artista religioso-existencial populista sin referentes sólidos, en formación, tensionado entre enriquecer el jardín burgués que quiere pisotear o saltar a opciones más radicales de ruptura.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/MALI</t>
+          <t>Cap 2 - Historia/Hueso Húmero 18</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - El poder y la ilusión. Pérdida y restauración del aura en la «República de Weimar peruana» 1980-1992 [MALI].md</t>
+          <t>Lama - Los años de la resaca (1983) [Hueso Húmero 18, pdf pp. 136-156].md</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>1980-1992</t>
+          <t>1974-1983 (con antecedentes en los años 60-70)</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico (versión MALI), 2013 [escrito 1991-1994]</t>
+          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; E.P.S. Huayco; Taller NN; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; Walter Benjamin; Jesús Ruiz Durand; Andy Warhol; Mirko Lauer; Museo de Arte de Lima (MALI); III Bienal de La Habana</t>
+          <t>Luis Lama; Hernán Pazos; Francisco Mariotti; Contacta; grupo Huayco; Juan Javier Salazar; Herbert Rodríguez; Alfonso Castrillón; Escuela Nacional de Bellas Artes; Galería Forum; Galería 9; Ugarte Eléspuru</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Ensayo seminal de Gustavo Buntinx —redactado entre 1991 y 1994, difundido en inglés en «Beyond the Fantastic» (1995) y publicado por primera vez en Perú en esta versión del MALI (2013)— que interpreta el radical cambio de época del arte peruano entre 1980 y 1992, periodo que denomina metafóricamente «República de Weimar peruana». Su marco conceptual adapta la dialéctica benjaminiana entre proximidad y distancia (el aura, su pérdida por la reproductibilidad técnica y su posible restauración) y las categorías de alegoría, montaje y apropiación de Owens, Foster y Craig Owens a una periferia extrema. El argumento se sostiene sobre el análisis iconográfico minucioso de dos o tres obras que abren y cierran la década. La primera, «Arte al paso» y sobre todo «Sarita Colonia» (1980) del taller E.P.S. Huayco: una enorme estampa de la santa migrante pintada sobre diez mil latas de leche y emplazada en la Panamericana Sur, que Buntinx lee como huaca (post)moderna y exvoto donde lo pequeñoburgués radical se articula figuradamente a lo popular en emergencia (el «pop achorado» y «chicha»). La segunda, «Maorilyn» / «Viva el maoísmo» (1989) del Taller NN: una serigrafía que travistió el rostro de Mao con labios warholianos, alegoría ambivalente de la violencia senderista y la estetización de la política. Su tesis vincula la desintegración social —hiperinflación, guerra civil, movida subte punk— con el desarrollo de una condición alegórica y neo-aurática; su aporte es un modelo teórico para leer el colectivismo y la (post)modernidad popular peruana.</t>
+          <t>Ensayo de Luis Lama que narra el paso de la "ebullición ideológica" de los años setenta a la "resaca" del segundo belaundismo, articulando historia social del arte y crítica biográfica. La primera parte reconstruye los antecedentes: el terremoto de 1974 y el reflujo de artistas jóvenes hacia Barranco, la gravitación de Francisco Mariotti que transforma el arte de sistemas en movimiento grupal con Contacta e Inkari bajo auspicio de SINAMOS, las tomas y la crisis de la Escuela Nacional de Bellas Artes (1974-1976), y la gestación del taller de Pedro de Osma que devendría núcleo del grupo Huayco (Juan Javier Salazar, Herbert Rodríguez, Charo Noriega, Fernando Bedoya, Lucy Angulo). Lama describe la consolidación paradójica del mercado del arte al amparo de la prohibición de importaciones, con galerías que proliferan mientras la formación académica alcanza sus niveles más bajos. Diagnostica el fin de los happenings sesenteros y el retorno de un expresionismo "de crisis" impulsado desde los predios católicos (Williams, Polanco, Velarde, Hamann), junto a indagaciones matéricas de Wiesse y el conceptualismo de Vainstein. La segunda mitad es un retrato extenso de Hernán Pazos: su formación entre Derecho, la Católica y París, su tránsito del conceptualismo (los cielos y nubes de Galería 9) a la abstracción cromática, las series de los Quipus y los dibujos infantiles, su gestión en Rama Dorada y su individualismo parricida. Lama lo consagra como el artista más destacado de la década, emblema lúcido de las "amargas frustraciones" nacionales bajo el liberalismo económico belaundista.</t>
         </is>
       </c>
     </row>
@@ -2686,27 +2686,27 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Lerner - Formando la colección de arte contemporáneo del MALI (2013).txt</t>
+          <t>Buntinx - El poder y la ilusión. Pérdida y restauración del aura en la «República de Weimar peruana» 1980-1992 [MALI].md</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>mediados de los años 60 - 2013 (con foco en 1980-2000)</t>
+          <t>1980-1992</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo de colección, 2013</t>
+          <t>Ensayo académico (versión MALI), 2013 [escrito 1991-1994]</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Museo de Arte de Lima (MALI); Tatiana Cuevas; Miguel A. López; Gustavo Buntinx; Rodrigo Quijano; Jorge Villacorta; Natalia Majluf; E.P.S. Huayco; Teresa Burga; Milagros de la Torre; Flavia Gandolfo</t>
+          <t>Gustavo Buntinx; E.P.S. Huayco; Taller NN; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; Walter Benjamin; Jesús Ruiz Durand; Andy Warhol; Mirko Lauer; Museo de Arte de Lima (MALI); III Bienal de La Habana</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Ensayo introductorio de Sharon Lerner al libro que presenta la colección de arte contemporáneo del Museo de Arte de Lima (MALI), articulado como una lectura —entre muchas posibles— de la historia del arte reciente peruano a partir del acervo. Su tesis metodológica es que en el Perú el tránsito a la contemporaneidad no ocurre como un quiebre radical, sino como una serie de pequeños cambios discontinuos, por lo que la colección se organiza en dos principios: identificar momentos de ruptura de fines del siglo XX y perfilar la producción reciente por ejes temáticos. El recorrido histórico parte de mediados de los sesenta (vanguardias pop, experimentalismo, no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, cuando la migración y la sentencia de Mirko Lauer —«En el Perú, hoy, solo lo popular es moderno»— enmarcan la obra de E.P.S. Huayco. Recorre luego la hegemonía de la abstracción en los ochenta, el arte de derechos humanos de Ricardo Wiesse y Eduardo Villanes bajo el fujimorato, la irrupción de la Bienal Iberoamericana de Lima (1997) y el «bienalismo», y la generación de los 2000 (Flavia Gandolfo, Gilda Mantilla, Armando Andrade Tudela) vinculada al espacio La Culpable. El texto presenta además los ensayos de Miguel López, Gustavo Buntinx y Rodrigo Quijano incluidos en el volumen y la conversación de seis críticos (2011). Su aporte es explicitar la política de adquisiciones del MALI y su ambición de llenar el vacío institucional y discursivo, construyendo un marco regional e internacional para el arte peruano.</t>
+          <t>Ensayo seminal de Gustavo Buntinx —redactado entre 1991 y 1994, difundido en inglés en «Beyond the Fantastic» (1995) y publicado por primera vez en Perú en esta versión del MALI (2013)— que interpreta el radical cambio de época del arte peruano entre 1980 y 1992, periodo que denomina metafóricamente «República de Weimar peruana». Su marco conceptual adapta la dialéctica benjaminiana entre proximidad y distancia (el aura, su pérdida por la reproductibilidad técnica y su posible restauración) y las categorías de alegoría, montaje y apropiación de Owens, Foster y Craig Owens a una periferia extrema. El argumento se sostiene sobre el análisis iconográfico minucioso de dos o tres obras que abren y cierran la década. La primera, «Arte al paso» y sobre todo «Sarita Colonia» (1980) del taller E.P.S. Huayco: una enorme estampa de la santa migrante pintada sobre diez mil latas de leche y emplazada en la Panamericana Sur, que Buntinx lee como huaca (post)moderna y exvoto donde lo pequeñoburgués radical se articula figuradamente a lo popular en emergencia (el «pop achorado» y «chicha»). La segunda, «Maorilyn» / «Viva el maoísmo» (1989) del Taller NN: una serigrafía que travistió el rostro de Mao con labios warholianos, alegoría ambivalente de la violencia senderista y la estetización de la política. Su tesis vincula la desintegración social —hiperinflación, guerra civil, movida subte punk— con el desarrollo de una condición alegórica y neo-aurática; su aporte es un modelo teórico para leer el colectivismo y la (post)modernidad popular peruana.</t>
         </is>
       </c>
     </row>
@@ -2718,27 +2718,27 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - F(r)icciones cosmopolitas. Redefiniciones estéticas y políticas de una idea de vanguardia en los años 60s.txt</t>
+          <t>Lerner - Formando la colección de arte contemporáneo del MALI (2013).txt</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>1960-1976 (con antecedentes desde 1942-1947)</t>
+          <t>mediados de los años 60 - 2013 (con foco en 1980-2000)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico / capítulo de catálogo (MALI), s/f</t>
+          <t>Ensayo de catálogo de colección, 2013</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Emilio Tarazona; Juan Acha; Fernando de Szyszlo; Jorge Romero Brest; Teresa Burga; Rafael Hastings; Grupo Arte Nuevo; Jesús Ruiz Durand; José Gómez Sicre; Marta Traba; Instituto de Arte Contemporáneo (IAC); MoMA / Instituto Di Tella</t>
+          <t>Sharon Lerner; Museo de Arte de Lima (MALI); Tatiana Cuevas; Miguel A. López; Gustavo Buntinx; Rodrigo Quijano; Jorge Villacorta; Natalia Majluf; E.P.S. Huayco; Teresa Burga; Milagros de la Torre; Flavia Gandolfo</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>López reconstruye las mutaciones semánticas y políticas de la noción de vanguardia en el Perú entre los años sesenta y setenta, argumentando que la euforia cosmopolita del periodo fue el espejismo de una modernidad desarrollista tan prometedora como inacabada en un país socialmente fracturado. El objeto de estudio son las plataformas institucionales privadas (IAC, galerías, bienales americanas, concursos empresariales) que, apuntaladas por el panamericanismo de la Guerra Fría, la Alianza para el Progreso y la política curatorial estadounidense de José Gómez Sicre, promovieron primero la abstracción y luego el arte óptico, el pop y las ambientaciones. El texto traza el paso del declive de la abstracción szyszliana hacia el experimentalismo detonado por las conferencias de Jorge Romero Brest (1965) y la irrupción beligerante del grupo Arte Nuevo (1966-1968) contra el Festival Americano de Pintura. El marco conceptual articula la relación entre desarrollismo y vanguardia, y su posterior tensión con el subdesarrollo, siguiendo la radicalización de Juan Acha, quien tras 1968 y el golpe de Velasco redefine la vanguardia como 'guerrilla cultural' y horizonte revolucionario, hasta su exilio a México en 1971. López destaca las reconversiones de Teresa Burga y Rafael Hastings, el 'pop achorado' de Ruiz Durand al servicio de la Reforma Agraria, los festivales Contacta y las Carreras de chasquis. Su aporte es mostrar cómo la condición local, provinciana y periférica de las prácticas de los setenta y ochenta (Paréntesis, E.P.S. Huayco, Grupo Chaclacayo) actualizó de modo radical las pretensiones críticas sesenteras, canibalizando los conceptos metropolitanos de arte conceptual.</t>
+          <t>Ensayo introductorio de Sharon Lerner al libro que presenta la colección de arte contemporáneo del Museo de Arte de Lima (MALI), articulado como una lectura —entre muchas posibles— de la historia del arte reciente peruano a partir del acervo. Su tesis metodológica es que en el Perú el tránsito a la contemporaneidad no ocurre como un quiebre radical, sino como una serie de pequeños cambios discontinuos, por lo que la colección se organiza en dos principios: identificar momentos de ruptura de fines del siglo XX y perfilar la producción reciente por ejes temáticos. El recorrido histórico parte de mediados de los sesenta (vanguardias pop, experimentalismo, no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, cuando la migración y la sentencia de Mirko Lauer —«En el Perú, hoy, solo lo popular es moderno»— enmarcan la obra de E.P.S. Huayco. Recorre luego la hegemonía de la abstracción en los ochenta, el arte de derechos humanos de Ricardo Wiesse y Eduardo Villanes bajo el fujimorato, la irrupción de la Bienal Iberoamericana de Lima (1997) y el «bienalismo», y la generación de los 2000 (Flavia Gandolfo, Gilda Mantilla, Armando Andrade Tudela) vinculada al espacio La Culpable. El texto presenta además los ensayos de Miguel López, Gustavo Buntinx y Rodrigo Quijano incluidos en el volumen y la conversación de seis críticos (2011). Su aporte es explicitar la política de adquisiciones del MALI y su ambición de llenar el vacío institucional y discursivo, construyendo un marco regional e internacional para el arte peruano.</t>
         </is>
       </c>
     </row>
@@ -2750,27 +2750,27 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Quijano - Notas incompletas sobre el sitio de la fotografía peruana.md</t>
+          <t>López, Miguel A. - F(r)icciones cosmopolitas. Redefiniciones estéticas y políticas de una idea de vanguardia en los años 60s.txt</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>1900-2011 (con énfasis en 1920-1998)</t>
+          <t>1960-1976 (con antecedentes desde 1942-1947)</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo (MALI), s/f</t>
+          <t>Ensayo académico / capítulo de catálogo (MALI), s/f</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Quijano; Martín Chambi; José María Eguren; Carlos 'Chino' Domínguez; Aaron Siskind; Jesús Ruiz Durand; Claudia Martínez Garay; Daniela Ortiz; Foto Galería Secuencia; TAFOS; Taller NN; E.P.S. Huayco</t>
+          <t>Miguel A. López; Emilio Tarazona; Juan Acha; Fernando de Szyszlo; Jorge Romero Brest; Teresa Burga; Rafael Hastings; Grupo Arte Nuevo; Jesús Ruiz Durand; José Gómez Sicre; Marta Traba; Instituto de Arte Contemporáneo (IAC); MoMA / Instituto Di Tella</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Quijano ensaya una genealogía del 'sitio' de la fotografía peruana, sosteniendo que este medio inauguró un margen de creación moderno al margen de la institucionalidad académica de las bellas artes, alcanzando una temprana ubicuidad territorial y una masividad que condicionó la percepción misma de una realidad nacional. El texto, de estructura fragmentaria y numerada, contrapone dos matrices fundacionales: Martín Chambi como 'modernista sin modernidad' y profesional de la imagen surgido de una familia campesina andina —una 'oportunidad nacional'— frente a la miniatura pinhole intimista y hermética de José María Eguren, que prefigura la figura del fotógrafo-artista individual. Analiza a Carlos 'Chino' Domínguez como ojo testimonial de la urbanización y la nueva cultura popular (La resaca del Inca, el 'Cholo' Sotil, el filme Cholo y su reedición Mi cholo de Gruenberg), y la experiencia de la fotogalería Secuencia (1977-1980), que reinventó una tradición y un discurso del oficio adoptando a Minor White y Aaron Siskind. El marco conceptual enlaza fotografía, prensa y democratización de la imagen en el contexto del auge sindical y la repolitización popular de fines de los setenta, y la aparición de la fotoserigrafía disidente (Bedoya, Williams, Mariotti, Salazar) como catalizador de una nueva condición fotográfica colectiva, desde E.P.S. Huayco hasta el Taller NN. El aporte del texto es leer la fotografía como dispositivo de documento, archivo, memoria y duelo frente a la violencia política (Uchuraccay, Yuyanapaq), rastreando su 'grado cero' icónico en obras de Ruiz Durand, Claudia Martínez Garay y Daniela Ortiz, que develan la mirada colonial y la invisibilización étnica.</t>
+          <t>López reconstruye las mutaciones semánticas y políticas de la noción de vanguardia en el Perú entre los años sesenta y setenta, argumentando que la euforia cosmopolita del periodo fue el espejismo de una modernidad desarrollista tan prometedora como inacabada en un país socialmente fracturado. El objeto de estudio son las plataformas institucionales privadas (IAC, galerías, bienales americanas, concursos empresariales) que, apuntaladas por el panamericanismo de la Guerra Fría, la Alianza para el Progreso y la política curatorial estadounidense de José Gómez Sicre, promovieron primero la abstracción y luego el arte óptico, el pop y las ambientaciones. El texto traza el paso del declive de la abstracción szyszliana hacia el experimentalismo detonado por las conferencias de Jorge Romero Brest (1965) y la irrupción beligerante del grupo Arte Nuevo (1966-1968) contra el Festival Americano de Pintura. El marco conceptual articula la relación entre desarrollismo y vanguardia, y su posterior tensión con el subdesarrollo, siguiendo la radicalización de Juan Acha, quien tras 1968 y el golpe de Velasco redefine la vanguardia como 'guerrilla cultural' y horizonte revolucionario, hasta su exilio a México en 1971. López destaca las reconversiones de Teresa Burga y Rafael Hastings, el 'pop achorado' de Ruiz Durand al servicio de la Reforma Agraria, los festivales Contacta y las Carreras de chasquis. Su aporte es mostrar cómo la condición local, provinciana y periférica de las prácticas de los setenta y ochenta (Paréntesis, E.P.S. Huayco, Grupo Chaclacayo) actualizó de modo radical las pretensiones críticas sesenteras, canibalizando los conceptos metropolitanos de arte conceptual.</t>
         </is>
       </c>
     </row>
@@ -2782,32 +2782,64 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
+          <t>Quijano - Notas incompletas sobre el sitio de la fotografía peruana.md</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>1900-2011 (con énfasis en 1920-1998)</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Ensayo de catálogo (MALI), s/f</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Rodrigo Quijano; Martín Chambi; José María Eguren; Carlos 'Chino' Domínguez; Aaron Siskind; Jesús Ruiz Durand; Claudia Martínez Garay; Daniela Ortiz; Foto Galería Secuencia; TAFOS; Taller NN; E.P.S. Huayco</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>Quijano ensaya una genealogía del 'sitio' de la fotografía peruana, sosteniendo que este medio inauguró un margen de creación moderno al margen de la institucionalidad académica de las bellas artes, alcanzando una temprana ubicuidad territorial y una masividad que condicionó la percepción misma de una realidad nacional. El texto, de estructura fragmentaria y numerada, contrapone dos matrices fundacionales: Martín Chambi como 'modernista sin modernidad' y profesional de la imagen surgido de una familia campesina andina —una 'oportunidad nacional'— frente a la miniatura pinhole intimista y hermética de José María Eguren, que prefigura la figura del fotógrafo-artista individual. Analiza a Carlos 'Chino' Domínguez como ojo testimonial de la urbanización y la nueva cultura popular (La resaca del Inca, el 'Cholo' Sotil, el filme Cholo y su reedición Mi cholo de Gruenberg), y la experiencia de la fotogalería Secuencia (1977-1980), que reinventó una tradición y un discurso del oficio adoptando a Minor White y Aaron Siskind. El marco conceptual enlaza fotografía, prensa y democratización de la imagen en el contexto del auge sindical y la repolitización popular de fines de los setenta, y la aparición de la fotoserigrafía disidente (Bedoya, Williams, Mariotti, Salazar) como catalizador de una nueva condición fotográfica colectiva, desde E.P.S. Huayco hasta el Taller NN. El aporte del texto es leer la fotografía como dispositivo de documento, archivo, memoria y duelo frente a la violencia política (Uchuraccay, Yuyanapaq), rastreando su 'grado cero' icónico en obras de Ruiz Durand, Claudia Martínez Garay y Daniela Ortiz, que develan la mirada colonial y la invisibilización étnica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Cap 2 - Historia/MALI</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
           <t>Villacorta (ed.) - ¿Un arte visual a contrapelo de los dictados metropolitanos? En el Perú, el arte moderno es un gesto tardío [conversación en el MALI, 2011].txt</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
         <is>
           <t>1947-2011 (con eje en 1960-2002)</t>
         </is>
       </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="D74" s="2" t="inlineStr">
         <is>
           <t>Transcripción editada de conversación (MALI), 2011</t>
         </is>
       </c>
-      <c r="E73" s="3" t="inlineStr">
+      <c r="E74" s="3" t="inlineStr">
         <is>
           <t>Jorge Villacorta; Gustavo Buntinx; Miguel A. López; Rodrigo Quijano; Tatiana Cuevas; Natalia Majluf; E.P.S. Huayco; Grupo Arte Nuevo; Taller NN; Grupo Chaclacayo; Christian Bendayán; Fernando Bryce; MALI / Micromuseo</t>
         </is>
       </c>
-      <c r="F73" s="3" t="inlineStr">
+      <c r="F74" s="3" t="inlineStr">
         <is>
           <t>Editada por Villacorta a partir de dos sesiones de 2011 en el MALI, esta conversación a seis voces indaga si lo moderno está clausurado en el arte peruano de modo que permita definir lo contemporáneo. La tesis articuladora, propuesta por Quijano, es que en el Perú lo moderno solo ha podido darse 'a contrapelo' y como 'gesto tardío', a destiempo de las modernidades metropolitanas; López y Buntinx la matizan con la idea de temporalidades dislocadas y friccionadas que impiden toda historia lineal. El objeto de estudio es la genealogía de la vanguardia local: la contraposición entre Arte Nuevo (1966-1968), leído como destello cosmopolita fugaz, y E.P.S. Huayco y Paréntesis, cuya apropiación de Sarita Colonia y el 'pop achorado' marca una ruptura más perdurable y pertinente al medio. Buntinx despliega una secuencia estilístico-conceptual en clave pop/místico-libidinal —de la Twiggy de Emilio Hernández a Quistococha de Bendayán, pasando por el afiche de Ruiz Durand, la Maoirilyn del Taller NN y La Pachakuti de Alfredo Márquez— ligada a periodos políticos (desarrollismo, velasquismo, utopía socialista, dictadura fujimorista, revolución capitalista). Majluf sitúa el quiebre epocal de fin de siglo en el ingreso de la 'referencia' fotográfica (Bryce, Milagros de la Torre, Juan Enrique Bedoya, Mantilla), frente al neobarroco. El texto discute además la construcción de públicos, la institucionalidad faltante, el rol del curador, el mercado 'social' peruano, las subastas del MALI y la 'normalización de la diferencia' como riesgo de la consagración institucional del pasado radical.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F73"/>
+  <autoFilter ref="A1:F74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Cataloga y analiza (baterías 2.3.3 y 2.3.4) Quijano «¿De qué puntos cardinales hablan?»
- Cataloga Cap 2 - Historia/ICAA-1146549.pdf (ensayo de Rodrigo Quijano,
  nov. 2001, catálogo «Puntos Cardinales») en tabla-cap2-historia.csv y
  regenera el Excel.
- Añade a analisis/ el informe de datos crudos aplicando la batería común
  B1-B13 y las propias de los tramos 2.3.3 (P1-P7) y 2.3.4 (P1-P8), con
  citas verbatim del OCR del ICAA y ubicación por § (sección).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bob4w11uQRyAcv1Qayw1V
</commit_message>
<xml_diff>
--- a/Sistematización/tablas-sistematizacion.xlsx
+++ b/Sistematización/tablas-sistematizacion.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Extras" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cap 3 - Análisis'!$A$1:$F$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Teoría'!$A$1:$F$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Extras'!$A$1:$F$4</definedName>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -894,27 +894,27 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>El Pabellón ha caído - Buntinx.md</t>
+          <t>EPS_HUAYCO_Buntinx_2005.txt</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>1980-1992 (violencia política; obra pictórica de 1992; masacre de El Frontón, 1986)</t>
+          <t>1979-1981 (con amplio contexto desde ca. 1968-1978; publicado en 2005)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Artículo de crítica de arte en prensa, 14-06-1992</t>
+          <t>Estudio histórico-crítico de historia del arte de Gustavo Buntinx (2005) sobre el colectivo E.P.S. Huayco; edición digital en OpenEdition Books («Combates por la historia», p. 12-16). La atribución al volumen E.P.S. Huayco. Documentos (MALI/IFEA, 2005) es deducida.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Elio Martuccelli; Juan Javier Salazar; Herbert Rodríguez; Jaime Higa; grupo Huayco; los NN; los Bestias; José Tola; Piero Quijano; Anselmo Carrera; Roy Lichtenstein; Diario La República (suplemento Culturas)</t>
+          <t>Gustavo Buntinx; E.P.S. Huayco; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; María Luy; Charo Noriega; Mariela Zevallos; Armando Williams; Mirko Lauer; Juan Acha; Sarita Colonia; Contacta 79; SINAMOS; Sendero Luminoso; Micromuseo</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Artículo de Gustavo Buntinx publicado en el suplemento "Culturas" del diario La República el 14 de junio de 1992, concebido como crónica reflexiva y no como mero juicio de valor. El texto lee la plástica peruana como escenario privilegiado para registrar la subjetividad de un "pequeño-burgués-ilustrado" durante los doce años de violencia (1980-1992), esa frágil "República de Weimar" peruana en su ocaso. El objeto de estudio central es la exposición "Se vende" de Elio Martuccelli, arquitecto de vocación teórica situado en los márgenes entre los grupos Bestias y NN y vinculado a la plástica alternativa que arranca de Huayco. Buntinx se concentra en un cuadríptico donde Martuccelli reproduce páginas de un cómic editado por la Marina de Guerra sobre Miguel Grau (centenario de 1979), cuyo último recuadro reza "¡El pabellón ha caído!". El marco conceptual articula apropiación, cita y "copia de la copia": Martuccelli mira a Lichtenstein a través del Pop achorado de Juan Javier Salazar (su lámina de presidentes, 1980), reivindicando la brocha gorda artesanal frente al refinamiento tecnológico del pop norteamericano como signo de una modernidad fallida y periférica. Mediante mínimas intervenciones -reencuadres, ocultamiento de la franja roja de la bandera, transformación de "fuego" en "ego"- la obra hace hablar las contradicciones reprimidas de la comunicación masiva y evoca el aniquilamiento de los presos de El Frontón y el crimen de María Elena Moyano. El aporte es una crítica que politiza lo íntimo: el pabellón caído figura el quiebre entre la intelectualidad joven y los mitos republicanos, irreversiblemente cancelados por defensores e impugnadores por igual.</t>
+          <t>Estudio histórico-crítico extenso (unas 82.000 palabras) de Gustavo Buntinx sobre el colectivo E.P.S. Huayco (1979-1981), concebido como la reconstrucción documental de referencia del grupo y de su obra mayor, el mosaico de Sarita Colonia levantado con miles de latas de leche vacías sobre la Panamericana Sur. Escrito desde la proximidad personal del autor con los integrantes, reivindica una «descripción factual de los hechos» apoyada en crítica de fuentes, filología, hermenéutica y heurística, y se propone corregir la «acumulación impresionante de errores» de la bibliografía reciente: la datación equivocada de Sarita Colonia en 1981, la confusión de Contacta 79 con las elecciones a la Asamblea Constituyente de 1978, y las tergiversaciones de autorías, fechas y títulos. Organizado en secciones («Definiciones», «La utopía socialista», «El fin de la inocencia. La reforma frustrada», «Revolución en la revolución. El cisma», entre otras), traza la genealogía del colectivo desde la crisis del reformismo velasquista y el horizonte de la nueva izquierda, y narra Contacta, la muestra Arte al paso, el «pop achorado», las salchipapas gigantes y la disolución del grupo, en el marco del inicio de la violencia senderista. Reúne a Francisco Mariotti, Herbert Rodríguez, Juan Javier Salazar, María Luy, Charo Noriega, Mariela Zevallos y Armando Williams, y discute a Mirko Lauer y Juan Acha. Es el «estudio de 2005» de referencia sobre Huayco al que remiten otras fuentes del capítulo; emplea «culminación» y «cristalización» al caracterizar el lugar del grupo, y no usa la fórmula «arte crítico».</t>
         </is>
       </c>
     </row>
@@ -926,27 +926,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Elera, Gonzales y Silva - Lunes de crítica 2017-2018. Convulsión y autoorganización.md</t>
+          <t>El Pabellón ha caído - Buntinx.md</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>2014-2018 (programa Lunes de Crítica, oct. 2017 - mar. 2018)</t>
+          <t>1980-1992 (violencia política; obra pictórica de 1992; masacre de El Frontón, 1986)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Capítulo/ensayo en publicación, c. 2019</t>
+          <t>Artículo de crítica de arte en prensa, 14-06-1992</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Andrea Elera; Gustavo Gonzales; Raúl Silva; Por una Comunidad de las Artes Visuales; Museo de Arte de San Marcos (MASM); Augusto del Valle; Juan Javier Salazar; Pabellón Peruano de la Bienal de Venecia; Proyecto Fugaz / Monumental Callao; Lugar de la Memoria (LUM); Sonia Cunliffe; PUCP-ENSABAP</t>
+          <t>Gustavo Buntinx; Elio Martuccelli; Juan Javier Salazar; Herbert Rodríguez; Jaime Higa; grupo Huayco; los NN; los Bestias; José Tola; Piero Quijano; Anselmo Carrera; Roy Lichtenstein; Diario La República (suplemento Culturas)</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Texto reflexivo de Andrea Elera, Gustavo Gonzales y Raúl Silva, integrantes del colectivo "Por una Comunidad de las Artes Visuales", que balancea la experiencia del programa "Lunes de Crítica" (quince mesas realizadas los lunes entre octubre de 2017 y marzo de 2018 en el Museo de Arte de San Marcos, MASM). El argumento central sostiene que la autoorganización y la subjetivación crítica de los trabajadores de las artes son respuestas necesarias frente a la informalidad laboral, la fragmentación y la captura privada del sistema artístico limeño. Los autores enumeran los "exabruptos" que entre 2014 y 2017 detonaron la formación del colectivo: el borrado de murales del Centro de Lima por la gestión de Castañeda Lossio, el plagio en el texto curatorial de "Pasaporte para un Artista", los vínculos de lavado de activos del proyecto Fugaz y la gentrificación de Monumental Callao, y sobre todo la polémica gestión y curaduría del Pabellón Peruano en la 57 Bienal de Venecia (2017), con la presentación póstuma de la obra de Juan Javier Salazar, que actuó como detonante organizativo. Describen la estructura pedagógica del programa en cinco unidades (sector público-privado, gestión cultural y ciudadanía, espacios en disputa, educación artística e investigación/crítica), reconociendo antecedentes en los "Lunes de Crítica" que Augusto del Valle dirigió en el MASM (2002-2004). El balance admite el desgaste logístico y el carácter autoformativo del proceso —más autoaprendizaje que aporte comunitario—, ejemplificado en la tensa mesa sobre Fugaz con Sonia Cunliffe, pero reivindica la articulación colectiva, la crítica devenida propuesta y la voz común como metas de largo aliento, asumiendo su sesgo limeño y centralista.</t>
+          <t>Artículo de Gustavo Buntinx publicado en el suplemento "Culturas" del diario La República el 14 de junio de 1992, concebido como crónica reflexiva y no como mero juicio de valor. El texto lee la plástica peruana como escenario privilegiado para registrar la subjetividad de un "pequeño-burgués-ilustrado" durante los doce años de violencia (1980-1992), esa frágil "República de Weimar" peruana en su ocaso. El objeto de estudio central es la exposición "Se vende" de Elio Martuccelli, arquitecto de vocación teórica situado en los márgenes entre los grupos Bestias y NN y vinculado a la plástica alternativa que arranca de Huayco. Buntinx se concentra en un cuadríptico donde Martuccelli reproduce páginas de un cómic editado por la Marina de Guerra sobre Miguel Grau (centenario de 1979), cuyo último recuadro reza "¡El pabellón ha caído!". El marco conceptual articula apropiación, cita y "copia de la copia": Martuccelli mira a Lichtenstein a través del Pop achorado de Juan Javier Salazar (su lámina de presidentes, 1980), reivindicando la brocha gorda artesanal frente al refinamiento tecnológico del pop norteamericano como signo de una modernidad fallida y periférica. Mediante mínimas intervenciones -reencuadres, ocultamiento de la franja roja de la bandera, transformación de "fuego" en "ego"- la obra hace hablar las contradicciones reprimidas de la comunicación masiva y evoca el aniquilamiento de los presos de El Frontón y el crimen de María Elena Moyano. El aporte es una crítica que politiza lo íntimo: el pabellón caído figura el quiebre entre la intelectualidad joven y los mitos republicanos, irreversiblemente cancelados por defensores e impugnadores por igual.</t>
         </is>
       </c>
     </row>
@@ -958,27 +958,27 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Flores Hora, David - 2026-04-16.transcripcion.md</t>
+          <t>Elera, Gonzales y Silva - Lunes de crítica 2017-2018. Convulsión y autoorganización.md</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2000-2020 (con referencias a los años 80)</t>
+          <t>2014-2018 (programa Lunes de Crítica, oct. 2017 - mar. 2018)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Entrevista, 16-04-2026</t>
+          <t>Capítulo/ensayo en publicación, c. 2019</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>David Flores Hora; Carlos Zevallos (entrevistador); Centro Cultural de España; Ricardo Ramón; Sala Luis Miró Quesada Garland; Luis Lama; Jorge Villacorta; José Carlos Mariátegui; Christian Bendayán; MALI; Natalia Majluf; Miguel López; ICPNA; Ministerio de Cultura (ARCOmadrid); LUM</t>
+          <t>Andrea Elera; Gustavo Gonzales; Raúl Silva; Por una Comunidad de las Artes Visuales; Museo de Arte de San Marcos (MASM); Augusto del Valle; Juan Javier Salazar; Pabellón Peruano de la Bienal de Venecia; Proyecto Fugaz / Monumental Callao; Lugar de la Memoria (LUM); Sonia Cunliffe; PUCP-ENSABAP</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Testimonio de David Flores Hora, historiador del arte sanmarquino y gestor cultural, recogido por Carlos Zevallos en el marco de una tesis doctoral sobre el «arte crítico» y su institucionalización en Lima. La entrevista reconstruye una trayectoria que enlaza la formación en San Marcos durante el ocaso del fujimorato (ingreso en 2000), la coordinación de artes visuales del Centro Cultural de España (2007-2010), el paso por la Sala Luis Miró Quesada Garland junto a Luis Lama, el ICPNA, el Ministerio de Cultura (coordinación de la presencia peruana en ARCOmadrid) y el LUM. Flores Hora sostiene una tesis periodizadora: la primera década de 2000 fue un momento de efervescencia donde «ser contemporáneo» equivalía a asumir una posición política y a intervenir el espacio expositivo, alimentada por la resaca de la Bienal de Lima y las redes latinoamericanas; a partir de 2011 sobreviene la institucionalización (viraje del MALI hacia lo contemporáneo hacia 2008), sucedida por lo que denomina «dictaduras» consecutivas de la crítica, la curaduría y, finalmente, el coleccionismo. El relato contrapone la libertad de un espacio de extranjería (España) a la precariedad estatal, y lamenta la pérdida del «potencial revolucionario» ante la economización del campo y el ascenso del artista global y del arte amazónico (Bendayán) como opción menos confrontacional. Menciona el proyecto de archivo CEDAP, portafolios con Natalia Majluf, Emilio Tarazona y Miguel López, y aboga por archivos vivos. Su posición combina nostalgia militante y una conciencia ética de la sobrevivencia profesional en un medio desfinanciado.</t>
+          <t>Texto reflexivo de Andrea Elera, Gustavo Gonzales y Raúl Silva, integrantes del colectivo "Por una Comunidad de las Artes Visuales", que balancea la experiencia del programa "Lunes de Crítica" (quince mesas realizadas los lunes entre octubre de 2017 y marzo de 2018 en el Museo de Arte de San Marcos, MASM). El argumento central sostiene que la autoorganización y la subjetivación crítica de los trabajadores de las artes son respuestas necesarias frente a la informalidad laboral, la fragmentación y la captura privada del sistema artístico limeño. Los autores enumeran los "exabruptos" que entre 2014 y 2017 detonaron la formación del colectivo: el borrado de murales del Centro de Lima por la gestión de Castañeda Lossio, el plagio en el texto curatorial de "Pasaporte para un Artista", los vínculos de lavado de activos del proyecto Fugaz y la gentrificación de Monumental Callao, y sobre todo la polémica gestión y curaduría del Pabellón Peruano en la 57 Bienal de Venecia (2017), con la presentación póstuma de la obra de Juan Javier Salazar, que actuó como detonante organizativo. Describen la estructura pedagógica del programa en cinco unidades (sector público-privado, gestión cultural y ciudadanía, espacios en disputa, educación artística e investigación/crítica), reconociendo antecedentes en los "Lunes de Crítica" que Augusto del Valle dirigió en el MASM (2002-2004). El balance admite el desgaste logístico y el carácter autoformativo del proceso —más autoaprendizaje que aporte comunitario—, ejemplificado en la tensa mesa sobre Fugaz con Sonia Cunliffe, pero reivindica la articulación colectiva, la crítica devenida propuesta y la voz común como metas de largo aliento, asumiendo su sesgo limeño y centralista.</t>
         </is>
       </c>
     </row>
@@ -990,27 +990,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Germaná, Gabriela - 20 de noviembre.transcripcion.md</t>
+          <t>Entrevista - Flores Hora, David - 2026-04-16.transcripcion.md</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Años 80 y 90 y 2013-2025</t>
+          <t>2000-2020 (con referencias a los años 80)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Entrevista, 20 de noviembre (año no precisado)</t>
+          <t>Entrevista, 16-04-2026</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Gabriela Germaná; Carlos Zevallos (entrevistador); Venuca Evanán; Violeta Quispe; tablas de Sarhua; MAC; MALI; Natalia Majluf; Miguel López; Pedro Pablo Alayza; ICPNA/IMNA; galería Ginsberg; Baró; Luis Lama; Claire Bishop</t>
+          <t>David Flores Hora; Carlos Zevallos (entrevistador); Centro Cultural de España; Ricardo Ramón; Sala Luis Miró Quesada Garland; Luis Lama; Jorge Villacorta; José Carlos Mariátegui; Christian Bendayán; MALI; Natalia Majluf; Miguel López; ICPNA; Ministerio de Cultura (ARCOmadrid); LUM</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Entrevista a la historiadora del arte y curadora Gabriela Germ&lt;200b&gt;aná, especialista en artes populares y tablas de Sarhua, conducida por Carlos Zevallos para tensionar su hipótesis del «mandato crítico». Germaná matiza la noción de mandato, pero reconoce que la institucionalidad contemporánea hoy «da la bienvenida» e incorpora de inmediato discursos críticos —género, indigenidad, decolonialidad— que en los años ochenta permanecían marginales y solo fueron reconocidos a posteriori. El argumento articula tres ejes: la periodización del arte político peruano (los colectivos de los ochenta como indispensables para entender la década, frente al arte pro-gubernamental del velasquismo); su propia práctica curatorial de reivindicación de sujetos marginados (paridad de género, artistas regionales) en jurados de concursos como el del ICPNA/IMNA, el MUSE y Cultura, donde persisten tensiones generacionales entre «calidad estética» y postura política; y el caso de Venuca Evanán y Violeta Quispe, cuyo giro crítico —género, erotismo, memoria, retablos por la memoria— fue la condición que les abrió las puertas del arte contemporáneo, diferenciándolas del campo costumbrista del arte popular (series Piras Causa y Éxodo de los noventa, ingreso al MALI). Germaná problematiza el «extractivismo» de galerías internacionales (Baró, Ginsberg) que demandan producción sin diálogo, la fragilidad institucional local (MAC, MALI, gestión de Pedro Pablo Alayza), la sospecha ante el arte amazónico como inversión no confrontacional del coleccionismo, y el contraste con una historia del arte estadounidense más atravesada por raza, género y clase que la conservadora academia peruana. Reflexiona, además, sobre los límites del juicio crítico ante la producción indígena.</t>
+          <t>Testimonio de David Flores Hora, historiador del arte sanmarquino y gestor cultural, recogido por Carlos Zevallos en el marco de una tesis doctoral sobre el «arte crítico» y su institucionalización en Lima. La entrevista reconstruye una trayectoria que enlaza la formación en San Marcos durante el ocaso del fujimorato (ingreso en 2000), la coordinación de artes visuales del Centro Cultural de España (2007-2010), el paso por la Sala Luis Miró Quesada Garland junto a Luis Lama, el ICPNA, el Ministerio de Cultura (coordinación de la presencia peruana en ARCOmadrid) y el LUM. Flores Hora sostiene una tesis periodizadora: la primera década de 2000 fue un momento de efervescencia donde «ser contemporáneo» equivalía a asumir una posición política y a intervenir el espacio expositivo, alimentada por la resaca de la Bienal de Lima y las redes latinoamericanas; a partir de 2011 sobreviene la institucionalización (viraje del MALI hacia lo contemporáneo hacia 2008), sucedida por lo que denomina «dictaduras» consecutivas de la crítica, la curaduría y, finalmente, el coleccionismo. El relato contrapone la libertad de un espacio de extranjería (España) a la precariedad estatal, y lamenta la pérdida del «potencial revolucionario» ante la economización del campo y el ascenso del artista global y del arte amazónico (Bendayán) como opción menos confrontacional. Menciona el proyecto de archivo CEDAP, portafolios con Natalia Majluf, Emilio Tarazona y Miguel López, y aboga por archivos vivos. Su posición combina nostalgia militante y una conciencia ética de la sobrevivencia profesional en un medio desfinanciado.</t>
         </is>
       </c>
     </row>
@@ -1022,27 +1022,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Hernández Calvo, Max - 7jul2025.transcripcion.md</t>
+          <t>Entrevista - Germaná, Gabriela - 20 de noviembre.transcripcion.md</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>1997-2015 (con referencias a los años 70)</t>
+          <t>Años 80 y 90 y 2013-2025</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Entrevista, 07-07-2025</t>
+          <t>Entrevista, 20 de noviembre (año no precisado)</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Max Hernández Calvo; Carlos Zevallos (entrevistador); Miguel López; Emilio Tarazona; Juan Peralta; Bienales de Lima; Teresa Burga; MALI; Bard College; ICPNA/IMNA; Juan Carlos Verme; Carlos Marsano; Eduardo Hochschild; Alfonso García Miró</t>
+          <t>Gabriela Germaná; Carlos Zevallos (entrevistador); Venuca Evanán; Violeta Quispe; tablas de Sarhua; MAC; MALI; Natalia Majluf; Miguel López; Pedro Pablo Alayza; ICPNA/IMNA; galería Ginsberg; Baró; Luis Lama; Claire Bishop</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Conversación con el crítico y curador Max Hernández Calvo, sostenida con Carlos Zevallos en julio de 2025, centrada en la genealogía del «mandato crítico» y de la «lógica de proyecto» en el arte contemporáneo peruano. Hernández Calvo homologa el arte crítico con la producción de discurso y argumenta que los artistas jóvenes no perciben un mandato porque han sido formados dentro de un sistema que exige conceptualización previa, statement y portafolio; quienes sí lo leen como imposición externa suelen carecer de discurso, malinterpretándolo en clave esencialista o conspirativa. Reconstruye hitos institucionales: las Bienales de Lima de fines de los noventa (con Juan Peralta) que impulsaron la postulación mediante proyectos de instalación; su propia experiencia en la Bienal Nacional (1998) y en el MFA de baja residencia de Bard College (2005-2007), cuya estructura de crítica grupal evidenciaba la centralidad del discurso. Sitúa entre 2010 y 2015 la consolidación del mandato, ligada al viraje del MALI hacia lo contemporáneo, la aparición de ferias (Lima Foto, ArtLima), galerías nuevas (Revólver) y el redescubrimiento de Teresa Burga y del conceptualismo de los sesenta-setenta por Miguel López y Emilio Tarazona. Analiza los concursos (IMNA desde 2018, Pasaporte para un Artista, Artus) como síntoma del cambio, y la formación de coleccionistas (CAAC, 2006; Verme, Marsano, Hochschild, García Miró) entrenados en circuitos internacionales orientados al discurso. Cierra con una tesis sobre el extractivismo: la escena local colapsa tras las crisis políticas de 2016-2021 y la pandemia, y el artista deviene materia prima exportable, sostenido económicamente por galerías y compradores extranjeros.</t>
+          <t>Entrevista a la historiadora del arte y curadora Gabriela Germ&lt;200b&gt;aná, especialista en artes populares y tablas de Sarhua, conducida por Carlos Zevallos para tensionar su hipótesis del «mandato crítico». Germaná matiza la noción de mandato, pero reconoce que la institucionalidad contemporánea hoy «da la bienvenida» e incorpora de inmediato discursos críticos —género, indigenidad, decolonialidad— que en los años ochenta permanecían marginales y solo fueron reconocidos a posteriori. El argumento articula tres ejes: la periodización del arte político peruano (los colectivos de los ochenta como indispensables para entender la década, frente al arte pro-gubernamental del velasquismo); su propia práctica curatorial de reivindicación de sujetos marginados (paridad de género, artistas regionales) en jurados de concursos como el del ICPNA/IMNA, el MUSE y Cultura, donde persisten tensiones generacionales entre «calidad estética» y postura política; y el caso de Venuca Evanán y Violeta Quispe, cuyo giro crítico —género, erotismo, memoria, retablos por la memoria— fue la condición que les abrió las puertas del arte contemporáneo, diferenciándolas del campo costumbrista del arte popular (series Piras Causa y Éxodo de los noventa, ingreso al MALI). Germaná problematiza el «extractivismo» de galerías internacionales (Baró, Ginsberg) que demandan producción sin diálogo, la fragilidad institucional local (MAC, MALI, gestión de Pedro Pablo Alayza), la sospecha ante el arte amazónico como inversión no confrontacional del coleccionismo, y el contraste con una historia del arte estadounidense más atravesada por raza, género y clase que la conservadora academia peruana. Reflexiona, además, sobre los límites del juicio crítico ante la producción indígena.</t>
         </is>
       </c>
     </row>
@@ -1054,27 +1054,27 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Lerner, Sharon - sin fecha.transcripcion.md</t>
+          <t>Entrevista - Hernández Calvo, Max - 7jul2025.transcripcion.md</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>2007-2025 (historia de la colección del MALI)</t>
+          <t>1997-2015 (con referencias a los años 70)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Entrevista, s/f (transcripción 2026)</t>
+          <t>Entrevista, 07-07-2025</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Carlos Zevallos (entrevistador); MALI; Natalia Majluf; Tatiana Cuevas; Jorge Villacorta; Rodrigo Quijano; Miguel López; Julieta González; Florencia Portocarrero; Goethe Institut; Ricardo Kusunoki</t>
+          <t>Max Hernández Calvo; Carlos Zevallos (entrevistador); Miguel López; Emilio Tarazona; Juan Peralta; Bienales de Lima; Teresa Burga; MALI; Bard College; ICPNA/IMNA; Juan Carlos Verme; Carlos Marsano; Eduardo Hochschild; Alfonso García Miró</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Entrevista a Sharon Lerner, curadora de arte contemporáneo y directora del MALI, realizada por Carlos Zevallos (transcripción de 2026). Lerner sostiene que el museo no maneja una definición taxativa de «arte contemporáneo»: se trata de un corte histórico en permanente redefinición, discutido cíclicamente con el comité académico, los asesores rotativos del Comité de Adquisiciones de Arte Contemporáneo y encuentros especializados. Reconstruye dos momentos de revisión: el volumen editado con fondo Sura (2013), heredado de Tatiana Cuevas, con ensayos de asesores (Villacorta, Quijano, Miguel López) y una conversación editada por Villacorta que expone tensiones y «discontinuidades»; y el encuentro de 2015 (con apoyo del Goethe Institut y a instancias de Julieta González) para la creación de un fondo amazónico, que reconocía institucionalmente una escena preexistente. Frente a la hipótesis del «mandato crítico», Lerner precisa que la criticidad es parte constitutiva de la práctica contemporánea, pero no un requisito excluyente ni un factor disuasivo: el museo posee obra crítica con la propia institución, y los criterios de adquisición (votación, pertinencia discursiva, conservación, precio) son múltiples. Distingue entre obras que «encarnan» (embody) discurso y aquellas meramente «formulaicas» que exhiben etiquetas. Subraya la ventaja comparativa del MALI como museo panorámico —que cruza lo precolombino, textil, popular y contemporáneo— y su rol de facto como único coleccionista sostenido ante la ausencia de otras instituciones. Explica que se expone solo por invitación curatorial, atendiendo vacíos (presencia femenina, perspectivas queer señaladas por Miguel López), y anuncia un futuro concurso de intervenciones y la proyectada expansión hacia salas del siglo XXI.</t>
+          <t>Conversación con el crítico y curador Max Hernández Calvo, sostenida con Carlos Zevallos en julio de 2025, centrada en la genealogía del «mandato crítico» y de la «lógica de proyecto» en el arte contemporáneo peruano. Hernández Calvo homologa el arte crítico con la producción de discurso y argumenta que los artistas jóvenes no perciben un mandato porque han sido formados dentro de un sistema que exige conceptualización previa, statement y portafolio; quienes sí lo leen como imposición externa suelen carecer de discurso, malinterpretándolo en clave esencialista o conspirativa. Reconstruye hitos institucionales: las Bienales de Lima de fines de los noventa (con Juan Peralta) que impulsaron la postulación mediante proyectos de instalación; su propia experiencia en la Bienal Nacional (1998) y en el MFA de baja residencia de Bard College (2005-2007), cuya estructura de crítica grupal evidenciaba la centralidad del discurso. Sitúa entre 2010 y 2015 la consolidación del mandato, ligada al viraje del MALI hacia lo contemporáneo, la aparición de ferias (Lima Foto, ArtLima), galerías nuevas (Revólver) y el redescubrimiento de Teresa Burga y del conceptualismo de los sesenta-setenta por Miguel López y Emilio Tarazona. Analiza los concursos (IMNA desde 2018, Pasaporte para un Artista, Artus) como síntoma del cambio, y la formación de coleccionistas (CAAC, 2006; Verme, Marsano, Hochschild, García Miró) entrenados en circuitos internacionales orientados al discurso. Cierra con una tesis sobre el extractivismo: la escena local colapsa tras las crisis políticas de 2016-2021 y la pandemia, y el artista deviene materia prima exportable, sostenido económicamente por galerías y compradores extranjeros.</t>
         </is>
       </c>
     </row>
@@ -1086,27 +1086,27 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Rebaza Torres, Alberto - 2023-10-12 (editada).docx</t>
+          <t>Entrevista - Lerner, Sharon - sin fecha.transcripcion.md</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 90 - 2023</t>
+          <t>2007-2025 (historia de la colección del MALI)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Entrevista, 12-10-2023 (editada)</t>
+          <t>Entrevista, s/f (transcripción 2026)</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Alberto Rebaza Torres; Carlos Zevallos Trigoso (entrevistador); MALI; CAAC; Ginette Fernández; Residencia de Al Lado; Bienal de Venecia; Museo Reina Sofía; Guggenheim; Eduardo Hochschild; Juan Carlos Verme; Carlos Marsano; ICPNA; Sandra Gamarra</t>
+          <t>Sharon Lerner; Carlos Zevallos (entrevistador); MALI; Natalia Majluf; Tatiana Cuevas; Jorge Villacorta; Rodrigo Quijano; Miguel López; Julieta González; Florencia Portocarrero; Goethe Institut; Ricardo Kusunoki</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Entrevista editada a Alberto Rebaza Torres —abogado, coleccionista y presidente del consejo directivo del MALI, además de expresidente del Comité de Adquisiciones de Arte Contemporáneo—, conducida por Carlos Zevallos Trigoso en octubre de 2023. Rebaza narra el origen de su coleccionismo a fines de los noventa, orientado inicial y deliberadamente al arte peruano contemporáneo y luego extendido a lo latinoamericano, bajo la convicción de una «misión»: que el coleccionismo local funcione como primera plataforma de desarrollo para los artistas. Ubica en 2006 la formación del CAAC como factor de cohesión de un grupo de coleccionistas peruanos que ganó visibilidad en ferias regionales e internacionales (ArteBA, ARTBO, Zona Maco, Art Basel). El testimonio articula una teoría del coleccionismo como «proselitismo del arte» que, con el tiempo, debilita la sensación de propiedad y migra hacia la filantropía y el fortalecimiento institucional, ante la ausencia del Estado. Distingue el potencial «colectivo» del coleccionista frente al potencial «de a uno» del galerista, y enfatiza la complementariedad de roles (galerías, ferias, curadores, residencias) en una carrera artística sin hitos claros. Reivindica su Residencia de Al Lado (con Ginette Fernández) y menciona a otros agentes (Hochschild-MAC, Verme-MALI, Marsano-ARTUS, Mulder, Barreda). Sobre su criterio personal, prioriza la tríada contenido, inteligencia y estética, y diferencia expresamente su línea de coleccionismo de la línea curatorial del MALI —más volcada a violencia, territorio, género e historia, próxima al Reina Sofía—. El documento es fuente clave para analizar la perspectiva del coleccionismo y la filantropía en la institucionalización del arte contemporáneo peruano.</t>
+          <t>Entrevista a Sharon Lerner, curadora de arte contemporáneo y directora del MALI, realizada por Carlos Zevallos (transcripción de 2026). Lerner sostiene que el museo no maneja una definición taxativa de «arte contemporáneo»: se trata de un corte histórico en permanente redefinición, discutido cíclicamente con el comité académico, los asesores rotativos del Comité de Adquisiciones de Arte Contemporáneo y encuentros especializados. Reconstruye dos momentos de revisión: el volumen editado con fondo Sura (2013), heredado de Tatiana Cuevas, con ensayos de asesores (Villacorta, Quijano, Miguel López) y una conversación editada por Villacorta que expone tensiones y «discontinuidades»; y el encuentro de 2015 (con apoyo del Goethe Institut y a instancias de Julieta González) para la creación de un fondo amazónico, que reconocía institucionalmente una escena preexistente. Frente a la hipótesis del «mandato crítico», Lerner precisa que la criticidad es parte constitutiva de la práctica contemporánea, pero no un requisito excluyente ni un factor disuasivo: el museo posee obra crítica con la propia institución, y los criterios de adquisición (votación, pertinencia discursiva, conservación, precio) son múltiples. Distingue entre obras que «encarnan» (embody) discurso y aquellas meramente «formulaicas» que exhiben etiquetas. Subraya la ventaja comparativa del MALI como museo panorámico —que cruza lo precolombino, textil, popular y contemporáneo— y su rol de facto como único coleccionista sostenido ante la ausencia de otras instituciones. Explica que se expone solo por invitación curatorial, atendiendo vacíos (presencia femenina, perspectivas queer señaladas por Miguel López), y anuncia un futuro concurso de intervenciones y la proyectada expansión hacia salas del siglo XXI.</t>
         </is>
       </c>
     </row>
@@ -1118,27 +1118,27 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Tokeshi, Eduardo - sin fecha.transcripcion.md</t>
+          <t>Entrevista - Rebaza Torres, Alberto - 2023-10-12 (editada).docx</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>1980-2002</t>
+          <t>Fines de los años 90 - 2023</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Entrevista, s/f</t>
+          <t>Entrevista, 12-10-2023 (editada)</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Eduardo Tokeshi; Carlos Zevallos (entrevistador); PUCP; Gustavo Buntinx; Luis Lama; E.P.S. Huayco; Herbert Rodríguez; Bienal de Lima; Emilio Rodríguez Larraín; Jorge Eduardo Eielson; Luis Camnitzer; Óscar Muñoz</t>
+          <t>Alberto Rebaza Torres; Carlos Zevallos Trigoso (entrevistador); MALI; CAAC; Ginette Fernández; Residencia de Al Lado; Bienal de Venecia; Museo Reina Sofía; Guggenheim; Eduardo Hochschild; Juan Carlos Verme; Carlos Marsano; ICPNA; Sandra Gamarra</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Entrevista al artista Eduardo Tokeshi (n. 1960), conducida por Carlos Zevallos, que reconstruye su formación y la génesis de su obra más reconocida en el contexto de la violencia política peruana. Tokeshi relata su tránsito de la arquitectura a la especialidad de pintura en la PUCP hacia 1983, dentro de la clásica división entre la Católica (abstracción) y Bellas Artes (figuración), y su desmarque del canon al incorporar recortes periodísticos, objetos y materiales no pictóricos. Sitúa en 1985 la primera «Bandera» —cosida, rellena, tensada—, realizada por pulsión antes que como gesto deliberadamente contemporáneo, que inaugura una serie sostenida hasta 2001-2002 como sublimación de la violencia, el duelo y la reconstrucción de la nación. El testimonio historiza el surgimiento de lo contemporáneo local: la muestra «Algo va a pasar» (1987) organizada por Gustavo Buntinx, la Bienal de Trujillo (1987), las Bienales de Lima de los noventa y la labor de Luis Lama trayendo a Camnitzer y Óscar Muñoz. Analiza la profesionalización del campo en los noventa (idea de «proyecto», statements, portafolios, cambios de currícula), el desfase o «refracción» respecto de los centros internacionales (São Paulo, León) y la posterior consolidación de la figura del curador. Contrapone su disidencia formativa —hacer lo deseado siempre que pudiera sustentarlo— a la incorporación curricular del perfil «crítico» como expectativa. Cierra describiendo el proceso material de «Bandera VIII», con bolsas de transfusión llenas de falsa sangre y sal (símbolo de la saladera), asociada a su pertenencia a un club RH negativo, como emblema de una patria en cuidados intensivos.</t>
+          <t>Entrevista editada a Alberto Rebaza Torres —abogado, coleccionista y presidente del consejo directivo del MALI, además de expresidente del Comité de Adquisiciones de Arte Contemporáneo—, conducida por Carlos Zevallos Trigoso en octubre de 2023. Rebaza narra el origen de su coleccionismo a fines de los noventa, orientado inicial y deliberadamente al arte peruano contemporáneo y luego extendido a lo latinoamericano, bajo la convicción de una «misión»: que el coleccionismo local funcione como primera plataforma de desarrollo para los artistas. Ubica en 2006 la formación del CAAC como factor de cohesión de un grupo de coleccionistas peruanos que ganó visibilidad en ferias regionales e internacionales (ArteBA, ARTBO, Zona Maco, Art Basel). El testimonio articula una teoría del coleccionismo como «proselitismo del arte» que, con el tiempo, debilita la sensación de propiedad y migra hacia la filantropía y el fortalecimiento institucional, ante la ausencia del Estado. Distingue el potencial «colectivo» del coleccionista frente al potencial «de a uno» del galerista, y enfatiza la complementariedad de roles (galerías, ferias, curadores, residencias) en una carrera artística sin hitos claros. Reivindica su Residencia de Al Lado (con Ginette Fernández) y menciona a otros agentes (Hochschild-MAC, Verme-MALI, Marsano-ARTUS, Mulder, Barreda). Sobre su criterio personal, prioriza la tríada contenido, inteligencia y estética, y diferencia expresamente su línea de coleccionismo de la línea curatorial del MALI —más volcada a violencia, territorio, género e historia, próxima al Reina Sofía—. El documento es fuente clave para analizar la perspectiva del coleccionismo y la filantropía en la institucionalización del arte contemporáneo peruano.</t>
         </is>
       </c>
     </row>
@@ -1150,27 +1150,27 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Villacorta, Jorge - 2026-05-06.transcripcion.md</t>
+          <t>Entrevista - Tokeshi, Eduardo - sin fecha.transcripcion.md</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>años 1970-2026 (énfasis en el arte crítico de los 80 a los 2020)</t>
+          <t>1980-2002</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Entrevista (transcripción sin refinar), 06-05-2026</t>
+          <t>Entrevista, s/f</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Andreas Huyssen; Mirko Lauer; Herbert Rodríguez; Hans Haacke; Elena Tejada; Giuliana Borea; Luis Lama; Sharon Lerner; Isaac Ernesto; MALI; Bienal de Lima; E.P.S. Huayco</t>
+          <t>Eduardo Tokeshi; Carlos Zevallos (entrevistador); PUCP; Gustavo Buntinx; Luis Lama; E.P.S. Huayco; Herbert Rodríguez; Bienal de Lima; Emilio Rodríguez Larraín; Jorge Eduardo Eielson; Luis Camnitzer; Óscar Muñoz</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Extensa entrevista al curador y crítico Jorge Villacorta conducida por un investigador que prepara una tesis sobre la institucionalización del arte crítico en el Perú. Villacorta reconstruye la genealogía personal de su noción de arte crítico, armada sin bibliografía sistemática a partir de lecturas dispersas (Huyssen, Buchloh, Osborne, Greil Marcus), del Dadá y el surrealismo vistos en 1972 en el Museo de Arte Italiano, del punk británico y del constructivismo soviético. Sostiene que lo crítico no es categoría académica sino que se construye en la brega, en las luchas simbólicas por derechos, y prefiere hablar de criticidad más que de arte crítico. El diálogo interroga cómo la alternatividad disidente de los años noventa ingresó al museo y devino mandato para artistas jóvenes, articulándose con el vocabulario institucional global de lo decolonial, el género y lo queer. Villacorta introduce la tesis de que en Lima el arte existe fuera de una esfera pública dinamitada, contrasta la consolidación del arte contemporáneo en la Bienal de Trujillo (1987) frente a la Bienal de Lima (1997), y analiza la crítica institucional ausente (Haacke, Hito Steyerl, Andrea Fraser). Comenta casos peruanos: la performance de Elena Tejada, el DNI gigante de Camposano, obras de Flavia Gandolfo, Javi Vargas, Pierina Márquez, la censura a Herbert Rodríguez y Juan Dávila, y el concepto foucaultiano de parresía aplicado a Eduardo Villanes e Isaac Ernesto. Reflexiona además sobre el tutelaje del curador, la lógica de proyecto, el statement y la ansiedad teórica en la formación artística universitaria, y la polémica de Luis Lama contra su curaduría del premio ICPNA.</t>
+          <t>Entrevista al artista Eduardo Tokeshi (n. 1960), conducida por Carlos Zevallos, que reconstruye su formación y la génesis de su obra más reconocida en el contexto de la violencia política peruana. Tokeshi relata su tránsito de la arquitectura a la especialidad de pintura en la PUCP hacia 1983, dentro de la clásica división entre la Católica (abstracción) y Bellas Artes (figuración), y su desmarque del canon al incorporar recortes periodísticos, objetos y materiales no pictóricos. Sitúa en 1985 la primera «Bandera» —cosida, rellena, tensada—, realizada por pulsión antes que como gesto deliberadamente contemporáneo, que inaugura una serie sostenida hasta 2001-2002 como sublimación de la violencia, el duelo y la reconstrucción de la nación. El testimonio historiza el surgimiento de lo contemporáneo local: la muestra «Algo va a pasar» (1987) organizada por Gustavo Buntinx, la Bienal de Trujillo (1987), las Bienales de Lima de los noventa y la labor de Luis Lama trayendo a Camnitzer y Óscar Muñoz. Analiza la profesionalización del campo en los noventa (idea de «proyecto», statements, portafolios, cambios de currícula), el desfase o «refracción» respecto de los centros internacionales (São Paulo, León) y la posterior consolidación de la figura del curador. Contrapone su disidencia formativa —hacer lo deseado siempre que pudiera sustentarlo— a la incorporación curricular del perfil «crítico» como expectativa. Cierra describiendo el proceso material de «Bandera VIII», con bolsas de transfusión llenas de falsa sangre y sal (símbolo de la saladera), asociada a su pertenencia a un club RH negativo, como emblema de una patria en cuidados intensivos.</t>
         </is>
       </c>
     </row>
@@ -1182,27 +1182,27 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Villacorta, Jorge - 2026-06-08.transcripcion.md</t>
+          <t>Entrevista - Villacorta, Jorge - 2026-05-06.transcripcion.md</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>años 1960-2026 (con foco en 1997-2001 y el arte crítico de los 80)</t>
+          <t>años 1970-2026 (énfasis en el arte crítico de los 80 a los 2020)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Entrevista (transcripción sin refinar), 08-06-2026</t>
+          <t>Entrevista (transcripción sin refinar), 06-05-2026</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Mirko Lauer; Juan Acha; Emilio Adolfo Westphalen (Cisneros/Szyszlo); Giuliana Borea; Gerardo Chávez; Sandra Gamarra; Sharon Lerner; Giselle Ordaz; Jacques Peignet; MALI; Alianza Francesa; Fundación Wiese; Pasaporte para un Artista</t>
+          <t>Jorge Villacorta; Andreas Huyssen; Mirko Lauer; Herbert Rodríguez; Hans Haacke; Elena Tejada; Giuliana Borea; Luis Lama; Sharon Lerner; Isaac Ernesto; MALI; Bienal de Lima; E.P.S. Huayco</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Segunda sesión de la entrevista a Jorge Villacorta, centrada en el origen de la crítica de arte peruana, el coleccionismo y la génesis del concurso Pasaporte para un Artista. Villacorta sitúa el nacimiento del arte crítico local en la tensión de los años setenta-ochenta entre críticos y artistas: el volante de Mirko Lauer para E.P.S. Huayco en Galería Forum, la polémica de Ortiz de Ceballos sobre Rafael Hastings y la respuesta de Szyszlo a sus críticos. Formula la hipótesis, que juzga irónica, de que la noción de arte crítico quedó instalada como sentido común justo cuando ya casi no hay críticos activos. Discute críticamente la periodización y los veinte conceptos que Giuliana Borea propone para el paso del arte moderno al contemporáneo, señalando que su libro mira la escena limeña por una ventana demasiado estrecha e ignora las motivaciones del coleccionismo. Caracteriza al coleccionista peruano como desapegado, no obsesivo y guiado por la decoración, contrastándolo con los mecenazgos brasileño y mexicano; cita el caso dramático del retorno de Gerardo Chávez y la 'nacionalización' española de Sandra Gamarra. Analiza la precariedad estructural de las instituciones (MALI, ICPNA), su hermetismo y estructura de comités, y aplica la lectura reparativa de Sedgwick frente a la paranoica. La parte más extensa reconstruye con detalle la creación de Pasaporte para un Artista (1997-1998) en el marco de la política cultural francesa, la Embajada, Mazzoni y Peignet, y las experiencias de los primeros ganadores (Bedoya, Fito Espinosa, Elena Tejada, Bendayán).</t>
+          <t>Extensa entrevista al curador y crítico Jorge Villacorta conducida por un investigador que prepara una tesis sobre la institucionalización del arte crítico en el Perú. Villacorta reconstruye la genealogía personal de su noción de arte crítico, armada sin bibliografía sistemática a partir de lecturas dispersas (Huyssen, Buchloh, Osborne, Greil Marcus), del Dadá y el surrealismo vistos en 1972 en el Museo de Arte Italiano, del punk británico y del constructivismo soviético. Sostiene que lo crítico no es categoría académica sino que se construye en la brega, en las luchas simbólicas por derechos, y prefiere hablar de criticidad más que de arte crítico. El diálogo interroga cómo la alternatividad disidente de los años noventa ingresó al museo y devino mandato para artistas jóvenes, articulándose con el vocabulario institucional global de lo decolonial, el género y lo queer. Villacorta introduce la tesis de que en Lima el arte existe fuera de una esfera pública dinamitada, contrasta la consolidación del arte contemporáneo en la Bienal de Trujillo (1987) frente a la Bienal de Lima (1997), y analiza la crítica institucional ausente (Haacke, Hito Steyerl, Andrea Fraser). Comenta casos peruanos: la performance de Elena Tejada, el DNI gigante de Camposano, obras de Flavia Gandolfo, Javi Vargas, Pierina Márquez, la censura a Herbert Rodríguez y Juan Dávila, y el concepto foucaultiano de parresía aplicado a Eduardo Villanes e Isaac Ernesto. Reflexiona además sobre el tutelaje del curador, la lógica de proyecto, el statement y la ansiedad teórica en la formación artística universitaria, y la polémica de Luis Lama contra su curaduría del premio ICPNA.</t>
         </is>
       </c>
     </row>
@@ -1214,27 +1214,27 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Flynn, Iñigo Clavo, Lemos y Portocarrero - Introduction. Artistic practice and the unmaking of coloniality (2026) [Unmaking to Make].md</t>
+          <t>Entrevista - Villacorta, Jorge - 2026-06-08.transcripcion.md</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>1990-2024 (giro decolonial contemporáneo, con referencia al legado colonial de 500 años)</t>
+          <t>años 1960-2026 (con foco en 1997-2001 y el arte crítico de los 80)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Introducción de libro académico (volumen editado), 2026</t>
+          <t>Entrevista (transcripción sin refinar), 08-06-2026</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Alex Ungprateeb Flynn; María Iñigo Clavo; Beatriz Lemos; Florencia Portocarrero; Sandra Gamarra; Cildo Meireles; Walter Mignolo; Aníbal Quijano; Silvia Rivera Cusicanqui; Grupo Modernidad/Colonialidad; MACBA; Bienal de Venecia</t>
+          <t>Jorge Villacorta; Mirko Lauer; Juan Acha; Emilio Adolfo Westphalen (Cisneros/Szyszlo); Giuliana Borea; Gerardo Chávez; Sandra Gamarra; Sharon Lerner; Giselle Ordaz; Jacques Peignet; MALI; Alianza Francesa; Fundación Wiese; Pasaporte para un Artista</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Introducción al volumen colectivo 'Unmaking to Make', que reorienta hacia América Latina el horizonte teórico de la práctica artística frente a la colonialidad. Los cuatro editores parten de la constatación de que el trabajo 'descolonizador' se ha vuelto norma institucional en el arte contemporáneo del Norte global, mera casilla a marcar, ilustrando cómo lo que fue posición periférica y experimental deviene marco hegemónico (ejemplificado con los bicentenarios latinoamericanos, la exposición 'Buen Gobierno' de Sandra Gamarra en Madrid, el simposio del MACBA, el informe Sarr-Savoy y la Bienal de Venecia 'Foreigners Everywhere'). Su tesis central es que la práctica artística no puede reducirse a hacer visibles teorías producidas por la academia: posee un potencial generativo y especulativo propio para imaginar y proponer mundos, situándose en relación de igualdad y no de subordinación respecto al trabajo académico. El texto revisa críticamente el corpus de la teoría decolonial del Grupo Modernidad/Colonialidad (Mignolo, Quijano, Grosfoguel, Escobar, Dussel, Lugones, Maldonado-Torres), sus diferencias con el poscolonialismo anglófono y las objeciones que ha recibido —de Rivera Cusicanqui, Aura Cumes, Adusei-Poku— por su elitismo, su tendencia a subsumir el pensamiento feminista negro y a apropiarse post hoc de autores. Frente a ello, los editores privilegian epistemologías situadas y la noción de pluriverso (de la Cadena, Blaser), conceptos como amefricanidade y contra-colonialismo, y una metodología curatorial y editorial atenta a la remuneración justa, la traducción y la asimetría de poder. Anuncian cuatro ejes: contragenealogías, instituciones, descolonización del lenguaje y futuros, abriendo con la obra 'Cruzeiro do Sul' de Cildo Meireles.</t>
+          <t>Segunda sesión de la entrevista a Jorge Villacorta, centrada en el origen de la crítica de arte peruana, el coleccionismo y la génesis del concurso Pasaporte para un Artista. Villacorta sitúa el nacimiento del arte crítico local en la tensión de los años setenta-ochenta entre críticos y artistas: el volante de Mirko Lauer para E.P.S. Huayco en Galería Forum, la polémica de Ortiz de Ceballos sobre Rafael Hastings y la respuesta de Szyszlo a sus críticos. Formula la hipótesis, que juzga irónica, de que la noción de arte crítico quedó instalada como sentido común justo cuando ya casi no hay críticos activos. Discute críticamente la periodización y los veinte conceptos que Giuliana Borea propone para el paso del arte moderno al contemporáneo, señalando que su libro mira la escena limeña por una ventana demasiado estrecha e ignora las motivaciones del coleccionismo. Caracteriza al coleccionista peruano como desapegado, no obsesivo y guiado por la decoración, contrastándolo con los mecenazgos brasileño y mexicano; cita el caso dramático del retorno de Gerardo Chávez y la 'nacionalización' española de Sandra Gamarra. Analiza la precariedad estructural de las instituciones (MALI, ICPNA), su hermetismo y estructura de comités, y aplica la lectura reparativa de Sedgwick frente a la paranoica. La parte más extensa reconstruye con detalle la creación de Pasaporte para un Artista (1997-1998) en el marco de la política cultural francesa, la Embajada, Mazzoni y Peignet, y las experiencias de los primeros ganadores (Bedoya, Fito Espinosa, Elena Tejada, Bendayán).</t>
         </is>
       </c>
     </row>
@@ -1246,27 +1246,27 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Gamboa - Fuego cruzado en la Bienal de Arte de Lima.md</t>
+          <t>Flynn, Iñigo Clavo, Lemos y Portocarrero - Introduction. Artistic practice and the unmaking of coloniality (2026) [Unmaking to Make].md</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>1997 (I Bienal de Arte de Lima)</t>
+          <t>1990-2024 (giro decolonial contemporáneo, con referencia al legado colonial de 500 años)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Artículo periodístico / crónica de revista, c. 1997</t>
+          <t>Introducción de libro académico (volumen editado), 2026</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Jeremías Gamboa; Luis Lama; Raquel Tibol; Néstor García Canclini; Llilian Llanés; Aracy Amaral; Bélgica Rodríguez; Edward Sullivan; Alberto Andrade; Luz María Bedoya; Natalia Iguíñiz; Centro de Artes Visuales de Lima</t>
+          <t>Alex Ungprateeb Flynn; María Iñigo Clavo; Beatriz Lemos; Florencia Portocarrero; Sandra Gamarra; Cildo Meireles; Walter Mignolo; Aníbal Quijano; Silvia Rivera Cusicanqui; Grupo Modernidad/Colonialidad; MACBA; Bienal de Venecia</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Crónica periodística de Jeremías Gamboa sobre la polémica desatada en la I Bienal de Arte de Lima (1997), organizada por Luis Lama con una inversión cercana al millón de dólares, más de 150 expositores y casi un millón y medio de visitantes en el centro histórico. El texto reconstruye el 'fuego cruzado' provocado por la crítica mexicana Raquel Tibol, quien en las mesas de conversación y luego en la revista Proceso denunció la falta de reflexión y rigor del evento y su desbalance grotesco: 129 peruanos frente a 33 extranjeros, lo que convertía la muestra en un festival de plástica peruana antes que en una bienal iberoamericana. Gamboa rastrea el origen del problema en la composición excesivamente numerosa y heterogénea del comité de selección —cuatro escuelas, trece galerías y ocho críticos, entre ellos Castrillón, Lauer, Majluf, Wuffarden y el propio Villacorta— cuyo criterio 'democrático' permitió que cualquiera con un solo voto expusiera, con proclividad de los galeristas hacia sus propios artistas. Contrasta este modelo con la depuración conceptual de la Bienal de La Habana (Llilian Llanés) y con la ausencia de un concepto integrador eficaz, señalando que la 'pluralidad cultural' figuraba en las bases pero pocos la advertían, salvo García Canclini. El artículo recoge además elogios internacionales al trabajo de Luz María Bedoya y Natalia Iguíñiz, y un recuadro dedicado al debate paralelo sobre la existencia o no de un 'arte latinoamericano', con posturas encontradas de Lama y Bélgica Rodríguez frente a García Canclini y Edward Sullivan.</t>
+          <t>Introducción al volumen colectivo 'Unmaking to Make', que reorienta hacia América Latina el horizonte teórico de la práctica artística frente a la colonialidad. Los cuatro editores parten de la constatación de que el trabajo 'descolonizador' se ha vuelto norma institucional en el arte contemporáneo del Norte global, mera casilla a marcar, ilustrando cómo lo que fue posición periférica y experimental deviene marco hegemónico (ejemplificado con los bicentenarios latinoamericanos, la exposición 'Buen Gobierno' de Sandra Gamarra en Madrid, el simposio del MACBA, el informe Sarr-Savoy y la Bienal de Venecia 'Foreigners Everywhere'). Su tesis central es que la práctica artística no puede reducirse a hacer visibles teorías producidas por la academia: posee un potencial generativo y especulativo propio para imaginar y proponer mundos, situándose en relación de igualdad y no de subordinación respecto al trabajo académico. El texto revisa críticamente el corpus de la teoría decolonial del Grupo Modernidad/Colonialidad (Mignolo, Quijano, Grosfoguel, Escobar, Dussel, Lugones, Maldonado-Torres), sus diferencias con el poscolonialismo anglófono y las objeciones que ha recibido —de Rivera Cusicanqui, Aura Cumes, Adusei-Poku— por su elitismo, su tendencia a subsumir el pensamiento feminista negro y a apropiarse post hoc de autores. Frente a ello, los editores privilegian epistemologías situadas y la noción de pluriverso (de la Cadena, Blaser), conceptos como amefricanidade y contra-colonialismo, y una metodología curatorial y editorial atenta a la remuneración justa, la traducción y la asimetría de poder. Anuncian cuatro ejes: contragenealogías, instituciones, descolonización del lenguaje y futuros, abriendo con la obra 'Cruzeiro do Sul' de Cildo Meireles.</t>
         </is>
       </c>
     </row>
@@ -1278,27 +1278,27 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Germaná y Portocarrero - The «Indigenous turn» and the rise of Amazonian art. Insights from the seminal work of the SHRA (2026) [Unmaking to Make, cap. 8].md</t>
+          <t>Gamboa - Fuego cruzado en la Bienal de Arte de Lima.md</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>1966-2025 (con foco en el 'giro indígena' de los años 90 en adelante)</t>
+          <t>1997 (I Bienal de Arte de Lima)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro académico, 2026</t>
+          <t>Artículo periodístico / crónica de revista, c. 1997</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Gabriela Germaná; Florencia Portocarrero; Pablo Macera; María Belén Soria; Gredna Landolt; Víctor Churay; Elena Valera; Roldán Pinedo; Lastenia Canayo; Sara Flores; Mirko Lauer; Natalia Majluf; SHRA (UNMSM); Fundación Telefónica; MALI; MASP</t>
+          <t>Jeremías Gamboa; Luis Lama; Raquel Tibol; Néstor García Canclini; Llilian Llanés; Aracy Amaral; Bélgica Rodríguez; Edward Sullivan; Alberto Andrade; Luz María Bedoya; Natalia Iguíñiz; Centro de Artes Visuales de Lima</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Capítulo que examina el 'giro indígena' global y el ascenso del arte amazónico en el Perú a partir de la labor seminal del Seminario de Historia Rural Andina (SHRA), instituto de la UNMSM fundado por Pablo Macera en 1966. Germaná y Portocarrero parten de la exclusión histórica de los creadores indígenas de la historia del arte oficial, relegados a la categoría de artesanía por una lógica racializada que niega la posibilidad de que algo sea simultáneamente arte e indígena. Apoyándose en 'Lo andino en el arte peruano' de Mirko Lauer (1980), describen el campo artístico estratificado en tres universos —alto arte, arte popular y arte prehispánico— y sus rupturas: el indigenismo de los años veinte, la redefinición política de la artesanía bajo el gobierno de Velasco (premio a Joaquín López Antay, 1975) y el giro indígena de los noventa ligado al multiculturalismo neoliberal. El eje del texto es la metodología colaborativa del SHRA, que desde 1997 —con Macera y María Belén Soria, inspirados por la experiencia de Gredna Landolt en Formabiap— trabajó con pintores amazónicos autodidactas (Víctor Churay, Elena Valera, Roldán Pinedo, Lastenia Canayo, Enrique Casanto) usando la ecuación pintura-escritura para recuperar la memoria oral. Destacan que el seminario reconoció la autoría individual, pagó por el trabajo y operó como 'zona de contacto' descolonial. Las autoras concluyen que este método, de raíz etnográfica, consolidó la pintura figurativa como criterio de legitimación —limitando otros medios y el kené—, y analizan las contradicciones de la inserción del arte indígena en el circuito global (Sara Flores en el MALI, la Bienal de Venecia de Pedrosa, testimonios de Yahuarcani y Mombaça).</t>
+          <t>Crónica periodística de Jeremías Gamboa sobre la polémica desatada en la I Bienal de Arte de Lima (1997), organizada por Luis Lama con una inversión cercana al millón de dólares, más de 150 expositores y casi un millón y medio de visitantes en el centro histórico. El texto reconstruye el 'fuego cruzado' provocado por la crítica mexicana Raquel Tibol, quien en las mesas de conversación y luego en la revista Proceso denunció la falta de reflexión y rigor del evento y su desbalance grotesco: 129 peruanos frente a 33 extranjeros, lo que convertía la muestra en un festival de plástica peruana antes que en una bienal iberoamericana. Gamboa rastrea el origen del problema en la composición excesivamente numerosa y heterogénea del comité de selección —cuatro escuelas, trece galerías y ocho críticos, entre ellos Castrillón, Lauer, Majluf, Wuffarden y el propio Villacorta— cuyo criterio 'democrático' permitió que cualquiera con un solo voto expusiera, con proclividad de los galeristas hacia sus propios artistas. Contrasta este modelo con la depuración conceptual de la Bienal de La Habana (Llilian Llanés) y con la ausencia de un concepto integrador eficaz, señalando que la 'pluralidad cultural' figuraba en las bases pero pocos la advertían, salvo García Canclini. El artículo recoge además elogios internacionales al trabajo de Luz María Bedoya y Natalia Iguíñiz, y un recuadro dedicado al debate paralelo sobre la existencia o no de un 'arte latinoamericano', con posturas encontradas de Lama y Bélgica Rodríguez frente a García Canclini y Edward Sullivan.</t>
         </is>
       </c>
     </row>
@@ -1310,27 +1310,27 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Hernández Calvo y Villacorta - Franquicias imaginarias. Las opciones estéticas en las artes plásticas en el Perú de fin de siglo (2002) [OCR A].md</t>
+          <t>Germaná y Portocarrero - The «Indigenous turn» and the rise of Amazonian art. Insights from the seminal work of the SHRA (2026) [Unmaking to Make, cap. 8].md</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>1950-2000 (segunda mitad del siglo XX, con énfasis en los años 90 y fin de siglo)</t>
+          <t>1966-2025 (con foco en el 'giro indígena' de los años 90 en adelante)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Libro / ensayo académico (Fondo Editorial PUCP), 2002</t>
+          <t>Capítulo de libro académico, 2026</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Max Hernández Calvo; Jorge Villacorta; Mirko Lauer; Fernando de Szyszlo; Luis Miró Quesada; Juan Acha; Ricardo Grau; Agrupación Espacio; IAC; Colectivo Sociedad Civil; Eduardo Villanes; Ricardo Wiesse; Alfredo Márquez; PUCP</t>
+          <t>Gabriela Germaná; Florencia Portocarrero; Pablo Macera; María Belén Soria; Gredna Landolt; Víctor Churay; Elena Valera; Roldán Pinedo; Lastenia Canayo; Sara Flores; Mirko Lauer; Natalia Majluf; SHRA (UNMSM); Fundación Telefónica; MALI; MASP</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Libro de Max Hernández Calvo y Jorge Villacorta que ofrece una lectura crítica y panorámica —no meramente cronológica— de las opciones estéticas en las artes plásticas peruanas de la segunda mitad del siglo XX, atendiendo especialmente a Lima y al fin de siglo. La tesis de fondo es la precariedad y fragmentación del sistema artístico local (ausencia de un museo de arte contemporáneo, mercado incipiente, divorcio entre producción y recepción crítica, escisión ficticia entre arte y comercio) que impide comprender lo artístico como sistema. El texto reconstruye la instauración del modelo moderno-tardío: la llegada de la abstracción con Szyszlo (1949), la Agrupación Espacio, Luis Miró Quesada y el IAC como brazos de un proyecto vinculado a la burguesía industrial y urbanizadora, el desplazamiento del indigenismo en crisis y la posterior 'abstracción de reminiscencia precolombina' como símbolo ficticio de integración nacional que soslaya las realidades sociales del país migrante. Analiza luego la vanguardia de los sesenta (Pop y Op, Arte Nuevo, Juan Acha, Teresa Burga), la institucionalización postideológica, las esferas subsidiarias y escenas alternativas, la introspección y el juego, la globalización y 'lo social desquerenciado'. Un capítulo central, 'En la estela de la política', documenta el auge del arte políticamente motivado en la crisis del fujimorato tardío: Runcie Tanaka, Miguel Cordero, Ricardo Wiesse (Cantuta), Eduardo Villanes ('Gloria Evaporada'), Emilio Santisteban, el Colectivo Sociedad Civil ('Lava la bandera') y Perú Fábrica, con su especulación sobre los espacios público y privado. Cierra advirtiendo que la postmodernidad no se consolida como marco crítico por la misma precariedad institucional.</t>
+          <t>Capítulo que examina el 'giro indígena' global y el ascenso del arte amazónico en el Perú a partir de la labor seminal del Seminario de Historia Rural Andina (SHRA), instituto de la UNMSM fundado por Pablo Macera en 1966. Germaná y Portocarrero parten de la exclusión histórica de los creadores indígenas de la historia del arte oficial, relegados a la categoría de artesanía por una lógica racializada que niega la posibilidad de que algo sea simultáneamente arte e indígena. Apoyándose en 'Lo andino en el arte peruano' de Mirko Lauer (1980), describen el campo artístico estratificado en tres universos —alto arte, arte popular y arte prehispánico— y sus rupturas: el indigenismo de los años veinte, la redefinición política de la artesanía bajo el gobierno de Velasco (premio a Joaquín López Antay, 1975) y el giro indígena de los noventa ligado al multiculturalismo neoliberal. El eje del texto es la metodología colaborativa del SHRA, que desde 1997 —con Macera y María Belén Soria, inspirados por la experiencia de Gredna Landolt en Formabiap— trabajó con pintores amazónicos autodidactas (Víctor Churay, Elena Valera, Roldán Pinedo, Lastenia Canayo, Enrique Casanto) usando la ecuación pintura-escritura para recuperar la memoria oral. Destacan que el seminario reconoció la autoría individual, pagó por el trabajo y operó como 'zona de contacto' descolonial. Las autoras concluyen que este método, de raíz etnográfica, consolidó la pintura figurativa como criterio de legitimación —limitando otros medios y el kené—, y analizan las contradicciones de la inserción del arte indígena en el circuito global (Sara Flores en el MALI, la Bienal de Venecia de Pedrosa, testimonios de Yahuarcani y Mombaça).</t>
         </is>
       </c>
     </row>
@@ -1342,27 +1342,27 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Hernández Calvo y Villacorta - Franquicias imaginarias. Las opciones estéticas en las artes plásticas en el Perú de fin de siglo (2002) [OCR B].md</t>
+          <t>Hernández Calvo y Villacorta - Franquicias imaginarias. Las opciones estéticas en las artes plásticas en el Perú de fin de siglo (2002) [OCR A].md</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>1950-2001 (con énfasis en los años 70, 80 y 90)</t>
+          <t>1950-2000 (segunda mitad del siglo XX, con énfasis en los años 90 y fin de siglo)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Libro/ensayo crítico (OCR), 2002</t>
+          <t>Libro / ensayo académico (Fondo Editorial PUCP), 2002</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Max Hernández Calvo; Jorge Villacorta; Fondo Editorial PUCP; Fernando de Szyszlo; Ricardo Grau; Juan Acha; Mirko Lauer; Cristina Planas; Milagros de la Torre; Carlos Runcie Tanaka; Ricardo Wiesse; Bienal de Lima / ICPNA</t>
+          <t>Max Hernández Calvo; Jorge Villacorta; Mirko Lauer; Fernando de Szyszlo; Luis Miró Quesada; Juan Acha; Ricardo Grau; Agrupación Espacio; IAC; Colectivo Sociedad Civil; Eduardo Villanes; Ricardo Wiesse; Alfredo Márquez; PUCP</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Ensayo panorámico que diagnostica el desarrollo de las artes visuales peruanas desde mediados del siglo XX hasta el cambio de milenio, sosteniendo que la reflexión crítica local ha permanecido en un vacío de casi tres décadas pese a la creciente diversificación de opciones estéticas, soportes y medios. Los autores conciben el arte como sistema y práctica social, y denuncian la precariedad institucional peruana: la ausencia de un museo de arte contemporáneo, un mercado incipiente, la escisión ficticia entre arte y comercio y una formación que divorcia producción manual de reflexión conceptual. El texto reconstruye una genealogía: la instauración dominante del modelo moderno-tardío y la abstracción (Szyszlo, Grau, Espacio, Miró Quesada) como desplazamiento programático del indigenismo hacia una base social burguesa e industrial; el frenesí pop y las vanguardias de los sesenta; la reforma velasquista y sus tensiones entre lo popular (artesanía) y lo culto. Avanza luego hacia la institucionalización postideológica, las esferas alternativas y la globalización "C.O.D.", cerrando con el retorno de lo social y lo político a fines de los noventa. Marco conceptual apoyado en Foster, Greenberg, García Canclini y sociología de la cultura (esfera pública, movimientos sociales). Analiza obras como La wuawua de Planas sobre Abimael Guzmán, las fotografías forenses de Milagros de la Torre, Uchuraccay, el memorial cantuta de Wiesse en Cieneguilla, los ensamblajes de Miguel Cordero sobre Barrios Altos y La Cantuta, y a Runcie Tanaka. Su aporte es ofrecer una lectura orgánica, temática y no meramente cronológica del "fin de siglo" limeño, situando lo estético como franquicia imaginativa para la comunicación ciudadana.</t>
+          <t>Libro de Max Hernández Calvo y Jorge Villacorta que ofrece una lectura crítica y panorámica —no meramente cronológica— de las opciones estéticas en las artes plásticas peruanas de la segunda mitad del siglo XX, atendiendo especialmente a Lima y al fin de siglo. La tesis de fondo es la precariedad y fragmentación del sistema artístico local (ausencia de un museo de arte contemporáneo, mercado incipiente, divorcio entre producción y recepción crítica, escisión ficticia entre arte y comercio) que impide comprender lo artístico como sistema. El texto reconstruye la instauración del modelo moderno-tardío: la llegada de la abstracción con Szyszlo (1949), la Agrupación Espacio, Luis Miró Quesada y el IAC como brazos de un proyecto vinculado a la burguesía industrial y urbanizadora, el desplazamiento del indigenismo en crisis y la posterior 'abstracción de reminiscencia precolombina' como símbolo ficticio de integración nacional que soslaya las realidades sociales del país migrante. Analiza luego la vanguardia de los sesenta (Pop y Op, Arte Nuevo, Juan Acha, Teresa Burga), la institucionalización postideológica, las esferas subsidiarias y escenas alternativas, la introspección y el juego, la globalización y 'lo social desquerenciado'. Un capítulo central, 'En la estela de la política', documenta el auge del arte políticamente motivado en la crisis del fujimorato tardío: Runcie Tanaka, Miguel Cordero, Ricardo Wiesse (Cantuta), Eduardo Villanes ('Gloria Evaporada'), Emilio Santisteban, el Colectivo Sociedad Civil ('Lava la bandera') y Perú Fábrica, con su especulación sobre los espacios público y privado. Cierra advirtiendo que la postmodernidad no se consolida como marco crítico por la misma precariedad institucional.</t>
         </is>
       </c>
     </row>
@@ -1374,27 +1374,27 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>ICAA-1138109.pdf</t>
+          <t>Hernández Calvo y Villacorta - Franquicias imaginarias. Las opciones estéticas en las artes plásticas en el Perú de fin de siglo (2002) [OCR B].md</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Debate del nacionalismo e indigenismo en la pintura peruana, c. décadas de 1940-1950</t>
+          <t>1950-2001 (con énfasis en los años 70, 80 y 90)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Artículo de prensa (Suplemento Dominical de El Comercio, Lima), c. 1957 (s/f exacta); digitalizado por ICAA-MFAH</t>
+          <t>Libro/ensayo crítico (OCR), 2002</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>J. Nahuaca (seudónimo); José Sabogal; Francisco Laso; Fernando de Szyszlo; Ricardo Grau; Fernando de Villegas / Villegas; Juan Manuel Ugarte Eléspuru; Pancho Fierro; César Vallejo; Inca Garcilaso; El Comercio (Suplemento Dominical); International Center for the Arts of the Americas (ICAA-MFAH)</t>
+          <t>Max Hernández Calvo; Jorge Villacorta; Fondo Editorial PUCP; Fernando de Szyszlo; Ricardo Grau; Juan Acha; Mirko Lauer; Cristina Planas; Milagros de la Torre; Carlos Runcie Tanaka; Ricardo Wiesse; Bienal de Lima / ICPNA</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Artículo "Conscripción peruana la pintura", firmado con el seudónimo J. Nahuaca y publicado en el Suplemento Dominical de El Comercio de Lima (hacia finales de los años cincuenta, a juzgar por las referencias contextuales), conservado en el archivo digital ICAA del Museum of Fine Arts, Houston. La tesis sostiene que la pintura peruana sufre la presión de fuerzas nacionalistas que operan "desde afuera" como verdaderas conscripciones que le imponen un destino en nombre de la peruanidad, esterilizando sus energías estéticas endógenas. El autor distingue tres conscripciones: la político-social, que reduce la pintura a panfleto, confesión o acto de fe redentor y la torna inoperante; la iconográfica, la más antigua, que exige amor a lo nacional mediante la anécdota histórica y costumbrista (Merino, Montero, Castillo) y culmina en el indigenismo de Sabogal -cuya nacionalización amorosa de la iconografía "termina siendo una montonera"-; y la espiritual, con dos modalidades: un humanismo telúrico o "vallejismo" pictórico (Laso, Ugarte Eléspuru) y una búsqueda del eslabón formal con el pasado prehispánico y colonial. El marco conceptual moviliza el determinismo de Taine, la estilización del arte preincaico (Chavín, Nazca, Paracas, Moche), la escuela cuzqueña y la continuidad estética que uniría Garcilaso con Vallejo. Nahuaca reivindica la autonomía "insobornable" de la pintura frente a las presiones nacionalizadoras, valorando en Dávila, Grau, Szyszlo y Villegas tanto el entronque con el pasado como su vigencia pictórica. El aporte es un alegato antiindigenista y formalista que reclama la sublimación estética por encima de la subordinación ideológica, en pleno debate sobre la identidad del arte peruano.</t>
+          <t>Ensayo panorámico que diagnostica el desarrollo de las artes visuales peruanas desde mediados del siglo XX hasta el cambio de milenio, sosteniendo que la reflexión crítica local ha permanecido en un vacío de casi tres décadas pese a la creciente diversificación de opciones estéticas, soportes y medios. Los autores conciben el arte como sistema y práctica social, y denuncian la precariedad institucional peruana: la ausencia de un museo de arte contemporáneo, un mercado incipiente, la escisión ficticia entre arte y comercio y una formación que divorcia producción manual de reflexión conceptual. El texto reconstruye una genealogía: la instauración dominante del modelo moderno-tardío y la abstracción (Szyszlo, Grau, Espacio, Miró Quesada) como desplazamiento programático del indigenismo hacia una base social burguesa e industrial; el frenesí pop y las vanguardias de los sesenta; la reforma velasquista y sus tensiones entre lo popular (artesanía) y lo culto. Avanza luego hacia la institucionalización postideológica, las esferas alternativas y la globalización "C.O.D.", cerrando con el retorno de lo social y lo político a fines de los noventa. Marco conceptual apoyado en Foster, Greenberg, García Canclini y sociología de la cultura (esfera pública, movimientos sociales). Analiza obras como La wuawua de Planas sobre Abimael Guzmán, las fotografías forenses de Milagros de la Torre, Uchuraccay, el memorial cantuta de Wiesse en Cieneguilla, los ensamblajes de Miguel Cordero sobre Barrios Altos y La Cantuta, y a Runcie Tanaka. Su aporte es ofrecer una lectura orgánica, temática y no meramente cronológica del "fin de siglo" limeño, situando lo estético como franquicia imaginativa para la comunicación ciudadana.</t>
         </is>
       </c>
     </row>
@@ -1406,12 +1406,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>ICAA-1272963.pdf</t>
+          <t>ICAA-1138109.pdf</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Debate sobre arte, doctrina y nacionalismo; revisión de las revoluciones cristiana, francesa, rusa y mexicana; c. décadas de 1940-1950</t>
+          <t>Debate del nacionalismo e indigenismo en la pintura peruana, c. décadas de 1940-1950</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1421,12 +1421,12 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>J. Nahuaca (seudónimo); Moisés Laymito; Gladys Zender; César Vallejo; Wilhelm Worringer; Arnold Hauser; Nicolai Hartmann; Charles Lalo; Jacques-Louis David; Kazimir Malevich; Wassily Kandinsky; Marc Chagall; El Comercio (Suplemento Dominical); ICAA-MFAH</t>
+          <t>J. Nahuaca (seudónimo); José Sabogal; Francisco Laso; Fernando de Szyszlo; Ricardo Grau; Fernando de Villegas / Villegas; Juan Manuel Ugarte Eléspuru; Pancho Fierro; César Vallejo; Inca Garcilaso; El Comercio (Suplemento Dominical); International Center for the Arts of the Americas (ICAA-MFAH)</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Segunda entrega del ensayo de J. Nahuaca, titulada "Ideas doctrinarias y la pintura", publicada en el Suplemento Dominical de El Comercio de Lima (fines de los cincuenta) y archivada en el ICAA-MFAH. Continúa la reflexión sobre las fuerzas que tensionan el arte peruano, distinguiendo entre energías subyacentes -lentas, sentimentales, nacionalizadoras, orientadas a la peruanidad- y fuerzas dinámicas que importan sistemas político-sociales para materializarlos de inmediato, sometiendo el arte a los valores sociales mediante una estética "demagógica y a la vez conservadora". El objeto central es la relación entre pintura e ideas doctrinarias, examinada a través de un recorrido histórico por cuatro revoluciones: la cristiana (que renuncia al arte pagano y desemboca en la iconoclasia), la francesa (que no crea estilo sino que adopta el clasicismo de David, oficializado por Napoleón), la rusa (que tras aliarse con la vanguardia -Malevich, Kandinsky, Chagall- recae en el realismo heroico reaccionario) y la mexicana (nacida sin doctrina, expresiva y muralista, que crea el mito de la revolución cumplida). El marco teórico cita a Worringer, Hauser, Nicolai Hartmann y Charles Lalo, y disuelve la antinomia forma-contenido cara a la estética marxista. Nahuaca argumenta que ninguna revolución ha mejorado ni creado un arte, que este pertenece a individuos y la colectividad solo lo usufructúa, y aboga por "desclasificar" la élite estética -verdadera valoradora- frente al monopolio de las clases dirigentes. Denuncia un "terrorismo en pintura" que exige conciencia social y concluye que el ímpetu nacionalizador peruano ha derivado en un mal menor: la peruanización de la iconografía como fin artístico. Incluye notas sobre el escultor Moisés Laymito y un retrato de Gladys Zender.</t>
+          <t>Artículo "Conscripción peruana la pintura", firmado con el seudónimo J. Nahuaca y publicado en el Suplemento Dominical de El Comercio de Lima (hacia finales de los años cincuenta, a juzgar por las referencias contextuales), conservado en el archivo digital ICAA del Museum of Fine Arts, Houston. La tesis sostiene que la pintura peruana sufre la presión de fuerzas nacionalistas que operan "desde afuera" como verdaderas conscripciones que le imponen un destino en nombre de la peruanidad, esterilizando sus energías estéticas endógenas. El autor distingue tres conscripciones: la político-social, que reduce la pintura a panfleto, confesión o acto de fe redentor y la torna inoperante; la iconográfica, la más antigua, que exige amor a lo nacional mediante la anécdota histórica y costumbrista (Merino, Montero, Castillo) y culmina en el indigenismo de Sabogal -cuya nacionalización amorosa de la iconografía "termina siendo una montonera"-; y la espiritual, con dos modalidades: un humanismo telúrico o "vallejismo" pictórico (Laso, Ugarte Eléspuru) y una búsqueda del eslabón formal con el pasado prehispánico y colonial. El marco conceptual moviliza el determinismo de Taine, la estilización del arte preincaico (Chavín, Nazca, Paracas, Moche), la escuela cuzqueña y la continuidad estética que uniría Garcilaso con Vallejo. Nahuaca reivindica la autonomía "insobornable" de la pintura frente a las presiones nacionalizadoras, valorando en Dávila, Grau, Szyszlo y Villegas tanto el entronque con el pasado como su vigencia pictórica. El aporte es un alegato antiindigenista y formalista que reclama la sublimación estética por encima de la subordinación ideológica, en pleno debate sobre la identidad del arte peruano.</t>
         </is>
       </c>
     </row>
@@ -1438,27 +1438,27 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>ICPNA Catalogo Bellas Artes FINAL.pdf</t>
+          <t>ICAA-1146549.pdf</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>1918-2018</t>
+          <t>«Última década» del s. XX (años 1990; dictadura de Fujimori 1990-2000), con antecedentes desde los 60-80</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de exposición / libro institucional, noviembre de 2018</t>
+          <t>Ensayo de catálogo (muestra «Puntos Cardinales»), noviembre de 2001; digitalizado por ICAA-MFAH (reg. 1146549); OCR muy dañado</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Escuela Nacional Superior Autónoma de Bellas Artes del Perú (ENSABAP); Instituto Cultural Peruano Norteamericano (ICPNA); Max Hernández Calvo; Augusto del Valle Cárdenas; Rocío Corcuera Ríos; Víctor Mejía Ticona; Miguel Sánchez Flores; Luis Carlos Valdez Espinoza; Roberto Hoyle; Municipalidad de Miraflores; E.P.S. Huayco; Grupo Paréntesis</t>
+          <t>Rodrigo Quijano; Fernando Bryce; Iván Esquivel «Plaztikk»; Sandra Gamarra; Gilda Mantilla; Gustavo Buntinx; Mirko Lauer; Augusto del Valle; Juan Javier Salazar; Eduardo Tokeshi; Colectivo Sociedad Civil; ENBA; Museo de Arte de Lima; Bienal de Lima; ICAA-MFAH</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>El volumen documenta 'Un siglo de arte desde la Escuela Nacional', ciclo de cuatro exposiciones organizado en 2018 para el centenario (1918-2018) de la Escuela Nacional Superior Autónoma de Bellas Artes del Perú (ENSABAP), coeditado con el Instituto Cultural Peruano Norteamericano (ICPNA). Bajo la curaduría general de Max Hernández Calvo y Augusto del Valle Cárdenas, con Rocío Corcuera, Víctor Mejía y Miguel Sánchez, el proyecto busca construir memoria institucional y revisar cien años de producción y pedagogía bellasartina, articulándola con la sociedad contemporánea. Las muestras se distribuyeron en cuatro sedes (galerías ICPNA Juan Pardo Heeren y Germán Krüger Espantoso, y salas municipales de Miraflores). 'Bellas Artes: voz y huella de los egresados' (Corcuera) parte de cuarenta entrevistas a egresados de 1951 a 2017 —de Ella Krebs a Andrés Yaques— y una línea de tiempo que vincula formación, testimonio y obra estudiantil. 'Del individuo al ser social' (Sánchez) estudia los colectivos surgidos desde los años setenta (E.P.S. Huayco, Paréntesis, Signo x Signo, C.H.O.L.O., entre otros) como gesto político frente al modelo del artista individual. 'Espacio público' (Mejía) analiza el centro de Lima como insumo estético y campo de intervención. 'Una trayectoria de imágenes' (Hernández Calvo y Del Valle) emplea los géneros académicos —bodegón, paisaje, retrato— para pensar el tránsito del arte moderno al contemporáneo. La tesis transversal cuestiona la narrativa figurativo/abstracto de la modernidad e introduce la pregunta por el ícono, uniendo lo global con las tradiciones locales y artesanales, para otorgar 'carta de ciudadanía' a prácticas invisibilizadas desde una escuela pública.</t>
+          <t>Ensayo de Rodrigo Quijano fechado «Noviembre, 2001», texto del catálogo de la muestra colectiva «Puntos Cardinales» (cuatro artistas: Fernando Bryce, Iván Esquivel «Plaztikk», Sandra Gamarra y Gilda Mantilla). Titulado «¿De qué puntos cardinales hablan? Anotaciones sobre la última década en las artes visuales peruanas», ofrece un balance de los años noventa organizado en doce secciones numeradas. Su hilo es que la década consolidó una orientación del arte contemporáneo local a la vez que se perdió «un norte definido»: la entrada abrupta de la escena al «orden internacional» y a un «mercado simbólico consolidado de la región» tras años de aislamiento, bajo la dictadura de Fujimori (1990-2000). Rastrea el fin de la «modernidad alternativa» anclada en lo popular (con referencias a Lauer y su «Teoría de las Raíces Nacionales» y a Buntinx), la represión de los colectivos jóvenes (el grupo Huayco como paradigma, N.N. «diezmado» y Alfredo Márquez encarcelado bajo falsos cargos de terrorismo) y la «reinstitucionalización» privada (MALI, Centro de Artes Visuales, concursos y bienales auspiciados por el sector privado, Bienal de Lima desde 1997). Analiza en detalle a los cuatro artistas y comenta la crisis de la ENBA (intervenida por la dictadura), los «vladivideos», La Cantuta, Barrios Altos y el «Lava la bandera» del Colectivo Sociedad Civil (2000). Cierra afirmando que «la escena crítica es proporcionalmente precaria e invisible». Fuente primaria sobre la escena limeña de los noventa; digitalizada por el ICAA-MFAH (registro 1146549), con OCR muy dañado.</t>
         </is>
       </c>
     </row>
@@ -1470,27 +1470,27 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Kusunoki y Lerner - Reconsidering the «art museum». Some reflections on the history of the MALI collections (2026) [Unmaking to Make, cap. 5].md</t>
+          <t>ICAA-1272963.pdf</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>1961-2022 (con referencias desde época prehispánica y los años 20)</t>
+          <t>Debate sobre arte, doctrina y nacionalismo; revisión de las revoluciones cristiana, francesa, rusa y mexicana; c. décadas de 1940-1950</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro, 2026</t>
+          <t>Artículo de prensa (Suplemento Dominical de El Comercio, Lima), c. 1957 (s/f exacta); digitalizado por ICAA-MFAH</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Ricardo Kusunoki; Sharon Lerner; Museo de Arte de Lima (MALI); Natalia Majluf; Gabriela Germaná; Gredna Landolt; ADAPS / Piraq Causa; Brus Rubio Churay; José Sabogal; Con/Vida; Matadero Madrid / ARCO; Julieta González</t>
+          <t>J. Nahuaca (seudónimo); Moisés Laymito; Gladys Zender; César Vallejo; Wilhelm Worringer; Arnold Hauser; Nicolai Hartmann; Charles Lalo; Jacques-Louis David; Kazimir Malevich; Wassily Kandinsky; Marc Chagall; El Comercio (Suplemento Dominical); ICAA-MFAH</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Capítulo que reflexiona sobre la historia de las colecciones del Museo de Arte de Lima (MALI) desde su fundación en 1961 para interrogar la propia categoría de "museo de arte". Kusunoki y Lerner parten de la condición fundacional del MALI: nacido tardíamente frente a otros museos latinoamericanos, sin conexión con centros de enseñanza y configurado por el azar de donaciones como la vasta y heterogénea Memoria Prado. Esa amplitud material, argumentan, contenía en estado latente la posibilidad de cuestionar cómo las narrativas nacionales se proyectan sobre el pasado. El eje conceptual es la tensión entre "arte culto" y "arte popular", categoría esta última formulada en los años veinte desde el indigenismo de Sabogal y cargada de una ficción de autenticidad vernácula. El estudio de caso central es la incorporación en 2017 de la serie Piraq Causa —31 tablas de Sarhua de la ADAPS, comisionadas por Peter Gaupp, que narran la violencia de Sendero Luminoso y los Sinchis en Ayacucho—, que complejizó el eje de los "años de violencia" (junto a Taller N.N., Wiesse, Villares) y obligó a reconocer las tablas como práctica intersticial entre lo rural, urbano, tradicional y contemporáneo. La tesis sostiene que integrar tales obras no debe significar instalarlas en el espacio "atemporal" del arte, sino desmantelar la estructura dicotómica de clase y etnia del campo artístico peruano, preservando su carácter ambivalente. Reseña además el eje amazónico (Brus Rubio, 2014-2015), la gestión de Natalia Majluf (1995-2018) y las exposiciones Amazonías, Otras historias posibles (2019) e Imaginarios contemporáneos (2021-2022), proponiendo una política de colección que reconstruya constelaciones históricamente situadas y transformables.</t>
+          <t>Segunda entrega del ensayo de J. Nahuaca, titulada "Ideas doctrinarias y la pintura", publicada en el Suplemento Dominical de El Comercio de Lima (fines de los cincuenta) y archivada en el ICAA-MFAH. Continúa la reflexión sobre las fuerzas que tensionan el arte peruano, distinguiendo entre energías subyacentes -lentas, sentimentales, nacionalizadoras, orientadas a la peruanidad- y fuerzas dinámicas que importan sistemas político-sociales para materializarlos de inmediato, sometiendo el arte a los valores sociales mediante una estética "demagógica y a la vez conservadora". El objeto central es la relación entre pintura e ideas doctrinarias, examinada a través de un recorrido histórico por cuatro revoluciones: la cristiana (que renuncia al arte pagano y desemboca en la iconoclasia), la francesa (que no crea estilo sino que adopta el clasicismo de David, oficializado por Napoleón), la rusa (que tras aliarse con la vanguardia -Malevich, Kandinsky, Chagall- recae en el realismo heroico reaccionario) y la mexicana (nacida sin doctrina, expresiva y muralista, que crea el mito de la revolución cumplida). El marco teórico cita a Worringer, Hauser, Nicolai Hartmann y Charles Lalo, y disuelve la antinomia forma-contenido cara a la estética marxista. Nahuaca argumenta que ninguna revolución ha mejorado ni creado un arte, que este pertenece a individuos y la colectividad solo lo usufructúa, y aboga por "desclasificar" la élite estética -verdadera valoradora- frente al monopolio de las clases dirigentes. Denuncia un "terrorismo en pintura" que exige conciencia social y concluye que el ímpetu nacionalizador peruano ha derivado en un mal menor: la peruanización de la iconografía como fin artístico. Incluye notas sobre el escultor Moisés Laymito y un retrato de Gladys Zender.</t>
         </is>
       </c>
     </row>
@@ -1502,27 +1502,27 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Lauer, Mirko - Arte al paso, Tome uno (1980) [volante Galería Forum, E.P.S. Huayco].md</t>
+          <t>ICPNA Catalogo Bellas Artes FINAL.pdf</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>1980 (exposición Arte al paso, E.P.S. Huayco; contexto de la plástica joven peruana de fin de los años 70)</t>
+          <t>1918-2018</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Volante/panfleto de exposición, mayo de 1980 (Galería Forum, Lima); transcripción manual de fotografía, 2026</t>
+          <t>Catálogo de exposición / libro institucional, noviembre de 2018</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Mirko Lauer (texto); E.P.S. Huayco; María Luy; Francisco Mariotti; Charo Noriega; Juan Javier Salazar; Mariela Zevallos; Guillermo Orbegoso; Roberto Cores; Galería Forum</t>
+          <t>Escuela Nacional Superior Autónoma de Bellas Artes del Perú (ENSABAP); Instituto Cultural Peruano Norteamericano (ICPNA); Max Hernández Calvo; Augusto del Valle Cárdenas; Rocío Corcuera Ríos; Víctor Mejía Ticona; Miguel Sánchez Flores; Luis Carlos Valdez Espinoza; Roberto Hoyle; Municipalidad de Miraflores; E.P.S. Huayco; Grupo Paréntesis</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Volante o panfleto bifronte («Arte al paso» / «Tome uno») escrito por Mirko Lauer para acompañar la exposición homónima del colectivo E.P.S. Huayco en la Galería Forum de Lima (mayo de 1980); el proyecto reúne a María Luy, Francisco Mariotti, Charo Noriega, Juan Javier Salazar y Mariela Zevallos, con fotografías de Guillermo Orbegoso y Roberto Cores. El texto, organizado como una serie de definiciones anafóricas («Arte al paso: …»), es un manifiesto programático del no-objetualismo peruano y del arte crítico. Lauer presenta la obra como una «contestación» que combina serigrafía, detritus industriales, fórmulas teóricas, fotos y «expendio de salchipapas» para sostener que «la realidad del arte es más compleja que la realidad de las 'Bellas Artes'». Articula tres operaciones críticas: contra el mercado y las galerías como «escaparates» de la transacción comercial; contra los «métodos religioso-expresionistas» que enseñan a «sentir y no pensar»; y contra «una falsa modernidad de importación», rematando con la consigna que se volvería célebre: «Sólo lo popular es realmente moderno hoy en el Perú». Reivindica el trabajo colectivo frente al «aislamiento» y el «desamparo teórico» del plástico joven, propone un «ejercicio ecológico» que revela el «cordón umbilical» entre los desechos de la ciudad y su arte, y ancla la práctica en «esa realidad fundamental del arte en América Latina que es la miseria». Contra el «arte bobo», postula un arte popular, político y antipublicitario. Constituye una fuente primaria clave para la historia del arte crítico y no-objetual peruano de fines de los años setenta e inicios de los ochenta.</t>
+          <t>El volumen documenta 'Un siglo de arte desde la Escuela Nacional', ciclo de cuatro exposiciones organizado en 2018 para el centenario (1918-2018) de la Escuela Nacional Superior Autónoma de Bellas Artes del Perú (ENSABAP), coeditado con el Instituto Cultural Peruano Norteamericano (ICPNA). Bajo la curaduría general de Max Hernández Calvo y Augusto del Valle Cárdenas, con Rocío Corcuera, Víctor Mejía y Miguel Sánchez, el proyecto busca construir memoria institucional y revisar cien años de producción y pedagogía bellasartina, articulándola con la sociedad contemporánea. Las muestras se distribuyeron en cuatro sedes (galerías ICPNA Juan Pardo Heeren y Germán Krüger Espantoso, y salas municipales de Miraflores). 'Bellas Artes: voz y huella de los egresados' (Corcuera) parte de cuarenta entrevistas a egresados de 1951 a 2017 —de Ella Krebs a Andrés Yaques— y una línea de tiempo que vincula formación, testimonio y obra estudiantil. 'Del individuo al ser social' (Sánchez) estudia los colectivos surgidos desde los años setenta (E.P.S. Huayco, Paréntesis, Signo x Signo, C.H.O.L.O., entre otros) como gesto político frente al modelo del artista individual. 'Espacio público' (Mejía) analiza el centro de Lima como insumo estético y campo de intervención. 'Una trayectoria de imágenes' (Hernández Calvo y Del Valle) emplea los géneros académicos —bodegón, paisaje, retrato— para pensar el tránsito del arte moderno al contemporáneo. La tesis transversal cuestiona la narrativa figurativo/abstracto de la modernidad e introduce la pregunta por el ícono, uniendo lo global con las tradiciones locales y artesanales, para otorgar 'carta de ciudadanía' a prácticas invisibilizadas desde una escuela pública.</t>
         </is>
       </c>
     </row>
@@ -1534,27 +1534,27 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. (ed.) - Hay algo incomestible en la garganta. Poéticas antipatriarcales y nueva escena en los años noventa (2021) [catálogo ICPNA].md</t>
+          <t>Kusunoki y Lerner - Reconsidering the «art museum». Some reflections on the history of the MALI collections (2026) [Unmaking to Make, cap. 5].md</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>1988-2002</t>
+          <t>1961-2022 (con referencias desde época prehispánica y los años 20)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de exposición, 2021</t>
+          <t>Capítulo de libro, 2026</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López (curaduría); Issela Ccoyllo; Carmen Ilizarbe; Susana Torres; María Eugenia Yllia; Montserrat Álvarez; Irene Rojas; Elena Tejada-Herrera; Natalia Iguíñiz; Flavia Gandolfo; Movimiento Manuela Ramos / TAFOS; ICPNA</t>
+          <t>Ricardo Kusunoki; Sharon Lerner; Museo de Arte de Lima (MALI); Natalia Majluf; Gabriela Germaná; Gredna Landolt; ADAPS / Piraq Causa; Brus Rubio Churay; José Sabogal; Con/Vida; Matadero Madrid / ARCO; Julieta González</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Catálogo bilingüe de la exposición homónima curada por Miguel A. López en el ICPNA de Lima con motivo del Bicentenario, que reúne más de doscientas obras de cerca de noventa creadoras, colectivas y talleres para examinar la producción visual y las transformaciones sociopolíticas peruanas entre 1988 y 2002. Su tesis central sostiene que, al cierre del siglo XX, fueron las mujeres y los cuerpos feminizados quienes reorientaron el rumbo del arte, desplegando lo que López denomina «poéticas antipatriarcales»: vocabularios estéticos surgidos para enfrentar una misoginia naturalizada y la violencia colonial, racial y patriarcal. El marco conceptual articula feminismo, crítica al neoliberalismo (el «hechizo» de la privatización y el individualismo), teoría social del arte y una lectura de clase del campo cultural, rechazando una absorción de la heterogeneidad bajo la categoría occidental de «arte». El proyecto yuxtapone deliberadamente circuitos antagónicos: obras de galerías, museos y bienales junto a arpilleras de asociaciones de mujeres y clubes de madres, los Talleres de Fotografía Social (TAFOS) y el proyecto Mercomujer del Movimiento Manuela Ramos. Se organiza en diez ejes temáticos (autorrepresentación, misoginia, deseo y disidencia de género, políticas de cuidado, acción colectiva, poder androcéntrico, reciprocidad, cuerpos gestantes, pieles e hilos, violencia política) y ensayos complementarios de Susana Torres, Issela Ccoyllo, María Eugenia Yllia y Carmen Ilizarbe. Su aporte reside en construir una genealogía transfeminista que rescata prácticas invisibilizadas —arpilleristas migrantes, artistas indígenas y campesinas, transformismo, autogestión— y las inscribe como agentes decisivas de la reconfiguración de la esfera pública peruana frente a la dictadura fujimorista.</t>
+          <t>Capítulo que reflexiona sobre la historia de las colecciones del Museo de Arte de Lima (MALI) desde su fundación en 1961 para interrogar la propia categoría de "museo de arte". Kusunoki y Lerner parten de la condición fundacional del MALI: nacido tardíamente frente a otros museos latinoamericanos, sin conexión con centros de enseñanza y configurado por el azar de donaciones como la vasta y heterogénea Memoria Prado. Esa amplitud material, argumentan, contenía en estado latente la posibilidad de cuestionar cómo las narrativas nacionales se proyectan sobre el pasado. El eje conceptual es la tensión entre "arte culto" y "arte popular", categoría esta última formulada en los años veinte desde el indigenismo de Sabogal y cargada de una ficción de autenticidad vernácula. El estudio de caso central es la incorporación en 2017 de la serie Piraq Causa —31 tablas de Sarhua de la ADAPS, comisionadas por Peter Gaupp, que narran la violencia de Sendero Luminoso y los Sinchis en Ayacucho—, que complejizó el eje de los "años de violencia" (junto a Taller N.N., Wiesse, Villares) y obligó a reconocer las tablas como práctica intersticial entre lo rural, urbano, tradicional y contemporáneo. La tesis sostiene que integrar tales obras no debe significar instalarlas en el espacio "atemporal" del arte, sino desmantelar la estructura dicotómica de clase y etnia del campo artístico peruano, preservando su carácter ambivalente. Reseña además el eje amazónico (Brus Rubio, 2014-2015), la gestión de Natalia Majluf (1995-2018) y las exposiciones Amazonías, Otras historias posibles (2019) e Imaginarios contemporáneos (2021-2022), proponiendo una política de colección que reconstruya constelaciones históricamente situadas y transformables.</t>
         </is>
       </c>
     </row>
@@ -1566,27 +1566,27 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - How Do We Know What Latin American Conceptualism Looks Like?.md</t>
+          <t>Lauer, Mirko - Arte al paso, Tome uno (1980) [volante Galería Forum, E.P.S. Huayco].md</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>años 60-70 (con foco en 1968: Tucumán Arde)</t>
+          <t>1980 (exposición Arte al paso, E.P.S. Huayco; contexto de la plástica joven peruana de fin de los años 70)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico (Afterall), ca. 2010</t>
+          <t>Volante/panfleto de exposición, mayo de 1980 (Galería Forum, Lima); transcripción manual de fotografía, 2026</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Mari Carmen Ramírez; Luis Camnitzer; Jane Farver; Rachel Weiss; Paul B. (Beatriz) Preciado; Graciela Carnevale; Ana Longoni; Fernando Davis; Eduardo Costa; Roberto Jacoby; Queens Museum of Art / MoMA / Red Conceptualismos del Sur</t>
+          <t>Mirko Lauer (texto); E.P.S. Huayco; María Luy; Francisco Mariotti; Charo Noriega; Juan Javier Salazar; Mariela Zevallos; Guillermo Orbegoso; Roberto Cores; Galería Forum</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Ensayo historiográfico de Miguel A. López que problematiza cómo se ha construido y estabilizado la categoría «conceptualismo latinoamericano». Su objeto de estudio son los dispositivos discursivos y expositivos que fijaron una imagen canónica de la producción crítica de los años sesenta y setenta, tomando como bisagras la muestra «Global Conceptualism: Points of Origin» (Queens Museum, 1999) y el ensayo fundacional «Blueprint Circuits» (1993) de Mari Carmen Ramírez. El marco conceptual proviene de una crítica queer de la representación: siguiendo a Paul B. Preciado y a Guattari, López contrapone una «cartografía de identidades» —que rastrea, clasifica y verifica obras conceptuales— a una «cartografía crítica» que expone las relaciones de poder y las tecnologías de producción de subjetividad implicadas en el acto de historizar. Argumenta que la distinción binaria entre un conceptualismo «analítico» anglosajón (Kosuth) y uno «ideológico» latinoamericano, consolidada por Ramírez y repetida por Osborne y Alberro, reinscribe la lógica centro/periferia que dice combatir y fija un estereotipo de arte subversivo. El texto examina la mitificación de «Tucumán Arde» (1968) y su recuperación en la exposición «Inventario 1965-1975. Archivo Graciela Carnevale» (Rosario, 2008), primer experimento curatorial de la Red Conceptualismos del Sur, que activa el archivo para desmontar la narrativa única. Recupera conceptos «menores» (desmaterialización de Masotta, no-objetualismo de Acha, deshabituación de Carreira) y cierra con la pieza de Eduardo Costa: su aporte es proponer una historiografía infiel, anacrónica y desestabilizadora que traicione las certezas del relato consensual.</t>
+          <t>Volante o panfleto bifronte («Arte al paso» / «Tome uno») escrito por Mirko Lauer para acompañar la exposición homónima del colectivo E.P.S. Huayco en la Galería Forum de Lima (mayo de 1980); el proyecto reúne a María Luy, Francisco Mariotti, Charo Noriega, Juan Javier Salazar y Mariela Zevallos, con fotografías de Guillermo Orbegoso y Roberto Cores. El texto, organizado como una serie de definiciones anafóricas («Arte al paso: …»), es un manifiesto programático del no-objetualismo peruano y del arte crítico. Lauer presenta la obra como una «contestación» que combina serigrafía, detritus industriales, fórmulas teóricas, fotos y «expendio de salchipapas» para sostener que «la realidad del arte es más compleja que la realidad de las 'Bellas Artes'». Articula tres operaciones críticas: contra el mercado y las galerías como «escaparates» de la transacción comercial; contra los «métodos religioso-expresionistas» que enseñan a «sentir y no pensar»; y contra «una falsa modernidad de importación», rematando con la consigna que se volvería célebre: «Sólo lo popular es realmente moderno hoy en el Perú». Reivindica el trabajo colectivo frente al «aislamiento» y el «desamparo teórico» del plástico joven, propone un «ejercicio ecológico» que revela el «cordón umbilical» entre los desechos de la ciudad y su arte, y ancla la práctica en «esa realidad fundamental del arte en América Latina que es la miseria». Contra el «arte bobo», postula un arte popular, político y antipublicitario. Constituye una fuente primaria clave para la historia del arte crítico y no-objetual peruano de fines de los años setenta e inicios de los ochenta.</t>
         </is>
       </c>
     </row>
@@ -1598,27 +1598,27 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - Los feminismos van a vencer. Una introducción [con presentación de Claudia Salazar Jiménez, dic. 2018].md</t>
+          <t>López, Miguel A. (ed.) - Hay algo incomestible en la garganta. Poéticas antipatriarcales y nueva escena en los años noventa (2021) [catálogo ICPNA].md</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>años 60-90 (textos escritos 2012-2018; activismo 2015-2018)</t>
+          <t>1988-2002</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Introducción de libro, 2018</t>
+          <t>Catálogo de exposición, 2021</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Claudia Salazar Jiménez; Rita Segato; Frantz Fanon; Julia Bryan-Wilson; Gladys Tzul Tzul; Aníbal Quijano; Paul B. Preciado; Giuseppe Campuzano; Víctor Manuel Rodríguez; TEOR/éTica / MACBA</t>
+          <t>Miguel A. López (curaduría); Issela Ccoyllo; Carmen Ilizarbe; Susana Torres; María Eugenia Yllia; Montserrat Álvarez; Irene Rojas; Elena Tejada-Herrera; Natalia Iguíñiz; Flavia Gandolfo; Movimiento Manuela Ramos / TAFOS; ICPNA</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Texto introductorio de López al libro que reúne sus ensayos sobre poéticas antipatriarcales (escritos entre 2012 y 2018), precedido por una presentación de la escritora Claudia Salazar Jiménez. Su tesis define los feminismos no como una identidad ni un periodo, sino como una «metodología para mirar» y un método de investigación afectivo: una política del afecto, la escucha y la resistencia colectiva que redefine el horizonte de acción y desconfía del esencialismo identitario. El marco conceptual entrelaza la «pedagogía de la crueldad» y el «mandato de la masculinidad» de Rita Segato, la distinción de Fanon entre «zona del ser» y «zona del no-ser», la «colonialidad del poder» de Aníbal Quijano y el «modelo metodológico afectivo» de Julia Bryan-Wilson, junto a referencias a Gladys Tzul Tzul y Paul B. Preciado. López sostiene que el arte, la performance y la escritura funcionan como refugio y resistencia frente a la exclusión, y que la tarea no es incorporar episodios omitidos a un inventario, sino analizar las condiciones políticas, materiales y afectivas que hacen emerger ciertas representaciones. Discute críticamente el rol de los museos como lugares de disputa capaces de redefinir la esfera pública, apoyándose en su experiencia en el MACBA y en la dirección colectiva de TEOR/éTica. Situado geopolíticamente en Lima pero atento a sus ausencias (la Amazonía, las provincias, el centralismo), el ensayo propone una genealogía transfeminista de la cultura visual que reactive «parientes extraviados» y reorganice la historia del arte como reserva de sororidad y alianzas.</t>
+          <t>Catálogo bilingüe de la exposición homónima curada por Miguel A. López en el ICPNA de Lima con motivo del Bicentenario, que reúne más de doscientas obras de cerca de noventa creadoras, colectivas y talleres para examinar la producción visual y las transformaciones sociopolíticas peruanas entre 1988 y 2002. Su tesis central sostiene que, al cierre del siglo XX, fueron las mujeres y los cuerpos feminizados quienes reorientaron el rumbo del arte, desplegando lo que López denomina «poéticas antipatriarcales»: vocabularios estéticos surgidos para enfrentar una misoginia naturalizada y la violencia colonial, racial y patriarcal. El marco conceptual articula feminismo, crítica al neoliberalismo (el «hechizo» de la privatización y el individualismo), teoría social del arte y una lectura de clase del campo cultural, rechazando una absorción de la heterogeneidad bajo la categoría occidental de «arte». El proyecto yuxtapone deliberadamente circuitos antagónicos: obras de galerías, museos y bienales junto a arpilleras de asociaciones de mujeres y clubes de madres, los Talleres de Fotografía Social (TAFOS) y el proyecto Mercomujer del Movimiento Manuela Ramos. Se organiza en diez ejes temáticos (autorrepresentación, misoginia, deseo y disidencia de género, políticas de cuidado, acción colectiva, poder androcéntrico, reciprocidad, cuerpos gestantes, pieles e hilos, violencia política) y ensayos complementarios de Susana Torres, Issela Ccoyllo, María Eugenia Yllia y Carmen Ilizarbe. Su aporte reside en construir una genealogía transfeminista que rescata prácticas invisibilizadas —arpilleristas migrantes, artistas indígenas y campesinas, transformismo, autogestión— y las inscribe como agentes decisivas de la reconfiguración de la esfera pública peruana frente a la dictadura fujimorista.</t>
         </is>
       </c>
     </row>
@@ -1630,27 +1630,27 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - Parientes extraviados, Cuerpo vehículo político y A contratiempo. Tres ensayos sobre poéticas antipatriarcales.md</t>
+          <t>López, Miguel A. - How Do We Know What Latin American Conceptualism Looks Like?.md</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>años 60-80 (con proyección al presente)</t>
+          <t>años 60-70 (con foco en 1968: Tucumán Arde)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Capítulos de libro, 2019</t>
+          <t>Artículo académico (Afterall), ca. 2010</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Teresa Burga; Gloria Gómez-Sánchez; Cristina Portocarrero; Victoria Santa Cruz; Johanna Hamann; Tilsa Tsuchiya; Marisa Godínez; María T-Ta (María Roncal); Grupo Chaclacayo; ALIMUPER / Movimiento Manuela Ramos / Centro Flora Tristán</t>
+          <t>Miguel A. López; Mari Carmen Ramírez; Luis Camnitzer; Jane Farver; Rachel Weiss; Paul B. (Beatriz) Preciado; Graciela Carnevale; Ana Longoni; Fernando Davis; Eduardo Costa; Roberto Jacoby; Queens Museum of Art / MoMA / Red Conceptualismos del Sur</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Conjunto de tres ensayos de López que trazan una genealogía de poéticas antipatriarcales en el arte peruano entre los años sesenta y ochenta, entendidas como «parientes extraviados» de las luchas feministas y sexodisidentes actuales. «Parientes extraviados» reconstruye la contribución de las artistas mujeres al experimentalismo: las ambientaciones y objetos de Teresa Burga y Gloria Gómez-Sánchez en el grupo Arte Nuevo (1966-1968), que desmantelaban el régimen masculino de la mirada; el tránsito de Cristina Portocarrero del arte a la militancia en ALIMUPER; y la revaloración de las artes de tradición andina (Apolonia Dorregaray) bajo el velasquismo. «Cuerpo, vehículo político» analiza cómo diversas creadoras abandonaron pintura y escultura para usar el propio cuerpo como crítica: el «Antiballet» de Yvonne von Mollendorff, el «Autorretrato» clínico de Burga (1972), la declamación antirracista «Me gritaron negra» de Victoria Santa Cruz, las «Barrigas» de Johanna Hamann y la gráfica militante de Marisa Godínez para Flora Tristán. Aborda además la teatralidad, el travestismo y lo performativo de los ochenta —Grupo Chaclacayo, Jaime Higa, la escena drag documentada por Flavia Gandolfo, la punk María T-Ta, Támira Bassallo, Susana Torres— como respuestas a una guerra tanto armada como misógina y homofóbica. El tercer ensayo, «A contratiempo», explora las «cronodisidencias» de Burga y su temporalidad improductiva del dibujo. El marco conceptual moviliza teoría feminista y queer (Preciado, Bryan-Wilson, Richard); su aporte es reinscribir prácticas borradas como antagonismo estético-político y desmentir el diagnóstico de su supuesta inexistencia.</t>
+          <t>Ensayo historiográfico de Miguel A. López que problematiza cómo se ha construido y estabilizado la categoría «conceptualismo latinoamericano». Su objeto de estudio son los dispositivos discursivos y expositivos que fijaron una imagen canónica de la producción crítica de los años sesenta y setenta, tomando como bisagras la muestra «Global Conceptualism: Points of Origin» (Queens Museum, 1999) y el ensayo fundacional «Blueprint Circuits» (1993) de Mari Carmen Ramírez. El marco conceptual proviene de una crítica queer de la representación: siguiendo a Paul B. Preciado y a Guattari, López contrapone una «cartografía de identidades» —que rastrea, clasifica y verifica obras conceptuales— a una «cartografía crítica» que expone las relaciones de poder y las tecnologías de producción de subjetividad implicadas en el acto de historizar. Argumenta que la distinción binaria entre un conceptualismo «analítico» anglosajón (Kosuth) y uno «ideológico» latinoamericano, consolidada por Ramírez y repetida por Osborne y Alberro, reinscribe la lógica centro/periferia que dice combatir y fija un estereotipo de arte subversivo. El texto examina la mitificación de «Tucumán Arde» (1968) y su recuperación en la exposición «Inventario 1965-1975. Archivo Graciela Carnevale» (Rosario, 2008), primer experimento curatorial de la Red Conceptualismos del Sur, que activa el archivo para desmontar la narrativa única. Recupera conceptos «menores» (desmaterialización de Masotta, no-objetualismo de Acha, deshabituación de Carreira) y cierra con la pieza de Eduardo Costa: su aporte es proponer una historiografía infiel, anacrónica y desestabilizadora que traicione las certezas del relato consensual.</t>
         </is>
       </c>
     </row>
@@ -1662,27 +1662,27 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Mesa - Arte contemporáneo peruano. Portocarrero, Aramburu y Lerner (2022) [MALBA].transcripcion.md</t>
+          <t>López, Miguel A. - Los feminismos van a vencer. Una introducción [con presentación de Claudia Salazar Jiménez, dic. 2018].md</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>1930-2022 (con énfasis en 1976-2022)</t>
+          <t>años 60-90 (textos escritos 2012-2018; activismo 2015-2018)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Transcripción de mesa redonda (MALBA/MALVA), 2022</t>
+          <t>Introducción de libro, 2018</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Florencia Portocarrero; Iosu Aramburu; Verónica Rossi; Ana Teresa Barboza; Mirko Lauer; Joaquín López Antay; Miguel Aguirre; Elvia Paucar; Centro de Textiles Tradicionales del Cusco; MALI</t>
+          <t>Miguel A. López; Claudia Salazar Jiménez; Rita Segato; Frantz Fanon; Julia Bryan-Wilson; Gladys Tzul Tzul; Aníbal Quijano; Paul B. Preciado; Giuseppe Campuzano; Víctor Manuel Rodríguez; TEOR/éTica / MACBA</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Transcripción (borrador sin refinar) de una mesa redonda organizada en torno a la exposición 'Tejer las Piedras' de Ana Teresa Barboza, que toma el pulso a los debates del arte contemporáneo peruano actual, con foco en la relación entre arte y artesanía. Sharon Lerner abre con un recorrido por veinte años de la obra de Barboza, desde el bordado autobiográfico de cuerpos y heridas —leído por Gabriela Germaná y Augusto del Valle como inversión de la representación sexista— hacia un trabajo colaborativo con tejido, telar de cintura y tintes naturales que reflexiona sobre paisaje, sostenibilidad y territorio, situándolo en la tradición anglosajona del craft y en la reinserción de lo personal, según Whitney Chadwick, característica del feminismo desde los setenta. Portocarrero y Aramburu estructuran su intervención con los tres 'universos estéticos' de Mirko Lauer (precolombino, erudito/bellas artes, tradicional/popular), entendidos como compartimentos estancos ligados a una estructura colonial y racista, y examinan sus cruces históricos: el Instituto de Arte Peruano indigenista, la apropiación de lo prehispánico en los sesenta, el escándalo del Premio Nacional a Joaquín López Antay (1976). El marco conceptual sostiene que, a diferencia de aquel premio otorgado por un jurado, artistas indígenas contemporáneos como Venuca Evanán y Chonon Bensho hoy postulan conscientemente e ingresan por agencia propia a los circuitos del arte contemporáneo. Se analizan la colaboración de largo aliento entre Miguel Aguirre y la tejedora Elvia Paucar y el proyecto Ser Payay en Cusco, como casos de 'vocabularios colaborados' que problematizan la coautoría, la mediación y las lógicas de mercado diferenciadas entre arte y artesanía.</t>
+          <t>Texto introductorio de López al libro que reúne sus ensayos sobre poéticas antipatriarcales (escritos entre 2012 y 2018), precedido por una presentación de la escritora Claudia Salazar Jiménez. Su tesis define los feminismos no como una identidad ni un periodo, sino como una «metodología para mirar» y un método de investigación afectivo: una política del afecto, la escucha y la resistencia colectiva que redefine el horizonte de acción y desconfía del esencialismo identitario. El marco conceptual entrelaza la «pedagogía de la crueldad» y el «mandato de la masculinidad» de Rita Segato, la distinción de Fanon entre «zona del ser» y «zona del no-ser», la «colonialidad del poder» de Aníbal Quijano y el «modelo metodológico afectivo» de Julia Bryan-Wilson, junto a referencias a Gladys Tzul Tzul y Paul B. Preciado. López sostiene que el arte, la performance y la escritura funcionan como refugio y resistencia frente a la exclusión, y que la tarea no es incorporar episodios omitidos a un inventario, sino analizar las condiciones políticas, materiales y afectivas que hacen emerger ciertas representaciones. Discute críticamente el rol de los museos como lugares de disputa capaces de redefinir la esfera pública, apoyándose en su experiencia en el MACBA y en la dirección colectiva de TEOR/éTica. Situado geopolíticamente en Lima pero atento a sus ausencias (la Amazonía, las provincias, el centralismo), el ensayo propone una genealogía transfeminista de la cultura visual que reactive «parientes extraviados» y reorganice la historia del arte como reserva de sororidad y alianzas.</t>
         </is>
       </c>
     </row>
@@ -1694,27 +1694,27 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Mesa - Coleccionando desde la institución (2025) [Charlas de colección, Foro Pinta Lima].transcripcion.md</t>
+          <t>López, Miguel A. - Parientes extraviados, Cuerpo vehículo político y A contratiempo. Tres ensayos sobre poéticas antipatriarcales.md</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>1960s-2025 (con eje en 2006-2025)</t>
+          <t>años 60-80 (con proyección al presente)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Transcripción de conversatorio (Foro Pinta Lima 2025), 2025</t>
+          <t>Capítulos de libro, 2019</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Pablo León de la Barra; Sharon Lerner; Manuel Segade; MALI; Museo Reina Sofía; Museo Guggenheim; Comité de Adquisiciones de Arte Contemporáneo del MALI; Suset Sánchez; Amanda de la Garza; Tatiana Cuevas; Fundación Museo Reina Sofía</t>
+          <t>Miguel A. López; Teresa Burga; Gloria Gómez-Sánchez; Cristina Portocarrero; Victoria Santa Cruz; Johanna Hamann; Tilsa Tsuchiya; Marisa Godínez; María T-Ta (María Roncal); Grupo Chaclacayo; ALIMUPER / Movimiento Manuela Ramos / Centro Flora Tristán</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Transcripción (borrador) del conversatorio 'Coleccionando desde la institución' del Foro Pinta Lima 2025, moderado por Pablo León de la Barra (Guggenheim), que confronta dos modelos museales públicos: el MALI de Lima y el Museo Reina Sofía de Madrid. La tesis compartida es que coleccionar implica un pensamiento crítico que puede cuestionar el canon, reparar asimetrías históricas de género, raza e identidad y llenar vacíos. Sharon Lerner expone la trayectoria del Comité de Adquisiciones de Arte Contemporáneo del MALI (casi veinte años, modelado sobre el Latin American Acquisitions Committee de la Tate), la curaduría contemporánea iniciada por Tatiana Cuevas en 2008, y el trabajo 'trenzado' entre colección histórica y contemporánea que atraviesa exposiciones como Arte al Paso, Amazonías y Otras historias posibles, y la reestructuración pospandemia con el programa Salas Abiertas. Detalla la visibilización de artistas amazónicos e indígenas (Sara Flores, Chonon Bensho, Venuca Evanán), la incorporación del textil y proyectos como Línea de Vida de Giuseppe Campuzano, junto a comisiones y trabajo comunitario con Cantagallo. Manuel Segade analiza la dimensión colonial del Reina Sofía —cuya colección latinoamericana se inauguró en 1992— y las condiciones estructurales, funcionariales y presupuestarias que la condicionan, citando las preguntas ontológicas de Suset Sánchez y el Instituto Cader de arte centroamericano como vía de restitución frente al extractivismo cultural. El diálogo aborda el rol de los públicos, la crispación política, la censura, el cierre del Lugar de la Memoria y la misión histórica del museo como plataforma de tensiones críticas de la sociedad civil.</t>
+          <t>Conjunto de tres ensayos de López que trazan una genealogía de poéticas antipatriarcales en el arte peruano entre los años sesenta y ochenta, entendidas como «parientes extraviados» de las luchas feministas y sexodisidentes actuales. «Parientes extraviados» reconstruye la contribución de las artistas mujeres al experimentalismo: las ambientaciones y objetos de Teresa Burga y Gloria Gómez-Sánchez en el grupo Arte Nuevo (1966-1968), que desmantelaban el régimen masculino de la mirada; el tránsito de Cristina Portocarrero del arte a la militancia en ALIMUPER; y la revaloración de las artes de tradición andina (Apolonia Dorregaray) bajo el velasquismo. «Cuerpo, vehículo político» analiza cómo diversas creadoras abandonaron pintura y escultura para usar el propio cuerpo como crítica: el «Antiballet» de Yvonne von Mollendorff, el «Autorretrato» clínico de Burga (1972), la declamación antirracista «Me gritaron negra» de Victoria Santa Cruz, las «Barrigas» de Johanna Hamann y la gráfica militante de Marisa Godínez para Flora Tristán. Aborda además la teatralidad, el travestismo y lo performativo de los ochenta —Grupo Chaclacayo, Jaime Higa, la escena drag documentada por Flavia Gandolfo, la punk María T-Ta, Támira Bassallo, Susana Torres— como respuestas a una guerra tanto armada como misógina y homofóbica. El tercer ensayo, «A contratiempo», explora las «cronodisidencias» de Burga y su temporalidad improductiva del dibujo. El marco conceptual moviliza teoría feminista y queer (Preciado, Bryan-Wilson, Richard); su aporte es reinscribir prácticas borradas como antagonismo estético-político y desmentir el diagnóstico de su supuesta inexistencia.</t>
         </is>
       </c>
     </row>
@@ -1726,27 +1726,27 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Ministerio de Cultura - Contemporáneos. Cinco mil años de visualidad peruana (2019) [catálogo, Perú país invitado ARCOmadrid].md</t>
+          <t>Mesa - Arte contemporáneo peruano. Portocarrero, Aramburu y Lerner (2022) [MALBA].transcripcion.md</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>200 a.C.-2019 (Nasca, virreinato y arte contemporáneo reciente)</t>
+          <t>1930-2022 (con énfasis en 1976-2022)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Catálogo institucional de feria/exposición (ARCOmadrid), 2019</t>
+          <t>Transcripción de mesa redonda (MALBA/MALVA), 2022</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Ministerio de Cultura del Perú; Jorge Villacorta; Sharon Lerner; Fietta Jarque; Miguel A. López; Teresa Burga; Fernando Bryce; Sandra Gamarra; Natalia Majluf; MALI; ARCOmadrid / IFEMA; Museo Reina Sofía / Museo del Prado</t>
+          <t>Sharon Lerner; Florencia Portocarrero; Iosu Aramburu; Verónica Rossi; Ana Teresa Barboza; Mirko Lauer; Joaquín López Antay; Miguel Aguirre; Elvia Paucar; Centro de Textiles Tradicionales del Cusco; MALI</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Catálogo institucional de la participación de Perú como País Invitado en ARCOmadrid 2019, que reúne los textos curatoriales del stand del Estado, la zona de galerías y el programa oficial de más de treinta exposiciones y actividades en Madrid. El ensayo de Jorge Villacorta, 'Contemporáneos: cinco mil años de visualidad peruana', propone lo contemporáneo como actitud y coexistencia antes que como novedad, avanzando la hipótesis de que la contemporaneidad peruana es continuidad de una matriz cultural andino-amazónica con incrustaciones occidentales, un tiempo cíclico que supera categorías como arte popular o artesanía. Sharon Lerner, en 'Texto, tactibilidad y trama', encuadra la selección de galerías —que por primera vez combina representación local e internacional— como un corte no representativo de un 'arte nacional', destacando líneas transversales: el uso del texto, la cita y el archivo para desmontar discursos de la historia oficial; las tensiones del colonialismo y los criterios étnicos y de clase; la mirada al territorio y a lo extractivo; y la fragilidad táctil del textil, la arcilla y el cuerpo. El catálogo perfila a artistas como Teresa Burga, Rita Ponce de León, Ximena Garrido Lecca, Herbert Rodríguez, Fernando Bryce, Sandra Gamarra, Milagros de la Torre y Antonio Paucar, y documenta las conferencias curadas por Miguel A. López sobre el Bicentenario, la contemporaneidad andina, indígena y amazónica, y las transformaciones institucionales y de mercado. El programa oficial, presentado por Fietta Jarque, articula un relato de cinco mil años: Nasca, el Matrimonio de Martín de Loyola, Huamán Poma, la revista Amauta de Mariátegui, Amazonías y colecciones privadas (Hochschild, CIFO, Jan Mulder).</t>
+          <t>Transcripción (borrador sin refinar) de una mesa redonda organizada en torno a la exposición 'Tejer las Piedras' de Ana Teresa Barboza, que toma el pulso a los debates del arte contemporáneo peruano actual, con foco en la relación entre arte y artesanía. Sharon Lerner abre con un recorrido por veinte años de la obra de Barboza, desde el bordado autobiográfico de cuerpos y heridas —leído por Gabriela Germaná y Augusto del Valle como inversión de la representación sexista— hacia un trabajo colaborativo con tejido, telar de cintura y tintes naturales que reflexiona sobre paisaje, sostenibilidad y territorio, situándolo en la tradición anglosajona del craft y en la reinserción de lo personal, según Whitney Chadwick, característica del feminismo desde los setenta. Portocarrero y Aramburu estructuran su intervención con los tres 'universos estéticos' de Mirko Lauer (precolombino, erudito/bellas artes, tradicional/popular), entendidos como compartimentos estancos ligados a una estructura colonial y racista, y examinan sus cruces históricos: el Instituto de Arte Peruano indigenista, la apropiación de lo prehispánico en los sesenta, el escándalo del Premio Nacional a Joaquín López Antay (1976). El marco conceptual sostiene que, a diferencia de aquel premio otorgado por un jurado, artistas indígenas contemporáneos como Venuca Evanán y Chonon Bensho hoy postulan conscientemente e ingresan por agencia propia a los circuitos del arte contemporáneo. Se analizan la colaboración de largo aliento entre Miguel Aguirre y la tejedora Elvia Paucar y el proyecto Ser Payay en Cusco, como casos de 'vocabularios colaborados' que problematizan la coautoría, la mediación y las lógicas de mercado diferenciadas entre arte y artesanía.</t>
         </is>
       </c>
     </row>
@@ -1758,27 +1758,27 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Mitrovic - Extravíos de la forma. Vanguardia, modernismo popular y arte contemporáneo en Lima desde los 60 (2019).md</t>
+          <t>Mesa - Coleccionando desde la institución (2025) [Charlas de colección, Foro Pinta Lima].transcripcion.md</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>1960-2018 (desde los sesenta hasta el presente)</t>
+          <t>1960s-2025 (con eje en 2006-2025)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Libro académico, 2019 (Fondo Editorial FAU-PUCP)</t>
+          <t>Transcripción de conversatorio (Foro Pinta Lima 2025), 2025</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Mijail Mitrovic; Gustavo Buntinx; Mirko Lauer; Sharon Lerner; Miguel A. López; Emilio Tarazona; Fernando de Szyszlo; E.P.S. Huayco; Taller NN; José Carlos Martinat; Museo de Arte de Lima (MALI); PUCP; Fredric Jameson</t>
+          <t>Pablo León de la Barra; Sharon Lerner; Manuel Segade; MALI; Museo Reina Sofía; Museo Guggenheim; Comité de Adquisiciones de Arte Contemporáneo del MALI; Suset Sánchez; Amanda de la Garza; Tatiana Cuevas; Fundación Museo Reina Sofía</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Ensayo de historia y teoría del arte que impugna el «relato convencional» sobre el arte contemporáneo en Lima, entendido como una fábula épica que narra el tránsito de la vanguardia de los sesenta al arte contemporáneo global mediante el «encuentro con lo popular». Desde un marco marxista-dialéctico (Adorno, Jameson, Bürger, Osborne, Lukács), Mitrovic reivindica la totalización y la periodización frente al historicismo posmoderno que celebra heterogeneidad y discontinuidad. Su tesis central es que la «desidealización» del arte —su reducción a hecho social e institucional— siguió en Lima una trayectoria específica: de la teoría de las raíces nacionales (Szyszlo, Lauer) y el altomodernismo, a la radicalización de la vanguardia bajo el velasquismo, que el autor conceptualiza como «modernismo popular» (E.P.S. Huayco, Paréntesis, la frase de Lauer «solo lo popular es moderno»). Con Sendero Luminoso y la crisis de los ochenta, la utopía colapsa y el arte se reorienta hacia la denuncia ética de la violencia, prolongada durante el fujimorato (Colectivo Sociedad Civil, «Lava la bandera»). El cambio de siglo consuma la «contemporaneización» mediante las Bienales de Lima y el mercado. El último capítulo analiza obras (Polanco, Guerra García, Huarcaya, Aguirre, Andrade Valdez, Martinat) para mostrar cómo lo popular deviene «neocostumbrismo» y «renta de monopolio»: sello local que certifica autenticidad cultural en el circuito global, mientras se evacúa el horizonte futuro y el «pueblo» se reduce a «población». Frente a la nostalgia y la reoligarquización simbólica, Mitrovic propone recuperar las potencialidades utópicas hoy reprimidas.</t>
+          <t>Transcripción (borrador) del conversatorio 'Coleccionando desde la institución' del Foro Pinta Lima 2025, moderado por Pablo León de la Barra (Guggenheim), que confronta dos modelos museales públicos: el MALI de Lima y el Museo Reina Sofía de Madrid. La tesis compartida es que coleccionar implica un pensamiento crítico que puede cuestionar el canon, reparar asimetrías históricas de género, raza e identidad y llenar vacíos. Sharon Lerner expone la trayectoria del Comité de Adquisiciones de Arte Contemporáneo del MALI (casi veinte años, modelado sobre el Latin American Acquisitions Committee de la Tate), la curaduría contemporánea iniciada por Tatiana Cuevas en 2008, y el trabajo 'trenzado' entre colección histórica y contemporánea que atraviesa exposiciones como Arte al Paso, Amazonías y Otras historias posibles, y la reestructuración pospandemia con el programa Salas Abiertas. Detalla la visibilización de artistas amazónicos e indígenas (Sara Flores, Chonon Bensho, Venuca Evanán), la incorporación del textil y proyectos como Línea de Vida de Giuseppe Campuzano, junto a comisiones y trabajo comunitario con Cantagallo. Manuel Segade analiza la dimensión colonial del Reina Sofía —cuya colección latinoamericana se inauguró en 1992— y las condiciones estructurales, funcionariales y presupuestarias que la condicionan, citando las preguntas ontológicas de Suset Sánchez y el Instituto Cader de arte centroamericano como vía de restitución frente al extractivismo cultural. El diálogo aborda el rol de los públicos, la crispación política, la censura, el cierre del Lugar de la Memoria y la misión histórica del museo como plataforma de tensiones críticas de la sociedad civil.</t>
         </is>
       </c>
     </row>
@@ -1790,27 +1790,27 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Peralta - Lo que la Bienal de Lima se llevó. Balance a cinco años de su desactivación.md</t>
+          <t>Ministerio de Cultura - Contemporáneos. Cinco mil años de visualidad peruana (2019) [catálogo, Perú país invitado ARCOmadrid].md</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>1997-2003 (Bienales de Lima y su desactivación)</t>
+          <t>200 a.C.-2019 (Nasca, virreinato y arte contemporáneo reciente)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Artículo/ensayo de balance, ca. 2007-2008</t>
+          <t>Catálogo institucional de feria/exposición (ARCOmadrid), 2019</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Juan Peralta; Luis Lama; Jorge Villacorta; Emilio Santisteban; Elena Tejada; Gustavo Buntinx; Alfonso Castrillón; Élida Román; Allora &amp; Calzadilla; Francis Alÿs; Cuauhtémoc Medina; Alberto Andrade; Luis Castañeda Lossio; Municipalidad Metropolitana de Lima; UCCI</t>
+          <t>Ministerio de Cultura del Perú; Jorge Villacorta; Sharon Lerner; Fietta Jarque; Miguel A. López; Teresa Burga; Fernando Bryce; Sandra Gamarra; Natalia Majluf; MALI; ARCOmadrid / IFEMA; Museo Reina Sofía / Museo del Prado</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Balance crítico sobre la desaparición de la Bienal de Lima, escrito por Juan Peralta a cinco años de su desactivación. El texto reconstruye el contexto político-cultural en que surgió el megaevento ideado por Luis Lama: el régimen fujimorista, el programa municipal «Volver al Centro» y el Plan Maestro del Centro Histórico impulsado por la gestión de Alberto Andrade, articulados con redes internacionales (UCCI, CIDEU) y el título de «Lima, Capital de la Cultura Iberoamericana». Peralta sostiene que la Bienal (1997-2002), en sus versiones nacional e iberoamericana, funcionó como núcleo de reactivación cultural y descentralización mediante salones regionales, atrajo atención internacional y sirvió de modelo de gestión, pero fue cancelada por desinterés político —especialmente de Luis Castañeda Lossio— y por la incapacidad del propio medio artístico de defender su función social. Documenta episodios polémicos: la crítica de Alfonso Castrillón a la autoría de una obra de García Zapatero, la performance «Señorita de buena presencia busca empleo» de Elena Tejada, la muestra paralela «Emergencia Artística» (1999) gestada por Emilio Santisteban y Gustavo Buntinx tras el veto a «Crisis», y la intervención «Chalk» de Allora &amp; Calzadilla, resignificada por trabajadores municipales. A través de testimonios (Santisteban, Élida Román, Natalia Velit, el propio Lama), el autor argumenta que la orfandad cultural persiste por la ausencia de políticas públicas y la subordinación al mercado. El texto se posiciona a favor de una gestión cultural audaz, descentralizada y socialmente participativa, lamentando que nada haya reemplazado la escala y el alcance de la Bienal.</t>
+          <t>Catálogo institucional de la participación de Perú como País Invitado en ARCOmadrid 2019, que reúne los textos curatoriales del stand del Estado, la zona de galerías y el programa oficial de más de treinta exposiciones y actividades en Madrid. El ensayo de Jorge Villacorta, 'Contemporáneos: cinco mil años de visualidad peruana', propone lo contemporáneo como actitud y coexistencia antes que como novedad, avanzando la hipótesis de que la contemporaneidad peruana es continuidad de una matriz cultural andino-amazónica con incrustaciones occidentales, un tiempo cíclico que supera categorías como arte popular o artesanía. Sharon Lerner, en 'Texto, tactibilidad y trama', encuadra la selección de galerías —que por primera vez combina representación local e internacional— como un corte no representativo de un 'arte nacional', destacando líneas transversales: el uso del texto, la cita y el archivo para desmontar discursos de la historia oficial; las tensiones del colonialismo y los criterios étnicos y de clase; la mirada al territorio y a lo extractivo; y la fragilidad táctil del textil, la arcilla y el cuerpo. El catálogo perfila a artistas como Teresa Burga, Rita Ponce de León, Ximena Garrido Lecca, Herbert Rodríguez, Fernando Bryce, Sandra Gamarra, Milagros de la Torre y Antonio Paucar, y documenta las conferencias curadas por Miguel A. López sobre el Bicentenario, la contemporaneidad andina, indígena y amazónica, y las transformaciones institucionales y de mercado. El programa oficial, presentado por Fietta Jarque, articula un relato de cinco mil años: Nasca, el Matrimonio de Martín de Loyola, Huamán Poma, la revista Amauta de Mariátegui, Amazonías y colecciones privadas (Hochschild, CIFO, Jan Mulder).</t>
         </is>
       </c>
     </row>
@@ -1822,27 +1822,27 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Ponencia - Villacorta, Jorge - Puntos cardinales (2019) [CEdA].transcripcion.txt</t>
+          <t>Mitrovic - Extravíos de la forma. Vanguardia, modernismo popular y arte contemporáneo en Lima desde los 60 (2019).md</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>1979-2019 (énfasis en 2001-2019: obra de los ochenta y ARCO 2019)</t>
+          <t>1960-2018 (desde los sesenta hasta el presente)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Transcripción de ponencia/conferencia, 2019 (Fundación SEDA-CEdA, Santiago)</t>
+          <t>Libro académico, 2019 (Fondo Editorial FAU-PUCP)</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Sebastián Vidal; Fundación SEDA; Sandra Gamarra (LiMac); Juan Javier Salazar; Herbert Rodríguez; Rodrigo Quijano; grupo Huayco; MALI; Fundación Reina Sofía; ARCOmadrid; galería Enrique Faria; galería Revólver; Alexis Fabri</t>
+          <t>Mijail Mitrovic; Gustavo Buntinx; Mirko Lauer; Sharon Lerner; Miguel A. López; Emilio Tarazona; Fernando de Szyszlo; E.P.S. Huayco; Taller NN; José Carlos Martinat; Museo de Arte de Lima (MALI); PUCP; Fredric Jameson</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Transcripción de una ponencia de Jorge Villacorta en la Fundación SEDA (Santiago de Chile), presentada por Sebastián Vidal, en el marco de su participación en el pabellón peruano de ARCOmadrid 2019. Partiendo de dos exposiciones fundacionales de Sandra Gamarra (Living Room, 2001; el proyecto LiMac, 2002), Villacorta reflexiona sobre la desconexión histórica del sistema del arte limeño respecto del circuito internacional y su condición estructuralmente «coja». El eje del argumento es un contraste entre dos artistas del grupo Huayco: Juan Javier Salazar y Herbert Rodríguez. Salazar, considerado durante dos décadas el artista contemporáneo peruano por excelencia (Perú País del Mañana, El cuartucho, los náufragos), cultivó una obra frágil, localista y ácida sobre la desidia nacional, pero fue «maltratado» tras su muerte: descartado en ARCO 2019, cosmetizado en la Bienal de Venecia 2017 y regateado por el capítulo peruano de la Fundación Reina Sofía. Rodríguez, artista afrodescendiente y sistemático archivista de su obra (fotocopias, murales antisenderistas en San Marcos, fotoserigrafía), experimenta en cambio un ascenso internacional inesperado (galería Enrique Faria, Reina Sofía, Fundación Cartier), pese al desdén histórico del medio limeño y del MALI. Villacorta articula estas trayectorias con una crítica al coleccionismo peruano, a la lógica del mercado (galería Revólver, ferias, matching funds de arteBA), a la desatención de la crítica y las galerías, y a las jerarquías raciales y clasistas del establishment cultural limeño (Szyszlo, Armando Andrade). El texto plantea el problema del legado, el valor simbólico y la posibilidad de un arte con «testigos» frente a un arte subordinado al mercado.</t>
+          <t>Ensayo de historia y teoría del arte que impugna el «relato convencional» sobre el arte contemporáneo en Lima, entendido como una fábula épica que narra el tránsito de la vanguardia de los sesenta al arte contemporáneo global mediante el «encuentro con lo popular». Desde un marco marxista-dialéctico (Adorno, Jameson, Bürger, Osborne, Lukács), Mitrovic reivindica la totalización y la periodización frente al historicismo posmoderno que celebra heterogeneidad y discontinuidad. Su tesis central es que la «desidealización» del arte —su reducción a hecho social e institucional— siguió en Lima una trayectoria específica: de la teoría de las raíces nacionales (Szyszlo, Lauer) y el altomodernismo, a la radicalización de la vanguardia bajo el velasquismo, que el autor conceptualiza como «modernismo popular» (E.P.S. Huayco, Paréntesis, la frase de Lauer «solo lo popular es moderno»). Con Sendero Luminoso y la crisis de los ochenta, la utopía colapsa y el arte se reorienta hacia la denuncia ética de la violencia, prolongada durante el fujimorato (Colectivo Sociedad Civil, «Lava la bandera»). El cambio de siglo consuma la «contemporaneización» mediante las Bienales de Lima y el mercado. El último capítulo analiza obras (Polanco, Guerra García, Huarcaya, Aguirre, Andrade Valdez, Martinat) para mostrar cómo lo popular deviene «neocostumbrismo» y «renta de monopolio»: sello local que certifica autenticidad cultural en el circuito global, mientras se evacúa el horizonte futuro y el «pueblo» se reduce a «población». Frente a la nostalgia y la reoligarquización simbólica, Mitrovic propone recuperar las potencialidades utópicas hoy reprimidas.</t>
         </is>
       </c>
     </row>
@@ -1854,27 +1854,27 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Por Qué no vivo en el Perú.md</t>
+          <t>Peralta - Lo que la Bienal de Lima se llevó. Balance a cinco años de su desactivación.md</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>ca. 1972 en adelante (emigración de Juan Acha a México y comparación Perú/México de los años setenta)</t>
+          <t>1997-2003 (Bienales de Lima y su desactivación)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Encuesta/testimonio en revista literaria (Hueso Húmero), ca. 1980; transcripción en Markdown, s/f</t>
+          <t>Artículo/ensayo de balance, ca. 2007-2008</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Juan Acha; revista Hueso Húmero; museos, institutos y universidades de México</t>
+          <t>Juan Peralta; Luis Lama; Jorge Villacorta; Emilio Santisteban; Elena Tejada; Gustavo Buntinx; Alfonso Castrillón; Élida Román; Allora &amp; Calzadilla; Francis Alÿs; Cuauhtémoc Medina; Alberto Andrade; Luis Castañeda Lossio; Municipalidad Metropolitana de Lima; UCCI</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Transcripción de la respuesta de Juan Acha a la encuesta 'Por qué no vivo en el Perú', iniciada por la revista Hueso Húmero para indagar las razones del éxodo de creadores e intelectuales peruanos. Acha —crítico y teórico del arte dedicado a los problemas latinoamericanos, radicado en México— distingue razones 'de afuera' y 'de adentro', otorgando mayor peso a las primeras: sólo abandona su país quien encuentra en otro las condiciones para desarrollar con dignidad su trabajo profesional, mientras que las circunstancias personales o los factores nacionales negativos serían secundarios en su caso. Enumera lo que México le ofreció y el Perú le negaba: amplias posibilidades de publicar en diarios y revistas, de colaborar en museos e institutos y de investigar y enseñar en universidades, todo ello remunerado con dignidad; libertad de expresión intelectual e intensa circulación de ideas marxistas en libros, revistas y simposios; prestigio nacional de las artes visuales con apoyo estatal, política museográfica y de simposios activa, y facilidades para viajar y contactar con el arte de otras latitudes. Valora, además, el mejor enfoque de los problemas artísticos y culturales latinoamericanos posible desde México, cuya escala demográfica y potente industria editorial concentran las investigaciones de toda la región y anticipan fenómenos que luego se difunden. El testimonio —que el archivo conserva incompleto, interrumpido al mencionar una 'identificación cultural más conflictiva y acorde a la realidad concreta'— condensa la autojustificación del exilio intelectual como decisión productiva antes que como queja, y funciona como documento sobre las carencias institucionales del campo artístico peruano frente a las condiciones del México de esos años.</t>
+          <t>Balance crítico sobre la desaparición de la Bienal de Lima, escrito por Juan Peralta a cinco años de su desactivación. El texto reconstruye el contexto político-cultural en que surgió el megaevento ideado por Luis Lama: el régimen fujimorista, el programa municipal «Volver al Centro» y el Plan Maestro del Centro Histórico impulsado por la gestión de Alberto Andrade, articulados con redes internacionales (UCCI, CIDEU) y el título de «Lima, Capital de la Cultura Iberoamericana». Peralta sostiene que la Bienal (1997-2002), en sus versiones nacional e iberoamericana, funcionó como núcleo de reactivación cultural y descentralización mediante salones regionales, atrajo atención internacional y sirvió de modelo de gestión, pero fue cancelada por desinterés político —especialmente de Luis Castañeda Lossio— y por la incapacidad del propio medio artístico de defender su función social. Documenta episodios polémicos: la crítica de Alfonso Castrillón a la autoría de una obra de García Zapatero, la performance «Señorita de buena presencia busca empleo» de Elena Tejada, la muestra paralela «Emergencia Artística» (1999) gestada por Emilio Santisteban y Gustavo Buntinx tras el veto a «Crisis», y la intervención «Chalk» de Allora &amp; Calzadilla, resignificada por trabajadores municipales. A través de testimonios (Santisteban, Élida Román, Natalia Velit, el propio Lama), el autor argumenta que la orfandad cultural persiste por la ausencia de políticas públicas y la subordinación al mercado. El texto se posiciona a favor de una gestión cultural audaz, descentralizada y socialmente participativa, lamentando que nada haya reemplazado la escala y el alcance de la Bienal.</t>
         </is>
       </c>
     </row>
@@ -1886,27 +1886,27 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>QUEHACER 19_watermark_p120-128.pdf</t>
+          <t>Ponencia - Villacorta, Jorge - Puntos cardinales (2019) [CEdA].transcripcion.txt</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>1940-1982 (arte peruano del siglo XX: indigenismo, velasquismo y transición belaundista)</t>
+          <t>1979-2019 (énfasis en 2001-2019: obra de los ochenta y ARCO 2019)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Entrevista en revista (Quehacer n.º 19, DESCO), ca. 1982</t>
+          <t>Transcripción de ponencia/conferencia, 2019 (Fundación SEDA-CEdA, Santiago)</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Mirko Lauer; Sebastián Gris; Juan Acha; DESCO; Alfonso Castrillón; José Sabogal; Josué Sánchez; Ramiro Llona; José Carlos Ramos; Joaquín López Antay; Fernando de Szyszlo; Juan Manuel Ugarte Eléspuru; Bienal de Medellín</t>
+          <t>Jorge Villacorta; Sebastián Vidal; Fundación SEDA; Sandra Gamarra (LiMac); Juan Javier Salazar; Herbert Rodríguez; Rodrigo Quijano; grupo Huayco; MALI; Fundación Reina Sofía; ARCOmadrid; galería Enrique Faria; galería Revólver; Alexis Fabri</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Entrevista de Sebastián Gris a Mirko Lauer publicada en la revista Quehacer (n.º 19, DESCO) bajo el título 'Está naciendo algo…'. El diálogo presenta el giro teórico de Lauer —poeta y crítico literario— hacia una teoría social de la cultura y del objeto plástico, formulada en su libro 'Crítica de la artesanía' y anticipada, junto al ausente Juan Acha, en el Coloquio de Arte No-objetual de Medellín. Lauer relee su 'Introducción a la pintura peruana del siglo XX': sostiene que hacia 1960 culmina, con la 'Teoría de las Raíces Nacionales', el ciclo abierto por el indigenismo de Sabogal, mientras los años setenta traen la revaloración del arte popular y su confluencia con una tradición artesanal. Critica el neo-indigenismo como coartada del populismo velasquista y de la Reforma Agraria: un país que, sin atreverse a enfrentar lo popular real, se inventa un seudo-país mistificado (el 'colmenazo', el arte turístico de José Carlos Ramos). Diagnostica, tras la restauración belaundista (posterior a 1977), una 'pérdida de direccionalidad' y un caos del mercado que ahora impone valor. Discute los límites de la propuesta conceptual y no-objetual, el Premio Nacional López Antay y la labor de Alfonso Castrillón, y reivindica la crítica de arte como oficio concreto —ni estética idealista ni 'estética marxista'—. Finalmente aborda la marginalidad y el desprecio hacia el intelectual peruano. Aparecen Josué Sánchez, Ramiro Llona, Szyszlo, Ugarte Eléspuru y la Bienal de Medellín. Su aporte es proponer el estudio del objeto plástico desde su existencia social y desde una perspectiva popular.</t>
+          <t>Transcripción de una ponencia de Jorge Villacorta en la Fundación SEDA (Santiago de Chile), presentada por Sebastián Vidal, en el marco de su participación en el pabellón peruano de ARCOmadrid 2019. Partiendo de dos exposiciones fundacionales de Sandra Gamarra (Living Room, 2001; el proyecto LiMac, 2002), Villacorta reflexiona sobre la desconexión histórica del sistema del arte limeño respecto del circuito internacional y su condición estructuralmente «coja». El eje del argumento es un contraste entre dos artistas del grupo Huayco: Juan Javier Salazar y Herbert Rodríguez. Salazar, considerado durante dos décadas el artista contemporáneo peruano por excelencia (Perú País del Mañana, El cuartucho, los náufragos), cultivó una obra frágil, localista y ácida sobre la desidia nacional, pero fue «maltratado» tras su muerte: descartado en ARCO 2019, cosmetizado en la Bienal de Venecia 2017 y regateado por el capítulo peruano de la Fundación Reina Sofía. Rodríguez, artista afrodescendiente y sistemático archivista de su obra (fotocopias, murales antisenderistas en San Marcos, fotoserigrafía), experimenta en cambio un ascenso internacional inesperado (galería Enrique Faria, Reina Sofía, Fundación Cartier), pese al desdén histórico del medio limeño y del MALI. Villacorta articula estas trayectorias con una crítica al coleccionismo peruano, a la lógica del mercado (galería Revólver, ferias, matching funds de arteBA), a la desatención de la crítica y las galerías, y a las jerarquías raciales y clasistas del establishment cultural limeño (Szyszlo, Armando Andrade). El texto plantea el problema del legado, el valor simbólico y la posibilidad de un arte con «testigos» frente a un arte subordinado al mercado.</t>
         </is>
       </c>
     </row>
@@ -1918,27 +1918,27 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Román, Elida - I Bienal Nacional de Lima. Algunos deslindes.md</t>
+          <t>Por Qué no vivo en el Perú.md</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>1997-1998 (I Bienal Nacional de Lima; referencias a 1987 y 1997)</t>
+          <t>ca. 1972 en adelante (emigración de Juan Acha a México y comparación Perú/México de los años setenta)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Artículo/reseña crítica, 1998</t>
+          <t>Encuesta/testimonio en revista literaria (Hueso Húmero), ca. 1980; transcripción en Markdown, s/f</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Élida Román; Luis Lama; UCCI; Municipalidad Metropolitana de Lima; Centro de Artes Visuales (CAV); Virginia Pérez-Ratton; Museo de Arte de Lima; Luz María Bedoya; Mariella Agois; Bienal de Trujillo</t>
+          <t>Juan Acha; revista Hueso Húmero; museos, institutos y universidades de México</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Nota crítica de la crítica de arte Élida Román sobre la I Bienal Nacional de Lima (1998), que deslinda sus antecedentes y examina su lógica organizativa. Román recuerda que un evento similar existió en la III Bienal de Trujillo (1987) con el núcleo «Mirada hacia adentro», y sitúa la Bienal Nacional como mecanismo para seleccionar —mediante salones regionales y comités— la representación peruana a la II Bienal Iberoamericana. Enmarca el evento en el proyecto municipal de recuperación del Centro Histórico y en la designación de Lima como «Plaza Mayor de la Cultura Iberoamericana» por la UCCI, señalando el apresuramiento organizativo y los defectos museográficos derivados del uso de casonas no adecuadas a fines museológicos. Su argumento central cuestiona el discurso «modernizador» y globalizador de los organizadores (Luis Lama), advirtiendo que tras las nociones de ruptura, novedad y globalización se esconden la moda, el esnobismo y «roles forzados» e intereses extraculturales. Critica el centralismo y paternalismo de los salones regionales, que perpetúan la posición privilegiada de Lima sin una política real de desarrollo en provincias. Román reclama definir los propósitos de la actividad artística e interroga la falsa dicotomía entre arte «popular» y «culto», recordando la polémica por el Premio Nacional otorgado a un artesano ayacuchano. Frente a la comparación con estándares metropolitanos, aboga por una modernidad entendida como apertura multidisciplinaria y actitud cohesionadora e identitaria, apoyada en la historia, la antropología y las ciencias sociales. El texto, denso en interrogantes, defiende la reflexión teórica y el debate, y cierra evocando la consigna «¡La imaginación al poder!».</t>
+          <t>Transcripción de la respuesta de Juan Acha a la encuesta 'Por qué no vivo en el Perú', iniciada por la revista Hueso Húmero para indagar las razones del éxodo de creadores e intelectuales peruanos. Acha —crítico y teórico del arte dedicado a los problemas latinoamericanos, radicado en México— distingue razones 'de afuera' y 'de adentro', otorgando mayor peso a las primeras: sólo abandona su país quien encuentra en otro las condiciones para desarrollar con dignidad su trabajo profesional, mientras que las circunstancias personales o los factores nacionales negativos serían secundarios en su caso. Enumera lo que México le ofreció y el Perú le negaba: amplias posibilidades de publicar en diarios y revistas, de colaborar en museos e institutos y de investigar y enseñar en universidades, todo ello remunerado con dignidad; libertad de expresión intelectual e intensa circulación de ideas marxistas en libros, revistas y simposios; prestigio nacional de las artes visuales con apoyo estatal, política museográfica y de simposios activa, y facilidades para viajar y contactar con el arte de otras latitudes. Valora, además, el mejor enfoque de los problemas artísticos y culturales latinoamericanos posible desde México, cuya escala demográfica y potente industria editorial concentran las investigaciones de toda la región y anticipan fenómenos que luego se difunden. El testimonio —que el archivo conserva incompleto, interrumpido al mencionar una 'identificación cultural más conflictiva y acorde a la realidad concreta'— condensa la autojustificación del exilio intelectual como decisión productiva antes que como queja, y funciona como documento sobre las carencias institucionales del campo artístico peruano frente a las condiciones del México de esos años.</t>
         </is>
       </c>
     </row>
@@ -1950,27 +1950,27 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Screen Shot 2026-07-16 at 08.22.07.png</t>
+          <t>QUEHACER 19_watermark_p120-128.pdf</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>1980-1981 (obra 'Arte al Paso' y culto vigente a Sarita Colonia); Sarita Colonia 1914-1940</t>
+          <t>1940-1982 (arte peruano del siglo XX: indigenismo, velasquismo y transición belaundista)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Captura de pantalla, 16-07-2026 (de artículo de la revista MARKA, Lima, 14-05-1981, p. 34; archivo UNMSM-CEDOC)</t>
+          <t>Entrevista en revista (Quehacer n.º 19, DESCO), ca. 1982</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Sarita Colonia; Taller de Estética de Proyección Social 'Huayco' (E.P.S. Huayco); Francisco Mariotti; María Luy; Gerbert Rodríguez; Mariella Zevallos; Armando Williams; Charo Noriega; revista MARKA; UNMSM-CEDOC</t>
+          <t>Mirko Lauer; Sebastián Gris; Juan Acha; DESCO; Alfonso Castrillón; José Sabogal; Josué Sánchez; Ramiro Llona; José Carlos Ramos; Joaquín López Antay; Fernando de Szyszlo; Juan Manuel Ugarte Eléspuru; Bienal de Medellín</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Captura de una página de la revista MARKA (Lima, 14 de mayo de 1981, p. 34; sello de archivo UNMSM-CEDOC) con el artículo 'La imagen y la fuerza milagrosa', dedicado al culto a Sarita Colonia y a su tratamiento en el arte. El texto interpreta la devoción popular a Sarita como caso patente de realización simbólica donde el elemento religioso se ensambla con el gusto estético popular, uniendo pensamiento mágico y realidad social inmediata; el símbolo religioso operaría como continente de mitos que resuelven imaginariamente las contradicciones de la vida. Recuerda que Sarita nació en Huaraz en 1914 y murió en el Callao en 1940, donde surgió su culto —hoy extendido entre los más desvalidos: el mundo del hampa, la prostitución, estibadores y choferes—, con un mausoleo-santuario rodeado de exvotos y comerciantes ambulantes. La sección 'Sarita en el arte' presenta y reproduce la obra 'Arte al Paso', un enorme rostro de Sarita compuesto con cerca de 12,000 latas de leche, realizado por un conjunto de artistas jóvenes reunidos en el Taller de Estética de Proyección Social 'Huayco' (E.P.S. Huayco): Francisco Mariotti, María Luy, Gerbert Rodríguez, Mariella Zevallos, Armando Williams y Charo Noriega. Instalada desde enero de ese año a la vera del sur, la obra recoge en clave colectiva la significación sociocultural de Sarita para ofrecer a viajeros y peregrinos una exposición permanente de esa imagen, integrando la escala monumental, la soledad del paisaje y una identificación plástica con el misterio cotidiano. Es documento clave sobre el vínculo entre religiosidad popular, migración andina y vanguardia peruana de inicios de los ochenta.</t>
+          <t>Entrevista de Sebastián Gris a Mirko Lauer publicada en la revista Quehacer (n.º 19, DESCO) bajo el título 'Está naciendo algo…'. El diálogo presenta el giro teórico de Lauer —poeta y crítico literario— hacia una teoría social de la cultura y del objeto plástico, formulada en su libro 'Crítica de la artesanía' y anticipada, junto al ausente Juan Acha, en el Coloquio de Arte No-objetual de Medellín. Lauer relee su 'Introducción a la pintura peruana del siglo XX': sostiene que hacia 1960 culmina, con la 'Teoría de las Raíces Nacionales', el ciclo abierto por el indigenismo de Sabogal, mientras los años setenta traen la revaloración del arte popular y su confluencia con una tradición artesanal. Critica el neo-indigenismo como coartada del populismo velasquista y de la Reforma Agraria: un país que, sin atreverse a enfrentar lo popular real, se inventa un seudo-país mistificado (el 'colmenazo', el arte turístico de José Carlos Ramos). Diagnostica, tras la restauración belaundista (posterior a 1977), una 'pérdida de direccionalidad' y un caos del mercado que ahora impone valor. Discute los límites de la propuesta conceptual y no-objetual, el Premio Nacional López Antay y la labor de Alfonso Castrillón, y reivindica la crítica de arte como oficio concreto —ni estética idealista ni 'estética marxista'—. Finalmente aborda la marginalidad y el desprecio hacia el intelectual peruano. Aparecen Josué Sánchez, Ramiro Llona, Szyszlo, Ugarte Eléspuru y la Bienal de Medellín. Su aporte es proponer el estudio del objeto plástico desde su existencia social y desde una perspectiva popular.</t>
         </is>
       </c>
     </row>
@@ -1982,27 +1982,27 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Screen Shot 2026-07-16 at 08.37.09.png</t>
+          <t>Román, Elida - I Bienal Nacional de Lima. Algunos deslindes.md</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>1965-1984</t>
+          <t>1997-1998 (I Bienal Nacional de Lima; referencias a 1987 y 1997)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Captura de pantalla, 16-07-2026 (de un cuadro/gráfico basado en el informe de Alfonso Castrillón, 'Reflexiones sobre el arte conceptual en el Perú y sus proyecciones', Hueso Húmero n.º 7; sello UNMSM)</t>
+          <t>Artículo/reseña crítica, 1998</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Alfonso Castrillón; Juan Acha; Teresa Burga; Emilio Hernández; Rafael Hastings; Francisco Mariotti; Luis Arias Vera; Jorge Eielson; Wiley Ludeña; Herbert Rodríguez; E.P.S. Huayco; Grupo Paréntesis; UNMSM</t>
+          <t>Élida Román; Luis Lama; UCCI; Municipalidad Metropolitana de Lima; Centro de Artes Visuales (CAV); Virginia Pérez-Ratton; Museo de Arte de Lima; Luz María Bedoya; Mariella Agois; Bienal de Trujillo</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Captura de pantalla de un cuadro cronológico ('Gráfico 1') que sistematiza el desarrollo del arte conceptual y no-objetual en el Perú entre 1965 y 1984, elaborado 'en base al informe de Alfonso Castrillón: Reflexiones sobre el arte conceptual en el Perú y sus proyecciones' (Hueso Húmero 7). El cuadro organiza la información en cuatro columnas —Fecha, Tendencia, Operador (artistas y grupos) y Lugar— trazando la sucesión de tendencias: pop y op (1965, Galería Lima, IAC), concepto y ambientes (1969-1970, con Juan Acha, 'Cultura y Libertad'), acciones y eventos (1972-1975: Teresa Burga, Rafael Hastings, Francisco Mariotti, CONTACTA, Premio López Antay, Festival Inkarri), y las prácticas de no-objeto y performance de fines de los setenta y de los ochenta. Registra los colectivos 'Signo x signo' (Patricia López, Armando Williams, Rossana Agois, Wiley Ludeña, Hugo Salazar), el Grupo USM de Alfonso Castrillón, 'Paréntesis' (Charo Noriega, Armando Williams, María Luy, Francisco Mariotti, Fernando Bedoya, Juan J. Salazar, Mariela Zevallos) y 'Huayco EPS' (Herbert Rodríguez, Lucy Angulo, José Morales), junto a nombres como Luis Arias Vera, Emilio Hernández, Jorge Eielson, Hernán Pazos, Esther Vainstein, Cecilia Paredes y Sergio Zevallos. Consigna hitos y sedes: encuestas, la Bienal no-objetual de Medellín, la Bienal de São Paulo (1983), la acción 'Cuidado pintores…', y espacios como el Instituto Italiano, la Universidad de San Marcos y galerías limeñas. Funciona como mapa genealógico de la vanguardia experimental peruana y de sus operadores institucionales, útil para periodizar el paso del conceptualismo a la performance y al arte no-objetual.</t>
+          <t>Nota crítica de la crítica de arte Élida Román sobre la I Bienal Nacional de Lima (1998), que deslinda sus antecedentes y examina su lógica organizativa. Román recuerda que un evento similar existió en la III Bienal de Trujillo (1987) con el núcleo «Mirada hacia adentro», y sitúa la Bienal Nacional como mecanismo para seleccionar —mediante salones regionales y comités— la representación peruana a la II Bienal Iberoamericana. Enmarca el evento en el proyecto municipal de recuperación del Centro Histórico y en la designación de Lima como «Plaza Mayor de la Cultura Iberoamericana» por la UCCI, señalando el apresuramiento organizativo y los defectos museográficos derivados del uso de casonas no adecuadas a fines museológicos. Su argumento central cuestiona el discurso «modernizador» y globalizador de los organizadores (Luis Lama), advirtiendo que tras las nociones de ruptura, novedad y globalización se esconden la moda, el esnobismo y «roles forzados» e intereses extraculturales. Critica el centralismo y paternalismo de los salones regionales, que perpetúan la posición privilegiada de Lima sin una política real de desarrollo en provincias. Román reclama definir los propósitos de la actividad artística e interroga la falsa dicotomía entre arte «popular» y «culto», recordando la polémica por el Premio Nacional otorgado a un artesano ayacuchano. Frente a la comparación con estándares metropolitanos, aboga por una modernidad entendida como apertura multidisciplinaria y actitud cohesionadora e identitaria, apoyada en la historia, la antropología y las ciencias sociales. El texto, denso en interrogantes, defiende la reflexión teórica y el debate, y cierra evocando la consigna «¡La imaginación al poder!».</t>
         </is>
       </c>
     </row>
@@ -2014,27 +2014,27 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Screen Shot 2026-07-16 at 13.03.35.png</t>
+          <t>Screen Shot 2026-07-16 at 08.22.07.png</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>1970-1981</t>
+          <t>1980-1981 (obra 'Arte al Paso' y culto vigente a Sarita Colonia); Sarita Colonia 1914-1940</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Captura de pantalla (16-07-2026) de artículo de revista, 1981</t>
+          <t>Captura de pantalla, 16-07-2026 (de artículo de la revista MARKA, Lima, 14-05-1981, p. 34; archivo UNMSM-CEDOC)</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Juan Acha; Hueso Húmero (revista); UNMSM; José Carlos Mariátegui (contexto marxista); El Sexto (prisión); México D.F.</t>
+          <t>Sarita Colonia; Taller de Estética de Proyección Social 'Huayco' (E.P.S. Huayco); Francisco Mariotti; María Luy; Gerbert Rodríguez; Mariella Zevallos; Armando Williams; Charo Noriega; revista MARKA; UNMSM-CEDOC</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>La captura reproduce la primera página del texto autobiográfico y ensayístico de Juan Acha titulado 'Por qué no vivo en el Perú', encabezado por una nota editorial de la revista Hueso Húmero que enmarca el escrito dentro de una indagación colectiva sobre los creadores e intelectuales peruanos que optaron por emigrar, problema que la publicación se propone tratar con seriedad y continuar en números sucesivos. Acha, crítico y teórico del arte dedicado a los problemas latinoamericanos, ordena sus razones para no residir en el Perú en dos clases jerarquizadas: las 'de afuera', que considera principales, y las 'de adentro', secundarias. Bajo las primeras enumera lo que encontró en México y le faltaba en su país: amplias posibilidades de publicar en diarios y revistas, colaborar en museos e institutos, investigar y enseñar en universidades como crítico de arte, todo ello remunerado con dignidad; libertad de expresión e intensa circulación de ideas marxistas en libros, revistas y simposios; y un prestigio nacional de las artes visuales sostenido por el Estado, con una activa política museográfica y de simposios además de facilidades para viajar y entrar en contacto con el arte de otras latitudes. El fragmento evidencia la tesis central del autor: la emigración no responde a un rechazo personal sino a la asimetría estructural entre el medio cultural peruano, precario y cerrado, y el mexicano, mejor equipado y más poroso al quehacer cultural latinoamericano. El documento funciona como fuente primaria sobre las condiciones institucionales del campo artístico peruano y sobre la trayectoria del propio Acha como figura clave de la teoría del arte no objetual en América Latina.</t>
+          <t>Captura de una página de la revista MARKA (Lima, 14 de mayo de 1981, p. 34; sello de archivo UNMSM-CEDOC) con el artículo 'La imagen y la fuerza milagrosa', dedicado al culto a Sarita Colonia y a su tratamiento en el arte. El texto interpreta la devoción popular a Sarita como caso patente de realización simbólica donde el elemento religioso se ensambla con el gusto estético popular, uniendo pensamiento mágico y realidad social inmediata; el símbolo religioso operaría como continente de mitos que resuelven imaginariamente las contradicciones de la vida. Recuerda que Sarita nació en Huaraz en 1914 y murió en el Callao en 1940, donde surgió su culto —hoy extendido entre los más desvalidos: el mundo del hampa, la prostitución, estibadores y choferes—, con un mausoleo-santuario rodeado de exvotos y comerciantes ambulantes. La sección 'Sarita en el arte' presenta y reproduce la obra 'Arte al Paso', un enorme rostro de Sarita compuesto con cerca de 12,000 latas de leche, realizado por un conjunto de artistas jóvenes reunidos en el Taller de Estética de Proyección Social 'Huayco' (E.P.S. Huayco): Francisco Mariotti, María Luy, Gerbert Rodríguez, Mariella Zevallos, Armando Williams y Charo Noriega. Instalada desde enero de ese año a la vera del sur, la obra recoge en clave colectiva la significación sociocultural de Sarita para ofrecer a viajeros y peregrinos una exposición permanente de esa imagen, integrando la escala monumental, la soledad del paisaje y una identificación plástica con el misterio cotidiano. Es documento clave sobre el vínculo entre religiosidad popular, migración andina y vanguardia peruana de inicios de los ochenta.</t>
         </is>
       </c>
     </row>
@@ -2046,27 +2046,27 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Screen Shot 2026-07-16 at 13.03.44.png</t>
+          <t>Screen Shot 2026-07-16 at 08.37.09.png</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>1970-1981</t>
+          <t>1965-1984</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Captura de pantalla (16-07-2026) de artículo de revista, 1981</t>
+          <t>Captura de pantalla, 16-07-2026 (de un cuadro/gráfico basado en el informe de Alfonso Castrillón, 'Reflexiones sobre el arte conceptual en el Perú y sus proyecciones', Hueso Húmero n.º 7; sello UNMSM)</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Juan Acha; Hueso Húmero (revista); El Sexto (prisión de Lima); México D.F.; UNMSM</t>
+          <t>Alfonso Castrillón; Juan Acha; Teresa Burga; Emilio Hernández; Rafael Hastings; Francisco Mariotti; Luis Arias Vera; Jorge Eielson; Wiley Ludeña; Herbert Rodríguez; E.P.S. Huayco; Grupo Paréntesis; UNMSM</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>La captura corresponde a la página 109 (sección 'Encuesta') y continúa el texto de Juan Acha 'Por qué no vivo en el Perú', cerrando la argumentación iniciada en la página anterior. Bajo las razones 'de afuera' Acha añade dos motivos vinculados a su vocación latinoamericanista: México ofrece un mejor enfoque de los problemas artísticos y culturales de 'nuestra América' porque, por su tamaño demográfico e importancia y por su industria editora, allí confluyen antes que en otros países los fenómenos y las investigaciones del resto de Latinoamérica; y propicia una identificación cultural más conflictiva y acorde a la realidad concreta, con un aprecio por la cultura popular en la que halla semejanzas con el Perú. Luego expone tres razones 'secundarias', personales, que lo empujaron a salir: haber vivido y formado universitariamente fuera del país trabajando como químico en varios países latinoamericanos, lo que facilitó su salida y le dio mejor visión de virtudes y defectos nacionales; el clima represivo y discriminante de la capital, producto del 'aristocratismo limeño' y su racismo disimulado, del nepotismo de las clases dominantes y la represión de lo popular; y, sobre todo, haber sido fichado en 1970 como supuesto inculpado de tráfico de drogas al asistir a una fiesta de artistas jóvenes, sufriendo diez días de vejaciones en la prisión El Sexto por negligencia judicial antes de ser declarado inocente. El texto, firmado en México D.F. en febrero de 1981, articula crítica estructural del campo cultural peruano con testimonio personal de exclusión y violencia institucional.</t>
+          <t>Captura de pantalla de un cuadro cronológico ('Gráfico 1') que sistematiza el desarrollo del arte conceptual y no-objetual en el Perú entre 1965 y 1984, elaborado 'en base al informe de Alfonso Castrillón: Reflexiones sobre el arte conceptual en el Perú y sus proyecciones' (Hueso Húmero 7). El cuadro organiza la información en cuatro columnas —Fecha, Tendencia, Operador (artistas y grupos) y Lugar— trazando la sucesión de tendencias: pop y op (1965, Galería Lima, IAC), concepto y ambientes (1969-1970, con Juan Acha, 'Cultura y Libertad'), acciones y eventos (1972-1975: Teresa Burga, Rafael Hastings, Francisco Mariotti, CONTACTA, Premio López Antay, Festival Inkarri), y las prácticas de no-objeto y performance de fines de los setenta y de los ochenta. Registra los colectivos 'Signo x signo' (Patricia López, Armando Williams, Rossana Agois, Wiley Ludeña, Hugo Salazar), el Grupo USM de Alfonso Castrillón, 'Paréntesis' (Charo Noriega, Armando Williams, María Luy, Francisco Mariotti, Fernando Bedoya, Juan J. Salazar, Mariela Zevallos) y 'Huayco EPS' (Herbert Rodríguez, Lucy Angulo, José Morales), junto a nombres como Luis Arias Vera, Emilio Hernández, Jorge Eielson, Hernán Pazos, Esther Vainstein, Cecilia Paredes y Sergio Zevallos. Consigna hitos y sedes: encuestas, la Bienal no-objetual de Medellín, la Bienal de São Paulo (1983), la acción 'Cuidado pintores…', y espacios como el Instituto Italiano, la Universidad de San Marcos y galerías limeñas. Funciona como mapa genealógico de la vanguardia experimental peruana y de sus operadores institucionales, útil para periodizar el paso del conceptualismo a la performance y al arte no-objetual.</t>
         </is>
       </c>
     </row>
@@ -2078,27 +2078,27 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>VVAA - El desencantamiento del arte. Conversación de egresados con Jorge Villacorta [Ansible].md</t>
+          <t>Screen Shot 2026-07-16 at 13.03.35.png</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>2013-2018 (coyuntura reciente, con referencias a los años ochenta)</t>
+          <t>1970-1981</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Conversación colectiva publicada en revista (Ansible), ca. 2018 (s/f exacta)</t>
+          <t>Captura de pantalla (16-07-2026) de artículo de revista, 1981</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Adriana Bickel; Rafael Nolte; Rox Monteverde; Kenji Quispe; Mariana Román; Raúl Silva; Michael Prado; Alfredo Bernal; PUCP; ENSABAP; Corriente Alterna; Centro de la Imagen; galería 80m2 Livia Benavides; Revolver; Mario Testino; Rodrigo Quijano</t>
+          <t>Juan Acha; Hueso Húmero (revista); UNMSM; José Carlos Mariátegui (contexto marxista); El Sexto (prisión); México D.F.</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Conversación colectiva entre egresados y estudiantes recientes de las principales escuelas de artes visuales de Lima (PUCP, ENSABAP-Bellas Artes, Corriente Alterna, Centro de la Imagen), con intervención del crítico Jorge Villacorta, publicada en la revista Ansible. El diálogo diagnostica un momento de «desencantamiento» e inflexión entre un pasado precario y un futuro incierto en el campo laboral del arte. Los participantes (Adriana Bickel, Rafael Nolte, Rox Monteverde, Kenji Quispe, Mariana Román, Raúl Silva, Michael Prado, Alfredo Bernal) analizan factores recientes: el surgimiento de ferias (P.Ar.C., Art Lima), la internacionalización de galerías (Revolver, 80m2 Livia Benavides), las vanity gallery, el coleccionismo concentrado de Hochschild y Verme, el libro de Mario Testino, la gentrificación de Monumental Callao y el escándalo del pabellón peruano en la Bienal de Venecia 2017 (obra de Juan Javier Salazar, retirada del curador Rodrigo Quijano). El eje conceptual gira en torno al mercado como fuerza hegemónica que guía la cultura, la ausencia de aparato crítico e histórico, el auge de la autogestión como «arma de doble filo» y la imposibilidad de agremiación en un medio fragmentado y competitivo. Villacorta aporta la memoria histórica de la ASPAP (años ochenta) y el contraste con la colegiatura profesional y la AICA. Se debaten la profesionalización, la legitimación externa del artista (por sociólogos, curadores, museos), la deficiente formación que provoca el éxodo de artistas, los cambios curriculares hacia el «artista-investigador» (2010-2011) y lo aspiracional del éxito comercial. El texto expone críticamente la vulnerabilidad estructural del artista joven limeño.</t>
+          <t>La captura reproduce la primera página del texto autobiográfico y ensayístico de Juan Acha titulado 'Por qué no vivo en el Perú', encabezado por una nota editorial de la revista Hueso Húmero que enmarca el escrito dentro de una indagación colectiva sobre los creadores e intelectuales peruanos que optaron por emigrar, problema que la publicación se propone tratar con seriedad y continuar en números sucesivos. Acha, crítico y teórico del arte dedicado a los problemas latinoamericanos, ordena sus razones para no residir en el Perú en dos clases jerarquizadas: las 'de afuera', que considera principales, y las 'de adentro', secundarias. Bajo las primeras enumera lo que encontró en México y le faltaba en su país: amplias posibilidades de publicar en diarios y revistas, colaborar en museos e institutos, investigar y enseñar en universidades como crítico de arte, todo ello remunerado con dignidad; libertad de expresión e intensa circulación de ideas marxistas en libros, revistas y simposios; y un prestigio nacional de las artes visuales sostenido por el Estado, con una activa política museográfica y de simposios además de facilidades para viajar y entrar en contacto con el arte de otras latitudes. El fragmento evidencia la tesis central del autor: la emigración no responde a un rechazo personal sino a la asimetría estructural entre el medio cultural peruano, precario y cerrado, y el mexicano, mejor equipado y más poroso al quehacer cultural latinoamericano. El documento funciona como fuente primaria sobre las condiciones institucionales del campo artístico peruano y sobre la trayectoria del propio Acha como figura clave de la teoría del arte no objetual en América Latina.</t>
         </is>
       </c>
     </row>
@@ -2110,27 +2110,27 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>VVAA - Lima se anima. Debates en la escena artística peruana (2009) [ramona 89].md</t>
+          <t>Screen Shot 2026-07-16 at 13.03.44.png</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>1997-2009 (última década, de la Bienal Iberoamericana al presente)</t>
+          <t>1970-1981</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Dossier de revista (ramona nº 89), abril 2009</t>
+          <t>Captura de pantalla (16-07-2026) de artículo de revista, 1981</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Quijano; Eliana Otta; Miguel López; Max Hernández-Calvo; Gustavo Buntinx; Jorge Villacorta; Alfredo Márquez; Fernando Bryce; Gilda Mantilla; Philippe Gruenberg; Giancarlo Scaglia; revista Juanacha; La Culpable; MALI; galería Revólver</t>
+          <t>Juan Acha; Hueso Húmero (revista); El Sexto (prisión de Lima); México D.F.; UNMSM</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Dossier «Lima se anima» de la revista argentina ramona (nº 89, abril 2009), coeditado con la publicación limeña Juanacha por Rodrigo Quijano y Eliana Otta, que ofrece una radiografía crítica de la escena artística peruana ante su reciente revinculación con el circuito internacional. Reúne una conversación entre artistas («Perú, ¿país blindado?») con Alfredo Márquez, Fernando Bryce, Gilda Mantilla, Philippe Gruenberg y Giancarlo Scaglia; ensayos de Miguel López y Max Hernández-Calvo; un debate virtual del blog Arte-Nuevo sobre las políticas museales; un texto de Gustavo Buntinx (Micromuseo) y una entrevista a Jorge Villacorta. El hilo común es la interrogación del supuesto «boom» del arte contemporáneo limeño de la última década: los participantes coinciden en que la internacionalización y el crecimiento del mercado y del coleccionismo (impulsado por el MALI) han producido una escena «contrahecha», con brazos de mercado pero sin instituciones, crítica, educación ni políticas culturales. Márquez denuncia el carácter colonial y exótico de esa visibilidad; López («Boo(o)m: Morir de éxito») teoriza un proceso de despolitización y domesticación que diluye el conflicto y convierte la autonomía en aquiescencia entre agentes; Hernández-Calvo («Una coyuntura que no fue») analiza cómo las Bienales de Lima (1997-2002) forzaron una «contemporaneización» de instalación y video sin sustento curatorial ni educativo, generando escisiones entre circuito oficial y alternativo. Se abordan además el éxodo de artistas por la deficiente formación, la toma estudiantil de Bellas Artes, la autogestión (La Culpable) y las disputas por el Museo de la Memoria. El dossier reivindica la autonomía, el disenso y el filo crítico histórico del arte peruano.</t>
+          <t>La captura corresponde a la página 109 (sección 'Encuesta') y continúa el texto de Juan Acha 'Por qué no vivo en el Perú', cerrando la argumentación iniciada en la página anterior. Bajo las razones 'de afuera' Acha añade dos motivos vinculados a su vocación latinoamericanista: México ofrece un mejor enfoque de los problemas artísticos y culturales de 'nuestra América' porque, por su tamaño demográfico e importancia y por su industria editora, allí confluyen antes que en otros países los fenómenos y las investigaciones del resto de Latinoamérica; y propicia una identificación cultural más conflictiva y acorde a la realidad concreta, con un aprecio por la cultura popular en la que halla semejanzas con el Perú. Luego expone tres razones 'secundarias', personales, que lo empujaron a salir: haber vivido y formado universitariamente fuera del país trabajando como químico en varios países latinoamericanos, lo que facilitó su salida y le dio mejor visión de virtudes y defectos nacionales; el clima represivo y discriminante de la capital, producto del 'aristocratismo limeño' y su racismo disimulado, del nepotismo de las clases dominantes y la represión de lo popular; y, sobre todo, haber sido fichado en 1970 como supuesto inculpado de tráfico de drogas al asistir a una fiesta de artistas jóvenes, sufriendo diez días de vejaciones en la prisión El Sexto por negligencia judicial antes de ser declarado inocente. El texto, firmado en México D.F. en febrero de 1981, articula crítica estructural del campo cultural peruano con testimonio personal de exclusión y violencia institucional.</t>
         </is>
       </c>
     </row>
@@ -2142,27 +2142,27 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>VVAA - Memorias del subdesarrollo. Arte y el giro descolonial en América Latina, 1960-1985 [catálogo MCASD].md</t>
+          <t>VVAA - El desencantamiento del arte. Conversación de egresados con Jorge Villacorta [Ansible].md</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>1960-1985 (con foco 1967-1981)</t>
+          <t>2013-2018 (coyuntura reciente, con referencias a los años ochenta)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de exposición / ensayo académico, 2018 (MCASD)</t>
+          <t>Conversación colectiva publicada en revista (Ansible), ca. 2018 (s/f exacta)</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Julieta González; Andrea Giunta; Jacopo Crivelli Visconti; Juan Acha; Marta Traba; Ferreira Gullar; Teresa Burga; E.P.S. Huayco; Grupo Paréntesis; Jesús Ruiz Durand; Fernando 'Coco' Bedoya; MALI; Museum of Contemporary Art San Diego</t>
+          <t>Jorge Villacorta; Adriana Bickel; Rafael Nolte; Rox Monteverde; Kenji Quispe; Mariana Román; Raúl Silva; Michael Prado; Alfredo Bernal; PUCP; ENSABAP; Corriente Alterna; Centro de la Imagen; galería 80m2 Livia Benavides; Revolver; Mario Testino; Rodrigo Quijano</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>El ensayo de Sharon Lerner incluido en el catálogo de la exposición 'Memorias del subdesarrollo: arte y el giro descolonial en América Latina, 1960-1985' inserta la escena peruana de 1967-1981 en una narrativa continental que postula una ruptura epistémica con lo moderno mediante la noción de subdesarrollo y el deseo de descolonizar los cánones estéticos impuestos. Su tesis desplaza el foco del paradigma formalista modernista hacia el contexto social, la apropiación de tradiciones locales y lo 'popular' como categoría clave, cuya heterogeneidad histórica advierte no homogeneizar. Reconstruye el debate entre Juan Acha y Marta Traba sobre el pop cosmopolita y la dependencia cultural, apoyándose en Mariátegui, Ferreira Gullar y Mário Pedrosa, y en la teoría de la dependencia. Analiza casos peruanos: los afiches de la Reforma Agraria de Jesús Ruiz Durand y su 'pop achorado' dentro de SINAMOS; los festivales Contacta y las Carreras de Chasquis de Luis Arias Vera bajo el velasquismo; el Grupo Paréntesis y el Contacta 79 (Becerro de oro, Coquito) de Fernando Bedoya; y sobre todo E.P.S. Huayco, con 'Arte al paso (Salchipapas)' y 'Sarita Colonia', leídos vía Buntinx y Lauer como articulación de lo popular urbano migrante. Suma el caso aislado de Teresa Burga y 'Perfil de la mujer peruana' (1980-81) como acercamiento conceptual a género y clase. Recurriendo a Bürger y Giunta, discute la definición de vanguardia y concluye que estas prácticas oscilaron entre dependencia y autonomía, sin lograr plataformas de continuidad, siendo Huayco el caso más próximo a una vanguardia local pese a su disolución.</t>
+          <t>Conversación colectiva entre egresados y estudiantes recientes de las principales escuelas de artes visuales de Lima (PUCP, ENSABAP-Bellas Artes, Corriente Alterna, Centro de la Imagen), con intervención del crítico Jorge Villacorta, publicada en la revista Ansible. El diálogo diagnostica un momento de «desencantamiento» e inflexión entre un pasado precario y un futuro incierto en el campo laboral del arte. Los participantes (Adriana Bickel, Rafael Nolte, Rox Monteverde, Kenji Quispe, Mariana Román, Raúl Silva, Michael Prado, Alfredo Bernal) analizan factores recientes: el surgimiento de ferias (P.Ar.C., Art Lima), la internacionalización de galerías (Revolver, 80m2 Livia Benavides), las vanity gallery, el coleccionismo concentrado de Hochschild y Verme, el libro de Mario Testino, la gentrificación de Monumental Callao y el escándalo del pabellón peruano en la Bienal de Venecia 2017 (obra de Juan Javier Salazar, retirada del curador Rodrigo Quijano). El eje conceptual gira en torno al mercado como fuerza hegemónica que guía la cultura, la ausencia de aparato crítico e histórico, el auge de la autogestión como «arma de doble filo» y la imposibilidad de agremiación en un medio fragmentado y competitivo. Villacorta aporta la memoria histórica de la ASPAP (años ochenta) y el contraste con la colegiatura profesional y la AICA. Se debaten la profesionalización, la legitimación externa del artista (por sociólogos, curadores, museos), la deficiente formación que provoca el éxodo de artistas, los cambios curriculares hacia el «artista-investigador» (2010-2011) y lo aspiracional del éxito comercial. El texto expone críticamente la vulnerabilidad estructural del artista joven limeño.</t>
         </is>
       </c>
     </row>
@@ -2174,27 +2174,27 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Vich - La violencia, la dictadura y la globalización. Arte y política en el Perú contemporáneo.md</t>
+          <t>VVAA - Lima se anima. Debates en la escena artística peruana (2009) [ramona 89].md</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>1980-2009 (violencia política, dictadura fujimorista y posconflicto)</t>
+          <t>1997-2009 (última década, de la Bienal Iberoamericana al presente)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Ensayo / capítulo de libro académico, c. 2013-2015</t>
+          <t>Dossier de revista (ramona nº 89), abril 2009</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Víctor Vich; Eduardo Tokeshi; Colectivo Sociedad Civil; Natalia Iguíñiz; Sandro Venturo; Piero Quijano; Luz Letts; Víctor Delfín; Miguel Cordero; Jaime Higa; Herbert Rodríguez; Claudia Martínez; Santiago Quintanilla; Rudolph Castro; Felipe López; Gustavo Buntinx</t>
+          <t>Rodrigo Quijano; Eliana Otta; Miguel López; Max Hernández-Calvo; Gustavo Buntinx; Jorge Villacorta; Alfredo Márquez; Fernando Bryce; Gilda Mantilla; Philippe Gruenberg; Giancarlo Scaglia; revista Juanacha; La Culpable; MALI; galería Revólver</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>Víctor Vich propone una lectura desde la crítica cultural del arte peruano contemporáneo, sosteniendo que, frente al discurso triunfalista del crecimiento económico, un sector de artistas sigue nombrando al país a partir de sus heridas históricas. Estructura el ensayo en torno a tres acontecimientos: la violencia política, el autoritarismo corrupto del fujimontesinismo y la globalización neoliberal. Apoyándose en Žižek, Hall, Jameson, Foucault y Badiou, entiende lo simbólico no como reflejo sino como soporte de la realidad y campo de batalla donde se disputan sentidos de ciudadanía. Analiza obras emblemáticas: 'Bandera VIII' (2000) de Eduardo Tokeshi, leída como 'la patria en cuidados intensivos'; 'Lava la bandera' del Colectivo Sociedad Civil; la instalación 'Patria' de Natalia Iguíñiz y Sandro Venturo; el afiche censurado de Piero Quijano sobre La Cantuta e Iwo Jima; 'El azar como destino' de Luz Letts; 'El hermoso general' de Víctor Delfín; el saco militar de Miguel Cordero; y las serigrafías de César Vallejo de Jaime Higa sobre posmodernismo y cultura de masas. En una segunda sección sobre memoria generacional examina a artistas nacidos en los ochenta que 'traducen' la violencia con lenguajes heredados de la infancia: la serie 'Invisible' de Claudia Martínez, el trabajo de archivo y cómic de Santiago Quintanilla, los juguetes siniestros (Lego, Playmobil) de Rudolph Castro y las fotografías de nichos ayacuchanos de Felipe López. Su aporte es articular teoría psicoanalítica y poscolonial con un corpus visual peruano, mostrando el arte crítico como agente que interrumpe la ficción neoliberal y recompone la comunidad desde el orden simbólico.</t>
+          <t>Dossier «Lima se anima» de la revista argentina ramona (nº 89, abril 2009), coeditado con la publicación limeña Juanacha por Rodrigo Quijano y Eliana Otta, que ofrece una radiografía crítica de la escena artística peruana ante su reciente revinculación con el circuito internacional. Reúne una conversación entre artistas («Perú, ¿país blindado?») con Alfredo Márquez, Fernando Bryce, Gilda Mantilla, Philippe Gruenberg y Giancarlo Scaglia; ensayos de Miguel López y Max Hernández-Calvo; un debate virtual del blog Arte-Nuevo sobre las políticas museales; un texto de Gustavo Buntinx (Micromuseo) y una entrevista a Jorge Villacorta. El hilo común es la interrogación del supuesto «boom» del arte contemporáneo limeño de la última década: los participantes coinciden en que la internacionalización y el crecimiento del mercado y del coleccionismo (impulsado por el MALI) han producido una escena «contrahecha», con brazos de mercado pero sin instituciones, crítica, educación ni políticas culturales. Márquez denuncia el carácter colonial y exótico de esa visibilidad; López («Boo(o)m: Morir de éxito») teoriza un proceso de despolitización y domesticación que diluye el conflicto y convierte la autonomía en aquiescencia entre agentes; Hernández-Calvo («Una coyuntura que no fue») analiza cómo las Bienales de Lima (1997-2002) forzaron una «contemporaneización» de instalación y video sin sustento curatorial ni educativo, generando escisiones entre circuito oficial y alternativo. Se abordan además el éxodo de artistas por la deficiente formación, la toma estudiantil de Bellas Artes, la autogestión (La Culpable) y las disputas por el Museo de la Memoria. El dossier reivindica la autonomía, el disenso y el filo crítico histórico del arte peruano.</t>
         </is>
       </c>
     </row>
@@ -2206,27 +2206,27 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Vidarte - Exhibiciones y adquisiciones para la construcción de narrativas en la historia del arte contemporáneo peruano.md</t>
+          <t>VVAA - Memorias del subdesarrollo. Arte y el giro descolonial en América Latina, 1960-1985 [catálogo MCASD].md</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>2015-2023</t>
+          <t>1960-1985 (con foco 1967-1981)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Ensayo curatorial de catálogo, 2023</t>
+          <t>Catálogo de exposición / ensayo académico, 2018 (MCASD)</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Giuliana Vidarte; ICPNA; Natalia Iguíñiz; Carlos García Montero; Venuca Evanán; Nereida Apaza; Gloria Quispe; Cristina Flores; Antonio Paucar; Andrés Argüelles Vigo; Carolina Estrada; Santiago Yahuarcani; Ana de Orbegoso</t>
+          <t>Sharon Lerner; Julieta González; Andrea Giunta; Jacopo Crivelli Visconti; Juan Acha; Marta Traba; Ferreira Gullar; Teresa Burga; E.P.S. Huayco; Grupo Paréntesis; Jesús Ruiz Durand; Fernando 'Coco' Bedoya; MALI; Museum of Contemporary Art San Diego</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Giuliana Vidarte reflexiona sobre la exposición 'Miradas contemporáneas. Nuevas adquisiciones en la colección ICPNA (2015-2023)', presentada en el Espacio Juan Pardo Heeren del ICPNA de Lima entre agosto y septiembre de 2023. Su argumento central es que las exhibiciones y adquisiciones institucionales son dispositivos para la construcción de narrativas y memoria crítica en la historia del arte contemporáneo peruano: una colección formada a partir de obras que fueron parte de la propia programación expositiva constituye un testimonio de los modos de creación y conserva la memoria de la historia de las exposiciones en el país. Parte de dos ganadoras del Premio ICPNA de Arte Contemporáneo, Venuca Evanán y Nereida Apaza, para introducir cómo el arte contribuye a pensar la realidad mediante reflexiones colectivas sobre violencia de género, identidad y nación. Describe los cinco ejes curatoriales de la muestra —revalorando intimidades, discursos críticos, develando entornos, reinterpretar tradiciones y estéticas disímiles— y analiza diálogos entre obras: el cuerpo y la caja torácica en Gloria Quispe, Cristina Flores y Antonio Paucar; la crítica a la representación colonial y republicana en Andrés Argüelles Vigo y Carolina Estrada/Teodoro Ramírez; el paisaje y la crisis medioambiental amazónica en Silvia Westphalen y Nicole Franchy; la reinterpretación de saberes ancestrales en Santiago Yahuarcani y Ana de Orbegoso. Destaca que las fichas incorporan citas de textos curatoriales previos, nutriendo la exposición del archivo documental institucional. Concluye que estos conjuntos abren líneas múltiples de lectura y afirman el valor del esfuerzo colectivo de gestores, curadores e investigadores en la formación de colecciones y en la escritura de la historia del arte peruano reciente.</t>
+          <t>El ensayo de Sharon Lerner incluido en el catálogo de la exposición 'Memorias del subdesarrollo: arte y el giro descolonial en América Latina, 1960-1985' inserta la escena peruana de 1967-1981 en una narrativa continental que postula una ruptura epistémica con lo moderno mediante la noción de subdesarrollo y el deseo de descolonizar los cánones estéticos impuestos. Su tesis desplaza el foco del paradigma formalista modernista hacia el contexto social, la apropiación de tradiciones locales y lo 'popular' como categoría clave, cuya heterogeneidad histórica advierte no homogeneizar. Reconstruye el debate entre Juan Acha y Marta Traba sobre el pop cosmopolita y la dependencia cultural, apoyándose en Mariátegui, Ferreira Gullar y Mário Pedrosa, y en la teoría de la dependencia. Analiza casos peruanos: los afiches de la Reforma Agraria de Jesús Ruiz Durand y su 'pop achorado' dentro de SINAMOS; los festivales Contacta y las Carreras de Chasquis de Luis Arias Vera bajo el velasquismo; el Grupo Paréntesis y el Contacta 79 (Becerro de oro, Coquito) de Fernando Bedoya; y sobre todo E.P.S. Huayco, con 'Arte al paso (Salchipapas)' y 'Sarita Colonia', leídos vía Buntinx y Lauer como articulación de lo popular urbano migrante. Suma el caso aislado de Teresa Burga y 'Perfil de la mujer peruana' (1980-81) como acercamiento conceptual a género y clase. Recurriendo a Bürger y Giunta, discute la definición de vanguardia y concluye que estas prácticas oscilaron entre dependencia y autonomía, sin lograr plataformas de continuidad, siendo Huayco el caso más próximo a una vanguardia local pese a su disolución.</t>
         </is>
       </c>
     </row>
@@ -2238,27 +2238,27 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Villacorta - La colección Hochschild.md</t>
+          <t>Vich - La violencia, la dictadura y la globalización. Arte y política en el Perú contemporáneo.md</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>1980-2016 (con énfasis en el arte peruano desde 2000)</t>
+          <t>1980-2009 (violencia política, dictadura fujimorista y posconflicto)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo de colección, c. 2016</t>
+          <t>Ensayo / capítulo de libro académico, c. 2013-2015</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta Chávez; Eduardo y Mariana Hochschild; Octavio Zaya; Luis Pérez Oramas; Giancarlo Scaglia; Fernando Bryce; Teresa Burga; Tilsa Tsuchiya; Jorge Eduardo Eielson; Regina Aprijaskis; MALI; MoMA; Tate Modern</t>
+          <t>Víctor Vich; Eduardo Tokeshi; Colectivo Sociedad Civil; Natalia Iguíñiz; Sandro Venturo; Piero Quijano; Luz Letts; Víctor Delfín; Miguel Cordero; Jaime Higa; Herbert Rodríguez; Claudia Martínez; Santiago Quintanilla; Rudolph Castro; Felipe López; Gustavo Buntinx</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta analiza la Colección Hochschild como caso paradigmático del coleccionismo privado de arte contemporáneo peruano, sosteniendo que todo desarrollo artístico notable requiere un coleccionismo a la altura de su ambición, junto con crítica y testimonio histórico escrito. El coleccionista, figura clave de todo sistema artístico moderno, opera a la vez como catalizador de la escena y motor del mercado. Iniciada en 2009 por Eduardo y Mariana Hochschild, la colección se distingue por seguir la dinámica actual del sistema de las artes visuales en un medio que careció de coleccionismo corporativo sostenido, escasa crítica periodística y pocas publicaciones especializadas —una 'orfandad' de los artistas. Villacorta subraya que los Hochschild rompieron el molde del coleccionismo centrado en el arte moderno al adquirir netamente arte contemporáneo con asesoramiento profesional (Luis Pérez Oramas, Giancarlo Scaglia) en ausencia de una historiografía orgánica del arte peruano desde 1980. Contextualiza el aislamiento económico y la violencia de los años ochenta y noventa que invisibilizaron a dos generaciones de artistas, y el dinamismo que trajeron la Bienal Iberoamericana de Lima (1997) y el Festival de Video/Arte Electrónico (1998). Comenta la selección de Octavio Zaya para 'Próxima parada' y la tríada Aprijaskis-Eielson-Burga como artistas que escapan al arte moderno local e inauguran lo contemporáneo. Ejemplifica el 'punto ciego' del coleccionista limeño con 'Atlas Perú' de Fernando Bryce, vendido al exterior, y aborda la tensión entre relevancia cultural nacional y reconocimiento del mercado internacional. Cita cimientos modernos (Sabogal, Szyszlo, Tsuchiya) y fortalezas en escultura, instalación y fotografía (Chambi, Testino, Martinat, Damiani), afirmando que la colección materializa una visión cabal del arte peruano contemporáneo.</t>
+          <t>Víctor Vich propone una lectura desde la crítica cultural del arte peruano contemporáneo, sosteniendo que, frente al discurso triunfalista del crecimiento económico, un sector de artistas sigue nombrando al país a partir de sus heridas históricas. Estructura el ensayo en torno a tres acontecimientos: la violencia política, el autoritarismo corrupto del fujimontesinismo y la globalización neoliberal. Apoyándose en Žižek, Hall, Jameson, Foucault y Badiou, entiende lo simbólico no como reflejo sino como soporte de la realidad y campo de batalla donde se disputan sentidos de ciudadanía. Analiza obras emblemáticas: 'Bandera VIII' (2000) de Eduardo Tokeshi, leída como 'la patria en cuidados intensivos'; 'Lava la bandera' del Colectivo Sociedad Civil; la instalación 'Patria' de Natalia Iguíñiz y Sandro Venturo; el afiche censurado de Piero Quijano sobre La Cantuta e Iwo Jima; 'El azar como destino' de Luz Letts; 'El hermoso general' de Víctor Delfín; el saco militar de Miguel Cordero; y las serigrafías de César Vallejo de Jaime Higa sobre posmodernismo y cultura de masas. En una segunda sección sobre memoria generacional examina a artistas nacidos en los ochenta que 'traducen' la violencia con lenguajes heredados de la infancia: la serie 'Invisible' de Claudia Martínez, el trabajo de archivo y cómic de Santiago Quintanilla, los juguetes siniestros (Lego, Playmobil) de Rudolph Castro y las fotografías de nichos ayacuchanos de Felipe López. Su aporte es articular teoría psicoanalítica y poscolonial con un corpus visual peruano, mostrando el arte crítico como agente que interrumpe la ficción neoliberal y recompone la comunidad desde el orden simbólico.</t>
         </is>
       </c>
     </row>
@@ -2270,27 +2270,27 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Villacorta - Un arte cuestionador. De Dadá a La Cantuta [Quehacer 102, pdf pp. 96-105].md</t>
+          <t>Vidarte - Exhibiciones y adquisiciones para la construcción de narrativas en la historia del arte contemporáneo peruano.md</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>1916-1996 (vanguardias históricas y arte peruano 1979-1995)</t>
+          <t>2015-2023</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Artículo de revista (Quehacer 102, DESCO), c. 1996</t>
+          <t>Ensayo curatorial de catálogo, 2023</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Francisco Mariotti; Herbert Rodríguez; Ricardo Wiesse; Eduardo Villanes; Hugo Salazar del Alcázar; E.P.S. Huayco; Grupo Paréntesis; Los Bestias; Carpa Teatro del Puente Santa Rosa; Sendero Luminoso</t>
+          <t>Giuliana Vidarte; ICPNA; Natalia Iguíñiz; Carlos García Montero; Venuca Evanán; Nereida Apaza; Gloria Quispe; Cristina Flores; Antonio Paucar; Andrés Argüelles Vigo; Carolina Estrada; Santiago Yahuarcani; Ana de Orbegoso</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>En este artículo para la revista Quehacer (DESCO), dedicado in memoriam a Hugo Salazar del Alcázar, Jorge Villacorta traza una genealogía del arte peruano contestatario que la generación más joven de artistas visuales estaría redescubriendo como una tradición alternativa o 'canon no-oficial', paralelo al aceptado. Su tesis vincula esa tradición local con las vanguardias históricas internacionales: la deuda con Dadá (Zúrich, 1916) como rechazo crítico de la civilización occidental tras la carnicería bélica, el manifiesto como obra del futurismo, y el constructivismo ruso con su noción de arte como agit-prop. Aplica ese marco a la 'movida barranquina' de fines de los años setenta, primera generación ligada a una cultura juvenil limeña irreverente y a los medios masivos, donde grupos como Paréntesis y Huayco entendieron la creación como provocación y enfrentamiento; destaca la serigrafía enseñada por Mariotti y la salida de Huayco de la galería hacia el kilómetro 54 de la Panamericana Sur. Narra luego cómo la violencia de Sendero Luminoso desde 1980, el fracaso de Izquierda Unida y la crisis marcaron el clima cultural: la exposición de Artistas Visuales Asociados (1983) y 'Por el Derecho a la Vida' (1985). Analiza la escena subterránea y la Carpa Teatro del Puente Santa Rosa (1986), con Los Bestias y el fanzine, y el proyecto solitario Arte Vida de Herbert Rodríguez en San Marcos entre 1986 y 1992. Concluye con la respuesta ética ante el caso La Cantuta: la exposición de Eduardo Villanes con cajas de leche Gloria (1994) y la acción ambiental de Ricardo Wiesse con flores de cantuta en Cieneguilla (1995), afirmando un arte que asume responsabilidades éticas frente a los desaparecidos.</t>
+          <t>Giuliana Vidarte reflexiona sobre la exposición 'Miradas contemporáneas. Nuevas adquisiciones en la colección ICPNA (2015-2023)', presentada en el Espacio Juan Pardo Heeren del ICPNA de Lima entre agosto y septiembre de 2023. Su argumento central es que las exhibiciones y adquisiciones institucionales son dispositivos para la construcción de narrativas y memoria crítica en la historia del arte contemporáneo peruano: una colección formada a partir de obras que fueron parte de la propia programación expositiva constituye un testimonio de los modos de creación y conserva la memoria de la historia de las exposiciones en el país. Parte de dos ganadoras del Premio ICPNA de Arte Contemporáneo, Venuca Evanán y Nereida Apaza, para introducir cómo el arte contribuye a pensar la realidad mediante reflexiones colectivas sobre violencia de género, identidad y nación. Describe los cinco ejes curatoriales de la muestra —revalorando intimidades, discursos críticos, develando entornos, reinterpretar tradiciones y estéticas disímiles— y analiza diálogos entre obras: el cuerpo y la caja torácica en Gloria Quispe, Cristina Flores y Antonio Paucar; la crítica a la representación colonial y republicana en Andrés Argüelles Vigo y Carolina Estrada/Teodoro Ramírez; el paisaje y la crisis medioambiental amazónica en Silvia Westphalen y Nicole Franchy; la reinterpretación de saberes ancestrales en Santiago Yahuarcani y Ana de Orbegoso. Destaca que las fichas incorporan citas de textos curatoriales previos, nutriendo la exposición del archivo documental institucional. Concluye que estos conjuntos abren líneas múltiples de lectura y afirman el valor del esfuerzo colectivo de gestores, curadores e investigadores en la formación de colecciones y en la escritura de la historia del arte peruano reciente.</t>
         </is>
       </c>
     </row>
@@ -2302,27 +2302,27 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Villacorta y Del Valle - Incertidumbre y certezas en el arte peruano reciente. Imaginarios de Lima en transformación 1980-2006 [Post-Ilusiones].txt</t>
+          <t>Villacorta - La colección Hochschild.md</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>1919-2006 (con eje central 1980-2006)</t>
+          <t>1980-2016 (con énfasis en el arte peruano desde 2000)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de libro/catálogo (Post-Ilusiones), c. 2007</t>
+          <t>Ensayo de catálogo de colección, c. 2016</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta Chávez; Augusto del Valle Cárdenas; José Sabogal; Juan Acha; Marta Traba; Fernando de Szyszlo; Jorge Eduardo Eielson; Emilio Rodríguez Larraín; E.P.S. Huayco; Escuela Nacional de Bellas Artes; IAC; Agrupación Espacio</t>
+          <t>Jorge Villacorta Chávez; Eduardo y Mariana Hochschild; Octavio Zaya; Luis Pérez Oramas; Giancarlo Scaglia; Fernando Bryce; Teresa Burga; Tilsa Tsuchiya; Jorge Eduardo Eielson; Regina Aprijaskis; MALI; MoMA; Tate Modern</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta y Augusto del Valle proponen un ensayo panorámico sobre el arte peruano reciente que lee la transformación de los imaginarios de Lima entre 1980 y 2006 a partir de una tesis de fondo: en el Perú la academia y sus modelos artísticos comenzaron tarde e hicieron crisis temprano. Recorren la fundación de la Escuela Nacional de Bellas Artes (1919), la retorización del indigenismo de Sabogal como vanguardia institucionalizada, el rol del IAC (1955-1972) en la difusión del arte 'culto' y su negociación con modelos norteamericanos, y la tensión entre 'alta' y 'baja' cultura heredada de la intelligentsia marxista tras la Revolución cubana. Interpretan el populismo cultural del gobierno militar (Velasco y Morales Bermúdez), el premio a López Antay (1975) y el receso de Bellas Artes (1977) como síntomas del agotamiento de una visión del arte, frente al modelo pedagógico expresivo-trascendente de Winternitz en la PUCP. El eje del texto es la categoría de no-objetualismo de Juan Acha, que articulan en dos oleadas: un primer no-objetualismo utópico de izquierda (E.P.S. Huayco) y un segundo, ligado a la Movida Subterránea y a la Carpa Teatro del Puente Santa Rosa (1986). Analizan la precariedad de los años ochenta bajo la violencia y la crisis del primer gobierno de García, el neoliberalismo autocrático fujimorista como silenciador del arte crítico y productor de espectáculo, y la centralidad creciente de la fotografía, el video y el arte electrónico desde las bienales de Lima (1997) y el Festival de Video (1998). Concluyen con el tránsito del no-objetualismo político al poético y con la 'choledad digital' y la globalización del imaginario como horizonte contemporáneo.</t>
+          <t>Jorge Villacorta analiza la Colección Hochschild como caso paradigmático del coleccionismo privado de arte contemporáneo peruano, sosteniendo que todo desarrollo artístico notable requiere un coleccionismo a la altura de su ambición, junto con crítica y testimonio histórico escrito. El coleccionista, figura clave de todo sistema artístico moderno, opera a la vez como catalizador de la escena y motor del mercado. Iniciada en 2009 por Eduardo y Mariana Hochschild, la colección se distingue por seguir la dinámica actual del sistema de las artes visuales en un medio que careció de coleccionismo corporativo sostenido, escasa crítica periodística y pocas publicaciones especializadas —una 'orfandad' de los artistas. Villacorta subraya que los Hochschild rompieron el molde del coleccionismo centrado en el arte moderno al adquirir netamente arte contemporáneo con asesoramiento profesional (Luis Pérez Oramas, Giancarlo Scaglia) en ausencia de una historiografía orgánica del arte peruano desde 1980. Contextualiza el aislamiento económico y la violencia de los años ochenta y noventa que invisibilizaron a dos generaciones de artistas, y el dinamismo que trajeron la Bienal Iberoamericana de Lima (1997) y el Festival de Video/Arte Electrónico (1998). Comenta la selección de Octavio Zaya para 'Próxima parada' y la tríada Aprijaskis-Eielson-Burga como artistas que escapan al arte moderno local e inauguran lo contemporáneo. Ejemplifica el 'punto ciego' del coleccionista limeño con 'Atlas Perú' de Fernando Bryce, vendido al exterior, y aborda la tensión entre relevancia cultural nacional y reconocimiento del mercado internacional. Cita cimientos modernos (Sabogal, Szyszlo, Tsuchiya) y fortalezas en escultura, instalación y fotografía (Chambi, Testino, Martinat, Damiani), afirmando que la colección materializa una visión cabal del arte peruano contemporáneo.</t>
         </is>
       </c>
     </row>
@@ -2334,27 +2334,27 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Villegas_Fernando_La_relacion_entre_arte.pdf</t>
+          <t>Villacorta - Un arte cuestionador. De Dadá a La Cantuta [Quehacer 102, pdf pp. 96-105].md</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>1920-1976 (con proyecciones hasta 2013)</t>
+          <t>1916-1996 (vanguardias históricas y arte peruano 1979-1995)</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico, 2013 (Revista de Historiografía, N.º 19)</t>
+          <t>Artículo de revista (Quehacer 102, DESCO), c. 1996</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Fernando Villegas; José Sabogal; Joaquín López Antay; José Carlos Mariátegui; Fernando de Szyszlo; Carlos Quízpez Asín; Instituto de Arte Peruano; Amauta; ASPAP; Juan Velasco Alvarado; Universidad Complutense de Madrid; Néstor García Canclini</t>
+          <t>Jorge Villacorta; Francisco Mariotti; Herbert Rodríguez; Ricardo Wiesse; Eduardo Villanes; Hugo Salazar del Alcázar; E.P.S. Huayco; Grupo Paréntesis; Los Bestias; Carpa Teatro del Puente Santa Rosa; Sendero Luminoso</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Artículo de Fernando Villegas (Universidad Complutense de Madrid), publicado en la Revista de Historiografía N.º 19 (2013, pp. 75-87), que rastrea la evolución de los enfoques ideológicos sobre el arte popular peruano vinculando arte y política en dos momentos clave. El primero es el proyecto mestizo de José Sabogal en los años veinte: tras su viaje a México (1923) y en sintonía con la búsqueda de peruanidad de Mariátegui y la revista Amauta, Sabogal revaloriza mates burilados, queros y retablos como productos mestizos, fusión de lo indígena precolombino y lo virreinal hispano. Desde el Instituto de Arte Peruano (1931) su grupo estudia la cerámica precolombina, el color y las artes populares, legitimando estos objetos por su origen indígena pero desplazando al artista popular como creador (los pintores urbanos se autoproclaman sus 'descubridores'). El segundo momento es la polémica de 1975-1976, cuando el gobierno militar de Velasco otorgó el Premio Nacional de Cultura al retablista ayacuchano Joaquín López Antay; la ASPAP y artistas académicos lo descalificaron como 'artesano', reproduciendo la jerarquía social y racial limeña. Villegas argumenta que ambos episodios responden a gobiernos autoritarios que legitimaron el arte popular para oponerse a la oligarquía limeña, y que el criterio de validación siempre fue estético-cronológico, ignorando el proceso histórico. El marco conceptual moviliza a Mariátegui, a Clifford (apropiación de objetos de otras culturas) y a García Canclini (descontextualización). Su aporte es evidenciar la ausencia del artista popular como sujeto de su propia obra y la carga étnica y de clase que desnaturaliza el proceso creativo andino en el circuito artístico peruano.</t>
+          <t>En este artículo para la revista Quehacer (DESCO), dedicado in memoriam a Hugo Salazar del Alcázar, Jorge Villacorta traza una genealogía del arte peruano contestatario que la generación más joven de artistas visuales estaría redescubriendo como una tradición alternativa o 'canon no-oficial', paralelo al aceptado. Su tesis vincula esa tradición local con las vanguardias históricas internacionales: la deuda con Dadá (Zúrich, 1916) como rechazo crítico de la civilización occidental tras la carnicería bélica, el manifiesto como obra del futurismo, y el constructivismo ruso con su noción de arte como agit-prop. Aplica ese marco a la 'movida barranquina' de fines de los años setenta, primera generación ligada a una cultura juvenil limeña irreverente y a los medios masivos, donde grupos como Paréntesis y Huayco entendieron la creación como provocación y enfrentamiento; destaca la serigrafía enseñada por Mariotti y la salida de Huayco de la galería hacia el kilómetro 54 de la Panamericana Sur. Narra luego cómo la violencia de Sendero Luminoso desde 1980, el fracaso de Izquierda Unida y la crisis marcaron el clima cultural: la exposición de Artistas Visuales Asociados (1983) y 'Por el Derecho a la Vida' (1985). Analiza la escena subterránea y la Carpa Teatro del Puente Santa Rosa (1986), con Los Bestias y el fanzine, y el proyecto solitario Arte Vida de Herbert Rodríguez en San Marcos entre 1986 y 1992. Concluye con la respuesta ética ante el caso La Cantuta: la exposición de Eduardo Villanes con cajas de leche Gloria (1994) y la acción ambiental de Ricardo Wiesse con flores de cantuta en Cieneguilla (1995), afirmando un arte que asume responsabilidades éticas frente a los desaparecidos.</t>
         </is>
       </c>
     </row>
@@ -2366,27 +2366,27 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>canepa_kg_2006_p132-167.pdf</t>
+          <t>Villacorta y Del Valle - Incertidumbre y certezas en el arte peruano reciente. Imaginarios de Lima en transformación 1980-2006 [Post-Ilusiones].txt</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>1970-2006 (con referencias históricas desde el siglo XIX)</t>
+          <t>1919-2006 (con eje central 1980-2006)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro, 2006</t>
+          <t>Ensayo de libro/catálogo (Post-Ilusiones), c. 2007</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Giuliana Borea Labarthe; Gisela Cánepa Koch (ed.); Sandra Gamarra (LiMAC); Instituto de Arte Contemporáneo (IAC); Fernando de Szyszlo; Gerardo Chávez; Mario Vargas Llosa; Ramiro Llona; Instituto Nacional de Cultura; ICOM; Museo de la Nación; Museo Nacional de la Cultura Peruana; Alfonso Castrillón</t>
+          <t>Jorge Villacorta Chávez; Augusto del Valle Cárdenas; José Sabogal; Juan Acha; Marta Traba; Fernando de Szyszlo; Jorge Eduardo Eielson; Emilio Rodríguez Larraín; E.P.S. Huayco; Escuela Nacional de Bellas Artes; IAC; Agrupación Espacio</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Capítulo de Giuliana Borea Labarthe ('Museos y esfera pública: espacio, discursos y prácticas. Reflexiones en torno a la ciudad de Lima') incluido en el volumen editado por Gisela Cánepa Koch, 'Mirando la esfera pública desde la cultura en el Perú' (2006). Partiendo de las nociones de esfera pública (Habermas), cultura pública (Appadurai) y de la nueva museología surgida de las crisis de los años 70-80 (Mesa de Santiago 1972, redefinición del ICOM 1974, ecomuseos), Borea concibe el museo como contenedor y contenido, plataforma y discurso, esfera de poder y arena de disputa por la representación. Analiza tres casos limeños. Primero, el posicionamiento urbano de los museos: mediante una encuesta a transeúntes y taxistas muestra que solo el Museo de la Nación y el Museo de Arte de Lima son hitos reconocidos, mientras la mayoría oscila entre lugar simbólico y lugar anónimo por la falta de señalización y de alianzas municipales. Segundo, la polémica de 2006 por el proyecto del Museo de Arte Contemporáneo (MAC) del IAC, detonada por el intento de nombrarlo 'Fernando de Szyszlo': reconstruye siete momentos del debate mediático (comunicados de artistas, la columna 'Escaramuzas en Liliput' de Vargas Llosa), la falta de plan museológico y de diálogo con artistas donantes y con Barranco, y destaca la contrapropuesta crítica LiMAC de Sandra Gamarra frente al silencio del INC. Tercero, compara las puestas en escena sobre peruanidad y diversidad de cinco museos (Cultura Peruana, de la Nación, Etnográfico, Inmigración Japonesa, MNAAHP), evidenciando discursos lejanos, fragmentados y ahistóricos en los grandes museos nacionales frente a autorrepresentaciones más políticas en los pequeños. Cierra con Castrillón: Lima como escenario de emplazamiento, no de reflexión.</t>
+          <t>Jorge Villacorta y Augusto del Valle proponen un ensayo panorámico sobre el arte peruano reciente que lee la transformación de los imaginarios de Lima entre 1980 y 2006 a partir de una tesis de fondo: en el Perú la academia y sus modelos artísticos comenzaron tarde e hicieron crisis temprano. Recorren la fundación de la Escuela Nacional de Bellas Artes (1919), la retorización del indigenismo de Sabogal como vanguardia institucionalizada, el rol del IAC (1955-1972) en la difusión del arte 'culto' y su negociación con modelos norteamericanos, y la tensión entre 'alta' y 'baja' cultura heredada de la intelligentsia marxista tras la Revolución cubana. Interpretan el populismo cultural del gobierno militar (Velasco y Morales Bermúdez), el premio a López Antay (1975) y el receso de Bellas Artes (1977) como síntomas del agotamiento de una visión del arte, frente al modelo pedagógico expresivo-trascendente de Winternitz en la PUCP. El eje del texto es la categoría de no-objetualismo de Juan Acha, que articulan en dos oleadas: un primer no-objetualismo utópico de izquierda (E.P.S. Huayco) y un segundo, ligado a la Movida Subterránea y a la Carpa Teatro del Puente Santa Rosa (1986). Analizan la precariedad de los años ochenta bajo la violencia y la crisis del primer gobierno de García, el neoliberalismo autocrático fujimorista como silenciador del arte crítico y productor de espectáculo, y la centralidad creciente de la fotografía, el video y el arte electrónico desde las bienales de Lima (1997) y el Festival de Video (1998). Concluyen con el tránsito del no-objetualismo político al poético y con la 'choledad digital' y la globalización del imaginario como horizonte contemporáneo.</t>
         </is>
       </c>
     </row>
@@ -2398,27 +2398,27 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>mac-proyecto-2008.md</t>
+          <t>Villegas_Fernando_La_relacion_entre_arte.pdf</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>2008 (exposición feb.–mar. 2008; con historia del sitio desde 1944)</t>
+          <t>1920-1976 (con proyecciones hasta 2013)</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de exposición, mayo 2008 (Instituto de Arte Contemporáneo — MAC-Lima; OCR)</t>
+          <t>Artículo académico, 2013 (Revista de Historiografía, N.º 19)</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Miguel Zegarra (curadores); Instituto de Arte Contemporáneo (IAC); MAC-Lima; Giuliana Borea; George Gruenberg; Ricardo Ramón Jarne; José Carlos Martinat; Ishmael Randall Weeks; Elena Damiani; Sergio Abugattás; Raura Oblitas</t>
+          <t>Fernando Villegas; José Sabogal; Joaquín López Antay; José Carlos Mariátegui; Fernando de Szyszlo; Carlos Quízpez Asín; Instituto de Arte Peruano; Amauta; ASPAP; Juan Velasco Alvarado; Universidad Complutense de Madrid; Néstor García Canclini</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Catálogo de la exposición «La Construcción del Lugar Común» (MAC-Lima, 5 de febrero–30 de marzo de 2008), editado por el Instituto de Arte Contemporáneo (IAC) y curado por Jorge Villacorta y Miguel Zegarra. Documenta una intervención colectiva de quince artistas peruanos emergentes —Sergio Abugattás, Miguel Andrade, Víctor Castro, Elena Damiani, Giuseppe De Bernardi, Nicole Franchy, Alejandro Jaime, Manuel Larrea, Martín Jiménez Paz, Christians Luna, José Carlos Martinat, José Miyashiro, Raura Oblitas, Ishmael Randall Weeks e Iliana Scheggia— que ocuparon el edificio del Museo de Arte Contemporáneo de Lima cuando aún estaba a medio construir. La muestra convirtió la arquitectura inconclusa y su entorno (el parque de la antigua «laguna» de Barranco) en soporte y tema: las obras tematizan la construcción/destrucción, el paisaje, la memoria del sitio y la disputa pública por el museo, cuyo proceso estuvo marcado por conflictos municipales y un intento de clausura respondido con el gesto «CLAUSURADO = INAUGURADO». El catálogo reúne textos institucionales (George Gruenberg, presidente del IAC), una pieza literaria de Ricardo Ramón Jarne («La maldición de la laguna»), un ensayo antropológico de Giuliana Borea sobre la construcción del lugar y el «lugar común» en la esfera pública (apoyado en Augé, Appadurai, Certeau y Casey), el texto curatorial de Villacorta y Zegarra, y los statements de cada artista. Como fuente histórica documenta un episodio clave de institucionalización del arte contemporáneo en Lima —la génesis del MAC— y las prácticas site-specific, de crítica institucional y de intervención en el espacio público de una generación emergente peruana de fines de la década de 2000.</t>
+          <t>Artículo de Fernando Villegas (Universidad Complutense de Madrid), publicado en la Revista de Historiografía N.º 19 (2013, pp. 75-87), que rastrea la evolución de los enfoques ideológicos sobre el arte popular peruano vinculando arte y política en dos momentos clave. El primero es el proyecto mestizo de José Sabogal en los años veinte: tras su viaje a México (1923) y en sintonía con la búsqueda de peruanidad de Mariátegui y la revista Amauta, Sabogal revaloriza mates burilados, queros y retablos como productos mestizos, fusión de lo indígena precolombino y lo virreinal hispano. Desde el Instituto de Arte Peruano (1931) su grupo estudia la cerámica precolombina, el color y las artes populares, legitimando estos objetos por su origen indígena pero desplazando al artista popular como creador (los pintores urbanos se autoproclaman sus 'descubridores'). El segundo momento es la polémica de 1975-1976, cuando el gobierno militar de Velasco otorgó el Premio Nacional de Cultura al retablista ayacuchano Joaquín López Antay; la ASPAP y artistas académicos lo descalificaron como 'artesano', reproduciendo la jerarquía social y racial limeña. Villegas argumenta que ambos episodios responden a gobiernos autoritarios que legitimaron el arte popular para oponerse a la oligarquía limeña, y que el criterio de validación siempre fue estético-cronológico, ignorando el proceso histórico. El marco conceptual moviliza a Mariátegui, a Clifford (apropiación de objetos de otras culturas) y a García Canclini (descontextualización). Su aporte es evidenciar la ausencia del artista popular como sujeto de su propia obra y la carga étnica y de clase que desnaturaliza el proceso creativo andino en el circuito artístico peruano.</t>
         </is>
       </c>
     </row>
@@ -2430,91 +2430,91 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>sura.md</t>
+          <t>canepa_kg_2006_p132-167.pdf</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>mediados de la década de 1960 a 2013 (arte contemporáneo peruano)</t>
+          <t>1970-2006 (con referencias históricas desde el siglo XIX)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de colección museística, 2013</t>
+          <t>Capítulo de libro, 2006</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner (ed.); Museo de Arte de Lima (MALI); Grupo SURA; Mirko Lauer; E.P.S. Huayco; Charo Noriega; Ramiro Llona; Flavia Gandolfo; Armando Andrade Tudela; Ricardo Wiesse; Eduardo Villanes; Miguel A. López; Rodrigo Quijano</t>
+          <t>Giuliana Borea Labarthe; Gisela Cánepa Koch (ed.); Sandra Gamarra (LiMAC); Instituto de Arte Contemporáneo (IAC); Fernando de Szyszlo; Gerardo Chávez; Mario Vargas Llosa; Ramiro Llona; Instituto Nacional de Cultura; ICOM; Museo de la Nación; Museo Nacional de la Cultura Peruana; Alfonso Castrillón</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Catálogo de la colección de arte contemporáneo del Museo de Arte de Lima (MALI), editado por la curadora Sharon Lerner y publicado con el patrocinio del grupo SURA. El volumen traza los derroteros del arte peruano reciente a partir del acervo del museo, sin pretender definir un 'arte peruano' esencial. La colección se articula bajo dos principios: identificar momentos de ruptura en la producción artística de fines del siglo XX y perfilar la producción reciente mediante ejes temáticos comunes. El ensayo central de Lerner establece como punto de partida mediados de la década de 1960 (grupos de vanguardia ligados al Pop y al no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, tras las reformas del Gobierno Militar, cuando —según la célebre frase de Mirko Lauer para la muestra Arte al paso del colectivo E.P.S. Huayco (1980)— 'en el Perú hoy solo lo popular es moderno'. Analiza la irrupción de la migración interna, el conflicto armado interno, el autogolpe de Fujimori (1992) y la virtual desaparición de la esfera pública, así como la Bienal Iberoamericana de Lima (1997) como puesta al día forzada y descontextualizada. El catálogo se organiza en núcleos temáticos: modernidad popular y transformación de Lima, f(r)icciones cosmopolitas, reconsideración del pasado y configuración del Perú, sistema artístico y utopías museales, desplazamientos, y signos de violencia, resistencia y memoria. Incluye obras de Charo Noriega, Ramiro Llona, Flavia Gandolfo, Armando Andrade Tudela, Herman Schwarz, Ricardo Wiesse y Eduardo Villanes, entre otros, y textos críticos complementarios. Su aporte es consolidar un relato historiográfico y crítico del arte contemporáneo peruano desde una institución museal.</t>
+          <t>Capítulo de Giuliana Borea Labarthe ('Museos y esfera pública: espacio, discursos y prácticas. Reflexiones en torno a la ciudad de Lima') incluido en el volumen editado por Gisela Cánepa Koch, 'Mirando la esfera pública desde la cultura en el Perú' (2006). Partiendo de las nociones de esfera pública (Habermas), cultura pública (Appadurai) y de la nueva museología surgida de las crisis de los años 70-80 (Mesa de Santiago 1972, redefinición del ICOM 1974, ecomuseos), Borea concibe el museo como contenedor y contenido, plataforma y discurso, esfera de poder y arena de disputa por la representación. Analiza tres casos limeños. Primero, el posicionamiento urbano de los museos: mediante una encuesta a transeúntes y taxistas muestra que solo el Museo de la Nación y el Museo de Arte de Lima son hitos reconocidos, mientras la mayoría oscila entre lugar simbólico y lugar anónimo por la falta de señalización y de alianzas municipales. Segundo, la polémica de 2006 por el proyecto del Museo de Arte Contemporáneo (MAC) del IAC, detonada por el intento de nombrarlo 'Fernando de Szyszlo': reconstruye siete momentos del debate mediático (comunicados de artistas, la columna 'Escaramuzas en Liliput' de Vargas Llosa), la falta de plan museológico y de diálogo con artistas donantes y con Barranco, y destaca la contrapropuesta crítica LiMAC de Sandra Gamarra frente al silencio del INC. Tercero, compara las puestas en escena sobre peruanidad y diversidad de cinco museos (Cultura Peruana, de la Nación, Etnográfico, Inmigración Japonesa, MNAAHP), evidenciando discursos lejanos, fragmentados y ahistóricos en los grandes museos nacionales frente a autorrepresentaciones más políticas en los pequeños. Cierra con Castrillón: Lima como escenario de emplazamiento, no de reflexión.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Arte al Paso 2011</t>
+          <t>Cap 2 - Historia</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Arte al Paso - Texto Investigación.md</t>
+          <t>mac-proyecto-2008.md</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 1960 – 2010 (con foco en las décadas de 1970-2000 y el conflicto armado interno 1980-2000)</t>
+          <t>2008 (exposición feb.–mar. 2008; con historia del sitio desde 1944)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Ensayo curatorial de catálogo (exposición Arte al paso, Pinacoteca do Estado de São Paulo, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Catálogo de exposición, mayo 2008 (Instituto de Arte Contemporáneo — MAC-Lima; OCR)</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Pinacoteca de São Paulo; Emilio Hernández Saavedra; E.P.S. Huayco; Jesús Ruiz Durand; Sandra Gamarra; Alfredo Márquez / Taller NN; Fernando Bryce; José Carlos Martinat; Susana Torres</t>
+          <t>Jorge Villacorta; Miguel Zegarra (curadores); Instituto de Arte Contemporáneo (IAC); MAC-Lima; Giuliana Borea; George Gruenberg; Ricardo Ramón Jarne; José Carlos Martinat; Ishmael Randall Weeks; Elena Damiani; Sergio Abugattás; Raura Oblitas</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Ensayo curatorial extenso y bilingüe (castellano/portugués) de Tatiana Cuevas y Rodrigo Quijano para la muestra Arte al paso, que exhibió la coleccion contemporanea del MALI en la Estacion Pinacoteca de Sao Paulo. El texto toma como punto de partida la imagen El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra para diagnosticar los vacios institucionales y la distancia entre el discurso cultural cosmopolita y la practica real en el Peru de la segunda mitad del siglo XX. Su argumento articula el arte contemporaneo peruano con las transformaciones sociales derivadas de la masiva migracion rural a Lima, la explosion de la economia informal y la emergencia de una nueva cultura popular urbana. Rastrea las primeras vinculaciones locales con vanguardias internacionales (op, pop, conceptualismo, no-objetualismo), el pop achorado de Jesus Ruiz Durand y sus afiches de la Reforma Agraria velasquista, y las experiencias colectivas Contacta 79 y Arte al paso de E.P.S. Huayco (1980), que propusieron un arte callejero y antiinstitucional. Analiza la critica a la institucionalidad faltante (el museo ficticio LiMAC de Sandra Gamarra), el uso ironico del pasado prehispanico (Susana Torres, Rodriguez Larrain, Bryce, Cordova, Martinat), el tema del paisaje y el territorio, y la irrupcion tardia de la fotografia y la serigrafia como medios. Dedica una seccion central a la memoria de la violencia del conflicto armado interno (1980-2000) —Sendero Luminoso, MRTA, la Comision de la Verdad, 69.280 muertos— y su tratamiento por el Taller NN, Alfredo Marquez (Katatay), Carlos Dominguez, Ricardo Wiesse, Eduardo Villanes, Fernando Bryce y Milagros de la Torre.</t>
+          <t>Catálogo de la exposición «La Construcción del Lugar Común» (MAC-Lima, 5 de febrero–30 de marzo de 2008), editado por el Instituto de Arte Contemporáneo (IAC) y curado por Jorge Villacorta y Miguel Zegarra. Documenta una intervención colectiva de quince artistas peruanos emergentes —Sergio Abugattás, Miguel Andrade, Víctor Castro, Elena Damiani, Giuseppe De Bernardi, Nicole Franchy, Alejandro Jaime, Manuel Larrea, Martín Jiménez Paz, Christians Luna, José Carlos Martinat, José Miyashiro, Raura Oblitas, Ishmael Randall Weeks e Iliana Scheggia— que ocuparon el edificio del Museo de Arte Contemporáneo de Lima cuando aún estaba a medio construir. La muestra convirtió la arquitectura inconclusa y su entorno (el parque de la antigua «laguna» de Barranco) en soporte y tema: las obras tematizan la construcción/destrucción, el paisaje, la memoria del sitio y la disputa pública por el museo, cuyo proceso estuvo marcado por conflictos municipales y un intento de clausura respondido con el gesto «CLAUSURADO = INAUGURADO». El catálogo reúne textos institucionales (George Gruenberg, presidente del IAC), una pieza literaria de Ricardo Ramón Jarne («La maldición de la laguna»), un ensayo antropológico de Giuliana Borea sobre la construcción del lugar y el «lugar común» en la esfera pública (apoyado en Augé, Appadurai, Certeau y Casey), el texto curatorial de Villacorta y Zegarra, y los statements de cada artista. Como fuente histórica documenta un episodio clave de institucionalización del arte contemporáneo en Lima —la génesis del MAC— y las prácticas site-specific, de crítica institucional y de intervención en el espacio público de una generación emergente peruana de fines de la década de 2000.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Arte al Paso 2011</t>
+          <t>Cap 2 - Historia</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Cronología Político Artistica - Arte al Paso 2011.md</t>
+          <t>sura.md</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>1962 – 2010</t>
+          <t>mediados de la década de 1960 a 2013 (arte contemporáneo peruano)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Cronología y bibliografía de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Catálogo de colección museística, 2013</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Museo de Arte de Lima (MALI); Grupo Arte Nuevo; Grupo Señal; E.P.S. Huayco; Taller NN; Colectivo Sociedad Civil; Gustavo Buntinx; Joaquín López Antay; Comisión de la Verdad y Reconciliación; Sendero Luminoso; Alberto Fujimori; Juan Velasco Alvarado</t>
+          <t>Sharon Lerner (ed.); Museo de Arte de Lima (MALI); Grupo SURA; Mirko Lauer; E.P.S. Huayco; Charo Noriega; Ramiro Llona; Flavia Gandolfo; Armando Andrade Tudela; Ricardo Wiesse; Eduardo Villanes; Miguel A. López; Rodrigo Quijano</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Cronologia politico-artistica bilingue (castellano/portugues) incluida en el catalogo Arte al paso, que entrelaza en paralelo tres series de acontecimientos —eventos politicos, eventos artisticos y adquisiciones de la coleccion de arte contemporaneo del MALI— entre 1962 y 2010. El documento funciona como aparato historiografico que contextualiza la escena artistica peruana dentro de sus convulsiones politicas: rebeliones campesinas y golpes militares de los anos sesenta, el Gobierno Revolucionario de las Fuerzas Armadas de Velasco Alvarado (1968) y la Reforma Agraria, el estallido del conflicto armado interno con Sendero Luminoso y el MRTA (1980), las masacres de Barrios Altos y La Cantuta, el autogolpe y la dictadura de Alberto Fujimori (1990-2000), la Marcha de los Cuatro Suyos y el Informe de la Comision de la Verdad y Reconciliacion (2003). En el plano artistico registra la formacion de los grupos Senal y Arte Nuevo, las Bienales de Lima e Iberoamericanas, los festivales Contacta e Inkarri, el Taller E.P.S. Huayco y el Taller NN, la premiacion de Joaquin Lopez Antay, y acciones de arte critico como Cantuta de Ricardo Wiesse, Gloria evaporada de Eduardo Villanes y Lava la bandera del Colectivo Sociedad Civil. Una tercera linea traza la institucionalizacion del MALI: el ciclo curatorial Miradas de fin de siglo, la creacion del Comite de Adquisiciones (2007) y la reapertura del museo (2010). Se acompana de una extensa bibliografia especializada (Buntinx, Castrillon, Lauer, Majluf, Lopez, Tarazona, Quijano, Villacorta), fuente clave para la historiografia del arte peruano contemporaneo.</t>
+          <t>Catálogo de la colección de arte contemporáneo del Museo de Arte de Lima (MALI), editado por la curadora Sharon Lerner y publicado con el patrocinio del grupo SURA. El volumen traza los derroteros del arte peruano reciente a partir del acervo del museo, sin pretender definir un 'arte peruano' esencial. La colección se articula bajo dos principios: identificar momentos de ruptura en la producción artística de fines del siglo XX y perfilar la producción reciente mediante ejes temáticos comunes. El ensayo central de Lerner establece como punto de partida mediados de la década de 1960 (grupos de vanguardia ligados al Pop y al no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, tras las reformas del Gobierno Militar, cuando —según la célebre frase de Mirko Lauer para la muestra Arte al paso del colectivo E.P.S. Huayco (1980)— 'en el Perú hoy solo lo popular es moderno'. Analiza la irrupción de la migración interna, el conflicto armado interno, el autogolpe de Fujimori (1992) y la virtual desaparición de la esfera pública, así como la Bienal Iberoamericana de Lima (1997) como puesta al día forzada y descontextualizada. El catálogo se organiza en núcleos temáticos: modernidad popular y transformación de Lima, f(r)icciones cosmopolitas, reconsideración del pasado y configuración del Perú, sistema artístico y utopías museales, desplazamientos, y signos de violencia, resistencia y memoria. Incluye obras de Charo Noriega, Ramiro Llona, Flavia Gandolfo, Armando Andrade Tudela, Herman Schwarz, Ricardo Wiesse y Eduardo Villanes, entre otros, y textos críticos complementarios. Su aporte es consolidar un relato historiográfico y crítico del arte contemporáneo peruano desde una institución museal.</t>
         </is>
       </c>
     </row>
@@ -2526,91 +2526,91 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Texto de la exposición Arte al Paso 2011.md</t>
+          <t>Arte al Paso - Texto Investigación.md</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 1960 – 2010 (unos 40 años; foco en las décadas de 1970-1980)</t>
+          <t>Fines de los años 1960 – 2010 (con foco en las décadas de 1970-2000 y el conflicto armado interno 1980-2000)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Texto de sala / presentación de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Ensayo curatorial de catálogo (exposición Arte al paso, Pinacoteca do Estado de São Paulo, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Emilio Hernández Saavedra; E.P.S. Huayco; Grupo Paréntesis; Sandra Gamarra; Susana Torres; Emilio Rodríguez Larraín; Juan Javier Salazar; William Cordova; José Carlos Martinat</t>
+          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Pinacoteca de São Paulo; Emilio Hernández Saavedra; E.P.S. Huayco; Jesús Ruiz Durand; Sandra Gamarra; Alfredo Márquez / Taller NN; Fernando Bryce; José Carlos Martinat; Susana Torres</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Texto de sala o presentacion general de la exposicion Arte al paso (coleccion contemporanea del MALI en la Pinacoteca de Sao Paulo), firmado por los curadores Tatiana Cuevas y Rodrigo Quijano, en edicion bilingue castellano/portugues. Es una version sintetica del argumento curatorial: parte nuevamente de El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra como metafora de la ausencia institucional y punto de arranque para examinar la escena artistica peruana desde fines de los anos sesenta. Explica el titulo de la muestra a partir de la accion Arte al paso de E.P.S. Huayco (1980) —que, aludiendo a los puestos informales de comida al paso surgidos con la migracion y la economia informal, propuso un arte para consumirse en la calle, opuesto al museo y la galeria ausentes, un arte para pensar y no para sentir que dejaba atras el modernismo conservador de mediados de siglo. Sintetiza cuarenta anos de produccion cultural marcados por oposiciones ocultas y explicitas, los primeros acercamientos al conceptualismo y a las vanguardias internacionales, y la creciente proyeccion internacional de artistas peruanos. Una segunda seccion, Critica ante una institucionalidad faltante y al poder redentor del pasado, reune a Hernandez Saavedra, los grupos Parentesis y E.P.S. Huayco y el museo ficticio de Sandra Gamarra como estrategias de critica institucional apropiadas del conceptualismo y del imaginario popular urbano, con recurrente uso del humor. Aborda ademas la critica a la explotacion comercial y politica de lo prehispanico (Museo Neo-Inka de Susana Torres) y el vinculo entre la retorica del glorioso pasado incaico y los fracasos politicos y economicos del presente en obras de Rodriguez Larrain, Salazar, Cordova y Martinat.</t>
+          <t>Ensayo curatorial extenso y bilingüe (castellano/portugués) de Tatiana Cuevas y Rodrigo Quijano para la muestra Arte al paso, que exhibió la coleccion contemporanea del MALI en la Estacion Pinacoteca de Sao Paulo. El texto toma como punto de partida la imagen El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra para diagnosticar los vacios institucionales y la distancia entre el discurso cultural cosmopolita y la practica real en el Peru de la segunda mitad del siglo XX. Su argumento articula el arte contemporaneo peruano con las transformaciones sociales derivadas de la masiva migracion rural a Lima, la explosion de la economia informal y la emergencia de una nueva cultura popular urbana. Rastrea las primeras vinculaciones locales con vanguardias internacionales (op, pop, conceptualismo, no-objetualismo), el pop achorado de Jesus Ruiz Durand y sus afiches de la Reforma Agraria velasquista, y las experiencias colectivas Contacta 79 y Arte al paso de E.P.S. Huayco (1980), que propusieron un arte callejero y antiinstitucional. Analiza la critica a la institucionalidad faltante (el museo ficticio LiMAC de Sandra Gamarra), el uso ironico del pasado prehispanico (Susana Torres, Rodriguez Larrain, Bryce, Cordova, Martinat), el tema del paisaje y el territorio, y la irrupcion tardia de la fotografia y la serigrafia como medios. Dedica una seccion central a la memoria de la violencia del conflicto armado interno (1980-2000) —Sendero Luminoso, MRTA, la Comision de la Verdad, 69.280 muertos— y su tratamiento por el Taller NN, Alfredo Marquez (Katatay), Carlos Dominguez, Ricardo Wiesse, Eduardo Villanes, Fernando Bryce y Milagros de la Torre.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Hueso Húmero 18</t>
+          <t>Cap 2 - Historia/Arte al Paso 2011</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - Arte joven peruano, ¿el sueño del mercado propio? Una conversación con Claudia Polar (1983) [Hueso Húmero 18, pp. 94-107].md</t>
+          <t>Cronología Político Artistica - Arte al Paso 2011.md</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>1974-1983</t>
+          <t>1962 – 2010</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Entrevista en revista (Hueso Húmero 18), 1983</t>
+          <t>Cronología y bibliografía de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Claudia Polar; Galería Forum; Elida Román; Hernán Pazos; Esther Vainstein; Ramiro Llona; Bill Caro; Herbert Rodríguez; EAPUC; ENBA; Hueso Húmero</t>
+          <t>Museo de Arte de Lima (MALI); Grupo Arte Nuevo; Grupo Señal; E.P.S. Huayco; Taller NN; Colectivo Sociedad Civil; Gustavo Buntinx; Joaquín López Antay; Comisión de la Verdad y Reconciliación; Sendero Luminoso; Alberto Fujimori; Juan Velasco Alvarado</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Entrevista conducida por Gustavo Buntinx a Claudia Polar, directora de la Galería Forum, concebida como contraparte de un reportaje previo a Elida Román para perfilar el mercado del arte joven peruano. Polar reconstruye la fundación de Forum en diciembre de 1974 como un espacio destinado a priorizar a los artistas jóvenes y a gestar deliberadamente un mercado y coleccionistas nuevos, mediante becas, premios, subvenciones informales (incluso marcos y pasajes) y una política de "riesgo total" sostenida por la venta de stock. El diálogo traza una periodización económica de la plástica: expansión del mercado hacia 1974-1976, auge en 1978 atribuido a la restricción de importaciones bajo Morales Bermúdez, y recesión desde 1980 con la apertura de Belaúnde, siendo 1983 el año más difícil. Se discute la naturaleza del público comprador (gente joven, profesionales, empresarios, bancos como el de Crédito y el Continental) y la débil proporción de compradores habituales, apenas un 5% con relación económica. Buntinx presiona sobre las mediaciones de clase: el vínculo de Forum con la Universidad Católica frente a la ENBA, la identidad ideológica compartida, y el papel de las relaciones públicas como "gatillo" de casi toda venta en un mercado de "sala de estar". Polar aborda la diferencia entre lo culto y lo popular, el fracaso de asociar galerías, las cotizaciones (Llona, Caro, Pazos, Vainstein) y la explotación del artista acostumbrado a vender barato. El aporte documental es excepcional: registra desde dentro la lógica comercial, simbólica y provinciana del circuito limeño de principios de los ochenta.</t>
+          <t>Cronologia politico-artistica bilingue (castellano/portugues) incluida en el catalogo Arte al paso, que entrelaza en paralelo tres series de acontecimientos —eventos politicos, eventos artisticos y adquisiciones de la coleccion de arte contemporaneo del MALI— entre 1962 y 2010. El documento funciona como aparato historiografico que contextualiza la escena artistica peruana dentro de sus convulsiones politicas: rebeliones campesinas y golpes militares de los anos sesenta, el Gobierno Revolucionario de las Fuerzas Armadas de Velasco Alvarado (1968) y la Reforma Agraria, el estallido del conflicto armado interno con Sendero Luminoso y el MRTA (1980), las masacres de Barrios Altos y La Cantuta, el autogolpe y la dictadura de Alberto Fujimori (1990-2000), la Marcha de los Cuatro Suyos y el Informe de la Comision de la Verdad y Reconciliacion (2003). En el plano artistico registra la formacion de los grupos Senal y Arte Nuevo, las Bienales de Lima e Iberoamericanas, los festivales Contacta e Inkarri, el Taller E.P.S. Huayco y el Taller NN, la premiacion de Joaquin Lopez Antay, y acciones de arte critico como Cantuta de Ricardo Wiesse, Gloria evaporada de Eduardo Villanes y Lava la bandera del Colectivo Sociedad Civil. Una tercera linea traza la institucionalizacion del MALI: el ciclo curatorial Miradas de fin de siglo, la creacion del Comite de Adquisiciones (2007) y la reapertura del museo (2010). Se acompana de una extensa bibliografia especializada (Buntinx, Castrillon, Lauer, Majluf, Lopez, Tarazona, Quijano, Villacorta), fuente clave para la historiografia del arte peruano contemporaneo.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Hueso Húmero 18</t>
+          <t>Cap 2 - Historia/Arte al Paso 2011</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - ¿Entre lo popular y lo moderno? Alternativas pretendidas o reales en la joven plástica peruana (1983) [Hueso Húmero 18, pp. 61-85].md</t>
+          <t>Texto de la exposición Arte al Paso 2011.md</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>1960-1984 (con énfasis en los años 70)</t>
+          <t>Fines de los años 1960 – 2010 (unos 40 años; foco en las décadas de 1970-1980)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
+          <t>Texto de sala / presentación de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Mirko Lauer; Juan Acha; Francisco Mariotti; Huayco E.P.S.; Herbert Rodríguez; Juan Javier Salazar; Jesús Ruiz Durand; Fernando de Szyszlo; IAC; Galería Forum; SINAMOS; Néstor García Canclini</t>
+          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Emilio Hernández Saavedra; E.P.S. Huayco; Grupo Paréntesis; Sandra Gamarra; Susana Torres; Emilio Rodríguez Larraín; Juan Javier Salazar; William Cordova; José Carlos Martinat</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Ensayo teórico-histórico que propone hipótesis de trabajo sobre lo que fue o pretendió ser alternativo en el arte erudito peruano desde la transición al primer belaundismo hasta los años ochenta, articulando dos tópicos móviles: lo popular y lo moderno. Retomando y ampliando a Mirko Lauer, Buntinx sostiene que las opciones estéticas no reflejan mecánicamente la época sino que reproducen una inserción particular en el mercado, entendido como trama compleja de producción, intermediación y consumo (soporte social). Recorre así una secuencia de "soportes": el corporativo (IAC financiado por IPC, IBM, Tecnoquímica) que sostuvo la Teoría de las Raíces Nacionales de Szyszlo; el soporte "de punta" del frenesí pop cosmopolita (Acha, Arte Nuevo, Fundación para las Artes, 1966-1969); el soporte estatal velasquista con sus cuatro alternativas (comunicación masiva de Ruiz Durand con su "pop achorado", festivales de arte-total como Contacta e Inkarri, revaloración de lo artesanal, López Antay); y la frustrada búsqueda de un soporte alternativo hacia 1977-1980. El caso central es Huayco E.P.S., cuyo proyecto Sarita Colonia codifica una modernidad sincrética limeña sostenida por una pequeña burguesía ilustrada radicalizada, y cuya dispersión coincide con el agotamiento de la izquierda y el repliegue hacia el mercado galerístico (Forum). El marco conceptual bebe de García Canclini. La tesis es incisiva: el tránsito de la imagen telúrica a la industrial, agraria y migrante revela apropiaciones sucesivas de una idea variable de lo popular, siempre con una radicalidad deficiente y una relación desigual con la cultura interpretada.</t>
+          <t>Texto de sala o presentacion general de la exposicion Arte al paso (coleccion contemporanea del MALI en la Pinacoteca de Sao Paulo), firmado por los curadores Tatiana Cuevas y Rodrigo Quijano, en edicion bilingue castellano/portugues. Es una version sintetica del argumento curatorial: parte nuevamente de El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra como metafora de la ausencia institucional y punto de arranque para examinar la escena artistica peruana desde fines de los anos sesenta. Explica el titulo de la muestra a partir de la accion Arte al paso de E.P.S. Huayco (1980) —que, aludiendo a los puestos informales de comida al paso surgidos con la migracion y la economia informal, propuso un arte para consumirse en la calle, opuesto al museo y la galeria ausentes, un arte para pensar y no para sentir que dejaba atras el modernismo conservador de mediados de siglo. Sintetiza cuarenta anos de produccion cultural marcados por oposiciones ocultas y explicitas, los primeros acercamientos al conceptualismo y a las vanguardias internacionales, y la creciente proyeccion internacional de artistas peruanos. Una segunda seccion, Critica ante una institucionalidad faltante y al poder redentor del pasado, reune a Hernandez Saavedra, los grupos Parentesis y E.P.S. Huayco y el museo ficticio de Sandra Gamarra como estrategias de critica institucional apropiadas del conceptualismo y del imaginario popular urbano, con recurrente uso del humor. Aborda ademas la critica a la explotacion comercial y politica de lo prehispanico (Museo Neo-Inka de Susana Torres) y el vinculo entre la retorica del glorioso pasado incaico y los fracasos politicos y economicos del presente en obras de Rodriguez Larrain, Salazar, Cordova y Martinat.</t>
         </is>
       </c>
     </row>
@@ -2622,27 +2622,27 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Freire - Herbert Rodríguez, azote y azúcar con el sistema (1983) [Hueso Húmero 18, pdf pp. 178-185].md</t>
+          <t>Buntinx - Arte joven peruano, ¿el sueño del mercado propio? Una conversación con Claudia Polar (1983) [Hueso Húmero 18, pp. 94-107].md</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>1979-1983 (con antecedentes desde 1968)</t>
+          <t>1974-1983</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Reseña crítica en revista (Hueso Húmero 18), 1983</t>
+          <t>Entrevista en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Luis Freire S.; Herbert Rodríguez; Francisco Mariotti; Huayco E.P.S.; Juan Acha; Fernando Bedoya; Juan Javier Salazar; Bienal de Sao Paulo; Galería La Rama Dorada; Galería Forum; EAPUC; ENBAP</t>
+          <t>Gustavo Buntinx; Claudia Polar; Galería Forum; Elida Román; Hernán Pazos; Esther Vainstein; Ramiro Llona; Bill Caro; Herbert Rodríguez; EAPUC; ENBA; Hueso Húmero</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Perfil crítico dedicado a Herbert Rodríguez Huachín en la sección "Individuales" de Hueso Húmero, escrito por Luis Freire, que examina el salto vertiginoso del artista desde la suspensión disciplinaria en la Escuela de Artes Plásticas de la Católica (1981) hasta su presencia en la XVII Bienal de Sao Paulo (1983). Freire sitúa a Rodríguez como imposible de explicar sin el proceso ideológico del populismo velasquista y sin la figura mediadora de Francisco Mariotti, artista suizo-peruano formado en la Documenta de Kassel y la vanguardia europea, catalizador de Contacta y de la EPS Huayco. El texto reconstruye la genealogía Mariotti-Huayco-Rodríguez: los ensamblajes y "reciclajes" del suizo-peruano derivan en los "altares" de Rodríguez, hibridación entre constructivismo geométrico, expresionismo "pobre" y antiestético, y estructuras rituales de la religiosidad popular andina. Argumenta que Rodríguez encarna las contradicciones de una pequeña burguesía radical: dinamita el circuito con una mano y lo enluce con la otra, camuflando "bellamente" materiales pobres y reciclados en obras a la vez contestatarias y comerciables, con lo que ironiza sobre el culto al oficio del arte establecido. Analiza su heterogeneidad de lenguajes (expresionismo abstracto, figuración dura, conceptualismo informal, collage, fotocopia, ensamblaje) como búsqueda pero también como crisis, y sus "altares al Yo" exhibidos en Forum (1983) y la Bienal. Freire lo define como un artista religioso-existencial populista sin referentes sólidos, en formación, tensionado entre enriquecer el jardín burgués que quiere pisotear o saltar a opciones más radicales de ruptura.</t>
+          <t>Entrevista conducida por Gustavo Buntinx a Claudia Polar, directora de la Galería Forum, concebida como contraparte de un reportaje previo a Elida Román para perfilar el mercado del arte joven peruano. Polar reconstruye la fundación de Forum en diciembre de 1974 como un espacio destinado a priorizar a los artistas jóvenes y a gestar deliberadamente un mercado y coleccionistas nuevos, mediante becas, premios, subvenciones informales (incluso marcos y pasajes) y una política de "riesgo total" sostenida por la venta de stock. El diálogo traza una periodización económica de la plástica: expansión del mercado hacia 1974-1976, auge en 1978 atribuido a la restricción de importaciones bajo Morales Bermúdez, y recesión desde 1980 con la apertura de Belaúnde, siendo 1983 el año más difícil. Se discute la naturaleza del público comprador (gente joven, profesionales, empresarios, bancos como el de Crédito y el Continental) y la débil proporción de compradores habituales, apenas un 5% con relación económica. Buntinx presiona sobre las mediaciones de clase: el vínculo de Forum con la Universidad Católica frente a la ENBA, la identidad ideológica compartida, y el papel de las relaciones públicas como "gatillo" de casi toda venta en un mercado de "sala de estar". Polar aborda la diferencia entre lo culto y lo popular, el fracaso de asociar galerías, las cotizaciones (Llona, Caro, Pazos, Vainstein) y la explotación del artista acostumbrado a vender barato. El aporte documental es excepcional: registra desde dentro la lógica comercial, simbólica y provinciana del circuito limeño de principios de los ochenta.</t>
         </is>
       </c>
     </row>
@@ -2654,12 +2654,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Lama - Los años de la resaca (1983) [Hueso Húmero 18, pdf pp. 136-156].md</t>
+          <t>Buntinx - ¿Entre lo popular y lo moderno? Alternativas pretendidas o reales en la joven plástica peruana (1983) [Hueso Húmero 18, pp. 61-85].md</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>1974-1983 (con antecedentes en los años 60-70)</t>
+          <t>1960-1984 (con énfasis en los años 70)</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -2669,76 +2669,76 @@
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Luis Lama; Hernán Pazos; Francisco Mariotti; Contacta; grupo Huayco; Juan Javier Salazar; Herbert Rodríguez; Alfonso Castrillón; Escuela Nacional de Bellas Artes; Galería Forum; Galería 9; Ugarte Eléspuru</t>
+          <t>Gustavo Buntinx; Mirko Lauer; Juan Acha; Francisco Mariotti; Huayco E.P.S.; Herbert Rodríguez; Juan Javier Salazar; Jesús Ruiz Durand; Fernando de Szyszlo; IAC; Galería Forum; SINAMOS; Néstor García Canclini</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Ensayo de Luis Lama que narra el paso de la "ebullición ideológica" de los años setenta a la "resaca" del segundo belaundismo, articulando historia social del arte y crítica biográfica. La primera parte reconstruye los antecedentes: el terremoto de 1974 y el reflujo de artistas jóvenes hacia Barranco, la gravitación de Francisco Mariotti que transforma el arte de sistemas en movimiento grupal con Contacta e Inkari bajo auspicio de SINAMOS, las tomas y la crisis de la Escuela Nacional de Bellas Artes (1974-1976), y la gestación del taller de Pedro de Osma que devendría núcleo del grupo Huayco (Juan Javier Salazar, Herbert Rodríguez, Charo Noriega, Fernando Bedoya, Lucy Angulo). Lama describe la consolidación paradójica del mercado del arte al amparo de la prohibición de importaciones, con galerías que proliferan mientras la formación académica alcanza sus niveles más bajos. Diagnostica el fin de los happenings sesenteros y el retorno de un expresionismo "de crisis" impulsado desde los predios católicos (Williams, Polanco, Velarde, Hamann), junto a indagaciones matéricas de Wiesse y el conceptualismo de Vainstein. La segunda mitad es un retrato extenso de Hernán Pazos: su formación entre Derecho, la Católica y París, su tránsito del conceptualismo (los cielos y nubes de Galería 9) a la abstracción cromática, las series de los Quipus y los dibujos infantiles, su gestión en Rama Dorada y su individualismo parricida. Lama lo consagra como el artista más destacado de la década, emblema lúcido de las "amargas frustraciones" nacionales bajo el liberalismo económico belaundista.</t>
+          <t>Ensayo teórico-histórico que propone hipótesis de trabajo sobre lo que fue o pretendió ser alternativo en el arte erudito peruano desde la transición al primer belaundismo hasta los años ochenta, articulando dos tópicos móviles: lo popular y lo moderno. Retomando y ampliando a Mirko Lauer, Buntinx sostiene que las opciones estéticas no reflejan mecánicamente la época sino que reproducen una inserción particular en el mercado, entendido como trama compleja de producción, intermediación y consumo (soporte social). Recorre así una secuencia de "soportes": el corporativo (IAC financiado por IPC, IBM, Tecnoquímica) que sostuvo la Teoría de las Raíces Nacionales de Szyszlo; el soporte "de punta" del frenesí pop cosmopolita (Acha, Arte Nuevo, Fundación para las Artes, 1966-1969); el soporte estatal velasquista con sus cuatro alternativas (comunicación masiva de Ruiz Durand con su "pop achorado", festivales de arte-total como Contacta e Inkarri, revaloración de lo artesanal, López Antay); y la frustrada búsqueda de un soporte alternativo hacia 1977-1980. El caso central es Huayco E.P.S., cuyo proyecto Sarita Colonia codifica una modernidad sincrética limeña sostenida por una pequeña burguesía ilustrada radicalizada, y cuya dispersión coincide con el agotamiento de la izquierda y el repliegue hacia el mercado galerístico (Forum). El marco conceptual bebe de García Canclini. La tesis es incisiva: el tránsito de la imagen telúrica a la industrial, agraria y migrante revela apropiaciones sucesivas de una idea variable de lo popular, siempre con una radicalidad deficiente y una relación desigual con la cultura interpretada.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/MALI</t>
+          <t>Cap 2 - Historia/Hueso Húmero 18</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - El poder y la ilusión. Pérdida y restauración del aura en la «República de Weimar peruana» 1980-1992 [MALI].md</t>
+          <t>Freire - Herbert Rodríguez, azote y azúcar con el sistema (1983) [Hueso Húmero 18, pdf pp. 178-185].md</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>1980-1992</t>
+          <t>1979-1983 (con antecedentes desde 1968)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico (versión MALI), 2013 [escrito 1991-1994]</t>
+          <t>Reseña crítica en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; E.P.S. Huayco; Taller NN; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; Walter Benjamin; Jesús Ruiz Durand; Andy Warhol; Mirko Lauer; Museo de Arte de Lima (MALI); III Bienal de La Habana</t>
+          <t>Luis Freire S.; Herbert Rodríguez; Francisco Mariotti; Huayco E.P.S.; Juan Acha; Fernando Bedoya; Juan Javier Salazar; Bienal de Sao Paulo; Galería La Rama Dorada; Galería Forum; EAPUC; ENBAP</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Ensayo seminal de Gustavo Buntinx —redactado entre 1991 y 1994, difundido en inglés en «Beyond the Fantastic» (1995) y publicado por primera vez en Perú en esta versión del MALI (2013)— que interpreta el radical cambio de época del arte peruano entre 1980 y 1992, periodo que denomina metafóricamente «República de Weimar peruana». Su marco conceptual adapta la dialéctica benjaminiana entre proximidad y distancia (el aura, su pérdida por la reproductibilidad técnica y su posible restauración) y las categorías de alegoría, montaje y apropiación de Owens, Foster y Craig Owens a una periferia extrema. El argumento se sostiene sobre el análisis iconográfico minucioso de dos o tres obras que abren y cierran la década. La primera, «Arte al paso» y sobre todo «Sarita Colonia» (1980) del taller E.P.S. Huayco: una enorme estampa de la santa migrante pintada sobre diez mil latas de leche y emplazada en la Panamericana Sur, que Buntinx lee como huaca (post)moderna y exvoto donde lo pequeñoburgués radical se articula figuradamente a lo popular en emergencia (el «pop achorado» y «chicha»). La segunda, «Maorilyn» / «Viva el maoísmo» (1989) del Taller NN: una serigrafía que travistió el rostro de Mao con labios warholianos, alegoría ambivalente de la violencia senderista y la estetización de la política. Su tesis vincula la desintegración social —hiperinflación, guerra civil, movida subte punk— con el desarrollo de una condición alegórica y neo-aurática; su aporte es un modelo teórico para leer el colectivismo y la (post)modernidad popular peruana.</t>
+          <t>Perfil crítico dedicado a Herbert Rodríguez Huachín en la sección "Individuales" de Hueso Húmero, escrito por Luis Freire, que examina el salto vertiginoso del artista desde la suspensión disciplinaria en la Escuela de Artes Plásticas de la Católica (1981) hasta su presencia en la XVII Bienal de Sao Paulo (1983). Freire sitúa a Rodríguez como imposible de explicar sin el proceso ideológico del populismo velasquista y sin la figura mediadora de Francisco Mariotti, artista suizo-peruano formado en la Documenta de Kassel y la vanguardia europea, catalizador de Contacta y de la EPS Huayco. El texto reconstruye la genealogía Mariotti-Huayco-Rodríguez: los ensamblajes y "reciclajes" del suizo-peruano derivan en los "altares" de Rodríguez, hibridación entre constructivismo geométrico, expresionismo "pobre" y antiestético, y estructuras rituales de la religiosidad popular andina. Argumenta que Rodríguez encarna las contradicciones de una pequeña burguesía radical: dinamita el circuito con una mano y lo enluce con la otra, camuflando "bellamente" materiales pobres y reciclados en obras a la vez contestatarias y comerciables, con lo que ironiza sobre el culto al oficio del arte establecido. Analiza su heterogeneidad de lenguajes (expresionismo abstracto, figuración dura, conceptualismo informal, collage, fotocopia, ensamblaje) como búsqueda pero también como crisis, y sus "altares al Yo" exhibidos en Forum (1983) y la Bienal. Freire lo define como un artista religioso-existencial populista sin referentes sólidos, en formación, tensionado entre enriquecer el jardín burgués que quiere pisotear o saltar a opciones más radicales de ruptura.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/MALI</t>
+          <t>Cap 2 - Historia/Hueso Húmero 18</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Lerner - Formando la colección de arte contemporáneo del MALI (2013).txt</t>
+          <t>Lama - Los años de la resaca (1983) [Hueso Húmero 18, pdf pp. 136-156].md</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>mediados de los años 60 - 2013 (con foco en 1980-2000)</t>
+          <t>1974-1983 (con antecedentes en los años 60-70)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo de colección, 2013</t>
+          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Museo de Arte de Lima (MALI); Tatiana Cuevas; Miguel A. López; Gustavo Buntinx; Rodrigo Quijano; Jorge Villacorta; Natalia Majluf; E.P.S. Huayco; Teresa Burga; Milagros de la Torre; Flavia Gandolfo</t>
+          <t>Luis Lama; Hernán Pazos; Francisco Mariotti; Contacta; grupo Huayco; Juan Javier Salazar; Herbert Rodríguez; Alfonso Castrillón; Escuela Nacional de Bellas Artes; Galería Forum; Galería 9; Ugarte Eléspuru</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Ensayo introductorio de Sharon Lerner al libro que presenta la colección de arte contemporáneo del Museo de Arte de Lima (MALI), articulado como una lectura —entre muchas posibles— de la historia del arte reciente peruano a partir del acervo. Su tesis metodológica es que en el Perú el tránsito a la contemporaneidad no ocurre como un quiebre radical, sino como una serie de pequeños cambios discontinuos, por lo que la colección se organiza en dos principios: identificar momentos de ruptura de fines del siglo XX y perfilar la producción reciente por ejes temáticos. El recorrido histórico parte de mediados de los sesenta (vanguardias pop, experimentalismo, no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, cuando la migración y la sentencia de Mirko Lauer —«En el Perú, hoy, solo lo popular es moderno»— enmarcan la obra de E.P.S. Huayco. Recorre luego la hegemonía de la abstracción en los ochenta, el arte de derechos humanos de Ricardo Wiesse y Eduardo Villanes bajo el fujimorato, la irrupción de la Bienal Iberoamericana de Lima (1997) y el «bienalismo», y la generación de los 2000 (Flavia Gandolfo, Gilda Mantilla, Armando Andrade Tudela) vinculada al espacio La Culpable. El texto presenta además los ensayos de Miguel López, Gustavo Buntinx y Rodrigo Quijano incluidos en el volumen y la conversación de seis críticos (2011). Su aporte es explicitar la política de adquisiciones del MALI y su ambición de llenar el vacío institucional y discursivo, construyendo un marco regional e internacional para el arte peruano.</t>
+          <t>Ensayo de Luis Lama que narra el paso de la "ebullición ideológica" de los años setenta a la "resaca" del segundo belaundismo, articulando historia social del arte y crítica biográfica. La primera parte reconstruye los antecedentes: el terremoto de 1974 y el reflujo de artistas jóvenes hacia Barranco, la gravitación de Francisco Mariotti que transforma el arte de sistemas en movimiento grupal con Contacta e Inkari bajo auspicio de SINAMOS, las tomas y la crisis de la Escuela Nacional de Bellas Artes (1974-1976), y la gestación del taller de Pedro de Osma que devendría núcleo del grupo Huayco (Juan Javier Salazar, Herbert Rodríguez, Charo Noriega, Fernando Bedoya, Lucy Angulo). Lama describe la consolidación paradójica del mercado del arte al amparo de la prohibición de importaciones, con galerías que proliferan mientras la formación académica alcanza sus niveles más bajos. Diagnostica el fin de los happenings sesenteros y el retorno de un expresionismo "de crisis" impulsado desde los predios católicos (Williams, Polanco, Velarde, Hamann), junto a indagaciones matéricas de Wiesse y el conceptualismo de Vainstein. La segunda mitad es un retrato extenso de Hernán Pazos: su formación entre Derecho, la Católica y París, su tránsito del conceptualismo (los cielos y nubes de Galería 9) a la abstracción cromática, las series de los Quipus y los dibujos infantiles, su gestión en Rama Dorada y su individualismo parricida. Lama lo consagra como el artista más destacado de la década, emblema lúcido de las "amargas frustraciones" nacionales bajo el liberalismo económico belaundista.</t>
         </is>
       </c>
     </row>
@@ -2750,27 +2750,27 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - F(r)icciones cosmopolitas. Redefiniciones estéticas y políticas de una idea de vanguardia en los años 60s.txt</t>
+          <t>Buntinx - El poder y la ilusión. Pérdida y restauración del aura en la «República de Weimar peruana» 1980-1992 [MALI].md</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>1960-1976 (con antecedentes desde 1942-1947)</t>
+          <t>1980-1992</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico / capítulo de catálogo (MALI), s/f</t>
+          <t>Ensayo académico (versión MALI), 2013 [escrito 1991-1994]</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Emilio Tarazona; Juan Acha; Fernando de Szyszlo; Jorge Romero Brest; Teresa Burga; Rafael Hastings; Grupo Arte Nuevo; Jesús Ruiz Durand; José Gómez Sicre; Marta Traba; Instituto de Arte Contemporáneo (IAC); MoMA / Instituto Di Tella</t>
+          <t>Gustavo Buntinx; E.P.S. Huayco; Taller NN; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; Walter Benjamin; Jesús Ruiz Durand; Andy Warhol; Mirko Lauer; Museo de Arte de Lima (MALI); III Bienal de La Habana</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>López reconstruye las mutaciones semánticas y políticas de la noción de vanguardia en el Perú entre los años sesenta y setenta, argumentando que la euforia cosmopolita del periodo fue el espejismo de una modernidad desarrollista tan prometedora como inacabada en un país socialmente fracturado. El objeto de estudio son las plataformas institucionales privadas (IAC, galerías, bienales americanas, concursos empresariales) que, apuntaladas por el panamericanismo de la Guerra Fría, la Alianza para el Progreso y la política curatorial estadounidense de José Gómez Sicre, promovieron primero la abstracción y luego el arte óptico, el pop y las ambientaciones. El texto traza el paso del declive de la abstracción szyszliana hacia el experimentalismo detonado por las conferencias de Jorge Romero Brest (1965) y la irrupción beligerante del grupo Arte Nuevo (1966-1968) contra el Festival Americano de Pintura. El marco conceptual articula la relación entre desarrollismo y vanguardia, y su posterior tensión con el subdesarrollo, siguiendo la radicalización de Juan Acha, quien tras 1968 y el golpe de Velasco redefine la vanguardia como 'guerrilla cultural' y horizonte revolucionario, hasta su exilio a México en 1971. López destaca las reconversiones de Teresa Burga y Rafael Hastings, el 'pop achorado' de Ruiz Durand al servicio de la Reforma Agraria, los festivales Contacta y las Carreras de chasquis. Su aporte es mostrar cómo la condición local, provinciana y periférica de las prácticas de los setenta y ochenta (Paréntesis, E.P.S. Huayco, Grupo Chaclacayo) actualizó de modo radical las pretensiones críticas sesenteras, canibalizando los conceptos metropolitanos de arte conceptual.</t>
+          <t>Ensayo seminal de Gustavo Buntinx —redactado entre 1991 y 1994, difundido en inglés en «Beyond the Fantastic» (1995) y publicado por primera vez en Perú en esta versión del MALI (2013)— que interpreta el radical cambio de época del arte peruano entre 1980 y 1992, periodo que denomina metafóricamente «República de Weimar peruana». Su marco conceptual adapta la dialéctica benjaminiana entre proximidad y distancia (el aura, su pérdida por la reproductibilidad técnica y su posible restauración) y las categorías de alegoría, montaje y apropiación de Owens, Foster y Craig Owens a una periferia extrema. El argumento se sostiene sobre el análisis iconográfico minucioso de dos o tres obras que abren y cierran la década. La primera, «Arte al paso» y sobre todo «Sarita Colonia» (1980) del taller E.P.S. Huayco: una enorme estampa de la santa migrante pintada sobre diez mil latas de leche y emplazada en la Panamericana Sur, que Buntinx lee como huaca (post)moderna y exvoto donde lo pequeñoburgués radical se articula figuradamente a lo popular en emergencia (el «pop achorado» y «chicha»). La segunda, «Maorilyn» / «Viva el maoísmo» (1989) del Taller NN: una serigrafía que travistió el rostro de Mao con labios warholianos, alegoría ambivalente de la violencia senderista y la estetización de la política. Su tesis vincula la desintegración social —hiperinflación, guerra civil, movida subte punk— con el desarrollo de una condición alegórica y neo-aurática; su aporte es un modelo teórico para leer el colectivismo y la (post)modernidad popular peruana.</t>
         </is>
       </c>
     </row>
@@ -2782,27 +2782,27 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Quijano - Notas incompletas sobre el sitio de la fotografía peruana.md</t>
+          <t>Lerner - Formando la colección de arte contemporáneo del MALI (2013).txt</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>1900-2011 (con énfasis en 1920-1998)</t>
+          <t>mediados de los años 60 - 2013 (con foco en 1980-2000)</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo (MALI), s/f</t>
+          <t>Ensayo de catálogo de colección, 2013</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Quijano; Martín Chambi; José María Eguren; Carlos 'Chino' Domínguez; Aaron Siskind; Jesús Ruiz Durand; Claudia Martínez Garay; Daniela Ortiz; Foto Galería Secuencia; TAFOS; Taller NN; E.P.S. Huayco</t>
+          <t>Sharon Lerner; Museo de Arte de Lima (MALI); Tatiana Cuevas; Miguel A. López; Gustavo Buntinx; Rodrigo Quijano; Jorge Villacorta; Natalia Majluf; E.P.S. Huayco; Teresa Burga; Milagros de la Torre; Flavia Gandolfo</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>Quijano ensaya una genealogía del 'sitio' de la fotografía peruana, sosteniendo que este medio inauguró un margen de creación moderno al margen de la institucionalidad académica de las bellas artes, alcanzando una temprana ubicuidad territorial y una masividad que condicionó la percepción misma de una realidad nacional. El texto, de estructura fragmentaria y numerada, contrapone dos matrices fundacionales: Martín Chambi como 'modernista sin modernidad' y profesional de la imagen surgido de una familia campesina andina —una 'oportunidad nacional'— frente a la miniatura pinhole intimista y hermética de José María Eguren, que prefigura la figura del fotógrafo-artista individual. Analiza a Carlos 'Chino' Domínguez como ojo testimonial de la urbanización y la nueva cultura popular (La resaca del Inca, el 'Cholo' Sotil, el filme Cholo y su reedición Mi cholo de Gruenberg), y la experiencia de la fotogalería Secuencia (1977-1980), que reinventó una tradición y un discurso del oficio adoptando a Minor White y Aaron Siskind. El marco conceptual enlaza fotografía, prensa y democratización de la imagen en el contexto del auge sindical y la repolitización popular de fines de los setenta, y la aparición de la fotoserigrafía disidente (Bedoya, Williams, Mariotti, Salazar) como catalizador de una nueva condición fotográfica colectiva, desde E.P.S. Huayco hasta el Taller NN. El aporte del texto es leer la fotografía como dispositivo de documento, archivo, memoria y duelo frente a la violencia política (Uchuraccay, Yuyanapaq), rastreando su 'grado cero' icónico en obras de Ruiz Durand, Claudia Martínez Garay y Daniela Ortiz, que develan la mirada colonial y la invisibilización étnica.</t>
+          <t>Ensayo introductorio de Sharon Lerner al libro que presenta la colección de arte contemporáneo del Museo de Arte de Lima (MALI), articulado como una lectura —entre muchas posibles— de la historia del arte reciente peruano a partir del acervo. Su tesis metodológica es que en el Perú el tránsito a la contemporaneidad no ocurre como un quiebre radical, sino como una serie de pequeños cambios discontinuos, por lo que la colección se organiza en dos principios: identificar momentos de ruptura de fines del siglo XX y perfilar la producción reciente por ejes temáticos. El recorrido histórico parte de mediados de los sesenta (vanguardias pop, experimentalismo, no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, cuando la migración y la sentencia de Mirko Lauer —«En el Perú, hoy, solo lo popular es moderno»— enmarcan la obra de E.P.S. Huayco. Recorre luego la hegemonía de la abstracción en los ochenta, el arte de derechos humanos de Ricardo Wiesse y Eduardo Villanes bajo el fujimorato, la irrupción de la Bienal Iberoamericana de Lima (1997) y el «bienalismo», y la generación de los 2000 (Flavia Gandolfo, Gilda Mantilla, Armando Andrade Tudela) vinculada al espacio La Culpable. El texto presenta además los ensayos de Miguel López, Gustavo Buntinx y Rodrigo Quijano incluidos en el volumen y la conversación de seis críticos (2011). Su aporte es explicitar la política de adquisiciones del MALI y su ambición de llenar el vacío institucional y discursivo, construyendo un marco regional e internacional para el arte peruano.</t>
         </is>
       </c>
     </row>
@@ -2814,32 +2814,96 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
+          <t>López, Miguel A. - F(r)icciones cosmopolitas. Redefiniciones estéticas y políticas de una idea de vanguardia en los años 60s.txt</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>1960-1976 (con antecedentes desde 1942-1947)</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Ensayo académico / capítulo de catálogo (MALI), s/f</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Miguel A. López; Emilio Tarazona; Juan Acha; Fernando de Szyszlo; Jorge Romero Brest; Teresa Burga; Rafael Hastings; Grupo Arte Nuevo; Jesús Ruiz Durand; José Gómez Sicre; Marta Traba; Instituto de Arte Contemporáneo (IAC); MoMA / Instituto Di Tella</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>López reconstruye las mutaciones semánticas y políticas de la noción de vanguardia en el Perú entre los años sesenta y setenta, argumentando que la euforia cosmopolita del periodo fue el espejismo de una modernidad desarrollista tan prometedora como inacabada en un país socialmente fracturado. El objeto de estudio son las plataformas institucionales privadas (IAC, galerías, bienales americanas, concursos empresariales) que, apuntaladas por el panamericanismo de la Guerra Fría, la Alianza para el Progreso y la política curatorial estadounidense de José Gómez Sicre, promovieron primero la abstracción y luego el arte óptico, el pop y las ambientaciones. El texto traza el paso del declive de la abstracción szyszliana hacia el experimentalismo detonado por las conferencias de Jorge Romero Brest (1965) y la irrupción beligerante del grupo Arte Nuevo (1966-1968) contra el Festival Americano de Pintura. El marco conceptual articula la relación entre desarrollismo y vanguardia, y su posterior tensión con el subdesarrollo, siguiendo la radicalización de Juan Acha, quien tras 1968 y el golpe de Velasco redefine la vanguardia como 'guerrilla cultural' y horizonte revolucionario, hasta su exilio a México en 1971. López destaca las reconversiones de Teresa Burga y Rafael Hastings, el 'pop achorado' de Ruiz Durand al servicio de la Reforma Agraria, los festivales Contacta y las Carreras de chasquis. Su aporte es mostrar cómo la condición local, provinciana y periférica de las prácticas de los setenta y ochenta (Paréntesis, E.P.S. Huayco, Grupo Chaclacayo) actualizó de modo radical las pretensiones críticas sesenteras, canibalizando los conceptos metropolitanos de arte conceptual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Cap 2 - Historia/MALI</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Quijano - Notas incompletas sobre el sitio de la fotografía peruana.md</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>1900-2011 (con énfasis en 1920-1998)</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Ensayo de catálogo (MALI), s/f</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Rodrigo Quijano; Martín Chambi; José María Eguren; Carlos 'Chino' Domínguez; Aaron Siskind; Jesús Ruiz Durand; Claudia Martínez Garay; Daniela Ortiz; Foto Galería Secuencia; TAFOS; Taller NN; E.P.S. Huayco</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>Quijano ensaya una genealogía del 'sitio' de la fotografía peruana, sosteniendo que este medio inauguró un margen de creación moderno al margen de la institucionalidad académica de las bellas artes, alcanzando una temprana ubicuidad territorial y una masividad que condicionó la percepción misma de una realidad nacional. El texto, de estructura fragmentaria y numerada, contrapone dos matrices fundacionales: Martín Chambi como 'modernista sin modernidad' y profesional de la imagen surgido de una familia campesina andina —una 'oportunidad nacional'— frente a la miniatura pinhole intimista y hermética de José María Eguren, que prefigura la figura del fotógrafo-artista individual. Analiza a Carlos 'Chino' Domínguez como ojo testimonial de la urbanización y la nueva cultura popular (La resaca del Inca, el 'Cholo' Sotil, el filme Cholo y su reedición Mi cholo de Gruenberg), y la experiencia de la fotogalería Secuencia (1977-1980), que reinventó una tradición y un discurso del oficio adoptando a Minor White y Aaron Siskind. El marco conceptual enlaza fotografía, prensa y democratización de la imagen en el contexto del auge sindical y la repolitización popular de fines de los setenta, y la aparición de la fotoserigrafía disidente (Bedoya, Williams, Mariotti, Salazar) como catalizador de una nueva condición fotográfica colectiva, desde E.P.S. Huayco hasta el Taller NN. El aporte del texto es leer la fotografía como dispositivo de documento, archivo, memoria y duelo frente a la violencia política (Uchuraccay, Yuyanapaq), rastreando su 'grado cero' icónico en obras de Ruiz Durand, Claudia Martínez Garay y Daniela Ortiz, que develan la mirada colonial y la invisibilización étnica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Cap 2 - Historia/MALI</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
           <t>Villacorta (ed.) - ¿Un arte visual a contrapelo de los dictados metropolitanos? En el Perú, el arte moderno es un gesto tardío [conversación en el MALI, 2011].txt</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>1947-2011 (con eje en 1960-2002)</t>
         </is>
       </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="D76" s="2" t="inlineStr">
         <is>
           <t>Transcripción editada de conversación (MALI), 2011</t>
         </is>
       </c>
-      <c r="E74" s="3" t="inlineStr">
+      <c r="E76" s="3" t="inlineStr">
         <is>
           <t>Jorge Villacorta; Gustavo Buntinx; Miguel A. López; Rodrigo Quijano; Tatiana Cuevas; Natalia Majluf; E.P.S. Huayco; Grupo Arte Nuevo; Taller NN; Grupo Chaclacayo; Christian Bendayán; Fernando Bryce; MALI / Micromuseo</t>
         </is>
       </c>
-      <c r="F74" s="3" t="inlineStr">
+      <c r="F76" s="3" t="inlineStr">
         <is>
           <t>Editada por Villacorta a partir de dos sesiones de 2011 en el MALI, esta conversación a seis voces indaga si lo moderno está clausurado en el arte peruano de modo que permita definir lo contemporáneo. La tesis articuladora, propuesta por Quijano, es que en el Perú lo moderno solo ha podido darse 'a contrapelo' y como 'gesto tardío', a destiempo de las modernidades metropolitanas; López y Buntinx la matizan con la idea de temporalidades dislocadas y friccionadas que impiden toda historia lineal. El objeto de estudio es la genealogía de la vanguardia local: la contraposición entre Arte Nuevo (1966-1968), leído como destello cosmopolita fugaz, y E.P.S. Huayco y Paréntesis, cuya apropiación de Sarita Colonia y el 'pop achorado' marca una ruptura más perdurable y pertinente al medio. Buntinx despliega una secuencia estilístico-conceptual en clave pop/místico-libidinal —de la Twiggy de Emilio Hernández a Quistococha de Bendayán, pasando por el afiche de Ruiz Durand, la Maoirilyn del Taller NN y La Pachakuti de Alfredo Márquez— ligada a periodos políticos (desarrollismo, velasquismo, utopía socialista, dictadura fujimorista, revolución capitalista). Majluf sitúa el quiebre epocal de fin de siglo en el ingreso de la 'referencia' fotográfica (Bryce, Milagros de la Torre, Juan Enrique Bedoya, Mantilla), frente al neobarroco. El texto discute además la construcción de públicos, la institucionalidad faltante, el rol del curador, el mercado 'social' peruano, las subastas del MALI y la 'normalización de la diferencia' como riesgo de la consagración institucional del pasado radical.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F74"/>
+  <autoFilter ref="A1:F76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Cataloga y analiza (2.3.3 y 2.3.4) Quijano «Contra el Consenso de Lima» (2009)
- Cataloga el PDF de Rodrigo Quijano «Contra el Consenso de Lima» (rev.
  chilena Plus / Trienal de Santiago; ArteBA 2009; captura del blog «arte
  nuevo» de Miguel López, 2009) en tabla-cap2-historia.csv; Excel al día.
- Añade a analisis/ el informe de datos crudos: batería común B1-B13 y
  propias de 2.3.3 (P1-P7) y 2.3.4 (P1-P8), separando el texto de Quijano
  del aparato del blog (presentación, comentarios, índices), con citas
  literales y ubicación por § de sección.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bob4w11uQRyAcv1Qayw1V
</commit_message>
<xml_diff>
--- a/Sistematización/tablas-sistematizacion.xlsx
+++ b/Sistematización/tablas-sistematizacion.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Extras" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$77</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cap 3 - Análisis'!$A$1:$F$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Teoría'!$A$1:$F$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Extras'!$A$1:$F$4</definedName>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2430,27 +2430,27 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>canepa_kg_2006_p132-167.pdf</t>
+          <t>arte nuevo_ Contra el Consenso de Lima_ Notas incompletas sobre las colectividades artísticas en el Perú, sus nuevas, viejas condiciones - Rodrigo Quijano.pdf</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>1970-2006 (con referencias históricas desde el siglo XIX)</t>
+          <t>Perú postdictatorial (años 2000); escrito en 2009 (masacre de Bagua, 5-jun-2009); colectivos 1979-1991 y «Consenso» desde fines de los 80</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro, 2006</t>
+          <t>Ensayo de revista (chilena «Plus», Trienal de Santiago; también en «Hacia el salón del siglo XXI», ArteBA, 2009, pp. 168-178); PDF = captura del blog «arte nuevo» (Miguel López), 29-dic-2009</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Giuliana Borea Labarthe; Gisela Cánepa Koch (ed.); Sandra Gamarra (LiMAC); Instituto de Arte Contemporáneo (IAC); Fernando de Szyszlo; Gerardo Chávez; Mario Vargas Llosa; Ramiro Llona; Instituto Nacional de Cultura; ICOM; Museo de la Nación; Museo Nacional de la Cultura Peruana; Alfonso Castrillón</t>
+          <t>Rodrigo Quijano; Miguel López (blog «arte nuevo»); Alfredo Márquez; Mario Vargas Llosa; Gustavo Buntinx; Ana Longoni; grupos Paréntesis, Huayco, N.N., La Culpable, Tupac, El Colectivo, Proyecto Cultural Noviembre; MALI; Museo de la Memoria; CVR; Trienal de Santiago; ArteBA</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Capítulo de Giuliana Borea Labarthe ('Museos y esfera pública: espacio, discursos y prácticas. Reflexiones en torno a la ciudad de Lima') incluido en el volumen editado por Gisela Cánepa Koch, 'Mirando la esfera pública desde la cultura en el Perú' (2006). Partiendo de las nociones de esfera pública (Habermas), cultura pública (Appadurai) y de la nueva museología surgida de las crisis de los años 70-80 (Mesa de Santiago 1972, redefinición del ICOM 1974, ecomuseos), Borea concibe el museo como contenedor y contenido, plataforma y discurso, esfera de poder y arena de disputa por la representación. Analiza tres casos limeños. Primero, el posicionamiento urbano de los museos: mediante una encuesta a transeúntes y taxistas muestra que solo el Museo de la Nación y el Museo de Arte de Lima son hitos reconocidos, mientras la mayoría oscila entre lugar simbólico y lugar anónimo por la falta de señalización y de alianzas municipales. Segundo, la polémica de 2006 por el proyecto del Museo de Arte Contemporáneo (MAC) del IAC, detonada por el intento de nombrarlo 'Fernando de Szyszlo': reconstruye siete momentos del debate mediático (comunicados de artistas, la columna 'Escaramuzas en Liliput' de Vargas Llosa), la falta de plan museológico y de diálogo con artistas donantes y con Barranco, y destaca la contrapropuesta crítica LiMAC de Sandra Gamarra frente al silencio del INC. Tercero, compara las puestas en escena sobre peruanidad y diversidad de cinco museos (Cultura Peruana, de la Nación, Etnográfico, Inmigración Japonesa, MNAAHP), evidenciando discursos lejanos, fragmentados y ahistóricos en los grandes museos nacionales frente a autorrepresentaciones más políticas en los pequeños. Cierra con Castrillón: Lima como escenario de emplazamiento, no de reflexión.</t>
+          <t>Ensayo de Rodrigo Quijano, «Contra el Consenso de Lima. Notas incompletas sobre las colectividades artísticas en el Perú, sus nuevas, viejas condiciones», publicado en la revista chilena «Plus» (Trienal de Santiago) y reproducido en «Hacia el salón del siglo XXI» (ArteBA Fundación, 2009, pp. 168-178). El PDF es una captura del blog «arte nuevo» de Miguel López, que lo reposteó el 29 de diciembre de 2009 (con la presentación de López, el índice de Ramona 89, los comentarios de lectores y el aparato del blog). Quijano acuña la noción de «Consenso de Lima» —por alusión al Consenso de Washington— para nombrar el «espeso consenso cultural y social» conformista impuesto por la dictadura fujimorista (1990-2000) y sostenido después: una «reoligarquización simbólica» del escenario nacional (iniciada tras el intento de estatizar la banca a fines de los 80, con Vargas Llosa), un neonacionalismo (pisco, caballo de paso, comida) y la reconcentración del «producto simbólico y artístico en pocas manos privadas», con su «nuevo coleccionismo y nueva musealidad» (MALI; un frustrado Museo de Arte Moderno; un futuro Museo de la Memoria ligado a la CVR). Frente a ese consenso sitúa a las «colectividades artísticas y críticas» surgidas «a contrapelo»: Paréntesis (1979), Huayco (1980-1981), N.N. (1986-1991) y, más recientes, La Culpable, Tupac, El Colectivo o el Proyecto Cultural Noviembre. La tercera sección lee la masacre de Bagua (5 de junio de 2009, gobierno de Alan García) como el episodio que «develó» y «contradijo» el Consenso. Fuente sobre arte, colectivos y política en el Perú postdictatorial.</t>
         </is>
       </c>
     </row>
@@ -2462,27 +2462,27 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>mac-proyecto-2008.md</t>
+          <t>canepa_kg_2006_p132-167.pdf</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>2008 (exposición feb.–mar. 2008; con historia del sitio desde 1944)</t>
+          <t>1970-2006 (con referencias históricas desde el siglo XIX)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de exposición, mayo 2008 (Instituto de Arte Contemporáneo — MAC-Lima; OCR)</t>
+          <t>Capítulo de libro, 2006</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Miguel Zegarra (curadores); Instituto de Arte Contemporáneo (IAC); MAC-Lima; Giuliana Borea; George Gruenberg; Ricardo Ramón Jarne; José Carlos Martinat; Ishmael Randall Weeks; Elena Damiani; Sergio Abugattás; Raura Oblitas</t>
+          <t>Giuliana Borea Labarthe; Gisela Cánepa Koch (ed.); Sandra Gamarra (LiMAC); Instituto de Arte Contemporáneo (IAC); Fernando de Szyszlo; Gerardo Chávez; Mario Vargas Llosa; Ramiro Llona; Instituto Nacional de Cultura; ICOM; Museo de la Nación; Museo Nacional de la Cultura Peruana; Alfonso Castrillón</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Catálogo de la exposición «La Construcción del Lugar Común» (MAC-Lima, 5 de febrero–30 de marzo de 2008), editado por el Instituto de Arte Contemporáneo (IAC) y curado por Jorge Villacorta y Miguel Zegarra. Documenta una intervención colectiva de quince artistas peruanos emergentes —Sergio Abugattás, Miguel Andrade, Víctor Castro, Elena Damiani, Giuseppe De Bernardi, Nicole Franchy, Alejandro Jaime, Manuel Larrea, Martín Jiménez Paz, Christians Luna, José Carlos Martinat, José Miyashiro, Raura Oblitas, Ishmael Randall Weeks e Iliana Scheggia— que ocuparon el edificio del Museo de Arte Contemporáneo de Lima cuando aún estaba a medio construir. La muestra convirtió la arquitectura inconclusa y su entorno (el parque de la antigua «laguna» de Barranco) en soporte y tema: las obras tematizan la construcción/destrucción, el paisaje, la memoria del sitio y la disputa pública por el museo, cuyo proceso estuvo marcado por conflictos municipales y un intento de clausura respondido con el gesto «CLAUSURADO = INAUGURADO». El catálogo reúne textos institucionales (George Gruenberg, presidente del IAC), una pieza literaria de Ricardo Ramón Jarne («La maldición de la laguna»), un ensayo antropológico de Giuliana Borea sobre la construcción del lugar y el «lugar común» en la esfera pública (apoyado en Augé, Appadurai, Certeau y Casey), el texto curatorial de Villacorta y Zegarra, y los statements de cada artista. Como fuente histórica documenta un episodio clave de institucionalización del arte contemporáneo en Lima —la génesis del MAC— y las prácticas site-specific, de crítica institucional y de intervención en el espacio público de una generación emergente peruana de fines de la década de 2000.</t>
+          <t>Capítulo de Giuliana Borea Labarthe ('Museos y esfera pública: espacio, discursos y prácticas. Reflexiones en torno a la ciudad de Lima') incluido en el volumen editado por Gisela Cánepa Koch, 'Mirando la esfera pública desde la cultura en el Perú' (2006). Partiendo de las nociones de esfera pública (Habermas), cultura pública (Appadurai) y de la nueva museología surgida de las crisis de los años 70-80 (Mesa de Santiago 1972, redefinición del ICOM 1974, ecomuseos), Borea concibe el museo como contenedor y contenido, plataforma y discurso, esfera de poder y arena de disputa por la representación. Analiza tres casos limeños. Primero, el posicionamiento urbano de los museos: mediante una encuesta a transeúntes y taxistas muestra que solo el Museo de la Nación y el Museo de Arte de Lima son hitos reconocidos, mientras la mayoría oscila entre lugar simbólico y lugar anónimo por la falta de señalización y de alianzas municipales. Segundo, la polémica de 2006 por el proyecto del Museo de Arte Contemporáneo (MAC) del IAC, detonada por el intento de nombrarlo 'Fernando de Szyszlo': reconstruye siete momentos del debate mediático (comunicados de artistas, la columna 'Escaramuzas en Liliput' de Vargas Llosa), la falta de plan museológico y de diálogo con artistas donantes y con Barranco, y destaca la contrapropuesta crítica LiMAC de Sandra Gamarra frente al silencio del INC. Tercero, compara las puestas en escena sobre peruanidad y diversidad de cinco museos (Cultura Peruana, de la Nación, Etnográfico, Inmigración Japonesa, MNAAHP), evidenciando discursos lejanos, fragmentados y ahistóricos en los grandes museos nacionales frente a autorrepresentaciones más políticas en los pequeños. Cierra con Castrillón: Lima como escenario de emplazamiento, no de reflexión.</t>
         </is>
       </c>
     </row>
@@ -2494,59 +2494,59 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>sura.md</t>
+          <t>mac-proyecto-2008.md</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>mediados de la década de 1960 a 2013 (arte contemporáneo peruano)</t>
+          <t>2008 (exposición feb.–mar. 2008; con historia del sitio desde 1944)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de colección museística, 2013</t>
+          <t>Catálogo de exposición, mayo 2008 (Instituto de Arte Contemporáneo — MAC-Lima; OCR)</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner (ed.); Museo de Arte de Lima (MALI); Grupo SURA; Mirko Lauer; E.P.S. Huayco; Charo Noriega; Ramiro Llona; Flavia Gandolfo; Armando Andrade Tudela; Ricardo Wiesse; Eduardo Villanes; Miguel A. López; Rodrigo Quijano</t>
+          <t>Jorge Villacorta; Miguel Zegarra (curadores); Instituto de Arte Contemporáneo (IAC); MAC-Lima; Giuliana Borea; George Gruenberg; Ricardo Ramón Jarne; José Carlos Martinat; Ishmael Randall Weeks; Elena Damiani; Sergio Abugattás; Raura Oblitas</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Catálogo de la colección de arte contemporáneo del Museo de Arte de Lima (MALI), editado por la curadora Sharon Lerner y publicado con el patrocinio del grupo SURA. El volumen traza los derroteros del arte peruano reciente a partir del acervo del museo, sin pretender definir un 'arte peruano' esencial. La colección se articula bajo dos principios: identificar momentos de ruptura en la producción artística de fines del siglo XX y perfilar la producción reciente mediante ejes temáticos comunes. El ensayo central de Lerner establece como punto de partida mediados de la década de 1960 (grupos de vanguardia ligados al Pop y al no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, tras las reformas del Gobierno Militar, cuando —según la célebre frase de Mirko Lauer para la muestra Arte al paso del colectivo E.P.S. Huayco (1980)— 'en el Perú hoy solo lo popular es moderno'. Analiza la irrupción de la migración interna, el conflicto armado interno, el autogolpe de Fujimori (1992) y la virtual desaparición de la esfera pública, así como la Bienal Iberoamericana de Lima (1997) como puesta al día forzada y descontextualizada. El catálogo se organiza en núcleos temáticos: modernidad popular y transformación de Lima, f(r)icciones cosmopolitas, reconsideración del pasado y configuración del Perú, sistema artístico y utopías museales, desplazamientos, y signos de violencia, resistencia y memoria. Incluye obras de Charo Noriega, Ramiro Llona, Flavia Gandolfo, Armando Andrade Tudela, Herman Schwarz, Ricardo Wiesse y Eduardo Villanes, entre otros, y textos críticos complementarios. Su aporte es consolidar un relato historiográfico y crítico del arte contemporáneo peruano desde una institución museal.</t>
+          <t>Catálogo de la exposición «La Construcción del Lugar Común» (MAC-Lima, 5 de febrero–30 de marzo de 2008), editado por el Instituto de Arte Contemporáneo (IAC) y curado por Jorge Villacorta y Miguel Zegarra. Documenta una intervención colectiva de quince artistas peruanos emergentes —Sergio Abugattás, Miguel Andrade, Víctor Castro, Elena Damiani, Giuseppe De Bernardi, Nicole Franchy, Alejandro Jaime, Manuel Larrea, Martín Jiménez Paz, Christians Luna, José Carlos Martinat, José Miyashiro, Raura Oblitas, Ishmael Randall Weeks e Iliana Scheggia— que ocuparon el edificio del Museo de Arte Contemporáneo de Lima cuando aún estaba a medio construir. La muestra convirtió la arquitectura inconclusa y su entorno (el parque de la antigua «laguna» de Barranco) en soporte y tema: las obras tematizan la construcción/destrucción, el paisaje, la memoria del sitio y la disputa pública por el museo, cuyo proceso estuvo marcado por conflictos municipales y un intento de clausura respondido con el gesto «CLAUSURADO = INAUGURADO». El catálogo reúne textos institucionales (George Gruenberg, presidente del IAC), una pieza literaria de Ricardo Ramón Jarne («La maldición de la laguna»), un ensayo antropológico de Giuliana Borea sobre la construcción del lugar y el «lugar común» en la esfera pública (apoyado en Augé, Appadurai, Certeau y Casey), el texto curatorial de Villacorta y Zegarra, y los statements de cada artista. Como fuente histórica documenta un episodio clave de institucionalización del arte contemporáneo en Lima —la génesis del MAC— y las prácticas site-specific, de crítica institucional y de intervención en el espacio público de una generación emergente peruana de fines de la década de 2000.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Arte al Paso 2011</t>
+          <t>Cap 2 - Historia</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Arte al Paso - Texto Investigación.md</t>
+          <t>sura.md</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 1960 – 2010 (con foco en las décadas de 1970-2000 y el conflicto armado interno 1980-2000)</t>
+          <t>mediados de la década de 1960 a 2013 (arte contemporáneo peruano)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Ensayo curatorial de catálogo (exposición Arte al paso, Pinacoteca do Estado de São Paulo, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Catálogo de colección museística, 2013</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Pinacoteca de São Paulo; Emilio Hernández Saavedra; E.P.S. Huayco; Jesús Ruiz Durand; Sandra Gamarra; Alfredo Márquez / Taller NN; Fernando Bryce; José Carlos Martinat; Susana Torres</t>
+          <t>Sharon Lerner (ed.); Museo de Arte de Lima (MALI); Grupo SURA; Mirko Lauer; E.P.S. Huayco; Charo Noriega; Ramiro Llona; Flavia Gandolfo; Armando Andrade Tudela; Ricardo Wiesse; Eduardo Villanes; Miguel A. López; Rodrigo Quijano</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Ensayo curatorial extenso y bilingüe (castellano/portugués) de Tatiana Cuevas y Rodrigo Quijano para la muestra Arte al paso, que exhibió la coleccion contemporanea del MALI en la Estacion Pinacoteca de Sao Paulo. El texto toma como punto de partida la imagen El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra para diagnosticar los vacios institucionales y la distancia entre el discurso cultural cosmopolita y la practica real en el Peru de la segunda mitad del siglo XX. Su argumento articula el arte contemporaneo peruano con las transformaciones sociales derivadas de la masiva migracion rural a Lima, la explosion de la economia informal y la emergencia de una nueva cultura popular urbana. Rastrea las primeras vinculaciones locales con vanguardias internacionales (op, pop, conceptualismo, no-objetualismo), el pop achorado de Jesus Ruiz Durand y sus afiches de la Reforma Agraria velasquista, y las experiencias colectivas Contacta 79 y Arte al paso de E.P.S. Huayco (1980), que propusieron un arte callejero y antiinstitucional. Analiza la critica a la institucionalidad faltante (el museo ficticio LiMAC de Sandra Gamarra), el uso ironico del pasado prehispanico (Susana Torres, Rodriguez Larrain, Bryce, Cordova, Martinat), el tema del paisaje y el territorio, y la irrupcion tardia de la fotografia y la serigrafia como medios. Dedica una seccion central a la memoria de la violencia del conflicto armado interno (1980-2000) —Sendero Luminoso, MRTA, la Comision de la Verdad, 69.280 muertos— y su tratamiento por el Taller NN, Alfredo Marquez (Katatay), Carlos Dominguez, Ricardo Wiesse, Eduardo Villanes, Fernando Bryce y Milagros de la Torre.</t>
+          <t>Catálogo de la colección de arte contemporáneo del Museo de Arte de Lima (MALI), editado por la curadora Sharon Lerner y publicado con el patrocinio del grupo SURA. El volumen traza los derroteros del arte peruano reciente a partir del acervo del museo, sin pretender definir un 'arte peruano' esencial. La colección se articula bajo dos principios: identificar momentos de ruptura en la producción artística de fines del siglo XX y perfilar la producción reciente mediante ejes temáticos comunes. El ensayo central de Lerner establece como punto de partida mediados de la década de 1960 (grupos de vanguardia ligados al Pop y al no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, tras las reformas del Gobierno Militar, cuando —según la célebre frase de Mirko Lauer para la muestra Arte al paso del colectivo E.P.S. Huayco (1980)— 'en el Perú hoy solo lo popular es moderno'. Analiza la irrupción de la migración interna, el conflicto armado interno, el autogolpe de Fujimori (1992) y la virtual desaparición de la esfera pública, así como la Bienal Iberoamericana de Lima (1997) como puesta al día forzada y descontextualizada. El catálogo se organiza en núcleos temáticos: modernidad popular y transformación de Lima, f(r)icciones cosmopolitas, reconsideración del pasado y configuración del Perú, sistema artístico y utopías museales, desplazamientos, y signos de violencia, resistencia y memoria. Incluye obras de Charo Noriega, Ramiro Llona, Flavia Gandolfo, Armando Andrade Tudela, Herman Schwarz, Ricardo Wiesse y Eduardo Villanes, entre otros, y textos críticos complementarios. Su aporte es consolidar un relato historiográfico y crítico del arte contemporáneo peruano desde una institución museal.</t>
         </is>
       </c>
     </row>
@@ -2558,27 +2558,27 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Cronología Político Artistica - Arte al Paso 2011.md</t>
+          <t>Arte al Paso - Texto Investigación.md</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>1962 – 2010</t>
+          <t>Fines de los años 1960 – 2010 (con foco en las décadas de 1970-2000 y el conflicto armado interno 1980-2000)</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Cronología y bibliografía de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Ensayo curatorial de catálogo (exposición Arte al paso, Pinacoteca do Estado de São Paulo, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Museo de Arte de Lima (MALI); Grupo Arte Nuevo; Grupo Señal; E.P.S. Huayco; Taller NN; Colectivo Sociedad Civil; Gustavo Buntinx; Joaquín López Antay; Comisión de la Verdad y Reconciliación; Sendero Luminoso; Alberto Fujimori; Juan Velasco Alvarado</t>
+          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Pinacoteca de São Paulo; Emilio Hernández Saavedra; E.P.S. Huayco; Jesús Ruiz Durand; Sandra Gamarra; Alfredo Márquez / Taller NN; Fernando Bryce; José Carlos Martinat; Susana Torres</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Cronologia politico-artistica bilingue (castellano/portugues) incluida en el catalogo Arte al paso, que entrelaza en paralelo tres series de acontecimientos —eventos politicos, eventos artisticos y adquisiciones de la coleccion de arte contemporaneo del MALI— entre 1962 y 2010. El documento funciona como aparato historiografico que contextualiza la escena artistica peruana dentro de sus convulsiones politicas: rebeliones campesinas y golpes militares de los anos sesenta, el Gobierno Revolucionario de las Fuerzas Armadas de Velasco Alvarado (1968) y la Reforma Agraria, el estallido del conflicto armado interno con Sendero Luminoso y el MRTA (1980), las masacres de Barrios Altos y La Cantuta, el autogolpe y la dictadura de Alberto Fujimori (1990-2000), la Marcha de los Cuatro Suyos y el Informe de la Comision de la Verdad y Reconciliacion (2003). En el plano artistico registra la formacion de los grupos Senal y Arte Nuevo, las Bienales de Lima e Iberoamericanas, los festivales Contacta e Inkarri, el Taller E.P.S. Huayco y el Taller NN, la premiacion de Joaquin Lopez Antay, y acciones de arte critico como Cantuta de Ricardo Wiesse, Gloria evaporada de Eduardo Villanes y Lava la bandera del Colectivo Sociedad Civil. Una tercera linea traza la institucionalizacion del MALI: el ciclo curatorial Miradas de fin de siglo, la creacion del Comite de Adquisiciones (2007) y la reapertura del museo (2010). Se acompana de una extensa bibliografia especializada (Buntinx, Castrillon, Lauer, Majluf, Lopez, Tarazona, Quijano, Villacorta), fuente clave para la historiografia del arte peruano contemporaneo.</t>
+          <t>Ensayo curatorial extenso y bilingüe (castellano/portugués) de Tatiana Cuevas y Rodrigo Quijano para la muestra Arte al paso, que exhibió la coleccion contemporanea del MALI en la Estacion Pinacoteca de Sao Paulo. El texto toma como punto de partida la imagen El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra para diagnosticar los vacios institucionales y la distancia entre el discurso cultural cosmopolita y la practica real en el Peru de la segunda mitad del siglo XX. Su argumento articula el arte contemporaneo peruano con las transformaciones sociales derivadas de la masiva migracion rural a Lima, la explosion de la economia informal y la emergencia de una nueva cultura popular urbana. Rastrea las primeras vinculaciones locales con vanguardias internacionales (op, pop, conceptualismo, no-objetualismo), el pop achorado de Jesus Ruiz Durand y sus afiches de la Reforma Agraria velasquista, y las experiencias colectivas Contacta 79 y Arte al paso de E.P.S. Huayco (1980), que propusieron un arte callejero y antiinstitucional. Analiza la critica a la institucionalidad faltante (el museo ficticio LiMAC de Sandra Gamarra), el uso ironico del pasado prehispanico (Susana Torres, Rodriguez Larrain, Bryce, Cordova, Martinat), el tema del paisaje y el territorio, y la irrupcion tardia de la fotografia y la serigrafia como medios. Dedica una seccion central a la memoria de la violencia del conflicto armado interno (1980-2000) —Sendero Luminoso, MRTA, la Comision de la Verdad, 69.280 muertos— y su tratamiento por el Taller NN, Alfredo Marquez (Katatay), Carlos Dominguez, Ricardo Wiesse, Eduardo Villanes, Fernando Bryce y Milagros de la Torre.</t>
         </is>
       </c>
     </row>
@@ -2590,59 +2590,59 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Texto de la exposición Arte al Paso 2011.md</t>
+          <t>Cronología Político Artistica - Arte al Paso 2011.md</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 1960 – 2010 (unos 40 años; foco en las décadas de 1970-1980)</t>
+          <t>1962 – 2010</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Texto de sala / presentación de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Cronología y bibliografía de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Emilio Hernández Saavedra; E.P.S. Huayco; Grupo Paréntesis; Sandra Gamarra; Susana Torres; Emilio Rodríguez Larraín; Juan Javier Salazar; William Cordova; José Carlos Martinat</t>
+          <t>Museo de Arte de Lima (MALI); Grupo Arte Nuevo; Grupo Señal; E.P.S. Huayco; Taller NN; Colectivo Sociedad Civil; Gustavo Buntinx; Joaquín López Antay; Comisión de la Verdad y Reconciliación; Sendero Luminoso; Alberto Fujimori; Juan Velasco Alvarado</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Texto de sala o presentacion general de la exposicion Arte al paso (coleccion contemporanea del MALI en la Pinacoteca de Sao Paulo), firmado por los curadores Tatiana Cuevas y Rodrigo Quijano, en edicion bilingue castellano/portugues. Es una version sintetica del argumento curatorial: parte nuevamente de El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra como metafora de la ausencia institucional y punto de arranque para examinar la escena artistica peruana desde fines de los anos sesenta. Explica el titulo de la muestra a partir de la accion Arte al paso de E.P.S. Huayco (1980) —que, aludiendo a los puestos informales de comida al paso surgidos con la migracion y la economia informal, propuso un arte para consumirse en la calle, opuesto al museo y la galeria ausentes, un arte para pensar y no para sentir que dejaba atras el modernismo conservador de mediados de siglo. Sintetiza cuarenta anos de produccion cultural marcados por oposiciones ocultas y explicitas, los primeros acercamientos al conceptualismo y a las vanguardias internacionales, y la creciente proyeccion internacional de artistas peruanos. Una segunda seccion, Critica ante una institucionalidad faltante y al poder redentor del pasado, reune a Hernandez Saavedra, los grupos Parentesis y E.P.S. Huayco y el museo ficticio de Sandra Gamarra como estrategias de critica institucional apropiadas del conceptualismo y del imaginario popular urbano, con recurrente uso del humor. Aborda ademas la critica a la explotacion comercial y politica de lo prehispanico (Museo Neo-Inka de Susana Torres) y el vinculo entre la retorica del glorioso pasado incaico y los fracasos politicos y economicos del presente en obras de Rodriguez Larrain, Salazar, Cordova y Martinat.</t>
+          <t>Cronologia politico-artistica bilingue (castellano/portugues) incluida en el catalogo Arte al paso, que entrelaza en paralelo tres series de acontecimientos —eventos politicos, eventos artisticos y adquisiciones de la coleccion de arte contemporaneo del MALI— entre 1962 y 2010. El documento funciona como aparato historiografico que contextualiza la escena artistica peruana dentro de sus convulsiones politicas: rebeliones campesinas y golpes militares de los anos sesenta, el Gobierno Revolucionario de las Fuerzas Armadas de Velasco Alvarado (1968) y la Reforma Agraria, el estallido del conflicto armado interno con Sendero Luminoso y el MRTA (1980), las masacres de Barrios Altos y La Cantuta, el autogolpe y la dictadura de Alberto Fujimori (1990-2000), la Marcha de los Cuatro Suyos y el Informe de la Comision de la Verdad y Reconciliacion (2003). En el plano artistico registra la formacion de los grupos Senal y Arte Nuevo, las Bienales de Lima e Iberoamericanas, los festivales Contacta e Inkarri, el Taller E.P.S. Huayco y el Taller NN, la premiacion de Joaquin Lopez Antay, y acciones de arte critico como Cantuta de Ricardo Wiesse, Gloria evaporada de Eduardo Villanes y Lava la bandera del Colectivo Sociedad Civil. Una tercera linea traza la institucionalizacion del MALI: el ciclo curatorial Miradas de fin de siglo, la creacion del Comite de Adquisiciones (2007) y la reapertura del museo (2010). Se acompana de una extensa bibliografia especializada (Buntinx, Castrillon, Lauer, Majluf, Lopez, Tarazona, Quijano, Villacorta), fuente clave para la historiografia del arte peruano contemporaneo.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Hueso Húmero 18</t>
+          <t>Cap 2 - Historia/Arte al Paso 2011</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - Arte joven peruano, ¿el sueño del mercado propio? Una conversación con Claudia Polar (1983) [Hueso Húmero 18, pp. 94-107].md</t>
+          <t>Texto de la exposición Arte al Paso 2011.md</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>1974-1983</t>
+          <t>Fines de los años 1960 – 2010 (unos 40 años; foco en las décadas de 1970-1980)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Entrevista en revista (Hueso Húmero 18), 1983</t>
+          <t>Texto de sala / presentación de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Claudia Polar; Galería Forum; Elida Román; Hernán Pazos; Esther Vainstein; Ramiro Llona; Bill Caro; Herbert Rodríguez; EAPUC; ENBA; Hueso Húmero</t>
+          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Emilio Hernández Saavedra; E.P.S. Huayco; Grupo Paréntesis; Sandra Gamarra; Susana Torres; Emilio Rodríguez Larraín; Juan Javier Salazar; William Cordova; José Carlos Martinat</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Entrevista conducida por Gustavo Buntinx a Claudia Polar, directora de la Galería Forum, concebida como contraparte de un reportaje previo a Elida Román para perfilar el mercado del arte joven peruano. Polar reconstruye la fundación de Forum en diciembre de 1974 como un espacio destinado a priorizar a los artistas jóvenes y a gestar deliberadamente un mercado y coleccionistas nuevos, mediante becas, premios, subvenciones informales (incluso marcos y pasajes) y una política de "riesgo total" sostenida por la venta de stock. El diálogo traza una periodización económica de la plástica: expansión del mercado hacia 1974-1976, auge en 1978 atribuido a la restricción de importaciones bajo Morales Bermúdez, y recesión desde 1980 con la apertura de Belaúnde, siendo 1983 el año más difícil. Se discute la naturaleza del público comprador (gente joven, profesionales, empresarios, bancos como el de Crédito y el Continental) y la débil proporción de compradores habituales, apenas un 5% con relación económica. Buntinx presiona sobre las mediaciones de clase: el vínculo de Forum con la Universidad Católica frente a la ENBA, la identidad ideológica compartida, y el papel de las relaciones públicas como "gatillo" de casi toda venta en un mercado de "sala de estar". Polar aborda la diferencia entre lo culto y lo popular, el fracaso de asociar galerías, las cotizaciones (Llona, Caro, Pazos, Vainstein) y la explotación del artista acostumbrado a vender barato. El aporte documental es excepcional: registra desde dentro la lógica comercial, simbólica y provinciana del circuito limeño de principios de los ochenta.</t>
+          <t>Texto de sala o presentacion general de la exposicion Arte al paso (coleccion contemporanea del MALI en la Pinacoteca de Sao Paulo), firmado por los curadores Tatiana Cuevas y Rodrigo Quijano, en edicion bilingue castellano/portugues. Es una version sintetica del argumento curatorial: parte nuevamente de El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra como metafora de la ausencia institucional y punto de arranque para examinar la escena artistica peruana desde fines de los anos sesenta. Explica el titulo de la muestra a partir de la accion Arte al paso de E.P.S. Huayco (1980) —que, aludiendo a los puestos informales de comida al paso surgidos con la migracion y la economia informal, propuso un arte para consumirse en la calle, opuesto al museo y la galeria ausentes, un arte para pensar y no para sentir que dejaba atras el modernismo conservador de mediados de siglo. Sintetiza cuarenta anos de produccion cultural marcados por oposiciones ocultas y explicitas, los primeros acercamientos al conceptualismo y a las vanguardias internacionales, y la creciente proyeccion internacional de artistas peruanos. Una segunda seccion, Critica ante una institucionalidad faltante y al poder redentor del pasado, reune a Hernandez Saavedra, los grupos Parentesis y E.P.S. Huayco y el museo ficticio de Sandra Gamarra como estrategias de critica institucional apropiadas del conceptualismo y del imaginario popular urbano, con recurrente uso del humor. Aborda ademas la critica a la explotacion comercial y politica de lo prehispanico (Museo Neo-Inka de Susana Torres) y el vinculo entre la retorica del glorioso pasado incaico y los fracasos politicos y economicos del presente en obras de Rodriguez Larrain, Salazar, Cordova y Martinat.</t>
         </is>
       </c>
     </row>
@@ -2654,27 +2654,27 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - ¿Entre lo popular y lo moderno? Alternativas pretendidas o reales en la joven plástica peruana (1983) [Hueso Húmero 18, pp. 61-85].md</t>
+          <t>Buntinx - Arte joven peruano, ¿el sueño del mercado propio? Una conversación con Claudia Polar (1983) [Hueso Húmero 18, pp. 94-107].md</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>1960-1984 (con énfasis en los años 70)</t>
+          <t>1974-1983</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
+          <t>Entrevista en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Mirko Lauer; Juan Acha; Francisco Mariotti; Huayco E.P.S.; Herbert Rodríguez; Juan Javier Salazar; Jesús Ruiz Durand; Fernando de Szyszlo; IAC; Galería Forum; SINAMOS; Néstor García Canclini</t>
+          <t>Gustavo Buntinx; Claudia Polar; Galería Forum; Elida Román; Hernán Pazos; Esther Vainstein; Ramiro Llona; Bill Caro; Herbert Rodríguez; EAPUC; ENBA; Hueso Húmero</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Ensayo teórico-histórico que propone hipótesis de trabajo sobre lo que fue o pretendió ser alternativo en el arte erudito peruano desde la transición al primer belaundismo hasta los años ochenta, articulando dos tópicos móviles: lo popular y lo moderno. Retomando y ampliando a Mirko Lauer, Buntinx sostiene que las opciones estéticas no reflejan mecánicamente la época sino que reproducen una inserción particular en el mercado, entendido como trama compleja de producción, intermediación y consumo (soporte social). Recorre así una secuencia de "soportes": el corporativo (IAC financiado por IPC, IBM, Tecnoquímica) que sostuvo la Teoría de las Raíces Nacionales de Szyszlo; el soporte "de punta" del frenesí pop cosmopolita (Acha, Arte Nuevo, Fundación para las Artes, 1966-1969); el soporte estatal velasquista con sus cuatro alternativas (comunicación masiva de Ruiz Durand con su "pop achorado", festivales de arte-total como Contacta e Inkarri, revaloración de lo artesanal, López Antay); y la frustrada búsqueda de un soporte alternativo hacia 1977-1980. El caso central es Huayco E.P.S., cuyo proyecto Sarita Colonia codifica una modernidad sincrética limeña sostenida por una pequeña burguesía ilustrada radicalizada, y cuya dispersión coincide con el agotamiento de la izquierda y el repliegue hacia el mercado galerístico (Forum). El marco conceptual bebe de García Canclini. La tesis es incisiva: el tránsito de la imagen telúrica a la industrial, agraria y migrante revela apropiaciones sucesivas de una idea variable de lo popular, siempre con una radicalidad deficiente y una relación desigual con la cultura interpretada.</t>
+          <t>Entrevista conducida por Gustavo Buntinx a Claudia Polar, directora de la Galería Forum, concebida como contraparte de un reportaje previo a Elida Román para perfilar el mercado del arte joven peruano. Polar reconstruye la fundación de Forum en diciembre de 1974 como un espacio destinado a priorizar a los artistas jóvenes y a gestar deliberadamente un mercado y coleccionistas nuevos, mediante becas, premios, subvenciones informales (incluso marcos y pasajes) y una política de "riesgo total" sostenida por la venta de stock. El diálogo traza una periodización económica de la plástica: expansión del mercado hacia 1974-1976, auge en 1978 atribuido a la restricción de importaciones bajo Morales Bermúdez, y recesión desde 1980 con la apertura de Belaúnde, siendo 1983 el año más difícil. Se discute la naturaleza del público comprador (gente joven, profesionales, empresarios, bancos como el de Crédito y el Continental) y la débil proporción de compradores habituales, apenas un 5% con relación económica. Buntinx presiona sobre las mediaciones de clase: el vínculo de Forum con la Universidad Católica frente a la ENBA, la identidad ideológica compartida, y el papel de las relaciones públicas como "gatillo" de casi toda venta en un mercado de "sala de estar". Polar aborda la diferencia entre lo culto y lo popular, el fracaso de asociar galerías, las cotizaciones (Llona, Caro, Pazos, Vainstein) y la explotación del artista acostumbrado a vender barato. El aporte documental es excepcional: registra desde dentro la lógica comercial, simbólica y provinciana del circuito limeño de principios de los ochenta.</t>
         </is>
       </c>
     </row>
@@ -2686,27 +2686,27 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Freire - Herbert Rodríguez, azote y azúcar con el sistema (1983) [Hueso Húmero 18, pdf pp. 178-185].md</t>
+          <t>Buntinx - ¿Entre lo popular y lo moderno? Alternativas pretendidas o reales en la joven plástica peruana (1983) [Hueso Húmero 18, pp. 61-85].md</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>1979-1983 (con antecedentes desde 1968)</t>
+          <t>1960-1984 (con énfasis en los años 70)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Reseña crítica en revista (Hueso Húmero 18), 1983</t>
+          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Luis Freire S.; Herbert Rodríguez; Francisco Mariotti; Huayco E.P.S.; Juan Acha; Fernando Bedoya; Juan Javier Salazar; Bienal de Sao Paulo; Galería La Rama Dorada; Galería Forum; EAPUC; ENBAP</t>
+          <t>Gustavo Buntinx; Mirko Lauer; Juan Acha; Francisco Mariotti; Huayco E.P.S.; Herbert Rodríguez; Juan Javier Salazar; Jesús Ruiz Durand; Fernando de Szyszlo; IAC; Galería Forum; SINAMOS; Néstor García Canclini</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Perfil crítico dedicado a Herbert Rodríguez Huachín en la sección "Individuales" de Hueso Húmero, escrito por Luis Freire, que examina el salto vertiginoso del artista desde la suspensión disciplinaria en la Escuela de Artes Plásticas de la Católica (1981) hasta su presencia en la XVII Bienal de Sao Paulo (1983). Freire sitúa a Rodríguez como imposible de explicar sin el proceso ideológico del populismo velasquista y sin la figura mediadora de Francisco Mariotti, artista suizo-peruano formado en la Documenta de Kassel y la vanguardia europea, catalizador de Contacta y de la EPS Huayco. El texto reconstruye la genealogía Mariotti-Huayco-Rodríguez: los ensamblajes y "reciclajes" del suizo-peruano derivan en los "altares" de Rodríguez, hibridación entre constructivismo geométrico, expresionismo "pobre" y antiestético, y estructuras rituales de la religiosidad popular andina. Argumenta que Rodríguez encarna las contradicciones de una pequeña burguesía radical: dinamita el circuito con una mano y lo enluce con la otra, camuflando "bellamente" materiales pobres y reciclados en obras a la vez contestatarias y comerciables, con lo que ironiza sobre el culto al oficio del arte establecido. Analiza su heterogeneidad de lenguajes (expresionismo abstracto, figuración dura, conceptualismo informal, collage, fotocopia, ensamblaje) como búsqueda pero también como crisis, y sus "altares al Yo" exhibidos en Forum (1983) y la Bienal. Freire lo define como un artista religioso-existencial populista sin referentes sólidos, en formación, tensionado entre enriquecer el jardín burgués que quiere pisotear o saltar a opciones más radicales de ruptura.</t>
+          <t>Ensayo teórico-histórico que propone hipótesis de trabajo sobre lo que fue o pretendió ser alternativo en el arte erudito peruano desde la transición al primer belaundismo hasta los años ochenta, articulando dos tópicos móviles: lo popular y lo moderno. Retomando y ampliando a Mirko Lauer, Buntinx sostiene que las opciones estéticas no reflejan mecánicamente la época sino que reproducen una inserción particular en el mercado, entendido como trama compleja de producción, intermediación y consumo (soporte social). Recorre así una secuencia de "soportes": el corporativo (IAC financiado por IPC, IBM, Tecnoquímica) que sostuvo la Teoría de las Raíces Nacionales de Szyszlo; el soporte "de punta" del frenesí pop cosmopolita (Acha, Arte Nuevo, Fundación para las Artes, 1966-1969); el soporte estatal velasquista con sus cuatro alternativas (comunicación masiva de Ruiz Durand con su "pop achorado", festivales de arte-total como Contacta e Inkarri, revaloración de lo artesanal, López Antay); y la frustrada búsqueda de un soporte alternativo hacia 1977-1980. El caso central es Huayco E.P.S., cuyo proyecto Sarita Colonia codifica una modernidad sincrética limeña sostenida por una pequeña burguesía ilustrada radicalizada, y cuya dispersión coincide con el agotamiento de la izquierda y el repliegue hacia el mercado galerístico (Forum). El marco conceptual bebe de García Canclini. La tesis es incisiva: el tránsito de la imagen telúrica a la industrial, agraria y migrante revela apropiaciones sucesivas de una idea variable de lo popular, siempre con una radicalidad deficiente y una relación desigual con la cultura interpretada.</t>
         </is>
       </c>
     </row>
@@ -2718,59 +2718,59 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Lama - Los años de la resaca (1983) [Hueso Húmero 18, pdf pp. 136-156].md</t>
+          <t>Freire - Herbert Rodríguez, azote y azúcar con el sistema (1983) [Hueso Húmero 18, pdf pp. 178-185].md</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>1974-1983 (con antecedentes en los años 60-70)</t>
+          <t>1979-1983 (con antecedentes desde 1968)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
+          <t>Reseña crítica en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Luis Lama; Hernán Pazos; Francisco Mariotti; Contacta; grupo Huayco; Juan Javier Salazar; Herbert Rodríguez; Alfonso Castrillón; Escuela Nacional de Bellas Artes; Galería Forum; Galería 9; Ugarte Eléspuru</t>
+          <t>Luis Freire S.; Herbert Rodríguez; Francisco Mariotti; Huayco E.P.S.; Juan Acha; Fernando Bedoya; Juan Javier Salazar; Bienal de Sao Paulo; Galería La Rama Dorada; Galería Forum; EAPUC; ENBAP</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Ensayo de Luis Lama que narra el paso de la "ebullición ideológica" de los años setenta a la "resaca" del segundo belaundismo, articulando historia social del arte y crítica biográfica. La primera parte reconstruye los antecedentes: el terremoto de 1974 y el reflujo de artistas jóvenes hacia Barranco, la gravitación de Francisco Mariotti que transforma el arte de sistemas en movimiento grupal con Contacta e Inkari bajo auspicio de SINAMOS, las tomas y la crisis de la Escuela Nacional de Bellas Artes (1974-1976), y la gestación del taller de Pedro de Osma que devendría núcleo del grupo Huayco (Juan Javier Salazar, Herbert Rodríguez, Charo Noriega, Fernando Bedoya, Lucy Angulo). Lama describe la consolidación paradójica del mercado del arte al amparo de la prohibición de importaciones, con galerías que proliferan mientras la formación académica alcanza sus niveles más bajos. Diagnostica el fin de los happenings sesenteros y el retorno de un expresionismo "de crisis" impulsado desde los predios católicos (Williams, Polanco, Velarde, Hamann), junto a indagaciones matéricas de Wiesse y el conceptualismo de Vainstein. La segunda mitad es un retrato extenso de Hernán Pazos: su formación entre Derecho, la Católica y París, su tránsito del conceptualismo (los cielos y nubes de Galería 9) a la abstracción cromática, las series de los Quipus y los dibujos infantiles, su gestión en Rama Dorada y su individualismo parricida. Lama lo consagra como el artista más destacado de la década, emblema lúcido de las "amargas frustraciones" nacionales bajo el liberalismo económico belaundista.</t>
+          <t>Perfil crítico dedicado a Herbert Rodríguez Huachín en la sección "Individuales" de Hueso Húmero, escrito por Luis Freire, que examina el salto vertiginoso del artista desde la suspensión disciplinaria en la Escuela de Artes Plásticas de la Católica (1981) hasta su presencia en la XVII Bienal de Sao Paulo (1983). Freire sitúa a Rodríguez como imposible de explicar sin el proceso ideológico del populismo velasquista y sin la figura mediadora de Francisco Mariotti, artista suizo-peruano formado en la Documenta de Kassel y la vanguardia europea, catalizador de Contacta y de la EPS Huayco. El texto reconstruye la genealogía Mariotti-Huayco-Rodríguez: los ensamblajes y "reciclajes" del suizo-peruano derivan en los "altares" de Rodríguez, hibridación entre constructivismo geométrico, expresionismo "pobre" y antiestético, y estructuras rituales de la religiosidad popular andina. Argumenta que Rodríguez encarna las contradicciones de una pequeña burguesía radical: dinamita el circuito con una mano y lo enluce con la otra, camuflando "bellamente" materiales pobres y reciclados en obras a la vez contestatarias y comerciables, con lo que ironiza sobre el culto al oficio del arte establecido. Analiza su heterogeneidad de lenguajes (expresionismo abstracto, figuración dura, conceptualismo informal, collage, fotocopia, ensamblaje) como búsqueda pero también como crisis, y sus "altares al Yo" exhibidos en Forum (1983) y la Bienal. Freire lo define como un artista religioso-existencial populista sin referentes sólidos, en formación, tensionado entre enriquecer el jardín burgués que quiere pisotear o saltar a opciones más radicales de ruptura.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/MALI</t>
+          <t>Cap 2 - Historia/Hueso Húmero 18</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - El poder y la ilusión. Pérdida y restauración del aura en la «República de Weimar peruana» 1980-1992 [MALI].md</t>
+          <t>Lama - Los años de la resaca (1983) [Hueso Húmero 18, pdf pp. 136-156].md</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>1980-1992</t>
+          <t>1974-1983 (con antecedentes en los años 60-70)</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico (versión MALI), 2013 [escrito 1991-1994]</t>
+          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; E.P.S. Huayco; Taller NN; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; Walter Benjamin; Jesús Ruiz Durand; Andy Warhol; Mirko Lauer; Museo de Arte de Lima (MALI); III Bienal de La Habana</t>
+          <t>Luis Lama; Hernán Pazos; Francisco Mariotti; Contacta; grupo Huayco; Juan Javier Salazar; Herbert Rodríguez; Alfonso Castrillón; Escuela Nacional de Bellas Artes; Galería Forum; Galería 9; Ugarte Eléspuru</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Ensayo seminal de Gustavo Buntinx —redactado entre 1991 y 1994, difundido en inglés en «Beyond the Fantastic» (1995) y publicado por primera vez en Perú en esta versión del MALI (2013)— que interpreta el radical cambio de época del arte peruano entre 1980 y 1992, periodo que denomina metafóricamente «República de Weimar peruana». Su marco conceptual adapta la dialéctica benjaminiana entre proximidad y distancia (el aura, su pérdida por la reproductibilidad técnica y su posible restauración) y las categorías de alegoría, montaje y apropiación de Owens, Foster y Craig Owens a una periferia extrema. El argumento se sostiene sobre el análisis iconográfico minucioso de dos o tres obras que abren y cierran la década. La primera, «Arte al paso» y sobre todo «Sarita Colonia» (1980) del taller E.P.S. Huayco: una enorme estampa de la santa migrante pintada sobre diez mil latas de leche y emplazada en la Panamericana Sur, que Buntinx lee como huaca (post)moderna y exvoto donde lo pequeñoburgués radical se articula figuradamente a lo popular en emergencia (el «pop achorado» y «chicha»). La segunda, «Maorilyn» / «Viva el maoísmo» (1989) del Taller NN: una serigrafía que travistió el rostro de Mao con labios warholianos, alegoría ambivalente de la violencia senderista y la estetización de la política. Su tesis vincula la desintegración social —hiperinflación, guerra civil, movida subte punk— con el desarrollo de una condición alegórica y neo-aurática; su aporte es un modelo teórico para leer el colectivismo y la (post)modernidad popular peruana.</t>
+          <t>Ensayo de Luis Lama que narra el paso de la "ebullición ideológica" de los años setenta a la "resaca" del segundo belaundismo, articulando historia social del arte y crítica biográfica. La primera parte reconstruye los antecedentes: el terremoto de 1974 y el reflujo de artistas jóvenes hacia Barranco, la gravitación de Francisco Mariotti que transforma el arte de sistemas en movimiento grupal con Contacta e Inkari bajo auspicio de SINAMOS, las tomas y la crisis de la Escuela Nacional de Bellas Artes (1974-1976), y la gestación del taller de Pedro de Osma que devendría núcleo del grupo Huayco (Juan Javier Salazar, Herbert Rodríguez, Charo Noriega, Fernando Bedoya, Lucy Angulo). Lama describe la consolidación paradójica del mercado del arte al amparo de la prohibición de importaciones, con galerías que proliferan mientras la formación académica alcanza sus niveles más bajos. Diagnostica el fin de los happenings sesenteros y el retorno de un expresionismo "de crisis" impulsado desde los predios católicos (Williams, Polanco, Velarde, Hamann), junto a indagaciones matéricas de Wiesse y el conceptualismo de Vainstein. La segunda mitad es un retrato extenso de Hernán Pazos: su formación entre Derecho, la Católica y París, su tránsito del conceptualismo (los cielos y nubes de Galería 9) a la abstracción cromática, las series de los Quipus y los dibujos infantiles, su gestión en Rama Dorada y su individualismo parricida. Lama lo consagra como el artista más destacado de la década, emblema lúcido de las "amargas frustraciones" nacionales bajo el liberalismo económico belaundista.</t>
         </is>
       </c>
     </row>
@@ -2782,27 +2782,27 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Lerner - Formando la colección de arte contemporáneo del MALI (2013).txt</t>
+          <t>Buntinx - El poder y la ilusión. Pérdida y restauración del aura en la «República de Weimar peruana» 1980-1992 [MALI].md</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>mediados de los años 60 - 2013 (con foco en 1980-2000)</t>
+          <t>1980-1992</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo de colección, 2013</t>
+          <t>Ensayo académico (versión MALI), 2013 [escrito 1991-1994]</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Museo de Arte de Lima (MALI); Tatiana Cuevas; Miguel A. López; Gustavo Buntinx; Rodrigo Quijano; Jorge Villacorta; Natalia Majluf; E.P.S. Huayco; Teresa Burga; Milagros de la Torre; Flavia Gandolfo</t>
+          <t>Gustavo Buntinx; E.P.S. Huayco; Taller NN; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; Walter Benjamin; Jesús Ruiz Durand; Andy Warhol; Mirko Lauer; Museo de Arte de Lima (MALI); III Bienal de La Habana</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>Ensayo introductorio de Sharon Lerner al libro que presenta la colección de arte contemporáneo del Museo de Arte de Lima (MALI), articulado como una lectura —entre muchas posibles— de la historia del arte reciente peruano a partir del acervo. Su tesis metodológica es que en el Perú el tránsito a la contemporaneidad no ocurre como un quiebre radical, sino como una serie de pequeños cambios discontinuos, por lo que la colección se organiza en dos principios: identificar momentos de ruptura de fines del siglo XX y perfilar la producción reciente por ejes temáticos. El recorrido histórico parte de mediados de los sesenta (vanguardias pop, experimentalismo, no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, cuando la migración y la sentencia de Mirko Lauer —«En el Perú, hoy, solo lo popular es moderno»— enmarcan la obra de E.P.S. Huayco. Recorre luego la hegemonía de la abstracción en los ochenta, el arte de derechos humanos de Ricardo Wiesse y Eduardo Villanes bajo el fujimorato, la irrupción de la Bienal Iberoamericana de Lima (1997) y el «bienalismo», y la generación de los 2000 (Flavia Gandolfo, Gilda Mantilla, Armando Andrade Tudela) vinculada al espacio La Culpable. El texto presenta además los ensayos de Miguel López, Gustavo Buntinx y Rodrigo Quijano incluidos en el volumen y la conversación de seis críticos (2011). Su aporte es explicitar la política de adquisiciones del MALI y su ambición de llenar el vacío institucional y discursivo, construyendo un marco regional e internacional para el arte peruano.</t>
+          <t>Ensayo seminal de Gustavo Buntinx —redactado entre 1991 y 1994, difundido en inglés en «Beyond the Fantastic» (1995) y publicado por primera vez en Perú en esta versión del MALI (2013)— que interpreta el radical cambio de época del arte peruano entre 1980 y 1992, periodo que denomina metafóricamente «República de Weimar peruana». Su marco conceptual adapta la dialéctica benjaminiana entre proximidad y distancia (el aura, su pérdida por la reproductibilidad técnica y su posible restauración) y las categorías de alegoría, montaje y apropiación de Owens, Foster y Craig Owens a una periferia extrema. El argumento se sostiene sobre el análisis iconográfico minucioso de dos o tres obras que abren y cierran la década. La primera, «Arte al paso» y sobre todo «Sarita Colonia» (1980) del taller E.P.S. Huayco: una enorme estampa de la santa migrante pintada sobre diez mil latas de leche y emplazada en la Panamericana Sur, que Buntinx lee como huaca (post)moderna y exvoto donde lo pequeñoburgués radical se articula figuradamente a lo popular en emergencia (el «pop achorado» y «chicha»). La segunda, «Maorilyn» / «Viva el maoísmo» (1989) del Taller NN: una serigrafía que travistió el rostro de Mao con labios warholianos, alegoría ambivalente de la violencia senderista y la estetización de la política. Su tesis vincula la desintegración social —hiperinflación, guerra civil, movida subte punk— con el desarrollo de una condición alegórica y neo-aurática; su aporte es un modelo teórico para leer el colectivismo y la (post)modernidad popular peruana.</t>
         </is>
       </c>
     </row>
@@ -2814,27 +2814,27 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - F(r)icciones cosmopolitas. Redefiniciones estéticas y políticas de una idea de vanguardia en los años 60s.txt</t>
+          <t>Lerner - Formando la colección de arte contemporáneo del MALI (2013).txt</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>1960-1976 (con antecedentes desde 1942-1947)</t>
+          <t>mediados de los años 60 - 2013 (con foco en 1980-2000)</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico / capítulo de catálogo (MALI), s/f</t>
+          <t>Ensayo de catálogo de colección, 2013</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Emilio Tarazona; Juan Acha; Fernando de Szyszlo; Jorge Romero Brest; Teresa Burga; Rafael Hastings; Grupo Arte Nuevo; Jesús Ruiz Durand; José Gómez Sicre; Marta Traba; Instituto de Arte Contemporáneo (IAC); MoMA / Instituto Di Tella</t>
+          <t>Sharon Lerner; Museo de Arte de Lima (MALI); Tatiana Cuevas; Miguel A. López; Gustavo Buntinx; Rodrigo Quijano; Jorge Villacorta; Natalia Majluf; E.P.S. Huayco; Teresa Burga; Milagros de la Torre; Flavia Gandolfo</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>López reconstruye las mutaciones semánticas y políticas de la noción de vanguardia en el Perú entre los años sesenta y setenta, argumentando que la euforia cosmopolita del periodo fue el espejismo de una modernidad desarrollista tan prometedora como inacabada en un país socialmente fracturado. El objeto de estudio son las plataformas institucionales privadas (IAC, galerías, bienales americanas, concursos empresariales) que, apuntaladas por el panamericanismo de la Guerra Fría, la Alianza para el Progreso y la política curatorial estadounidense de José Gómez Sicre, promovieron primero la abstracción y luego el arte óptico, el pop y las ambientaciones. El texto traza el paso del declive de la abstracción szyszliana hacia el experimentalismo detonado por las conferencias de Jorge Romero Brest (1965) y la irrupción beligerante del grupo Arte Nuevo (1966-1968) contra el Festival Americano de Pintura. El marco conceptual articula la relación entre desarrollismo y vanguardia, y su posterior tensión con el subdesarrollo, siguiendo la radicalización de Juan Acha, quien tras 1968 y el golpe de Velasco redefine la vanguardia como 'guerrilla cultural' y horizonte revolucionario, hasta su exilio a México en 1971. López destaca las reconversiones de Teresa Burga y Rafael Hastings, el 'pop achorado' de Ruiz Durand al servicio de la Reforma Agraria, los festivales Contacta y las Carreras de chasquis. Su aporte es mostrar cómo la condición local, provinciana y periférica de las prácticas de los setenta y ochenta (Paréntesis, E.P.S. Huayco, Grupo Chaclacayo) actualizó de modo radical las pretensiones críticas sesenteras, canibalizando los conceptos metropolitanos de arte conceptual.</t>
+          <t>Ensayo introductorio de Sharon Lerner al libro que presenta la colección de arte contemporáneo del Museo de Arte de Lima (MALI), articulado como una lectura —entre muchas posibles— de la historia del arte reciente peruano a partir del acervo. Su tesis metodológica es que en el Perú el tránsito a la contemporaneidad no ocurre como un quiebre radical, sino como una serie de pequeños cambios discontinuos, por lo que la colección se organiza en dos principios: identificar momentos de ruptura de fines del siglo XX y perfilar la producción reciente por ejes temáticos. El recorrido histórico parte de mediados de los sesenta (vanguardias pop, experimentalismo, no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, cuando la migración y la sentencia de Mirko Lauer —«En el Perú, hoy, solo lo popular es moderno»— enmarcan la obra de E.P.S. Huayco. Recorre luego la hegemonía de la abstracción en los ochenta, el arte de derechos humanos de Ricardo Wiesse y Eduardo Villanes bajo el fujimorato, la irrupción de la Bienal Iberoamericana de Lima (1997) y el «bienalismo», y la generación de los 2000 (Flavia Gandolfo, Gilda Mantilla, Armando Andrade Tudela) vinculada al espacio La Culpable. El texto presenta además los ensayos de Miguel López, Gustavo Buntinx y Rodrigo Quijano incluidos en el volumen y la conversación de seis críticos (2011). Su aporte es explicitar la política de adquisiciones del MALI y su ambición de llenar el vacío institucional y discursivo, construyendo un marco regional e internacional para el arte peruano.</t>
         </is>
       </c>
     </row>
@@ -2846,27 +2846,27 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Quijano - Notas incompletas sobre el sitio de la fotografía peruana.md</t>
+          <t>López, Miguel A. - F(r)icciones cosmopolitas. Redefiniciones estéticas y políticas de una idea de vanguardia en los años 60s.txt</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>1900-2011 (con énfasis en 1920-1998)</t>
+          <t>1960-1976 (con antecedentes desde 1942-1947)</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo (MALI), s/f</t>
+          <t>Ensayo académico / capítulo de catálogo (MALI), s/f</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Quijano; Martín Chambi; José María Eguren; Carlos 'Chino' Domínguez; Aaron Siskind; Jesús Ruiz Durand; Claudia Martínez Garay; Daniela Ortiz; Foto Galería Secuencia; TAFOS; Taller NN; E.P.S. Huayco</t>
+          <t>Miguel A. López; Emilio Tarazona; Juan Acha; Fernando de Szyszlo; Jorge Romero Brest; Teresa Burga; Rafael Hastings; Grupo Arte Nuevo; Jesús Ruiz Durand; José Gómez Sicre; Marta Traba; Instituto de Arte Contemporáneo (IAC); MoMA / Instituto Di Tella</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Quijano ensaya una genealogía del 'sitio' de la fotografía peruana, sosteniendo que este medio inauguró un margen de creación moderno al margen de la institucionalidad académica de las bellas artes, alcanzando una temprana ubicuidad territorial y una masividad que condicionó la percepción misma de una realidad nacional. El texto, de estructura fragmentaria y numerada, contrapone dos matrices fundacionales: Martín Chambi como 'modernista sin modernidad' y profesional de la imagen surgido de una familia campesina andina —una 'oportunidad nacional'— frente a la miniatura pinhole intimista y hermética de José María Eguren, que prefigura la figura del fotógrafo-artista individual. Analiza a Carlos 'Chino' Domínguez como ojo testimonial de la urbanización y la nueva cultura popular (La resaca del Inca, el 'Cholo' Sotil, el filme Cholo y su reedición Mi cholo de Gruenberg), y la experiencia de la fotogalería Secuencia (1977-1980), que reinventó una tradición y un discurso del oficio adoptando a Minor White y Aaron Siskind. El marco conceptual enlaza fotografía, prensa y democratización de la imagen en el contexto del auge sindical y la repolitización popular de fines de los setenta, y la aparición de la fotoserigrafía disidente (Bedoya, Williams, Mariotti, Salazar) como catalizador de una nueva condición fotográfica colectiva, desde E.P.S. Huayco hasta el Taller NN. El aporte del texto es leer la fotografía como dispositivo de documento, archivo, memoria y duelo frente a la violencia política (Uchuraccay, Yuyanapaq), rastreando su 'grado cero' icónico en obras de Ruiz Durand, Claudia Martínez Garay y Daniela Ortiz, que develan la mirada colonial y la invisibilización étnica.</t>
+          <t>López reconstruye las mutaciones semánticas y políticas de la noción de vanguardia en el Perú entre los años sesenta y setenta, argumentando que la euforia cosmopolita del periodo fue el espejismo de una modernidad desarrollista tan prometedora como inacabada en un país socialmente fracturado. El objeto de estudio son las plataformas institucionales privadas (IAC, galerías, bienales americanas, concursos empresariales) que, apuntaladas por el panamericanismo de la Guerra Fría, la Alianza para el Progreso y la política curatorial estadounidense de José Gómez Sicre, promovieron primero la abstracción y luego el arte óptico, el pop y las ambientaciones. El texto traza el paso del declive de la abstracción szyszliana hacia el experimentalismo detonado por las conferencias de Jorge Romero Brest (1965) y la irrupción beligerante del grupo Arte Nuevo (1966-1968) contra el Festival Americano de Pintura. El marco conceptual articula la relación entre desarrollismo y vanguardia, y su posterior tensión con el subdesarrollo, siguiendo la radicalización de Juan Acha, quien tras 1968 y el golpe de Velasco redefine la vanguardia como 'guerrilla cultural' y horizonte revolucionario, hasta su exilio a México en 1971. López destaca las reconversiones de Teresa Burga y Rafael Hastings, el 'pop achorado' de Ruiz Durand al servicio de la Reforma Agraria, los festivales Contacta y las Carreras de chasquis. Su aporte es mostrar cómo la condición local, provinciana y periférica de las prácticas de los setenta y ochenta (Paréntesis, E.P.S. Huayco, Grupo Chaclacayo) actualizó de modo radical las pretensiones críticas sesenteras, canibalizando los conceptos metropolitanos de arte conceptual.</t>
         </is>
       </c>
     </row>
@@ -2878,32 +2878,64 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
+          <t>Quijano - Notas incompletas sobre el sitio de la fotografía peruana.md</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>1900-2011 (con énfasis en 1920-1998)</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Ensayo de catálogo (MALI), s/f</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>Rodrigo Quijano; Martín Chambi; José María Eguren; Carlos 'Chino' Domínguez; Aaron Siskind; Jesús Ruiz Durand; Claudia Martínez Garay; Daniela Ortiz; Foto Galería Secuencia; TAFOS; Taller NN; E.P.S. Huayco</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>Quijano ensaya una genealogía del 'sitio' de la fotografía peruana, sosteniendo que este medio inauguró un margen de creación moderno al margen de la institucionalidad académica de las bellas artes, alcanzando una temprana ubicuidad territorial y una masividad que condicionó la percepción misma de una realidad nacional. El texto, de estructura fragmentaria y numerada, contrapone dos matrices fundacionales: Martín Chambi como 'modernista sin modernidad' y profesional de la imagen surgido de una familia campesina andina —una 'oportunidad nacional'— frente a la miniatura pinhole intimista y hermética de José María Eguren, que prefigura la figura del fotógrafo-artista individual. Analiza a Carlos 'Chino' Domínguez como ojo testimonial de la urbanización y la nueva cultura popular (La resaca del Inca, el 'Cholo' Sotil, el filme Cholo y su reedición Mi cholo de Gruenberg), y la experiencia de la fotogalería Secuencia (1977-1980), que reinventó una tradición y un discurso del oficio adoptando a Minor White y Aaron Siskind. El marco conceptual enlaza fotografía, prensa y democratización de la imagen en el contexto del auge sindical y la repolitización popular de fines de los setenta, y la aparición de la fotoserigrafía disidente (Bedoya, Williams, Mariotti, Salazar) como catalizador de una nueva condición fotográfica colectiva, desde E.P.S. Huayco hasta el Taller NN. El aporte del texto es leer la fotografía como dispositivo de documento, archivo, memoria y duelo frente a la violencia política (Uchuraccay, Yuyanapaq), rastreando su 'grado cero' icónico en obras de Ruiz Durand, Claudia Martínez Garay y Daniela Ortiz, que develan la mirada colonial y la invisibilización étnica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Cap 2 - Historia/MALI</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
           <t>Villacorta (ed.) - ¿Un arte visual a contrapelo de los dictados metropolitanos? En el Perú, el arte moderno es un gesto tardío [conversación en el MALI, 2011].txt</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>1947-2011 (con eje en 1960-2002)</t>
         </is>
       </c>
-      <c r="D76" s="2" t="inlineStr">
+      <c r="D77" s="2" t="inlineStr">
         <is>
           <t>Transcripción editada de conversación (MALI), 2011</t>
         </is>
       </c>
-      <c r="E76" s="3" t="inlineStr">
+      <c r="E77" s="3" t="inlineStr">
         <is>
           <t>Jorge Villacorta; Gustavo Buntinx; Miguel A. López; Rodrigo Quijano; Tatiana Cuevas; Natalia Majluf; E.P.S. Huayco; Grupo Arte Nuevo; Taller NN; Grupo Chaclacayo; Christian Bendayán; Fernando Bryce; MALI / Micromuseo</t>
         </is>
       </c>
-      <c r="F76" s="3" t="inlineStr">
+      <c r="F77" s="3" t="inlineStr">
         <is>
           <t>Editada por Villacorta a partir de dos sesiones de 2011 en el MALI, esta conversación a seis voces indaga si lo moderno está clausurado en el arte peruano de modo que permita definir lo contemporáneo. La tesis articuladora, propuesta por Quijano, es que en el Perú lo moderno solo ha podido darse 'a contrapelo' y como 'gesto tardío', a destiempo de las modernidades metropolitanas; López y Buntinx la matizan con la idea de temporalidades dislocadas y friccionadas que impiden toda historia lineal. El objeto de estudio es la genealogía de la vanguardia local: la contraposición entre Arte Nuevo (1966-1968), leído como destello cosmopolita fugaz, y E.P.S. Huayco y Paréntesis, cuya apropiación de Sarita Colonia y el 'pop achorado' marca una ruptura más perdurable y pertinente al medio. Buntinx despliega una secuencia estilístico-conceptual en clave pop/místico-libidinal —de la Twiggy de Emilio Hernández a Quistococha de Bendayán, pasando por el afiche de Ruiz Durand, la Maoirilyn del Taller NN y La Pachakuti de Alfredo Márquez— ligada a periodos políticos (desarrollismo, velasquismo, utopía socialista, dictadura fujimorista, revolución capitalista). Majluf sitúa el quiebre epocal de fin de siglo en el ingreso de la 'referencia' fotográfica (Bryce, Milagros de la Torre, Juan Enrique Bedoya, Mantilla), frente al neobarroco. El texto discute además la construcción de públicos, la institucionalidad faltante, el rol del curador, el mercado 'social' peruano, las subastas del MALI y la 'normalización de la diferencia' como riesgo de la consagración institucional del pasado radical.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F76"/>
+  <autoFilter ref="A1:F77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Cataloga 4 fuentes ICPNA/ARTUS y añade mapa de aportes al «mandato crítico»
- Añade 4 filas a tabla-cap2-historia.csv (Premio ICPNA 2026, Beca ARTUS-ICPNA WIELS 2026, podcast EP12 Marzano, conversatorio ARTUS en Park) y regenera el .xlsx.
- Nuevo documento en analisis/ que historiza cómo estas fuentes aportan al «mandato crítico» (dimensión de la gestión operando; llena el vacío del Comité de Adquisiciones del MALI), con separación estricta cita literal / [lectura].

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bob4w11uQRyAcv1Qayw1V
</commit_message>
<xml_diff>
--- a/Sistematización/tablas-sistematizacion.xlsx
+++ b/Sistematización/tablas-sistematizacion.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Extras" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$81</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cap 3 - Análisis'!$A$1:$F$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Teoría'!$A$1:$F$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Extras'!$A$1:$F$4</definedName>
@@ -37,7 +37,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -86,13 +86,13 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -542,27 +542,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Biczel - Sobre la imposibilidad de trazar un mapa. El «fracaso» de la Bienal de Lima 1997-2002 [Caiana].md</t>
+          <t>BASES-PREMIO-ICPNA-ARTE-CONTEMPORANEO-2026.pdf</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>1997-2002</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico (revista Caiana n.º 11, CAIA), 2017</t>
+          <t>Documento normativo (bases de concurso), 2026; exposición 24 sep–20 dic 2026; premiación 26 nov 2026</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Dorota Biczel; Francis Alÿs; Allora &amp; Calzadilla; Rogelio López Cuenca; Tupac*Caput; Luis Lama; Cuauhtémoc Medina; Miwon Kwon; Grant Kester; Bienal Iberoamericana de Lima; Municipalidad Metropolitana de Lima; Alberto Fujimori</t>
+          <t>ICPNA (Instituto Cultural Peruano Norteamericano); curador designado por el ICPNA; jurado de tres profesionales del campo artístico designados por el ICPNA; Espacio Juan Pardo Heeren (Cercado de Lima)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>El ensayo interroga por qué la Bienal Iberoamericana de Lima (1997, 1999, 2002) fracasó como plataforma de legitimación dentro del circuito global de bienales de los noventa, pese a haber alojado proyectos hoy canónicos del “arte participativo”. Biczel rechaza la explicación habitual —la pérdida del apoyo municipal tras la llegada del alcalde Castañeda Lossio— y propone que el fracaso obedeció a una tensión estructural entre la noción de sitio manejada por los organizadores (Luis Lama, la Municipalidad) y la que movilizaron los artistas internacionales invitados. Apoyándose en Miwon Kwon, rastrea el desplazamiento noventero del site-specific desde un lugar físico y fijo hacia un “sitio discursivo” fluido y desterritorializado, coincidente con el “giro social” del arte. Analiza tres obras de la tercera edición: Cuando la fe mueve montañas de Francis Alÿs, Tiza de Allora &amp; Calzadilla y Lima i[NN]memoriam de Rogelio López Cuenca con el grupo Tupac*Caput. Muestra que las dos primeras alcanzaron enorme visibilidad internacional precisamente porque su localidad se volvió abstracta e intercambiable, mientras que la obra de López Cuenca —anclada en catorce “sitios de memoria” reales del conflicto armado y la violencia urbana— permaneció invisible fuera de Lima. Recurriendo a Kester, Bishop y Thompson, critica cómo el marco interpretativo del arte colaborativo borra las jerarquías de poder entre artistas extranjeros y participantes peruanos. Tesis central: la Bienal fracasó por aferrarse a un modelo identitario y a una localidad estable (el Centro Histórico) inservible en un circuito global supuestamente posidentitario, agravado por la caída del régimen de Fujimori, que desdibujó la legibilidad de la ciudad como sitio.</t>
+          <t>Bases oficiales del Premio ICPNA de Arte Contemporáneo 2026. Documento normativo que fija las condiciones de participación de un concurso de arte contemporáneo abierto a artistas peruanos residentes en el Perú o el extranjero y a extranjeros residentes en el Perú, mayores de edad, en disciplinas de pintura, dibujo, fotografía, grabado, acuarela, escultura, técnica mixta, instalación y video, con temática libre. El concurso se estructura en tres etapas: (1) evaluación de expedientes digitales (ficha, CV de máx. 700 palabras, portafolio con texto de presentación de máx. 500 palabras y hasta siete imágenes de obra reciente); (2) selección de obras para exposición a cargo de 'un curador designado por el ICPNA'; y (3) premiación por 'un jurado integrado por tres profesionales del campo artístico, designados por el ICPNA'. El jurado otorga un único premio y tres menciones honrosas, no puede declarar desierto el premio ni compartirlo, y su decisión es inapelable pero fundamentada por escrito. El ganador recibe S/ 30 000 y una exposición individual en un espacio del ICPNA; se especifica que 'el premio no implica la adquisición de la obra por parte del ICPNA'. Fija dimensiones máximas de obra, restricciones de materiales (nada orgánico perecible ni punzocortante), plazos (envío hasta el 14 de agosto; selección publicada el 21 de agosto) y la exhibición del 24 de septiembre al 20 de diciembre de 2026. Fuente primaria institucional que documenta los criterios, la autoridad curatorial y los mecanismos de valoración con que una institución delimita y premia el arte contemporáneo joven en Lima.</t>
         </is>
       </c>
     </row>
@@ -574,27 +574,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Borea - Configuring the New Lima Art Scene. An Anthropological Analysis of Contemporary Art in Latin America (2021).md</t>
+          <t>Bases-de-Convovatoria-ARTUS-ICPNA-2026.pdf</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>1997-2014</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Libro / monografía académica (Routledge), 2021</t>
+          <t>Documento normativo (bases de convocatoria), 2026; residencia 1 oct–31 dic 2026; inscripción 29 abr–1 jun 2026</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Giuliana Borea; Museo de Arte de Lima (MALI); Fernando Bryce; Natalia Iguiñiz; Rember Yahuarcani; Elena Damiani; Bienal de Lima; ArtLima; PArC; Micromuseo; Routledge; PUCP; Universidad de Essex</t>
+          <t>ICPNA; ARTUS; WIELS (laboratorio internacional de arte contemporáneo, Bruselas, Bélgica); comité especializado de selección; artistas visuales peruanos jóvenes</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Monografía antropológica que examina la configuración de la escena de arte contemporáneo en Lima entre 1997 y 2014, articulándola con la renovación social posterior al régimen de Fujimori, la transformación neoliberal de Lima como “ciudad creativa” y el fortalecimiento de las redes de arte latinoamericano. Borea identifica tres momentos: (1) exploraciones artísticas y nuevas narrativas curatoriales durante la transición democrática (fines de los noventa a 2006), detonadas por la Bienal de Lima y las movilizaciones antifujimoristas, cuando se consolida la figura del curador local y se amplía lo “contemporáneo” para incluir el arte amazónico; (2) reforzamiento del museo y de las redes regionales (2006-2013), con el protagonismo del MALI, el auge del coleccionista y la participación de agentes peruanos como clase cultural transnacional; (3) el ascenso del mercado (desde 2010), que culmina en la aparición simultánea de dos ferias (ArtLima y PArC). El marco conceptual dialoga críticamente con Bourdieu (campo), Latour (redes de actores), Turner (arenas), Clifford (articulaciones), Appadurai (imaginación) y la Teoría Social del Arte latinoamericana (Acha), atendiendo a clase, raza, género y generación, y a las categorías de “cholo”, “indígena” y “arte popular”. Su tesis: la articulación de Lima con el “mundo global del arte” y con el proyecto de la “ciudad creativa” no difunde nuevos valores estéticos sino que expande formatos, prototipos y lógicas de mercado dominantes, movilizados por élites transnacionales; hay una “movilización de lo político sin política”. Combina capítulos analíticos con “trayectorias” de artistas (Bryce, Iguiñiz, Yahuarcani, Damiani) y una sección curatorial sobre la autorreflexión de la escena.</t>
+          <t>Bases de la Beca ARTUS-ICPNA WIELS 2026. Documento normativo que reglamenta una convocatoria conjunta del ICPNA y ARTUS para financiar una residencia artística de tres meses (octubre–diciembre de 2026) en WIELS, Bruselas, presentado como 'laboratorio internacional para la creación y difusión del arte contemporáneo'. La beca se dirige a artistas visuales de nacionalidad peruana, mayores de edad y con dominio del inglés, y busca 'proporcionar la movilidad internacional a un artista visual peruano' y 'establecer conexiones entre la escena artística de Bélgica y del Perú'. Detalla la documentación de postulación (CV, declaración del artista de máx. 250 palabras, declaración de propósito de máx. 300 palabras, tres referencias, portafolio de hasta diez imágenes, certificación en estudios de arte). El mecanismo de selección es de doble instancia: 'un comité especializado de selección', cuyos miembros son 'designados por las partes involucradas en la organización de la beca', preselecciona los diez portafolios más destacados, y 'será responsabilidad de WIELS seleccionar al único ganador'. La dotación incluye pasajes, estudio de 40 m², alojamiento y '800 euros por cada mes de estancia'. Precisa plazos (inscripción del 29 de abril al 1 de junio; finalistas el 17 de junio; ganador el 30 de junio) y cláusulas de propiedad intelectual y derechos de imagen a favor de ICPNA y ARTUS. Fuente primaria que documenta la infraestructura de becas, los criterios de elegibilidad y la cadena de decisión (comité local + institución extranjera) con que se selecciona y proyecta internacionalmente al arte joven peruano.</t>
         </is>
       </c>
     </row>
@@ -606,27 +606,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - Lava la bandera. The Colectivo Sociedad Civil and the Cultural Overthrow of the Fujimori-Montesinos Dictatorship (2017) [Collective Situations, cap. 1].md</t>
+          <t>Biczel - Sobre la imposibilidad de trazar un mapa. El «fracaso» de la Bienal de Lima 1997-2002 [Caiana].md</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2000-2001</t>
+          <t>1997-2002</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro (Collective Situations, Duke University Press), 2017; basado en texto en español de 2006</t>
+          <t>Artículo académico (revista Caiana n.º 11, CAIA), 2017</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Colectivo Sociedad Civil; Fernando Bryce; Emilio Santisteban; Susana Torres; Claudia Coca; Natalia Iguiñiz; Alberto Fujimori; Vladimiro Montesinos; Walter Benjamin; Micromuseo; CADA</t>
+          <t>Dorota Biczel; Francis Alÿs; Allora &amp; Calzadilla; Rogelio López Cuenca; Tupac*Caput; Luis Lama; Cuauhtémoc Medina; Miwon Kwon; Grant Kester; Bienal Iberoamericana de Lima; Municipalidad Metropolitana de Lima; Alberto Fujimori</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Capítulo que documenta y teoriza la acción Lava la bandera del Colectivo Sociedad Civil (CSC) como contribución artística al “derrocamiento cultural” de la dictadura de Fujimori-Montesinos. Buntinx sostiene que el derrocamiento de una dictadura tiene una dimensión cultural tan decisiva como la económica, política o militar: la construcción de un consenso democrático y de una ciudadanía activa mediante la lucha por el poder simbólico en el espacio público. Reconstruye la génesis del CSC —surgido tras el fraude electoral de abril de 2000, con antecedentes en la exposición Emergencia artística (1999)— y describe el ritual iniciado en mayo de 2000 en la Plaza Mayor de Lima: ciudadanos lavando banderas peruanas de tela con agua y jabón y colgándolas en tendederos, en un gesto de purificación patriótica que resignifica los emblemas nacionales. Analiza su masiva replicación nacional e internacional, la represión estatal y las infiltraciones del SIN, así como variantes posteriores como Cose la bandera (Sana tu país, 2001), vinculada a la campaña por la Comisión de la Verdad. En lo conceptual apela a Walter Benjamin (aura, ritual, valor de culto, politización del arte frente a la estetización fascista de la política) y a antecedentes como el Siluetazo argentino y el CADA chileno. Su tesis clave es que el CSC no buscaba producir “obras” sino “situaciones” apropiables por la ciudadanía, diluyendo la especificidad artística: el arte opera como laboratorio de acciones comunicativas cuyo criterio de verdad está fuera del arte. Reivindica un “heroísmo de la vida cotidiana” y una religiosidad cívica, doméstica y casi pop, capaz de instaurar una nueva ciudadanía.</t>
+          <t>El ensayo interroga por qué la Bienal Iberoamericana de Lima (1997, 1999, 2002) fracasó como plataforma de legitimación dentro del circuito global de bienales de los noventa, pese a haber alojado proyectos hoy canónicos del “arte participativo”. Biczel rechaza la explicación habitual —la pérdida del apoyo municipal tras la llegada del alcalde Castañeda Lossio— y propone que el fracaso obedeció a una tensión estructural entre la noción de sitio manejada por los organizadores (Luis Lama, la Municipalidad) y la que movilizaron los artistas internacionales invitados. Apoyándose en Miwon Kwon, rastrea el desplazamiento noventero del site-specific desde un lugar físico y fijo hacia un “sitio discursivo” fluido y desterritorializado, coincidente con el “giro social” del arte. Analiza tres obras de la tercera edición: Cuando la fe mueve montañas de Francis Alÿs, Tiza de Allora &amp; Calzadilla y Lima i[NN]memoriam de Rogelio López Cuenca con el grupo Tupac*Caput. Muestra que las dos primeras alcanzaron enorme visibilidad internacional precisamente porque su localidad se volvió abstracta e intercambiable, mientras que la obra de López Cuenca —anclada en catorce “sitios de memoria” reales del conflicto armado y la violencia urbana— permaneció invisible fuera de Lima. Recurriendo a Kester, Bishop y Thompson, critica cómo el marco interpretativo del arte colaborativo borra las jerarquías de poder entre artistas extranjeros y participantes peruanos. Tesis central: la Bienal fracasó por aferrarse a un modelo identitario y a una localidad estable (el Centro Histórico) inservible en un circuito global supuestamente posidentitario, agravado por la caída del régimen de Fujimori, que desdibujó la legibilidad de la ciudad como sitio.</t>
         </is>
       </c>
     </row>
@@ -638,27 +638,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - Los signos mesiánicos. Fardos y banderas en la obra de Eduardo Tokeshi durante la «República de Weimar peruana» 1980-1992.md</t>
+          <t>Borea - Configuring the New Lima Art Scene. An Anthropological Analysis of Contemporary Art in Latin America (2021).md</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>1980-1992</t>
+          <t>1997-2014</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico / catálogo de exposición (Galería Fórum), reformulado hacia 2001-2002 a partir de una ponencia de 1994 (publicada en 1995)</t>
+          <t>Libro / monografía académica (Routledge), 2021</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Eduardo Tokeshi; Jaime Higa; Armando Williams; Juan Javier Salazar; Jorge Eduardo Eielson; Jasper Johns; Christo Javacheff; Sendero Luminoso; Galería Fórum; Museo de Arte de la UNMSM</t>
+          <t>Giuliana Borea; Museo de Arte de Lima (MALI); Fernando Bryce; Natalia Iguiñiz; Rember Yahuarcani; Elena Damiani; Bienal de Lima; ArtLima; PArC; Micromuseo; Routledge; PUCP; Universidad de Essex</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Ensayo (versión corregida y aumentada de una ponencia de 1994) que analiza la iconografía del fardo funerario y la bandera en la obra de Eduardo Tokeshi durante la “República de Weimar peruana”, concepto acuñado por Buntinx para nombrar la frágil democracia electoral entre 1980 y el autogolpe de Fujimori de 1992. Tesis: en un país de tiempos dislocados y superpuestos, atravesado por la guerra interna (Sendero Luminoso, MRTA, represión estatal), cierta pequeña burguesía ilustrada procesa la violencia mediante signos mesiánicos ligados al fardo —momia, feto y semilla a la vez (malki)—, imagen que enlaza muerte, represión y resurrección de una cultura andina reprimida, asociada al mito de Inkarrí y al Pachakuti. El marco conceptual moviliza a Benjamin (alegoría), Freud (lo unheimlich, el retorno de lo reprimido) y categorías locales como el “pop achorado”. Recorre la evolución de Tokeshi: piezas tempranas de 1985 con fardos y fotografías carnet borradas; Uchuraccay (1985, con Jaime Higa), que sustituye el cadáver embolsado por el fardo tras la masacre de los periodistas; la serie Bandera I-VI (1985-1992), donde el estandarte patrio funciona a la vez como vientre y sudario; y su deriva hacia la introspección y el desencanto (Sólo nubes veo para ti, Últimos refugios, Matasueños) a medida que la violencia alcanza a las clases medias limeñas (atentado de Tarata, 1992). Buntinx lee las desapariciones forzadas y las resurrecciones míticas como una tensión irresuelta, contrasta a Tokeshi con Juan Javier Salazar y Armando Williams, y recupera la controversia política por la exposición Algo va a pasar (1987).</t>
+          <t>Monografía antropológica que examina la configuración de la escena de arte contemporáneo en Lima entre 1997 y 2014, articulándola con la renovación social posterior al régimen de Fujimori, la transformación neoliberal de Lima como “ciudad creativa” y el fortalecimiento de las redes de arte latinoamericano. Borea identifica tres momentos: (1) exploraciones artísticas y nuevas narrativas curatoriales durante la transición democrática (fines de los noventa a 2006), detonadas por la Bienal de Lima y las movilizaciones antifujimoristas, cuando se consolida la figura del curador local y se amplía lo “contemporáneo” para incluir el arte amazónico; (2) reforzamiento del museo y de las redes regionales (2006-2013), con el protagonismo del MALI, el auge del coleccionista y la participación de agentes peruanos como clase cultural transnacional; (3) el ascenso del mercado (desde 2010), que culmina en la aparición simultánea de dos ferias (ArtLima y PArC). El marco conceptual dialoga críticamente con Bourdieu (campo), Latour (redes de actores), Turner (arenas), Clifford (articulaciones), Appadurai (imaginación) y la Teoría Social del Arte latinoamericana (Acha), atendiendo a clase, raza, género y generación, y a las categorías de “cholo”, “indígena” y “arte popular”. Su tesis: la articulación de Lima con el “mundo global del arte” y con el proyecto de la “ciudad creativa” no difunde nuevos valores estéticos sino que expande formatos, prototipos y lógicas de mercado dominantes, movilizados por élites transnacionales; hay una “movilización de lo político sin política”. Combina capítulos analíticos con “trayectorias” de artistas (Bryce, Iguiñiz, Yahuarcani, Damiani) y una sección curatorial sobre la autorreflexión de la escena.</t>
         </is>
       </c>
     </row>
@@ -670,27 +670,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - The Power and the Illusion. Aura, Lost and Restored in the «Peruvian Weimar Republic» 1980-1992 [EN].md</t>
+          <t>Buntinx - Lava la bandera. The Colectivo Sociedad Civil and the Cultural Overthrow of the Fujimori-Montesinos Dictatorship (2017) [Collective Situations, cap. 1].md</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>1980-1992</t>
+          <t>2000-2001</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Ensayo / capítulo de libro en inglés (Beyond the Fantastic, ed. Gerardo Mosquera), 1995</t>
+          <t>Capítulo de libro (Collective Situations, Duke University Press), 2017; basado en texto en español de 2006</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Huayco E.P.S.; Francisco Mariotti; Taller NN; Herbert Rodríguez; Juan Javier Salazar; Armando Williams; Jesús Ruiz Durand; Walter Benjamin; Sarita Colonia; Gerardo Mosquera; Galería Fórum</t>
+          <t>Gustavo Buntinx; Colectivo Sociedad Civil; Fernando Bryce; Emilio Santisteban; Susana Torres; Claudia Coca; Natalia Iguiñiz; Alberto Fujimori; Vladimiro Montesinos; Walter Benjamin; Micromuseo; CADA</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Ensayo (publicado en inglés en el volumen Beyond the Fantastic, editado por Gerardo Mosquera, 1995) que reelabora, mediante el concepto benjaminiano de aura, la producción de las artes plásticas radicales durante la “República de Weimar peruana” (1980-1992). Buntinx analiza en detalle obras que “abren y cierran” la década, rastreando el movimiento entre la pérdida cosmopolita del aura y su restauración “provinciana”. Del colectivo Huayco (E.P.S.) examina Arte al paso (1980), tapiz de 10.000 latas vacías de leche evaporada sobre las que se pinta una ración de salchipapas —crítica al hambre y a las transnacionales, y homenaje al reciclaje de las barriadas— y Sarita Colonia (1980), retrato de la santa popular instalado a la intemperie junto a la Panamericana, cerca de Pachacamac, que funciona simultáneamente como arte de vanguardia y como ícono religioso reapropiado por los migrantes: una “huaca moderna”, un ex-voto que restaura el aura. Del Taller NN analiza Viva el maoísmo / Maorilyn (c. 1990), collage-emblema que ataca alegóricamente el aura del “Gran Timonel”. El marco conceptual convoca a Benjamin (aura, montaje, símbolo frente a alegoría, Trauerspiel), Adorno y las categorías del “pop achorado” y lo “chicha”. Tesis: en esta periferia extrema las estrategias posmodernas de desmitificación se canibalizan para remitificar; los gestos contrahegemónicos se orientan a nuevas hegemonías, fundiendo tradiciones andinas y horizonte socialista en una “modernidad popular”. El aura se restaura en el mismo gesto que enuncia su pérdida, reflejando la ambivalencia del propio Benjamin entre misticismo y materialismo.</t>
+          <t>Capítulo que documenta y teoriza la acción Lava la bandera del Colectivo Sociedad Civil (CSC) como contribución artística al “derrocamiento cultural” de la dictadura de Fujimori-Montesinos. Buntinx sostiene que el derrocamiento de una dictadura tiene una dimensión cultural tan decisiva como la económica, política o militar: la construcción de un consenso democrático y de una ciudadanía activa mediante la lucha por el poder simbólico en el espacio público. Reconstruye la génesis del CSC —surgido tras el fraude electoral de abril de 2000, con antecedentes en la exposición Emergencia artística (1999)— y describe el ritual iniciado en mayo de 2000 en la Plaza Mayor de Lima: ciudadanos lavando banderas peruanas de tela con agua y jabón y colgándolas en tendederos, en un gesto de purificación patriótica que resignifica los emblemas nacionales. Analiza su masiva replicación nacional e internacional, la represión estatal y las infiltraciones del SIN, así como variantes posteriores como Cose la bandera (Sana tu país, 2001), vinculada a la campaña por la Comisión de la Verdad. En lo conceptual apela a Walter Benjamin (aura, ritual, valor de culto, politización del arte frente a la estetización fascista de la política) y a antecedentes como el Siluetazo argentino y el CADA chileno. Su tesis clave es que el CSC no buscaba producir “obras” sino “situaciones” apropiables por la ciudadanía, diluyendo la especificidad artística: el arte opera como laboratorio de acciones comunicativas cuyo criterio de verdad está fuera del arte. Reivindica un “heroísmo de la vida cotidiana” y una religiosidad cívica, doméstica y casi pop, capaz de instaurar una nueva ciudadanía.</t>
         </is>
       </c>
     </row>
@@ -702,27 +702,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Castrillón - La generación del 68. Entre la agonía y la fiesta de la modernidad.md</t>
+          <t>Buntinx - Los signos mesiánicos. Fardos y banderas en la obra de Eduardo Tokeshi durante la «República de Weimar peruana» 1980-1992.md</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>1963-1980 (con antecedentes desde los años 50)</t>
+          <t>1980-1992</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro de historia del arte, s/f (posterior a 2002)</t>
+          <t>Ensayo académico / catálogo de exposición (Galería Fórum), reformulado hacia 2001-2002 a partir de una ponencia de 1994 (publicada en 1995)</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Alfonso Castrillón; Juan Acha; Grupo Arte Nuevo; Teresa Burga; Gloria Gómez Sánchez; Emilio Hernández Saavedra; Luis Arias Vera; Rafael Hastings; Jesús Ruiz Durand; Joaquín López Antay; Fernando de Szyszlo; Instituto de Arte Contemporáneo (IAC)</t>
+          <t>Gustavo Buntinx; Eduardo Tokeshi; Jaime Higa; Armando Williams; Juan Javier Salazar; Jorge Eduardo Eielson; Jasper Johns; Christo Javacheff; Sendero Luminoso; Galería Fórum; Museo de Arte de la UNMSM</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Capítulo de historia del arte peruano dedicado a la “generación del 68”, los artistas de vanguardia que hacia los años sesenta y setenta adoptaron el Pop, el Op, el Hard-Edge (filo duro) y el arte conceptual/no-objetual, en convivencia con el surrealismo, la nueva figuración y el expresionismo abstracto supérstite. Castrillón enmarca el periodo entre el gobierno de Belaúnde (1963) y el régimen militar de Velasco (1968-1975), atendiendo a la vida política, el desarrollo educativo, el crecimiento de las galerías y del mercado limeño. El eje conceptual es la figura del crítico Juan Acha, cuya defensa de una modernidad universalista contra el “provincianismo” indigenista y las “conscripciones” de la peruanidad, su teoría del arte como sistema de producción-distribución-consumo y sus conferencias de 1969 sobre mass media, estructuralismo y no-objetualismo articularon el ingreso de las vanguardias. Reconstruye la protesta del grupo Arte Nuevo (1966) frente al Festival Americano de Pintura y su muestra en la galería El ombligo de Adán, con Luis Arias Vera, Teresa Burga, Gloria Gómez Sánchez, Emilio Hernández Saavedra, Rafael Hastings y otros; traza el informalismo (Gómez Sánchez), los surrealismos (Quintanilla, Chávez, Tsuchiya, Revilla), la figuración (Bill Caro, Palao), el “pop achorado” de Ruiz Durand y el conceptualismo pionero de Burga y Hastings. Discute la polémica de 1975 por el Premio Nacional otorgado al retablista popular Joaquín López Antay, que planteó el reconocimiento del arte popular en la historia del arte peruano. La tesis, sugerida por el título “entre la agonía y la fiesta”, es la tensión de una modernidad rezagada y dependiente de importaciones estéticas que exigían ser asimiladas con recursos y nutrientes locales.</t>
+          <t>Ensayo (versión corregida y aumentada de una ponencia de 1994) que analiza la iconografía del fardo funerario y la bandera en la obra de Eduardo Tokeshi durante la “República de Weimar peruana”, concepto acuñado por Buntinx para nombrar la frágil democracia electoral entre 1980 y el autogolpe de Fujimori de 1992. Tesis: en un país de tiempos dislocados y superpuestos, atravesado por la guerra interna (Sendero Luminoso, MRTA, represión estatal), cierta pequeña burguesía ilustrada procesa la violencia mediante signos mesiánicos ligados al fardo —momia, feto y semilla a la vez (malki)—, imagen que enlaza muerte, represión y resurrección de una cultura andina reprimida, asociada al mito de Inkarrí y al Pachakuti. El marco conceptual moviliza a Benjamin (alegoría), Freud (lo unheimlich, el retorno de lo reprimido) y categorías locales como el “pop achorado”. Recorre la evolución de Tokeshi: piezas tempranas de 1985 con fardos y fotografías carnet borradas; Uchuraccay (1985, con Jaime Higa), que sustituye el cadáver embolsado por el fardo tras la masacre de los periodistas; la serie Bandera I-VI (1985-1992), donde el estandarte patrio funciona a la vez como vientre y sudario; y su deriva hacia la introspección y el desencanto (Sólo nubes veo para ti, Últimos refugios, Matasueños) a medida que la violencia alcanza a las clases medias limeñas (atentado de Tarata, 1992). Buntinx lee las desapariciones forzadas y las resurrecciones míticas como una tensión irresuelta, contrasta a Tokeshi con Juan Javier Salazar y Armando Williams, y recupera la controversia política por la exposición Algo va a pasar (1987).</t>
         </is>
       </c>
     </row>
@@ -734,27 +734,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Castrillón - Reflexiones sobre el arte conceptual en Perú y sus proyecciones.md</t>
+          <t>Buntinx - The Power and the Illusion. Aura, Lost and Restored in the «Peruvian Weimar Republic» 1980-1992 [EN].md</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Años 60-70 en Perú (con antecedentes desde 1436 y del Dadá/Duchamp)</t>
+          <t>1980-1992</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Ponencia de coloquio (arte no-objetual), 1981 (reed. c. 2007)</t>
+          <t>Ensayo / capítulo de libro en inglés (Beyond the Fantastic, ed. Gerardo Mosquera), 1995</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Alfonso Castrillón Vizcarra; Juan Acha; Teresa Burga; Rafael Hastings; Emilio Hernández; Joaquín López Antay; Fernando de Szyszlo; Jorge Romero Brest; Ruiz Durand; Grupo Espacio; Instituto de Arte Contemporáneo (IAC); Universidad Nacional Mayor de San Marcos</t>
+          <t>Gustavo Buntinx; Huayco E.P.S.; Francisco Mariotti; Taller NN; Herbert Rodríguez; Juan Javier Salazar; Armando Williams; Jesús Ruiz Durand; Walter Benjamin; Sarita Colonia; Gerardo Mosquera; Galería Fórum</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Ponencia leída por Alfonso Castrillón en el Primer Coloquio Latinoamericano sobre Arte No-Objetual (Medellín, 1981) que discute la pertinencia de la categoría "no-objetualismo" y propone, en su lugar, una historia de la progresiva desaparición del objeto artístico. Castrillón rastrea la conciencia del concepto desde Alberti, Leonardo y Miguel Ángel, para argumentar que la objetualidad y sus atractivos sensibles prevalecieron durante siglos hasta que, hacia 1966, el Conceptual Art desplazó esa intención tradicional. Sostiene que no existe un no-objetual absoluto, pues toda manifestación se apoya en un soporte material; prefiere hablar de una crisis de la sensibilidad y del objeto-mercancía, gestada desde el impresionismo, el cubismo, el futurismo, Dadá, Duchamp y el minimalismo. El aporte central es su lectura del caso peruano: describe la vanguardia como fenómeno atípico y desfasado respecto de una industrialización incipiente (desde Odría), reconstruyendo hitos del pop, op y conceptual local (Luis Arias Vera, Gloria Gómez Sánchez, Teresa Burga, Ruiz Durand), la irradiación de Romero Brest y, sobre todo, la crítica activa de Juan Acha, cuyo entusiasmo por el "desarrollo" juzga estimulante pero sin eco material. Valora experiencias conceptuales de Emilio Hernández, el Autorretrato de Teresa Burga y las acciones de Rafael Hastings. Su tesis más provocadora considera la premiación de Joaquín López Antay (1975) como la mejor acción de arte conceptual peruana, por golpear desde dentro la ideología estética señorial. Concluye reivindicando el arte conceptual como crítica operativa, efímera y útil en ámbitos universitarios, y aboga por un arte de la vida frente a la mercancía.</t>
+          <t>Ensayo (publicado en inglés en el volumen Beyond the Fantastic, editado por Gerardo Mosquera, 1995) que reelabora, mediante el concepto benjaminiano de aura, la producción de las artes plásticas radicales durante la “República de Weimar peruana” (1980-1992). Buntinx analiza en detalle obras que “abren y cierran” la década, rastreando el movimiento entre la pérdida cosmopolita del aura y su restauración “provinciana”. Del colectivo Huayco (E.P.S.) examina Arte al paso (1980), tapiz de 10.000 latas vacías de leche evaporada sobre las que se pinta una ración de salchipapas —crítica al hambre y a las transnacionales, y homenaje al reciclaje de las barriadas— y Sarita Colonia (1980), retrato de la santa popular instalado a la intemperie junto a la Panamericana, cerca de Pachacamac, que funciona simultáneamente como arte de vanguardia y como ícono religioso reapropiado por los migrantes: una “huaca moderna”, un ex-voto que restaura el aura. Del Taller NN analiza Viva el maoísmo / Maorilyn (c. 1990), collage-emblema que ataca alegóricamente el aura del “Gran Timonel”. El marco conceptual convoca a Benjamin (aura, montaje, símbolo frente a alegoría, Trauerspiel), Adorno y las categorías del “pop achorado” y lo “chicha”. Tesis: en esta periferia extrema las estrategias posmodernas de desmitificación se canibalizan para remitificar; los gestos contrahegemónicos se orientan a nuevas hegemonías, fundiendo tradiciones andinas y horizonte socialista en una “modernidad popular”. El aura se restaura en el mismo gesto que enuncia su pérdida, reflejando la ambivalencia del propio Benjamin entre misticismo y materialismo.</t>
         </is>
       </c>
     </row>
@@ -766,27 +766,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Conversatorio - Hay algo incomestible en la garganta - 2021-10-13 [Sala de Lectura].transcripcion.md</t>
+          <t>Castrillón - La generación del 68. Entre la agonía y la fiesta de la modernidad.md</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>1988-2002 (años 90)</t>
+          <t>1963-1980 (con antecedentes desde los años 50)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Transcripción de conversatorio, 13-10-2021</t>
+          <t>Capítulo de libro de historia del arte, s/f (posterior a 2002)</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Elena Tejada-Herrera; Susana Torres; Cecilia (autora de La máquina de carne); Jorge Villacorta; galería Parafernalia; ICPNA; Natalia Iguíñiz; Gilda Mantilla; Elena Valera; Seminario de Historia Rural Andina; Sala de Lectura</t>
+          <t>Alfonso Castrillón; Juan Acha; Grupo Arte Nuevo; Teresa Burga; Gloria Gómez Sánchez; Emilio Hernández Saavedra; Luis Arias Vera; Rafael Hastings; Jesús Ruiz Durand; Joaquín López Antay; Fernando de Szyszlo; Instituto de Arte Contemporáneo (IAC)</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Transcripción del conversatorio de cierre de la exposición "Hay algo incomestible en la garganta. Poéticas antipatriarcales y nueva escena en los años noventa" (curaduría de Miguel A. López, ICPNA, 2021), con las artistas Elena Tejada-Herrera, Susana Torres y Cecilia (autora de La máquina de carne). López enmarca la muestra entre 1988 y 2002 y en el contexto de la dictadura fujimorista, el neoliberalismo y la violencia política, proponiendo dos ejes: la emergencia de representaciones que desafían estructuras misóginas y la reconfiguración de los bordes de la escena artística. Las artistas comentan obras concretas: Tejada-Herrera describe performances como "Recuerdo" (1998), realizada en San Marcos tomada por el ejército en alusión a los desaparecidos de La Cantuta, y "La mujer yo-yo", que subvierte el imaginario del peruano doliente; Torres narra su tránsito del modelaje al autorretrato y a la serie de banderas exhibida en Parafernalia con Jorge Villacorta, y su descubrimiento del feminismo vía Flora Tristán; Cecilia explica el fotomatón interactivo "Máquina de carne" (2000-2001) como dispositivo sobre sexualidad, cuerpo y foto carnet, y su recorrido por distintos estratos sociales. El diálogo articula la noción de un "arte de urgencia" intuitivo y anterior al vocabulario feminista instalado hacia 2021, discute la relectura histórica que permite la muestra, la sororidad, la censura y la recontextualización de obras. Se mencionan trayectorias paralelas (Iguíñiz, Mantilla, Bedoya, Gandolfo, Rocío Rodrigo, Johanna Hamann) y la incorporación de artistas amazónicas (Elena Valera, Astrid Canayo) y del Seminario de Historia Rural Andina, ampliando el canon de la escena limeña noventera.</t>
+          <t>Capítulo de historia del arte peruano dedicado a la “generación del 68”, los artistas de vanguardia que hacia los años sesenta y setenta adoptaron el Pop, el Op, el Hard-Edge (filo duro) y el arte conceptual/no-objetual, en convivencia con el surrealismo, la nueva figuración y el expresionismo abstracto supérstite. Castrillón enmarca el periodo entre el gobierno de Belaúnde (1963) y el régimen militar de Velasco (1968-1975), atendiendo a la vida política, el desarrollo educativo, el crecimiento de las galerías y del mercado limeño. El eje conceptual es la figura del crítico Juan Acha, cuya defensa de una modernidad universalista contra el “provincianismo” indigenista y las “conscripciones” de la peruanidad, su teoría del arte como sistema de producción-distribución-consumo y sus conferencias de 1969 sobre mass media, estructuralismo y no-objetualismo articularon el ingreso de las vanguardias. Reconstruye la protesta del grupo Arte Nuevo (1966) frente al Festival Americano de Pintura y su muestra en la galería El ombligo de Adán, con Luis Arias Vera, Teresa Burga, Gloria Gómez Sánchez, Emilio Hernández Saavedra, Rafael Hastings y otros; traza el informalismo (Gómez Sánchez), los surrealismos (Quintanilla, Chávez, Tsuchiya, Revilla), la figuración (Bill Caro, Palao), el “pop achorado” de Ruiz Durand y el conceptualismo pionero de Burga y Hastings. Discute la polémica de 1975 por el Premio Nacional otorgado al retablista popular Joaquín López Antay, que planteó el reconocimiento del arte popular en la historia del arte peruano. La tesis, sugerida por el título “entre la agonía y la fiesta”, es la tensión de una modernidad rezagada y dependiente de importaciones estéticas que exigían ser asimiladas con recursos y nutrientes locales.</t>
         </is>
       </c>
     </row>
@@ -798,27 +798,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Del Valle - La fiesta del no-objetualismo. Polémicas sobre arte contemporáneo en América Latina.md</t>
+          <t>Castrillón - Reflexiones sobre el arte conceptual en Perú y sus proyecciones.md</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>1970-1981 (esp. Coloquio de Medellín, mayo 1981)</t>
+          <t>Años 60-70 en Perú (con antecedentes desde 1436 y del Dadá/Duchamp)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico, 2007</t>
+          <t>Ponencia de coloquio (arte no-objetual), 1981 (reed. c. 2007)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Augusto del Valle; Juan Acha; Mirko Lauer; Aracy Amaral; Mário Pedrosa; Néstor García Canclini; Rita Eder; Nelly Richard; Alfonso Castrillón; Álvaro Barrios; Marta Traba; Museo de Arte Moderno de Medellín</t>
+          <t>Alfonso Castrillón Vizcarra; Juan Acha; Teresa Burga; Rafael Hastings; Emilio Hernández; Joaquín López Antay; Fernando de Szyszlo; Jorge Romero Brest; Ruiz Durand; Grupo Espacio; Instituto de Arte Contemporáneo (IAC); Universidad Nacional Mayor de San Marcos</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Ensayo de Augusto del Valle (fechado en marzo de 2007) que toma como objeto el Primer Coloquio Latinoamericano sobre Arte No-Objetual y Arte Urbano (Medellín, mayo de 1981), dirigido por Juan Acha, para reconstruir el origen, vigencia y olvido de la categoría "no-objetualismo" y evaluar su potencial crítico. La tesis central lee ese coloquio como el pico de una deriva identitaria y latinoamericanista, situada entre la I Bienal Latinoamericana de São Paulo (1978) y la I Bienal de La Habana (1984), y determinada por el endeudamiento de la "década perdida" y la posterior recomposición neoliberal y multicultural que obliteró esos proyectos. Del Valle organiza el análisis contrastando a los ponentes que rechazaron la categoría desde la comunicación o la historia del arte (García Canclini, María Elena Ramos, Jorge Glusberg, Castrillón) con quienes la aceptaron mediante informes nacionales (Aracy Amaral en Brasil, Rita Eder en México, Álvaro Barrios en Colombia, Nelly Richard en Chile, Lauer y Castrillón en Perú). Marco conceptual: teoría social del arte, valor de uso/valor de cambio, aura benjaminiana y crítica de la modernización capitalista. Destaca la asociación entre no-objetualismo y acción corporal, el fenómeno mexicano de "los grupos", el retablo andino en Mirko Lauer como experimento social involuntario y la vanguardia peruana según Castrillón. Cierra dialogando con el conceptualismo global (Camnitzer, Mari Carmen Ramírez, Longoni, Cuauhtémoc Medina) y reivindica el no-objetualismo como archivo semántico capaz de recuperar autores y polémicas silenciadas frente a la homogeneización curatorial contemporánea.</t>
+          <t>Ponencia leída por Alfonso Castrillón en el Primer Coloquio Latinoamericano sobre Arte No-Objetual (Medellín, 1981) que discute la pertinencia de la categoría "no-objetualismo" y propone, en su lugar, una historia de la progresiva desaparición del objeto artístico. Castrillón rastrea la conciencia del concepto desde Alberti, Leonardo y Miguel Ángel, para argumentar que la objetualidad y sus atractivos sensibles prevalecieron durante siglos hasta que, hacia 1966, el Conceptual Art desplazó esa intención tradicional. Sostiene que no existe un no-objetual absoluto, pues toda manifestación se apoya en un soporte material; prefiere hablar de una crisis de la sensibilidad y del objeto-mercancía, gestada desde el impresionismo, el cubismo, el futurismo, Dadá, Duchamp y el minimalismo. El aporte central es su lectura del caso peruano: describe la vanguardia como fenómeno atípico y desfasado respecto de una industrialización incipiente (desde Odría), reconstruyendo hitos del pop, op y conceptual local (Luis Arias Vera, Gloria Gómez Sánchez, Teresa Burga, Ruiz Durand), la irradiación de Romero Brest y, sobre todo, la crítica activa de Juan Acha, cuyo entusiasmo por el "desarrollo" juzga estimulante pero sin eco material. Valora experiencias conceptuales de Emilio Hernández, el Autorretrato de Teresa Burga y las acciones de Rafael Hastings. Su tesis más provocadora considera la premiación de Joaquín López Antay (1975) como la mejor acción de arte conceptual peruana, por golpear desde dentro la ideología estética señorial. Concluye reivindicando el arte conceptual como crítica operativa, efímera y útil en ámbitos universitarios, y aboga por un arte de la vida frente a la mercancía.</t>
         </is>
       </c>
     </row>
@@ -830,27 +830,27 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Del Valle - Memoria sin territorio, territorio sin memoria.md</t>
+          <t>Conversatorio - Hay algo incomestible en la garganta - 2021-10-13 [Sala de Lectura].transcripcion.md</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>1997-1998 (I Bienal Iberoamericana de Lima; contexto 1980-1998)</t>
+          <t>1988-2002 (años 90)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Ensayo/artículo crítico, c. 1998 (Hueso Húmero 34)</t>
+          <t>Transcripción de conversatorio, 13-10-2021</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Augusto del Valle; Cristina Planas; Francisco Guerra García; Carlos Runcie Tanaka; Eduardo Tokeshi; Emilio Santisteban; Luz María Bedoya; Elena Tejada; Gustavo Buntinx; Élida Román; Jorge Villacorta; Centro de Artes Visuales (I Bienal Iberoamericana de Lima)</t>
+          <t>Miguel A. López; Elena Tejada-Herrera; Susana Torres; Cecilia (autora de La máquina de carne); Jorge Villacorta; galería Parafernalia; ICPNA; Natalia Iguíñiz; Gilda Mantilla; Elena Valera; Seminario de Historia Rural Andina; Sala de Lectura</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Ensayo crítico de Augusto del Valle sobre la participación peruana en la Primera Bienal Iberoamericana de Lima (organizada por el Centro de Artes Visuales, octubre-diciembre de 1997, bajo el lema "Nuevos conceptos de arte en Latinoamérica"). Su marco conceptual gira en torno a la noción de imaginario social "amoderno" y a la tensión entre memoria histórica y forma plástica, articulando el análisis en tres ejes: lo político como tema versus lo político como mentalidad; el refugio del esteticismo; y el laberinto del pluralismo. A través de estudios de caso, el autor argumenta que buena parte de la "generación del noventa" desplazó lo político hacia lo introspectivo y estetizante. Analiza La wuawua de Cristina Planas (imagen de Abimael Guzmán, censurada) y el Último partido de Guerra García como estéticas de la subjetividad que entran en cortocircuito con sus referentes populares; valora Tiempo detenido de Carlos Runcie Tanaka —ex rehén de la embajada de Japón— como transformación plástica de una testificación histórica hacia un arquetipo; critica el esteticismo de Vida y milagros del hombre invisible de Eduardo Tokeshi, cuyo virtuosismo obliteraría su discurso identitario; y examina la instalación de Emilio Santisteban, el Punto Ciego de Luz María Bedoya y la performance disruptiva de Elena Tejada en el Museo de Arte de Lima. Del Valle sostiene que en Perú no existe dialéctica entre institucionalidad y marginalidad, y que la escena oscila entre el "brillo de lo exótico" demandado por el mercado internacional y la "inestabilidad del exilio", proponiendo situar las obras respecto de sus contextos locales sin métodos comparativos descontextualizados.</t>
+          <t>Transcripción del conversatorio de cierre de la exposición "Hay algo incomestible en la garganta. Poéticas antipatriarcales y nueva escena en los años noventa" (curaduría de Miguel A. López, ICPNA, 2021), con las artistas Elena Tejada-Herrera, Susana Torres y Cecilia (autora de La máquina de carne). López enmarca la muestra entre 1988 y 2002 y en el contexto de la dictadura fujimorista, el neoliberalismo y la violencia política, proponiendo dos ejes: la emergencia de representaciones que desafían estructuras misóginas y la reconfiguración de los bordes de la escena artística. Las artistas comentan obras concretas: Tejada-Herrera describe performances como "Recuerdo" (1998), realizada en San Marcos tomada por el ejército en alusión a los desaparecidos de La Cantuta, y "La mujer yo-yo", que subvierte el imaginario del peruano doliente; Torres narra su tránsito del modelaje al autorretrato y a la serie de banderas exhibida en Parafernalia con Jorge Villacorta, y su descubrimiento del feminismo vía Flora Tristán; Cecilia explica el fotomatón interactivo "Máquina de carne" (2000-2001) como dispositivo sobre sexualidad, cuerpo y foto carnet, y su recorrido por distintos estratos sociales. El diálogo articula la noción de un "arte de urgencia" intuitivo y anterior al vocabulario feminista instalado hacia 2021, discute la relectura histórica que permite la muestra, la sororidad, la censura y la recontextualización de obras. Se mencionan trayectorias paralelas (Iguíñiz, Mantilla, Bedoya, Gandolfo, Rocío Rodrigo, Johanna Hamann) y la incorporación de artistas amazónicas (Elena Valera, Astrid Canayo) y del Seminario de Historia Rural Andina, ampliando el canon de la escena limeña noventera.</t>
         </is>
       </c>
     </row>
@@ -862,27 +862,27 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>E.P.S. Huayco - Arte al paso (1981) [librillo bilingüe español-alemán del video de 28 min, Edizioni Flaviana, Locarno].pdf</t>
+          <t>Del Valle - La fiesta del no-objetualismo. Polémicas sobre arte contemporáneo en América Latina.md</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>1979-1981</t>
+          <t>1970-1981 (esp. Coloquio de Medellín, mayo 1981)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Librillo/catálogo bilingüe de videoarte, 1981 (Edizioni Flaviana, Locarno)</t>
+          <t>Ensayo académico, 2007</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>E.P.S. Huayco; Francisco Mariotti; María Luy; Juan Javier Salazar; Herbert Rodríguez; Armando Williams; Rosario Noriega; Mirko Lauer; Manuel Lajo; Juan Acha; Edizioni Flaviana Locarno; UNMSM / Universidad de Lima</t>
+          <t>Augusto del Valle; Juan Acha; Mirko Lauer; Aracy Amaral; Mário Pedrosa; Néstor García Canclini; Rita Eder; Nelly Richard; Alfonso Castrillón; Álvaro Barrios; Marta Traba; Museo de Arte Moderno de Medellín</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Librillo bilingüe español-alemán, editado por Edizioni Flaviana (Locarno, 1981), que acompaña el video de 28 minutos "Arte al Paso" del colectivo peruano E.P.S. Huayco (Francisco Mariotti, María Luy, Rosario Noriega, Mariela Zevallos, Juan Javier Salazar, Herbert Rodríguez, Armando Williams). El proyecto se define como un intento de acercamiento y diálogo de un grupo de artistas plásticos con un público popular urbano, en contraposición al público "culto" que frecuenta galerías y controla los sistemas económicos, políticos y culturales del país. El video documenta las dificultades y logros de esa comunicación con la cultura popular e incluye una encuesta de preferencias estéticas realizada en diciembre de 1980 y enero de 1981 en dos plazas de Lima —el Parque Universitario y el Parque Central de Miraflores—, con apoyo del Programa de Historia del Arte de la UNMSM y del Programa de Ciencias de la Comunicación de la Universidad de Lima; sus resultados contrastan las preferencias por lo religioso, figurativo y abstracto (Taytacha, cabeza Chavín, tejido Huari, Cristo de Giotto, mujer que llora de Picasso, composición de Mondrian) según el origen social del público. El folleto reproduce el Manifiesto del Festival de Arte Total Contacta 79 (Barranco, julio de 1979), un texto de Manuel Lajo sobre la dependencia alimentaria y las transnacionales lácteas (Nestlé, Carnation, Leche Gloria) —trasfondo de la obra Sarita Colonia hecha con latas—, y citas de Federico Morais y Juan Acha. Destaca el comentario crítico de Mirko Lauer, que juzga la propuesta valiosa pero insuficientemente radical y asimilable por el establishment plástico limeño.</t>
+          <t>Ensayo de Augusto del Valle (fechado en marzo de 2007) que toma como objeto el Primer Coloquio Latinoamericano sobre Arte No-Objetual y Arte Urbano (Medellín, mayo de 1981), dirigido por Juan Acha, para reconstruir el origen, vigencia y olvido de la categoría "no-objetualismo" y evaluar su potencial crítico. La tesis central lee ese coloquio como el pico de una deriva identitaria y latinoamericanista, situada entre la I Bienal Latinoamericana de São Paulo (1978) y la I Bienal de La Habana (1984), y determinada por el endeudamiento de la "década perdida" y la posterior recomposición neoliberal y multicultural que obliteró esos proyectos. Del Valle organiza el análisis contrastando a los ponentes que rechazaron la categoría desde la comunicación o la historia del arte (García Canclini, María Elena Ramos, Jorge Glusberg, Castrillón) con quienes la aceptaron mediante informes nacionales (Aracy Amaral en Brasil, Rita Eder en México, Álvaro Barrios en Colombia, Nelly Richard en Chile, Lauer y Castrillón en Perú). Marco conceptual: teoría social del arte, valor de uso/valor de cambio, aura benjaminiana y crítica de la modernización capitalista. Destaca la asociación entre no-objetualismo y acción corporal, el fenómeno mexicano de "los grupos", el retablo andino en Mirko Lauer como experimento social involuntario y la vanguardia peruana según Castrillón. Cierra dialogando con el conceptualismo global (Camnitzer, Mari Carmen Ramírez, Longoni, Cuauhtémoc Medina) y reivindica el no-objetualismo como archivo semántico capaz de recuperar autores y polémicas silenciadas frente a la homogeneización curatorial contemporánea.</t>
         </is>
       </c>
     </row>
@@ -894,27 +894,27 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>EPS_HUAYCO_Buntinx_2005.txt</t>
+          <t>Del Valle - Memoria sin territorio, territorio sin memoria.md</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>1979-1981 (con amplio contexto desde ca. 1968-1978; publicado en 2005)</t>
+          <t>1997-1998 (I Bienal Iberoamericana de Lima; contexto 1980-1998)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Estudio histórico-crítico de historia del arte de Gustavo Buntinx (2005) sobre el colectivo E.P.S. Huayco; edición digital en OpenEdition Books («Combates por la historia», p. 12-16). La atribución al volumen E.P.S. Huayco. Documentos (MALI/IFEA, 2005) es deducida.</t>
+          <t>Ensayo/artículo crítico, c. 1998 (Hueso Húmero 34)</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; E.P.S. Huayco; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; María Luy; Charo Noriega; Mariela Zevallos; Armando Williams; Mirko Lauer; Juan Acha; Sarita Colonia; Contacta 79; SINAMOS; Sendero Luminoso; Micromuseo</t>
+          <t>Augusto del Valle; Cristina Planas; Francisco Guerra García; Carlos Runcie Tanaka; Eduardo Tokeshi; Emilio Santisteban; Luz María Bedoya; Elena Tejada; Gustavo Buntinx; Élida Román; Jorge Villacorta; Centro de Artes Visuales (I Bienal Iberoamericana de Lima)</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Estudio histórico-crítico extenso (unas 82.000 palabras) de Gustavo Buntinx sobre el colectivo E.P.S. Huayco (1979-1981), concebido como la reconstrucción documental de referencia del grupo y de su obra mayor, el mosaico de Sarita Colonia levantado con miles de latas de leche vacías sobre la Panamericana Sur. Escrito desde la proximidad personal del autor con los integrantes, reivindica una «descripción factual de los hechos» apoyada en crítica de fuentes, filología, hermenéutica y heurística, y se propone corregir la «acumulación impresionante de errores» de la bibliografía reciente: la datación equivocada de Sarita Colonia en 1981, la confusión de Contacta 79 con las elecciones a la Asamblea Constituyente de 1978, y las tergiversaciones de autorías, fechas y títulos. Organizado en secciones («Definiciones», «La utopía socialista», «El fin de la inocencia. La reforma frustrada», «Revolución en la revolución. El cisma», entre otras), traza la genealogía del colectivo desde la crisis del reformismo velasquista y el horizonte de la nueva izquierda, y narra Contacta, la muestra Arte al paso, el «pop achorado», las salchipapas gigantes y la disolución del grupo, en el marco del inicio de la violencia senderista. Reúne a Francisco Mariotti, Herbert Rodríguez, Juan Javier Salazar, María Luy, Charo Noriega, Mariela Zevallos y Armando Williams, y discute a Mirko Lauer y Juan Acha. Es el «estudio de 2005» de referencia sobre Huayco al que remiten otras fuentes del capítulo; emplea «culminación» y «cristalización» al caracterizar el lugar del grupo, y no usa la fórmula «arte crítico».</t>
+          <t>Ensayo crítico de Augusto del Valle sobre la participación peruana en la Primera Bienal Iberoamericana de Lima (organizada por el Centro de Artes Visuales, octubre-diciembre de 1997, bajo el lema "Nuevos conceptos de arte en Latinoamérica"). Su marco conceptual gira en torno a la noción de imaginario social "amoderno" y a la tensión entre memoria histórica y forma plástica, articulando el análisis en tres ejes: lo político como tema versus lo político como mentalidad; el refugio del esteticismo; y el laberinto del pluralismo. A través de estudios de caso, el autor argumenta que buena parte de la "generación del noventa" desplazó lo político hacia lo introspectivo y estetizante. Analiza La wuawua de Cristina Planas (imagen de Abimael Guzmán, censurada) y el Último partido de Guerra García como estéticas de la subjetividad que entran en cortocircuito con sus referentes populares; valora Tiempo detenido de Carlos Runcie Tanaka —ex rehén de la embajada de Japón— como transformación plástica de una testificación histórica hacia un arquetipo; critica el esteticismo de Vida y milagros del hombre invisible de Eduardo Tokeshi, cuyo virtuosismo obliteraría su discurso identitario; y examina la instalación de Emilio Santisteban, el Punto Ciego de Luz María Bedoya y la performance disruptiva de Elena Tejada en el Museo de Arte de Lima. Del Valle sostiene que en Perú no existe dialéctica entre institucionalidad y marginalidad, y que la escena oscila entre el "brillo de lo exótico" demandado por el mercado internacional y la "inestabilidad del exilio", proponiendo situar las obras respecto de sus contextos locales sin métodos comparativos descontextualizados.</t>
         </is>
       </c>
     </row>
@@ -926,27 +926,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>El Pabellón ha caído - Buntinx.md</t>
+          <t>E.P.S. Huayco - Arte al paso (1981) [librillo bilingüe español-alemán del video de 28 min, Edizioni Flaviana, Locarno].pdf</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>1980-1992 (violencia política; obra pictórica de 1992; masacre de El Frontón, 1986)</t>
+          <t>1979-1981</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Artículo de crítica de arte en prensa, 14-06-1992</t>
+          <t>Librillo/catálogo bilingüe de videoarte, 1981 (Edizioni Flaviana, Locarno)</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Elio Martuccelli; Juan Javier Salazar; Herbert Rodríguez; Jaime Higa; grupo Huayco; los NN; los Bestias; José Tola; Piero Quijano; Anselmo Carrera; Roy Lichtenstein; Diario La República (suplemento Culturas)</t>
+          <t>E.P.S. Huayco; Francisco Mariotti; María Luy; Juan Javier Salazar; Herbert Rodríguez; Armando Williams; Rosario Noriega; Mirko Lauer; Manuel Lajo; Juan Acha; Edizioni Flaviana Locarno; UNMSM / Universidad de Lima</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Artículo de Gustavo Buntinx publicado en el suplemento "Culturas" del diario La República el 14 de junio de 1992, concebido como crónica reflexiva y no como mero juicio de valor. El texto lee la plástica peruana como escenario privilegiado para registrar la subjetividad de un "pequeño-burgués-ilustrado" durante los doce años de violencia (1980-1992), esa frágil "República de Weimar" peruana en su ocaso. El objeto de estudio central es la exposición "Se vende" de Elio Martuccelli, arquitecto de vocación teórica situado en los márgenes entre los grupos Bestias y NN y vinculado a la plástica alternativa que arranca de Huayco. Buntinx se concentra en un cuadríptico donde Martuccelli reproduce páginas de un cómic editado por la Marina de Guerra sobre Miguel Grau (centenario de 1979), cuyo último recuadro reza "¡El pabellón ha caído!". El marco conceptual articula apropiación, cita y "copia de la copia": Martuccelli mira a Lichtenstein a través del Pop achorado de Juan Javier Salazar (su lámina de presidentes, 1980), reivindicando la brocha gorda artesanal frente al refinamiento tecnológico del pop norteamericano como signo de una modernidad fallida y periférica. Mediante mínimas intervenciones -reencuadres, ocultamiento de la franja roja de la bandera, transformación de "fuego" en "ego"- la obra hace hablar las contradicciones reprimidas de la comunicación masiva y evoca el aniquilamiento de los presos de El Frontón y el crimen de María Elena Moyano. El aporte es una crítica que politiza lo íntimo: el pabellón caído figura el quiebre entre la intelectualidad joven y los mitos republicanos, irreversiblemente cancelados por defensores e impugnadores por igual.</t>
+          <t>Librillo bilingüe español-alemán, editado por Edizioni Flaviana (Locarno, 1981), que acompaña el video de 28 minutos "Arte al Paso" del colectivo peruano E.P.S. Huayco (Francisco Mariotti, María Luy, Rosario Noriega, Mariela Zevallos, Juan Javier Salazar, Herbert Rodríguez, Armando Williams). El proyecto se define como un intento de acercamiento y diálogo de un grupo de artistas plásticos con un público popular urbano, en contraposición al público "culto" que frecuenta galerías y controla los sistemas económicos, políticos y culturales del país. El video documenta las dificultades y logros de esa comunicación con la cultura popular e incluye una encuesta de preferencias estéticas realizada en diciembre de 1980 y enero de 1981 en dos plazas de Lima —el Parque Universitario y el Parque Central de Miraflores—, con apoyo del Programa de Historia del Arte de la UNMSM y del Programa de Ciencias de la Comunicación de la Universidad de Lima; sus resultados contrastan las preferencias por lo religioso, figurativo y abstracto (Taytacha, cabeza Chavín, tejido Huari, Cristo de Giotto, mujer que llora de Picasso, composición de Mondrian) según el origen social del público. El folleto reproduce el Manifiesto del Festival de Arte Total Contacta 79 (Barranco, julio de 1979), un texto de Manuel Lajo sobre la dependencia alimentaria y las transnacionales lácteas (Nestlé, Carnation, Leche Gloria) —trasfondo de la obra Sarita Colonia hecha con latas—, y citas de Federico Morais y Juan Acha. Destaca el comentario crítico de Mirko Lauer, que juzga la propuesta valiosa pero insuficientemente radical y asimilable por el establishment plástico limeño.</t>
         </is>
       </c>
     </row>
@@ -958,27 +958,27 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Elera, Gonzales y Silva - Lunes de crítica 2017-2018. Convulsión y autoorganización.md</t>
+          <t>EP12_El_hombre_de_Artus__transcripcion_refinada.md</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2014-2018 (programa Lunes de Crítica, oct. 2017 - mar. 2018)</t>
+          <t>s. f. (transcripción); menciones de 1996, 2007, 2013 y hasta el presente reciente (2025)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Capítulo/ensayo en publicación, c. 2019</t>
+          <t>Transcripción de podcast ('Desde la Azotea', EP12); conversación reciente (posterior a 2023 por sus menciones)</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Andrea Elera; Gustavo Gonzales; Raúl Silva; Por una Comunidad de las Artes Visuales; Museo de Arte de San Marcos (MASM); Augusto del Valle; Juan Javier Salazar; Pabellón Peruano de la Bienal de Venecia; Proyecto Fugaz / Monumental Callao; Lugar de la Memoria (LUM); Sonia Cunliffe; PUCP-ENSABAP</t>
+          <t>Alberto Casari, Carlos Marzano (coleccionista/gestor de ARTUS), María Alejandra Massa; ARTUS; ICPNA; MALI (comité de adquisiciones; Sharon Lerner, Caroline Briceño); Delfina Foundation, Gasworks, WIELS, Pivô (São Paulo); MAC Barranco; galerías Fórum, Revólver, 80m2 Livia Benavides</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Texto reflexivo de Andrea Elera, Gustavo Gonzales y Raúl Silva, integrantes del colectivo "Por una Comunidad de las Artes Visuales", que balancea la experiencia del programa "Lunes de Crítica" (quince mesas realizadas los lunes entre octubre de 2017 y marzo de 2018 en el Museo de Arte de San Marcos, MASM). El argumento central sostiene que la autoorganización y la subjetivación crítica de los trabajadores de las artes son respuestas necesarias frente a la informalidad laboral, la fragmentación y la captura privada del sistema artístico limeño. Los autores enumeran los "exabruptos" que entre 2014 y 2017 detonaron la formación del colectivo: el borrado de murales del Centro de Lima por la gestión de Castañeda Lossio, el plagio en el texto curatorial de "Pasaporte para un Artista", los vínculos de lavado de activos del proyecto Fugaz y la gentrificación de Monumental Callao, y sobre todo la polémica gestión y curaduría del Pabellón Peruano en la 57 Bienal de Venecia (2017), con la presentación póstuma de la obra de Juan Javier Salazar, que actuó como detonante organizativo. Describen la estructura pedagógica del programa en cinco unidades (sector público-privado, gestión cultural y ciudadanía, espacios en disputa, educación artística e investigación/crítica), reconociendo antecedentes en los "Lunes de Crítica" que Augusto del Valle dirigió en el MASM (2002-2004). El balance admite el desgaste logístico y el carácter autoformativo del proceso —más autoaprendizaje que aporte comunitario—, ejemplificado en la tensa mesa sobre Fugaz con Sonia Cunliffe, pero reivindica la articulación colectiva, la crítica devenida propuesta y la voz común como metas de largo aliento, asumiendo su sesgo limeño y centralista.</t>
+          <t>Transcripción refinada del episodio 12 del podcast 'Desde la Azotea', conducido por Alberto Casari y María Alejandra Massa, con Carlos Marzano como invitado. Marzano se presenta como coleccionista, productor y gestor del proyecto ARTUS, asociación de cuatro fundadores que financia residencias internacionales para artistas peruanos jóvenes (más de 17 enviados a Gasworks, Delfina, WIELS, Pivô São Paulo, entre otros). Expone su concepción del coleccionismo —'la acumulación es parte del coleccionista, pero el coleccionismo es mucho más que acumular'; el poseedor tiene 'el deber moral de que esa obra circule'— y su modelo de residencia como 'ecosistemas de pensamiento'. El documento aporta información primaria sobre la institucionalidad artística limeña: la centralidad del MALI, el rol del MAC Barranco, el estado del sistema de galerías ('un negocio de sobrevivencia', del que 'solo queda Fórum' entre las icónicas, más la nueva generación Revólver, 80m2 Livia Benavides). Contiene un dato relevante para el corpus: Marzano declara haber sido 'presidente del comité de adquisiciones' del MALI durante dos años, con Sharon Lerner en la dirección y dos curadores internacionales invitados, grupo que 'continúa armando la colección contemporánea'. La transcripción incluye marcas de revisión y notas de la propia transcripción sobre datos a verificar (fechas incompatibles, nombres con posible corrupción de reconocimiento automático de voz, señalados con '[corr.]', '[¿?]' o '[nota:]'). Fuente oral primaria sobre coleccionismo, mecenazgo privado y la relación entre iniciativa privada e institución en el circuito del arte contemporáneo peruano.</t>
         </is>
       </c>
     </row>
@@ -990,27 +990,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Flores Hora, David - 2026-04-16.transcripcion.md</t>
+          <t>EPS_HUAYCO_Buntinx_2005.txt</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>2000-2020 (con referencias a los años 80)</t>
+          <t>1979-1981 (con amplio contexto desde ca. 1968-1978; publicado en 2005)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Entrevista, 16-04-2026</t>
+          <t>Estudio histórico-crítico de historia del arte de Gustavo Buntinx (2005) sobre el colectivo E.P.S. Huayco; edición digital en OpenEdition Books («Combates por la historia», p. 12-16). La atribución al volumen E.P.S. Huayco. Documentos (MALI/IFEA, 2005) es deducida.</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>David Flores Hora; Carlos Zevallos (entrevistador); Centro Cultural de España; Ricardo Ramón; Sala Luis Miró Quesada Garland; Luis Lama; Jorge Villacorta; José Carlos Mariátegui; Christian Bendayán; MALI; Natalia Majluf; Miguel López; ICPNA; Ministerio de Cultura (ARCOmadrid); LUM</t>
+          <t>Gustavo Buntinx; E.P.S. Huayco; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; María Luy; Charo Noriega; Mariela Zevallos; Armando Williams; Mirko Lauer; Juan Acha; Sarita Colonia; Contacta 79; SINAMOS; Sendero Luminoso; Micromuseo</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Testimonio de David Flores Hora, historiador del arte sanmarquino y gestor cultural, recogido por Carlos Zevallos en el marco de una tesis doctoral sobre el «arte crítico» y su institucionalización en Lima. La entrevista reconstruye una trayectoria que enlaza la formación en San Marcos durante el ocaso del fujimorato (ingreso en 2000), la coordinación de artes visuales del Centro Cultural de España (2007-2010), el paso por la Sala Luis Miró Quesada Garland junto a Luis Lama, el ICPNA, el Ministerio de Cultura (coordinación de la presencia peruana en ARCOmadrid) y el LUM. Flores Hora sostiene una tesis periodizadora: la primera década de 2000 fue un momento de efervescencia donde «ser contemporáneo» equivalía a asumir una posición política y a intervenir el espacio expositivo, alimentada por la resaca de la Bienal de Lima y las redes latinoamericanas; a partir de 2011 sobreviene la institucionalización (viraje del MALI hacia lo contemporáneo hacia 2008), sucedida por lo que denomina «dictaduras» consecutivas de la crítica, la curaduría y, finalmente, el coleccionismo. El relato contrapone la libertad de un espacio de extranjería (España) a la precariedad estatal, y lamenta la pérdida del «potencial revolucionario» ante la economización del campo y el ascenso del artista global y del arte amazónico (Bendayán) como opción menos confrontacional. Menciona el proyecto de archivo CEDAP, portafolios con Natalia Majluf, Emilio Tarazona y Miguel López, y aboga por archivos vivos. Su posición combina nostalgia militante y una conciencia ética de la sobrevivencia profesional en un medio desfinanciado.</t>
+          <t>Estudio histórico-crítico extenso (unas 82.000 palabras) de Gustavo Buntinx sobre el colectivo E.P.S. Huayco (1979-1981), concebido como la reconstrucción documental de referencia del grupo y de su obra mayor, el mosaico de Sarita Colonia levantado con miles de latas de leche vacías sobre la Panamericana Sur. Escrito desde la proximidad personal del autor con los integrantes, reivindica una «descripción factual de los hechos» apoyada en crítica de fuentes, filología, hermenéutica y heurística, y se propone corregir la «acumulación impresionante de errores» de la bibliografía reciente: la datación equivocada de Sarita Colonia en 1981, la confusión de Contacta 79 con las elecciones a la Asamblea Constituyente de 1978, y las tergiversaciones de autorías, fechas y títulos. Organizado en secciones («Definiciones», «La utopía socialista», «El fin de la inocencia. La reforma frustrada», «Revolución en la revolución. El cisma», entre otras), traza la genealogía del colectivo desde la crisis del reformismo velasquista y el horizonte de la nueva izquierda, y narra Contacta, la muestra Arte al paso, el «pop achorado», las salchipapas gigantes y la disolución del grupo, en el marco del inicio de la violencia senderista. Reúne a Francisco Mariotti, Herbert Rodríguez, Juan Javier Salazar, María Luy, Charo Noriega, Mariela Zevallos y Armando Williams, y discute a Mirko Lauer y Juan Acha. Es el «estudio de 2005» de referencia sobre Huayco al que remiten otras fuentes del capítulo; emplea «culminación» y «cristalización» al caracterizar el lugar del grupo, y no usa la fórmula «arte crítico».</t>
         </is>
       </c>
     </row>
@@ -1022,27 +1022,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Germaná, Gabriela - 20 de noviembre.transcripcion.md</t>
+          <t>El Pabellón ha caído - Buntinx.md</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Años 80 y 90 y 2013-2025</t>
+          <t>1980-1992 (violencia política; obra pictórica de 1992; masacre de El Frontón, 1986)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Entrevista, 20 de noviembre (año no precisado)</t>
+          <t>Artículo de crítica de arte en prensa, 14-06-1992</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Gabriela Germaná; Carlos Zevallos (entrevistador); Venuca Evanán; Violeta Quispe; tablas de Sarhua; MAC; MALI; Natalia Majluf; Miguel López; Pedro Pablo Alayza; ICPNA/IMNA; galería Ginsberg; Baró; Luis Lama; Claire Bishop</t>
+          <t>Gustavo Buntinx; Elio Martuccelli; Juan Javier Salazar; Herbert Rodríguez; Jaime Higa; grupo Huayco; los NN; los Bestias; José Tola; Piero Quijano; Anselmo Carrera; Roy Lichtenstein; Diario La República (suplemento Culturas)</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Entrevista a la historiadora del arte y curadora Gabriela Germ&lt;200b&gt;aná, especialista en artes populares y tablas de Sarhua, conducida por Carlos Zevallos para tensionar su hipótesis del «mandato crítico». Germaná matiza la noción de mandato, pero reconoce que la institucionalidad contemporánea hoy «da la bienvenida» e incorpora de inmediato discursos críticos —género, indigenidad, decolonialidad— que en los años ochenta permanecían marginales y solo fueron reconocidos a posteriori. El argumento articula tres ejes: la periodización del arte político peruano (los colectivos de los ochenta como indispensables para entender la década, frente al arte pro-gubernamental del velasquismo); su propia práctica curatorial de reivindicación de sujetos marginados (paridad de género, artistas regionales) en jurados de concursos como el del ICPNA/IMNA, el MUSE y Cultura, donde persisten tensiones generacionales entre «calidad estética» y postura política; y el caso de Venuca Evanán y Violeta Quispe, cuyo giro crítico —género, erotismo, memoria, retablos por la memoria— fue la condición que les abrió las puertas del arte contemporáneo, diferenciándolas del campo costumbrista del arte popular (series Piras Causa y Éxodo de los noventa, ingreso al MALI). Germaná problematiza el «extractivismo» de galerías internacionales (Baró, Ginsberg) que demandan producción sin diálogo, la fragilidad institucional local (MAC, MALI, gestión de Pedro Pablo Alayza), la sospecha ante el arte amazónico como inversión no confrontacional del coleccionismo, y el contraste con una historia del arte estadounidense más atravesada por raza, género y clase que la conservadora academia peruana. Reflexiona, además, sobre los límites del juicio crítico ante la producción indígena.</t>
+          <t>Artículo de Gustavo Buntinx publicado en el suplemento "Culturas" del diario La República el 14 de junio de 1992, concebido como crónica reflexiva y no como mero juicio de valor. El texto lee la plástica peruana como escenario privilegiado para registrar la subjetividad de un "pequeño-burgués-ilustrado" durante los doce años de violencia (1980-1992), esa frágil "República de Weimar" peruana en su ocaso. El objeto de estudio central es la exposición "Se vende" de Elio Martuccelli, arquitecto de vocación teórica situado en los márgenes entre los grupos Bestias y NN y vinculado a la plástica alternativa que arranca de Huayco. Buntinx se concentra en un cuadríptico donde Martuccelli reproduce páginas de un cómic editado por la Marina de Guerra sobre Miguel Grau (centenario de 1979), cuyo último recuadro reza "¡El pabellón ha caído!". El marco conceptual articula apropiación, cita y "copia de la copia": Martuccelli mira a Lichtenstein a través del Pop achorado de Juan Javier Salazar (su lámina de presidentes, 1980), reivindicando la brocha gorda artesanal frente al refinamiento tecnológico del pop norteamericano como signo de una modernidad fallida y periférica. Mediante mínimas intervenciones -reencuadres, ocultamiento de la franja roja de la bandera, transformación de "fuego" en "ego"- la obra hace hablar las contradicciones reprimidas de la comunicación masiva y evoca el aniquilamiento de los presos de El Frontón y el crimen de María Elena Moyano. El aporte es una crítica que politiza lo íntimo: el pabellón caído figura el quiebre entre la intelectualidad joven y los mitos republicanos, irreversiblemente cancelados por defensores e impugnadores por igual.</t>
         </is>
       </c>
     </row>
@@ -1054,27 +1054,27 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Hernández Calvo, Max - 7jul2025.transcripcion.md</t>
+          <t>Elera, Gonzales y Silva - Lunes de crítica 2017-2018. Convulsión y autoorganización.md</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>1997-2015 (con referencias a los años 70)</t>
+          <t>2014-2018 (programa Lunes de Crítica, oct. 2017 - mar. 2018)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Entrevista, 07-07-2025</t>
+          <t>Capítulo/ensayo en publicación, c. 2019</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Max Hernández Calvo; Carlos Zevallos (entrevistador); Miguel López; Emilio Tarazona; Juan Peralta; Bienales de Lima; Teresa Burga; MALI; Bard College; ICPNA/IMNA; Juan Carlos Verme; Carlos Marsano; Eduardo Hochschild; Alfonso García Miró</t>
+          <t>Andrea Elera; Gustavo Gonzales; Raúl Silva; Por una Comunidad de las Artes Visuales; Museo de Arte de San Marcos (MASM); Augusto del Valle; Juan Javier Salazar; Pabellón Peruano de la Bienal de Venecia; Proyecto Fugaz / Monumental Callao; Lugar de la Memoria (LUM); Sonia Cunliffe; PUCP-ENSABAP</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Conversación con el crítico y curador Max Hernández Calvo, sostenida con Carlos Zevallos en julio de 2025, centrada en la genealogía del «mandato crítico» y de la «lógica de proyecto» en el arte contemporáneo peruano. Hernández Calvo homologa el arte crítico con la producción de discurso y argumenta que los artistas jóvenes no perciben un mandato porque han sido formados dentro de un sistema que exige conceptualización previa, statement y portafolio; quienes sí lo leen como imposición externa suelen carecer de discurso, malinterpretándolo en clave esencialista o conspirativa. Reconstruye hitos institucionales: las Bienales de Lima de fines de los noventa (con Juan Peralta) que impulsaron la postulación mediante proyectos de instalación; su propia experiencia en la Bienal Nacional (1998) y en el MFA de baja residencia de Bard College (2005-2007), cuya estructura de crítica grupal evidenciaba la centralidad del discurso. Sitúa entre 2010 y 2015 la consolidación del mandato, ligada al viraje del MALI hacia lo contemporáneo, la aparición de ferias (Lima Foto, ArtLima), galerías nuevas (Revólver) y el redescubrimiento de Teresa Burga y del conceptualismo de los sesenta-setenta por Miguel López y Emilio Tarazona. Analiza los concursos (IMNA desde 2018, Pasaporte para un Artista, Artus) como síntoma del cambio, y la formación de coleccionistas (CAAC, 2006; Verme, Marsano, Hochschild, García Miró) entrenados en circuitos internacionales orientados al discurso. Cierra con una tesis sobre el extractivismo: la escena local colapsa tras las crisis políticas de 2016-2021 y la pandemia, y el artista deviene materia prima exportable, sostenido económicamente por galerías y compradores extranjeros.</t>
+          <t>Texto reflexivo de Andrea Elera, Gustavo Gonzales y Raúl Silva, integrantes del colectivo "Por una Comunidad de las Artes Visuales", que balancea la experiencia del programa "Lunes de Crítica" (quince mesas realizadas los lunes entre octubre de 2017 y marzo de 2018 en el Museo de Arte de San Marcos, MASM). El argumento central sostiene que la autoorganización y la subjetivación crítica de los trabajadores de las artes son respuestas necesarias frente a la informalidad laboral, la fragmentación y la captura privada del sistema artístico limeño. Los autores enumeran los "exabruptos" que entre 2014 y 2017 detonaron la formación del colectivo: el borrado de murales del Centro de Lima por la gestión de Castañeda Lossio, el plagio en el texto curatorial de "Pasaporte para un Artista", los vínculos de lavado de activos del proyecto Fugaz y la gentrificación de Monumental Callao, y sobre todo la polémica gestión y curaduría del Pabellón Peruano en la 57 Bienal de Venecia (2017), con la presentación póstuma de la obra de Juan Javier Salazar, que actuó como detonante organizativo. Describen la estructura pedagógica del programa en cinco unidades (sector público-privado, gestión cultural y ciudadanía, espacios en disputa, educación artística e investigación/crítica), reconociendo antecedentes en los "Lunes de Crítica" que Augusto del Valle dirigió en el MASM (2002-2004). El balance admite el desgaste logístico y el carácter autoformativo del proceso —más autoaprendizaje que aporte comunitario—, ejemplificado en la tensa mesa sobre Fugaz con Sonia Cunliffe, pero reivindica la articulación colectiva, la crítica devenida propuesta y la voz común como metas de largo aliento, asumiendo su sesgo limeño y centralista.</t>
         </is>
       </c>
     </row>
@@ -1086,27 +1086,27 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Lerner, Sharon - sin fecha.transcripcion.md</t>
+          <t>Entrevista - Flores Hora, David - 2026-04-16.transcripcion.md</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>2007-2025 (historia de la colección del MALI)</t>
+          <t>2000-2020 (con referencias a los años 80)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Entrevista, s/f (transcripción 2026)</t>
+          <t>Entrevista, 16-04-2026</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Carlos Zevallos (entrevistador); MALI; Natalia Majluf; Tatiana Cuevas; Jorge Villacorta; Rodrigo Quijano; Miguel López; Julieta González; Florencia Portocarrero; Goethe Institut; Ricardo Kusunoki</t>
+          <t>David Flores Hora; Carlos Zevallos (entrevistador); Centro Cultural de España; Ricardo Ramón; Sala Luis Miró Quesada Garland; Luis Lama; Jorge Villacorta; José Carlos Mariátegui; Christian Bendayán; MALI; Natalia Majluf; Miguel López; ICPNA; Ministerio de Cultura (ARCOmadrid); LUM</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Entrevista a Sharon Lerner, curadora de arte contemporáneo y directora del MALI, realizada por Carlos Zevallos (transcripción de 2026). Lerner sostiene que el museo no maneja una definición taxativa de «arte contemporáneo»: se trata de un corte histórico en permanente redefinición, discutido cíclicamente con el comité académico, los asesores rotativos del Comité de Adquisiciones de Arte Contemporáneo y encuentros especializados. Reconstruye dos momentos de revisión: el volumen editado con fondo Sura (2013), heredado de Tatiana Cuevas, con ensayos de asesores (Villacorta, Quijano, Miguel López) y una conversación editada por Villacorta que expone tensiones y «discontinuidades»; y el encuentro de 2015 (con apoyo del Goethe Institut y a instancias de Julieta González) para la creación de un fondo amazónico, que reconocía institucionalmente una escena preexistente. Frente a la hipótesis del «mandato crítico», Lerner precisa que la criticidad es parte constitutiva de la práctica contemporánea, pero no un requisito excluyente ni un factor disuasivo: el museo posee obra crítica con la propia institución, y los criterios de adquisición (votación, pertinencia discursiva, conservación, precio) son múltiples. Distingue entre obras que «encarnan» (embody) discurso y aquellas meramente «formulaicas» que exhiben etiquetas. Subraya la ventaja comparativa del MALI como museo panorámico —que cruza lo precolombino, textil, popular y contemporáneo— y su rol de facto como único coleccionista sostenido ante la ausencia de otras instituciones. Explica que se expone solo por invitación curatorial, atendiendo vacíos (presencia femenina, perspectivas queer señaladas por Miguel López), y anuncia un futuro concurso de intervenciones y la proyectada expansión hacia salas del siglo XXI.</t>
+          <t>Testimonio de David Flores Hora, historiador del arte sanmarquino y gestor cultural, recogido por Carlos Zevallos en el marco de una tesis doctoral sobre el «arte crítico» y su institucionalización en Lima. La entrevista reconstruye una trayectoria que enlaza la formación en San Marcos durante el ocaso del fujimorato (ingreso en 2000), la coordinación de artes visuales del Centro Cultural de España (2007-2010), el paso por la Sala Luis Miró Quesada Garland junto a Luis Lama, el ICPNA, el Ministerio de Cultura (coordinación de la presencia peruana en ARCOmadrid) y el LUM. Flores Hora sostiene una tesis periodizadora: la primera década de 2000 fue un momento de efervescencia donde «ser contemporáneo» equivalía a asumir una posición política y a intervenir el espacio expositivo, alimentada por la resaca de la Bienal de Lima y las redes latinoamericanas; a partir de 2011 sobreviene la institucionalización (viraje del MALI hacia lo contemporáneo hacia 2008), sucedida por lo que denomina «dictaduras» consecutivas de la crítica, la curaduría y, finalmente, el coleccionismo. El relato contrapone la libertad de un espacio de extranjería (España) a la precariedad estatal, y lamenta la pérdida del «potencial revolucionario» ante la economización del campo y el ascenso del artista global y del arte amazónico (Bendayán) como opción menos confrontacional. Menciona el proyecto de archivo CEDAP, portafolios con Natalia Majluf, Emilio Tarazona y Miguel López, y aboga por archivos vivos. Su posición combina nostalgia militante y una conciencia ética de la sobrevivencia profesional en un medio desfinanciado.</t>
         </is>
       </c>
     </row>
@@ -1118,27 +1118,27 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Rebaza Torres, Alberto - 2023-10-12 (editada).docx</t>
+          <t>Entrevista - Germaná, Gabriela - 20 de noviembre.transcripcion.md</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 90 - 2023</t>
+          <t>Años 80 y 90 y 2013-2025</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Entrevista, 12-10-2023 (editada)</t>
+          <t>Entrevista, 20 de noviembre (año no precisado)</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Alberto Rebaza Torres; Carlos Zevallos Trigoso (entrevistador); MALI; CAAC; Ginette Fernández; Residencia de Al Lado; Bienal de Venecia; Museo Reina Sofía; Guggenheim; Eduardo Hochschild; Juan Carlos Verme; Carlos Marsano; ICPNA; Sandra Gamarra</t>
+          <t>Gabriela Germaná; Carlos Zevallos (entrevistador); Venuca Evanán; Violeta Quispe; tablas de Sarhua; MAC; MALI; Natalia Majluf; Miguel López; Pedro Pablo Alayza; ICPNA/IMNA; galería Ginsberg; Baró; Luis Lama; Claire Bishop</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Entrevista editada a Alberto Rebaza Torres —abogado, coleccionista y presidente del consejo directivo del MALI, además de expresidente del Comité de Adquisiciones de Arte Contemporáneo—, conducida por Carlos Zevallos Trigoso en octubre de 2023. Rebaza narra el origen de su coleccionismo a fines de los noventa, orientado inicial y deliberadamente al arte peruano contemporáneo y luego extendido a lo latinoamericano, bajo la convicción de una «misión»: que el coleccionismo local funcione como primera plataforma de desarrollo para los artistas. Ubica en 2006 la formación del CAAC como factor de cohesión de un grupo de coleccionistas peruanos que ganó visibilidad en ferias regionales e internacionales (ArteBA, ARTBO, Zona Maco, Art Basel). El testimonio articula una teoría del coleccionismo como «proselitismo del arte» que, con el tiempo, debilita la sensación de propiedad y migra hacia la filantropía y el fortalecimiento institucional, ante la ausencia del Estado. Distingue el potencial «colectivo» del coleccionista frente al potencial «de a uno» del galerista, y enfatiza la complementariedad de roles (galerías, ferias, curadores, residencias) en una carrera artística sin hitos claros. Reivindica su Residencia de Al Lado (con Ginette Fernández) y menciona a otros agentes (Hochschild-MAC, Verme-MALI, Marsano-ARTUS, Mulder, Barreda). Sobre su criterio personal, prioriza la tríada contenido, inteligencia y estética, y diferencia expresamente su línea de coleccionismo de la línea curatorial del MALI —más volcada a violencia, territorio, género e historia, próxima al Reina Sofía—. El documento es fuente clave para analizar la perspectiva del coleccionismo y la filantropía en la institucionalización del arte contemporáneo peruano.</t>
+          <t>Entrevista a la historiadora del arte y curadora Gabriela Germ&lt;200b&gt;aná, especialista en artes populares y tablas de Sarhua, conducida por Carlos Zevallos para tensionar su hipótesis del «mandato crítico». Germaná matiza la noción de mandato, pero reconoce que la institucionalidad contemporánea hoy «da la bienvenida» e incorpora de inmediato discursos críticos —género, indigenidad, decolonialidad— que en los años ochenta permanecían marginales y solo fueron reconocidos a posteriori. El argumento articula tres ejes: la periodización del arte político peruano (los colectivos de los ochenta como indispensables para entender la década, frente al arte pro-gubernamental del velasquismo); su propia práctica curatorial de reivindicación de sujetos marginados (paridad de género, artistas regionales) en jurados de concursos como el del ICPNA/IMNA, el MUSE y Cultura, donde persisten tensiones generacionales entre «calidad estética» y postura política; y el caso de Venuca Evanán y Violeta Quispe, cuyo giro crítico —género, erotismo, memoria, retablos por la memoria— fue la condición que les abrió las puertas del arte contemporáneo, diferenciándolas del campo costumbrista del arte popular (series Piras Causa y Éxodo de los noventa, ingreso al MALI). Germaná problematiza el «extractivismo» de galerías internacionales (Baró, Ginsberg) que demandan producción sin diálogo, la fragilidad institucional local (MAC, MALI, gestión de Pedro Pablo Alayza), la sospecha ante el arte amazónico como inversión no confrontacional del coleccionismo, y el contraste con una historia del arte estadounidense más atravesada por raza, género y clase que la conservadora academia peruana. Reflexiona, además, sobre los límites del juicio crítico ante la producción indígena.</t>
         </is>
       </c>
     </row>
@@ -1150,27 +1150,27 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Tokeshi, Eduardo - sin fecha.transcripcion.md</t>
+          <t>Entrevista - Hernández Calvo, Max - 7jul2025.transcripcion.md</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>1980-2002</t>
+          <t>1997-2015 (con referencias a los años 70)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Entrevista, s/f</t>
+          <t>Entrevista, 07-07-2025</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Eduardo Tokeshi; Carlos Zevallos (entrevistador); PUCP; Gustavo Buntinx; Luis Lama; E.P.S. Huayco; Herbert Rodríguez; Bienal de Lima; Emilio Rodríguez Larraín; Jorge Eduardo Eielson; Luis Camnitzer; Óscar Muñoz</t>
+          <t>Max Hernández Calvo; Carlos Zevallos (entrevistador); Miguel López; Emilio Tarazona; Juan Peralta; Bienales de Lima; Teresa Burga; MALI; Bard College; ICPNA/IMNA; Juan Carlos Verme; Carlos Marsano; Eduardo Hochschild; Alfonso García Miró</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Entrevista al artista Eduardo Tokeshi (n. 1960), conducida por Carlos Zevallos, que reconstruye su formación y la génesis de su obra más reconocida en el contexto de la violencia política peruana. Tokeshi relata su tránsito de la arquitectura a la especialidad de pintura en la PUCP hacia 1983, dentro de la clásica división entre la Católica (abstracción) y Bellas Artes (figuración), y su desmarque del canon al incorporar recortes periodísticos, objetos y materiales no pictóricos. Sitúa en 1985 la primera «Bandera» —cosida, rellena, tensada—, realizada por pulsión antes que como gesto deliberadamente contemporáneo, que inaugura una serie sostenida hasta 2001-2002 como sublimación de la violencia, el duelo y la reconstrucción de la nación. El testimonio historiza el surgimiento de lo contemporáneo local: la muestra «Algo va a pasar» (1987) organizada por Gustavo Buntinx, la Bienal de Trujillo (1987), las Bienales de Lima de los noventa y la labor de Luis Lama trayendo a Camnitzer y Óscar Muñoz. Analiza la profesionalización del campo en los noventa (idea de «proyecto», statements, portafolios, cambios de currícula), el desfase o «refracción» respecto de los centros internacionales (São Paulo, León) y la posterior consolidación de la figura del curador. Contrapone su disidencia formativa —hacer lo deseado siempre que pudiera sustentarlo— a la incorporación curricular del perfil «crítico» como expectativa. Cierra describiendo el proceso material de «Bandera VIII», con bolsas de transfusión llenas de falsa sangre y sal (símbolo de la saladera), asociada a su pertenencia a un club RH negativo, como emblema de una patria en cuidados intensivos.</t>
+          <t>Conversación con el crítico y curador Max Hernández Calvo, sostenida con Carlos Zevallos en julio de 2025, centrada en la genealogía del «mandato crítico» y de la «lógica de proyecto» en el arte contemporáneo peruano. Hernández Calvo homologa el arte crítico con la producción de discurso y argumenta que los artistas jóvenes no perciben un mandato porque han sido formados dentro de un sistema que exige conceptualización previa, statement y portafolio; quienes sí lo leen como imposición externa suelen carecer de discurso, malinterpretándolo en clave esencialista o conspirativa. Reconstruye hitos institucionales: las Bienales de Lima de fines de los noventa (con Juan Peralta) que impulsaron la postulación mediante proyectos de instalación; su propia experiencia en la Bienal Nacional (1998) y en el MFA de baja residencia de Bard College (2005-2007), cuya estructura de crítica grupal evidenciaba la centralidad del discurso. Sitúa entre 2010 y 2015 la consolidación del mandato, ligada al viraje del MALI hacia lo contemporáneo, la aparición de ferias (Lima Foto, ArtLima), galerías nuevas (Revólver) y el redescubrimiento de Teresa Burga y del conceptualismo de los sesenta-setenta por Miguel López y Emilio Tarazona. Analiza los concursos (IMNA desde 2018, Pasaporte para un Artista, Artus) como síntoma del cambio, y la formación de coleccionistas (CAAC, 2006; Verme, Marsano, Hochschild, García Miró) entrenados en circuitos internacionales orientados al discurso. Cierra con una tesis sobre el extractivismo: la escena local colapsa tras las crisis políticas de 2016-2021 y la pandemia, y el artista deviene materia prima exportable, sostenido económicamente por galerías y compradores extranjeros.</t>
         </is>
       </c>
     </row>
@@ -1182,27 +1182,27 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Villacorta, Jorge - 2026-05-06.transcripcion.md</t>
+          <t>Entrevista - Lerner, Sharon - sin fecha.transcripcion.md</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>años 1970-2026 (énfasis en el arte crítico de los 80 a los 2020)</t>
+          <t>2007-2025 (historia de la colección del MALI)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Entrevista (transcripción sin refinar), 06-05-2026</t>
+          <t>Entrevista, s/f (transcripción 2026)</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Andreas Huyssen; Mirko Lauer; Herbert Rodríguez; Hans Haacke; Elena Tejada; Giuliana Borea; Luis Lama; Sharon Lerner; Isaac Ernesto; MALI; Bienal de Lima; E.P.S. Huayco</t>
+          <t>Sharon Lerner; Carlos Zevallos (entrevistador); MALI; Natalia Majluf; Tatiana Cuevas; Jorge Villacorta; Rodrigo Quijano; Miguel López; Julieta González; Florencia Portocarrero; Goethe Institut; Ricardo Kusunoki</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Extensa entrevista al curador y crítico Jorge Villacorta conducida por un investigador que prepara una tesis sobre la institucionalización del arte crítico en el Perú. Villacorta reconstruye la genealogía personal de su noción de arte crítico, armada sin bibliografía sistemática a partir de lecturas dispersas (Huyssen, Buchloh, Osborne, Greil Marcus), del Dadá y el surrealismo vistos en 1972 en el Museo de Arte Italiano, del punk británico y del constructivismo soviético. Sostiene que lo crítico no es categoría académica sino que se construye en la brega, en las luchas simbólicas por derechos, y prefiere hablar de criticidad más que de arte crítico. El diálogo interroga cómo la alternatividad disidente de los años noventa ingresó al museo y devino mandato para artistas jóvenes, articulándose con el vocabulario institucional global de lo decolonial, el género y lo queer. Villacorta introduce la tesis de que en Lima el arte existe fuera de una esfera pública dinamitada, contrasta la consolidación del arte contemporáneo en la Bienal de Trujillo (1987) frente a la Bienal de Lima (1997), y analiza la crítica institucional ausente (Haacke, Hito Steyerl, Andrea Fraser). Comenta casos peruanos: la performance de Elena Tejada, el DNI gigante de Camposano, obras de Flavia Gandolfo, Javi Vargas, Pierina Márquez, la censura a Herbert Rodríguez y Juan Dávila, y el concepto foucaultiano de parresía aplicado a Eduardo Villanes e Isaac Ernesto. Reflexiona además sobre el tutelaje del curador, la lógica de proyecto, el statement y la ansiedad teórica en la formación artística universitaria, y la polémica de Luis Lama contra su curaduría del premio ICPNA.</t>
+          <t>Entrevista a Sharon Lerner, curadora de arte contemporáneo y directora del MALI, realizada por Carlos Zevallos (transcripción de 2026). Lerner sostiene que el museo no maneja una definición taxativa de «arte contemporáneo»: se trata de un corte histórico en permanente redefinición, discutido cíclicamente con el comité académico, los asesores rotativos del Comité de Adquisiciones de Arte Contemporáneo y encuentros especializados. Reconstruye dos momentos de revisión: el volumen editado con fondo Sura (2013), heredado de Tatiana Cuevas, con ensayos de asesores (Villacorta, Quijano, Miguel López) y una conversación editada por Villacorta que expone tensiones y «discontinuidades»; y el encuentro de 2015 (con apoyo del Goethe Institut y a instancias de Julieta González) para la creación de un fondo amazónico, que reconocía institucionalmente una escena preexistente. Frente a la hipótesis del «mandato crítico», Lerner precisa que la criticidad es parte constitutiva de la práctica contemporánea, pero no un requisito excluyente ni un factor disuasivo: el museo posee obra crítica con la propia institución, y los criterios de adquisición (votación, pertinencia discursiva, conservación, precio) son múltiples. Distingue entre obras que «encarnan» (embody) discurso y aquellas meramente «formulaicas» que exhiben etiquetas. Subraya la ventaja comparativa del MALI como museo panorámico —que cruza lo precolombino, textil, popular y contemporáneo— y su rol de facto como único coleccionista sostenido ante la ausencia de otras instituciones. Explica que se expone solo por invitación curatorial, atendiendo vacíos (presencia femenina, perspectivas queer señaladas por Miguel López), y anuncia un futuro concurso de intervenciones y la proyectada expansión hacia salas del siglo XXI.</t>
         </is>
       </c>
     </row>
@@ -1214,27 +1214,27 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Entrevista - Villacorta, Jorge - 2026-06-08.transcripcion.md</t>
+          <t>Entrevista - Rebaza Torres, Alberto - 2023-10-12 (editada).docx</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>años 1960-2026 (con foco en 1997-2001 y el arte crítico de los 80)</t>
+          <t>Fines de los años 90 - 2023</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Entrevista (transcripción sin refinar), 08-06-2026</t>
+          <t>Entrevista, 12-10-2023 (editada)</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Mirko Lauer; Juan Acha; Emilio Adolfo Westphalen (Cisneros/Szyszlo); Giuliana Borea; Gerardo Chávez; Sandra Gamarra; Sharon Lerner; Giselle Ordaz; Jacques Peignet; MALI; Alianza Francesa; Fundación Wiese; Pasaporte para un Artista</t>
+          <t>Alberto Rebaza Torres; Carlos Zevallos Trigoso (entrevistador); MALI; CAAC; Ginette Fernández; Residencia de Al Lado; Bienal de Venecia; Museo Reina Sofía; Guggenheim; Eduardo Hochschild; Juan Carlos Verme; Carlos Marsano; ICPNA; Sandra Gamarra</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Segunda sesión de la entrevista a Jorge Villacorta, centrada en el origen de la crítica de arte peruana, el coleccionismo y la génesis del concurso Pasaporte para un Artista. Villacorta sitúa el nacimiento del arte crítico local en la tensión de los años setenta-ochenta entre críticos y artistas: el volante de Mirko Lauer para E.P.S. Huayco en Galería Forum, la polémica de Ortiz de Ceballos sobre Rafael Hastings y la respuesta de Szyszlo a sus críticos. Formula la hipótesis, que juzga irónica, de que la noción de arte crítico quedó instalada como sentido común justo cuando ya casi no hay críticos activos. Discute críticamente la periodización y los veinte conceptos que Giuliana Borea propone para el paso del arte moderno al contemporáneo, señalando que su libro mira la escena limeña por una ventana demasiado estrecha e ignora las motivaciones del coleccionismo. Caracteriza al coleccionista peruano como desapegado, no obsesivo y guiado por la decoración, contrastándolo con los mecenazgos brasileño y mexicano; cita el caso dramático del retorno de Gerardo Chávez y la 'nacionalización' española de Sandra Gamarra. Analiza la precariedad estructural de las instituciones (MALI, ICPNA), su hermetismo y estructura de comités, y aplica la lectura reparativa de Sedgwick frente a la paranoica. La parte más extensa reconstruye con detalle la creación de Pasaporte para un Artista (1997-1998) en el marco de la política cultural francesa, la Embajada, Mazzoni y Peignet, y las experiencias de los primeros ganadores (Bedoya, Fito Espinosa, Elena Tejada, Bendayán).</t>
+          <t>Entrevista editada a Alberto Rebaza Torres —abogado, coleccionista y presidente del consejo directivo del MALI, además de expresidente del Comité de Adquisiciones de Arte Contemporáneo—, conducida por Carlos Zevallos Trigoso en octubre de 2023. Rebaza narra el origen de su coleccionismo a fines de los noventa, orientado inicial y deliberadamente al arte peruano contemporáneo y luego extendido a lo latinoamericano, bajo la convicción de una «misión»: que el coleccionismo local funcione como primera plataforma de desarrollo para los artistas. Ubica en 2006 la formación del CAAC como factor de cohesión de un grupo de coleccionistas peruanos que ganó visibilidad en ferias regionales e internacionales (ArteBA, ARTBO, Zona Maco, Art Basel). El testimonio articula una teoría del coleccionismo como «proselitismo del arte» que, con el tiempo, debilita la sensación de propiedad y migra hacia la filantropía y el fortalecimiento institucional, ante la ausencia del Estado. Distingue el potencial «colectivo» del coleccionista frente al potencial «de a uno» del galerista, y enfatiza la complementariedad de roles (galerías, ferias, curadores, residencias) en una carrera artística sin hitos claros. Reivindica su Residencia de Al Lado (con Ginette Fernández) y menciona a otros agentes (Hochschild-MAC, Verme-MALI, Marsano-ARTUS, Mulder, Barreda). Sobre su criterio personal, prioriza la tríada contenido, inteligencia y estética, y diferencia expresamente su línea de coleccionismo de la línea curatorial del MALI —más volcada a violencia, territorio, género e historia, próxima al Reina Sofía—. El documento es fuente clave para analizar la perspectiva del coleccionismo y la filantropía en la institucionalización del arte contemporáneo peruano.</t>
         </is>
       </c>
     </row>
@@ -1246,27 +1246,27 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Flynn, Iñigo Clavo, Lemos y Portocarrero - Introduction. Artistic practice and the unmaking of coloniality (2026) [Unmaking to Make].md</t>
+          <t>Entrevista - Tokeshi, Eduardo - sin fecha.transcripcion.md</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>1990-2024 (giro decolonial contemporáneo, con referencia al legado colonial de 500 años)</t>
+          <t>1980-2002</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Introducción de libro académico (volumen editado), 2026</t>
+          <t>Entrevista, s/f</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Alex Ungprateeb Flynn; María Iñigo Clavo; Beatriz Lemos; Florencia Portocarrero; Sandra Gamarra; Cildo Meireles; Walter Mignolo; Aníbal Quijano; Silvia Rivera Cusicanqui; Grupo Modernidad/Colonialidad; MACBA; Bienal de Venecia</t>
+          <t>Eduardo Tokeshi; Carlos Zevallos (entrevistador); PUCP; Gustavo Buntinx; Luis Lama; E.P.S. Huayco; Herbert Rodríguez; Bienal de Lima; Emilio Rodríguez Larraín; Jorge Eduardo Eielson; Luis Camnitzer; Óscar Muñoz</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Introducción al volumen colectivo 'Unmaking to Make', que reorienta hacia América Latina el horizonte teórico de la práctica artística frente a la colonialidad. Los cuatro editores parten de la constatación de que el trabajo 'descolonizador' se ha vuelto norma institucional en el arte contemporáneo del Norte global, mera casilla a marcar, ilustrando cómo lo que fue posición periférica y experimental deviene marco hegemónico (ejemplificado con los bicentenarios latinoamericanos, la exposición 'Buen Gobierno' de Sandra Gamarra en Madrid, el simposio del MACBA, el informe Sarr-Savoy y la Bienal de Venecia 'Foreigners Everywhere'). Su tesis central es que la práctica artística no puede reducirse a hacer visibles teorías producidas por la academia: posee un potencial generativo y especulativo propio para imaginar y proponer mundos, situándose en relación de igualdad y no de subordinación respecto al trabajo académico. El texto revisa críticamente el corpus de la teoría decolonial del Grupo Modernidad/Colonialidad (Mignolo, Quijano, Grosfoguel, Escobar, Dussel, Lugones, Maldonado-Torres), sus diferencias con el poscolonialismo anglófono y las objeciones que ha recibido —de Rivera Cusicanqui, Aura Cumes, Adusei-Poku— por su elitismo, su tendencia a subsumir el pensamiento feminista negro y a apropiarse post hoc de autores. Frente a ello, los editores privilegian epistemologías situadas y la noción de pluriverso (de la Cadena, Blaser), conceptos como amefricanidade y contra-colonialismo, y una metodología curatorial y editorial atenta a la remuneración justa, la traducción y la asimetría de poder. Anuncian cuatro ejes: contragenealogías, instituciones, descolonización del lenguaje y futuros, abriendo con la obra 'Cruzeiro do Sul' de Cildo Meireles.</t>
+          <t>Entrevista al artista Eduardo Tokeshi (n. 1960), conducida por Carlos Zevallos, que reconstruye su formación y la génesis de su obra más reconocida en el contexto de la violencia política peruana. Tokeshi relata su tránsito de la arquitectura a la especialidad de pintura en la PUCP hacia 1983, dentro de la clásica división entre la Católica (abstracción) y Bellas Artes (figuración), y su desmarque del canon al incorporar recortes periodísticos, objetos y materiales no pictóricos. Sitúa en 1985 la primera «Bandera» —cosida, rellena, tensada—, realizada por pulsión antes que como gesto deliberadamente contemporáneo, que inaugura una serie sostenida hasta 2001-2002 como sublimación de la violencia, el duelo y la reconstrucción de la nación. El testimonio historiza el surgimiento de lo contemporáneo local: la muestra «Algo va a pasar» (1987) organizada por Gustavo Buntinx, la Bienal de Trujillo (1987), las Bienales de Lima de los noventa y la labor de Luis Lama trayendo a Camnitzer y Óscar Muñoz. Analiza la profesionalización del campo en los noventa (idea de «proyecto», statements, portafolios, cambios de currícula), el desfase o «refracción» respecto de los centros internacionales (São Paulo, León) y la posterior consolidación de la figura del curador. Contrapone su disidencia formativa —hacer lo deseado siempre que pudiera sustentarlo— a la incorporación curricular del perfil «crítico» como expectativa. Cierra describiendo el proceso material de «Bandera VIII», con bolsas de transfusión llenas de falsa sangre y sal (símbolo de la saladera), asociada a su pertenencia a un club RH negativo, como emblema de una patria en cuidados intensivos.</t>
         </is>
       </c>
     </row>
@@ -1278,27 +1278,27 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Gamboa - Fuego cruzado en la Bienal de Arte de Lima.md</t>
+          <t>Entrevista - Villacorta, Jorge - 2026-05-06.transcripcion.md</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>1997 (I Bienal de Arte de Lima)</t>
+          <t>años 1970-2026 (énfasis en el arte crítico de los 80 a los 2020)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Artículo periodístico / crónica de revista, c. 1997</t>
+          <t>Entrevista (transcripción sin refinar), 06-05-2026</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Jeremías Gamboa; Luis Lama; Raquel Tibol; Néstor García Canclini; Llilian Llanés; Aracy Amaral; Bélgica Rodríguez; Edward Sullivan; Alberto Andrade; Luz María Bedoya; Natalia Iguíñiz; Centro de Artes Visuales de Lima</t>
+          <t>Jorge Villacorta; Andreas Huyssen; Mirko Lauer; Herbert Rodríguez; Hans Haacke; Elena Tejada; Giuliana Borea; Luis Lama; Sharon Lerner; Isaac Ernesto; MALI; Bienal de Lima; E.P.S. Huayco</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Crónica periodística de Jeremías Gamboa sobre la polémica desatada en la I Bienal de Arte de Lima (1997), organizada por Luis Lama con una inversión cercana al millón de dólares, más de 150 expositores y casi un millón y medio de visitantes en el centro histórico. El texto reconstruye el 'fuego cruzado' provocado por la crítica mexicana Raquel Tibol, quien en las mesas de conversación y luego en la revista Proceso denunció la falta de reflexión y rigor del evento y su desbalance grotesco: 129 peruanos frente a 33 extranjeros, lo que convertía la muestra en un festival de plástica peruana antes que en una bienal iberoamericana. Gamboa rastrea el origen del problema en la composición excesivamente numerosa y heterogénea del comité de selección —cuatro escuelas, trece galerías y ocho críticos, entre ellos Castrillón, Lauer, Majluf, Wuffarden y el propio Villacorta— cuyo criterio 'democrático' permitió que cualquiera con un solo voto expusiera, con proclividad de los galeristas hacia sus propios artistas. Contrasta este modelo con la depuración conceptual de la Bienal de La Habana (Llilian Llanés) y con la ausencia de un concepto integrador eficaz, señalando que la 'pluralidad cultural' figuraba en las bases pero pocos la advertían, salvo García Canclini. El artículo recoge además elogios internacionales al trabajo de Luz María Bedoya y Natalia Iguíñiz, y un recuadro dedicado al debate paralelo sobre la existencia o no de un 'arte latinoamericano', con posturas encontradas de Lama y Bélgica Rodríguez frente a García Canclini y Edward Sullivan.</t>
+          <t>Extensa entrevista al curador y crítico Jorge Villacorta conducida por un investigador que prepara una tesis sobre la institucionalización del arte crítico en el Perú. Villacorta reconstruye la genealogía personal de su noción de arte crítico, armada sin bibliografía sistemática a partir de lecturas dispersas (Huyssen, Buchloh, Osborne, Greil Marcus), del Dadá y el surrealismo vistos en 1972 en el Museo de Arte Italiano, del punk británico y del constructivismo soviético. Sostiene que lo crítico no es categoría académica sino que se construye en la brega, en las luchas simbólicas por derechos, y prefiere hablar de criticidad más que de arte crítico. El diálogo interroga cómo la alternatividad disidente de los años noventa ingresó al museo y devino mandato para artistas jóvenes, articulándose con el vocabulario institucional global de lo decolonial, el género y lo queer. Villacorta introduce la tesis de que en Lima el arte existe fuera de una esfera pública dinamitada, contrasta la consolidación del arte contemporáneo en la Bienal de Trujillo (1987) frente a la Bienal de Lima (1997), y analiza la crítica institucional ausente (Haacke, Hito Steyerl, Andrea Fraser). Comenta casos peruanos: la performance de Elena Tejada, el DNI gigante de Camposano, obras de Flavia Gandolfo, Javi Vargas, Pierina Márquez, la censura a Herbert Rodríguez y Juan Dávila, y el concepto foucaultiano de parresía aplicado a Eduardo Villanes e Isaac Ernesto. Reflexiona además sobre el tutelaje del curador, la lógica de proyecto, el statement y la ansiedad teórica en la formación artística universitaria, y la polémica de Luis Lama contra su curaduría del premio ICPNA.</t>
         </is>
       </c>
     </row>
@@ -1310,27 +1310,27 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Germaná y Portocarrero - The «Indigenous turn» and the rise of Amazonian art. Insights from the seminal work of the SHRA (2026) [Unmaking to Make, cap. 8].md</t>
+          <t>Entrevista - Villacorta, Jorge - 2026-06-08.transcripcion.md</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>1966-2025 (con foco en el 'giro indígena' de los años 90 en adelante)</t>
+          <t>años 1960-2026 (con foco en 1997-2001 y el arte crítico de los 80)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro académico, 2026</t>
+          <t>Entrevista (transcripción sin refinar), 08-06-2026</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Gabriela Germaná; Florencia Portocarrero; Pablo Macera; María Belén Soria; Gredna Landolt; Víctor Churay; Elena Valera; Roldán Pinedo; Lastenia Canayo; Sara Flores; Mirko Lauer; Natalia Majluf; SHRA (UNMSM); Fundación Telefónica; MALI; MASP</t>
+          <t>Jorge Villacorta; Mirko Lauer; Juan Acha; Emilio Adolfo Westphalen (Cisneros/Szyszlo); Giuliana Borea; Gerardo Chávez; Sandra Gamarra; Sharon Lerner; Giselle Ordaz; Jacques Peignet; MALI; Alianza Francesa; Fundación Wiese; Pasaporte para un Artista</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Capítulo que examina el 'giro indígena' global y el ascenso del arte amazónico en el Perú a partir de la labor seminal del Seminario de Historia Rural Andina (SHRA), instituto de la UNMSM fundado por Pablo Macera en 1966. Germaná y Portocarrero parten de la exclusión histórica de los creadores indígenas de la historia del arte oficial, relegados a la categoría de artesanía por una lógica racializada que niega la posibilidad de que algo sea simultáneamente arte e indígena. Apoyándose en 'Lo andino en el arte peruano' de Mirko Lauer (1980), describen el campo artístico estratificado en tres universos —alto arte, arte popular y arte prehispánico— y sus rupturas: el indigenismo de los años veinte, la redefinición política de la artesanía bajo el gobierno de Velasco (premio a Joaquín López Antay, 1975) y el giro indígena de los noventa ligado al multiculturalismo neoliberal. El eje del texto es la metodología colaborativa del SHRA, que desde 1997 —con Macera y María Belén Soria, inspirados por la experiencia de Gredna Landolt en Formabiap— trabajó con pintores amazónicos autodidactas (Víctor Churay, Elena Valera, Roldán Pinedo, Lastenia Canayo, Enrique Casanto) usando la ecuación pintura-escritura para recuperar la memoria oral. Destacan que el seminario reconoció la autoría individual, pagó por el trabajo y operó como 'zona de contacto' descolonial. Las autoras concluyen que este método, de raíz etnográfica, consolidó la pintura figurativa como criterio de legitimación —limitando otros medios y el kené—, y analizan las contradicciones de la inserción del arte indígena en el circuito global (Sara Flores en el MALI, la Bienal de Venecia de Pedrosa, testimonios de Yahuarcani y Mombaça).</t>
+          <t>Segunda sesión de la entrevista a Jorge Villacorta, centrada en el origen de la crítica de arte peruana, el coleccionismo y la génesis del concurso Pasaporte para un Artista. Villacorta sitúa el nacimiento del arte crítico local en la tensión de los años setenta-ochenta entre críticos y artistas: el volante de Mirko Lauer para E.P.S. Huayco en Galería Forum, la polémica de Ortiz de Ceballos sobre Rafael Hastings y la respuesta de Szyszlo a sus críticos. Formula la hipótesis, que juzga irónica, de que la noción de arte crítico quedó instalada como sentido común justo cuando ya casi no hay críticos activos. Discute críticamente la periodización y los veinte conceptos que Giuliana Borea propone para el paso del arte moderno al contemporáneo, señalando que su libro mira la escena limeña por una ventana demasiado estrecha e ignora las motivaciones del coleccionismo. Caracteriza al coleccionista peruano como desapegado, no obsesivo y guiado por la decoración, contrastándolo con los mecenazgos brasileño y mexicano; cita el caso dramático del retorno de Gerardo Chávez y la 'nacionalización' española de Sandra Gamarra. Analiza la precariedad estructural de las instituciones (MALI, ICPNA), su hermetismo y estructura de comités, y aplica la lectura reparativa de Sedgwick frente a la paranoica. La parte más extensa reconstruye con detalle la creación de Pasaporte para un Artista (1997-1998) en el marco de la política cultural francesa, la Embajada, Mazzoni y Peignet, y las experiencias de los primeros ganadores (Bedoya, Fito Espinosa, Elena Tejada, Bendayán).</t>
         </is>
       </c>
     </row>
@@ -1342,27 +1342,27 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Hernández Calvo y Villacorta - Franquicias imaginarias. Las opciones estéticas en las artes plásticas en el Perú de fin de siglo (2002) [OCR A].md</t>
+          <t>Flynn, Iñigo Clavo, Lemos y Portocarrero - Introduction. Artistic practice and the unmaking of coloniality (2026) [Unmaking to Make].md</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>1950-2000 (segunda mitad del siglo XX, con énfasis en los años 90 y fin de siglo)</t>
+          <t>1990-2024 (giro decolonial contemporáneo, con referencia al legado colonial de 500 años)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Libro / ensayo académico (Fondo Editorial PUCP), 2002</t>
+          <t>Introducción de libro académico (volumen editado), 2026</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Max Hernández Calvo; Jorge Villacorta; Mirko Lauer; Fernando de Szyszlo; Luis Miró Quesada; Juan Acha; Ricardo Grau; Agrupación Espacio; IAC; Colectivo Sociedad Civil; Eduardo Villanes; Ricardo Wiesse; Alfredo Márquez; PUCP</t>
+          <t>Alex Ungprateeb Flynn; María Iñigo Clavo; Beatriz Lemos; Florencia Portocarrero; Sandra Gamarra; Cildo Meireles; Walter Mignolo; Aníbal Quijano; Silvia Rivera Cusicanqui; Grupo Modernidad/Colonialidad; MACBA; Bienal de Venecia</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Libro de Max Hernández Calvo y Jorge Villacorta que ofrece una lectura crítica y panorámica —no meramente cronológica— de las opciones estéticas en las artes plásticas peruanas de la segunda mitad del siglo XX, atendiendo especialmente a Lima y al fin de siglo. La tesis de fondo es la precariedad y fragmentación del sistema artístico local (ausencia de un museo de arte contemporáneo, mercado incipiente, divorcio entre producción y recepción crítica, escisión ficticia entre arte y comercio) que impide comprender lo artístico como sistema. El texto reconstruye la instauración del modelo moderno-tardío: la llegada de la abstracción con Szyszlo (1949), la Agrupación Espacio, Luis Miró Quesada y el IAC como brazos de un proyecto vinculado a la burguesía industrial y urbanizadora, el desplazamiento del indigenismo en crisis y la posterior 'abstracción de reminiscencia precolombina' como símbolo ficticio de integración nacional que soslaya las realidades sociales del país migrante. Analiza luego la vanguardia de los sesenta (Pop y Op, Arte Nuevo, Juan Acha, Teresa Burga), la institucionalización postideológica, las esferas subsidiarias y escenas alternativas, la introspección y el juego, la globalización y 'lo social desquerenciado'. Un capítulo central, 'En la estela de la política', documenta el auge del arte políticamente motivado en la crisis del fujimorato tardío: Runcie Tanaka, Miguel Cordero, Ricardo Wiesse (Cantuta), Eduardo Villanes ('Gloria Evaporada'), Emilio Santisteban, el Colectivo Sociedad Civil ('Lava la bandera') y Perú Fábrica, con su especulación sobre los espacios público y privado. Cierra advirtiendo que la postmodernidad no se consolida como marco crítico por la misma precariedad institucional.</t>
+          <t>Introducción al volumen colectivo 'Unmaking to Make', que reorienta hacia América Latina el horizonte teórico de la práctica artística frente a la colonialidad. Los cuatro editores parten de la constatación de que el trabajo 'descolonizador' se ha vuelto norma institucional en el arte contemporáneo del Norte global, mera casilla a marcar, ilustrando cómo lo que fue posición periférica y experimental deviene marco hegemónico (ejemplificado con los bicentenarios latinoamericanos, la exposición 'Buen Gobierno' de Sandra Gamarra en Madrid, el simposio del MACBA, el informe Sarr-Savoy y la Bienal de Venecia 'Foreigners Everywhere'). Su tesis central es que la práctica artística no puede reducirse a hacer visibles teorías producidas por la academia: posee un potencial generativo y especulativo propio para imaginar y proponer mundos, situándose en relación de igualdad y no de subordinación respecto al trabajo académico. El texto revisa críticamente el corpus de la teoría decolonial del Grupo Modernidad/Colonialidad (Mignolo, Quijano, Grosfoguel, Escobar, Dussel, Lugones, Maldonado-Torres), sus diferencias con el poscolonialismo anglófono y las objeciones que ha recibido —de Rivera Cusicanqui, Aura Cumes, Adusei-Poku— por su elitismo, su tendencia a subsumir el pensamiento feminista negro y a apropiarse post hoc de autores. Frente a ello, los editores privilegian epistemologías situadas y la noción de pluriverso (de la Cadena, Blaser), conceptos como amefricanidade y contra-colonialismo, y una metodología curatorial y editorial atenta a la remuneración justa, la traducción y la asimetría de poder. Anuncian cuatro ejes: contragenealogías, instituciones, descolonización del lenguaje y futuros, abriendo con la obra 'Cruzeiro do Sul' de Cildo Meireles.</t>
         </is>
       </c>
     </row>
@@ -1374,27 +1374,27 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Hernández Calvo y Villacorta - Franquicias imaginarias. Las opciones estéticas en las artes plásticas en el Perú de fin de siglo (2002) [OCR B].md</t>
+          <t>Gamboa - Fuego cruzado en la Bienal de Arte de Lima.md</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>1950-2001 (con énfasis en los años 70, 80 y 90)</t>
+          <t>1997 (I Bienal de Arte de Lima)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Libro/ensayo crítico (OCR), 2002</t>
+          <t>Artículo periodístico / crónica de revista, c. 1997</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Max Hernández Calvo; Jorge Villacorta; Fondo Editorial PUCP; Fernando de Szyszlo; Ricardo Grau; Juan Acha; Mirko Lauer; Cristina Planas; Milagros de la Torre; Carlos Runcie Tanaka; Ricardo Wiesse; Bienal de Lima / ICPNA</t>
+          <t>Jeremías Gamboa; Luis Lama; Raquel Tibol; Néstor García Canclini; Llilian Llanés; Aracy Amaral; Bélgica Rodríguez; Edward Sullivan; Alberto Andrade; Luz María Bedoya; Natalia Iguíñiz; Centro de Artes Visuales de Lima</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Ensayo panorámico que diagnostica el desarrollo de las artes visuales peruanas desde mediados del siglo XX hasta el cambio de milenio, sosteniendo que la reflexión crítica local ha permanecido en un vacío de casi tres décadas pese a la creciente diversificación de opciones estéticas, soportes y medios. Los autores conciben el arte como sistema y práctica social, y denuncian la precariedad institucional peruana: la ausencia de un museo de arte contemporáneo, un mercado incipiente, la escisión ficticia entre arte y comercio y una formación que divorcia producción manual de reflexión conceptual. El texto reconstruye una genealogía: la instauración dominante del modelo moderno-tardío y la abstracción (Szyszlo, Grau, Espacio, Miró Quesada) como desplazamiento programático del indigenismo hacia una base social burguesa e industrial; el frenesí pop y las vanguardias de los sesenta; la reforma velasquista y sus tensiones entre lo popular (artesanía) y lo culto. Avanza luego hacia la institucionalización postideológica, las esferas alternativas y la globalización "C.O.D.", cerrando con el retorno de lo social y lo político a fines de los noventa. Marco conceptual apoyado en Foster, Greenberg, García Canclini y sociología de la cultura (esfera pública, movimientos sociales). Analiza obras como La wuawua de Planas sobre Abimael Guzmán, las fotografías forenses de Milagros de la Torre, Uchuraccay, el memorial cantuta de Wiesse en Cieneguilla, los ensamblajes de Miguel Cordero sobre Barrios Altos y La Cantuta, y a Runcie Tanaka. Su aporte es ofrecer una lectura orgánica, temática y no meramente cronológica del "fin de siglo" limeño, situando lo estético como franquicia imaginativa para la comunicación ciudadana.</t>
+          <t>Crónica periodística de Jeremías Gamboa sobre la polémica desatada en la I Bienal de Arte de Lima (1997), organizada por Luis Lama con una inversión cercana al millón de dólares, más de 150 expositores y casi un millón y medio de visitantes en el centro histórico. El texto reconstruye el 'fuego cruzado' provocado por la crítica mexicana Raquel Tibol, quien en las mesas de conversación y luego en la revista Proceso denunció la falta de reflexión y rigor del evento y su desbalance grotesco: 129 peruanos frente a 33 extranjeros, lo que convertía la muestra en un festival de plástica peruana antes que en una bienal iberoamericana. Gamboa rastrea el origen del problema en la composición excesivamente numerosa y heterogénea del comité de selección —cuatro escuelas, trece galerías y ocho críticos, entre ellos Castrillón, Lauer, Majluf, Wuffarden y el propio Villacorta— cuyo criterio 'democrático' permitió que cualquiera con un solo voto expusiera, con proclividad de los galeristas hacia sus propios artistas. Contrasta este modelo con la depuración conceptual de la Bienal de La Habana (Llilian Llanés) y con la ausencia de un concepto integrador eficaz, señalando que la 'pluralidad cultural' figuraba en las bases pero pocos la advertían, salvo García Canclini. El artículo recoge además elogios internacionales al trabajo de Luz María Bedoya y Natalia Iguíñiz, y un recuadro dedicado al debate paralelo sobre la existencia o no de un 'arte latinoamericano', con posturas encontradas de Lama y Bélgica Rodríguez frente a García Canclini y Edward Sullivan.</t>
         </is>
       </c>
     </row>
@@ -1406,27 +1406,27 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>ICAA-1138109.pdf</t>
+          <t>Germaná y Portocarrero - The «Indigenous turn» and the rise of Amazonian art. Insights from the seminal work of the SHRA (2026) [Unmaking to Make, cap. 8].md</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Debate del nacionalismo e indigenismo en la pintura peruana, c. décadas de 1940-1950</t>
+          <t>1966-2025 (con foco en el 'giro indígena' de los años 90 en adelante)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Artículo de prensa (Suplemento Dominical de El Comercio, Lima), c. 1957 (s/f exacta); digitalizado por ICAA-MFAH</t>
+          <t>Capítulo de libro académico, 2026</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>J. Nahuaca (seudónimo); José Sabogal; Francisco Laso; Fernando de Szyszlo; Ricardo Grau; Fernando de Villegas / Villegas; Juan Manuel Ugarte Eléspuru; Pancho Fierro; César Vallejo; Inca Garcilaso; El Comercio (Suplemento Dominical); International Center for the Arts of the Americas (ICAA-MFAH)</t>
+          <t>Gabriela Germaná; Florencia Portocarrero; Pablo Macera; María Belén Soria; Gredna Landolt; Víctor Churay; Elena Valera; Roldán Pinedo; Lastenia Canayo; Sara Flores; Mirko Lauer; Natalia Majluf; SHRA (UNMSM); Fundación Telefónica; MALI; MASP</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Artículo "Conscripción peruana la pintura", firmado con el seudónimo J. Nahuaca y publicado en el Suplemento Dominical de El Comercio de Lima (hacia finales de los años cincuenta, a juzgar por las referencias contextuales), conservado en el archivo digital ICAA del Museum of Fine Arts, Houston. La tesis sostiene que la pintura peruana sufre la presión de fuerzas nacionalistas que operan "desde afuera" como verdaderas conscripciones que le imponen un destino en nombre de la peruanidad, esterilizando sus energías estéticas endógenas. El autor distingue tres conscripciones: la político-social, que reduce la pintura a panfleto, confesión o acto de fe redentor y la torna inoperante; la iconográfica, la más antigua, que exige amor a lo nacional mediante la anécdota histórica y costumbrista (Merino, Montero, Castillo) y culmina en el indigenismo de Sabogal -cuya nacionalización amorosa de la iconografía "termina siendo una montonera"-; y la espiritual, con dos modalidades: un humanismo telúrico o "vallejismo" pictórico (Laso, Ugarte Eléspuru) y una búsqueda del eslabón formal con el pasado prehispánico y colonial. El marco conceptual moviliza el determinismo de Taine, la estilización del arte preincaico (Chavín, Nazca, Paracas, Moche), la escuela cuzqueña y la continuidad estética que uniría Garcilaso con Vallejo. Nahuaca reivindica la autonomía "insobornable" de la pintura frente a las presiones nacionalizadoras, valorando en Dávila, Grau, Szyszlo y Villegas tanto el entronque con el pasado como su vigencia pictórica. El aporte es un alegato antiindigenista y formalista que reclama la sublimación estética por encima de la subordinación ideológica, en pleno debate sobre la identidad del arte peruano.</t>
+          <t>Capítulo que examina el 'giro indígena' global y el ascenso del arte amazónico en el Perú a partir de la labor seminal del Seminario de Historia Rural Andina (SHRA), instituto de la UNMSM fundado por Pablo Macera en 1966. Germaná y Portocarrero parten de la exclusión histórica de los creadores indígenas de la historia del arte oficial, relegados a la categoría de artesanía por una lógica racializada que niega la posibilidad de que algo sea simultáneamente arte e indígena. Apoyándose en 'Lo andino en el arte peruano' de Mirko Lauer (1980), describen el campo artístico estratificado en tres universos —alto arte, arte popular y arte prehispánico— y sus rupturas: el indigenismo de los años veinte, la redefinición política de la artesanía bajo el gobierno de Velasco (premio a Joaquín López Antay, 1975) y el giro indígena de los noventa ligado al multiculturalismo neoliberal. El eje del texto es la metodología colaborativa del SHRA, que desde 1997 —con Macera y María Belén Soria, inspirados por la experiencia de Gredna Landolt en Formabiap— trabajó con pintores amazónicos autodidactas (Víctor Churay, Elena Valera, Roldán Pinedo, Lastenia Canayo, Enrique Casanto) usando la ecuación pintura-escritura para recuperar la memoria oral. Destacan que el seminario reconoció la autoría individual, pagó por el trabajo y operó como 'zona de contacto' descolonial. Las autoras concluyen que este método, de raíz etnográfica, consolidó la pintura figurativa como criterio de legitimación —limitando otros medios y el kené—, y analizan las contradicciones de la inserción del arte indígena en el circuito global (Sara Flores en el MALI, la Bienal de Venecia de Pedrosa, testimonios de Yahuarcani y Mombaça).</t>
         </is>
       </c>
     </row>
@@ -1438,27 +1438,27 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>ICAA-1146549.pdf</t>
+          <t>Hernández Calvo y Villacorta - Franquicias imaginarias. Las opciones estéticas en las artes plásticas en el Perú de fin de siglo (2002) [OCR A].md</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>«Última década» del s. XX (años 1990; dictadura de Fujimori 1990-2000), con antecedentes desde los 60-80</t>
+          <t>1950-2000 (segunda mitad del siglo XX, con énfasis en los años 90 y fin de siglo)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo (muestra «Puntos Cardinales»), noviembre de 2001; digitalizado por ICAA-MFAH (reg. 1146549); OCR muy dañado</t>
+          <t>Libro / ensayo académico (Fondo Editorial PUCP), 2002</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Quijano; Fernando Bryce; Iván Esquivel «Plaztikk»; Sandra Gamarra; Gilda Mantilla; Gustavo Buntinx; Mirko Lauer; Augusto del Valle; Juan Javier Salazar; Eduardo Tokeshi; Colectivo Sociedad Civil; ENBA; Museo de Arte de Lima; Bienal de Lima; ICAA-MFAH</t>
+          <t>Max Hernández Calvo; Jorge Villacorta; Mirko Lauer; Fernando de Szyszlo; Luis Miró Quesada; Juan Acha; Ricardo Grau; Agrupación Espacio; IAC; Colectivo Sociedad Civil; Eduardo Villanes; Ricardo Wiesse; Alfredo Márquez; PUCP</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Ensayo de Rodrigo Quijano fechado «Noviembre, 2001», texto del catálogo de la muestra colectiva «Puntos Cardinales» (cuatro artistas: Fernando Bryce, Iván Esquivel «Plaztikk», Sandra Gamarra y Gilda Mantilla). Titulado «¿De qué puntos cardinales hablan? Anotaciones sobre la última década en las artes visuales peruanas», ofrece un balance de los años noventa organizado en doce secciones numeradas. Su hilo es que la década consolidó una orientación del arte contemporáneo local a la vez que se perdió «un norte definido»: la entrada abrupta de la escena al «orden internacional» y a un «mercado simbólico consolidado de la región» tras años de aislamiento, bajo la dictadura de Fujimori (1990-2000). Rastrea el fin de la «modernidad alternativa» anclada en lo popular (con referencias a Lauer y su «Teoría de las Raíces Nacionales» y a Buntinx), la represión de los colectivos jóvenes (el grupo Huayco como paradigma, N.N. «diezmado» y Alfredo Márquez encarcelado bajo falsos cargos de terrorismo) y la «reinstitucionalización» privada (MALI, Centro de Artes Visuales, concursos y bienales auspiciados por el sector privado, Bienal de Lima desde 1997). Analiza en detalle a los cuatro artistas y comenta la crisis de la ENBA (intervenida por la dictadura), los «vladivideos», La Cantuta, Barrios Altos y el «Lava la bandera» del Colectivo Sociedad Civil (2000). Cierra afirmando que «la escena crítica es proporcionalmente precaria e invisible». Fuente primaria sobre la escena limeña de los noventa; digitalizada por el ICAA-MFAH (registro 1146549), con OCR muy dañado.</t>
+          <t>Libro de Max Hernández Calvo y Jorge Villacorta que ofrece una lectura crítica y panorámica —no meramente cronológica— de las opciones estéticas en las artes plásticas peruanas de la segunda mitad del siglo XX, atendiendo especialmente a Lima y al fin de siglo. La tesis de fondo es la precariedad y fragmentación del sistema artístico local (ausencia de un museo de arte contemporáneo, mercado incipiente, divorcio entre producción y recepción crítica, escisión ficticia entre arte y comercio) que impide comprender lo artístico como sistema. El texto reconstruye la instauración del modelo moderno-tardío: la llegada de la abstracción con Szyszlo (1949), la Agrupación Espacio, Luis Miró Quesada y el IAC como brazos de un proyecto vinculado a la burguesía industrial y urbanizadora, el desplazamiento del indigenismo en crisis y la posterior 'abstracción de reminiscencia precolombina' como símbolo ficticio de integración nacional que soslaya las realidades sociales del país migrante. Analiza luego la vanguardia de los sesenta (Pop y Op, Arte Nuevo, Juan Acha, Teresa Burga), la institucionalización postideológica, las esferas subsidiarias y escenas alternativas, la introspección y el juego, la globalización y 'lo social desquerenciado'. Un capítulo central, 'En la estela de la política', documenta el auge del arte políticamente motivado en la crisis del fujimorato tardío: Runcie Tanaka, Miguel Cordero, Ricardo Wiesse (Cantuta), Eduardo Villanes ('Gloria Evaporada'), Emilio Santisteban, el Colectivo Sociedad Civil ('Lava la bandera') y Perú Fábrica, con su especulación sobre los espacios público y privado. Cierra advirtiendo que la postmodernidad no se consolida como marco crítico por la misma precariedad institucional.</t>
         </is>
       </c>
     </row>
@@ -1470,27 +1470,27 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>ICAA-1272963.pdf</t>
+          <t>Hernández Calvo y Villacorta - Franquicias imaginarias. Las opciones estéticas en las artes plásticas en el Perú de fin de siglo (2002) [OCR B].md</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Debate sobre arte, doctrina y nacionalismo; revisión de las revoluciones cristiana, francesa, rusa y mexicana; c. décadas de 1940-1950</t>
+          <t>1950-2001 (con énfasis en los años 70, 80 y 90)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Artículo de prensa (Suplemento Dominical de El Comercio, Lima), c. 1957 (s/f exacta); digitalizado por ICAA-MFAH</t>
+          <t>Libro/ensayo crítico (OCR), 2002</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>J. Nahuaca (seudónimo); Moisés Laymito; Gladys Zender; César Vallejo; Wilhelm Worringer; Arnold Hauser; Nicolai Hartmann; Charles Lalo; Jacques-Louis David; Kazimir Malevich; Wassily Kandinsky; Marc Chagall; El Comercio (Suplemento Dominical); ICAA-MFAH</t>
+          <t>Max Hernández Calvo; Jorge Villacorta; Fondo Editorial PUCP; Fernando de Szyszlo; Ricardo Grau; Juan Acha; Mirko Lauer; Cristina Planas; Milagros de la Torre; Carlos Runcie Tanaka; Ricardo Wiesse; Bienal de Lima / ICPNA</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Segunda entrega del ensayo de J. Nahuaca, titulada "Ideas doctrinarias y la pintura", publicada en el Suplemento Dominical de El Comercio de Lima (fines de los cincuenta) y archivada en el ICAA-MFAH. Continúa la reflexión sobre las fuerzas que tensionan el arte peruano, distinguiendo entre energías subyacentes -lentas, sentimentales, nacionalizadoras, orientadas a la peruanidad- y fuerzas dinámicas que importan sistemas político-sociales para materializarlos de inmediato, sometiendo el arte a los valores sociales mediante una estética "demagógica y a la vez conservadora". El objeto central es la relación entre pintura e ideas doctrinarias, examinada a través de un recorrido histórico por cuatro revoluciones: la cristiana (que renuncia al arte pagano y desemboca en la iconoclasia), la francesa (que no crea estilo sino que adopta el clasicismo de David, oficializado por Napoleón), la rusa (que tras aliarse con la vanguardia -Malevich, Kandinsky, Chagall- recae en el realismo heroico reaccionario) y la mexicana (nacida sin doctrina, expresiva y muralista, que crea el mito de la revolución cumplida). El marco teórico cita a Worringer, Hauser, Nicolai Hartmann y Charles Lalo, y disuelve la antinomia forma-contenido cara a la estética marxista. Nahuaca argumenta que ninguna revolución ha mejorado ni creado un arte, que este pertenece a individuos y la colectividad solo lo usufructúa, y aboga por "desclasificar" la élite estética -verdadera valoradora- frente al monopolio de las clases dirigentes. Denuncia un "terrorismo en pintura" que exige conciencia social y concluye que el ímpetu nacionalizador peruano ha derivado en un mal menor: la peruanización de la iconografía como fin artístico. Incluye notas sobre el escultor Moisés Laymito y un retrato de Gladys Zender.</t>
+          <t>Ensayo panorámico que diagnostica el desarrollo de las artes visuales peruanas desde mediados del siglo XX hasta el cambio de milenio, sosteniendo que la reflexión crítica local ha permanecido en un vacío de casi tres décadas pese a la creciente diversificación de opciones estéticas, soportes y medios. Los autores conciben el arte como sistema y práctica social, y denuncian la precariedad institucional peruana: la ausencia de un museo de arte contemporáneo, un mercado incipiente, la escisión ficticia entre arte y comercio y una formación que divorcia producción manual de reflexión conceptual. El texto reconstruye una genealogía: la instauración dominante del modelo moderno-tardío y la abstracción (Szyszlo, Grau, Espacio, Miró Quesada) como desplazamiento programático del indigenismo hacia una base social burguesa e industrial; el frenesí pop y las vanguardias de los sesenta; la reforma velasquista y sus tensiones entre lo popular (artesanía) y lo culto. Avanza luego hacia la institucionalización postideológica, las esferas alternativas y la globalización "C.O.D.", cerrando con el retorno de lo social y lo político a fines de los noventa. Marco conceptual apoyado en Foster, Greenberg, García Canclini y sociología de la cultura (esfera pública, movimientos sociales). Analiza obras como La wuawua de Planas sobre Abimael Guzmán, las fotografías forenses de Milagros de la Torre, Uchuraccay, el memorial cantuta de Wiesse en Cieneguilla, los ensamblajes de Miguel Cordero sobre Barrios Altos y La Cantuta, y a Runcie Tanaka. Su aporte es ofrecer una lectura orgánica, temática y no meramente cronológica del "fin de siglo" limeño, situando lo estético como franquicia imaginativa para la comunicación ciudadana.</t>
         </is>
       </c>
     </row>
@@ -1502,27 +1502,27 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>ICPNA Catalogo Bellas Artes FINAL.pdf</t>
+          <t>ICAA-1138109.pdf</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>1918-2018</t>
+          <t>Debate del nacionalismo e indigenismo en la pintura peruana, c. décadas de 1940-1950</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de exposición / libro institucional, noviembre de 2018</t>
+          <t>Artículo de prensa (Suplemento Dominical de El Comercio, Lima), c. 1957 (s/f exacta); digitalizado por ICAA-MFAH</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Escuela Nacional Superior Autónoma de Bellas Artes del Perú (ENSABAP); Instituto Cultural Peruano Norteamericano (ICPNA); Max Hernández Calvo; Augusto del Valle Cárdenas; Rocío Corcuera Ríos; Víctor Mejía Ticona; Miguel Sánchez Flores; Luis Carlos Valdez Espinoza; Roberto Hoyle; Municipalidad de Miraflores; E.P.S. Huayco; Grupo Paréntesis</t>
+          <t>J. Nahuaca (seudónimo); José Sabogal; Francisco Laso; Fernando de Szyszlo; Ricardo Grau; Fernando de Villegas / Villegas; Juan Manuel Ugarte Eléspuru; Pancho Fierro; César Vallejo; Inca Garcilaso; El Comercio (Suplemento Dominical); International Center for the Arts of the Americas (ICAA-MFAH)</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>El volumen documenta 'Un siglo de arte desde la Escuela Nacional', ciclo de cuatro exposiciones organizado en 2018 para el centenario (1918-2018) de la Escuela Nacional Superior Autónoma de Bellas Artes del Perú (ENSABAP), coeditado con el Instituto Cultural Peruano Norteamericano (ICPNA). Bajo la curaduría general de Max Hernández Calvo y Augusto del Valle Cárdenas, con Rocío Corcuera, Víctor Mejía y Miguel Sánchez, el proyecto busca construir memoria institucional y revisar cien años de producción y pedagogía bellasartina, articulándola con la sociedad contemporánea. Las muestras se distribuyeron en cuatro sedes (galerías ICPNA Juan Pardo Heeren y Germán Krüger Espantoso, y salas municipales de Miraflores). 'Bellas Artes: voz y huella de los egresados' (Corcuera) parte de cuarenta entrevistas a egresados de 1951 a 2017 —de Ella Krebs a Andrés Yaques— y una línea de tiempo que vincula formación, testimonio y obra estudiantil. 'Del individuo al ser social' (Sánchez) estudia los colectivos surgidos desde los años setenta (E.P.S. Huayco, Paréntesis, Signo x Signo, C.H.O.L.O., entre otros) como gesto político frente al modelo del artista individual. 'Espacio público' (Mejía) analiza el centro de Lima como insumo estético y campo de intervención. 'Una trayectoria de imágenes' (Hernández Calvo y Del Valle) emplea los géneros académicos —bodegón, paisaje, retrato— para pensar el tránsito del arte moderno al contemporáneo. La tesis transversal cuestiona la narrativa figurativo/abstracto de la modernidad e introduce la pregunta por el ícono, uniendo lo global con las tradiciones locales y artesanales, para otorgar 'carta de ciudadanía' a prácticas invisibilizadas desde una escuela pública.</t>
+          <t>Artículo "Conscripción peruana la pintura", firmado con el seudónimo J. Nahuaca y publicado en el Suplemento Dominical de El Comercio de Lima (hacia finales de los años cincuenta, a juzgar por las referencias contextuales), conservado en el archivo digital ICAA del Museum of Fine Arts, Houston. La tesis sostiene que la pintura peruana sufre la presión de fuerzas nacionalistas que operan "desde afuera" como verdaderas conscripciones que le imponen un destino en nombre de la peruanidad, esterilizando sus energías estéticas endógenas. El autor distingue tres conscripciones: la político-social, que reduce la pintura a panfleto, confesión o acto de fe redentor y la torna inoperante; la iconográfica, la más antigua, que exige amor a lo nacional mediante la anécdota histórica y costumbrista (Merino, Montero, Castillo) y culmina en el indigenismo de Sabogal -cuya nacionalización amorosa de la iconografía "termina siendo una montonera"-; y la espiritual, con dos modalidades: un humanismo telúrico o "vallejismo" pictórico (Laso, Ugarte Eléspuru) y una búsqueda del eslabón formal con el pasado prehispánico y colonial. El marco conceptual moviliza el determinismo de Taine, la estilización del arte preincaico (Chavín, Nazca, Paracas, Moche), la escuela cuzqueña y la continuidad estética que uniría Garcilaso con Vallejo. Nahuaca reivindica la autonomía "insobornable" de la pintura frente a las presiones nacionalizadoras, valorando en Dávila, Grau, Szyszlo y Villegas tanto el entronque con el pasado como su vigencia pictórica. El aporte es un alegato antiindigenista y formalista que reclama la sublimación estética por encima de la subordinación ideológica, en pleno debate sobre la identidad del arte peruano.</t>
         </is>
       </c>
     </row>
@@ -1534,27 +1534,27 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Kusunoki y Lerner - Reconsidering the «art museum». Some reflections on the history of the MALI collections (2026) [Unmaking to Make, cap. 5].md</t>
+          <t>ICAA-1146549.pdf</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>1961-2022 (con referencias desde época prehispánica y los años 20)</t>
+          <t>«Última década» del s. XX (años 1990; dictadura de Fujimori 1990-2000), con antecedentes desde los 60-80</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro, 2026</t>
+          <t>Ensayo de catálogo (muestra «Puntos Cardinales»), noviembre de 2001; digitalizado por ICAA-MFAH (reg. 1146549); OCR muy dañado</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Ricardo Kusunoki; Sharon Lerner; Museo de Arte de Lima (MALI); Natalia Majluf; Gabriela Germaná; Gredna Landolt; ADAPS / Piraq Causa; Brus Rubio Churay; José Sabogal; Con/Vida; Matadero Madrid / ARCO; Julieta González</t>
+          <t>Rodrigo Quijano; Fernando Bryce; Iván Esquivel «Plaztikk»; Sandra Gamarra; Gilda Mantilla; Gustavo Buntinx; Mirko Lauer; Augusto del Valle; Juan Javier Salazar; Eduardo Tokeshi; Colectivo Sociedad Civil; ENBA; Museo de Arte de Lima; Bienal de Lima; ICAA-MFAH</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Capítulo que reflexiona sobre la historia de las colecciones del Museo de Arte de Lima (MALI) desde su fundación en 1961 para interrogar la propia categoría de "museo de arte". Kusunoki y Lerner parten de la condición fundacional del MALI: nacido tardíamente frente a otros museos latinoamericanos, sin conexión con centros de enseñanza y configurado por el azar de donaciones como la vasta y heterogénea Memoria Prado. Esa amplitud material, argumentan, contenía en estado latente la posibilidad de cuestionar cómo las narrativas nacionales se proyectan sobre el pasado. El eje conceptual es la tensión entre "arte culto" y "arte popular", categoría esta última formulada en los años veinte desde el indigenismo de Sabogal y cargada de una ficción de autenticidad vernácula. El estudio de caso central es la incorporación en 2017 de la serie Piraq Causa —31 tablas de Sarhua de la ADAPS, comisionadas por Peter Gaupp, que narran la violencia de Sendero Luminoso y los Sinchis en Ayacucho—, que complejizó el eje de los "años de violencia" (junto a Taller N.N., Wiesse, Villares) y obligó a reconocer las tablas como práctica intersticial entre lo rural, urbano, tradicional y contemporáneo. La tesis sostiene que integrar tales obras no debe significar instalarlas en el espacio "atemporal" del arte, sino desmantelar la estructura dicotómica de clase y etnia del campo artístico peruano, preservando su carácter ambivalente. Reseña además el eje amazónico (Brus Rubio, 2014-2015), la gestión de Natalia Majluf (1995-2018) y las exposiciones Amazonías, Otras historias posibles (2019) e Imaginarios contemporáneos (2021-2022), proponiendo una política de colección que reconstruya constelaciones históricamente situadas y transformables.</t>
+          <t>Ensayo de Rodrigo Quijano fechado «Noviembre, 2001», texto del catálogo de la muestra colectiva «Puntos Cardinales» (cuatro artistas: Fernando Bryce, Iván Esquivel «Plaztikk», Sandra Gamarra y Gilda Mantilla). Titulado «¿De qué puntos cardinales hablan? Anotaciones sobre la última década en las artes visuales peruanas», ofrece un balance de los años noventa organizado en doce secciones numeradas. Su hilo es que la década consolidó una orientación del arte contemporáneo local a la vez que se perdió «un norte definido»: la entrada abrupta de la escena al «orden internacional» y a un «mercado simbólico consolidado de la región» tras años de aislamiento, bajo la dictadura de Fujimori (1990-2000). Rastrea el fin de la «modernidad alternativa» anclada en lo popular (con referencias a Lauer y su «Teoría de las Raíces Nacionales» y a Buntinx), la represión de los colectivos jóvenes (el grupo Huayco como paradigma, N.N. «diezmado» y Alfredo Márquez encarcelado bajo falsos cargos de terrorismo) y la «reinstitucionalización» privada (MALI, Centro de Artes Visuales, concursos y bienales auspiciados por el sector privado, Bienal de Lima desde 1997). Analiza en detalle a los cuatro artistas y comenta la crisis de la ENBA (intervenida por la dictadura), los «vladivideos», La Cantuta, Barrios Altos y el «Lava la bandera» del Colectivo Sociedad Civil (2000). Cierra afirmando que «la escena crítica es proporcionalmente precaria e invisible». Fuente primaria sobre la escena limeña de los noventa; digitalizada por el ICAA-MFAH (registro 1146549), con OCR muy dañado.</t>
         </is>
       </c>
     </row>
@@ -1566,27 +1566,27 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Lauer, Mirko - Arte al paso, Tome uno (1980) [volante Galería Forum, E.P.S. Huayco].md</t>
+          <t>ICAA-1272963.pdf</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>1980 (exposición Arte al paso, E.P.S. Huayco; contexto de la plástica joven peruana de fin de los años 70)</t>
+          <t>Debate sobre arte, doctrina y nacionalismo; revisión de las revoluciones cristiana, francesa, rusa y mexicana; c. décadas de 1940-1950</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Volante/panfleto de exposición, mayo de 1980 (Galería Forum, Lima); transcripción manual de fotografía, 2026</t>
+          <t>Artículo de prensa (Suplemento Dominical de El Comercio, Lima), c. 1957 (s/f exacta); digitalizado por ICAA-MFAH</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Mirko Lauer (texto); E.P.S. Huayco; María Luy; Francisco Mariotti; Charo Noriega; Juan Javier Salazar; Mariela Zevallos; Guillermo Orbegoso; Roberto Cores; Galería Forum</t>
+          <t>J. Nahuaca (seudónimo); Moisés Laymito; Gladys Zender; César Vallejo; Wilhelm Worringer; Arnold Hauser; Nicolai Hartmann; Charles Lalo; Jacques-Louis David; Kazimir Malevich; Wassily Kandinsky; Marc Chagall; El Comercio (Suplemento Dominical); ICAA-MFAH</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Volante o panfleto bifronte («Arte al paso» / «Tome uno») escrito por Mirko Lauer para acompañar la exposición homónima del colectivo E.P.S. Huayco en la Galería Forum de Lima (mayo de 1980); el proyecto reúne a María Luy, Francisco Mariotti, Charo Noriega, Juan Javier Salazar y Mariela Zevallos, con fotografías de Guillermo Orbegoso y Roberto Cores. El texto, organizado como una serie de definiciones anafóricas («Arte al paso: …»), es un manifiesto programático del no-objetualismo peruano y del arte crítico. Lauer presenta la obra como una «contestación» que combina serigrafía, detritus industriales, fórmulas teóricas, fotos y «expendio de salchipapas» para sostener que «la realidad del arte es más compleja que la realidad de las 'Bellas Artes'». Articula tres operaciones críticas: contra el mercado y las galerías como «escaparates» de la transacción comercial; contra los «métodos religioso-expresionistas» que enseñan a «sentir y no pensar»; y contra «una falsa modernidad de importación», rematando con la consigna que se volvería célebre: «Sólo lo popular es realmente moderno hoy en el Perú». Reivindica el trabajo colectivo frente al «aislamiento» y el «desamparo teórico» del plástico joven, propone un «ejercicio ecológico» que revela el «cordón umbilical» entre los desechos de la ciudad y su arte, y ancla la práctica en «esa realidad fundamental del arte en América Latina que es la miseria». Contra el «arte bobo», postula un arte popular, político y antipublicitario. Constituye una fuente primaria clave para la historia del arte crítico y no-objetual peruano de fines de los años setenta e inicios de los ochenta.</t>
+          <t>Segunda entrega del ensayo de J. Nahuaca, titulada "Ideas doctrinarias y la pintura", publicada en el Suplemento Dominical de El Comercio de Lima (fines de los cincuenta) y archivada en el ICAA-MFAH. Continúa la reflexión sobre las fuerzas que tensionan el arte peruano, distinguiendo entre energías subyacentes -lentas, sentimentales, nacionalizadoras, orientadas a la peruanidad- y fuerzas dinámicas que importan sistemas político-sociales para materializarlos de inmediato, sometiendo el arte a los valores sociales mediante una estética "demagógica y a la vez conservadora". El objeto central es la relación entre pintura e ideas doctrinarias, examinada a través de un recorrido histórico por cuatro revoluciones: la cristiana (que renuncia al arte pagano y desemboca en la iconoclasia), la francesa (que no crea estilo sino que adopta el clasicismo de David, oficializado por Napoleón), la rusa (que tras aliarse con la vanguardia -Malevich, Kandinsky, Chagall- recae en el realismo heroico reaccionario) y la mexicana (nacida sin doctrina, expresiva y muralista, que crea el mito de la revolución cumplida). El marco teórico cita a Worringer, Hauser, Nicolai Hartmann y Charles Lalo, y disuelve la antinomia forma-contenido cara a la estética marxista. Nahuaca argumenta que ninguna revolución ha mejorado ni creado un arte, que este pertenece a individuos y la colectividad solo lo usufructúa, y aboga por "desclasificar" la élite estética -verdadera valoradora- frente al monopolio de las clases dirigentes. Denuncia un "terrorismo en pintura" que exige conciencia social y concluye que el ímpetu nacionalizador peruano ha derivado en un mal menor: la peruanización de la iconografía como fin artístico. Incluye notas sobre el escultor Moisés Laymito y un retrato de Gladys Zender.</t>
         </is>
       </c>
     </row>
@@ -1598,27 +1598,27 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. (ed.) - Hay algo incomestible en la garganta. Poéticas antipatriarcales y nueva escena en los años noventa (2021) [catálogo ICPNA].md</t>
+          <t>ICPNA Catalogo Bellas Artes FINAL.pdf</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>1988-2002</t>
+          <t>1918-2018</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de exposición, 2021</t>
+          <t>Catálogo de exposición / libro institucional, noviembre de 2018</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López (curaduría); Issela Ccoyllo; Carmen Ilizarbe; Susana Torres; María Eugenia Yllia; Montserrat Álvarez; Irene Rojas; Elena Tejada-Herrera; Natalia Iguíñiz; Flavia Gandolfo; Movimiento Manuela Ramos / TAFOS; ICPNA</t>
+          <t>Escuela Nacional Superior Autónoma de Bellas Artes del Perú (ENSABAP); Instituto Cultural Peruano Norteamericano (ICPNA); Max Hernández Calvo; Augusto del Valle Cárdenas; Rocío Corcuera Ríos; Víctor Mejía Ticona; Miguel Sánchez Flores; Luis Carlos Valdez Espinoza; Roberto Hoyle; Municipalidad de Miraflores; E.P.S. Huayco; Grupo Paréntesis</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Catálogo bilingüe de la exposición homónima curada por Miguel A. López en el ICPNA de Lima con motivo del Bicentenario, que reúne más de doscientas obras de cerca de noventa creadoras, colectivas y talleres para examinar la producción visual y las transformaciones sociopolíticas peruanas entre 1988 y 2002. Su tesis central sostiene que, al cierre del siglo XX, fueron las mujeres y los cuerpos feminizados quienes reorientaron el rumbo del arte, desplegando lo que López denomina «poéticas antipatriarcales»: vocabularios estéticos surgidos para enfrentar una misoginia naturalizada y la violencia colonial, racial y patriarcal. El marco conceptual articula feminismo, crítica al neoliberalismo (el «hechizo» de la privatización y el individualismo), teoría social del arte y una lectura de clase del campo cultural, rechazando una absorción de la heterogeneidad bajo la categoría occidental de «arte». El proyecto yuxtapone deliberadamente circuitos antagónicos: obras de galerías, museos y bienales junto a arpilleras de asociaciones de mujeres y clubes de madres, los Talleres de Fotografía Social (TAFOS) y el proyecto Mercomujer del Movimiento Manuela Ramos. Se organiza en diez ejes temáticos (autorrepresentación, misoginia, deseo y disidencia de género, políticas de cuidado, acción colectiva, poder androcéntrico, reciprocidad, cuerpos gestantes, pieles e hilos, violencia política) y ensayos complementarios de Susana Torres, Issela Ccoyllo, María Eugenia Yllia y Carmen Ilizarbe. Su aporte reside en construir una genealogía transfeminista que rescata prácticas invisibilizadas —arpilleristas migrantes, artistas indígenas y campesinas, transformismo, autogestión— y las inscribe como agentes decisivas de la reconfiguración de la esfera pública peruana frente a la dictadura fujimorista.</t>
+          <t>El volumen documenta 'Un siglo de arte desde la Escuela Nacional', ciclo de cuatro exposiciones organizado en 2018 para el centenario (1918-2018) de la Escuela Nacional Superior Autónoma de Bellas Artes del Perú (ENSABAP), coeditado con el Instituto Cultural Peruano Norteamericano (ICPNA). Bajo la curaduría general de Max Hernández Calvo y Augusto del Valle Cárdenas, con Rocío Corcuera, Víctor Mejía y Miguel Sánchez, el proyecto busca construir memoria institucional y revisar cien años de producción y pedagogía bellasartina, articulándola con la sociedad contemporánea. Las muestras se distribuyeron en cuatro sedes (galerías ICPNA Juan Pardo Heeren y Germán Krüger Espantoso, y salas municipales de Miraflores). 'Bellas Artes: voz y huella de los egresados' (Corcuera) parte de cuarenta entrevistas a egresados de 1951 a 2017 —de Ella Krebs a Andrés Yaques— y una línea de tiempo que vincula formación, testimonio y obra estudiantil. 'Del individuo al ser social' (Sánchez) estudia los colectivos surgidos desde los años setenta (E.P.S. Huayco, Paréntesis, Signo x Signo, C.H.O.L.O., entre otros) como gesto político frente al modelo del artista individual. 'Espacio público' (Mejía) analiza el centro de Lima como insumo estético y campo de intervención. 'Una trayectoria de imágenes' (Hernández Calvo y Del Valle) emplea los géneros académicos —bodegón, paisaje, retrato— para pensar el tránsito del arte moderno al contemporáneo. La tesis transversal cuestiona la narrativa figurativo/abstracto de la modernidad e introduce la pregunta por el ícono, uniendo lo global con las tradiciones locales y artesanales, para otorgar 'carta de ciudadanía' a prácticas invisibilizadas desde una escuela pública.</t>
         </is>
       </c>
     </row>
@@ -1630,27 +1630,27 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - How Do We Know What Latin American Conceptualism Looks Like?.md</t>
+          <t>Kusunoki y Lerner - Reconsidering the «art museum». Some reflections on the history of the MALI collections (2026) [Unmaking to Make, cap. 5].md</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>años 60-70 (con foco en 1968: Tucumán Arde)</t>
+          <t>1961-2022 (con referencias desde época prehispánica y los años 20)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico (Afterall), ca. 2010</t>
+          <t>Capítulo de libro, 2026</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Mari Carmen Ramírez; Luis Camnitzer; Jane Farver; Rachel Weiss; Paul B. (Beatriz) Preciado; Graciela Carnevale; Ana Longoni; Fernando Davis; Eduardo Costa; Roberto Jacoby; Queens Museum of Art / MoMA / Red Conceptualismos del Sur</t>
+          <t>Ricardo Kusunoki; Sharon Lerner; Museo de Arte de Lima (MALI); Natalia Majluf; Gabriela Germaná; Gredna Landolt; ADAPS / Piraq Causa; Brus Rubio Churay; José Sabogal; Con/Vida; Matadero Madrid / ARCO; Julieta González</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Ensayo historiográfico de Miguel A. López que problematiza cómo se ha construido y estabilizado la categoría «conceptualismo latinoamericano». Su objeto de estudio son los dispositivos discursivos y expositivos que fijaron una imagen canónica de la producción crítica de los años sesenta y setenta, tomando como bisagras la muestra «Global Conceptualism: Points of Origin» (Queens Museum, 1999) y el ensayo fundacional «Blueprint Circuits» (1993) de Mari Carmen Ramírez. El marco conceptual proviene de una crítica queer de la representación: siguiendo a Paul B. Preciado y a Guattari, López contrapone una «cartografía de identidades» —que rastrea, clasifica y verifica obras conceptuales— a una «cartografía crítica» que expone las relaciones de poder y las tecnologías de producción de subjetividad implicadas en el acto de historizar. Argumenta que la distinción binaria entre un conceptualismo «analítico» anglosajón (Kosuth) y uno «ideológico» latinoamericano, consolidada por Ramírez y repetida por Osborne y Alberro, reinscribe la lógica centro/periferia que dice combatir y fija un estereotipo de arte subversivo. El texto examina la mitificación de «Tucumán Arde» (1968) y su recuperación en la exposición «Inventario 1965-1975. Archivo Graciela Carnevale» (Rosario, 2008), primer experimento curatorial de la Red Conceptualismos del Sur, que activa el archivo para desmontar la narrativa única. Recupera conceptos «menores» (desmaterialización de Masotta, no-objetualismo de Acha, deshabituación de Carreira) y cierra con la pieza de Eduardo Costa: su aporte es proponer una historiografía infiel, anacrónica y desestabilizadora que traicione las certezas del relato consensual.</t>
+          <t>Capítulo que reflexiona sobre la historia de las colecciones del Museo de Arte de Lima (MALI) desde su fundación en 1961 para interrogar la propia categoría de "museo de arte". Kusunoki y Lerner parten de la condición fundacional del MALI: nacido tardíamente frente a otros museos latinoamericanos, sin conexión con centros de enseñanza y configurado por el azar de donaciones como la vasta y heterogénea Memoria Prado. Esa amplitud material, argumentan, contenía en estado latente la posibilidad de cuestionar cómo las narrativas nacionales se proyectan sobre el pasado. El eje conceptual es la tensión entre "arte culto" y "arte popular", categoría esta última formulada en los años veinte desde el indigenismo de Sabogal y cargada de una ficción de autenticidad vernácula. El estudio de caso central es la incorporación en 2017 de la serie Piraq Causa —31 tablas de Sarhua de la ADAPS, comisionadas por Peter Gaupp, que narran la violencia de Sendero Luminoso y los Sinchis en Ayacucho—, que complejizó el eje de los "años de violencia" (junto a Taller N.N., Wiesse, Villares) y obligó a reconocer las tablas como práctica intersticial entre lo rural, urbano, tradicional y contemporáneo. La tesis sostiene que integrar tales obras no debe significar instalarlas en el espacio "atemporal" del arte, sino desmantelar la estructura dicotómica de clase y etnia del campo artístico peruano, preservando su carácter ambivalente. Reseña además el eje amazónico (Brus Rubio, 2014-2015), la gestión de Natalia Majluf (1995-2018) y las exposiciones Amazonías, Otras historias posibles (2019) e Imaginarios contemporáneos (2021-2022), proponiendo una política de colección que reconstruya constelaciones históricamente situadas y transformables.</t>
         </is>
       </c>
     </row>
@@ -1662,27 +1662,27 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - Los feminismos van a vencer. Una introducción [con presentación de Claudia Salazar Jiménez, dic. 2018].md</t>
+          <t>Lauer, Mirko - Arte al paso, Tome uno (1980) [volante Galería Forum, E.P.S. Huayco].md</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>años 60-90 (textos escritos 2012-2018; activismo 2015-2018)</t>
+          <t>1980 (exposición Arte al paso, E.P.S. Huayco; contexto de la plástica joven peruana de fin de los años 70)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Introducción de libro, 2018</t>
+          <t>Volante/panfleto de exposición, mayo de 1980 (Galería Forum, Lima); transcripción manual de fotografía, 2026</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Claudia Salazar Jiménez; Rita Segato; Frantz Fanon; Julia Bryan-Wilson; Gladys Tzul Tzul; Aníbal Quijano; Paul B. Preciado; Giuseppe Campuzano; Víctor Manuel Rodríguez; TEOR/éTica / MACBA</t>
+          <t>Mirko Lauer (texto); E.P.S. Huayco; María Luy; Francisco Mariotti; Charo Noriega; Juan Javier Salazar; Mariela Zevallos; Guillermo Orbegoso; Roberto Cores; Galería Forum</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Texto introductorio de López al libro que reúne sus ensayos sobre poéticas antipatriarcales (escritos entre 2012 y 2018), precedido por una presentación de la escritora Claudia Salazar Jiménez. Su tesis define los feminismos no como una identidad ni un periodo, sino como una «metodología para mirar» y un método de investigación afectivo: una política del afecto, la escucha y la resistencia colectiva que redefine el horizonte de acción y desconfía del esencialismo identitario. El marco conceptual entrelaza la «pedagogía de la crueldad» y el «mandato de la masculinidad» de Rita Segato, la distinción de Fanon entre «zona del ser» y «zona del no-ser», la «colonialidad del poder» de Aníbal Quijano y el «modelo metodológico afectivo» de Julia Bryan-Wilson, junto a referencias a Gladys Tzul Tzul y Paul B. Preciado. López sostiene que el arte, la performance y la escritura funcionan como refugio y resistencia frente a la exclusión, y que la tarea no es incorporar episodios omitidos a un inventario, sino analizar las condiciones políticas, materiales y afectivas que hacen emerger ciertas representaciones. Discute críticamente el rol de los museos como lugares de disputa capaces de redefinir la esfera pública, apoyándose en su experiencia en el MACBA y en la dirección colectiva de TEOR/éTica. Situado geopolíticamente en Lima pero atento a sus ausencias (la Amazonía, las provincias, el centralismo), el ensayo propone una genealogía transfeminista de la cultura visual que reactive «parientes extraviados» y reorganice la historia del arte como reserva de sororidad y alianzas.</t>
+          <t>Volante o panfleto bifronte («Arte al paso» / «Tome uno») escrito por Mirko Lauer para acompañar la exposición homónima del colectivo E.P.S. Huayco en la Galería Forum de Lima (mayo de 1980); el proyecto reúne a María Luy, Francisco Mariotti, Charo Noriega, Juan Javier Salazar y Mariela Zevallos, con fotografías de Guillermo Orbegoso y Roberto Cores. El texto, organizado como una serie de definiciones anafóricas («Arte al paso: …»), es un manifiesto programático del no-objetualismo peruano y del arte crítico. Lauer presenta la obra como una «contestación» que combina serigrafía, detritus industriales, fórmulas teóricas, fotos y «expendio de salchipapas» para sostener que «la realidad del arte es más compleja que la realidad de las 'Bellas Artes'». Articula tres operaciones críticas: contra el mercado y las galerías como «escaparates» de la transacción comercial; contra los «métodos religioso-expresionistas» que enseñan a «sentir y no pensar»; y contra «una falsa modernidad de importación», rematando con la consigna que se volvería célebre: «Sólo lo popular es realmente moderno hoy en el Perú». Reivindica el trabajo colectivo frente al «aislamiento» y el «desamparo teórico» del plástico joven, propone un «ejercicio ecológico» que revela el «cordón umbilical» entre los desechos de la ciudad y su arte, y ancla la práctica en «esa realidad fundamental del arte en América Latina que es la miseria». Contra el «arte bobo», postula un arte popular, político y antipublicitario. Constituye una fuente primaria clave para la historia del arte crítico y no-objetual peruano de fines de los años setenta e inicios de los ochenta.</t>
         </is>
       </c>
     </row>
@@ -1694,27 +1694,27 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - Parientes extraviados, Cuerpo vehículo político y A contratiempo. Tres ensayos sobre poéticas antipatriarcales.md</t>
+          <t>López, Miguel A. (ed.) - Hay algo incomestible en la garganta. Poéticas antipatriarcales y nueva escena en los años noventa (2021) [catálogo ICPNA].md</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>años 60-80 (con proyección al presente)</t>
+          <t>1988-2002</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Capítulos de libro, 2019</t>
+          <t>Catálogo de exposición, 2021</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Teresa Burga; Gloria Gómez-Sánchez; Cristina Portocarrero; Victoria Santa Cruz; Johanna Hamann; Tilsa Tsuchiya; Marisa Godínez; María T-Ta (María Roncal); Grupo Chaclacayo; ALIMUPER / Movimiento Manuela Ramos / Centro Flora Tristán</t>
+          <t>Miguel A. López (curaduría); Issela Ccoyllo; Carmen Ilizarbe; Susana Torres; María Eugenia Yllia; Montserrat Álvarez; Irene Rojas; Elena Tejada-Herrera; Natalia Iguíñiz; Flavia Gandolfo; Movimiento Manuela Ramos / TAFOS; ICPNA</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Conjunto de tres ensayos de López que trazan una genealogía de poéticas antipatriarcales en el arte peruano entre los años sesenta y ochenta, entendidas como «parientes extraviados» de las luchas feministas y sexodisidentes actuales. «Parientes extraviados» reconstruye la contribución de las artistas mujeres al experimentalismo: las ambientaciones y objetos de Teresa Burga y Gloria Gómez-Sánchez en el grupo Arte Nuevo (1966-1968), que desmantelaban el régimen masculino de la mirada; el tránsito de Cristina Portocarrero del arte a la militancia en ALIMUPER; y la revaloración de las artes de tradición andina (Apolonia Dorregaray) bajo el velasquismo. «Cuerpo, vehículo político» analiza cómo diversas creadoras abandonaron pintura y escultura para usar el propio cuerpo como crítica: el «Antiballet» de Yvonne von Mollendorff, el «Autorretrato» clínico de Burga (1972), la declamación antirracista «Me gritaron negra» de Victoria Santa Cruz, las «Barrigas» de Johanna Hamann y la gráfica militante de Marisa Godínez para Flora Tristán. Aborda además la teatralidad, el travestismo y lo performativo de los ochenta —Grupo Chaclacayo, Jaime Higa, la escena drag documentada por Flavia Gandolfo, la punk María T-Ta, Támira Bassallo, Susana Torres— como respuestas a una guerra tanto armada como misógina y homofóbica. El tercer ensayo, «A contratiempo», explora las «cronodisidencias» de Burga y su temporalidad improductiva del dibujo. El marco conceptual moviliza teoría feminista y queer (Preciado, Bryan-Wilson, Richard); su aporte es reinscribir prácticas borradas como antagonismo estético-político y desmentir el diagnóstico de su supuesta inexistencia.</t>
+          <t>Catálogo bilingüe de la exposición homónima curada por Miguel A. López en el ICPNA de Lima con motivo del Bicentenario, que reúne más de doscientas obras de cerca de noventa creadoras, colectivas y talleres para examinar la producción visual y las transformaciones sociopolíticas peruanas entre 1988 y 2002. Su tesis central sostiene que, al cierre del siglo XX, fueron las mujeres y los cuerpos feminizados quienes reorientaron el rumbo del arte, desplegando lo que López denomina «poéticas antipatriarcales»: vocabularios estéticos surgidos para enfrentar una misoginia naturalizada y la violencia colonial, racial y patriarcal. El marco conceptual articula feminismo, crítica al neoliberalismo (el «hechizo» de la privatización y el individualismo), teoría social del arte y una lectura de clase del campo cultural, rechazando una absorción de la heterogeneidad bajo la categoría occidental de «arte». El proyecto yuxtapone deliberadamente circuitos antagónicos: obras de galerías, museos y bienales junto a arpilleras de asociaciones de mujeres y clubes de madres, los Talleres de Fotografía Social (TAFOS) y el proyecto Mercomujer del Movimiento Manuela Ramos. Se organiza en diez ejes temáticos (autorrepresentación, misoginia, deseo y disidencia de género, políticas de cuidado, acción colectiva, poder androcéntrico, reciprocidad, cuerpos gestantes, pieles e hilos, violencia política) y ensayos complementarios de Susana Torres, Issela Ccoyllo, María Eugenia Yllia y Carmen Ilizarbe. Su aporte reside en construir una genealogía transfeminista que rescata prácticas invisibilizadas —arpilleristas migrantes, artistas indígenas y campesinas, transformismo, autogestión— y las inscribe como agentes decisivas de la reconfiguración de la esfera pública peruana frente a la dictadura fujimorista.</t>
         </is>
       </c>
     </row>
@@ -1726,27 +1726,27 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Mesa - Arte contemporáneo peruano. Portocarrero, Aramburu y Lerner (2022) [MALBA].transcripcion.md</t>
+          <t>López, Miguel A. - How Do We Know What Latin American Conceptualism Looks Like?.md</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>1930-2022 (con énfasis en 1976-2022)</t>
+          <t>años 60-70 (con foco en 1968: Tucumán Arde)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Transcripción de mesa redonda (MALBA/MALVA), 2022</t>
+          <t>Artículo académico (Afterall), ca. 2010</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Florencia Portocarrero; Iosu Aramburu; Verónica Rossi; Ana Teresa Barboza; Mirko Lauer; Joaquín López Antay; Miguel Aguirre; Elvia Paucar; Centro de Textiles Tradicionales del Cusco; MALI</t>
+          <t>Miguel A. López; Mari Carmen Ramírez; Luis Camnitzer; Jane Farver; Rachel Weiss; Paul B. (Beatriz) Preciado; Graciela Carnevale; Ana Longoni; Fernando Davis; Eduardo Costa; Roberto Jacoby; Queens Museum of Art / MoMA / Red Conceptualismos del Sur</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Transcripción (borrador sin refinar) de una mesa redonda organizada en torno a la exposición 'Tejer las Piedras' de Ana Teresa Barboza, que toma el pulso a los debates del arte contemporáneo peruano actual, con foco en la relación entre arte y artesanía. Sharon Lerner abre con un recorrido por veinte años de la obra de Barboza, desde el bordado autobiográfico de cuerpos y heridas —leído por Gabriela Germaná y Augusto del Valle como inversión de la representación sexista— hacia un trabajo colaborativo con tejido, telar de cintura y tintes naturales que reflexiona sobre paisaje, sostenibilidad y territorio, situándolo en la tradición anglosajona del craft y en la reinserción de lo personal, según Whitney Chadwick, característica del feminismo desde los setenta. Portocarrero y Aramburu estructuran su intervención con los tres 'universos estéticos' de Mirko Lauer (precolombino, erudito/bellas artes, tradicional/popular), entendidos como compartimentos estancos ligados a una estructura colonial y racista, y examinan sus cruces históricos: el Instituto de Arte Peruano indigenista, la apropiación de lo prehispánico en los sesenta, el escándalo del Premio Nacional a Joaquín López Antay (1976). El marco conceptual sostiene que, a diferencia de aquel premio otorgado por un jurado, artistas indígenas contemporáneos como Venuca Evanán y Chonon Bensho hoy postulan conscientemente e ingresan por agencia propia a los circuitos del arte contemporáneo. Se analizan la colaboración de largo aliento entre Miguel Aguirre y la tejedora Elvia Paucar y el proyecto Ser Payay en Cusco, como casos de 'vocabularios colaborados' que problematizan la coautoría, la mediación y las lógicas de mercado diferenciadas entre arte y artesanía.</t>
+          <t>Ensayo historiográfico de Miguel A. López que problematiza cómo se ha construido y estabilizado la categoría «conceptualismo latinoamericano». Su objeto de estudio son los dispositivos discursivos y expositivos que fijaron una imagen canónica de la producción crítica de los años sesenta y setenta, tomando como bisagras la muestra «Global Conceptualism: Points of Origin» (Queens Museum, 1999) y el ensayo fundacional «Blueprint Circuits» (1993) de Mari Carmen Ramírez. El marco conceptual proviene de una crítica queer de la representación: siguiendo a Paul B. Preciado y a Guattari, López contrapone una «cartografía de identidades» —que rastrea, clasifica y verifica obras conceptuales— a una «cartografía crítica» que expone las relaciones de poder y las tecnologías de producción de subjetividad implicadas en el acto de historizar. Argumenta que la distinción binaria entre un conceptualismo «analítico» anglosajón (Kosuth) y uno «ideológico» latinoamericano, consolidada por Ramírez y repetida por Osborne y Alberro, reinscribe la lógica centro/periferia que dice combatir y fija un estereotipo de arte subversivo. El texto examina la mitificación de «Tucumán Arde» (1968) y su recuperación en la exposición «Inventario 1965-1975. Archivo Graciela Carnevale» (Rosario, 2008), primer experimento curatorial de la Red Conceptualismos del Sur, que activa el archivo para desmontar la narrativa única. Recupera conceptos «menores» (desmaterialización de Masotta, no-objetualismo de Acha, deshabituación de Carreira) y cierra con la pieza de Eduardo Costa: su aporte es proponer una historiografía infiel, anacrónica y desestabilizadora que traicione las certezas del relato consensual.</t>
         </is>
       </c>
     </row>
@@ -1758,27 +1758,27 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Mesa - Coleccionando desde la institución (2025) [Charlas de colección, Foro Pinta Lima].transcripcion.md</t>
+          <t>López, Miguel A. - Los feminismos van a vencer. Una introducción [con presentación de Claudia Salazar Jiménez, dic. 2018].md</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>1960s-2025 (con eje en 2006-2025)</t>
+          <t>años 60-90 (textos escritos 2012-2018; activismo 2015-2018)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Transcripción de conversatorio (Foro Pinta Lima 2025), 2025</t>
+          <t>Introducción de libro, 2018</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Pablo León de la Barra; Sharon Lerner; Manuel Segade; MALI; Museo Reina Sofía; Museo Guggenheim; Comité de Adquisiciones de Arte Contemporáneo del MALI; Suset Sánchez; Amanda de la Garza; Tatiana Cuevas; Fundación Museo Reina Sofía</t>
+          <t>Miguel A. López; Claudia Salazar Jiménez; Rita Segato; Frantz Fanon; Julia Bryan-Wilson; Gladys Tzul Tzul; Aníbal Quijano; Paul B. Preciado; Giuseppe Campuzano; Víctor Manuel Rodríguez; TEOR/éTica / MACBA</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Transcripción (borrador) del conversatorio 'Coleccionando desde la institución' del Foro Pinta Lima 2025, moderado por Pablo León de la Barra (Guggenheim), que confronta dos modelos museales públicos: el MALI de Lima y el Museo Reina Sofía de Madrid. La tesis compartida es que coleccionar implica un pensamiento crítico que puede cuestionar el canon, reparar asimetrías históricas de género, raza e identidad y llenar vacíos. Sharon Lerner expone la trayectoria del Comité de Adquisiciones de Arte Contemporáneo del MALI (casi veinte años, modelado sobre el Latin American Acquisitions Committee de la Tate), la curaduría contemporánea iniciada por Tatiana Cuevas en 2008, y el trabajo 'trenzado' entre colección histórica y contemporánea que atraviesa exposiciones como Arte al Paso, Amazonías y Otras historias posibles, y la reestructuración pospandemia con el programa Salas Abiertas. Detalla la visibilización de artistas amazónicos e indígenas (Sara Flores, Chonon Bensho, Venuca Evanán), la incorporación del textil y proyectos como Línea de Vida de Giuseppe Campuzano, junto a comisiones y trabajo comunitario con Cantagallo. Manuel Segade analiza la dimensión colonial del Reina Sofía —cuya colección latinoamericana se inauguró en 1992— y las condiciones estructurales, funcionariales y presupuestarias que la condicionan, citando las preguntas ontológicas de Suset Sánchez y el Instituto Cader de arte centroamericano como vía de restitución frente al extractivismo cultural. El diálogo aborda el rol de los públicos, la crispación política, la censura, el cierre del Lugar de la Memoria y la misión histórica del museo como plataforma de tensiones críticas de la sociedad civil.</t>
+          <t>Texto introductorio de López al libro que reúne sus ensayos sobre poéticas antipatriarcales (escritos entre 2012 y 2018), precedido por una presentación de la escritora Claudia Salazar Jiménez. Su tesis define los feminismos no como una identidad ni un periodo, sino como una «metodología para mirar» y un método de investigación afectivo: una política del afecto, la escucha y la resistencia colectiva que redefine el horizonte de acción y desconfía del esencialismo identitario. El marco conceptual entrelaza la «pedagogía de la crueldad» y el «mandato de la masculinidad» de Rita Segato, la distinción de Fanon entre «zona del ser» y «zona del no-ser», la «colonialidad del poder» de Aníbal Quijano y el «modelo metodológico afectivo» de Julia Bryan-Wilson, junto a referencias a Gladys Tzul Tzul y Paul B. Preciado. López sostiene que el arte, la performance y la escritura funcionan como refugio y resistencia frente a la exclusión, y que la tarea no es incorporar episodios omitidos a un inventario, sino analizar las condiciones políticas, materiales y afectivas que hacen emerger ciertas representaciones. Discute críticamente el rol de los museos como lugares de disputa capaces de redefinir la esfera pública, apoyándose en su experiencia en el MACBA y en la dirección colectiva de TEOR/éTica. Situado geopolíticamente en Lima pero atento a sus ausencias (la Amazonía, las provincias, el centralismo), el ensayo propone una genealogía transfeminista de la cultura visual que reactive «parientes extraviados» y reorganice la historia del arte como reserva de sororidad y alianzas.</t>
         </is>
       </c>
     </row>
@@ -1790,27 +1790,27 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Ministerio de Cultura - Contemporáneos. Cinco mil años de visualidad peruana (2019) [catálogo, Perú país invitado ARCOmadrid].md</t>
+          <t>López, Miguel A. - Parientes extraviados, Cuerpo vehículo político y A contratiempo. Tres ensayos sobre poéticas antipatriarcales.md</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>200 a.C.-2019 (Nasca, virreinato y arte contemporáneo reciente)</t>
+          <t>años 60-80 (con proyección al presente)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Catálogo institucional de feria/exposición (ARCOmadrid), 2019</t>
+          <t>Capítulos de libro, 2019</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Ministerio de Cultura del Perú; Jorge Villacorta; Sharon Lerner; Fietta Jarque; Miguel A. López; Teresa Burga; Fernando Bryce; Sandra Gamarra; Natalia Majluf; MALI; ARCOmadrid / IFEMA; Museo Reina Sofía / Museo del Prado</t>
+          <t>Miguel A. López; Teresa Burga; Gloria Gómez-Sánchez; Cristina Portocarrero; Victoria Santa Cruz; Johanna Hamann; Tilsa Tsuchiya; Marisa Godínez; María T-Ta (María Roncal); Grupo Chaclacayo; ALIMUPER / Movimiento Manuela Ramos / Centro Flora Tristán</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Catálogo institucional de la participación de Perú como País Invitado en ARCOmadrid 2019, que reúne los textos curatoriales del stand del Estado, la zona de galerías y el programa oficial de más de treinta exposiciones y actividades en Madrid. El ensayo de Jorge Villacorta, 'Contemporáneos: cinco mil años de visualidad peruana', propone lo contemporáneo como actitud y coexistencia antes que como novedad, avanzando la hipótesis de que la contemporaneidad peruana es continuidad de una matriz cultural andino-amazónica con incrustaciones occidentales, un tiempo cíclico que supera categorías como arte popular o artesanía. Sharon Lerner, en 'Texto, tactibilidad y trama', encuadra la selección de galerías —que por primera vez combina representación local e internacional— como un corte no representativo de un 'arte nacional', destacando líneas transversales: el uso del texto, la cita y el archivo para desmontar discursos de la historia oficial; las tensiones del colonialismo y los criterios étnicos y de clase; la mirada al territorio y a lo extractivo; y la fragilidad táctil del textil, la arcilla y el cuerpo. El catálogo perfila a artistas como Teresa Burga, Rita Ponce de León, Ximena Garrido Lecca, Herbert Rodríguez, Fernando Bryce, Sandra Gamarra, Milagros de la Torre y Antonio Paucar, y documenta las conferencias curadas por Miguel A. López sobre el Bicentenario, la contemporaneidad andina, indígena y amazónica, y las transformaciones institucionales y de mercado. El programa oficial, presentado por Fietta Jarque, articula un relato de cinco mil años: Nasca, el Matrimonio de Martín de Loyola, Huamán Poma, la revista Amauta de Mariátegui, Amazonías y colecciones privadas (Hochschild, CIFO, Jan Mulder).</t>
+          <t>Conjunto de tres ensayos de López que trazan una genealogía de poéticas antipatriarcales en el arte peruano entre los años sesenta y ochenta, entendidas como «parientes extraviados» de las luchas feministas y sexodisidentes actuales. «Parientes extraviados» reconstruye la contribución de las artistas mujeres al experimentalismo: las ambientaciones y objetos de Teresa Burga y Gloria Gómez-Sánchez en el grupo Arte Nuevo (1966-1968), que desmantelaban el régimen masculino de la mirada; el tránsito de Cristina Portocarrero del arte a la militancia en ALIMUPER; y la revaloración de las artes de tradición andina (Apolonia Dorregaray) bajo el velasquismo. «Cuerpo, vehículo político» analiza cómo diversas creadoras abandonaron pintura y escultura para usar el propio cuerpo como crítica: el «Antiballet» de Yvonne von Mollendorff, el «Autorretrato» clínico de Burga (1972), la declamación antirracista «Me gritaron negra» de Victoria Santa Cruz, las «Barrigas» de Johanna Hamann y la gráfica militante de Marisa Godínez para Flora Tristán. Aborda además la teatralidad, el travestismo y lo performativo de los ochenta —Grupo Chaclacayo, Jaime Higa, la escena drag documentada por Flavia Gandolfo, la punk María T-Ta, Támira Bassallo, Susana Torres— como respuestas a una guerra tanto armada como misógina y homofóbica. El tercer ensayo, «A contratiempo», explora las «cronodisidencias» de Burga y su temporalidad improductiva del dibujo. El marco conceptual moviliza teoría feminista y queer (Preciado, Bryan-Wilson, Richard); su aporte es reinscribir prácticas borradas como antagonismo estético-político y desmentir el diagnóstico de su supuesta inexistencia.</t>
         </is>
       </c>
     </row>
@@ -1822,27 +1822,27 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Mitrovic - Extravíos de la forma. Vanguardia, modernismo popular y arte contemporáneo en Lima desde los 60 (2019).md</t>
+          <t>Mesa - Arte contemporáneo peruano. Portocarrero, Aramburu y Lerner (2022) [MALBA].transcripcion.md</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>1960-2018 (desde los sesenta hasta el presente)</t>
+          <t>1930-2022 (con énfasis en 1976-2022)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Libro académico, 2019 (Fondo Editorial FAU-PUCP)</t>
+          <t>Transcripción de mesa redonda (MALBA/MALVA), 2022</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Mijail Mitrovic; Gustavo Buntinx; Mirko Lauer; Sharon Lerner; Miguel A. López; Emilio Tarazona; Fernando de Szyszlo; E.P.S. Huayco; Taller NN; José Carlos Martinat; Museo de Arte de Lima (MALI); PUCP; Fredric Jameson</t>
+          <t>Sharon Lerner; Florencia Portocarrero; Iosu Aramburu; Verónica Rossi; Ana Teresa Barboza; Mirko Lauer; Joaquín López Antay; Miguel Aguirre; Elvia Paucar; Centro de Textiles Tradicionales del Cusco; MALI</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Ensayo de historia y teoría del arte que impugna el «relato convencional» sobre el arte contemporáneo en Lima, entendido como una fábula épica que narra el tránsito de la vanguardia de los sesenta al arte contemporáneo global mediante el «encuentro con lo popular». Desde un marco marxista-dialéctico (Adorno, Jameson, Bürger, Osborne, Lukács), Mitrovic reivindica la totalización y la periodización frente al historicismo posmoderno que celebra heterogeneidad y discontinuidad. Su tesis central es que la «desidealización» del arte —su reducción a hecho social e institucional— siguió en Lima una trayectoria específica: de la teoría de las raíces nacionales (Szyszlo, Lauer) y el altomodernismo, a la radicalización de la vanguardia bajo el velasquismo, que el autor conceptualiza como «modernismo popular» (E.P.S. Huayco, Paréntesis, la frase de Lauer «solo lo popular es moderno»). Con Sendero Luminoso y la crisis de los ochenta, la utopía colapsa y el arte se reorienta hacia la denuncia ética de la violencia, prolongada durante el fujimorato (Colectivo Sociedad Civil, «Lava la bandera»). El cambio de siglo consuma la «contemporaneización» mediante las Bienales de Lima y el mercado. El último capítulo analiza obras (Polanco, Guerra García, Huarcaya, Aguirre, Andrade Valdez, Martinat) para mostrar cómo lo popular deviene «neocostumbrismo» y «renta de monopolio»: sello local que certifica autenticidad cultural en el circuito global, mientras se evacúa el horizonte futuro y el «pueblo» se reduce a «población». Frente a la nostalgia y la reoligarquización simbólica, Mitrovic propone recuperar las potencialidades utópicas hoy reprimidas.</t>
+          <t>Transcripción (borrador sin refinar) de una mesa redonda organizada en torno a la exposición 'Tejer las Piedras' de Ana Teresa Barboza, que toma el pulso a los debates del arte contemporáneo peruano actual, con foco en la relación entre arte y artesanía. Sharon Lerner abre con un recorrido por veinte años de la obra de Barboza, desde el bordado autobiográfico de cuerpos y heridas —leído por Gabriela Germaná y Augusto del Valle como inversión de la representación sexista— hacia un trabajo colaborativo con tejido, telar de cintura y tintes naturales que reflexiona sobre paisaje, sostenibilidad y territorio, situándolo en la tradición anglosajona del craft y en la reinserción de lo personal, según Whitney Chadwick, característica del feminismo desde los setenta. Portocarrero y Aramburu estructuran su intervención con los tres 'universos estéticos' de Mirko Lauer (precolombino, erudito/bellas artes, tradicional/popular), entendidos como compartimentos estancos ligados a una estructura colonial y racista, y examinan sus cruces históricos: el Instituto de Arte Peruano indigenista, la apropiación de lo prehispánico en los sesenta, el escándalo del Premio Nacional a Joaquín López Antay (1976). El marco conceptual sostiene que, a diferencia de aquel premio otorgado por un jurado, artistas indígenas contemporáneos como Venuca Evanán y Chonon Bensho hoy postulan conscientemente e ingresan por agencia propia a los circuitos del arte contemporáneo. Se analizan la colaboración de largo aliento entre Miguel Aguirre y la tejedora Elvia Paucar y el proyecto Ser Payay en Cusco, como casos de 'vocabularios colaborados' que problematizan la coautoría, la mediación y las lógicas de mercado diferenciadas entre arte y artesanía.</t>
         </is>
       </c>
     </row>
@@ -1854,27 +1854,27 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Peralta - Lo que la Bienal de Lima se llevó. Balance a cinco años de su desactivación.md</t>
+          <t>Mesa - Coleccionando desde la institución (2025) [Charlas de colección, Foro Pinta Lima].transcripcion.md</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>1997-2003 (Bienales de Lima y su desactivación)</t>
+          <t>1960s-2025 (con eje en 2006-2025)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Artículo/ensayo de balance, ca. 2007-2008</t>
+          <t>Transcripción de conversatorio (Foro Pinta Lima 2025), 2025</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Juan Peralta; Luis Lama; Jorge Villacorta; Emilio Santisteban; Elena Tejada; Gustavo Buntinx; Alfonso Castrillón; Élida Román; Allora &amp; Calzadilla; Francis Alÿs; Cuauhtémoc Medina; Alberto Andrade; Luis Castañeda Lossio; Municipalidad Metropolitana de Lima; UCCI</t>
+          <t>Pablo León de la Barra; Sharon Lerner; Manuel Segade; MALI; Museo Reina Sofía; Museo Guggenheim; Comité de Adquisiciones de Arte Contemporáneo del MALI; Suset Sánchez; Amanda de la Garza; Tatiana Cuevas; Fundación Museo Reina Sofía</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Balance crítico sobre la desaparición de la Bienal de Lima, escrito por Juan Peralta a cinco años de su desactivación. El texto reconstruye el contexto político-cultural en que surgió el megaevento ideado por Luis Lama: el régimen fujimorista, el programa municipal «Volver al Centro» y el Plan Maestro del Centro Histórico impulsado por la gestión de Alberto Andrade, articulados con redes internacionales (UCCI, CIDEU) y el título de «Lima, Capital de la Cultura Iberoamericana». Peralta sostiene que la Bienal (1997-2002), en sus versiones nacional e iberoamericana, funcionó como núcleo de reactivación cultural y descentralización mediante salones regionales, atrajo atención internacional y sirvió de modelo de gestión, pero fue cancelada por desinterés político —especialmente de Luis Castañeda Lossio— y por la incapacidad del propio medio artístico de defender su función social. Documenta episodios polémicos: la crítica de Alfonso Castrillón a la autoría de una obra de García Zapatero, la performance «Señorita de buena presencia busca empleo» de Elena Tejada, la muestra paralela «Emergencia Artística» (1999) gestada por Emilio Santisteban y Gustavo Buntinx tras el veto a «Crisis», y la intervención «Chalk» de Allora &amp; Calzadilla, resignificada por trabajadores municipales. A través de testimonios (Santisteban, Élida Román, Natalia Velit, el propio Lama), el autor argumenta que la orfandad cultural persiste por la ausencia de políticas públicas y la subordinación al mercado. El texto se posiciona a favor de una gestión cultural audaz, descentralizada y socialmente participativa, lamentando que nada haya reemplazado la escala y el alcance de la Bienal.</t>
+          <t>Transcripción (borrador) del conversatorio 'Coleccionando desde la institución' del Foro Pinta Lima 2025, moderado por Pablo León de la Barra (Guggenheim), que confronta dos modelos museales públicos: el MALI de Lima y el Museo Reina Sofía de Madrid. La tesis compartida es que coleccionar implica un pensamiento crítico que puede cuestionar el canon, reparar asimetrías históricas de género, raza e identidad y llenar vacíos. Sharon Lerner expone la trayectoria del Comité de Adquisiciones de Arte Contemporáneo del MALI (casi veinte años, modelado sobre el Latin American Acquisitions Committee de la Tate), la curaduría contemporánea iniciada por Tatiana Cuevas en 2008, y el trabajo 'trenzado' entre colección histórica y contemporánea que atraviesa exposiciones como Arte al Paso, Amazonías y Otras historias posibles, y la reestructuración pospandemia con el programa Salas Abiertas. Detalla la visibilización de artistas amazónicos e indígenas (Sara Flores, Chonon Bensho, Venuca Evanán), la incorporación del textil y proyectos como Línea de Vida de Giuseppe Campuzano, junto a comisiones y trabajo comunitario con Cantagallo. Manuel Segade analiza la dimensión colonial del Reina Sofía —cuya colección latinoamericana se inauguró en 1992— y las condiciones estructurales, funcionariales y presupuestarias que la condicionan, citando las preguntas ontológicas de Suset Sánchez y el Instituto Cader de arte centroamericano como vía de restitución frente al extractivismo cultural. El diálogo aborda el rol de los públicos, la crispación política, la censura, el cierre del Lugar de la Memoria y la misión histórica del museo como plataforma de tensiones críticas de la sociedad civil.</t>
         </is>
       </c>
     </row>
@@ -1886,27 +1886,27 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Ponencia - Villacorta, Jorge - Puntos cardinales (2019) [CEdA].transcripcion.txt</t>
+          <t>Ministerio de Cultura - Contemporáneos. Cinco mil años de visualidad peruana (2019) [catálogo, Perú país invitado ARCOmadrid].md</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>1979-2019 (énfasis en 2001-2019: obra de los ochenta y ARCO 2019)</t>
+          <t>200 a.C.-2019 (Nasca, virreinato y arte contemporáneo reciente)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Transcripción de ponencia/conferencia, 2019 (Fundación SEDA-CEdA, Santiago)</t>
+          <t>Catálogo institucional de feria/exposición (ARCOmadrid), 2019</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Sebastián Vidal; Fundación SEDA; Sandra Gamarra (LiMac); Juan Javier Salazar; Herbert Rodríguez; Rodrigo Quijano; grupo Huayco; MALI; Fundación Reina Sofía; ARCOmadrid; galería Enrique Faria; galería Revólver; Alexis Fabri</t>
+          <t>Ministerio de Cultura del Perú; Jorge Villacorta; Sharon Lerner; Fietta Jarque; Miguel A. López; Teresa Burga; Fernando Bryce; Sandra Gamarra; Natalia Majluf; MALI; ARCOmadrid / IFEMA; Museo Reina Sofía / Museo del Prado</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Transcripción de una ponencia de Jorge Villacorta en la Fundación SEDA (Santiago de Chile), presentada por Sebastián Vidal, en el marco de su participación en el pabellón peruano de ARCOmadrid 2019. Partiendo de dos exposiciones fundacionales de Sandra Gamarra (Living Room, 2001; el proyecto LiMac, 2002), Villacorta reflexiona sobre la desconexión histórica del sistema del arte limeño respecto del circuito internacional y su condición estructuralmente «coja». El eje del argumento es un contraste entre dos artistas del grupo Huayco: Juan Javier Salazar y Herbert Rodríguez. Salazar, considerado durante dos décadas el artista contemporáneo peruano por excelencia (Perú País del Mañana, El cuartucho, los náufragos), cultivó una obra frágil, localista y ácida sobre la desidia nacional, pero fue «maltratado» tras su muerte: descartado en ARCO 2019, cosmetizado en la Bienal de Venecia 2017 y regateado por el capítulo peruano de la Fundación Reina Sofía. Rodríguez, artista afrodescendiente y sistemático archivista de su obra (fotocopias, murales antisenderistas en San Marcos, fotoserigrafía), experimenta en cambio un ascenso internacional inesperado (galería Enrique Faria, Reina Sofía, Fundación Cartier), pese al desdén histórico del medio limeño y del MALI. Villacorta articula estas trayectorias con una crítica al coleccionismo peruano, a la lógica del mercado (galería Revólver, ferias, matching funds de arteBA), a la desatención de la crítica y las galerías, y a las jerarquías raciales y clasistas del establishment cultural limeño (Szyszlo, Armando Andrade). El texto plantea el problema del legado, el valor simbólico y la posibilidad de un arte con «testigos» frente a un arte subordinado al mercado.</t>
+          <t>Catálogo institucional de la participación de Perú como País Invitado en ARCOmadrid 2019, que reúne los textos curatoriales del stand del Estado, la zona de galerías y el programa oficial de más de treinta exposiciones y actividades en Madrid. El ensayo de Jorge Villacorta, 'Contemporáneos: cinco mil años de visualidad peruana', propone lo contemporáneo como actitud y coexistencia antes que como novedad, avanzando la hipótesis de que la contemporaneidad peruana es continuidad de una matriz cultural andino-amazónica con incrustaciones occidentales, un tiempo cíclico que supera categorías como arte popular o artesanía. Sharon Lerner, en 'Texto, tactibilidad y trama', encuadra la selección de galerías —que por primera vez combina representación local e internacional— como un corte no representativo de un 'arte nacional', destacando líneas transversales: el uso del texto, la cita y el archivo para desmontar discursos de la historia oficial; las tensiones del colonialismo y los criterios étnicos y de clase; la mirada al territorio y a lo extractivo; y la fragilidad táctil del textil, la arcilla y el cuerpo. El catálogo perfila a artistas como Teresa Burga, Rita Ponce de León, Ximena Garrido Lecca, Herbert Rodríguez, Fernando Bryce, Sandra Gamarra, Milagros de la Torre y Antonio Paucar, y documenta las conferencias curadas por Miguel A. López sobre el Bicentenario, la contemporaneidad andina, indígena y amazónica, y las transformaciones institucionales y de mercado. El programa oficial, presentado por Fietta Jarque, articula un relato de cinco mil años: Nasca, el Matrimonio de Martín de Loyola, Huamán Poma, la revista Amauta de Mariátegui, Amazonías y colecciones privadas (Hochschild, CIFO, Jan Mulder).</t>
         </is>
       </c>
     </row>
@@ -1918,27 +1918,27 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Por Qué no vivo en el Perú.md</t>
+          <t>Mitrovic - Extravíos de la forma. Vanguardia, modernismo popular y arte contemporáneo en Lima desde los 60 (2019).md</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>ca. 1972 en adelante (emigración de Juan Acha a México y comparación Perú/México de los años setenta)</t>
+          <t>1960-2018 (desde los sesenta hasta el presente)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Encuesta/testimonio en revista literaria (Hueso Húmero), ca. 1980; transcripción en Markdown, s/f</t>
+          <t>Libro académico, 2019 (Fondo Editorial FAU-PUCP)</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Juan Acha; revista Hueso Húmero; museos, institutos y universidades de México</t>
+          <t>Mijail Mitrovic; Gustavo Buntinx; Mirko Lauer; Sharon Lerner; Miguel A. López; Emilio Tarazona; Fernando de Szyszlo; E.P.S. Huayco; Taller NN; José Carlos Martinat; Museo de Arte de Lima (MALI); PUCP; Fredric Jameson</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Transcripción de la respuesta de Juan Acha a la encuesta 'Por qué no vivo en el Perú', iniciada por la revista Hueso Húmero para indagar las razones del éxodo de creadores e intelectuales peruanos. Acha —crítico y teórico del arte dedicado a los problemas latinoamericanos, radicado en México— distingue razones 'de afuera' y 'de adentro', otorgando mayor peso a las primeras: sólo abandona su país quien encuentra en otro las condiciones para desarrollar con dignidad su trabajo profesional, mientras que las circunstancias personales o los factores nacionales negativos serían secundarios en su caso. Enumera lo que México le ofreció y el Perú le negaba: amplias posibilidades de publicar en diarios y revistas, de colaborar en museos e institutos y de investigar y enseñar en universidades, todo ello remunerado con dignidad; libertad de expresión intelectual e intensa circulación de ideas marxistas en libros, revistas y simposios; prestigio nacional de las artes visuales con apoyo estatal, política museográfica y de simposios activa, y facilidades para viajar y contactar con el arte de otras latitudes. Valora, además, el mejor enfoque de los problemas artísticos y culturales latinoamericanos posible desde México, cuya escala demográfica y potente industria editorial concentran las investigaciones de toda la región y anticipan fenómenos que luego se difunden. El testimonio —que el archivo conserva incompleto, interrumpido al mencionar una 'identificación cultural más conflictiva y acorde a la realidad concreta'— condensa la autojustificación del exilio intelectual como decisión productiva antes que como queja, y funciona como documento sobre las carencias institucionales del campo artístico peruano frente a las condiciones del México de esos años.</t>
+          <t>Ensayo de historia y teoría del arte que impugna el «relato convencional» sobre el arte contemporáneo en Lima, entendido como una fábula épica que narra el tránsito de la vanguardia de los sesenta al arte contemporáneo global mediante el «encuentro con lo popular». Desde un marco marxista-dialéctico (Adorno, Jameson, Bürger, Osborne, Lukács), Mitrovic reivindica la totalización y la periodización frente al historicismo posmoderno que celebra heterogeneidad y discontinuidad. Su tesis central es que la «desidealización» del arte —su reducción a hecho social e institucional— siguió en Lima una trayectoria específica: de la teoría de las raíces nacionales (Szyszlo, Lauer) y el altomodernismo, a la radicalización de la vanguardia bajo el velasquismo, que el autor conceptualiza como «modernismo popular» (E.P.S. Huayco, Paréntesis, la frase de Lauer «solo lo popular es moderno»). Con Sendero Luminoso y la crisis de los ochenta, la utopía colapsa y el arte se reorienta hacia la denuncia ética de la violencia, prolongada durante el fujimorato (Colectivo Sociedad Civil, «Lava la bandera»). El cambio de siglo consuma la «contemporaneización» mediante las Bienales de Lima y el mercado. El último capítulo analiza obras (Polanco, Guerra García, Huarcaya, Aguirre, Andrade Valdez, Martinat) para mostrar cómo lo popular deviene «neocostumbrismo» y «renta de monopolio»: sello local que certifica autenticidad cultural en el circuito global, mientras se evacúa el horizonte futuro y el «pueblo» se reduce a «población». Frente a la nostalgia y la reoligarquización simbólica, Mitrovic propone recuperar las potencialidades utópicas hoy reprimidas.</t>
         </is>
       </c>
     </row>
@@ -1950,27 +1950,27 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>QUEHACER 19_watermark_p120-128.pdf</t>
+          <t>Peralta - Lo que la Bienal de Lima se llevó. Balance a cinco años de su desactivación.md</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>1940-1982 (arte peruano del siglo XX: indigenismo, velasquismo y transición belaundista)</t>
+          <t>1997-2003 (Bienales de Lima y su desactivación)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Entrevista en revista (Quehacer n.º 19, DESCO), ca. 1982</t>
+          <t>Artículo/ensayo de balance, ca. 2007-2008</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Mirko Lauer; Sebastián Gris; Juan Acha; DESCO; Alfonso Castrillón; José Sabogal; Josué Sánchez; Ramiro Llona; José Carlos Ramos; Joaquín López Antay; Fernando de Szyszlo; Juan Manuel Ugarte Eléspuru; Bienal de Medellín</t>
+          <t>Juan Peralta; Luis Lama; Jorge Villacorta; Emilio Santisteban; Elena Tejada; Gustavo Buntinx; Alfonso Castrillón; Élida Román; Allora &amp; Calzadilla; Francis Alÿs; Cuauhtémoc Medina; Alberto Andrade; Luis Castañeda Lossio; Municipalidad Metropolitana de Lima; UCCI</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Entrevista de Sebastián Gris a Mirko Lauer publicada en la revista Quehacer (n.º 19, DESCO) bajo el título 'Está naciendo algo…'. El diálogo presenta el giro teórico de Lauer —poeta y crítico literario— hacia una teoría social de la cultura y del objeto plástico, formulada en su libro 'Crítica de la artesanía' y anticipada, junto al ausente Juan Acha, en el Coloquio de Arte No-objetual de Medellín. Lauer relee su 'Introducción a la pintura peruana del siglo XX': sostiene que hacia 1960 culmina, con la 'Teoría de las Raíces Nacionales', el ciclo abierto por el indigenismo de Sabogal, mientras los años setenta traen la revaloración del arte popular y su confluencia con una tradición artesanal. Critica el neo-indigenismo como coartada del populismo velasquista y de la Reforma Agraria: un país que, sin atreverse a enfrentar lo popular real, se inventa un seudo-país mistificado (el 'colmenazo', el arte turístico de José Carlos Ramos). Diagnostica, tras la restauración belaundista (posterior a 1977), una 'pérdida de direccionalidad' y un caos del mercado que ahora impone valor. Discute los límites de la propuesta conceptual y no-objetual, el Premio Nacional López Antay y la labor de Alfonso Castrillón, y reivindica la crítica de arte como oficio concreto —ni estética idealista ni 'estética marxista'—. Finalmente aborda la marginalidad y el desprecio hacia el intelectual peruano. Aparecen Josué Sánchez, Ramiro Llona, Szyszlo, Ugarte Eléspuru y la Bienal de Medellín. Su aporte es proponer el estudio del objeto plástico desde su existencia social y desde una perspectiva popular.</t>
+          <t>Balance crítico sobre la desaparición de la Bienal de Lima, escrito por Juan Peralta a cinco años de su desactivación. El texto reconstruye el contexto político-cultural en que surgió el megaevento ideado por Luis Lama: el régimen fujimorista, el programa municipal «Volver al Centro» y el Plan Maestro del Centro Histórico impulsado por la gestión de Alberto Andrade, articulados con redes internacionales (UCCI, CIDEU) y el título de «Lima, Capital de la Cultura Iberoamericana». Peralta sostiene que la Bienal (1997-2002), en sus versiones nacional e iberoamericana, funcionó como núcleo de reactivación cultural y descentralización mediante salones regionales, atrajo atención internacional y sirvió de modelo de gestión, pero fue cancelada por desinterés político —especialmente de Luis Castañeda Lossio— y por la incapacidad del propio medio artístico de defender su función social. Documenta episodios polémicos: la crítica de Alfonso Castrillón a la autoría de una obra de García Zapatero, la performance «Señorita de buena presencia busca empleo» de Elena Tejada, la muestra paralela «Emergencia Artística» (1999) gestada por Emilio Santisteban y Gustavo Buntinx tras el veto a «Crisis», y la intervención «Chalk» de Allora &amp; Calzadilla, resignificada por trabajadores municipales. A través de testimonios (Santisteban, Élida Román, Natalia Velit, el propio Lama), el autor argumenta que la orfandad cultural persiste por la ausencia de políticas públicas y la subordinación al mercado. El texto se posiciona a favor de una gestión cultural audaz, descentralizada y socialmente participativa, lamentando que nada haya reemplazado la escala y el alcance de la Bienal.</t>
         </is>
       </c>
     </row>
@@ -1982,27 +1982,27 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Román, Elida - I Bienal Nacional de Lima. Algunos deslindes.md</t>
+          <t>Ponencia - Villacorta, Jorge - Puntos cardinales (2019) [CEdA].transcripcion.txt</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>1997-1998 (I Bienal Nacional de Lima; referencias a 1987 y 1997)</t>
+          <t>1979-2019 (énfasis en 2001-2019: obra de los ochenta y ARCO 2019)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Artículo/reseña crítica, 1998</t>
+          <t>Transcripción de ponencia/conferencia, 2019 (Fundación SEDA-CEdA, Santiago)</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Élida Román; Luis Lama; UCCI; Municipalidad Metropolitana de Lima; Centro de Artes Visuales (CAV); Virginia Pérez-Ratton; Museo de Arte de Lima; Luz María Bedoya; Mariella Agois; Bienal de Trujillo</t>
+          <t>Jorge Villacorta; Sebastián Vidal; Fundación SEDA; Sandra Gamarra (LiMac); Juan Javier Salazar; Herbert Rodríguez; Rodrigo Quijano; grupo Huayco; MALI; Fundación Reina Sofía; ARCOmadrid; galería Enrique Faria; galería Revólver; Alexis Fabri</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Nota crítica de la crítica de arte Élida Román sobre la I Bienal Nacional de Lima (1998), que deslinda sus antecedentes y examina su lógica organizativa. Román recuerda que un evento similar existió en la III Bienal de Trujillo (1987) con el núcleo «Mirada hacia adentro», y sitúa la Bienal Nacional como mecanismo para seleccionar —mediante salones regionales y comités— la representación peruana a la II Bienal Iberoamericana. Enmarca el evento en el proyecto municipal de recuperación del Centro Histórico y en la designación de Lima como «Plaza Mayor de la Cultura Iberoamericana» por la UCCI, señalando el apresuramiento organizativo y los defectos museográficos derivados del uso de casonas no adecuadas a fines museológicos. Su argumento central cuestiona el discurso «modernizador» y globalizador de los organizadores (Luis Lama), advirtiendo que tras las nociones de ruptura, novedad y globalización se esconden la moda, el esnobismo y «roles forzados» e intereses extraculturales. Critica el centralismo y paternalismo de los salones regionales, que perpetúan la posición privilegiada de Lima sin una política real de desarrollo en provincias. Román reclama definir los propósitos de la actividad artística e interroga la falsa dicotomía entre arte «popular» y «culto», recordando la polémica por el Premio Nacional otorgado a un artesano ayacuchano. Frente a la comparación con estándares metropolitanos, aboga por una modernidad entendida como apertura multidisciplinaria y actitud cohesionadora e identitaria, apoyada en la historia, la antropología y las ciencias sociales. El texto, denso en interrogantes, defiende la reflexión teórica y el debate, y cierra evocando la consigna «¡La imaginación al poder!».</t>
+          <t>Transcripción de una ponencia de Jorge Villacorta en la Fundación SEDA (Santiago de Chile), presentada por Sebastián Vidal, en el marco de su participación en el pabellón peruano de ARCOmadrid 2019. Partiendo de dos exposiciones fundacionales de Sandra Gamarra (Living Room, 2001; el proyecto LiMac, 2002), Villacorta reflexiona sobre la desconexión histórica del sistema del arte limeño respecto del circuito internacional y su condición estructuralmente «coja». El eje del argumento es un contraste entre dos artistas del grupo Huayco: Juan Javier Salazar y Herbert Rodríguez. Salazar, considerado durante dos décadas el artista contemporáneo peruano por excelencia (Perú País del Mañana, El cuartucho, los náufragos), cultivó una obra frágil, localista y ácida sobre la desidia nacional, pero fue «maltratado» tras su muerte: descartado en ARCO 2019, cosmetizado en la Bienal de Venecia 2017 y regateado por el capítulo peruano de la Fundación Reina Sofía. Rodríguez, artista afrodescendiente y sistemático archivista de su obra (fotocopias, murales antisenderistas en San Marcos, fotoserigrafía), experimenta en cambio un ascenso internacional inesperado (galería Enrique Faria, Reina Sofía, Fundación Cartier), pese al desdén histórico del medio limeño y del MALI. Villacorta articula estas trayectorias con una crítica al coleccionismo peruano, a la lógica del mercado (galería Revólver, ferias, matching funds de arteBA), a la desatención de la crítica y las galerías, y a las jerarquías raciales y clasistas del establishment cultural limeño (Szyszlo, Armando Andrade). El texto plantea el problema del legado, el valor simbólico y la posibilidad de un arte con «testigos» frente a un arte subordinado al mercado.</t>
         </is>
       </c>
     </row>
@@ -2014,27 +2014,27 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Screen Shot 2026-07-16 at 08.22.07.png</t>
+          <t>Por Qué no vivo en el Perú.md</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>1980-1981 (obra 'Arte al Paso' y culto vigente a Sarita Colonia); Sarita Colonia 1914-1940</t>
+          <t>ca. 1972 en adelante (emigración de Juan Acha a México y comparación Perú/México de los años setenta)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Captura de pantalla, 16-07-2026 (de artículo de la revista MARKA, Lima, 14-05-1981, p. 34; archivo UNMSM-CEDOC)</t>
+          <t>Encuesta/testimonio en revista literaria (Hueso Húmero), ca. 1980; transcripción en Markdown, s/f</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Sarita Colonia; Taller de Estética de Proyección Social 'Huayco' (E.P.S. Huayco); Francisco Mariotti; María Luy; Gerbert Rodríguez; Mariella Zevallos; Armando Williams; Charo Noriega; revista MARKA; UNMSM-CEDOC</t>
+          <t>Juan Acha; revista Hueso Húmero; museos, institutos y universidades de México</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Captura de una página de la revista MARKA (Lima, 14 de mayo de 1981, p. 34; sello de archivo UNMSM-CEDOC) con el artículo 'La imagen y la fuerza milagrosa', dedicado al culto a Sarita Colonia y a su tratamiento en el arte. El texto interpreta la devoción popular a Sarita como caso patente de realización simbólica donde el elemento religioso se ensambla con el gusto estético popular, uniendo pensamiento mágico y realidad social inmediata; el símbolo religioso operaría como continente de mitos que resuelven imaginariamente las contradicciones de la vida. Recuerda que Sarita nació en Huaraz en 1914 y murió en el Callao en 1940, donde surgió su culto —hoy extendido entre los más desvalidos: el mundo del hampa, la prostitución, estibadores y choferes—, con un mausoleo-santuario rodeado de exvotos y comerciantes ambulantes. La sección 'Sarita en el arte' presenta y reproduce la obra 'Arte al Paso', un enorme rostro de Sarita compuesto con cerca de 12,000 latas de leche, realizado por un conjunto de artistas jóvenes reunidos en el Taller de Estética de Proyección Social 'Huayco' (E.P.S. Huayco): Francisco Mariotti, María Luy, Gerbert Rodríguez, Mariella Zevallos, Armando Williams y Charo Noriega. Instalada desde enero de ese año a la vera del sur, la obra recoge en clave colectiva la significación sociocultural de Sarita para ofrecer a viajeros y peregrinos una exposición permanente de esa imagen, integrando la escala monumental, la soledad del paisaje y una identificación plástica con el misterio cotidiano. Es documento clave sobre el vínculo entre religiosidad popular, migración andina y vanguardia peruana de inicios de los ochenta.</t>
+          <t>Transcripción de la respuesta de Juan Acha a la encuesta 'Por qué no vivo en el Perú', iniciada por la revista Hueso Húmero para indagar las razones del éxodo de creadores e intelectuales peruanos. Acha —crítico y teórico del arte dedicado a los problemas latinoamericanos, radicado en México— distingue razones 'de afuera' y 'de adentro', otorgando mayor peso a las primeras: sólo abandona su país quien encuentra en otro las condiciones para desarrollar con dignidad su trabajo profesional, mientras que las circunstancias personales o los factores nacionales negativos serían secundarios en su caso. Enumera lo que México le ofreció y el Perú le negaba: amplias posibilidades de publicar en diarios y revistas, de colaborar en museos e institutos y de investigar y enseñar en universidades, todo ello remunerado con dignidad; libertad de expresión intelectual e intensa circulación de ideas marxistas en libros, revistas y simposios; prestigio nacional de las artes visuales con apoyo estatal, política museográfica y de simposios activa, y facilidades para viajar y contactar con el arte de otras latitudes. Valora, además, el mejor enfoque de los problemas artísticos y culturales latinoamericanos posible desde México, cuya escala demográfica y potente industria editorial concentran las investigaciones de toda la región y anticipan fenómenos que luego se difunden. El testimonio —que el archivo conserva incompleto, interrumpido al mencionar una 'identificación cultural más conflictiva y acorde a la realidad concreta'— condensa la autojustificación del exilio intelectual como decisión productiva antes que como queja, y funciona como documento sobre las carencias institucionales del campo artístico peruano frente a las condiciones del México de esos años.</t>
         </is>
       </c>
     </row>
@@ -2046,27 +2046,27 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Screen Shot 2026-07-16 at 08.37.09.png</t>
+          <t>Presentaci_n del programa ARTUS _ Beca de Artistas (transcript).mp4.pdf.txt</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>1965-1984</t>
+          <t>c. 2020 (menciona la pandemia de coronavirus en curso)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Captura de pantalla, 16-07-2026 (de un cuadro/gráfico basado en el informe de Alfonso Castrillón, 'Reflexiones sobre el arte conceptual en el Perú y sus proyecciones', Hueso Húmero n.º 7; sello UNMSM)</t>
+          <t>Transcripción de conversatorio en línea (plataforma Park); época de la pandemia (c. 2020)</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Alfonso Castrillón; Juan Acha; Teresa Burga; Emilio Hernández; Rafael Hastings; Francisco Mariotti; Luis Arias Vera; Jorge Eielson; Wiley Ludeña; Herbert Rodríguez; E.P.S. Huayco; Grupo Paréntesis; UNMSM</t>
+          <t>Max Hernández Calvo (moderador); Carlos Marzano y Patricia Exequio (cofundadores de ARTUS); Seneta Barsi y Augusto Valls (artistas becados) [nombres con corrupción de ASR]; ARTUS; ICPNA; Park; WIELS; Delfina; Gasworks; Pivô</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Captura de pantalla de un cuadro cronológico ('Gráfico 1') que sistematiza el desarrollo del arte conceptual y no-objetual en el Perú entre 1965 y 1984, elaborado 'en base al informe de Alfonso Castrillón: Reflexiones sobre el arte conceptual en el Perú y sus proyecciones' (Hueso Húmero 7). El cuadro organiza la información en cuatro columnas —Fecha, Tendencia, Operador (artistas y grupos) y Lugar— trazando la sucesión de tendencias: pop y op (1965, Galería Lima, IAC), concepto y ambientes (1969-1970, con Juan Acha, 'Cultura y Libertad'), acciones y eventos (1972-1975: Teresa Burga, Rafael Hastings, Francisco Mariotti, CONTACTA, Premio López Antay, Festival Inkarri), y las prácticas de no-objeto y performance de fines de los setenta y de los ochenta. Registra los colectivos 'Signo x signo' (Patricia López, Armando Williams, Rossana Agois, Wiley Ludeña, Hugo Salazar), el Grupo USM de Alfonso Castrillón, 'Paréntesis' (Charo Noriega, Armando Williams, María Luy, Francisco Mariotti, Fernando Bedoya, Juan J. Salazar, Mariela Zevallos) y 'Huayco EPS' (Herbert Rodríguez, Lucy Angulo, José Morales), junto a nombres como Luis Arias Vera, Emilio Hernández, Jorge Eielson, Hernán Pazos, Esther Vainstein, Cecilia Paredes y Sergio Zevallos. Consigna hitos y sedes: encuestas, la Bienal no-objetual de Medellín, la Bienal de São Paulo (1983), la acción 'Cuidado pintores…', y espacios como el Instituto Italiano, la Universidad de San Marcos y galerías limeñas. Funciona como mapa genealógico de la vanguardia experimental peruana y de sus operadores institucionales, útil para periodizar el paso del conceptualismo a la performance y al arte no-objetual.</t>
+          <t>Transcripción (con notoria corrupción de reconocimiento automático de voz) de un conversatorio del ciclo de la plataforma Park sobre el programa de becas ARTUS, moderado por el crítico y curador Max Hernández Calvo, con los cofundadores Carlos Marzano y Patricia Exequio y dos artistas que realizaron residencias. La conversación, situada durante la pandemia (se pregunta por su impacto en las residencias), expone el modelo de financiamiento de ARTUS: 'un grupo de patronos de 34 benefactores que nos ayudan con una cuota anual a poder financiar el costo de estas residencias', y el anuncio de haber logrado 'el primer sponsor institucional' (el ICPNA). Marzano describe el mecanismo de selección —'una comunidad de profesionales, de curadores locales y extranjeros que son los que hacen la selección de los trabajos y evalúan el cuerpo artístico e intelectual de los postulantes'— y el criterio para elegir residencias ('hacemos una labor de investigación de cuáles son las mejores residencias del mundo… hablamos con curadores, con instituciones fuera y con artistas'). Los dos artistas relatan sus procesos de selección y la experiencia de residencia (entrevistas con curadores, valor del 'tiempo para pensar' y de 'interlocutores que te ayuden a mirar diferente tu propia práctica'). Debido a la baja calidad de la transcripción automática, varios nombres propios aparecen corruptos ('Beca Sartus', 'Arthur', 'pivot' por Pivô) y requieren verificación contra el audio original. Fuente oral primaria sobre el mecenazgo privado, los criterios de selección y la articulación entre coleccionistas, curadores e institución en el apoyo al arte joven peruano.</t>
         </is>
       </c>
     </row>
@@ -2078,27 +2078,27 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Screen Shot 2026-07-16 at 13.03.35.png</t>
+          <t>QUEHACER 19_watermark_p120-128.pdf</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>1970-1981</t>
+          <t>1940-1982 (arte peruano del siglo XX: indigenismo, velasquismo y transición belaundista)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Captura de pantalla (16-07-2026) de artículo de revista, 1981</t>
+          <t>Entrevista en revista (Quehacer n.º 19, DESCO), ca. 1982</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Juan Acha; Hueso Húmero (revista); UNMSM; José Carlos Mariátegui (contexto marxista); El Sexto (prisión); México D.F.</t>
+          <t>Mirko Lauer; Sebastián Gris; Juan Acha; DESCO; Alfonso Castrillón; José Sabogal; Josué Sánchez; Ramiro Llona; José Carlos Ramos; Joaquín López Antay; Fernando de Szyszlo; Juan Manuel Ugarte Eléspuru; Bienal de Medellín</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>La captura reproduce la primera página del texto autobiográfico y ensayístico de Juan Acha titulado 'Por qué no vivo en el Perú', encabezado por una nota editorial de la revista Hueso Húmero que enmarca el escrito dentro de una indagación colectiva sobre los creadores e intelectuales peruanos que optaron por emigrar, problema que la publicación se propone tratar con seriedad y continuar en números sucesivos. Acha, crítico y teórico del arte dedicado a los problemas latinoamericanos, ordena sus razones para no residir en el Perú en dos clases jerarquizadas: las 'de afuera', que considera principales, y las 'de adentro', secundarias. Bajo las primeras enumera lo que encontró en México y le faltaba en su país: amplias posibilidades de publicar en diarios y revistas, colaborar en museos e institutos, investigar y enseñar en universidades como crítico de arte, todo ello remunerado con dignidad; libertad de expresión e intensa circulación de ideas marxistas en libros, revistas y simposios; y un prestigio nacional de las artes visuales sostenido por el Estado, con una activa política museográfica y de simposios además de facilidades para viajar y entrar en contacto con el arte de otras latitudes. El fragmento evidencia la tesis central del autor: la emigración no responde a un rechazo personal sino a la asimetría estructural entre el medio cultural peruano, precario y cerrado, y el mexicano, mejor equipado y más poroso al quehacer cultural latinoamericano. El documento funciona como fuente primaria sobre las condiciones institucionales del campo artístico peruano y sobre la trayectoria del propio Acha como figura clave de la teoría del arte no objetual en América Latina.</t>
+          <t>Entrevista de Sebastián Gris a Mirko Lauer publicada en la revista Quehacer (n.º 19, DESCO) bajo el título 'Está naciendo algo…'. El diálogo presenta el giro teórico de Lauer —poeta y crítico literario— hacia una teoría social de la cultura y del objeto plástico, formulada en su libro 'Crítica de la artesanía' y anticipada, junto al ausente Juan Acha, en el Coloquio de Arte No-objetual de Medellín. Lauer relee su 'Introducción a la pintura peruana del siglo XX': sostiene que hacia 1960 culmina, con la 'Teoría de las Raíces Nacionales', el ciclo abierto por el indigenismo de Sabogal, mientras los años setenta traen la revaloración del arte popular y su confluencia con una tradición artesanal. Critica el neo-indigenismo como coartada del populismo velasquista y de la Reforma Agraria: un país que, sin atreverse a enfrentar lo popular real, se inventa un seudo-país mistificado (el 'colmenazo', el arte turístico de José Carlos Ramos). Diagnostica, tras la restauración belaundista (posterior a 1977), una 'pérdida de direccionalidad' y un caos del mercado que ahora impone valor. Discute los límites de la propuesta conceptual y no-objetual, el Premio Nacional López Antay y la labor de Alfonso Castrillón, y reivindica la crítica de arte como oficio concreto —ni estética idealista ni 'estética marxista'—. Finalmente aborda la marginalidad y el desprecio hacia el intelectual peruano. Aparecen Josué Sánchez, Ramiro Llona, Szyszlo, Ugarte Eléspuru y la Bienal de Medellín. Su aporte es proponer el estudio del objeto plástico desde su existencia social y desde una perspectiva popular.</t>
         </is>
       </c>
     </row>
@@ -2110,27 +2110,27 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Screen Shot 2026-07-16 at 13.03.44.png</t>
+          <t>Román, Elida - I Bienal Nacional de Lima. Algunos deslindes.md</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>1970-1981</t>
+          <t>1997-1998 (I Bienal Nacional de Lima; referencias a 1987 y 1997)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Captura de pantalla (16-07-2026) de artículo de revista, 1981</t>
+          <t>Artículo/reseña crítica, 1998</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Juan Acha; Hueso Húmero (revista); El Sexto (prisión de Lima); México D.F.; UNMSM</t>
+          <t>Élida Román; Luis Lama; UCCI; Municipalidad Metropolitana de Lima; Centro de Artes Visuales (CAV); Virginia Pérez-Ratton; Museo de Arte de Lima; Luz María Bedoya; Mariella Agois; Bienal de Trujillo</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>La captura corresponde a la página 109 (sección 'Encuesta') y continúa el texto de Juan Acha 'Por qué no vivo en el Perú', cerrando la argumentación iniciada en la página anterior. Bajo las razones 'de afuera' Acha añade dos motivos vinculados a su vocación latinoamericanista: México ofrece un mejor enfoque de los problemas artísticos y culturales de 'nuestra América' porque, por su tamaño demográfico e importancia y por su industria editora, allí confluyen antes que en otros países los fenómenos y las investigaciones del resto de Latinoamérica; y propicia una identificación cultural más conflictiva y acorde a la realidad concreta, con un aprecio por la cultura popular en la que halla semejanzas con el Perú. Luego expone tres razones 'secundarias', personales, que lo empujaron a salir: haber vivido y formado universitariamente fuera del país trabajando como químico en varios países latinoamericanos, lo que facilitó su salida y le dio mejor visión de virtudes y defectos nacionales; el clima represivo y discriminante de la capital, producto del 'aristocratismo limeño' y su racismo disimulado, del nepotismo de las clases dominantes y la represión de lo popular; y, sobre todo, haber sido fichado en 1970 como supuesto inculpado de tráfico de drogas al asistir a una fiesta de artistas jóvenes, sufriendo diez días de vejaciones en la prisión El Sexto por negligencia judicial antes de ser declarado inocente. El texto, firmado en México D.F. en febrero de 1981, articula crítica estructural del campo cultural peruano con testimonio personal de exclusión y violencia institucional.</t>
+          <t>Nota crítica de la crítica de arte Élida Román sobre la I Bienal Nacional de Lima (1998), que deslinda sus antecedentes y examina su lógica organizativa. Román recuerda que un evento similar existió en la III Bienal de Trujillo (1987) con el núcleo «Mirada hacia adentro», y sitúa la Bienal Nacional como mecanismo para seleccionar —mediante salones regionales y comités— la representación peruana a la II Bienal Iberoamericana. Enmarca el evento en el proyecto municipal de recuperación del Centro Histórico y en la designación de Lima como «Plaza Mayor de la Cultura Iberoamericana» por la UCCI, señalando el apresuramiento organizativo y los defectos museográficos derivados del uso de casonas no adecuadas a fines museológicos. Su argumento central cuestiona el discurso «modernizador» y globalizador de los organizadores (Luis Lama), advirtiendo que tras las nociones de ruptura, novedad y globalización se esconden la moda, el esnobismo y «roles forzados» e intereses extraculturales. Critica el centralismo y paternalismo de los salones regionales, que perpetúan la posición privilegiada de Lima sin una política real de desarrollo en provincias. Román reclama definir los propósitos de la actividad artística e interroga la falsa dicotomía entre arte «popular» y «culto», recordando la polémica por el Premio Nacional otorgado a un artesano ayacuchano. Frente a la comparación con estándares metropolitanos, aboga por una modernidad entendida como apertura multidisciplinaria y actitud cohesionadora e identitaria, apoyada en la historia, la antropología y las ciencias sociales. El texto, denso en interrogantes, defiende la reflexión teórica y el debate, y cierra evocando la consigna «¡La imaginación al poder!».</t>
         </is>
       </c>
     </row>
@@ -2142,27 +2142,27 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>VVAA - El desencantamiento del arte. Conversación de egresados con Jorge Villacorta [Ansible].md</t>
+          <t>Screen Shot 2026-07-16 at 08.22.07.png</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>2013-2018 (coyuntura reciente, con referencias a los años ochenta)</t>
+          <t>1980-1981 (obra 'Arte al Paso' y culto vigente a Sarita Colonia); Sarita Colonia 1914-1940</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Conversación colectiva publicada en revista (Ansible), ca. 2018 (s/f exacta)</t>
+          <t>Captura de pantalla, 16-07-2026 (de artículo de la revista MARKA, Lima, 14-05-1981, p. 34; archivo UNMSM-CEDOC)</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Adriana Bickel; Rafael Nolte; Rox Monteverde; Kenji Quispe; Mariana Román; Raúl Silva; Michael Prado; Alfredo Bernal; PUCP; ENSABAP; Corriente Alterna; Centro de la Imagen; galería 80m2 Livia Benavides; Revolver; Mario Testino; Rodrigo Quijano</t>
+          <t>Sarita Colonia; Taller de Estética de Proyección Social 'Huayco' (E.P.S. Huayco); Francisco Mariotti; María Luy; Gerbert Rodríguez; Mariella Zevallos; Armando Williams; Charo Noriega; revista MARKA; UNMSM-CEDOC</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>Conversación colectiva entre egresados y estudiantes recientes de las principales escuelas de artes visuales de Lima (PUCP, ENSABAP-Bellas Artes, Corriente Alterna, Centro de la Imagen), con intervención del crítico Jorge Villacorta, publicada en la revista Ansible. El diálogo diagnostica un momento de «desencantamiento» e inflexión entre un pasado precario y un futuro incierto en el campo laboral del arte. Los participantes (Adriana Bickel, Rafael Nolte, Rox Monteverde, Kenji Quispe, Mariana Román, Raúl Silva, Michael Prado, Alfredo Bernal) analizan factores recientes: el surgimiento de ferias (P.Ar.C., Art Lima), la internacionalización de galerías (Revolver, 80m2 Livia Benavides), las vanity gallery, el coleccionismo concentrado de Hochschild y Verme, el libro de Mario Testino, la gentrificación de Monumental Callao y el escándalo del pabellón peruano en la Bienal de Venecia 2017 (obra de Juan Javier Salazar, retirada del curador Rodrigo Quijano). El eje conceptual gira en torno al mercado como fuerza hegemónica que guía la cultura, la ausencia de aparato crítico e histórico, el auge de la autogestión como «arma de doble filo» y la imposibilidad de agremiación en un medio fragmentado y competitivo. Villacorta aporta la memoria histórica de la ASPAP (años ochenta) y el contraste con la colegiatura profesional y la AICA. Se debaten la profesionalización, la legitimación externa del artista (por sociólogos, curadores, museos), la deficiente formación que provoca el éxodo de artistas, los cambios curriculares hacia el «artista-investigador» (2010-2011) y lo aspiracional del éxito comercial. El texto expone críticamente la vulnerabilidad estructural del artista joven limeño.</t>
+          <t>Captura de una página de la revista MARKA (Lima, 14 de mayo de 1981, p. 34; sello de archivo UNMSM-CEDOC) con el artículo 'La imagen y la fuerza milagrosa', dedicado al culto a Sarita Colonia y a su tratamiento en el arte. El texto interpreta la devoción popular a Sarita como caso patente de realización simbólica donde el elemento religioso se ensambla con el gusto estético popular, uniendo pensamiento mágico y realidad social inmediata; el símbolo religioso operaría como continente de mitos que resuelven imaginariamente las contradicciones de la vida. Recuerda que Sarita nació en Huaraz en 1914 y murió en el Callao en 1940, donde surgió su culto —hoy extendido entre los más desvalidos: el mundo del hampa, la prostitución, estibadores y choferes—, con un mausoleo-santuario rodeado de exvotos y comerciantes ambulantes. La sección 'Sarita en el arte' presenta y reproduce la obra 'Arte al Paso', un enorme rostro de Sarita compuesto con cerca de 12,000 latas de leche, realizado por un conjunto de artistas jóvenes reunidos en el Taller de Estética de Proyección Social 'Huayco' (E.P.S. Huayco): Francisco Mariotti, María Luy, Gerbert Rodríguez, Mariella Zevallos, Armando Williams y Charo Noriega. Instalada desde enero de ese año a la vera del sur, la obra recoge en clave colectiva la significación sociocultural de Sarita para ofrecer a viajeros y peregrinos una exposición permanente de esa imagen, integrando la escala monumental, la soledad del paisaje y una identificación plástica con el misterio cotidiano. Es documento clave sobre el vínculo entre religiosidad popular, migración andina y vanguardia peruana de inicios de los ochenta.</t>
         </is>
       </c>
     </row>
@@ -2174,27 +2174,27 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>VVAA - Lima se anima. Debates en la escena artística peruana (2009) [ramona 89].md</t>
+          <t>Screen Shot 2026-07-16 at 08.37.09.png</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>1997-2009 (última década, de la Bienal Iberoamericana al presente)</t>
+          <t>1965-1984</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Dossier de revista (ramona nº 89), abril 2009</t>
+          <t>Captura de pantalla, 16-07-2026 (de un cuadro/gráfico basado en el informe de Alfonso Castrillón, 'Reflexiones sobre el arte conceptual en el Perú y sus proyecciones', Hueso Húmero n.º 7; sello UNMSM)</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Quijano; Eliana Otta; Miguel López; Max Hernández-Calvo; Gustavo Buntinx; Jorge Villacorta; Alfredo Márquez; Fernando Bryce; Gilda Mantilla; Philippe Gruenberg; Giancarlo Scaglia; revista Juanacha; La Culpable; MALI; galería Revólver</t>
+          <t>Alfonso Castrillón; Juan Acha; Teresa Burga; Emilio Hernández; Rafael Hastings; Francisco Mariotti; Luis Arias Vera; Jorge Eielson; Wiley Ludeña; Herbert Rodríguez; E.P.S. Huayco; Grupo Paréntesis; UNMSM</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>Dossier «Lima se anima» de la revista argentina ramona (nº 89, abril 2009), coeditado con la publicación limeña Juanacha por Rodrigo Quijano y Eliana Otta, que ofrece una radiografía crítica de la escena artística peruana ante su reciente revinculación con el circuito internacional. Reúne una conversación entre artistas («Perú, ¿país blindado?») con Alfredo Márquez, Fernando Bryce, Gilda Mantilla, Philippe Gruenberg y Giancarlo Scaglia; ensayos de Miguel López y Max Hernández-Calvo; un debate virtual del blog Arte-Nuevo sobre las políticas museales; un texto de Gustavo Buntinx (Micromuseo) y una entrevista a Jorge Villacorta. El hilo común es la interrogación del supuesto «boom» del arte contemporáneo limeño de la última década: los participantes coinciden en que la internacionalización y el crecimiento del mercado y del coleccionismo (impulsado por el MALI) han producido una escena «contrahecha», con brazos de mercado pero sin instituciones, crítica, educación ni políticas culturales. Márquez denuncia el carácter colonial y exótico de esa visibilidad; López («Boo(o)m: Morir de éxito») teoriza un proceso de despolitización y domesticación que diluye el conflicto y convierte la autonomía en aquiescencia entre agentes; Hernández-Calvo («Una coyuntura que no fue») analiza cómo las Bienales de Lima (1997-2002) forzaron una «contemporaneización» de instalación y video sin sustento curatorial ni educativo, generando escisiones entre circuito oficial y alternativo. Se abordan además el éxodo de artistas por la deficiente formación, la toma estudiantil de Bellas Artes, la autogestión (La Culpable) y las disputas por el Museo de la Memoria. El dossier reivindica la autonomía, el disenso y el filo crítico histórico del arte peruano.</t>
+          <t>Captura de pantalla de un cuadro cronológico ('Gráfico 1') que sistematiza el desarrollo del arte conceptual y no-objetual en el Perú entre 1965 y 1984, elaborado 'en base al informe de Alfonso Castrillón: Reflexiones sobre el arte conceptual en el Perú y sus proyecciones' (Hueso Húmero 7). El cuadro organiza la información en cuatro columnas —Fecha, Tendencia, Operador (artistas y grupos) y Lugar— trazando la sucesión de tendencias: pop y op (1965, Galería Lima, IAC), concepto y ambientes (1969-1970, con Juan Acha, 'Cultura y Libertad'), acciones y eventos (1972-1975: Teresa Burga, Rafael Hastings, Francisco Mariotti, CONTACTA, Premio López Antay, Festival Inkarri), y las prácticas de no-objeto y performance de fines de los setenta y de los ochenta. Registra los colectivos 'Signo x signo' (Patricia López, Armando Williams, Rossana Agois, Wiley Ludeña, Hugo Salazar), el Grupo USM de Alfonso Castrillón, 'Paréntesis' (Charo Noriega, Armando Williams, María Luy, Francisco Mariotti, Fernando Bedoya, Juan J. Salazar, Mariela Zevallos) y 'Huayco EPS' (Herbert Rodríguez, Lucy Angulo, José Morales), junto a nombres como Luis Arias Vera, Emilio Hernández, Jorge Eielson, Hernán Pazos, Esther Vainstein, Cecilia Paredes y Sergio Zevallos. Consigna hitos y sedes: encuestas, la Bienal no-objetual de Medellín, la Bienal de São Paulo (1983), la acción 'Cuidado pintores…', y espacios como el Instituto Italiano, la Universidad de San Marcos y galerías limeñas. Funciona como mapa genealógico de la vanguardia experimental peruana y de sus operadores institucionales, útil para periodizar el paso del conceptualismo a la performance y al arte no-objetual.</t>
         </is>
       </c>
     </row>
@@ -2206,27 +2206,27 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>VVAA - Memorias del subdesarrollo. Arte y el giro descolonial en América Latina, 1960-1985 [catálogo MCASD].md</t>
+          <t>Screen Shot 2026-07-16 at 13.03.35.png</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>1960-1985 (con foco 1967-1981)</t>
+          <t>1970-1981</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de exposición / ensayo académico, 2018 (MCASD)</t>
+          <t>Captura de pantalla (16-07-2026) de artículo de revista, 1981</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Julieta González; Andrea Giunta; Jacopo Crivelli Visconti; Juan Acha; Marta Traba; Ferreira Gullar; Teresa Burga; E.P.S. Huayco; Grupo Paréntesis; Jesús Ruiz Durand; Fernando 'Coco' Bedoya; MALI; Museum of Contemporary Art San Diego</t>
+          <t>Juan Acha; Hueso Húmero (revista); UNMSM; José Carlos Mariátegui (contexto marxista); El Sexto (prisión); México D.F.</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>El ensayo de Sharon Lerner incluido en el catálogo de la exposición 'Memorias del subdesarrollo: arte y el giro descolonial en América Latina, 1960-1985' inserta la escena peruana de 1967-1981 en una narrativa continental que postula una ruptura epistémica con lo moderno mediante la noción de subdesarrollo y el deseo de descolonizar los cánones estéticos impuestos. Su tesis desplaza el foco del paradigma formalista modernista hacia el contexto social, la apropiación de tradiciones locales y lo 'popular' como categoría clave, cuya heterogeneidad histórica advierte no homogeneizar. Reconstruye el debate entre Juan Acha y Marta Traba sobre el pop cosmopolita y la dependencia cultural, apoyándose en Mariátegui, Ferreira Gullar y Mário Pedrosa, y en la teoría de la dependencia. Analiza casos peruanos: los afiches de la Reforma Agraria de Jesús Ruiz Durand y su 'pop achorado' dentro de SINAMOS; los festivales Contacta y las Carreras de Chasquis de Luis Arias Vera bajo el velasquismo; el Grupo Paréntesis y el Contacta 79 (Becerro de oro, Coquito) de Fernando Bedoya; y sobre todo E.P.S. Huayco, con 'Arte al paso (Salchipapas)' y 'Sarita Colonia', leídos vía Buntinx y Lauer como articulación de lo popular urbano migrante. Suma el caso aislado de Teresa Burga y 'Perfil de la mujer peruana' (1980-81) como acercamiento conceptual a género y clase. Recurriendo a Bürger y Giunta, discute la definición de vanguardia y concluye que estas prácticas oscilaron entre dependencia y autonomía, sin lograr plataformas de continuidad, siendo Huayco el caso más próximo a una vanguardia local pese a su disolución.</t>
+          <t>La captura reproduce la primera página del texto autobiográfico y ensayístico de Juan Acha titulado 'Por qué no vivo en el Perú', encabezado por una nota editorial de la revista Hueso Húmero que enmarca el escrito dentro de una indagación colectiva sobre los creadores e intelectuales peruanos que optaron por emigrar, problema que la publicación se propone tratar con seriedad y continuar en números sucesivos. Acha, crítico y teórico del arte dedicado a los problemas latinoamericanos, ordena sus razones para no residir en el Perú en dos clases jerarquizadas: las 'de afuera', que considera principales, y las 'de adentro', secundarias. Bajo las primeras enumera lo que encontró en México y le faltaba en su país: amplias posibilidades de publicar en diarios y revistas, colaborar en museos e institutos, investigar y enseñar en universidades como crítico de arte, todo ello remunerado con dignidad; libertad de expresión e intensa circulación de ideas marxistas en libros, revistas y simposios; y un prestigio nacional de las artes visuales sostenido por el Estado, con una activa política museográfica y de simposios además de facilidades para viajar y entrar en contacto con el arte de otras latitudes. El fragmento evidencia la tesis central del autor: la emigración no responde a un rechazo personal sino a la asimetría estructural entre el medio cultural peruano, precario y cerrado, y el mexicano, mejor equipado y más poroso al quehacer cultural latinoamericano. El documento funciona como fuente primaria sobre las condiciones institucionales del campo artístico peruano y sobre la trayectoria del propio Acha como figura clave de la teoría del arte no objetual en América Latina.</t>
         </is>
       </c>
     </row>
@@ -2238,27 +2238,27 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Vich - La violencia, la dictadura y la globalización. Arte y política en el Perú contemporáneo.md</t>
+          <t>Screen Shot 2026-07-16 at 13.03.44.png</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>1980-2009 (violencia política, dictadura fujimorista y posconflicto)</t>
+          <t>1970-1981</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Ensayo / capítulo de libro académico, c. 2013-2015</t>
+          <t>Captura de pantalla (16-07-2026) de artículo de revista, 1981</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Víctor Vich; Eduardo Tokeshi; Colectivo Sociedad Civil; Natalia Iguíñiz; Sandro Venturo; Piero Quijano; Luz Letts; Víctor Delfín; Miguel Cordero; Jaime Higa; Herbert Rodríguez; Claudia Martínez; Santiago Quintanilla; Rudolph Castro; Felipe López; Gustavo Buntinx</t>
+          <t>Juan Acha; Hueso Húmero (revista); El Sexto (prisión de Lima); México D.F.; UNMSM</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Víctor Vich propone una lectura desde la crítica cultural del arte peruano contemporáneo, sosteniendo que, frente al discurso triunfalista del crecimiento económico, un sector de artistas sigue nombrando al país a partir de sus heridas históricas. Estructura el ensayo en torno a tres acontecimientos: la violencia política, el autoritarismo corrupto del fujimontesinismo y la globalización neoliberal. Apoyándose en Žižek, Hall, Jameson, Foucault y Badiou, entiende lo simbólico no como reflejo sino como soporte de la realidad y campo de batalla donde se disputan sentidos de ciudadanía. Analiza obras emblemáticas: 'Bandera VIII' (2000) de Eduardo Tokeshi, leída como 'la patria en cuidados intensivos'; 'Lava la bandera' del Colectivo Sociedad Civil; la instalación 'Patria' de Natalia Iguíñiz y Sandro Venturo; el afiche censurado de Piero Quijano sobre La Cantuta e Iwo Jima; 'El azar como destino' de Luz Letts; 'El hermoso general' de Víctor Delfín; el saco militar de Miguel Cordero; y las serigrafías de César Vallejo de Jaime Higa sobre posmodernismo y cultura de masas. En una segunda sección sobre memoria generacional examina a artistas nacidos en los ochenta que 'traducen' la violencia con lenguajes heredados de la infancia: la serie 'Invisible' de Claudia Martínez, el trabajo de archivo y cómic de Santiago Quintanilla, los juguetes siniestros (Lego, Playmobil) de Rudolph Castro y las fotografías de nichos ayacuchanos de Felipe López. Su aporte es articular teoría psicoanalítica y poscolonial con un corpus visual peruano, mostrando el arte crítico como agente que interrumpe la ficción neoliberal y recompone la comunidad desde el orden simbólico.</t>
+          <t>La captura corresponde a la página 109 (sección 'Encuesta') y continúa el texto de Juan Acha 'Por qué no vivo en el Perú', cerrando la argumentación iniciada en la página anterior. Bajo las razones 'de afuera' Acha añade dos motivos vinculados a su vocación latinoamericanista: México ofrece un mejor enfoque de los problemas artísticos y culturales de 'nuestra América' porque, por su tamaño demográfico e importancia y por su industria editora, allí confluyen antes que en otros países los fenómenos y las investigaciones del resto de Latinoamérica; y propicia una identificación cultural más conflictiva y acorde a la realidad concreta, con un aprecio por la cultura popular en la que halla semejanzas con el Perú. Luego expone tres razones 'secundarias', personales, que lo empujaron a salir: haber vivido y formado universitariamente fuera del país trabajando como químico en varios países latinoamericanos, lo que facilitó su salida y le dio mejor visión de virtudes y defectos nacionales; el clima represivo y discriminante de la capital, producto del 'aristocratismo limeño' y su racismo disimulado, del nepotismo de las clases dominantes y la represión de lo popular; y, sobre todo, haber sido fichado en 1970 como supuesto inculpado de tráfico de drogas al asistir a una fiesta de artistas jóvenes, sufriendo diez días de vejaciones en la prisión El Sexto por negligencia judicial antes de ser declarado inocente. El texto, firmado en México D.F. en febrero de 1981, articula crítica estructural del campo cultural peruano con testimonio personal de exclusión y violencia institucional.</t>
         </is>
       </c>
     </row>
@@ -2270,27 +2270,27 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Vidarte - Exhibiciones y adquisiciones para la construcción de narrativas en la historia del arte contemporáneo peruano.md</t>
+          <t>VVAA - El desencantamiento del arte. Conversación de egresados con Jorge Villacorta [Ansible].md</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>2015-2023</t>
+          <t>2013-2018 (coyuntura reciente, con referencias a los años ochenta)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Ensayo curatorial de catálogo, 2023</t>
+          <t>Conversación colectiva publicada en revista (Ansible), ca. 2018 (s/f exacta)</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Giuliana Vidarte; ICPNA; Natalia Iguíñiz; Carlos García Montero; Venuca Evanán; Nereida Apaza; Gloria Quispe; Cristina Flores; Antonio Paucar; Andrés Argüelles Vigo; Carolina Estrada; Santiago Yahuarcani; Ana de Orbegoso</t>
+          <t>Jorge Villacorta; Adriana Bickel; Rafael Nolte; Rox Monteverde; Kenji Quispe; Mariana Román; Raúl Silva; Michael Prado; Alfredo Bernal; PUCP; ENSABAP; Corriente Alterna; Centro de la Imagen; galería 80m2 Livia Benavides; Revolver; Mario Testino; Rodrigo Quijano</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Giuliana Vidarte reflexiona sobre la exposición 'Miradas contemporáneas. Nuevas adquisiciones en la colección ICPNA (2015-2023)', presentada en el Espacio Juan Pardo Heeren del ICPNA de Lima entre agosto y septiembre de 2023. Su argumento central es que las exhibiciones y adquisiciones institucionales son dispositivos para la construcción de narrativas y memoria crítica en la historia del arte contemporáneo peruano: una colección formada a partir de obras que fueron parte de la propia programación expositiva constituye un testimonio de los modos de creación y conserva la memoria de la historia de las exposiciones en el país. Parte de dos ganadoras del Premio ICPNA de Arte Contemporáneo, Venuca Evanán y Nereida Apaza, para introducir cómo el arte contribuye a pensar la realidad mediante reflexiones colectivas sobre violencia de género, identidad y nación. Describe los cinco ejes curatoriales de la muestra —revalorando intimidades, discursos críticos, develando entornos, reinterpretar tradiciones y estéticas disímiles— y analiza diálogos entre obras: el cuerpo y la caja torácica en Gloria Quispe, Cristina Flores y Antonio Paucar; la crítica a la representación colonial y republicana en Andrés Argüelles Vigo y Carolina Estrada/Teodoro Ramírez; el paisaje y la crisis medioambiental amazónica en Silvia Westphalen y Nicole Franchy; la reinterpretación de saberes ancestrales en Santiago Yahuarcani y Ana de Orbegoso. Destaca que las fichas incorporan citas de textos curatoriales previos, nutriendo la exposición del archivo documental institucional. Concluye que estos conjuntos abren líneas múltiples de lectura y afirman el valor del esfuerzo colectivo de gestores, curadores e investigadores en la formación de colecciones y en la escritura de la historia del arte peruano reciente.</t>
+          <t>Conversación colectiva entre egresados y estudiantes recientes de las principales escuelas de artes visuales de Lima (PUCP, ENSABAP-Bellas Artes, Corriente Alterna, Centro de la Imagen), con intervención del crítico Jorge Villacorta, publicada en la revista Ansible. El diálogo diagnostica un momento de «desencantamiento» e inflexión entre un pasado precario y un futuro incierto en el campo laboral del arte. Los participantes (Adriana Bickel, Rafael Nolte, Rox Monteverde, Kenji Quispe, Mariana Román, Raúl Silva, Michael Prado, Alfredo Bernal) analizan factores recientes: el surgimiento de ferias (P.Ar.C., Art Lima), la internacionalización de galerías (Revolver, 80m2 Livia Benavides), las vanity gallery, el coleccionismo concentrado de Hochschild y Verme, el libro de Mario Testino, la gentrificación de Monumental Callao y el escándalo del pabellón peruano en la Bienal de Venecia 2017 (obra de Juan Javier Salazar, retirada del curador Rodrigo Quijano). El eje conceptual gira en torno al mercado como fuerza hegemónica que guía la cultura, la ausencia de aparato crítico e histórico, el auge de la autogestión como «arma de doble filo» y la imposibilidad de agremiación en un medio fragmentado y competitivo. Villacorta aporta la memoria histórica de la ASPAP (años ochenta) y el contraste con la colegiatura profesional y la AICA. Se debaten la profesionalización, la legitimación externa del artista (por sociólogos, curadores, museos), la deficiente formación que provoca el éxodo de artistas, los cambios curriculares hacia el «artista-investigador» (2010-2011) y lo aspiracional del éxito comercial. El texto expone críticamente la vulnerabilidad estructural del artista joven limeño.</t>
         </is>
       </c>
     </row>
@@ -2302,27 +2302,27 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Villacorta - La colección Hochschild.md</t>
+          <t>VVAA - Lima se anima. Debates en la escena artística peruana (2009) [ramona 89].md</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>1980-2016 (con énfasis en el arte peruano desde 2000)</t>
+          <t>1997-2009 (última década, de la Bienal Iberoamericana al presente)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo de colección, c. 2016</t>
+          <t>Dossier de revista (ramona nº 89), abril 2009</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta Chávez; Eduardo y Mariana Hochschild; Octavio Zaya; Luis Pérez Oramas; Giancarlo Scaglia; Fernando Bryce; Teresa Burga; Tilsa Tsuchiya; Jorge Eduardo Eielson; Regina Aprijaskis; MALI; MoMA; Tate Modern</t>
+          <t>Rodrigo Quijano; Eliana Otta; Miguel López; Max Hernández-Calvo; Gustavo Buntinx; Jorge Villacorta; Alfredo Márquez; Fernando Bryce; Gilda Mantilla; Philippe Gruenberg; Giancarlo Scaglia; revista Juanacha; La Culpable; MALI; galería Revólver</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta analiza la Colección Hochschild como caso paradigmático del coleccionismo privado de arte contemporáneo peruano, sosteniendo que todo desarrollo artístico notable requiere un coleccionismo a la altura de su ambición, junto con crítica y testimonio histórico escrito. El coleccionista, figura clave de todo sistema artístico moderno, opera a la vez como catalizador de la escena y motor del mercado. Iniciada en 2009 por Eduardo y Mariana Hochschild, la colección se distingue por seguir la dinámica actual del sistema de las artes visuales en un medio que careció de coleccionismo corporativo sostenido, escasa crítica periodística y pocas publicaciones especializadas —una 'orfandad' de los artistas. Villacorta subraya que los Hochschild rompieron el molde del coleccionismo centrado en el arte moderno al adquirir netamente arte contemporáneo con asesoramiento profesional (Luis Pérez Oramas, Giancarlo Scaglia) en ausencia de una historiografía orgánica del arte peruano desde 1980. Contextualiza el aislamiento económico y la violencia de los años ochenta y noventa que invisibilizaron a dos generaciones de artistas, y el dinamismo que trajeron la Bienal Iberoamericana de Lima (1997) y el Festival de Video/Arte Electrónico (1998). Comenta la selección de Octavio Zaya para 'Próxima parada' y la tríada Aprijaskis-Eielson-Burga como artistas que escapan al arte moderno local e inauguran lo contemporáneo. Ejemplifica el 'punto ciego' del coleccionista limeño con 'Atlas Perú' de Fernando Bryce, vendido al exterior, y aborda la tensión entre relevancia cultural nacional y reconocimiento del mercado internacional. Cita cimientos modernos (Sabogal, Szyszlo, Tsuchiya) y fortalezas en escultura, instalación y fotografía (Chambi, Testino, Martinat, Damiani), afirmando que la colección materializa una visión cabal del arte peruano contemporáneo.</t>
+          <t>Dossier «Lima se anima» de la revista argentina ramona (nº 89, abril 2009), coeditado con la publicación limeña Juanacha por Rodrigo Quijano y Eliana Otta, que ofrece una radiografía crítica de la escena artística peruana ante su reciente revinculación con el circuito internacional. Reúne una conversación entre artistas («Perú, ¿país blindado?») con Alfredo Márquez, Fernando Bryce, Gilda Mantilla, Philippe Gruenberg y Giancarlo Scaglia; ensayos de Miguel López y Max Hernández-Calvo; un debate virtual del blog Arte-Nuevo sobre las políticas museales; un texto de Gustavo Buntinx (Micromuseo) y una entrevista a Jorge Villacorta. El hilo común es la interrogación del supuesto «boom» del arte contemporáneo limeño de la última década: los participantes coinciden en que la internacionalización y el crecimiento del mercado y del coleccionismo (impulsado por el MALI) han producido una escena «contrahecha», con brazos de mercado pero sin instituciones, crítica, educación ni políticas culturales. Márquez denuncia el carácter colonial y exótico de esa visibilidad; López («Boo(o)m: Morir de éxito») teoriza un proceso de despolitización y domesticación que diluye el conflicto y convierte la autonomía en aquiescencia entre agentes; Hernández-Calvo («Una coyuntura que no fue») analiza cómo las Bienales de Lima (1997-2002) forzaron una «contemporaneización» de instalación y video sin sustento curatorial ni educativo, generando escisiones entre circuito oficial y alternativo. Se abordan además el éxodo de artistas por la deficiente formación, la toma estudiantil de Bellas Artes, la autogestión (La Culpable) y las disputas por el Museo de la Memoria. El dossier reivindica la autonomía, el disenso y el filo crítico histórico del arte peruano.</t>
         </is>
       </c>
     </row>
@@ -2334,27 +2334,27 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Villacorta - Un arte cuestionador. De Dadá a La Cantuta [Quehacer 102, pdf pp. 96-105].md</t>
+          <t>VVAA - Memorias del subdesarrollo. Arte y el giro descolonial en América Latina, 1960-1985 [catálogo MCASD].md</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>1916-1996 (vanguardias históricas y arte peruano 1979-1995)</t>
+          <t>1960-1985 (con foco 1967-1981)</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Artículo de revista (Quehacer 102, DESCO), c. 1996</t>
+          <t>Catálogo de exposición / ensayo académico, 2018 (MCASD)</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Francisco Mariotti; Herbert Rodríguez; Ricardo Wiesse; Eduardo Villanes; Hugo Salazar del Alcázar; E.P.S. Huayco; Grupo Paréntesis; Los Bestias; Carpa Teatro del Puente Santa Rosa; Sendero Luminoso</t>
+          <t>Sharon Lerner; Julieta González; Andrea Giunta; Jacopo Crivelli Visconti; Juan Acha; Marta Traba; Ferreira Gullar; Teresa Burga; E.P.S. Huayco; Grupo Paréntesis; Jesús Ruiz Durand; Fernando 'Coco' Bedoya; MALI; Museum of Contemporary Art San Diego</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>En este artículo para la revista Quehacer (DESCO), dedicado in memoriam a Hugo Salazar del Alcázar, Jorge Villacorta traza una genealogía del arte peruano contestatario que la generación más joven de artistas visuales estaría redescubriendo como una tradición alternativa o 'canon no-oficial', paralelo al aceptado. Su tesis vincula esa tradición local con las vanguardias históricas internacionales: la deuda con Dadá (Zúrich, 1916) como rechazo crítico de la civilización occidental tras la carnicería bélica, el manifiesto como obra del futurismo, y el constructivismo ruso con su noción de arte como agit-prop. Aplica ese marco a la 'movida barranquina' de fines de los años setenta, primera generación ligada a una cultura juvenil limeña irreverente y a los medios masivos, donde grupos como Paréntesis y Huayco entendieron la creación como provocación y enfrentamiento; destaca la serigrafía enseñada por Mariotti y la salida de Huayco de la galería hacia el kilómetro 54 de la Panamericana Sur. Narra luego cómo la violencia de Sendero Luminoso desde 1980, el fracaso de Izquierda Unida y la crisis marcaron el clima cultural: la exposición de Artistas Visuales Asociados (1983) y 'Por el Derecho a la Vida' (1985). Analiza la escena subterránea y la Carpa Teatro del Puente Santa Rosa (1986), con Los Bestias y el fanzine, y el proyecto solitario Arte Vida de Herbert Rodríguez en San Marcos entre 1986 y 1992. Concluye con la respuesta ética ante el caso La Cantuta: la exposición de Eduardo Villanes con cajas de leche Gloria (1994) y la acción ambiental de Ricardo Wiesse con flores de cantuta en Cieneguilla (1995), afirmando un arte que asume responsabilidades éticas frente a los desaparecidos.</t>
+          <t>El ensayo de Sharon Lerner incluido en el catálogo de la exposición 'Memorias del subdesarrollo: arte y el giro descolonial en América Latina, 1960-1985' inserta la escena peruana de 1967-1981 en una narrativa continental que postula una ruptura epistémica con lo moderno mediante la noción de subdesarrollo y el deseo de descolonizar los cánones estéticos impuestos. Su tesis desplaza el foco del paradigma formalista modernista hacia el contexto social, la apropiación de tradiciones locales y lo 'popular' como categoría clave, cuya heterogeneidad histórica advierte no homogeneizar. Reconstruye el debate entre Juan Acha y Marta Traba sobre el pop cosmopolita y la dependencia cultural, apoyándose en Mariátegui, Ferreira Gullar y Mário Pedrosa, y en la teoría de la dependencia. Analiza casos peruanos: los afiches de la Reforma Agraria de Jesús Ruiz Durand y su 'pop achorado' dentro de SINAMOS; los festivales Contacta y las Carreras de Chasquis de Luis Arias Vera bajo el velasquismo; el Grupo Paréntesis y el Contacta 79 (Becerro de oro, Coquito) de Fernando Bedoya; y sobre todo E.P.S. Huayco, con 'Arte al paso (Salchipapas)' y 'Sarita Colonia', leídos vía Buntinx y Lauer como articulación de lo popular urbano migrante. Suma el caso aislado de Teresa Burga y 'Perfil de la mujer peruana' (1980-81) como acercamiento conceptual a género y clase. Recurriendo a Bürger y Giunta, discute la definición de vanguardia y concluye que estas prácticas oscilaron entre dependencia y autonomía, sin lograr plataformas de continuidad, siendo Huayco el caso más próximo a una vanguardia local pese a su disolución.</t>
         </is>
       </c>
     </row>
@@ -2366,27 +2366,27 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Villacorta y Del Valle - Incertidumbre y certezas en el arte peruano reciente. Imaginarios de Lima en transformación 1980-2006 [Post-Ilusiones].txt</t>
+          <t>Vich - La violencia, la dictadura y la globalización. Arte y política en el Perú contemporáneo.md</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>1919-2006 (con eje central 1980-2006)</t>
+          <t>1980-2009 (violencia política, dictadura fujimorista y posconflicto)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de libro/catálogo (Post-Ilusiones), c. 2007</t>
+          <t>Ensayo / capítulo de libro académico, c. 2013-2015</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta Chávez; Augusto del Valle Cárdenas; José Sabogal; Juan Acha; Marta Traba; Fernando de Szyszlo; Jorge Eduardo Eielson; Emilio Rodríguez Larraín; E.P.S. Huayco; Escuela Nacional de Bellas Artes; IAC; Agrupación Espacio</t>
+          <t>Víctor Vich; Eduardo Tokeshi; Colectivo Sociedad Civil; Natalia Iguíñiz; Sandro Venturo; Piero Quijano; Luz Letts; Víctor Delfín; Miguel Cordero; Jaime Higa; Herbert Rodríguez; Claudia Martínez; Santiago Quintanilla; Rudolph Castro; Felipe López; Gustavo Buntinx</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta y Augusto del Valle proponen un ensayo panorámico sobre el arte peruano reciente que lee la transformación de los imaginarios de Lima entre 1980 y 2006 a partir de una tesis de fondo: en el Perú la academia y sus modelos artísticos comenzaron tarde e hicieron crisis temprano. Recorren la fundación de la Escuela Nacional de Bellas Artes (1919), la retorización del indigenismo de Sabogal como vanguardia institucionalizada, el rol del IAC (1955-1972) en la difusión del arte 'culto' y su negociación con modelos norteamericanos, y la tensión entre 'alta' y 'baja' cultura heredada de la intelligentsia marxista tras la Revolución cubana. Interpretan el populismo cultural del gobierno militar (Velasco y Morales Bermúdez), el premio a López Antay (1975) y el receso de Bellas Artes (1977) como síntomas del agotamiento de una visión del arte, frente al modelo pedagógico expresivo-trascendente de Winternitz en la PUCP. El eje del texto es la categoría de no-objetualismo de Juan Acha, que articulan en dos oleadas: un primer no-objetualismo utópico de izquierda (E.P.S. Huayco) y un segundo, ligado a la Movida Subterránea y a la Carpa Teatro del Puente Santa Rosa (1986). Analizan la precariedad de los años ochenta bajo la violencia y la crisis del primer gobierno de García, el neoliberalismo autocrático fujimorista como silenciador del arte crítico y productor de espectáculo, y la centralidad creciente de la fotografía, el video y el arte electrónico desde las bienales de Lima (1997) y el Festival de Video (1998). Concluyen con el tránsito del no-objetualismo político al poético y con la 'choledad digital' y la globalización del imaginario como horizonte contemporáneo.</t>
+          <t>Víctor Vich propone una lectura desde la crítica cultural del arte peruano contemporáneo, sosteniendo que, frente al discurso triunfalista del crecimiento económico, un sector de artistas sigue nombrando al país a partir de sus heridas históricas. Estructura el ensayo en torno a tres acontecimientos: la violencia política, el autoritarismo corrupto del fujimontesinismo y la globalización neoliberal. Apoyándose en Žižek, Hall, Jameson, Foucault y Badiou, entiende lo simbólico no como reflejo sino como soporte de la realidad y campo de batalla donde se disputan sentidos de ciudadanía. Analiza obras emblemáticas: 'Bandera VIII' (2000) de Eduardo Tokeshi, leída como 'la patria en cuidados intensivos'; 'Lava la bandera' del Colectivo Sociedad Civil; la instalación 'Patria' de Natalia Iguíñiz y Sandro Venturo; el afiche censurado de Piero Quijano sobre La Cantuta e Iwo Jima; 'El azar como destino' de Luz Letts; 'El hermoso general' de Víctor Delfín; el saco militar de Miguel Cordero; y las serigrafías de César Vallejo de Jaime Higa sobre posmodernismo y cultura de masas. En una segunda sección sobre memoria generacional examina a artistas nacidos en los ochenta que 'traducen' la violencia con lenguajes heredados de la infancia: la serie 'Invisible' de Claudia Martínez, el trabajo de archivo y cómic de Santiago Quintanilla, los juguetes siniestros (Lego, Playmobil) de Rudolph Castro y las fotografías de nichos ayacuchanos de Felipe López. Su aporte es articular teoría psicoanalítica y poscolonial con un corpus visual peruano, mostrando el arte crítico como agente que interrumpe la ficción neoliberal y recompone la comunidad desde el orden simbólico.</t>
         </is>
       </c>
     </row>
@@ -2398,27 +2398,27 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Villegas_Fernando_La_relacion_entre_arte.pdf</t>
+          <t>Vidarte - Exhibiciones y adquisiciones para la construcción de narrativas en la historia del arte contemporáneo peruano.md</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>1920-1976 (con proyecciones hasta 2013)</t>
+          <t>2015-2023</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Artículo académico, 2013 (Revista de Historiografía, N.º 19)</t>
+          <t>Ensayo curatorial de catálogo, 2023</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Fernando Villegas; José Sabogal; Joaquín López Antay; José Carlos Mariátegui; Fernando de Szyszlo; Carlos Quízpez Asín; Instituto de Arte Peruano; Amauta; ASPAP; Juan Velasco Alvarado; Universidad Complutense de Madrid; Néstor García Canclini</t>
+          <t>Giuliana Vidarte; ICPNA; Natalia Iguíñiz; Carlos García Montero; Venuca Evanán; Nereida Apaza; Gloria Quispe; Cristina Flores; Antonio Paucar; Andrés Argüelles Vigo; Carolina Estrada; Santiago Yahuarcani; Ana de Orbegoso</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Artículo de Fernando Villegas (Universidad Complutense de Madrid), publicado en la Revista de Historiografía N.º 19 (2013, pp. 75-87), que rastrea la evolución de los enfoques ideológicos sobre el arte popular peruano vinculando arte y política en dos momentos clave. El primero es el proyecto mestizo de José Sabogal en los años veinte: tras su viaje a México (1923) y en sintonía con la búsqueda de peruanidad de Mariátegui y la revista Amauta, Sabogal revaloriza mates burilados, queros y retablos como productos mestizos, fusión de lo indígena precolombino y lo virreinal hispano. Desde el Instituto de Arte Peruano (1931) su grupo estudia la cerámica precolombina, el color y las artes populares, legitimando estos objetos por su origen indígena pero desplazando al artista popular como creador (los pintores urbanos se autoproclaman sus 'descubridores'). El segundo momento es la polémica de 1975-1976, cuando el gobierno militar de Velasco otorgó el Premio Nacional de Cultura al retablista ayacuchano Joaquín López Antay; la ASPAP y artistas académicos lo descalificaron como 'artesano', reproduciendo la jerarquía social y racial limeña. Villegas argumenta que ambos episodios responden a gobiernos autoritarios que legitimaron el arte popular para oponerse a la oligarquía limeña, y que el criterio de validación siempre fue estético-cronológico, ignorando el proceso histórico. El marco conceptual moviliza a Mariátegui, a Clifford (apropiación de objetos de otras culturas) y a García Canclini (descontextualización). Su aporte es evidenciar la ausencia del artista popular como sujeto de su propia obra y la carga étnica y de clase que desnaturaliza el proceso creativo andino en el circuito artístico peruano.</t>
+          <t>Giuliana Vidarte reflexiona sobre la exposición 'Miradas contemporáneas. Nuevas adquisiciones en la colección ICPNA (2015-2023)', presentada en el Espacio Juan Pardo Heeren del ICPNA de Lima entre agosto y septiembre de 2023. Su argumento central es que las exhibiciones y adquisiciones institucionales son dispositivos para la construcción de narrativas y memoria crítica en la historia del arte contemporáneo peruano: una colección formada a partir de obras que fueron parte de la propia programación expositiva constituye un testimonio de los modos de creación y conserva la memoria de la historia de las exposiciones en el país. Parte de dos ganadoras del Premio ICPNA de Arte Contemporáneo, Venuca Evanán y Nereida Apaza, para introducir cómo el arte contribuye a pensar la realidad mediante reflexiones colectivas sobre violencia de género, identidad y nación. Describe los cinco ejes curatoriales de la muestra —revalorando intimidades, discursos críticos, develando entornos, reinterpretar tradiciones y estéticas disímiles— y analiza diálogos entre obras: el cuerpo y la caja torácica en Gloria Quispe, Cristina Flores y Antonio Paucar; la crítica a la representación colonial y republicana en Andrés Argüelles Vigo y Carolina Estrada/Teodoro Ramírez; el paisaje y la crisis medioambiental amazónica en Silvia Westphalen y Nicole Franchy; la reinterpretación de saberes ancestrales en Santiago Yahuarcani y Ana de Orbegoso. Destaca que las fichas incorporan citas de textos curatoriales previos, nutriendo la exposición del archivo documental institucional. Concluye que estos conjuntos abren líneas múltiples de lectura y afirman el valor del esfuerzo colectivo de gestores, curadores e investigadores en la formación de colecciones y en la escritura de la historia del arte peruano reciente.</t>
         </is>
       </c>
     </row>
@@ -2430,27 +2430,27 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>arte nuevo_ Contra el Consenso de Lima_ Notas incompletas sobre las colectividades artísticas en el Perú, sus nuevas, viejas condiciones - Rodrigo Quijano.pdf</t>
+          <t>Villacorta - La colección Hochschild.md</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Perú postdictatorial (años 2000); escrito en 2009 (masacre de Bagua, 5-jun-2009); colectivos 1979-1991 y «Consenso» desde fines de los 80</t>
+          <t>1980-2016 (con énfasis en el arte peruano desde 2000)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de revista (chilena «Plus», Trienal de Santiago; también en «Hacia el salón del siglo XXI», ArteBA, 2009, pp. 168-178); PDF = captura del blog «arte nuevo» (Miguel López), 29-dic-2009</t>
+          <t>Ensayo de catálogo de colección, c. 2016</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Quijano; Miguel López (blog «arte nuevo»); Alfredo Márquez; Mario Vargas Llosa; Gustavo Buntinx; Ana Longoni; grupos Paréntesis, Huayco, N.N., La Culpable, Tupac, El Colectivo, Proyecto Cultural Noviembre; MALI; Museo de la Memoria; CVR; Trienal de Santiago; ArteBA</t>
+          <t>Jorge Villacorta Chávez; Eduardo y Mariana Hochschild; Octavio Zaya; Luis Pérez Oramas; Giancarlo Scaglia; Fernando Bryce; Teresa Burga; Tilsa Tsuchiya; Jorge Eduardo Eielson; Regina Aprijaskis; MALI; MoMA; Tate Modern</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Ensayo de Rodrigo Quijano, «Contra el Consenso de Lima. Notas incompletas sobre las colectividades artísticas en el Perú, sus nuevas, viejas condiciones», publicado en la revista chilena «Plus» (Trienal de Santiago) y reproducido en «Hacia el salón del siglo XXI» (ArteBA Fundación, 2009, pp. 168-178). El PDF es una captura del blog «arte nuevo» de Miguel López, que lo reposteó el 29 de diciembre de 2009 (con la presentación de López, el índice de Ramona 89, los comentarios de lectores y el aparato del blog). Quijano acuña la noción de «Consenso de Lima» —por alusión al Consenso de Washington— para nombrar el «espeso consenso cultural y social» conformista impuesto por la dictadura fujimorista (1990-2000) y sostenido después: una «reoligarquización simbólica» del escenario nacional (iniciada tras el intento de estatizar la banca a fines de los 80, con Vargas Llosa), un neonacionalismo (pisco, caballo de paso, comida) y la reconcentración del «producto simbólico y artístico en pocas manos privadas», con su «nuevo coleccionismo y nueva musealidad» (MALI; un frustrado Museo de Arte Moderno; un futuro Museo de la Memoria ligado a la CVR). Frente a ese consenso sitúa a las «colectividades artísticas y críticas» surgidas «a contrapelo»: Paréntesis (1979), Huayco (1980-1981), N.N. (1986-1991) y, más recientes, La Culpable, Tupac, El Colectivo o el Proyecto Cultural Noviembre. La tercera sección lee la masacre de Bagua (5 de junio de 2009, gobierno de Alan García) como el episodio que «develó» y «contradijo» el Consenso. Fuente sobre arte, colectivos y política en el Perú postdictatorial.</t>
+          <t>Jorge Villacorta analiza la Colección Hochschild como caso paradigmático del coleccionismo privado de arte contemporáneo peruano, sosteniendo que todo desarrollo artístico notable requiere un coleccionismo a la altura de su ambición, junto con crítica y testimonio histórico escrito. El coleccionista, figura clave de todo sistema artístico moderno, opera a la vez como catalizador de la escena y motor del mercado. Iniciada en 2009 por Eduardo y Mariana Hochschild, la colección se distingue por seguir la dinámica actual del sistema de las artes visuales en un medio que careció de coleccionismo corporativo sostenido, escasa crítica periodística y pocas publicaciones especializadas —una 'orfandad' de los artistas. Villacorta subraya que los Hochschild rompieron el molde del coleccionismo centrado en el arte moderno al adquirir netamente arte contemporáneo con asesoramiento profesional (Luis Pérez Oramas, Giancarlo Scaglia) en ausencia de una historiografía orgánica del arte peruano desde 1980. Contextualiza el aislamiento económico y la violencia de los años ochenta y noventa que invisibilizaron a dos generaciones de artistas, y el dinamismo que trajeron la Bienal Iberoamericana de Lima (1997) y el Festival de Video/Arte Electrónico (1998). Comenta la selección de Octavio Zaya para 'Próxima parada' y la tríada Aprijaskis-Eielson-Burga como artistas que escapan al arte moderno local e inauguran lo contemporáneo. Ejemplifica el 'punto ciego' del coleccionista limeño con 'Atlas Perú' de Fernando Bryce, vendido al exterior, y aborda la tensión entre relevancia cultural nacional y reconocimiento del mercado internacional. Cita cimientos modernos (Sabogal, Szyszlo, Tsuchiya) y fortalezas en escultura, instalación y fotografía (Chambi, Testino, Martinat, Damiani), afirmando que la colección materializa una visión cabal del arte peruano contemporáneo.</t>
         </is>
       </c>
     </row>
@@ -2462,27 +2462,27 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>canepa_kg_2006_p132-167.pdf</t>
+          <t>Villacorta - Un arte cuestionador. De Dadá a La Cantuta [Quehacer 102, pdf pp. 96-105].md</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>1970-2006 (con referencias históricas desde el siglo XIX)</t>
+          <t>1916-1996 (vanguardias históricas y arte peruano 1979-1995)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Capítulo de libro, 2006</t>
+          <t>Artículo de revista (Quehacer 102, DESCO), c. 1996</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Giuliana Borea Labarthe; Gisela Cánepa Koch (ed.); Sandra Gamarra (LiMAC); Instituto de Arte Contemporáneo (IAC); Fernando de Szyszlo; Gerardo Chávez; Mario Vargas Llosa; Ramiro Llona; Instituto Nacional de Cultura; ICOM; Museo de la Nación; Museo Nacional de la Cultura Peruana; Alfonso Castrillón</t>
+          <t>Jorge Villacorta; Francisco Mariotti; Herbert Rodríguez; Ricardo Wiesse; Eduardo Villanes; Hugo Salazar del Alcázar; E.P.S. Huayco; Grupo Paréntesis; Los Bestias; Carpa Teatro del Puente Santa Rosa; Sendero Luminoso</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Capítulo de Giuliana Borea Labarthe ('Museos y esfera pública: espacio, discursos y prácticas. Reflexiones en torno a la ciudad de Lima') incluido en el volumen editado por Gisela Cánepa Koch, 'Mirando la esfera pública desde la cultura en el Perú' (2006). Partiendo de las nociones de esfera pública (Habermas), cultura pública (Appadurai) y de la nueva museología surgida de las crisis de los años 70-80 (Mesa de Santiago 1972, redefinición del ICOM 1974, ecomuseos), Borea concibe el museo como contenedor y contenido, plataforma y discurso, esfera de poder y arena de disputa por la representación. Analiza tres casos limeños. Primero, el posicionamiento urbano de los museos: mediante una encuesta a transeúntes y taxistas muestra que solo el Museo de la Nación y el Museo de Arte de Lima son hitos reconocidos, mientras la mayoría oscila entre lugar simbólico y lugar anónimo por la falta de señalización y de alianzas municipales. Segundo, la polémica de 2006 por el proyecto del Museo de Arte Contemporáneo (MAC) del IAC, detonada por el intento de nombrarlo 'Fernando de Szyszlo': reconstruye siete momentos del debate mediático (comunicados de artistas, la columna 'Escaramuzas en Liliput' de Vargas Llosa), la falta de plan museológico y de diálogo con artistas donantes y con Barranco, y destaca la contrapropuesta crítica LiMAC de Sandra Gamarra frente al silencio del INC. Tercero, compara las puestas en escena sobre peruanidad y diversidad de cinco museos (Cultura Peruana, de la Nación, Etnográfico, Inmigración Japonesa, MNAAHP), evidenciando discursos lejanos, fragmentados y ahistóricos en los grandes museos nacionales frente a autorrepresentaciones más políticas en los pequeños. Cierra con Castrillón: Lima como escenario de emplazamiento, no de reflexión.</t>
+          <t>En este artículo para la revista Quehacer (DESCO), dedicado in memoriam a Hugo Salazar del Alcázar, Jorge Villacorta traza una genealogía del arte peruano contestatario que la generación más joven de artistas visuales estaría redescubriendo como una tradición alternativa o 'canon no-oficial', paralelo al aceptado. Su tesis vincula esa tradición local con las vanguardias históricas internacionales: la deuda con Dadá (Zúrich, 1916) como rechazo crítico de la civilización occidental tras la carnicería bélica, el manifiesto como obra del futurismo, y el constructivismo ruso con su noción de arte como agit-prop. Aplica ese marco a la 'movida barranquina' de fines de los años setenta, primera generación ligada a una cultura juvenil limeña irreverente y a los medios masivos, donde grupos como Paréntesis y Huayco entendieron la creación como provocación y enfrentamiento; destaca la serigrafía enseñada por Mariotti y la salida de Huayco de la galería hacia el kilómetro 54 de la Panamericana Sur. Narra luego cómo la violencia de Sendero Luminoso desde 1980, el fracaso de Izquierda Unida y la crisis marcaron el clima cultural: la exposición de Artistas Visuales Asociados (1983) y 'Por el Derecho a la Vida' (1985). Analiza la escena subterránea y la Carpa Teatro del Puente Santa Rosa (1986), con Los Bestias y el fanzine, y el proyecto solitario Arte Vida de Herbert Rodríguez en San Marcos entre 1986 y 1992. Concluye con la respuesta ética ante el caso La Cantuta: la exposición de Eduardo Villanes con cajas de leche Gloria (1994) y la acción ambiental de Ricardo Wiesse con flores de cantuta en Cieneguilla (1995), afirmando un arte que asume responsabilidades éticas frente a los desaparecidos.</t>
         </is>
       </c>
     </row>
@@ -2494,27 +2494,27 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>mac-proyecto-2008.md</t>
+          <t>Villacorta y Del Valle - Incertidumbre y certezas en el arte peruano reciente. Imaginarios de Lima en transformación 1980-2006 [Post-Ilusiones].txt</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>2008 (exposición feb.–mar. 2008; con historia del sitio desde 1944)</t>
+          <t>1919-2006 (con eje central 1980-2006)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de exposición, mayo 2008 (Instituto de Arte Contemporáneo — MAC-Lima; OCR)</t>
+          <t>Ensayo de libro/catálogo (Post-Ilusiones), c. 2007</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Jorge Villacorta; Miguel Zegarra (curadores); Instituto de Arte Contemporáneo (IAC); MAC-Lima; Giuliana Borea; George Gruenberg; Ricardo Ramón Jarne; José Carlos Martinat; Ishmael Randall Weeks; Elena Damiani; Sergio Abugattás; Raura Oblitas</t>
+          <t>Jorge Villacorta Chávez; Augusto del Valle Cárdenas; José Sabogal; Juan Acha; Marta Traba; Fernando de Szyszlo; Jorge Eduardo Eielson; Emilio Rodríguez Larraín; E.P.S. Huayco; Escuela Nacional de Bellas Artes; IAC; Agrupación Espacio</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Catálogo de la exposición «La Construcción del Lugar Común» (MAC-Lima, 5 de febrero–30 de marzo de 2008), editado por el Instituto de Arte Contemporáneo (IAC) y curado por Jorge Villacorta y Miguel Zegarra. Documenta una intervención colectiva de quince artistas peruanos emergentes —Sergio Abugattás, Miguel Andrade, Víctor Castro, Elena Damiani, Giuseppe De Bernardi, Nicole Franchy, Alejandro Jaime, Manuel Larrea, Martín Jiménez Paz, Christians Luna, José Carlos Martinat, José Miyashiro, Raura Oblitas, Ishmael Randall Weeks e Iliana Scheggia— que ocuparon el edificio del Museo de Arte Contemporáneo de Lima cuando aún estaba a medio construir. La muestra convirtió la arquitectura inconclusa y su entorno (el parque de la antigua «laguna» de Barranco) en soporte y tema: las obras tematizan la construcción/destrucción, el paisaje, la memoria del sitio y la disputa pública por el museo, cuyo proceso estuvo marcado por conflictos municipales y un intento de clausura respondido con el gesto «CLAUSURADO = INAUGURADO». El catálogo reúne textos institucionales (George Gruenberg, presidente del IAC), una pieza literaria de Ricardo Ramón Jarne («La maldición de la laguna»), un ensayo antropológico de Giuliana Borea sobre la construcción del lugar y el «lugar común» en la esfera pública (apoyado en Augé, Appadurai, Certeau y Casey), el texto curatorial de Villacorta y Zegarra, y los statements de cada artista. Como fuente histórica documenta un episodio clave de institucionalización del arte contemporáneo en Lima —la génesis del MAC— y las prácticas site-specific, de crítica institucional y de intervención en el espacio público de una generación emergente peruana de fines de la década de 2000.</t>
+          <t>Jorge Villacorta y Augusto del Valle proponen un ensayo panorámico sobre el arte peruano reciente que lee la transformación de los imaginarios de Lima entre 1980 y 2006 a partir de una tesis de fondo: en el Perú la academia y sus modelos artísticos comenzaron tarde e hicieron crisis temprano. Recorren la fundación de la Escuela Nacional de Bellas Artes (1919), la retorización del indigenismo de Sabogal como vanguardia institucionalizada, el rol del IAC (1955-1972) en la difusión del arte 'culto' y su negociación con modelos norteamericanos, y la tensión entre 'alta' y 'baja' cultura heredada de la intelligentsia marxista tras la Revolución cubana. Interpretan el populismo cultural del gobierno militar (Velasco y Morales Bermúdez), el premio a López Antay (1975) y el receso de Bellas Artes (1977) como síntomas del agotamiento de una visión del arte, frente al modelo pedagógico expresivo-trascendente de Winternitz en la PUCP. El eje del texto es la categoría de no-objetualismo de Juan Acha, que articulan en dos oleadas: un primer no-objetualismo utópico de izquierda (E.P.S. Huayco) y un segundo, ligado a la Movida Subterránea y a la Carpa Teatro del Puente Santa Rosa (1986). Analizan la precariedad de los años ochenta bajo la violencia y la crisis del primer gobierno de García, el neoliberalismo autocrático fujimorista como silenciador del arte crítico y productor de espectáculo, y la centralidad creciente de la fotografía, el video y el arte electrónico desde las bienales de Lima (1997) y el Festival de Video (1998). Concluyen con el tránsito del no-objetualismo político al poético y con la 'choledad digital' y la globalización del imaginario como horizonte contemporáneo.</t>
         </is>
       </c>
     </row>
@@ -2526,379 +2526,379 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>sura.md</t>
+          <t>Villegas_Fernando_La_relacion_entre_arte.pdf</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>mediados de la década de 1960 a 2013 (arte contemporáneo peruano)</t>
+          <t>1920-1976 (con proyecciones hasta 2013)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de colección museística, 2013</t>
+          <t>Artículo académico, 2013 (Revista de Historiografía, N.º 19)</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner (ed.); Museo de Arte de Lima (MALI); Grupo SURA; Mirko Lauer; E.P.S. Huayco; Charo Noriega; Ramiro Llona; Flavia Gandolfo; Armando Andrade Tudela; Ricardo Wiesse; Eduardo Villanes; Miguel A. López; Rodrigo Quijano</t>
+          <t>Fernando Villegas; José Sabogal; Joaquín López Antay; José Carlos Mariátegui; Fernando de Szyszlo; Carlos Quízpez Asín; Instituto de Arte Peruano; Amauta; ASPAP; Juan Velasco Alvarado; Universidad Complutense de Madrid; Néstor García Canclini</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Catálogo de la colección de arte contemporáneo del Museo de Arte de Lima (MALI), editado por la curadora Sharon Lerner y publicado con el patrocinio del grupo SURA. El volumen traza los derroteros del arte peruano reciente a partir del acervo del museo, sin pretender definir un 'arte peruano' esencial. La colección se articula bajo dos principios: identificar momentos de ruptura en la producción artística de fines del siglo XX y perfilar la producción reciente mediante ejes temáticos comunes. El ensayo central de Lerner establece como punto de partida mediados de la década de 1960 (grupos de vanguardia ligados al Pop y al no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, tras las reformas del Gobierno Militar, cuando —según la célebre frase de Mirko Lauer para la muestra Arte al paso del colectivo E.P.S. Huayco (1980)— 'en el Perú hoy solo lo popular es moderno'. Analiza la irrupción de la migración interna, el conflicto armado interno, el autogolpe de Fujimori (1992) y la virtual desaparición de la esfera pública, así como la Bienal Iberoamericana de Lima (1997) como puesta al día forzada y descontextualizada. El catálogo se organiza en núcleos temáticos: modernidad popular y transformación de Lima, f(r)icciones cosmopolitas, reconsideración del pasado y configuración del Perú, sistema artístico y utopías museales, desplazamientos, y signos de violencia, resistencia y memoria. Incluye obras de Charo Noriega, Ramiro Llona, Flavia Gandolfo, Armando Andrade Tudela, Herman Schwarz, Ricardo Wiesse y Eduardo Villanes, entre otros, y textos críticos complementarios. Su aporte es consolidar un relato historiográfico y crítico del arte contemporáneo peruano desde una institución museal.</t>
+          <t>Artículo de Fernando Villegas (Universidad Complutense de Madrid), publicado en la Revista de Historiografía N.º 19 (2013, pp. 75-87), que rastrea la evolución de los enfoques ideológicos sobre el arte popular peruano vinculando arte y política en dos momentos clave. El primero es el proyecto mestizo de José Sabogal en los años veinte: tras su viaje a México (1923) y en sintonía con la búsqueda de peruanidad de Mariátegui y la revista Amauta, Sabogal revaloriza mates burilados, queros y retablos como productos mestizos, fusión de lo indígena precolombino y lo virreinal hispano. Desde el Instituto de Arte Peruano (1931) su grupo estudia la cerámica precolombina, el color y las artes populares, legitimando estos objetos por su origen indígena pero desplazando al artista popular como creador (los pintores urbanos se autoproclaman sus 'descubridores'). El segundo momento es la polémica de 1975-1976, cuando el gobierno militar de Velasco otorgó el Premio Nacional de Cultura al retablista ayacuchano Joaquín López Antay; la ASPAP y artistas académicos lo descalificaron como 'artesano', reproduciendo la jerarquía social y racial limeña. Villegas argumenta que ambos episodios responden a gobiernos autoritarios que legitimaron el arte popular para oponerse a la oligarquía limeña, y que el criterio de validación siempre fue estético-cronológico, ignorando el proceso histórico. El marco conceptual moviliza a Mariátegui, a Clifford (apropiación de objetos de otras culturas) y a García Canclini (descontextualización). Su aporte es evidenciar la ausencia del artista popular como sujeto de su propia obra y la carga étnica y de clase que desnaturaliza el proceso creativo andino en el circuito artístico peruano.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Arte al Paso 2011</t>
+          <t>Cap 2 - Historia</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Arte al Paso - Texto Investigación.md</t>
+          <t>arte nuevo_ Contra el Consenso de Lima_ Notas incompletas sobre las colectividades artísticas en el Perú, sus nuevas, viejas condiciones - Rodrigo Quijano.pdf</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 1960 – 2010 (con foco en las décadas de 1970-2000 y el conflicto armado interno 1980-2000)</t>
+          <t>Perú postdictatorial (años 2000); escrito en 2009 (masacre de Bagua, 5-jun-2009); colectivos 1979-1991 y «Consenso» desde fines de los 80</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Ensayo curatorial de catálogo (exposición Arte al paso, Pinacoteca do Estado de São Paulo, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Ensayo de revista (chilena «Plus», Trienal de Santiago; también en «Hacia el salón del siglo XXI», ArteBA, 2009, pp. 168-178); PDF = captura del blog «arte nuevo» (Miguel López), 29-dic-2009</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Pinacoteca de São Paulo; Emilio Hernández Saavedra; E.P.S. Huayco; Jesús Ruiz Durand; Sandra Gamarra; Alfredo Márquez / Taller NN; Fernando Bryce; José Carlos Martinat; Susana Torres</t>
+          <t>Rodrigo Quijano; Miguel López (blog «arte nuevo»); Alfredo Márquez; Mario Vargas Llosa; Gustavo Buntinx; Ana Longoni; grupos Paréntesis, Huayco, N.N., La Culpable, Tupac, El Colectivo, Proyecto Cultural Noviembre; MALI; Museo de la Memoria; CVR; Trienal de Santiago; ArteBA</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Ensayo curatorial extenso y bilingüe (castellano/portugués) de Tatiana Cuevas y Rodrigo Quijano para la muestra Arte al paso, que exhibió la coleccion contemporanea del MALI en la Estacion Pinacoteca de Sao Paulo. El texto toma como punto de partida la imagen El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra para diagnosticar los vacios institucionales y la distancia entre el discurso cultural cosmopolita y la practica real en el Peru de la segunda mitad del siglo XX. Su argumento articula el arte contemporaneo peruano con las transformaciones sociales derivadas de la masiva migracion rural a Lima, la explosion de la economia informal y la emergencia de una nueva cultura popular urbana. Rastrea las primeras vinculaciones locales con vanguardias internacionales (op, pop, conceptualismo, no-objetualismo), el pop achorado de Jesus Ruiz Durand y sus afiches de la Reforma Agraria velasquista, y las experiencias colectivas Contacta 79 y Arte al paso de E.P.S. Huayco (1980), que propusieron un arte callejero y antiinstitucional. Analiza la critica a la institucionalidad faltante (el museo ficticio LiMAC de Sandra Gamarra), el uso ironico del pasado prehispanico (Susana Torres, Rodriguez Larrain, Bryce, Cordova, Martinat), el tema del paisaje y el territorio, y la irrupcion tardia de la fotografia y la serigrafia como medios. Dedica una seccion central a la memoria de la violencia del conflicto armado interno (1980-2000) —Sendero Luminoso, MRTA, la Comision de la Verdad, 69.280 muertos— y su tratamiento por el Taller NN, Alfredo Marquez (Katatay), Carlos Dominguez, Ricardo Wiesse, Eduardo Villanes, Fernando Bryce y Milagros de la Torre.</t>
+          <t>Ensayo de Rodrigo Quijano, «Contra el Consenso de Lima. Notas incompletas sobre las colectividades artísticas en el Perú, sus nuevas, viejas condiciones», publicado en la revista chilena «Plus» (Trienal de Santiago) y reproducido en «Hacia el salón del siglo XXI» (ArteBA Fundación, 2009, pp. 168-178). El PDF es una captura del blog «arte nuevo» de Miguel López, que lo reposteó el 29 de diciembre de 2009 (con la presentación de López, el índice de Ramona 89, los comentarios de lectores y el aparato del blog). Quijano acuña la noción de «Consenso de Lima» —por alusión al Consenso de Washington— para nombrar el «espeso consenso cultural y social» conformista impuesto por la dictadura fujimorista (1990-2000) y sostenido después: una «reoligarquización simbólica» del escenario nacional (iniciada tras el intento de estatizar la banca a fines de los 80, con Vargas Llosa), un neonacionalismo (pisco, caballo de paso, comida) y la reconcentración del «producto simbólico y artístico en pocas manos privadas», con su «nuevo coleccionismo y nueva musealidad» (MALI; un frustrado Museo de Arte Moderno; un futuro Museo de la Memoria ligado a la CVR). Frente a ese consenso sitúa a las «colectividades artísticas y críticas» surgidas «a contrapelo»: Paréntesis (1979), Huayco (1980-1981), N.N. (1986-1991) y, más recientes, La Culpable, Tupac, El Colectivo o el Proyecto Cultural Noviembre. La tercera sección lee la masacre de Bagua (5 de junio de 2009, gobierno de Alan García) como el episodio que «develó» y «contradijo» el Consenso. Fuente sobre arte, colectivos y política en el Perú postdictatorial.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Arte al Paso 2011</t>
+          <t>Cap 2 - Historia</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Cronología Político Artistica - Arte al Paso 2011.md</t>
+          <t>canepa_kg_2006_p132-167.pdf</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>1962 – 2010</t>
+          <t>1970-2006 (con referencias históricas desde el siglo XIX)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Cronología y bibliografía de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Capítulo de libro, 2006</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Museo de Arte de Lima (MALI); Grupo Arte Nuevo; Grupo Señal; E.P.S. Huayco; Taller NN; Colectivo Sociedad Civil; Gustavo Buntinx; Joaquín López Antay; Comisión de la Verdad y Reconciliación; Sendero Luminoso; Alberto Fujimori; Juan Velasco Alvarado</t>
+          <t>Giuliana Borea Labarthe; Gisela Cánepa Koch (ed.); Sandra Gamarra (LiMAC); Instituto de Arte Contemporáneo (IAC); Fernando de Szyszlo; Gerardo Chávez; Mario Vargas Llosa; Ramiro Llona; Instituto Nacional de Cultura; ICOM; Museo de la Nación; Museo Nacional de la Cultura Peruana; Alfonso Castrillón</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Cronologia politico-artistica bilingue (castellano/portugues) incluida en el catalogo Arte al paso, que entrelaza en paralelo tres series de acontecimientos —eventos politicos, eventos artisticos y adquisiciones de la coleccion de arte contemporaneo del MALI— entre 1962 y 2010. El documento funciona como aparato historiografico que contextualiza la escena artistica peruana dentro de sus convulsiones politicas: rebeliones campesinas y golpes militares de los anos sesenta, el Gobierno Revolucionario de las Fuerzas Armadas de Velasco Alvarado (1968) y la Reforma Agraria, el estallido del conflicto armado interno con Sendero Luminoso y el MRTA (1980), las masacres de Barrios Altos y La Cantuta, el autogolpe y la dictadura de Alberto Fujimori (1990-2000), la Marcha de los Cuatro Suyos y el Informe de la Comision de la Verdad y Reconciliacion (2003). En el plano artistico registra la formacion de los grupos Senal y Arte Nuevo, las Bienales de Lima e Iberoamericanas, los festivales Contacta e Inkarri, el Taller E.P.S. Huayco y el Taller NN, la premiacion de Joaquin Lopez Antay, y acciones de arte critico como Cantuta de Ricardo Wiesse, Gloria evaporada de Eduardo Villanes y Lava la bandera del Colectivo Sociedad Civil. Una tercera linea traza la institucionalizacion del MALI: el ciclo curatorial Miradas de fin de siglo, la creacion del Comite de Adquisiciones (2007) y la reapertura del museo (2010). Se acompana de una extensa bibliografia especializada (Buntinx, Castrillon, Lauer, Majluf, Lopez, Tarazona, Quijano, Villacorta), fuente clave para la historiografia del arte peruano contemporaneo.</t>
+          <t>Capítulo de Giuliana Borea Labarthe ('Museos y esfera pública: espacio, discursos y prácticas. Reflexiones en torno a la ciudad de Lima') incluido en el volumen editado por Gisela Cánepa Koch, 'Mirando la esfera pública desde la cultura en el Perú' (2006). Partiendo de las nociones de esfera pública (Habermas), cultura pública (Appadurai) y de la nueva museología surgida de las crisis de los años 70-80 (Mesa de Santiago 1972, redefinición del ICOM 1974, ecomuseos), Borea concibe el museo como contenedor y contenido, plataforma y discurso, esfera de poder y arena de disputa por la representación. Analiza tres casos limeños. Primero, el posicionamiento urbano de los museos: mediante una encuesta a transeúntes y taxistas muestra que solo el Museo de la Nación y el Museo de Arte de Lima son hitos reconocidos, mientras la mayoría oscila entre lugar simbólico y lugar anónimo por la falta de señalización y de alianzas municipales. Segundo, la polémica de 2006 por el proyecto del Museo de Arte Contemporáneo (MAC) del IAC, detonada por el intento de nombrarlo 'Fernando de Szyszlo': reconstruye siete momentos del debate mediático (comunicados de artistas, la columna 'Escaramuzas en Liliput' de Vargas Llosa), la falta de plan museológico y de diálogo con artistas donantes y con Barranco, y destaca la contrapropuesta crítica LiMAC de Sandra Gamarra frente al silencio del INC. Tercero, compara las puestas en escena sobre peruanidad y diversidad de cinco museos (Cultura Peruana, de la Nación, Etnográfico, Inmigración Japonesa, MNAAHP), evidenciando discursos lejanos, fragmentados y ahistóricos en los grandes museos nacionales frente a autorrepresentaciones más políticas en los pequeños. Cierra con Castrillón: Lima como escenario de emplazamiento, no de reflexión.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Arte al Paso 2011</t>
+          <t>Cap 2 - Historia</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Texto de la exposición Arte al Paso 2011.md</t>
+          <t>mac-proyecto-2008.md</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 1960 – 2010 (unos 40 años; foco en las décadas de 1970-1980)</t>
+          <t>2008 (exposición feb.–mar. 2008; con historia del sitio desde 1944)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Texto de sala / presentación de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Catálogo de exposición, mayo 2008 (Instituto de Arte Contemporáneo — MAC-Lima; OCR)</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Emilio Hernández Saavedra; E.P.S. Huayco; Grupo Paréntesis; Sandra Gamarra; Susana Torres; Emilio Rodríguez Larraín; Juan Javier Salazar; William Cordova; José Carlos Martinat</t>
+          <t>Jorge Villacorta; Miguel Zegarra (curadores); Instituto de Arte Contemporáneo (IAC); MAC-Lima; Giuliana Borea; George Gruenberg; Ricardo Ramón Jarne; José Carlos Martinat; Ishmael Randall Weeks; Elena Damiani; Sergio Abugattás; Raura Oblitas</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Texto de sala o presentacion general de la exposicion Arte al paso (coleccion contemporanea del MALI en la Pinacoteca de Sao Paulo), firmado por los curadores Tatiana Cuevas y Rodrigo Quijano, en edicion bilingue castellano/portugues. Es una version sintetica del argumento curatorial: parte nuevamente de El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra como metafora de la ausencia institucional y punto de arranque para examinar la escena artistica peruana desde fines de los anos sesenta. Explica el titulo de la muestra a partir de la accion Arte al paso de E.P.S. Huayco (1980) —que, aludiendo a los puestos informales de comida al paso surgidos con la migracion y la economia informal, propuso un arte para consumirse en la calle, opuesto al museo y la galeria ausentes, un arte para pensar y no para sentir que dejaba atras el modernismo conservador de mediados de siglo. Sintetiza cuarenta anos de produccion cultural marcados por oposiciones ocultas y explicitas, los primeros acercamientos al conceptualismo y a las vanguardias internacionales, y la creciente proyeccion internacional de artistas peruanos. Una segunda seccion, Critica ante una institucionalidad faltante y al poder redentor del pasado, reune a Hernandez Saavedra, los grupos Parentesis y E.P.S. Huayco y el museo ficticio de Sandra Gamarra como estrategias de critica institucional apropiadas del conceptualismo y del imaginario popular urbano, con recurrente uso del humor. Aborda ademas la critica a la explotacion comercial y politica de lo prehispanico (Museo Neo-Inka de Susana Torres) y el vinculo entre la retorica del glorioso pasado incaico y los fracasos politicos y economicos del presente en obras de Rodriguez Larrain, Salazar, Cordova y Martinat.</t>
+          <t>Catálogo de la exposición «La Construcción del Lugar Común» (MAC-Lima, 5 de febrero–30 de marzo de 2008), editado por el Instituto de Arte Contemporáneo (IAC) y curado por Jorge Villacorta y Miguel Zegarra. Documenta una intervención colectiva de quince artistas peruanos emergentes —Sergio Abugattás, Miguel Andrade, Víctor Castro, Elena Damiani, Giuseppe De Bernardi, Nicole Franchy, Alejandro Jaime, Manuel Larrea, Martín Jiménez Paz, Christians Luna, José Carlos Martinat, José Miyashiro, Raura Oblitas, Ishmael Randall Weeks e Iliana Scheggia— que ocuparon el edificio del Museo de Arte Contemporáneo de Lima cuando aún estaba a medio construir. La muestra convirtió la arquitectura inconclusa y su entorno (el parque de la antigua «laguna» de Barranco) en soporte y tema: las obras tematizan la construcción/destrucción, el paisaje, la memoria del sitio y la disputa pública por el museo, cuyo proceso estuvo marcado por conflictos municipales y un intento de clausura respondido con el gesto «CLAUSURADO = INAUGURADO». El catálogo reúne textos institucionales (George Gruenberg, presidente del IAC), una pieza literaria de Ricardo Ramón Jarne («La maldición de la laguna»), un ensayo antropológico de Giuliana Borea sobre la construcción del lugar y el «lugar común» en la esfera pública (apoyado en Augé, Appadurai, Certeau y Casey), el texto curatorial de Villacorta y Zegarra, y los statements de cada artista. Como fuente histórica documenta un episodio clave de institucionalización del arte contemporáneo en Lima —la génesis del MAC— y las prácticas site-specific, de crítica institucional y de intervención en el espacio público de una generación emergente peruana de fines de la década de 2000.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Hueso Húmero 18</t>
+          <t>Cap 2 - Historia</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - Arte joven peruano, ¿el sueño del mercado propio? Una conversación con Claudia Polar (1983) [Hueso Húmero 18, pp. 94-107].md</t>
+          <t>sura.md</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>1974-1983</t>
+          <t>mediados de la década de 1960 a 2013 (arte contemporáneo peruano)</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Entrevista en revista (Hueso Húmero 18), 1983</t>
+          <t>Catálogo de colección museística, 2013</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Claudia Polar; Galería Forum; Elida Román; Hernán Pazos; Esther Vainstein; Ramiro Llona; Bill Caro; Herbert Rodríguez; EAPUC; ENBA; Hueso Húmero</t>
+          <t>Sharon Lerner (ed.); Museo de Arte de Lima (MALI); Grupo SURA; Mirko Lauer; E.P.S. Huayco; Charo Noriega; Ramiro Llona; Flavia Gandolfo; Armando Andrade Tudela; Ricardo Wiesse; Eduardo Villanes; Miguel A. López; Rodrigo Quijano</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Entrevista conducida por Gustavo Buntinx a Claudia Polar, directora de la Galería Forum, concebida como contraparte de un reportaje previo a Elida Román para perfilar el mercado del arte joven peruano. Polar reconstruye la fundación de Forum en diciembre de 1974 como un espacio destinado a priorizar a los artistas jóvenes y a gestar deliberadamente un mercado y coleccionistas nuevos, mediante becas, premios, subvenciones informales (incluso marcos y pasajes) y una política de "riesgo total" sostenida por la venta de stock. El diálogo traza una periodización económica de la plástica: expansión del mercado hacia 1974-1976, auge en 1978 atribuido a la restricción de importaciones bajo Morales Bermúdez, y recesión desde 1980 con la apertura de Belaúnde, siendo 1983 el año más difícil. Se discute la naturaleza del público comprador (gente joven, profesionales, empresarios, bancos como el de Crédito y el Continental) y la débil proporción de compradores habituales, apenas un 5% con relación económica. Buntinx presiona sobre las mediaciones de clase: el vínculo de Forum con la Universidad Católica frente a la ENBA, la identidad ideológica compartida, y el papel de las relaciones públicas como "gatillo" de casi toda venta en un mercado de "sala de estar". Polar aborda la diferencia entre lo culto y lo popular, el fracaso de asociar galerías, las cotizaciones (Llona, Caro, Pazos, Vainstein) y la explotación del artista acostumbrado a vender barato. El aporte documental es excepcional: registra desde dentro la lógica comercial, simbólica y provinciana del circuito limeño de principios de los ochenta.</t>
+          <t>Catálogo de la colección de arte contemporáneo del Museo de Arte de Lima (MALI), editado por la curadora Sharon Lerner y publicado con el patrocinio del grupo SURA. El volumen traza los derroteros del arte peruano reciente a partir del acervo del museo, sin pretender definir un 'arte peruano' esencial. La colección se articula bajo dos principios: identificar momentos de ruptura en la producción artística de fines del siglo XX y perfilar la producción reciente mediante ejes temáticos comunes. El ensayo central de Lerner establece como punto de partida mediados de la década de 1960 (grupos de vanguardia ligados al Pop y al no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, tras las reformas del Gobierno Militar, cuando —según la célebre frase de Mirko Lauer para la muestra Arte al paso del colectivo E.P.S. Huayco (1980)— 'en el Perú hoy solo lo popular es moderno'. Analiza la irrupción de la migración interna, el conflicto armado interno, el autogolpe de Fujimori (1992) y la virtual desaparición de la esfera pública, así como la Bienal Iberoamericana de Lima (1997) como puesta al día forzada y descontextualizada. El catálogo se organiza en núcleos temáticos: modernidad popular y transformación de Lima, f(r)icciones cosmopolitas, reconsideración del pasado y configuración del Perú, sistema artístico y utopías museales, desplazamientos, y signos de violencia, resistencia y memoria. Incluye obras de Charo Noriega, Ramiro Llona, Flavia Gandolfo, Armando Andrade Tudela, Herman Schwarz, Ricardo Wiesse y Eduardo Villanes, entre otros, y textos críticos complementarios. Su aporte es consolidar un relato historiográfico y crítico del arte contemporáneo peruano desde una institución museal.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Hueso Húmero 18</t>
+          <t>Cap 2 - Historia/Arte al Paso 2011</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - ¿Entre lo popular y lo moderno? Alternativas pretendidas o reales en la joven plástica peruana (1983) [Hueso Húmero 18, pp. 61-85].md</t>
+          <t>Arte al Paso - Texto Investigación.md</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>1960-1984 (con énfasis en los años 70)</t>
+          <t>Fines de los años 1960 – 2010 (con foco en las décadas de 1970-2000 y el conflicto armado interno 1980-2000)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
+          <t>Ensayo curatorial de catálogo (exposición Arte al paso, Pinacoteca do Estado de São Paulo, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Mirko Lauer; Juan Acha; Francisco Mariotti; Huayco E.P.S.; Herbert Rodríguez; Juan Javier Salazar; Jesús Ruiz Durand; Fernando de Szyszlo; IAC; Galería Forum; SINAMOS; Néstor García Canclini</t>
+          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Pinacoteca de São Paulo; Emilio Hernández Saavedra; E.P.S. Huayco; Jesús Ruiz Durand; Sandra Gamarra; Alfredo Márquez / Taller NN; Fernando Bryce; José Carlos Martinat; Susana Torres</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Ensayo teórico-histórico que propone hipótesis de trabajo sobre lo que fue o pretendió ser alternativo en el arte erudito peruano desde la transición al primer belaundismo hasta los años ochenta, articulando dos tópicos móviles: lo popular y lo moderno. Retomando y ampliando a Mirko Lauer, Buntinx sostiene que las opciones estéticas no reflejan mecánicamente la época sino que reproducen una inserción particular en el mercado, entendido como trama compleja de producción, intermediación y consumo (soporte social). Recorre así una secuencia de "soportes": el corporativo (IAC financiado por IPC, IBM, Tecnoquímica) que sostuvo la Teoría de las Raíces Nacionales de Szyszlo; el soporte "de punta" del frenesí pop cosmopolita (Acha, Arte Nuevo, Fundación para las Artes, 1966-1969); el soporte estatal velasquista con sus cuatro alternativas (comunicación masiva de Ruiz Durand con su "pop achorado", festivales de arte-total como Contacta e Inkarri, revaloración de lo artesanal, López Antay); y la frustrada búsqueda de un soporte alternativo hacia 1977-1980. El caso central es Huayco E.P.S., cuyo proyecto Sarita Colonia codifica una modernidad sincrética limeña sostenida por una pequeña burguesía ilustrada radicalizada, y cuya dispersión coincide con el agotamiento de la izquierda y el repliegue hacia el mercado galerístico (Forum). El marco conceptual bebe de García Canclini. La tesis es incisiva: el tránsito de la imagen telúrica a la industrial, agraria y migrante revela apropiaciones sucesivas de una idea variable de lo popular, siempre con una radicalidad deficiente y una relación desigual con la cultura interpretada.</t>
+          <t>Ensayo curatorial extenso y bilingüe (castellano/portugués) de Tatiana Cuevas y Rodrigo Quijano para la muestra Arte al paso, que exhibió la coleccion contemporanea del MALI en la Estacion Pinacoteca de Sao Paulo. El texto toma como punto de partida la imagen El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra para diagnosticar los vacios institucionales y la distancia entre el discurso cultural cosmopolita y la practica real en el Peru de la segunda mitad del siglo XX. Su argumento articula el arte contemporaneo peruano con las transformaciones sociales derivadas de la masiva migracion rural a Lima, la explosion de la economia informal y la emergencia de una nueva cultura popular urbana. Rastrea las primeras vinculaciones locales con vanguardias internacionales (op, pop, conceptualismo, no-objetualismo), el pop achorado de Jesus Ruiz Durand y sus afiches de la Reforma Agraria velasquista, y las experiencias colectivas Contacta 79 y Arte al paso de E.P.S. Huayco (1980), que propusieron un arte callejero y antiinstitucional. Analiza la critica a la institucionalidad faltante (el museo ficticio LiMAC de Sandra Gamarra), el uso ironico del pasado prehispanico (Susana Torres, Rodriguez Larrain, Bryce, Cordova, Martinat), el tema del paisaje y el territorio, y la irrupcion tardia de la fotografia y la serigrafia como medios. Dedica una seccion central a la memoria de la violencia del conflicto armado interno (1980-2000) —Sendero Luminoso, MRTA, la Comision de la Verdad, 69.280 muertos— y su tratamiento por el Taller NN, Alfredo Marquez (Katatay), Carlos Dominguez, Ricardo Wiesse, Eduardo Villanes, Fernando Bryce y Milagros de la Torre.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Hueso Húmero 18</t>
+          <t>Cap 2 - Historia/Arte al Paso 2011</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Freire - Herbert Rodríguez, azote y azúcar con el sistema (1983) [Hueso Húmero 18, pdf pp. 178-185].md</t>
+          <t>Cronología Político Artistica - Arte al Paso 2011.md</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>1979-1983 (con antecedentes desde 1968)</t>
+          <t>1962 – 2010</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Reseña crítica en revista (Hueso Húmero 18), 1983</t>
+          <t>Cronología y bibliografía de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Luis Freire S.; Herbert Rodríguez; Francisco Mariotti; Huayco E.P.S.; Juan Acha; Fernando Bedoya; Juan Javier Salazar; Bienal de Sao Paulo; Galería La Rama Dorada; Galería Forum; EAPUC; ENBAP</t>
+          <t>Museo de Arte de Lima (MALI); Grupo Arte Nuevo; Grupo Señal; E.P.S. Huayco; Taller NN; Colectivo Sociedad Civil; Gustavo Buntinx; Joaquín López Antay; Comisión de la Verdad y Reconciliación; Sendero Luminoso; Alberto Fujimori; Juan Velasco Alvarado</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Perfil crítico dedicado a Herbert Rodríguez Huachín en la sección "Individuales" de Hueso Húmero, escrito por Luis Freire, que examina el salto vertiginoso del artista desde la suspensión disciplinaria en la Escuela de Artes Plásticas de la Católica (1981) hasta su presencia en la XVII Bienal de Sao Paulo (1983). Freire sitúa a Rodríguez como imposible de explicar sin el proceso ideológico del populismo velasquista y sin la figura mediadora de Francisco Mariotti, artista suizo-peruano formado en la Documenta de Kassel y la vanguardia europea, catalizador de Contacta y de la EPS Huayco. El texto reconstruye la genealogía Mariotti-Huayco-Rodríguez: los ensamblajes y "reciclajes" del suizo-peruano derivan en los "altares" de Rodríguez, hibridación entre constructivismo geométrico, expresionismo "pobre" y antiestético, y estructuras rituales de la religiosidad popular andina. Argumenta que Rodríguez encarna las contradicciones de una pequeña burguesía radical: dinamita el circuito con una mano y lo enluce con la otra, camuflando "bellamente" materiales pobres y reciclados en obras a la vez contestatarias y comerciables, con lo que ironiza sobre el culto al oficio del arte establecido. Analiza su heterogeneidad de lenguajes (expresionismo abstracto, figuración dura, conceptualismo informal, collage, fotocopia, ensamblaje) como búsqueda pero también como crisis, y sus "altares al Yo" exhibidos en Forum (1983) y la Bienal. Freire lo define como un artista religioso-existencial populista sin referentes sólidos, en formación, tensionado entre enriquecer el jardín burgués que quiere pisotear o saltar a opciones más radicales de ruptura.</t>
+          <t>Cronologia politico-artistica bilingue (castellano/portugues) incluida en el catalogo Arte al paso, que entrelaza en paralelo tres series de acontecimientos —eventos politicos, eventos artisticos y adquisiciones de la coleccion de arte contemporaneo del MALI— entre 1962 y 2010. El documento funciona como aparato historiografico que contextualiza la escena artistica peruana dentro de sus convulsiones politicas: rebeliones campesinas y golpes militares de los anos sesenta, el Gobierno Revolucionario de las Fuerzas Armadas de Velasco Alvarado (1968) y la Reforma Agraria, el estallido del conflicto armado interno con Sendero Luminoso y el MRTA (1980), las masacres de Barrios Altos y La Cantuta, el autogolpe y la dictadura de Alberto Fujimori (1990-2000), la Marcha de los Cuatro Suyos y el Informe de la Comision de la Verdad y Reconciliacion (2003). En el plano artistico registra la formacion de los grupos Senal y Arte Nuevo, las Bienales de Lima e Iberoamericanas, los festivales Contacta e Inkarri, el Taller E.P.S. Huayco y el Taller NN, la premiacion de Joaquin Lopez Antay, y acciones de arte critico como Cantuta de Ricardo Wiesse, Gloria evaporada de Eduardo Villanes y Lava la bandera del Colectivo Sociedad Civil. Una tercera linea traza la institucionalizacion del MALI: el ciclo curatorial Miradas de fin de siglo, la creacion del Comite de Adquisiciones (2007) y la reapertura del museo (2010). Se acompana de una extensa bibliografia especializada (Buntinx, Castrillon, Lauer, Majluf, Lopez, Tarazona, Quijano, Villacorta), fuente clave para la historiografia del arte peruano contemporaneo.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Hueso Húmero 18</t>
+          <t>Cap 2 - Historia/Arte al Paso 2011</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Lama - Los años de la resaca (1983) [Hueso Húmero 18, pdf pp. 136-156].md</t>
+          <t>Texto de la exposición Arte al Paso 2011.md</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>1974-1983 (con antecedentes en los años 60-70)</t>
+          <t>Fines de los años 1960 – 2010 (unos 40 años; foco en las décadas de 1970-1980)</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
+          <t>Texto de sala / presentación de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Luis Lama; Hernán Pazos; Francisco Mariotti; Contacta; grupo Huayco; Juan Javier Salazar; Herbert Rodríguez; Alfonso Castrillón; Escuela Nacional de Bellas Artes; Galería Forum; Galería 9; Ugarte Eléspuru</t>
+          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Emilio Hernández Saavedra; E.P.S. Huayco; Grupo Paréntesis; Sandra Gamarra; Susana Torres; Emilio Rodríguez Larraín; Juan Javier Salazar; William Cordova; José Carlos Martinat</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Ensayo de Luis Lama que narra el paso de la "ebullición ideológica" de los años setenta a la "resaca" del segundo belaundismo, articulando historia social del arte y crítica biográfica. La primera parte reconstruye los antecedentes: el terremoto de 1974 y el reflujo de artistas jóvenes hacia Barranco, la gravitación de Francisco Mariotti que transforma el arte de sistemas en movimiento grupal con Contacta e Inkari bajo auspicio de SINAMOS, las tomas y la crisis de la Escuela Nacional de Bellas Artes (1974-1976), y la gestación del taller de Pedro de Osma que devendría núcleo del grupo Huayco (Juan Javier Salazar, Herbert Rodríguez, Charo Noriega, Fernando Bedoya, Lucy Angulo). Lama describe la consolidación paradójica del mercado del arte al amparo de la prohibición de importaciones, con galerías que proliferan mientras la formación académica alcanza sus niveles más bajos. Diagnostica el fin de los happenings sesenteros y el retorno de un expresionismo "de crisis" impulsado desde los predios católicos (Williams, Polanco, Velarde, Hamann), junto a indagaciones matéricas de Wiesse y el conceptualismo de Vainstein. La segunda mitad es un retrato extenso de Hernán Pazos: su formación entre Derecho, la Católica y París, su tránsito del conceptualismo (los cielos y nubes de Galería 9) a la abstracción cromática, las series de los Quipus y los dibujos infantiles, su gestión en Rama Dorada y su individualismo parricida. Lama lo consagra como el artista más destacado de la década, emblema lúcido de las "amargas frustraciones" nacionales bajo el liberalismo económico belaundista.</t>
+          <t>Texto de sala o presentacion general de la exposicion Arte al paso (coleccion contemporanea del MALI en la Pinacoteca de Sao Paulo), firmado por los curadores Tatiana Cuevas y Rodrigo Quijano, en edicion bilingue castellano/portugues. Es una version sintetica del argumento curatorial: parte nuevamente de El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra como metafora de la ausencia institucional y punto de arranque para examinar la escena artistica peruana desde fines de los anos sesenta. Explica el titulo de la muestra a partir de la accion Arte al paso de E.P.S. Huayco (1980) —que, aludiendo a los puestos informales de comida al paso surgidos con la migracion y la economia informal, propuso un arte para consumirse en la calle, opuesto al museo y la galeria ausentes, un arte para pensar y no para sentir que dejaba atras el modernismo conservador de mediados de siglo. Sintetiza cuarenta anos de produccion cultural marcados por oposiciones ocultas y explicitas, los primeros acercamientos al conceptualismo y a las vanguardias internacionales, y la creciente proyeccion internacional de artistas peruanos. Una segunda seccion, Critica ante una institucionalidad faltante y al poder redentor del pasado, reune a Hernandez Saavedra, los grupos Parentesis y E.P.S. Huayco y el museo ficticio de Sandra Gamarra como estrategias de critica institucional apropiadas del conceptualismo y del imaginario popular urbano, con recurrente uso del humor. Aborda ademas la critica a la explotacion comercial y politica de lo prehispanico (Museo Neo-Inka de Susana Torres) y el vinculo entre la retorica del glorioso pasado incaico y los fracasos politicos y economicos del presente en obras de Rodriguez Larrain, Salazar, Cordova y Martinat.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/MALI</t>
+          <t>Cap 2 - Historia/Hueso Húmero 18</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - El poder y la ilusión. Pérdida y restauración del aura en la «República de Weimar peruana» 1980-1992 [MALI].md</t>
+          <t>Buntinx - Arte joven peruano, ¿el sueño del mercado propio? Una conversación con Claudia Polar (1983) [Hueso Húmero 18, pp. 94-107].md</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>1980-1992</t>
+          <t>1974-1983</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico (versión MALI), 2013 [escrito 1991-1994]</t>
+          <t>Entrevista en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; E.P.S. Huayco; Taller NN; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; Walter Benjamin; Jesús Ruiz Durand; Andy Warhol; Mirko Lauer; Museo de Arte de Lima (MALI); III Bienal de La Habana</t>
+          <t>Gustavo Buntinx; Claudia Polar; Galería Forum; Elida Román; Hernán Pazos; Esther Vainstein; Ramiro Llona; Bill Caro; Herbert Rodríguez; EAPUC; ENBA; Hueso Húmero</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>Ensayo seminal de Gustavo Buntinx —redactado entre 1991 y 1994, difundido en inglés en «Beyond the Fantastic» (1995) y publicado por primera vez en Perú en esta versión del MALI (2013)— que interpreta el radical cambio de época del arte peruano entre 1980 y 1992, periodo que denomina metafóricamente «República de Weimar peruana». Su marco conceptual adapta la dialéctica benjaminiana entre proximidad y distancia (el aura, su pérdida por la reproductibilidad técnica y su posible restauración) y las categorías de alegoría, montaje y apropiación de Owens, Foster y Craig Owens a una periferia extrema. El argumento se sostiene sobre el análisis iconográfico minucioso de dos o tres obras que abren y cierran la década. La primera, «Arte al paso» y sobre todo «Sarita Colonia» (1980) del taller E.P.S. Huayco: una enorme estampa de la santa migrante pintada sobre diez mil latas de leche y emplazada en la Panamericana Sur, que Buntinx lee como huaca (post)moderna y exvoto donde lo pequeñoburgués radical se articula figuradamente a lo popular en emergencia (el «pop achorado» y «chicha»). La segunda, «Maorilyn» / «Viva el maoísmo» (1989) del Taller NN: una serigrafía que travistió el rostro de Mao con labios warholianos, alegoría ambivalente de la violencia senderista y la estetización de la política. Su tesis vincula la desintegración social —hiperinflación, guerra civil, movida subte punk— con el desarrollo de una condición alegórica y neo-aurática; su aporte es un modelo teórico para leer el colectivismo y la (post)modernidad popular peruana.</t>
+          <t>Entrevista conducida por Gustavo Buntinx a Claudia Polar, directora de la Galería Forum, concebida como contraparte de un reportaje previo a Elida Román para perfilar el mercado del arte joven peruano. Polar reconstruye la fundación de Forum en diciembre de 1974 como un espacio destinado a priorizar a los artistas jóvenes y a gestar deliberadamente un mercado y coleccionistas nuevos, mediante becas, premios, subvenciones informales (incluso marcos y pasajes) y una política de "riesgo total" sostenida por la venta de stock. El diálogo traza una periodización económica de la plástica: expansión del mercado hacia 1974-1976, auge en 1978 atribuido a la restricción de importaciones bajo Morales Bermúdez, y recesión desde 1980 con la apertura de Belaúnde, siendo 1983 el año más difícil. Se discute la naturaleza del público comprador (gente joven, profesionales, empresarios, bancos como el de Crédito y el Continental) y la débil proporción de compradores habituales, apenas un 5% con relación económica. Buntinx presiona sobre las mediaciones de clase: el vínculo de Forum con la Universidad Católica frente a la ENBA, la identidad ideológica compartida, y el papel de las relaciones públicas como "gatillo" de casi toda venta en un mercado de "sala de estar". Polar aborda la diferencia entre lo culto y lo popular, el fracaso de asociar galerías, las cotizaciones (Llona, Caro, Pazos, Vainstein) y la explotación del artista acostumbrado a vender barato. El aporte documental es excepcional: registra desde dentro la lógica comercial, simbólica y provinciana del circuito limeño de principios de los ochenta.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/MALI</t>
+          <t>Cap 2 - Historia/Hueso Húmero 18</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Lerner - Formando la colección de arte contemporáneo del MALI (2013).txt</t>
+          <t>Buntinx - ¿Entre lo popular y lo moderno? Alternativas pretendidas o reales en la joven plástica peruana (1983) [Hueso Húmero 18, pp. 61-85].md</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>mediados de los años 60 - 2013 (con foco en 1980-2000)</t>
+          <t>1960-1984 (con énfasis en los años 70)</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo de colección, 2013</t>
+          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Museo de Arte de Lima (MALI); Tatiana Cuevas; Miguel A. López; Gustavo Buntinx; Rodrigo Quijano; Jorge Villacorta; Natalia Majluf; E.P.S. Huayco; Teresa Burga; Milagros de la Torre; Flavia Gandolfo</t>
+          <t>Gustavo Buntinx; Mirko Lauer; Juan Acha; Francisco Mariotti; Huayco E.P.S.; Herbert Rodríguez; Juan Javier Salazar; Jesús Ruiz Durand; Fernando de Szyszlo; IAC; Galería Forum; SINAMOS; Néstor García Canclini</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Ensayo introductorio de Sharon Lerner al libro que presenta la colección de arte contemporáneo del Museo de Arte de Lima (MALI), articulado como una lectura —entre muchas posibles— de la historia del arte reciente peruano a partir del acervo. Su tesis metodológica es que en el Perú el tránsito a la contemporaneidad no ocurre como un quiebre radical, sino como una serie de pequeños cambios discontinuos, por lo que la colección se organiza en dos principios: identificar momentos de ruptura de fines del siglo XX y perfilar la producción reciente por ejes temáticos. El recorrido histórico parte de mediados de los sesenta (vanguardias pop, experimentalismo, no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, cuando la migración y la sentencia de Mirko Lauer —«En el Perú, hoy, solo lo popular es moderno»— enmarcan la obra de E.P.S. Huayco. Recorre luego la hegemonía de la abstracción en los ochenta, el arte de derechos humanos de Ricardo Wiesse y Eduardo Villanes bajo el fujimorato, la irrupción de la Bienal Iberoamericana de Lima (1997) y el «bienalismo», y la generación de los 2000 (Flavia Gandolfo, Gilda Mantilla, Armando Andrade Tudela) vinculada al espacio La Culpable. El texto presenta además los ensayos de Miguel López, Gustavo Buntinx y Rodrigo Quijano incluidos en el volumen y la conversación de seis críticos (2011). Su aporte es explicitar la política de adquisiciones del MALI y su ambición de llenar el vacío institucional y discursivo, construyendo un marco regional e internacional para el arte peruano.</t>
+          <t>Ensayo teórico-histórico que propone hipótesis de trabajo sobre lo que fue o pretendió ser alternativo en el arte erudito peruano desde la transición al primer belaundismo hasta los años ochenta, articulando dos tópicos móviles: lo popular y lo moderno. Retomando y ampliando a Mirko Lauer, Buntinx sostiene que las opciones estéticas no reflejan mecánicamente la época sino que reproducen una inserción particular en el mercado, entendido como trama compleja de producción, intermediación y consumo (soporte social). Recorre así una secuencia de "soportes": el corporativo (IAC financiado por IPC, IBM, Tecnoquímica) que sostuvo la Teoría de las Raíces Nacionales de Szyszlo; el soporte "de punta" del frenesí pop cosmopolita (Acha, Arte Nuevo, Fundación para las Artes, 1966-1969); el soporte estatal velasquista con sus cuatro alternativas (comunicación masiva de Ruiz Durand con su "pop achorado", festivales de arte-total como Contacta e Inkarri, revaloración de lo artesanal, López Antay); y la frustrada búsqueda de un soporte alternativo hacia 1977-1980. El caso central es Huayco E.P.S., cuyo proyecto Sarita Colonia codifica una modernidad sincrética limeña sostenida por una pequeña burguesía ilustrada radicalizada, y cuya dispersión coincide con el agotamiento de la izquierda y el repliegue hacia el mercado galerístico (Forum). El marco conceptual bebe de García Canclini. La tesis es incisiva: el tránsito de la imagen telúrica a la industrial, agraria y migrante revela apropiaciones sucesivas de una idea variable de lo popular, siempre con una radicalidad deficiente y una relación desigual con la cultura interpretada.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/MALI</t>
+          <t>Cap 2 - Historia/Hueso Húmero 18</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - F(r)icciones cosmopolitas. Redefiniciones estéticas y políticas de una idea de vanguardia en los años 60s.txt</t>
+          <t>Freire - Herbert Rodríguez, azote y azúcar con el sistema (1983) [Hueso Húmero 18, pdf pp. 178-185].md</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>1960-1976 (con antecedentes desde 1942-1947)</t>
+          <t>1979-1983 (con antecedentes desde 1968)</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico / capítulo de catálogo (MALI), s/f</t>
+          <t>Reseña crítica en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Emilio Tarazona; Juan Acha; Fernando de Szyszlo; Jorge Romero Brest; Teresa Burga; Rafael Hastings; Grupo Arte Nuevo; Jesús Ruiz Durand; José Gómez Sicre; Marta Traba; Instituto de Arte Contemporáneo (IAC); MoMA / Instituto Di Tella</t>
+          <t>Luis Freire S.; Herbert Rodríguez; Francisco Mariotti; Huayco E.P.S.; Juan Acha; Fernando Bedoya; Juan Javier Salazar; Bienal de Sao Paulo; Galería La Rama Dorada; Galería Forum; EAPUC; ENBAP</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>López reconstruye las mutaciones semánticas y políticas de la noción de vanguardia en el Perú entre los años sesenta y setenta, argumentando que la euforia cosmopolita del periodo fue el espejismo de una modernidad desarrollista tan prometedora como inacabada en un país socialmente fracturado. El objeto de estudio son las plataformas institucionales privadas (IAC, galerías, bienales americanas, concursos empresariales) que, apuntaladas por el panamericanismo de la Guerra Fría, la Alianza para el Progreso y la política curatorial estadounidense de José Gómez Sicre, promovieron primero la abstracción y luego el arte óptico, el pop y las ambientaciones. El texto traza el paso del declive de la abstracción szyszliana hacia el experimentalismo detonado por las conferencias de Jorge Romero Brest (1965) y la irrupción beligerante del grupo Arte Nuevo (1966-1968) contra el Festival Americano de Pintura. El marco conceptual articula la relación entre desarrollismo y vanguardia, y su posterior tensión con el subdesarrollo, siguiendo la radicalización de Juan Acha, quien tras 1968 y el golpe de Velasco redefine la vanguardia como 'guerrilla cultural' y horizonte revolucionario, hasta su exilio a México en 1971. López destaca las reconversiones de Teresa Burga y Rafael Hastings, el 'pop achorado' de Ruiz Durand al servicio de la Reforma Agraria, los festivales Contacta y las Carreras de chasquis. Su aporte es mostrar cómo la condición local, provinciana y periférica de las prácticas de los setenta y ochenta (Paréntesis, E.P.S. Huayco, Grupo Chaclacayo) actualizó de modo radical las pretensiones críticas sesenteras, canibalizando los conceptos metropolitanos de arte conceptual.</t>
+          <t>Perfil crítico dedicado a Herbert Rodríguez Huachín en la sección "Individuales" de Hueso Húmero, escrito por Luis Freire, que examina el salto vertiginoso del artista desde la suspensión disciplinaria en la Escuela de Artes Plásticas de la Católica (1981) hasta su presencia en la XVII Bienal de Sao Paulo (1983). Freire sitúa a Rodríguez como imposible de explicar sin el proceso ideológico del populismo velasquista y sin la figura mediadora de Francisco Mariotti, artista suizo-peruano formado en la Documenta de Kassel y la vanguardia europea, catalizador de Contacta y de la EPS Huayco. El texto reconstruye la genealogía Mariotti-Huayco-Rodríguez: los ensamblajes y "reciclajes" del suizo-peruano derivan en los "altares" de Rodríguez, hibridación entre constructivismo geométrico, expresionismo "pobre" y antiestético, y estructuras rituales de la religiosidad popular andina. Argumenta que Rodríguez encarna las contradicciones de una pequeña burguesía radical: dinamita el circuito con una mano y lo enluce con la otra, camuflando "bellamente" materiales pobres y reciclados en obras a la vez contestatarias y comerciables, con lo que ironiza sobre el culto al oficio del arte establecido. Analiza su heterogeneidad de lenguajes (expresionismo abstracto, figuración dura, conceptualismo informal, collage, fotocopia, ensamblaje) como búsqueda pero también como crisis, y sus "altares al Yo" exhibidos en Forum (1983) y la Bienal. Freire lo define como un artista religioso-existencial populista sin referentes sólidos, en formación, tensionado entre enriquecer el jardín burgués que quiere pisotear o saltar a opciones más radicales de ruptura.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/MALI</t>
+          <t>Cap 2 - Historia/Hueso Húmero 18</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Quijano - Notas incompletas sobre el sitio de la fotografía peruana.md</t>
+          <t>Lama - Los años de la resaca (1983) [Hueso Húmero 18, pdf pp. 136-156].md</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>1900-2011 (con énfasis en 1920-1998)</t>
+          <t>1974-1983 (con antecedentes en los años 60-70)</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo (MALI), s/f</t>
+          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Quijano; Martín Chambi; José María Eguren; Carlos 'Chino' Domínguez; Aaron Siskind; Jesús Ruiz Durand; Claudia Martínez Garay; Daniela Ortiz; Foto Galería Secuencia; TAFOS; Taller NN; E.P.S. Huayco</t>
+          <t>Luis Lama; Hernán Pazos; Francisco Mariotti; Contacta; grupo Huayco; Juan Javier Salazar; Herbert Rodríguez; Alfonso Castrillón; Escuela Nacional de Bellas Artes; Galería Forum; Galería 9; Ugarte Eléspuru</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Quijano ensaya una genealogía del 'sitio' de la fotografía peruana, sosteniendo que este medio inauguró un margen de creación moderno al margen de la institucionalidad académica de las bellas artes, alcanzando una temprana ubicuidad territorial y una masividad que condicionó la percepción misma de una realidad nacional. El texto, de estructura fragmentaria y numerada, contrapone dos matrices fundacionales: Martín Chambi como 'modernista sin modernidad' y profesional de la imagen surgido de una familia campesina andina —una 'oportunidad nacional'— frente a la miniatura pinhole intimista y hermética de José María Eguren, que prefigura la figura del fotógrafo-artista individual. Analiza a Carlos 'Chino' Domínguez como ojo testimonial de la urbanización y la nueva cultura popular (La resaca del Inca, el 'Cholo' Sotil, el filme Cholo y su reedición Mi cholo de Gruenberg), y la experiencia de la fotogalería Secuencia (1977-1980), que reinventó una tradición y un discurso del oficio adoptando a Minor White y Aaron Siskind. El marco conceptual enlaza fotografía, prensa y democratización de la imagen en el contexto del auge sindical y la repolitización popular de fines de los setenta, y la aparición de la fotoserigrafía disidente (Bedoya, Williams, Mariotti, Salazar) como catalizador de una nueva condición fotográfica colectiva, desde E.P.S. Huayco hasta el Taller NN. El aporte del texto es leer la fotografía como dispositivo de documento, archivo, memoria y duelo frente a la violencia política (Uchuraccay, Yuyanapaq), rastreando su 'grado cero' icónico en obras de Ruiz Durand, Claudia Martínez Garay y Daniela Ortiz, que develan la mirada colonial y la invisibilización étnica.</t>
+          <t>Ensayo de Luis Lama que narra el paso de la "ebullición ideológica" de los años setenta a la "resaca" del segundo belaundismo, articulando historia social del arte y crítica biográfica. La primera parte reconstruye los antecedentes: el terremoto de 1974 y el reflujo de artistas jóvenes hacia Barranco, la gravitación de Francisco Mariotti que transforma el arte de sistemas en movimiento grupal con Contacta e Inkari bajo auspicio de SINAMOS, las tomas y la crisis de la Escuela Nacional de Bellas Artes (1974-1976), y la gestación del taller de Pedro de Osma que devendría núcleo del grupo Huayco (Juan Javier Salazar, Herbert Rodríguez, Charo Noriega, Fernando Bedoya, Lucy Angulo). Lama describe la consolidación paradójica del mercado del arte al amparo de la prohibición de importaciones, con galerías que proliferan mientras la formación académica alcanza sus niveles más bajos. Diagnostica el fin de los happenings sesenteros y el retorno de un expresionismo "de crisis" impulsado desde los predios católicos (Williams, Polanco, Velarde, Hamann), junto a indagaciones matéricas de Wiesse y el conceptualismo de Vainstein. La segunda mitad es un retrato extenso de Hernán Pazos: su formación entre Derecho, la Católica y París, su tránsito del conceptualismo (los cielos y nubes de Galería 9) a la abstracción cromática, las series de los Quipus y los dibujos infantiles, su gestión en Rama Dorada y su individualismo parricida. Lama lo consagra como el artista más destacado de la década, emblema lúcido de las "amargas frustraciones" nacionales bajo el liberalismo económico belaundista.</t>
         </is>
       </c>
     </row>
@@ -2910,32 +2910,160 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
+          <t>Buntinx - El poder y la ilusión. Pérdida y restauración del aura en la «República de Weimar peruana» 1980-1992 [MALI].md</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>1980-1992</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Ensayo académico (versión MALI), 2013 [escrito 1991-1994]</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>Gustavo Buntinx; E.P.S. Huayco; Taller NN; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; Walter Benjamin; Jesús Ruiz Durand; Andy Warhol; Mirko Lauer; Museo de Arte de Lima (MALI); III Bienal de La Habana</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>Ensayo seminal de Gustavo Buntinx —redactado entre 1991 y 1994, difundido en inglés en «Beyond the Fantastic» (1995) y publicado por primera vez en Perú en esta versión del MALI (2013)— que interpreta el radical cambio de época del arte peruano entre 1980 y 1992, periodo que denomina metafóricamente «República de Weimar peruana». Su marco conceptual adapta la dialéctica benjaminiana entre proximidad y distancia (el aura, su pérdida por la reproductibilidad técnica y su posible restauración) y las categorías de alegoría, montaje y apropiación de Owens, Foster y Craig Owens a una periferia extrema. El argumento se sostiene sobre el análisis iconográfico minucioso de dos o tres obras que abren y cierran la década. La primera, «Arte al paso» y sobre todo «Sarita Colonia» (1980) del taller E.P.S. Huayco: una enorme estampa de la santa migrante pintada sobre diez mil latas de leche y emplazada en la Panamericana Sur, que Buntinx lee como huaca (post)moderna y exvoto donde lo pequeñoburgués radical se articula figuradamente a lo popular en emergencia (el «pop achorado» y «chicha»). La segunda, «Maorilyn» / «Viva el maoísmo» (1989) del Taller NN: una serigrafía que travistió el rostro de Mao con labios warholianos, alegoría ambivalente de la violencia senderista y la estetización de la política. Su tesis vincula la desintegración social —hiperinflación, guerra civil, movida subte punk— con el desarrollo de una condición alegórica y neo-aurática; su aporte es un modelo teórico para leer el colectivismo y la (post)modernidad popular peruana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Cap 2 - Historia/MALI</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Lerner - Formando la colección de arte contemporáneo del MALI (2013).txt</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>mediados de los años 60 - 2013 (con foco en 1980-2000)</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Ensayo de catálogo de colección, 2013</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>Sharon Lerner; Museo de Arte de Lima (MALI); Tatiana Cuevas; Miguel A. López; Gustavo Buntinx; Rodrigo Quijano; Jorge Villacorta; Natalia Majluf; E.P.S. Huayco; Teresa Burga; Milagros de la Torre; Flavia Gandolfo</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>Ensayo introductorio de Sharon Lerner al libro que presenta la colección de arte contemporáneo del Museo de Arte de Lima (MALI), articulado como una lectura —entre muchas posibles— de la historia del arte reciente peruano a partir del acervo. Su tesis metodológica es que en el Perú el tránsito a la contemporaneidad no ocurre como un quiebre radical, sino como una serie de pequeños cambios discontinuos, por lo que la colección se organiza en dos principios: identificar momentos de ruptura de fines del siglo XX y perfilar la producción reciente por ejes temáticos. El recorrido histórico parte de mediados de los sesenta (vanguardias pop, experimentalismo, no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, cuando la migración y la sentencia de Mirko Lauer —«En el Perú, hoy, solo lo popular es moderno»— enmarcan la obra de E.P.S. Huayco. Recorre luego la hegemonía de la abstracción en los ochenta, el arte de derechos humanos de Ricardo Wiesse y Eduardo Villanes bajo el fujimorato, la irrupción de la Bienal Iberoamericana de Lima (1997) y el «bienalismo», y la generación de los 2000 (Flavia Gandolfo, Gilda Mantilla, Armando Andrade Tudela) vinculada al espacio La Culpable. El texto presenta además los ensayos de Miguel López, Gustavo Buntinx y Rodrigo Quijano incluidos en el volumen y la conversación de seis críticos (2011). Su aporte es explicitar la política de adquisiciones del MALI y su ambición de llenar el vacío institucional y discursivo, construyendo un marco regional e internacional para el arte peruano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Cap 2 - Historia/MALI</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>López, Miguel A. - F(r)icciones cosmopolitas. Redefiniciones estéticas y políticas de una idea de vanguardia en los años 60s.txt</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>1960-1976 (con antecedentes desde 1942-1947)</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Ensayo académico / capítulo de catálogo (MALI), s/f</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Miguel A. López; Emilio Tarazona; Juan Acha; Fernando de Szyszlo; Jorge Romero Brest; Teresa Burga; Rafael Hastings; Grupo Arte Nuevo; Jesús Ruiz Durand; José Gómez Sicre; Marta Traba; Instituto de Arte Contemporáneo (IAC); MoMA / Instituto Di Tella</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>López reconstruye las mutaciones semánticas y políticas de la noción de vanguardia en el Perú entre los años sesenta y setenta, argumentando que la euforia cosmopolita del periodo fue el espejismo de una modernidad desarrollista tan prometedora como inacabada en un país socialmente fracturado. El objeto de estudio son las plataformas institucionales privadas (IAC, galerías, bienales americanas, concursos empresariales) que, apuntaladas por el panamericanismo de la Guerra Fría, la Alianza para el Progreso y la política curatorial estadounidense de José Gómez Sicre, promovieron primero la abstracción y luego el arte óptico, el pop y las ambientaciones. El texto traza el paso del declive de la abstracción szyszliana hacia el experimentalismo detonado por las conferencias de Jorge Romero Brest (1965) y la irrupción beligerante del grupo Arte Nuevo (1966-1968) contra el Festival Americano de Pintura. El marco conceptual articula la relación entre desarrollismo y vanguardia, y su posterior tensión con el subdesarrollo, siguiendo la radicalización de Juan Acha, quien tras 1968 y el golpe de Velasco redefine la vanguardia como 'guerrilla cultural' y horizonte revolucionario, hasta su exilio a México en 1971. López destaca las reconversiones de Teresa Burga y Rafael Hastings, el 'pop achorado' de Ruiz Durand al servicio de la Reforma Agraria, los festivales Contacta y las Carreras de chasquis. Su aporte es mostrar cómo la condición local, provinciana y periférica de las prácticas de los setenta y ochenta (Paréntesis, E.P.S. Huayco, Grupo Chaclacayo) actualizó de modo radical las pretensiones críticas sesenteras, canibalizando los conceptos metropolitanos de arte conceptual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Cap 2 - Historia/MALI</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Quijano - Notas incompletas sobre el sitio de la fotografía peruana.md</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>1900-2011 (con énfasis en 1920-1998)</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Ensayo de catálogo (MALI), s/f</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Rodrigo Quijano; Martín Chambi; José María Eguren; Carlos 'Chino' Domínguez; Aaron Siskind; Jesús Ruiz Durand; Claudia Martínez Garay; Daniela Ortiz; Foto Galería Secuencia; TAFOS; Taller NN; E.P.S. Huayco</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>Quijano ensaya una genealogía del 'sitio' de la fotografía peruana, sosteniendo que este medio inauguró un margen de creación moderno al margen de la institucionalidad académica de las bellas artes, alcanzando una temprana ubicuidad territorial y una masividad que condicionó la percepción misma de una realidad nacional. El texto, de estructura fragmentaria y numerada, contrapone dos matrices fundacionales: Martín Chambi como 'modernista sin modernidad' y profesional de la imagen surgido de una familia campesina andina —una 'oportunidad nacional'— frente a la miniatura pinhole intimista y hermética de José María Eguren, que prefigura la figura del fotógrafo-artista individual. Analiza a Carlos 'Chino' Domínguez como ojo testimonial de la urbanización y la nueva cultura popular (La resaca del Inca, el 'Cholo' Sotil, el filme Cholo y su reedición Mi cholo de Gruenberg), y la experiencia de la fotogalería Secuencia (1977-1980), que reinventó una tradición y un discurso del oficio adoptando a Minor White y Aaron Siskind. El marco conceptual enlaza fotografía, prensa y democratización de la imagen en el contexto del auge sindical y la repolitización popular de fines de los setenta, y la aparición de la fotoserigrafía disidente (Bedoya, Williams, Mariotti, Salazar) como catalizador de una nueva condición fotográfica colectiva, desde E.P.S. Huayco hasta el Taller NN. El aporte del texto es leer la fotografía como dispositivo de documento, archivo, memoria y duelo frente a la violencia política (Uchuraccay, Yuyanapaq), rastreando su 'grado cero' icónico en obras de Ruiz Durand, Claudia Martínez Garay y Daniela Ortiz, que develan la mirada colonial y la invisibilización étnica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Cap 2 - Historia/MALI</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
           <t>Villacorta (ed.) - ¿Un arte visual a contrapelo de los dictados metropolitanos? En el Perú, el arte moderno es un gesto tardío [conversación en el MALI, 2011].txt</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C81" s="2" t="inlineStr">
         <is>
           <t>1947-2011 (con eje en 1960-2002)</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D81" s="2" t="inlineStr">
         <is>
           <t>Transcripción editada de conversación (MALI), 2011</t>
         </is>
       </c>
-      <c r="E77" s="3" t="inlineStr">
+      <c r="E81" s="3" t="inlineStr">
         <is>
           <t>Jorge Villacorta; Gustavo Buntinx; Miguel A. López; Rodrigo Quijano; Tatiana Cuevas; Natalia Majluf; E.P.S. Huayco; Grupo Arte Nuevo; Taller NN; Grupo Chaclacayo; Christian Bendayán; Fernando Bryce; MALI / Micromuseo</t>
         </is>
       </c>
-      <c r="F77" s="3" t="inlineStr">
+      <c r="F81" s="3" t="inlineStr">
         <is>
           <t>Editada por Villacorta a partir de dos sesiones de 2011 en el MALI, esta conversación a seis voces indaga si lo moderno está clausurado en el arte peruano de modo que permita definir lo contemporáneo. La tesis articuladora, propuesta por Quijano, es que en el Perú lo moderno solo ha podido darse 'a contrapelo' y como 'gesto tardío', a destiempo de las modernidades metropolitanas; López y Buntinx la matizan con la idea de temporalidades dislocadas y friccionadas que impiden toda historia lineal. El objeto de estudio es la genealogía de la vanguardia local: la contraposición entre Arte Nuevo (1966-1968), leído como destello cosmopolita fugaz, y E.P.S. Huayco y Paréntesis, cuya apropiación de Sarita Colonia y el 'pop achorado' marca una ruptura más perdurable y pertinente al medio. Buntinx despliega una secuencia estilístico-conceptual en clave pop/místico-libidinal —de la Twiggy de Emilio Hernández a Quistococha de Bendayán, pasando por el afiche de Ruiz Durand, la Maoirilyn del Taller NN y La Pachakuti de Alfredo Márquez— ligada a periodos políticos (desarrollismo, velasquismo, utopía socialista, dictadura fujimorista, revolución capitalista). Majluf sitúa el quiebre epocal de fin de siglo en el ingreso de la 'referencia' fotográfica (Bryce, Milagros de la Torre, Juan Enrique Bedoya, Mantilla), frente al neobarroco. El texto discute además la construcción de públicos, la institucionalidad faltante, el rol del curador, el mercado 'social' peruano, las subastas del MALI y la 'normalización de la diferencia' como riesgo de la consagración institucional del pasado radical.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F77"/>
+  <autoFilter ref="A1:F81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Cataloga archivo de exposiciones del MALL (mali_exposiciones_2026-07-18) en Cap 2 - Historia
- Añade una fila a tabla-cap2-historia.csv (80 -> 81) para la recopilación de 64 exposiciones del MALI (2016-2026) y regenera el .xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bob4w11uQRyAcv1Qayw1V
</commit_message>
<xml_diff>
--- a/Sistematización/tablas-sistematizacion.xlsx
+++ b/Sistematización/tablas-sistematizacion.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Extras" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cap 2 - Historia'!$A$1:$F$82</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cap 3 - Análisis'!$A$1:$F$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Teoría'!$A$1:$F$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Extras'!$A$1:$F$4</definedName>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2654,59 +2654,59 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>sura.md</t>
+          <t>mali_exposiciones_2026-07-18.md</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>mediados de la década de 1960 a 2013 (arte contemporáneo peruano)</t>
+          <t>2016–2026 (exposiciones documentadas de agosto 2016 a julio 2026)</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Catálogo de colección museística, 2013</t>
+          <t>Archivo/recopilación del sitio web del MALI (mali.pe), generado el 18/07/2026</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner (ed.); Museo de Arte de Lima (MALI); Grupo SURA; Mirko Lauer; E.P.S. Huayco; Charo Noriega; Ramiro Llona; Flavia Gandolfo; Armando Andrade Tudela; Ricardo Wiesse; Eduardo Villanes; Miguel A. López; Rodrigo Quijano</t>
+          <t>Museo de Arte de Lima (MALI); curadores del museo (Luis Eduardo Wuffarden, Ricardo Kusunoki, María Eugenia Yllia, Carlo Trivelli, entre otros); numerosos artistas peruanos e internacionales (Julia Codesido, Olinda Silvano, Sara Flores, Francis Alÿs, Not Vital, Richard Tuttle, Abraham Cruzvillegas, Sandra Gamarra, Armando Andrade Tudela, Eielson, etc.); Bank of America y otros patrocinadores</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Catálogo de la colección de arte contemporáneo del Museo de Arte de Lima (MALI), editado por la curadora Sharon Lerner y publicado con el patrocinio del grupo SURA. El volumen traza los derroteros del arte peruano reciente a partir del acervo del museo, sin pretender definir un 'arte peruano' esencial. La colección se articula bajo dos principios: identificar momentos de ruptura en la producción artística de fines del siglo XX y perfilar la producción reciente mediante ejes temáticos comunes. El ensayo central de Lerner establece como punto de partida mediados de la década de 1960 (grupos de vanguardia ligados al Pop y al no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, tras las reformas del Gobierno Militar, cuando —según la célebre frase de Mirko Lauer para la muestra Arte al paso del colectivo E.P.S. Huayco (1980)— 'en el Perú hoy solo lo popular es moderno'. Analiza la irrupción de la migración interna, el conflicto armado interno, el autogolpe de Fujimori (1992) y la virtual desaparición de la esfera pública, así como la Bienal Iberoamericana de Lima (1997) como puesta al día forzada y descontextualizada. El catálogo se organiza en núcleos temáticos: modernidad popular y transformación de Lima, f(r)icciones cosmopolitas, reconsideración del pasado y configuración del Perú, sistema artístico y utopías museales, desplazamientos, y signos de violencia, resistencia y memoria. Incluye obras de Charo Noriega, Ramiro Llona, Flavia Gandolfo, Armando Andrade Tudela, Herman Schwarz, Ricardo Wiesse y Eduardo Villanes, entre otros, y textos críticos complementarios. Su aporte es consolidar un relato historiográfico y crítico del arte contemporáneo peruano desde una institución museal.</t>
+          <t>Recopilación (scraping) del archivo de exposiciones publicado en el sitio web del Museo de Arte de Lima (mali.pe), generada el 18 de julio de 2026. Reúne 64 exposiciones ordenadas de la más reciente a la más antigua, cubriendo una década de programación del museo (agosto de 2016 a julio de 2026). Cada entrada consigna el título de la muestra, la fecha y hora de apertura, el lugar exacto dentro del museo (sala y piso), un conjunto de etiquetas temáticas ('arte contemporáneo', 'arte moderno', 'arte peruano', 'fotografía', 'instalación', 'intervenciones MALI') y el texto curatorial oficial del museo, además del enlace a la ficha en mali.pe. El corpus abarca un espectro amplio: arte moderno e histórico peruano (Julia Codesido, 'Los años sesenta', Eielson), arte contemporáneo internacional (Not Vital, Francis Alÿs, Richard Tuttle, Abraham Cruzvillegas, Rosa Barba), arte indígena y amazónico (Olinda Silvano y el kené shipibo-konibo, Sara Flores, 'Amazonías'), fotografía, y muestras que exhiben la propia colección y sus incorporaciones recientes —notablemente 'MALI Colecciones. Adquisiciones y donaciones (2019–2023)' y 'MALI Colecciones. Primera etapa: Intervenciones Contemporáneas'—. Como fuente, documenta de manera sistemática qué programa, cura, exhibe y valoriza la principal institución museística del país a lo largo de diez años; los textos son copy institucional (la voz del museo enunciando el valor de cada muestra), por lo que constituyen discurso de la gestión cultural más que descripción neutral. Fuente primaria clave para la dimensión de la gestión operando sobre el arte contemporáneo (programación, curaduría, coleccionismo institucional) y para el giro descolonial/indígena y la inserción global en el circuito museístico limeño.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Arte al Paso 2011</t>
+          <t>Cap 2 - Historia</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Arte al Paso - Texto Investigación.md</t>
+          <t>sura.md</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 1960 – 2010 (con foco en las décadas de 1970-2000 y el conflicto armado interno 1980-2000)</t>
+          <t>mediados de la década de 1960 a 2013 (arte contemporáneo peruano)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Ensayo curatorial de catálogo (exposición Arte al paso, Pinacoteca do Estado de São Paulo, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Catálogo de colección museística, 2013</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Pinacoteca de São Paulo; Emilio Hernández Saavedra; E.P.S. Huayco; Jesús Ruiz Durand; Sandra Gamarra; Alfredo Márquez / Taller NN; Fernando Bryce; José Carlos Martinat; Susana Torres</t>
+          <t>Sharon Lerner (ed.); Museo de Arte de Lima (MALI); Grupo SURA; Mirko Lauer; E.P.S. Huayco; Charo Noriega; Ramiro Llona; Flavia Gandolfo; Armando Andrade Tudela; Ricardo Wiesse; Eduardo Villanes; Miguel A. López; Rodrigo Quijano</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Ensayo curatorial extenso y bilingüe (castellano/portugués) de Tatiana Cuevas y Rodrigo Quijano para la muestra Arte al paso, que exhibió la coleccion contemporanea del MALI en la Estacion Pinacoteca de Sao Paulo. El texto toma como punto de partida la imagen El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra para diagnosticar los vacios institucionales y la distancia entre el discurso cultural cosmopolita y la practica real en el Peru de la segunda mitad del siglo XX. Su argumento articula el arte contemporaneo peruano con las transformaciones sociales derivadas de la masiva migracion rural a Lima, la explosion de la economia informal y la emergencia de una nueva cultura popular urbana. Rastrea las primeras vinculaciones locales con vanguardias internacionales (op, pop, conceptualismo, no-objetualismo), el pop achorado de Jesus Ruiz Durand y sus afiches de la Reforma Agraria velasquista, y las experiencias colectivas Contacta 79 y Arte al paso de E.P.S. Huayco (1980), que propusieron un arte callejero y antiinstitucional. Analiza la critica a la institucionalidad faltante (el museo ficticio LiMAC de Sandra Gamarra), el uso ironico del pasado prehispanico (Susana Torres, Rodriguez Larrain, Bryce, Cordova, Martinat), el tema del paisaje y el territorio, y la irrupcion tardia de la fotografia y la serigrafia como medios. Dedica una seccion central a la memoria de la violencia del conflicto armado interno (1980-2000) —Sendero Luminoso, MRTA, la Comision de la Verdad, 69.280 muertos— y su tratamiento por el Taller NN, Alfredo Marquez (Katatay), Carlos Dominguez, Ricardo Wiesse, Eduardo Villanes, Fernando Bryce y Milagros de la Torre.</t>
+          <t>Catálogo de la colección de arte contemporáneo del Museo de Arte de Lima (MALI), editado por la curadora Sharon Lerner y publicado con el patrocinio del grupo SURA. El volumen traza los derroteros del arte peruano reciente a partir del acervo del museo, sin pretender definir un 'arte peruano' esencial. La colección se articula bajo dos principios: identificar momentos de ruptura en la producción artística de fines del siglo XX y perfilar la producción reciente mediante ejes temáticos comunes. El ensayo central de Lerner establece como punto de partida mediados de la década de 1960 (grupos de vanguardia ligados al Pop y al no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, tras las reformas del Gobierno Militar, cuando —según la célebre frase de Mirko Lauer para la muestra Arte al paso del colectivo E.P.S. Huayco (1980)— 'en el Perú hoy solo lo popular es moderno'. Analiza la irrupción de la migración interna, el conflicto armado interno, el autogolpe de Fujimori (1992) y la virtual desaparición de la esfera pública, así como la Bienal Iberoamericana de Lima (1997) como puesta al día forzada y descontextualizada. El catálogo se organiza en núcleos temáticos: modernidad popular y transformación de Lima, f(r)icciones cosmopolitas, reconsideración del pasado y configuración del Perú, sistema artístico y utopías museales, desplazamientos, y signos de violencia, resistencia y memoria. Incluye obras de Charo Noriega, Ramiro Llona, Flavia Gandolfo, Armando Andrade Tudela, Herman Schwarz, Ricardo Wiesse y Eduardo Villanes, entre otros, y textos críticos complementarios. Su aporte es consolidar un relato historiográfico y crítico del arte contemporáneo peruano desde una institución museal.</t>
         </is>
       </c>
     </row>
@@ -2718,27 +2718,27 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Cronología Político Artistica - Arte al Paso 2011.md</t>
+          <t>Arte al Paso - Texto Investigación.md</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>1962 – 2010</t>
+          <t>Fines de los años 1960 – 2010 (con foco en las décadas de 1970-2000 y el conflicto armado interno 1980-2000)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Cronología y bibliografía de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Ensayo curatorial de catálogo (exposición Arte al paso, Pinacoteca do Estado de São Paulo, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Museo de Arte de Lima (MALI); Grupo Arte Nuevo; Grupo Señal; E.P.S. Huayco; Taller NN; Colectivo Sociedad Civil; Gustavo Buntinx; Joaquín López Antay; Comisión de la Verdad y Reconciliación; Sendero Luminoso; Alberto Fujimori; Juan Velasco Alvarado</t>
+          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Pinacoteca de São Paulo; Emilio Hernández Saavedra; E.P.S. Huayco; Jesús Ruiz Durand; Sandra Gamarra; Alfredo Márquez / Taller NN; Fernando Bryce; José Carlos Martinat; Susana Torres</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Cronologia politico-artistica bilingue (castellano/portugues) incluida en el catalogo Arte al paso, que entrelaza en paralelo tres series de acontecimientos —eventos politicos, eventos artisticos y adquisiciones de la coleccion de arte contemporaneo del MALI— entre 1962 y 2010. El documento funciona como aparato historiografico que contextualiza la escena artistica peruana dentro de sus convulsiones politicas: rebeliones campesinas y golpes militares de los anos sesenta, el Gobierno Revolucionario de las Fuerzas Armadas de Velasco Alvarado (1968) y la Reforma Agraria, el estallido del conflicto armado interno con Sendero Luminoso y el MRTA (1980), las masacres de Barrios Altos y La Cantuta, el autogolpe y la dictadura de Alberto Fujimori (1990-2000), la Marcha de los Cuatro Suyos y el Informe de la Comision de la Verdad y Reconciliacion (2003). En el plano artistico registra la formacion de los grupos Senal y Arte Nuevo, las Bienales de Lima e Iberoamericanas, los festivales Contacta e Inkarri, el Taller E.P.S. Huayco y el Taller NN, la premiacion de Joaquin Lopez Antay, y acciones de arte critico como Cantuta de Ricardo Wiesse, Gloria evaporada de Eduardo Villanes y Lava la bandera del Colectivo Sociedad Civil. Una tercera linea traza la institucionalizacion del MALI: el ciclo curatorial Miradas de fin de siglo, la creacion del Comite de Adquisiciones (2007) y la reapertura del museo (2010). Se acompana de una extensa bibliografia especializada (Buntinx, Castrillon, Lauer, Majluf, Lopez, Tarazona, Quijano, Villacorta), fuente clave para la historiografia del arte peruano contemporaneo.</t>
+          <t>Ensayo curatorial extenso y bilingüe (castellano/portugués) de Tatiana Cuevas y Rodrigo Quijano para la muestra Arte al paso, que exhibió la coleccion contemporanea del MALI en la Estacion Pinacoteca de Sao Paulo. El texto toma como punto de partida la imagen El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra para diagnosticar los vacios institucionales y la distancia entre el discurso cultural cosmopolita y la practica real en el Peru de la segunda mitad del siglo XX. Su argumento articula el arte contemporaneo peruano con las transformaciones sociales derivadas de la masiva migracion rural a Lima, la explosion de la economia informal y la emergencia de una nueva cultura popular urbana. Rastrea las primeras vinculaciones locales con vanguardias internacionales (op, pop, conceptualismo, no-objetualismo), el pop achorado de Jesus Ruiz Durand y sus afiches de la Reforma Agraria velasquista, y las experiencias colectivas Contacta 79 y Arte al paso de E.P.S. Huayco (1980), que propusieron un arte callejero y antiinstitucional. Analiza la critica a la institucionalidad faltante (el museo ficticio LiMAC de Sandra Gamarra), el uso ironico del pasado prehispanico (Susana Torres, Rodriguez Larrain, Bryce, Cordova, Martinat), el tema del paisaje y el territorio, y la irrupcion tardia de la fotografia y la serigrafia como medios. Dedica una seccion central a la memoria de la violencia del conflicto armado interno (1980-2000) —Sendero Luminoso, MRTA, la Comision de la Verdad, 69.280 muertos— y su tratamiento por el Taller NN, Alfredo Marquez (Katatay), Carlos Dominguez, Ricardo Wiesse, Eduardo Villanes, Fernando Bryce y Milagros de la Torre.</t>
         </is>
       </c>
     </row>
@@ -2750,59 +2750,59 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Texto de la exposición Arte al Paso 2011.md</t>
+          <t>Cronología Político Artistica - Arte al Paso 2011.md</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Fines de los años 1960 – 2010 (unos 40 años; foco en las décadas de 1970-1980)</t>
+          <t>1962 – 2010</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Texto de sala / presentación de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
+          <t>Cronología y bibliografía de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Emilio Hernández Saavedra; E.P.S. Huayco; Grupo Paréntesis; Sandra Gamarra; Susana Torres; Emilio Rodríguez Larraín; Juan Javier Salazar; William Cordova; José Carlos Martinat</t>
+          <t>Museo de Arte de Lima (MALI); Grupo Arte Nuevo; Grupo Señal; E.P.S. Huayco; Taller NN; Colectivo Sociedad Civil; Gustavo Buntinx; Joaquín López Antay; Comisión de la Verdad y Reconciliación; Sendero Luminoso; Alberto Fujimori; Juan Velasco Alvarado</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Texto de sala o presentacion general de la exposicion Arte al paso (coleccion contemporanea del MALI en la Pinacoteca de Sao Paulo), firmado por los curadores Tatiana Cuevas y Rodrigo Quijano, en edicion bilingue castellano/portugues. Es una version sintetica del argumento curatorial: parte nuevamente de El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra como metafora de la ausencia institucional y punto de arranque para examinar la escena artistica peruana desde fines de los anos sesenta. Explica el titulo de la muestra a partir de la accion Arte al paso de E.P.S. Huayco (1980) —que, aludiendo a los puestos informales de comida al paso surgidos con la migracion y la economia informal, propuso un arte para consumirse en la calle, opuesto al museo y la galeria ausentes, un arte para pensar y no para sentir que dejaba atras el modernismo conservador de mediados de siglo. Sintetiza cuarenta anos de produccion cultural marcados por oposiciones ocultas y explicitas, los primeros acercamientos al conceptualismo y a las vanguardias internacionales, y la creciente proyeccion internacional de artistas peruanos. Una segunda seccion, Critica ante una institucionalidad faltante y al poder redentor del pasado, reune a Hernandez Saavedra, los grupos Parentesis y E.P.S. Huayco y el museo ficticio de Sandra Gamarra como estrategias de critica institucional apropiadas del conceptualismo y del imaginario popular urbano, con recurrente uso del humor. Aborda ademas la critica a la explotacion comercial y politica de lo prehispanico (Museo Neo-Inka de Susana Torres) y el vinculo entre la retorica del glorioso pasado incaico y los fracasos politicos y economicos del presente en obras de Rodriguez Larrain, Salazar, Cordova y Martinat.</t>
+          <t>Cronologia politico-artistica bilingue (castellano/portugues) incluida en el catalogo Arte al paso, que entrelaza en paralelo tres series de acontecimientos —eventos politicos, eventos artisticos y adquisiciones de la coleccion de arte contemporaneo del MALI— entre 1962 y 2010. El documento funciona como aparato historiografico que contextualiza la escena artistica peruana dentro de sus convulsiones politicas: rebeliones campesinas y golpes militares de los anos sesenta, el Gobierno Revolucionario de las Fuerzas Armadas de Velasco Alvarado (1968) y la Reforma Agraria, el estallido del conflicto armado interno con Sendero Luminoso y el MRTA (1980), las masacres de Barrios Altos y La Cantuta, el autogolpe y la dictadura de Alberto Fujimori (1990-2000), la Marcha de los Cuatro Suyos y el Informe de la Comision de la Verdad y Reconciliacion (2003). En el plano artistico registra la formacion de los grupos Senal y Arte Nuevo, las Bienales de Lima e Iberoamericanas, los festivales Contacta e Inkarri, el Taller E.P.S. Huayco y el Taller NN, la premiacion de Joaquin Lopez Antay, y acciones de arte critico como Cantuta de Ricardo Wiesse, Gloria evaporada de Eduardo Villanes y Lava la bandera del Colectivo Sociedad Civil. Una tercera linea traza la institucionalizacion del MALI: el ciclo curatorial Miradas de fin de siglo, la creacion del Comite de Adquisiciones (2007) y la reapertura del museo (2010). Se acompana de una extensa bibliografia especializada (Buntinx, Castrillon, Lauer, Majluf, Lopez, Tarazona, Quijano, Villacorta), fuente clave para la historiografia del arte peruano contemporaneo.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/Hueso Húmero 18</t>
+          <t>Cap 2 - Historia/Arte al Paso 2011</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - Arte joven peruano, ¿el sueño del mercado propio? Una conversación con Claudia Polar (1983) [Hueso Húmero 18, pp. 94-107].md</t>
+          <t>Texto de la exposición Arte al Paso 2011.md</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>1974-1983</t>
+          <t>Fines de los años 1960 – 2010 (unos 40 años; foco en las décadas de 1970-1980)</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Entrevista en revista (Hueso Húmero 18), 1983</t>
+          <t>Texto de sala / presentación de catálogo (exposición Arte al paso, 2011); archivo digitalizado por OCR el 16-07-2026</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Claudia Polar; Galería Forum; Elida Román; Hernán Pazos; Esther Vainstein; Ramiro Llona; Bill Caro; Herbert Rodríguez; EAPUC; ENBA; Hueso Húmero</t>
+          <t>Tatiana Cuevas; Rodrigo Quijano; Museo de Arte de Lima (MALI); Emilio Hernández Saavedra; E.P.S. Huayco; Grupo Paréntesis; Sandra Gamarra; Susana Torres; Emilio Rodríguez Larraín; Juan Javier Salazar; William Cordova; José Carlos Martinat</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>Entrevista conducida por Gustavo Buntinx a Claudia Polar, directora de la Galería Forum, concebida como contraparte de un reportaje previo a Elida Román para perfilar el mercado del arte joven peruano. Polar reconstruye la fundación de Forum en diciembre de 1974 como un espacio destinado a priorizar a los artistas jóvenes y a gestar deliberadamente un mercado y coleccionistas nuevos, mediante becas, premios, subvenciones informales (incluso marcos y pasajes) y una política de "riesgo total" sostenida por la venta de stock. El diálogo traza una periodización económica de la plástica: expansión del mercado hacia 1974-1976, auge en 1978 atribuido a la restricción de importaciones bajo Morales Bermúdez, y recesión desde 1980 con la apertura de Belaúnde, siendo 1983 el año más difícil. Se discute la naturaleza del público comprador (gente joven, profesionales, empresarios, bancos como el de Crédito y el Continental) y la débil proporción de compradores habituales, apenas un 5% con relación económica. Buntinx presiona sobre las mediaciones de clase: el vínculo de Forum con la Universidad Católica frente a la ENBA, la identidad ideológica compartida, y el papel de las relaciones públicas como "gatillo" de casi toda venta en un mercado de "sala de estar". Polar aborda la diferencia entre lo culto y lo popular, el fracaso de asociar galerías, las cotizaciones (Llona, Caro, Pazos, Vainstein) y la explotación del artista acostumbrado a vender barato. El aporte documental es excepcional: registra desde dentro la lógica comercial, simbólica y provinciana del circuito limeño de principios de los ochenta.</t>
+          <t>Texto de sala o presentacion general de la exposicion Arte al paso (coleccion contemporanea del MALI en la Pinacoteca de Sao Paulo), firmado por los curadores Tatiana Cuevas y Rodrigo Quijano, en edicion bilingue castellano/portugues. Es una version sintetica del argumento curatorial: parte nuevamente de El Museo de Arte borrado (1970) de Emilio Hernandez Saavedra como metafora de la ausencia institucional y punto de arranque para examinar la escena artistica peruana desde fines de los anos sesenta. Explica el titulo de la muestra a partir de la accion Arte al paso de E.P.S. Huayco (1980) —que, aludiendo a los puestos informales de comida al paso surgidos con la migracion y la economia informal, propuso un arte para consumirse en la calle, opuesto al museo y la galeria ausentes, un arte para pensar y no para sentir que dejaba atras el modernismo conservador de mediados de siglo. Sintetiza cuarenta anos de produccion cultural marcados por oposiciones ocultas y explicitas, los primeros acercamientos al conceptualismo y a las vanguardias internacionales, y la creciente proyeccion internacional de artistas peruanos. Una segunda seccion, Critica ante una institucionalidad faltante y al poder redentor del pasado, reune a Hernandez Saavedra, los grupos Parentesis y E.P.S. Huayco y el museo ficticio de Sandra Gamarra como estrategias de critica institucional apropiadas del conceptualismo y del imaginario popular urbano, con recurrente uso del humor. Aborda ademas la critica a la explotacion comercial y politica de lo prehispanico (Museo Neo-Inka de Susana Torres) y el vinculo entre la retorica del glorioso pasado incaico y los fracasos politicos y economicos del presente en obras de Rodriguez Larrain, Salazar, Cordova y Martinat.</t>
         </is>
       </c>
     </row>
@@ -2814,27 +2814,27 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - ¿Entre lo popular y lo moderno? Alternativas pretendidas o reales en la joven plástica peruana (1983) [Hueso Húmero 18, pp. 61-85].md</t>
+          <t>Buntinx - Arte joven peruano, ¿el sueño del mercado propio? Una conversación con Claudia Polar (1983) [Hueso Húmero 18, pp. 94-107].md</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>1960-1984 (con énfasis en los años 70)</t>
+          <t>1974-1983</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
+          <t>Entrevista en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; Mirko Lauer; Juan Acha; Francisco Mariotti; Huayco E.P.S.; Herbert Rodríguez; Juan Javier Salazar; Jesús Ruiz Durand; Fernando de Szyszlo; IAC; Galería Forum; SINAMOS; Néstor García Canclini</t>
+          <t>Gustavo Buntinx; Claudia Polar; Galería Forum; Elida Román; Hernán Pazos; Esther Vainstein; Ramiro Llona; Bill Caro; Herbert Rodríguez; EAPUC; ENBA; Hueso Húmero</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Ensayo teórico-histórico que propone hipótesis de trabajo sobre lo que fue o pretendió ser alternativo en el arte erudito peruano desde la transición al primer belaundismo hasta los años ochenta, articulando dos tópicos móviles: lo popular y lo moderno. Retomando y ampliando a Mirko Lauer, Buntinx sostiene que las opciones estéticas no reflejan mecánicamente la época sino que reproducen una inserción particular en el mercado, entendido como trama compleja de producción, intermediación y consumo (soporte social). Recorre así una secuencia de "soportes": el corporativo (IAC financiado por IPC, IBM, Tecnoquímica) que sostuvo la Teoría de las Raíces Nacionales de Szyszlo; el soporte "de punta" del frenesí pop cosmopolita (Acha, Arte Nuevo, Fundación para las Artes, 1966-1969); el soporte estatal velasquista con sus cuatro alternativas (comunicación masiva de Ruiz Durand con su "pop achorado", festivales de arte-total como Contacta e Inkarri, revaloración de lo artesanal, López Antay); y la frustrada búsqueda de un soporte alternativo hacia 1977-1980. El caso central es Huayco E.P.S., cuyo proyecto Sarita Colonia codifica una modernidad sincrética limeña sostenida por una pequeña burguesía ilustrada radicalizada, y cuya dispersión coincide con el agotamiento de la izquierda y el repliegue hacia el mercado galerístico (Forum). El marco conceptual bebe de García Canclini. La tesis es incisiva: el tránsito de la imagen telúrica a la industrial, agraria y migrante revela apropiaciones sucesivas de una idea variable de lo popular, siempre con una radicalidad deficiente y una relación desigual con la cultura interpretada.</t>
+          <t>Entrevista conducida por Gustavo Buntinx a Claudia Polar, directora de la Galería Forum, concebida como contraparte de un reportaje previo a Elida Román para perfilar el mercado del arte joven peruano. Polar reconstruye la fundación de Forum en diciembre de 1974 como un espacio destinado a priorizar a los artistas jóvenes y a gestar deliberadamente un mercado y coleccionistas nuevos, mediante becas, premios, subvenciones informales (incluso marcos y pasajes) y una política de "riesgo total" sostenida por la venta de stock. El diálogo traza una periodización económica de la plástica: expansión del mercado hacia 1974-1976, auge en 1978 atribuido a la restricción de importaciones bajo Morales Bermúdez, y recesión desde 1980 con la apertura de Belaúnde, siendo 1983 el año más difícil. Se discute la naturaleza del público comprador (gente joven, profesionales, empresarios, bancos como el de Crédito y el Continental) y la débil proporción de compradores habituales, apenas un 5% con relación económica. Buntinx presiona sobre las mediaciones de clase: el vínculo de Forum con la Universidad Católica frente a la ENBA, la identidad ideológica compartida, y el papel de las relaciones públicas como "gatillo" de casi toda venta en un mercado de "sala de estar". Polar aborda la diferencia entre lo culto y lo popular, el fracaso de asociar galerías, las cotizaciones (Llona, Caro, Pazos, Vainstein) y la explotación del artista acostumbrado a vender barato. El aporte documental es excepcional: registra desde dentro la lógica comercial, simbólica y provinciana del circuito limeño de principios de los ochenta.</t>
         </is>
       </c>
     </row>
@@ -2846,27 +2846,27 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Freire - Herbert Rodríguez, azote y azúcar con el sistema (1983) [Hueso Húmero 18, pdf pp. 178-185].md</t>
+          <t>Buntinx - ¿Entre lo popular y lo moderno? Alternativas pretendidas o reales en la joven plástica peruana (1983) [Hueso Húmero 18, pp. 61-85].md</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>1979-1983 (con antecedentes desde 1968)</t>
+          <t>1960-1984 (con énfasis en los años 70)</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Reseña crítica en revista (Hueso Húmero 18), 1983</t>
+          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Luis Freire S.; Herbert Rodríguez; Francisco Mariotti; Huayco E.P.S.; Juan Acha; Fernando Bedoya; Juan Javier Salazar; Bienal de Sao Paulo; Galería La Rama Dorada; Galería Forum; EAPUC; ENBAP</t>
+          <t>Gustavo Buntinx; Mirko Lauer; Juan Acha; Francisco Mariotti; Huayco E.P.S.; Herbert Rodríguez; Juan Javier Salazar; Jesús Ruiz Durand; Fernando de Szyszlo; IAC; Galería Forum; SINAMOS; Néstor García Canclini</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Perfil crítico dedicado a Herbert Rodríguez Huachín en la sección "Individuales" de Hueso Húmero, escrito por Luis Freire, que examina el salto vertiginoso del artista desde la suspensión disciplinaria en la Escuela de Artes Plásticas de la Católica (1981) hasta su presencia en la XVII Bienal de Sao Paulo (1983). Freire sitúa a Rodríguez como imposible de explicar sin el proceso ideológico del populismo velasquista y sin la figura mediadora de Francisco Mariotti, artista suizo-peruano formado en la Documenta de Kassel y la vanguardia europea, catalizador de Contacta y de la EPS Huayco. El texto reconstruye la genealogía Mariotti-Huayco-Rodríguez: los ensamblajes y "reciclajes" del suizo-peruano derivan en los "altares" de Rodríguez, hibridación entre constructivismo geométrico, expresionismo "pobre" y antiestético, y estructuras rituales de la religiosidad popular andina. Argumenta que Rodríguez encarna las contradicciones de una pequeña burguesía radical: dinamita el circuito con una mano y lo enluce con la otra, camuflando "bellamente" materiales pobres y reciclados en obras a la vez contestatarias y comerciables, con lo que ironiza sobre el culto al oficio del arte establecido. Analiza su heterogeneidad de lenguajes (expresionismo abstracto, figuración dura, conceptualismo informal, collage, fotocopia, ensamblaje) como búsqueda pero también como crisis, y sus "altares al Yo" exhibidos en Forum (1983) y la Bienal. Freire lo define como un artista religioso-existencial populista sin referentes sólidos, en formación, tensionado entre enriquecer el jardín burgués que quiere pisotear o saltar a opciones más radicales de ruptura.</t>
+          <t>Ensayo teórico-histórico que propone hipótesis de trabajo sobre lo que fue o pretendió ser alternativo en el arte erudito peruano desde la transición al primer belaundismo hasta los años ochenta, articulando dos tópicos móviles: lo popular y lo moderno. Retomando y ampliando a Mirko Lauer, Buntinx sostiene que las opciones estéticas no reflejan mecánicamente la época sino que reproducen una inserción particular en el mercado, entendido como trama compleja de producción, intermediación y consumo (soporte social). Recorre así una secuencia de "soportes": el corporativo (IAC financiado por IPC, IBM, Tecnoquímica) que sostuvo la Teoría de las Raíces Nacionales de Szyszlo; el soporte "de punta" del frenesí pop cosmopolita (Acha, Arte Nuevo, Fundación para las Artes, 1966-1969); el soporte estatal velasquista con sus cuatro alternativas (comunicación masiva de Ruiz Durand con su "pop achorado", festivales de arte-total como Contacta e Inkarri, revaloración de lo artesanal, López Antay); y la frustrada búsqueda de un soporte alternativo hacia 1977-1980. El caso central es Huayco E.P.S., cuyo proyecto Sarita Colonia codifica una modernidad sincrética limeña sostenida por una pequeña burguesía ilustrada radicalizada, y cuya dispersión coincide con el agotamiento de la izquierda y el repliegue hacia el mercado galerístico (Forum). El marco conceptual bebe de García Canclini. La tesis es incisiva: el tránsito de la imagen telúrica a la industrial, agraria y migrante revela apropiaciones sucesivas de una idea variable de lo popular, siempre con una radicalidad deficiente y una relación desigual con la cultura interpretada.</t>
         </is>
       </c>
     </row>
@@ -2878,59 +2878,59 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Lama - Los años de la resaca (1983) [Hueso Húmero 18, pdf pp. 136-156].md</t>
+          <t>Freire - Herbert Rodríguez, azote y azúcar con el sistema (1983) [Hueso Húmero 18, pdf pp. 178-185].md</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>1974-1983 (con antecedentes en los años 60-70)</t>
+          <t>1979-1983 (con antecedentes desde 1968)</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
+          <t>Reseña crítica en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>Luis Lama; Hernán Pazos; Francisco Mariotti; Contacta; grupo Huayco; Juan Javier Salazar; Herbert Rodríguez; Alfonso Castrillón; Escuela Nacional de Bellas Artes; Galería Forum; Galería 9; Ugarte Eléspuru</t>
+          <t>Luis Freire S.; Herbert Rodríguez; Francisco Mariotti; Huayco E.P.S.; Juan Acha; Fernando Bedoya; Juan Javier Salazar; Bienal de Sao Paulo; Galería La Rama Dorada; Galería Forum; EAPUC; ENBAP</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Ensayo de Luis Lama que narra el paso de la "ebullición ideológica" de los años setenta a la "resaca" del segundo belaundismo, articulando historia social del arte y crítica biográfica. La primera parte reconstruye los antecedentes: el terremoto de 1974 y el reflujo de artistas jóvenes hacia Barranco, la gravitación de Francisco Mariotti que transforma el arte de sistemas en movimiento grupal con Contacta e Inkari bajo auspicio de SINAMOS, las tomas y la crisis de la Escuela Nacional de Bellas Artes (1974-1976), y la gestación del taller de Pedro de Osma que devendría núcleo del grupo Huayco (Juan Javier Salazar, Herbert Rodríguez, Charo Noriega, Fernando Bedoya, Lucy Angulo). Lama describe la consolidación paradójica del mercado del arte al amparo de la prohibición de importaciones, con galerías que proliferan mientras la formación académica alcanza sus niveles más bajos. Diagnostica el fin de los happenings sesenteros y el retorno de un expresionismo "de crisis" impulsado desde los predios católicos (Williams, Polanco, Velarde, Hamann), junto a indagaciones matéricas de Wiesse y el conceptualismo de Vainstein. La segunda mitad es un retrato extenso de Hernán Pazos: su formación entre Derecho, la Católica y París, su tránsito del conceptualismo (los cielos y nubes de Galería 9) a la abstracción cromática, las series de los Quipus y los dibujos infantiles, su gestión en Rama Dorada y su individualismo parricida. Lama lo consagra como el artista más destacado de la década, emblema lúcido de las "amargas frustraciones" nacionales bajo el liberalismo económico belaundista.</t>
+          <t>Perfil crítico dedicado a Herbert Rodríguez Huachín en la sección "Individuales" de Hueso Húmero, escrito por Luis Freire, que examina el salto vertiginoso del artista desde la suspensión disciplinaria en la Escuela de Artes Plásticas de la Católica (1981) hasta su presencia en la XVII Bienal de Sao Paulo (1983). Freire sitúa a Rodríguez como imposible de explicar sin el proceso ideológico del populismo velasquista y sin la figura mediadora de Francisco Mariotti, artista suizo-peruano formado en la Documenta de Kassel y la vanguardia europea, catalizador de Contacta y de la EPS Huayco. El texto reconstruye la genealogía Mariotti-Huayco-Rodríguez: los ensamblajes y "reciclajes" del suizo-peruano derivan en los "altares" de Rodríguez, hibridación entre constructivismo geométrico, expresionismo "pobre" y antiestético, y estructuras rituales de la religiosidad popular andina. Argumenta que Rodríguez encarna las contradicciones de una pequeña burguesía radical: dinamita el circuito con una mano y lo enluce con la otra, camuflando "bellamente" materiales pobres y reciclados en obras a la vez contestatarias y comerciables, con lo que ironiza sobre el culto al oficio del arte establecido. Analiza su heterogeneidad de lenguajes (expresionismo abstracto, figuración dura, conceptualismo informal, collage, fotocopia, ensamblaje) como búsqueda pero también como crisis, y sus "altares al Yo" exhibidos en Forum (1983) y la Bienal. Freire lo define como un artista religioso-existencial populista sin referentes sólidos, en formación, tensionado entre enriquecer el jardín burgués que quiere pisotear o saltar a opciones más radicales de ruptura.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Cap 2 - Historia/MALI</t>
+          <t>Cap 2 - Historia/Hueso Húmero 18</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Buntinx - El poder y la ilusión. Pérdida y restauración del aura en la «República de Weimar peruana» 1980-1992 [MALI].md</t>
+          <t>Lama - Los años de la resaca (1983) [Hueso Húmero 18, pdf pp. 136-156].md</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>1980-1992</t>
+          <t>1974-1983 (con antecedentes en los años 60-70)</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico (versión MALI), 2013 [escrito 1991-1994]</t>
+          <t>Ensayo en revista (Hueso Húmero 18), 1983</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Buntinx; E.P.S. Huayco; Taller NN; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; Walter Benjamin; Jesús Ruiz Durand; Andy Warhol; Mirko Lauer; Museo de Arte de Lima (MALI); III Bienal de La Habana</t>
+          <t>Luis Lama; Hernán Pazos; Francisco Mariotti; Contacta; grupo Huayco; Juan Javier Salazar; Herbert Rodríguez; Alfonso Castrillón; Escuela Nacional de Bellas Artes; Galería Forum; Galería 9; Ugarte Eléspuru</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Ensayo seminal de Gustavo Buntinx —redactado entre 1991 y 1994, difundido en inglés en «Beyond the Fantastic» (1995) y publicado por primera vez en Perú en esta versión del MALI (2013)— que interpreta el radical cambio de época del arte peruano entre 1980 y 1992, periodo que denomina metafóricamente «República de Weimar peruana». Su marco conceptual adapta la dialéctica benjaminiana entre proximidad y distancia (el aura, su pérdida por la reproductibilidad técnica y su posible restauración) y las categorías de alegoría, montaje y apropiación de Owens, Foster y Craig Owens a una periferia extrema. El argumento se sostiene sobre el análisis iconográfico minucioso de dos o tres obras que abren y cierran la década. La primera, «Arte al paso» y sobre todo «Sarita Colonia» (1980) del taller E.P.S. Huayco: una enorme estampa de la santa migrante pintada sobre diez mil latas de leche y emplazada en la Panamericana Sur, que Buntinx lee como huaca (post)moderna y exvoto donde lo pequeñoburgués radical se articula figuradamente a lo popular en emergencia (el «pop achorado» y «chicha»). La segunda, «Maorilyn» / «Viva el maoísmo» (1989) del Taller NN: una serigrafía que travistió el rostro de Mao con labios warholianos, alegoría ambivalente de la violencia senderista y la estetización de la política. Su tesis vincula la desintegración social —hiperinflación, guerra civil, movida subte punk— con el desarrollo de una condición alegórica y neo-aurática; su aporte es un modelo teórico para leer el colectivismo y la (post)modernidad popular peruana.</t>
+          <t>Ensayo de Luis Lama que narra el paso de la "ebullición ideológica" de los años setenta a la "resaca" del segundo belaundismo, articulando historia social del arte y crítica biográfica. La primera parte reconstruye los antecedentes: el terremoto de 1974 y el reflujo de artistas jóvenes hacia Barranco, la gravitación de Francisco Mariotti que transforma el arte de sistemas en movimiento grupal con Contacta e Inkari bajo auspicio de SINAMOS, las tomas y la crisis de la Escuela Nacional de Bellas Artes (1974-1976), y la gestación del taller de Pedro de Osma que devendría núcleo del grupo Huayco (Juan Javier Salazar, Herbert Rodríguez, Charo Noriega, Fernando Bedoya, Lucy Angulo). Lama describe la consolidación paradójica del mercado del arte al amparo de la prohibición de importaciones, con galerías que proliferan mientras la formación académica alcanza sus niveles más bajos. Diagnostica el fin de los happenings sesenteros y el retorno de un expresionismo "de crisis" impulsado desde los predios católicos (Williams, Polanco, Velarde, Hamann), junto a indagaciones matéricas de Wiesse y el conceptualismo de Vainstein. La segunda mitad es un retrato extenso de Hernán Pazos: su formación entre Derecho, la Católica y París, su tránsito del conceptualismo (los cielos y nubes de Galería 9) a la abstracción cromática, las series de los Quipus y los dibujos infantiles, su gestión en Rama Dorada y su individualismo parricida. Lama lo consagra como el artista más destacado de la década, emblema lúcido de las "amargas frustraciones" nacionales bajo el liberalismo económico belaundista.</t>
         </is>
       </c>
     </row>
@@ -2942,27 +2942,27 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Lerner - Formando la colección de arte contemporáneo del MALI (2013).txt</t>
+          <t>Buntinx - El poder y la ilusión. Pérdida y restauración del aura en la «República de Weimar peruana» 1980-1992 [MALI].md</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>mediados de los años 60 - 2013 (con foco en 1980-2000)</t>
+          <t>1980-1992</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo de colección, 2013</t>
+          <t>Ensayo académico (versión MALI), 2013 [escrito 1991-1994]</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>Sharon Lerner; Museo de Arte de Lima (MALI); Tatiana Cuevas; Miguel A. López; Gustavo Buntinx; Rodrigo Quijano; Jorge Villacorta; Natalia Majluf; E.P.S. Huayco; Teresa Burga; Milagros de la Torre; Flavia Gandolfo</t>
+          <t>Gustavo Buntinx; E.P.S. Huayco; Taller NN; Francisco Mariotti; Herbert Rodríguez; Juan Javier Salazar; Walter Benjamin; Jesús Ruiz Durand; Andy Warhol; Mirko Lauer; Museo de Arte de Lima (MALI); III Bienal de La Habana</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>Ensayo introductorio de Sharon Lerner al libro que presenta la colección de arte contemporáneo del Museo de Arte de Lima (MALI), articulado como una lectura —entre muchas posibles— de la historia del arte reciente peruano a partir del acervo. Su tesis metodológica es que en el Perú el tránsito a la contemporaneidad no ocurre como un quiebre radical, sino como una serie de pequeños cambios discontinuos, por lo que la colección se organiza en dos principios: identificar momentos de ruptura de fines del siglo XX y perfilar la producción reciente por ejes temáticos. El recorrido histórico parte de mediados de los sesenta (vanguardias pop, experimentalismo, no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, cuando la migración y la sentencia de Mirko Lauer —«En el Perú, hoy, solo lo popular es moderno»— enmarcan la obra de E.P.S. Huayco. Recorre luego la hegemonía de la abstracción en los ochenta, el arte de derechos humanos de Ricardo Wiesse y Eduardo Villanes bajo el fujimorato, la irrupción de la Bienal Iberoamericana de Lima (1997) y el «bienalismo», y la generación de los 2000 (Flavia Gandolfo, Gilda Mantilla, Armando Andrade Tudela) vinculada al espacio La Culpable. El texto presenta además los ensayos de Miguel López, Gustavo Buntinx y Rodrigo Quijano incluidos en el volumen y la conversación de seis críticos (2011). Su aporte es explicitar la política de adquisiciones del MALI y su ambición de llenar el vacío institucional y discursivo, construyendo un marco regional e internacional para el arte peruano.</t>
+          <t>Ensayo seminal de Gustavo Buntinx —redactado entre 1991 y 1994, difundido en inglés en «Beyond the Fantastic» (1995) y publicado por primera vez en Perú en esta versión del MALI (2013)— que interpreta el radical cambio de época del arte peruano entre 1980 y 1992, periodo que denomina metafóricamente «República de Weimar peruana». Su marco conceptual adapta la dialéctica benjaminiana entre proximidad y distancia (el aura, su pérdida por la reproductibilidad técnica y su posible restauración) y las categorías de alegoría, montaje y apropiación de Owens, Foster y Craig Owens a una periferia extrema. El argumento se sostiene sobre el análisis iconográfico minucioso de dos o tres obras que abren y cierran la década. La primera, «Arte al paso» y sobre todo «Sarita Colonia» (1980) del taller E.P.S. Huayco: una enorme estampa de la santa migrante pintada sobre diez mil latas de leche y emplazada en la Panamericana Sur, que Buntinx lee como huaca (post)moderna y exvoto donde lo pequeñoburgués radical se articula figuradamente a lo popular en emergencia (el «pop achorado» y «chicha»). La segunda, «Maorilyn» / «Viva el maoísmo» (1989) del Taller NN: una serigrafía que travistió el rostro de Mao con labios warholianos, alegoría ambivalente de la violencia senderista y la estetización de la política. Su tesis vincula la desintegración social —hiperinflación, guerra civil, movida subte punk— con el desarrollo de una condición alegórica y neo-aurática; su aporte es un modelo teórico para leer el colectivismo y la (post)modernidad popular peruana.</t>
         </is>
       </c>
     </row>
@@ -2974,27 +2974,27 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>López, Miguel A. - F(r)icciones cosmopolitas. Redefiniciones estéticas y políticas de una idea de vanguardia en los años 60s.txt</t>
+          <t>Lerner - Formando la colección de arte contemporáneo del MALI (2013).txt</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>1960-1976 (con antecedentes desde 1942-1947)</t>
+          <t>mediados de los años 60 - 2013 (con foco en 1980-2000)</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Ensayo académico / capítulo de catálogo (MALI), s/f</t>
+          <t>Ensayo de catálogo de colección, 2013</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Miguel A. López; Emilio Tarazona; Juan Acha; Fernando de Szyszlo; Jorge Romero Brest; Teresa Burga; Rafael Hastings; Grupo Arte Nuevo; Jesús Ruiz Durand; José Gómez Sicre; Marta Traba; Instituto de Arte Contemporáneo (IAC); MoMA / Instituto Di Tella</t>
+          <t>Sharon Lerner; Museo de Arte de Lima (MALI); Tatiana Cuevas; Miguel A. López; Gustavo Buntinx; Rodrigo Quijano; Jorge Villacorta; Natalia Majluf; E.P.S. Huayco; Teresa Burga; Milagros de la Torre; Flavia Gandolfo</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>López reconstruye las mutaciones semánticas y políticas de la noción de vanguardia en el Perú entre los años sesenta y setenta, argumentando que la euforia cosmopolita del periodo fue el espejismo de una modernidad desarrollista tan prometedora como inacabada en un país socialmente fracturado. El objeto de estudio son las plataformas institucionales privadas (IAC, galerías, bienales americanas, concursos empresariales) que, apuntaladas por el panamericanismo de la Guerra Fría, la Alianza para el Progreso y la política curatorial estadounidense de José Gómez Sicre, promovieron primero la abstracción y luego el arte óptico, el pop y las ambientaciones. El texto traza el paso del declive de la abstracción szyszliana hacia el experimentalismo detonado por las conferencias de Jorge Romero Brest (1965) y la irrupción beligerante del grupo Arte Nuevo (1966-1968) contra el Festival Americano de Pintura. El marco conceptual articula la relación entre desarrollismo y vanguardia, y su posterior tensión con el subdesarrollo, siguiendo la radicalización de Juan Acha, quien tras 1968 y el golpe de Velasco redefine la vanguardia como 'guerrilla cultural' y horizonte revolucionario, hasta su exilio a México en 1971. López destaca las reconversiones de Teresa Burga y Rafael Hastings, el 'pop achorado' de Ruiz Durand al servicio de la Reforma Agraria, los festivales Contacta y las Carreras de chasquis. Su aporte es mostrar cómo la condición local, provinciana y periférica de las prácticas de los setenta y ochenta (Paréntesis, E.P.S. Huayco, Grupo Chaclacayo) actualizó de modo radical las pretensiones críticas sesenteras, canibalizando los conceptos metropolitanos de arte conceptual.</t>
+          <t>Ensayo introductorio de Sharon Lerner al libro que presenta la colección de arte contemporáneo del Museo de Arte de Lima (MALI), articulado como una lectura —entre muchas posibles— de la historia del arte reciente peruano a partir del acervo. Su tesis metodológica es que en el Perú el tránsito a la contemporaneidad no ocurre como un quiebre radical, sino como una serie de pequeños cambios discontinuos, por lo que la colección se organiza en dos principios: identificar momentos de ruptura de fines del siglo XX y perfilar la producción reciente por ejes temáticos. El recorrido histórico parte de mediados de los sesenta (vanguardias pop, experimentalismo, no-objetualismo) y sitúa el verdadero cambio de paradigma a fines de los setenta, cuando la migración y la sentencia de Mirko Lauer —«En el Perú, hoy, solo lo popular es moderno»— enmarcan la obra de E.P.S. Huayco. Recorre luego la hegemonía de la abstracción en los ochenta, el arte de derechos humanos de Ricardo Wiesse y Eduardo Villanes bajo el fujimorato, la irrupción de la Bienal Iberoamericana de Lima (1997) y el «bienalismo», y la generación de los 2000 (Flavia Gandolfo, Gilda Mantilla, Armando Andrade Tudela) vinculada al espacio La Culpable. El texto presenta además los ensayos de Miguel López, Gustavo Buntinx y Rodrigo Quijano incluidos en el volumen y la conversación de seis críticos (2011). Su aporte es explicitar la política de adquisiciones del MALI y su ambición de llenar el vacío institucional y discursivo, construyendo un marco regional e internacional para el arte peruano.</t>
         </is>
       </c>
     </row>
@@ -3006,27 +3006,27 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Quijano - Notas incompletas sobre el sitio de la fotografía peruana.md</t>
+          <t>López, Miguel A. - F(r)icciones cosmopolitas. Redefiniciones estéticas y políticas de una idea de vanguardia en los años 60s.txt</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>1900-2011 (con énfasis en 1920-1998)</t>
+          <t>1960-1976 (con antecedentes desde 1942-1947)</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Ensayo de catálogo (MALI), s/f</t>
+          <t>Ensayo académico / capítulo de catálogo (MALI), s/f</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Rodrigo Quijano; Martín Chambi; José María Eguren; Carlos 'Chino' Domínguez; Aaron Siskind; Jesús Ruiz Durand; Claudia Martínez Garay; Daniela Ortiz; Foto Galería Secuencia; TAFOS; Taller NN; E.P.S. Huayco</t>
+          <t>Miguel A. López; Emilio Tarazona; Juan Acha; Fernando de Szyszlo; Jorge Romero Brest; Teresa Burga; Rafael Hastings; Grupo Arte Nuevo; Jesús Ruiz Durand; José Gómez Sicre; Marta Traba; Instituto de Arte Contemporáneo (IAC); MoMA / Instituto Di Tella</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>Quijano ensaya una genealogía del 'sitio' de la fotografía peruana, sosteniendo que este medio inauguró un margen de creación moderno al margen de la institucionalidad académica de las bellas artes, alcanzando una temprana ubicuidad territorial y una masividad que condicionó la percepción misma de una realidad nacional. El texto, de estructura fragmentaria y numerada, contrapone dos matrices fundacionales: Martín Chambi como 'modernista sin modernidad' y profesional de la imagen surgido de una familia campesina andina —una 'oportunidad nacional'— frente a la miniatura pinhole intimista y hermética de José María Eguren, que prefigura la figura del fotógrafo-artista individual. Analiza a Carlos 'Chino' Domínguez como ojo testimonial de la urbanización y la nueva cultura popular (La resaca del Inca, el 'Cholo' Sotil, el filme Cholo y su reedición Mi cholo de Gruenberg), y la experiencia de la fotogalería Secuencia (1977-1980), que reinventó una tradición y un discurso del oficio adoptando a Minor White y Aaron Siskind. El marco conceptual enlaza fotografía, prensa y democratización de la imagen en el contexto del auge sindical y la repolitización popular de fines de los setenta, y la aparición de la fotoserigrafía disidente (Bedoya, Williams, Mariotti, Salazar) como catalizador de una nueva condición fotográfica colectiva, desde E.P.S. Huayco hasta el Taller NN. El aporte del texto es leer la fotografía como dispositivo de documento, archivo, memoria y duelo frente a la violencia política (Uchuraccay, Yuyanapaq), rastreando su 'grado cero' icónico en obras de Ruiz Durand, Claudia Martínez Garay y Daniela Ortiz, que develan la mirada colonial y la invisibilización étnica.</t>
+          <t>López reconstruye las mutaciones semánticas y políticas de la noción de vanguardia en el Perú entre los años sesenta y setenta, argumentando que la euforia cosmopolita del periodo fue el espejismo de una modernidad desarrollista tan prometedora como inacabada en un país socialmente fracturado. El objeto de estudio son las plataformas institucionales privadas (IAC, galerías, bienales americanas, concursos empresariales) que, apuntaladas por el panamericanismo de la Guerra Fría, la Alianza para el Progreso y la política curatorial estadounidense de José Gómez Sicre, promovieron primero la abstracción y luego el arte óptico, el pop y las ambientaciones. El texto traza el paso del declive de la abstracción szyszliana hacia el experimentalismo detonado por las conferencias de Jorge Romero Brest (1965) y la irrupción beligerante del grupo Arte Nuevo (1966-1968) contra el Festival Americano de Pintura. El marco conceptual articula la relación entre desarrollismo y vanguardia, y su posterior tensión con el subdesarrollo, siguiendo la radicalización de Juan Acha, quien tras 1968 y el golpe de Velasco redefine la vanguardia como 'guerrilla cultural' y horizonte revolucionario, hasta su exilio a México en 1971. López destaca las reconversiones de Teresa Burga y Rafael Hastings, el 'pop achorado' de Ruiz Durand al servicio de la Reforma Agraria, los festivales Contacta y las Carreras de chasquis. Su aporte es mostrar cómo la condición local, provinciana y periférica de las prácticas de los setenta y ochenta (Paréntesis, E.P.S. Huayco, Grupo Chaclacayo) actualizó de modo radical las pretensiones críticas sesenteras, canibalizando los conceptos metropolitanos de arte conceptual.</t>
         </is>
       </c>
     </row>
@@ -3038,32 +3038,64 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
+          <t>Quijano - Notas incompletas sobre el sitio de la fotografía peruana.md</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>1900-2011 (con énfasis en 1920-1998)</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Ensayo de catálogo (MALI), s/f</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>Rodrigo Quijano; Martín Chambi; José María Eguren; Carlos 'Chino' Domínguez; Aaron Siskind; Jesús Ruiz Durand; Claudia Martínez Garay; Daniela Ortiz; Foto Galería Secuencia; TAFOS; Taller NN; E.P.S. Huayco</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>Quijano ensaya una genealogía del 'sitio' de la fotografía peruana, sosteniendo que este medio inauguró un margen de creación moderno al margen de la institucionalidad académica de las bellas artes, alcanzando una temprana ubicuidad territorial y una masividad que condicionó la percepción misma de una realidad nacional. El texto, de estructura fragmentaria y numerada, contrapone dos matrices fundacionales: Martín Chambi como 'modernista sin modernidad' y profesional de la imagen surgido de una familia campesina andina —una 'oportunidad nacional'— frente a la miniatura pinhole intimista y hermética de José María Eguren, que prefigura la figura del fotógrafo-artista individual. Analiza a Carlos 'Chino' Domínguez como ojo testimonial de la urbanización y la nueva cultura popular (La resaca del Inca, el 'Cholo' Sotil, el filme Cholo y su reedición Mi cholo de Gruenberg), y la experiencia de la fotogalería Secuencia (1977-1980), que reinventó una tradición y un discurso del oficio adoptando a Minor White y Aaron Siskind. El marco conceptual enlaza fotografía, prensa y democratización de la imagen en el contexto del auge sindical y la repolitización popular de fines de los setenta, y la aparición de la fotoserigrafía disidente (Bedoya, Williams, Mariotti, Salazar) como catalizador de una nueva condición fotográfica colectiva, desde E.P.S. Huayco hasta el Taller NN. El aporte del texto es leer la fotografía como dispositivo de documento, archivo, memoria y duelo frente a la violencia política (Uchuraccay, Yuyanapaq), rastreando su 'grado cero' icónico en obras de Ruiz Durand, Claudia Martínez Garay y Daniela Ortiz, que develan la mirada colonial y la invisibilización étnica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Cap 2 - Historia/MALI</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
           <t>Villacorta (ed.) - ¿Un arte visual a contrapelo de los dictados metropolitanos? En el Perú, el arte moderno es un gesto tardío [conversación en el MALI, 2011].txt</t>
         </is>
       </c>
-      <c r="C81" s="2" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>1947-2011 (con eje en 1960-2002)</t>
         </is>
       </c>
-      <c r="D81" s="2" t="inlineStr">
+      <c r="D82" s="2" t="inlineStr">
         <is>
           <t>Transcripción editada de conversación (MALI), 2011</t>
         </is>
       </c>
-      <c r="E81" s="3" t="inlineStr">
+      <c r="E82" s="3" t="inlineStr">
         <is>
           <t>Jorge Villacorta; Gustavo Buntinx; Miguel A. López; Rodrigo Quijano; Tatiana Cuevas; Natalia Majluf; E.P.S. Huayco; Grupo Arte Nuevo; Taller NN; Grupo Chaclacayo; Christian Bendayán; Fernando Bryce; MALI / Micromuseo</t>
         </is>
       </c>
-      <c r="F81" s="3" t="inlineStr">
+      <c r="F82" s="3" t="inlineStr">
         <is>
           <t>Editada por Villacorta a partir de dos sesiones de 2011 en el MALI, esta conversación a seis voces indaga si lo moderno está clausurado en el arte peruano de modo que permita definir lo contemporáneo. La tesis articuladora, propuesta por Quijano, es que en el Perú lo moderno solo ha podido darse 'a contrapelo' y como 'gesto tardío', a destiempo de las modernidades metropolitanas; López y Buntinx la matizan con la idea de temporalidades dislocadas y friccionadas que impiden toda historia lineal. El objeto de estudio es la genealogía de la vanguardia local: la contraposición entre Arte Nuevo (1966-1968), leído como destello cosmopolita fugaz, y E.P.S. Huayco y Paréntesis, cuya apropiación de Sarita Colonia y el 'pop achorado' marca una ruptura más perdurable y pertinente al medio. Buntinx despliega una secuencia estilístico-conceptual en clave pop/místico-libidinal —de la Twiggy de Emilio Hernández a Quistococha de Bendayán, pasando por el afiche de Ruiz Durand, la Maoirilyn del Taller NN y La Pachakuti de Alfredo Márquez— ligada a periodos políticos (desarrollismo, velasquismo, utopía socialista, dictadura fujimorista, revolución capitalista). Majluf sitúa el quiebre epocal de fin de siglo en el ingreso de la 'referencia' fotográfica (Bryce, Milagros de la Torre, Juan Enrique Bedoya, Mantilla), frente al neobarroco. El texto discute además la construcción de públicos, la institucionalidad faltante, el rol del curador, el mercado 'social' peruano, las subastas del MALI y la 'normalización de la diferencia' como riesgo de la consagración institucional del pasado radical.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F81"/>
+  <autoFilter ref="A1:F82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>